<commit_message>
051425 - updated path to Week 2 results
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AF085A-653B-A142-B331-4B8594B8F56F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05896015-2EE1-2B47-8D47-2DD04256C773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9380" yWindow="1140" windowWidth="27640" windowHeight="16940" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -311,7 +311,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -824,37 +824,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -964,124 +938,130 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1433,65 +1413,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="51" t="s">
+      <c r="B1" s="56"/>
+      <c r="C1" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="53" t="s">
+      <c r="D1" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="53" t="s">
+      <c r="E1" s="64"/>
+      <c r="F1" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="G1" s="54"/>
-      <c r="H1" s="55" t="s">
+      <c r="G1" s="64"/>
+      <c r="H1" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="58" t="s">
+      <c r="I1" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="60"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="77"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="47"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="61">
+      <c r="A2" s="57"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="65">
         <v>45782</v>
       </c>
-      <c r="E2" s="62"/>
-      <c r="F2" s="61">
+      <c r="E2" s="66"/>
+      <c r="F2" s="65">
         <v>45789</v>
       </c>
-      <c r="G2" s="62"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="63" t="s">
+      <c r="G2" s="66"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="65" t="s">
+      <c r="J2" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="K2" s="67" t="s">
+      <c r="K2" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="L2" s="63" t="s">
+      <c r="L2" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="43" t="s">
+      <c r="M2" s="78" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="49"/>
-      <c r="B3" s="50"/>
-      <c r="C3" s="52"/>
+      <c r="A3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="62"/>
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1504,12 +1484,12 @@
       <c r="G3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="57"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="69"/>
-      <c r="M3" s="44"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="79"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
@@ -1521,19 +1501,18 @@
       <c r="C4" s="5">
         <v>15</v>
       </c>
-      <c r="D4" s="70" t="s">
+      <c r="D4" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="71"/>
+      <c r="E4" s="48"/>
       <c r="F4" s="6">
         <v>42</v>
       </c>
       <c r="G4" s="7">
         <v>27</v>
       </c>
-      <c r="H4" s="8" t="str">
-        <f t="shared" ref="H4:H15" si="0">D4</f>
-        <v>RAIN OUT</v>
+      <c r="H4" s="8">
+        <v>42</v>
       </c>
       <c r="I4" s="9">
         <v>1</v>
@@ -1541,10 +1520,10 @@
       <c r="J4" s="10"/>
       <c r="K4" s="7"/>
       <c r="L4" s="8">
-        <f>E4+G4+J4+K4</f>
+        <f t="shared" ref="L4:L12" si="0">E4+G4+J4+K4</f>
         <v>27</v>
       </c>
-      <c r="M4" s="72">
+      <c r="M4" s="43">
         <f t="shared" ref="M4:M12" si="1">L4/I4</f>
         <v>27</v>
       </c>
@@ -1559,8 +1538,8 @@
       <c r="C5" s="13">
         <v>13</v>
       </c>
-      <c r="D5" s="73"/>
-      <c r="E5" s="74"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="50"/>
       <c r="F5" s="14">
         <v>42</v>
       </c>
@@ -1568,8 +1547,7 @@
         <v>25</v>
       </c>
       <c r="H5" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="I5" s="17">
         <v>1</v>
@@ -1579,10 +1557,10 @@
       </c>
       <c r="K5" s="15"/>
       <c r="L5" s="16">
-        <f>E5+G5+J5+K5</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="M5" s="75">
+      <c r="M5" s="44">
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
@@ -1597,8 +1575,8 @@
       <c r="C6" s="13">
         <v>22</v>
       </c>
-      <c r="D6" s="73"/>
-      <c r="E6" s="74"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="50"/>
       <c r="F6" s="19">
         <v>53</v>
       </c>
@@ -1606,8 +1584,7 @@
         <v>23</v>
       </c>
       <c r="H6" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="I6" s="17">
         <v>1</v>
@@ -1615,10 +1592,10 @@
       <c r="J6" s="18"/>
       <c r="K6" s="15"/>
       <c r="L6" s="16">
-        <f>E6+G6+J6+K6</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="M6" s="75">
+      <c r="M6" s="44">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
@@ -1633,8 +1610,8 @@
       <c r="C7" s="13">
         <v>8</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="74"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="50"/>
       <c r="F7" s="20">
         <v>45</v>
       </c>
@@ -1642,8 +1619,7 @@
         <v>17</v>
       </c>
       <c r="H7" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I7" s="17">
         <v>1</v>
@@ -1653,10 +1629,10 @@
         <v>1</v>
       </c>
       <c r="L7" s="16">
-        <f>E7+G7+J7+K7</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="M7" s="75">
+      <c r="M7" s="44">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -1671,8 +1647,8 @@
       <c r="C8" s="13">
         <v>22</v>
       </c>
-      <c r="D8" s="73"/>
-      <c r="E8" s="74"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="50"/>
       <c r="F8" s="19">
         <v>59</v>
       </c>
@@ -1680,8 +1656,7 @@
         <v>17</v>
       </c>
       <c r="H8" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="I8" s="17">
         <v>1</v>
@@ -1689,10 +1664,10 @@
       <c r="J8" s="18"/>
       <c r="K8" s="15"/>
       <c r="L8" s="16">
-        <f>E8+G8+J8+K8</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="M8" s="75">
+      <c r="M8" s="44">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
@@ -1707,8 +1682,8 @@
       <c r="C9" s="13">
         <v>8</v>
       </c>
-      <c r="D9" s="73"/>
-      <c r="E9" s="74"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
       <c r="F9" s="19">
         <v>46</v>
       </c>
@@ -1716,8 +1691,7 @@
         <v>16</v>
       </c>
       <c r="H9" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="I9" s="17">
         <v>1</v>
@@ -1725,10 +1699,10 @@
       <c r="J9" s="18"/>
       <c r="K9" s="15"/>
       <c r="L9" s="16">
-        <f>E9+G9+J9+K9</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="M9" s="75">
+      <c r="M9" s="44">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -1743,8 +1717,8 @@
       <c r="C10" s="13">
         <v>17</v>
       </c>
-      <c r="D10" s="73"/>
-      <c r="E10" s="74"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
       <c r="F10" s="19">
         <v>55</v>
       </c>
@@ -1752,8 +1726,7 @@
         <v>16</v>
       </c>
       <c r="H10" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I10" s="17">
         <v>1</v>
@@ -1761,10 +1734,10 @@
       <c r="J10" s="18"/>
       <c r="K10" s="15"/>
       <c r="L10" s="16">
-        <f>E10+G10+J10+K10</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="M10" s="75">
+      <c r="M10" s="44">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -1779,8 +1752,8 @@
       <c r="C11" s="13">
         <v>18</v>
       </c>
-      <c r="D11" s="73"/>
-      <c r="E11" s="74"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
       <c r="F11" s="19">
         <v>56</v>
       </c>
@@ -1788,8 +1761,7 @@
         <v>16</v>
       </c>
       <c r="H11" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="I11" s="17">
         <v>1</v>
@@ -1797,10 +1769,10 @@
       <c r="J11" s="18"/>
       <c r="K11" s="15"/>
       <c r="L11" s="16">
-        <f>E11+G11+J11+K11</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="M11" s="75">
+      <c r="M11" s="44">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -1815,8 +1787,8 @@
       <c r="C12" s="13">
         <v>21</v>
       </c>
-      <c r="D12" s="73"/>
-      <c r="E12" s="74"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
       <c r="F12" s="21">
         <v>61</v>
       </c>
@@ -1824,8 +1796,7 @@
         <v>14</v>
       </c>
       <c r="H12" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="I12" s="17">
         <v>1</v>
@@ -1835,10 +1806,10 @@
       </c>
       <c r="K12" s="15"/>
       <c r="L12" s="16">
-        <f>E12+G12+J12+K12</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="M12" s="75">
+      <c r="M12" s="44">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
@@ -1853,15 +1824,14 @@
       <c r="C13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="73"/>
-      <c r="E13" s="74"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
       <c r="F13" s="19">
         <v>41</v>
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I13" s="17">
         <v>1</v>
@@ -1869,7 +1839,7 @@
       <c r="J13" s="18"/>
       <c r="K13" s="15"/>
       <c r="L13" s="16"/>
-      <c r="M13" s="75"/>
+      <c r="M13" s="44"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
@@ -1881,23 +1851,22 @@
       <c r="C14" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="73"/>
-      <c r="E14" s="74"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
       <c r="F14" s="19">
         <v>46</v>
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="I14" s="17">
         <v>1</v>
       </c>
       <c r="J14" s="19"/>
-      <c r="K14" s="76"/>
+      <c r="K14" s="45"/>
       <c r="L14" s="16"/>
-      <c r="M14" s="75"/>
+      <c r="M14" s="44"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
@@ -1909,15 +1878,14 @@
       <c r="C15" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="73"/>
-      <c r="E15" s="74"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
       <c r="F15" s="19">
         <v>51</v>
       </c>
       <c r="G15" s="15"/>
       <c r="H15" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I15" s="17">
         <v>1</v>
@@ -1925,7 +1893,7 @@
       <c r="J15" s="18"/>
       <c r="K15" s="15"/>
       <c r="L15" s="16"/>
-      <c r="M15" s="75"/>
+      <c r="M15" s="44"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
@@ -1937,8 +1905,8 @@
       <c r="C16" s="13">
         <v>13</v>
       </c>
-      <c r="D16" s="73"/>
-      <c r="E16" s="74"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
       <c r="F16" s="22"/>
       <c r="G16" s="15"/>
       <c r="H16" s="16"/>
@@ -1946,7 +1914,7 @@
       <c r="J16" s="18"/>
       <c r="K16" s="15"/>
       <c r="L16" s="16"/>
-      <c r="M16" s="75"/>
+      <c r="M16" s="44"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
@@ -1958,8 +1926,8 @@
       <c r="C17" s="13">
         <v>2</v>
       </c>
-      <c r="D17" s="73"/>
-      <c r="E17" s="74"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
       <c r="F17" s="23"/>
       <c r="G17" s="15"/>
       <c r="H17" s="16"/>
@@ -1967,7 +1935,7 @@
       <c r="J17" s="18"/>
       <c r="K17" s="15"/>
       <c r="L17" s="16"/>
-      <c r="M17" s="75"/>
+      <c r="M17" s="44"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
@@ -1979,8 +1947,8 @@
       <c r="C18" s="13">
         <v>15</v>
       </c>
-      <c r="D18" s="73"/>
-      <c r="E18" s="74"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
       <c r="F18" s="19"/>
       <c r="G18" s="15"/>
       <c r="H18" s="16"/>
@@ -1988,7 +1956,7 @@
       <c r="J18" s="18"/>
       <c r="K18" s="15"/>
       <c r="L18" s="16"/>
-      <c r="M18" s="75"/>
+      <c r="M18" s="44"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
@@ -2000,8 +1968,8 @@
       <c r="C19" s="13">
         <v>11</v>
       </c>
-      <c r="D19" s="73"/>
-      <c r="E19" s="74"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
       <c r="F19" s="19"/>
       <c r="G19" s="15"/>
       <c r="H19" s="16"/>
@@ -2009,7 +1977,7 @@
       <c r="J19" s="18"/>
       <c r="K19" s="15"/>
       <c r="L19" s="16"/>
-      <c r="M19" s="75"/>
+      <c r="M19" s="44"/>
     </row>
     <row r="20" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
@@ -2021,8 +1989,8 @@
       <c r="C20" s="26">
         <v>15</v>
       </c>
-      <c r="D20" s="77"/>
-      <c r="E20" s="78"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="52"/>
       <c r="F20" s="27"/>
       <c r="G20" s="28"/>
       <c r="H20" s="29"/>
@@ -2030,23 +1998,20 @@
       <c r="J20" s="31"/>
       <c r="K20" s="28"/>
       <c r="L20" s="29"/>
-      <c r="M20" s="79"/>
+      <c r="M20" s="46"/>
     </row>
     <row r="21" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="80"/>
       <c r="B21" s="81"/>
-      <c r="C21" s="81"/>
-      <c r="D21" s="82" t="e">
-        <f>AVERAGEIF(D4:D20,"&gt;0")</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E21" s="82"/>
-      <c r="F21" s="82">
+      <c r="C21" s="82"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83">
         <f>AVERAGEIF(F4:F20,"&gt;0")</f>
         <v>49.75</v>
       </c>
-      <c r="G21" s="82"/>
-      <c r="H21" s="81"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="84"/>
       <c r="I21" s="32"/>
       <c r="J21" s="32"/>
       <c r="K21" s="32"/>

</xml_diff>

<commit_message>
060125 - updated week 4 scores
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05896015-2EE1-2B47-8D47-2DD04256C773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32126D39-CE49-184A-9648-86A3A1F6E622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9380" yWindow="1140" windowWidth="27640" windowHeight="16940" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="10760" yWindow="3400" windowWidth="27640" windowHeight="16940" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -171,32 +171,29 @@
     <t>Closest #4</t>
   </si>
   <si>
-    <t>RED</t>
-  </si>
-  <si>
     <t>Closest #7</t>
   </si>
   <si>
-    <t>GREEN</t>
-  </si>
-  <si>
-    <t>Both</t>
-  </si>
-  <si>
-    <t>BLUE</t>
-  </si>
-  <si>
     <t>WEEK 2</t>
   </si>
   <si>
     <t>RAIN OUT</t>
+  </si>
+  <si>
+    <t>WEEK 3</t>
+  </si>
+  <si>
+    <t>WEEK 4</t>
+  </si>
+  <si>
+    <t>Closest Both</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -290,6 +287,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -311,7 +315,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="40">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -587,6 +591,21 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="medium">
         <color indexed="64"/>
@@ -594,34 +613,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="medium">
         <color indexed="64"/>
@@ -664,6 +655,129 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
       <top style="medium">
         <color indexed="64"/>
@@ -674,54 +788,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -732,90 +799,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -828,7 +813,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -837,75 +822,66 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
@@ -938,17 +914,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
@@ -968,10 +965,43 @@
     <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1004,66 +1034,21 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1398,80 +1383,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.33203125" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="7" width="7.5" customWidth="1"/>
-    <col min="8" max="8" width="7.1640625" customWidth="1"/>
-    <col min="9" max="9" width="9.1640625" customWidth="1"/>
-    <col min="10" max="10" width="6.5" customWidth="1"/>
-    <col min="11" max="11" width="6.33203125" customWidth="1"/>
-    <col min="12" max="12" width="7.6640625" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="4" max="5" width="5.83203125" hidden="1" customWidth="1"/>
+    <col min="6" max="11" width="5.83203125" customWidth="1"/>
+    <col min="12" max="16" width="6.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:17" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="61" t="s">
+      <c r="B1" s="71"/>
+      <c r="C1" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="63" t="s">
+      <c r="D1" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="64"/>
-      <c r="F1" s="63" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="64"/>
-      <c r="H1" s="72" t="s">
+      <c r="E1" s="79"/>
+      <c r="F1" s="78" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="79"/>
+      <c r="H1" s="78" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" s="79"/>
+      <c r="J1" s="78" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="79"/>
+      <c r="L1" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="75" t="s">
+      <c r="M1" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="77"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="57"/>
-      <c r="B2" s="58"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="65">
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="61"/>
+    </row>
+    <row r="2" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="72"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="62">
         <v>45782</v>
       </c>
-      <c r="E2" s="66"/>
-      <c r="F2" s="65">
+      <c r="E2" s="63"/>
+      <c r="F2" s="62">
         <v>45789</v>
       </c>
-      <c r="G2" s="66"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="53" t="s">
+      <c r="G2" s="63"/>
+      <c r="H2" s="62">
+        <v>45796</v>
+      </c>
+      <c r="I2" s="63"/>
+      <c r="J2" s="62">
+        <v>45803</v>
+      </c>
+      <c r="K2" s="63"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="68" t="s">
+      <c r="N2" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="K2" s="70" t="s">
+      <c r="O2" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="L2" s="53" t="s">
+      <c r="P2" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="78" t="s">
+      <c r="Q2" s="81" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59"/>
-      <c r="B3" s="60"/>
-      <c r="C3" s="62"/>
+    <row r="3" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="74"/>
+      <c r="B3" s="75"/>
+      <c r="C3" s="77"/>
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1484,14 +1483,26 @@
       <c r="G3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="74"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="54"/>
-      <c r="M3" s="79"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="58"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="82"/>
+    </row>
+    <row r="4" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -1501,578 +1512,713 @@
       <c r="C4" s="5">
         <v>15</v>
       </c>
-      <c r="D4" s="47" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="48"/>
+      <c r="D4" s="51" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="52"/>
       <c r="F4" s="6">
         <v>42</v>
       </c>
       <c r="G4" s="7">
         <v>27</v>
       </c>
-      <c r="H4" s="8">
-        <v>42</v>
-      </c>
-      <c r="I4" s="9">
-        <v>1</v>
-      </c>
-      <c r="J4" s="10"/>
+      <c r="H4" s="51" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="52"/>
+      <c r="J4" s="6"/>
       <c r="K4" s="7"/>
       <c r="L4" s="8">
-        <f t="shared" ref="L4:L12" si="0">E4+G4+J4+K4</f>
+        <f t="shared" ref="L4:L13" si="0">F4+J4</f>
+        <v>42</v>
+      </c>
+      <c r="M4" s="47">
+        <v>1</v>
+      </c>
+      <c r="N4" s="9"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="8">
+        <f t="shared" ref="P4:P20" si="1">G4+K4+N4+O4</f>
         <v>27</v>
       </c>
-      <c r="M4" s="43">
-        <f t="shared" ref="M4:M12" si="1">L4/I4</f>
+      <c r="Q4" s="40">
+        <f t="shared" ref="Q4:Q13" si="2">P4/M4</f>
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="12">
         <v>13</v>
       </c>
-      <c r="D5" s="49"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="14">
+      <c r="D5" s="53"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="83">
         <v>42</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="14">
         <v>25</v>
       </c>
-      <c r="H5" s="16">
+      <c r="H5" s="53"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="15">
+        <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="I5" s="17">
+      <c r="M5" s="48">
         <v>1</v>
       </c>
-      <c r="J5" s="18">
+      <c r="N5" s="16">
         <v>1</v>
       </c>
-      <c r="K5" s="15"/>
-      <c r="L5" s="16">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="M5" s="44">
+      <c r="O5" s="14"/>
+      <c r="P5" s="15">
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+      <c r="Q5" s="41">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="12">
         <v>22</v>
       </c>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="19">
+      <c r="D6" s="53"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="17">
         <v>53</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="14">
         <v>23</v>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="53"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="15">
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="I6" s="17">
+      <c r="M6" s="48">
         <v>1</v>
       </c>
-      <c r="J6" s="18"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="16">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="M6" s="44">
+      <c r="N6" s="16"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="15">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
+      <c r="Q6" s="41">
+        <f t="shared" si="2"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="12">
         <v>8</v>
       </c>
-      <c r="D7" s="49"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="20">
+      <c r="D7" s="53"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="18">
         <v>45</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="14">
         <v>17</v>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="53"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="15">
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="I7" s="17">
+      <c r="M7" s="48">
         <v>1</v>
       </c>
-      <c r="J7" s="18"/>
-      <c r="K7" s="15">
+      <c r="N7" s="16"/>
+      <c r="O7" s="14">
         <v>1</v>
       </c>
-      <c r="L7" s="16">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="M7" s="44">
+      <c r="P7" s="15">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
+      <c r="Q7" s="41">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="12">
+        <v>21</v>
+      </c>
+      <c r="D8" s="53"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="19">
+        <v>61</v>
+      </c>
+      <c r="G8" s="14">
+        <v>14</v>
+      </c>
+      <c r="H8" s="53"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="19">
+        <v>56</v>
+      </c>
+      <c r="K8" s="14">
         <v>19</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="L8" s="15">
+        <f t="shared" si="0"/>
+        <v>117</v>
+      </c>
+      <c r="M8" s="48">
+        <v>2</v>
+      </c>
+      <c r="N8" s="16">
+        <v>2</v>
+      </c>
+      <c r="O8" s="14"/>
+      <c r="P8" s="15">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="Q8" s="41">
+        <f t="shared" si="2"/>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C9" s="12">
         <v>22</v>
       </c>
-      <c r="D8" s="49"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="19">
+      <c r="D9" s="53"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="17">
         <v>59</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G9" s="14">
         <v>17</v>
       </c>
-      <c r="H8" s="16">
+      <c r="H9" s="53"/>
+      <c r="I9" s="54"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="15">
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="I8" s="17">
+      <c r="M9" s="48">
         <v>1</v>
       </c>
-      <c r="J8" s="18"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="16">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="M8" s="44">
+      <c r="N9" s="16"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="15">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="13">
-        <v>8</v>
-      </c>
-      <c r="D9" s="49"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="19">
-        <v>46</v>
-      </c>
-      <c r="G9" s="15">
+      <c r="Q9" s="41">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="12">
+        <v>15</v>
+      </c>
+      <c r="D10" s="53"/>
+      <c r="E10" s="54"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="53"/>
+      <c r="I10" s="54"/>
+      <c r="J10" s="17">
+        <v>52</v>
+      </c>
+      <c r="K10" s="14">
+        <v>17</v>
+      </c>
+      <c r="L10" s="15">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="M10" s="48">
+        <v>1</v>
+      </c>
+      <c r="N10" s="16"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="15">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="Q10" s="41">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A11" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="12">
+        <v>18</v>
+      </c>
+      <c r="D11" s="53"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="17">
+        <v>56</v>
+      </c>
+      <c r="G11" s="14">
         <v>16</v>
       </c>
-      <c r="H9" s="16">
-        <v>46</v>
-      </c>
-      <c r="I9" s="17">
+      <c r="H11" s="53"/>
+      <c r="I11" s="54"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="15">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+      <c r="M11" s="48">
         <v>1</v>
       </c>
-      <c r="J9" s="18"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="16">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="M9" s="44">
+      <c r="N11" s="16"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="15">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="13">
-        <v>17</v>
-      </c>
-      <c r="D10" s="49"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="19">
-        <v>55</v>
-      </c>
-      <c r="G10" s="15">
+      <c r="Q11" s="41">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="H10" s="16">
-        <v>55</v>
-      </c>
-      <c r="I10" s="17">
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="12">
+        <v>8</v>
+      </c>
+      <c r="D12" s="53"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="17">
+        <v>46</v>
+      </c>
+      <c r="G12" s="14">
+        <v>16</v>
+      </c>
+      <c r="H12" s="53"/>
+      <c r="I12" s="54"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="15">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="M12" s="48">
         <v>1</v>
       </c>
-      <c r="J10" s="18"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="16">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="M10" s="44">
+      <c r="N12" s="16"/>
+      <c r="O12" s="14"/>
+      <c r="P12" s="15">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="13">
-        <v>18</v>
-      </c>
-      <c r="D11" s="49"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="19">
-        <v>56</v>
-      </c>
-      <c r="G11" s="15">
+      <c r="Q12" s="41">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="H11" s="16">
-        <v>56</v>
-      </c>
-      <c r="I11" s="17">
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A13" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="12">
+        <v>17</v>
+      </c>
+      <c r="D13" s="53"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="17">
+        <v>55</v>
+      </c>
+      <c r="G13" s="14">
+        <v>16</v>
+      </c>
+      <c r="H13" s="53"/>
+      <c r="I13" s="54"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="15">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="M13" s="48">
         <v>1</v>
       </c>
-      <c r="J11" s="18"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="16">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="M11" s="44">
+      <c r="N13" s="16"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="15">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="13">
-        <v>21</v>
-      </c>
-      <c r="D12" s="49"/>
-      <c r="E12" s="50"/>
-      <c r="F12" s="21">
-        <v>61</v>
-      </c>
-      <c r="G12" s="15">
-        <v>14</v>
-      </c>
-      <c r="H12" s="16">
-        <v>61</v>
-      </c>
-      <c r="I12" s="17">
+      <c r="Q13" s="41">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="12">
+        <v>13</v>
+      </c>
+      <c r="D14" s="53"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="53"/>
+      <c r="I14" s="54"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="48"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="14"/>
+      <c r="P14" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="41"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="12">
+        <v>2</v>
+      </c>
+      <c r="D15" s="53"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="53"/>
+      <c r="I15" s="54"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="48"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="14"/>
+      <c r="P15" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="41"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="53"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="17">
+        <v>51</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="53"/>
+      <c r="I16" s="54"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="15">
+        <f>F16+J16</f>
+        <v>51</v>
+      </c>
+      <c r="M16" s="48">
         <v>1</v>
       </c>
-      <c r="J12" s="18">
+      <c r="N16" s="16"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q16" s="41"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="53"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="17">
+        <v>46</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="53"/>
+      <c r="I17" s="54"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="15">
+        <f>F17+J17</f>
+        <v>46</v>
+      </c>
+      <c r="M17" s="48">
         <v>1</v>
       </c>
-      <c r="K12" s="15"/>
-      <c r="L12" s="16">
-        <f t="shared" si="0"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="42"/>
+      <c r="P17" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="41"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A18" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="53"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="17">
+        <v>41</v>
+      </c>
+      <c r="G18" s="14"/>
+      <c r="H18" s="53"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="15">
+        <f>F18+J18</f>
+        <v>41</v>
+      </c>
+      <c r="M18" s="48">
+        <v>1</v>
+      </c>
+      <c r="N18" s="16"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="41"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A19" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="12">
         <v>15</v>
       </c>
-      <c r="M12" s="44">
+      <c r="D19" s="53"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="53"/>
+      <c r="I19" s="54"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="48"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="15">
         <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="49"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="19">
-        <v>41</v>
-      </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="16">
-        <v>41</v>
-      </c>
-      <c r="I13" s="17">
-        <v>1</v>
-      </c>
-      <c r="J13" s="18"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="44"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="49"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="19">
-        <v>46</v>
-      </c>
-      <c r="G14" s="15"/>
-      <c r="H14" s="16">
-        <v>46</v>
-      </c>
-      <c r="I14" s="17">
-        <v>1</v>
-      </c>
-      <c r="J14" s="19"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="44"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="41"/>
+    </row>
+    <row r="20" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="49"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="19">
-        <v>51</v>
-      </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16">
-        <v>51</v>
-      </c>
-      <c r="I15" s="17">
-        <v>1</v>
-      </c>
-      <c r="J15" s="18"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="44"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="13">
-        <v>13</v>
-      </c>
-      <c r="D16" s="49"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="44"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="13">
-        <v>2</v>
-      </c>
-      <c r="D17" s="49"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="44"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" s="13">
-        <v>15</v>
-      </c>
-      <c r="D18" s="49"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="44"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="12" t="s">
+      <c r="B20" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C20" s="24">
         <v>11</v>
       </c>
-      <c r="D19" s="49"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="44"/>
-    </row>
-    <row r="20" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="26">
-        <v>15</v>
-      </c>
-      <c r="D20" s="51"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="46"/>
-    </row>
-    <row r="21" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="80"/>
-      <c r="B21" s="81"/>
-      <c r="C21" s="82"/>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="83">
+      <c r="D20" s="55"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="56"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="49"/>
+      <c r="N20" s="28"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="27">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="43"/>
+    </row>
+    <row r="21" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="44"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46">
         <f>AVERAGEIF(F4:F20,"&gt;0")</f>
         <v>49.75</v>
       </c>
-      <c r="G21" s="83"/>
-      <c r="H21" s="84"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C22" s="33"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="34"/>
-      <c r="M22" s="36"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C23" s="37" t="s">
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46">
+        <f>AVERAGEIF(J4:J20,"&gt;0")</f>
+        <v>54</v>
+      </c>
+      <c r="K21" s="46"/>
+      <c r="L21" s="50"/>
+      <c r="M21" s="29"/>
+      <c r="N21" s="29"/>
+      <c r="O21" s="29"/>
+      <c r="P21" s="29"/>
+      <c r="Q21" s="29"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C22" s="30"/>
+      <c r="L22" s="31"/>
+      <c r="M22" s="31"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="31"/>
+      <c r="Q22" s="33"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C23" s="84" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="F23" s="35"/>
+      <c r="H23" s="35"/>
+      <c r="J23" s="34"/>
+      <c r="K23" s="35"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C24" s="85" t="s">
         <v>44</v>
       </c>
-      <c r="F23" s="38"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C24" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="39" t="s">
-        <v>46</v>
-      </c>
-      <c r="F24" s="39"/>
-      <c r="H24" s="40"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C25" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="E25" s="42"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="42"/>
+      <c r="F24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="J24" s="34"/>
+      <c r="K24" s="36"/>
+      <c r="L24" s="37"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C25" s="86" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="39"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="34"/>
+      <c r="K25" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="19">
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
     <mergeCell ref="D4:E20"/>
-    <mergeCell ref="L2:L3"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:H3"/>
-    <mergeCell ref="I1:M1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="H4:I20"/>
+    <mergeCell ref="L1:L3"/>
+    <mergeCell ref="M1:Q1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
060425 - posted scores from week 5 (June 2nd)
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32126D39-CE49-184A-9648-86A3A1F6E622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE152A4-F732-8C46-9333-4E5C8BE3F51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10760" yWindow="3400" windowWidth="27640" windowHeight="16940" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -187,13 +187,31 @@
   </si>
   <si>
     <t>Closest Both</t>
+  </si>
+  <si>
+    <t>WEEK 5</t>
+  </si>
+  <si>
+    <t>Drew</t>
+  </si>
+  <si>
+    <t>Kandrak</t>
+  </si>
+  <si>
+    <t>RED</t>
+  </si>
+  <si>
+    <t>GREEN</t>
+  </si>
+  <si>
+    <t>BLUE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -294,6 +312,11 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -315,7 +338,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -777,7 +800,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
@@ -789,6 +814,21 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -800,7 +840,35 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -813,7 +881,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -835,9 +903,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -852,9 +917,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -884,9 +946,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -901,9 +960,6 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -935,18 +991,24 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -965,6 +1027,30 @@
     <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -980,12 +1066,6 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -998,57 +1078,78 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1383,94 +1484,106 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" customWidth="1"/>
     <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="5" width="5.83203125" hidden="1" customWidth="1"/>
-    <col min="6" max="11" width="5.83203125" customWidth="1"/>
-    <col min="12" max="16" width="6.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.6640625" customWidth="1"/>
+    <col min="4" max="7" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="8" max="13" width="6.83203125" customWidth="1"/>
+    <col min="14" max="14" width="6.33203125" customWidth="1"/>
+    <col min="15" max="15" width="6.83203125" customWidth="1"/>
+    <col min="16" max="16" width="6" customWidth="1"/>
+    <col min="17" max="17" width="5.6640625" customWidth="1"/>
+    <col min="18" max="18" width="5.83203125" customWidth="1"/>
+    <col min="19" max="19" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+    <row r="1" spans="1:19" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="76" t="s">
+      <c r="B1" s="56"/>
+      <c r="C1" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="78" t="s">
+      <c r="D1" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="79"/>
-      <c r="F1" s="78" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="79"/>
-      <c r="H1" s="78" t="s">
+      <c r="G1" s="45"/>
+      <c r="H1" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="79"/>
-      <c r="J1" s="78" t="s">
+      <c r="I1" s="45"/>
+      <c r="J1" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="K1" s="79"/>
-      <c r="L1" s="57" t="s">
+      <c r="K1" s="45"/>
+      <c r="L1" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" s="45"/>
+      <c r="N1" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="59" t="s">
+      <c r="O1" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="61"/>
-    </row>
-    <row r="2" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="72"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="62">
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="67"/>
+    </row>
+    <row r="2" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="57"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="46">
         <v>45782</v>
       </c>
-      <c r="E2" s="63"/>
-      <c r="F2" s="62">
+      <c r="E2" s="47"/>
+      <c r="F2" s="46">
         <v>45789</v>
       </c>
-      <c r="G2" s="63"/>
-      <c r="H2" s="62">
+      <c r="G2" s="47"/>
+      <c r="H2" s="46">
         <v>45796</v>
       </c>
-      <c r="I2" s="63"/>
-      <c r="J2" s="62">
+      <c r="I2" s="47"/>
+      <c r="J2" s="46">
         <v>45803</v>
       </c>
-      <c r="K2" s="63"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="68" t="s">
+      <c r="K2" s="47"/>
+      <c r="L2" s="46">
+        <v>45810</v>
+      </c>
+      <c r="M2" s="47"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="64" t="s">
+      <c r="P2" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="O2" s="66" t="s">
+      <c r="Q2" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="P2" s="68" t="s">
+      <c r="R2" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="Q2" s="81" t="s">
+      <c r="S2" s="73" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="74"/>
-      <c r="B3" s="75"/>
-      <c r="C3" s="77"/>
+    <row r="3" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="62"/>
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1495,730 +1608,853 @@
       <c r="K3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="58"/>
-      <c r="M3" s="80"/>
-      <c r="N3" s="65"/>
-      <c r="O3" s="67"/>
+      <c r="L3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N3" s="64"/>
+      <c r="O3" s="72"/>
       <c r="P3" s="69"/>
-      <c r="Q3" s="82"/>
-    </row>
-    <row r="4" spans="1:17" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q3" s="71"/>
+      <c r="R3" s="72"/>
+      <c r="S3" s="74"/>
+    </row>
+    <row r="4" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C4" s="5">
-        <v>15</v>
-      </c>
-      <c r="D4" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="75"/>
+      <c r="E4" s="93"/>
+      <c r="F4" s="6">
+        <v>53</v>
+      </c>
+      <c r="G4" s="7">
+        <v>23</v>
+      </c>
+      <c r="H4" s="49" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="F4" s="6">
-        <v>42</v>
-      </c>
-      <c r="G4" s="7">
-        <v>27</v>
-      </c>
-      <c r="H4" s="51" t="s">
-        <v>46</v>
-      </c>
-      <c r="I4" s="52"/>
+      <c r="I4" s="50"/>
       <c r="J4" s="6"/>
       <c r="K4" s="7"/>
-      <c r="L4" s="8">
-        <f t="shared" ref="L4:L13" si="0">F4+J4</f>
+      <c r="L4" s="6"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="76">
+        <f>F4+J4+L4</f>
+        <v>53</v>
+      </c>
+      <c r="O4" s="8">
+        <f>COUNTIF(D4:L4,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P4" s="77"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="78">
+        <f>SUMIF(G4:M4, "&lt;30")+P4+Q4</f>
+        <v>23</v>
+      </c>
+      <c r="S4" s="36">
+        <f>R4/O4</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="11">
+        <v>15</v>
+      </c>
+      <c r="D5" s="79" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="94"/>
+      <c r="F5" s="15">
         <v>42</v>
       </c>
-      <c r="M4" s="47">
+      <c r="G5" s="13">
+        <v>27</v>
+      </c>
+      <c r="H5" s="51"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="15">
+        <v>54</v>
+      </c>
+      <c r="M5" s="13">
+        <v>15</v>
+      </c>
+      <c r="N5" s="80">
+        <f>F5+J5+L5</f>
+        <v>96</v>
+      </c>
+      <c r="O5" s="14">
+        <f>COUNTIF(D5:L5,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="P5" s="81"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="82">
+        <f>SUMIF(G5:M5, "&lt;30")+P5+Q5</f>
+        <v>42</v>
+      </c>
+      <c r="S5" s="37">
+        <f>R5/O5</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="11">
+        <v>13</v>
+      </c>
+      <c r="D6" s="79"/>
+      <c r="E6" s="94"/>
+      <c r="F6" s="12">
+        <v>42</v>
+      </c>
+      <c r="G6" s="13">
+        <v>25</v>
+      </c>
+      <c r="H6" s="51"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="83">
+        <v>51</v>
+      </c>
+      <c r="M6" s="13">
+        <v>16</v>
+      </c>
+      <c r="N6" s="80">
+        <f>F6+J6+L6</f>
+        <v>93</v>
+      </c>
+      <c r="O6" s="14">
+        <f>COUNTIF(D6:L6,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="P6" s="81">
         <v>1</v>
       </c>
-      <c r="N4" s="9"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="8">
-        <f t="shared" ref="P4:P20" si="1">G4+K4+N4+O4</f>
+      <c r="Q6" s="13"/>
+      <c r="R6" s="82">
+        <f>SUMIF(G6:M6, "&lt;30")+P6+Q6</f>
+        <v>42</v>
+      </c>
+      <c r="S6" s="37">
+        <f>R6/O6</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="11">
+        <v>8</v>
+      </c>
+      <c r="D7" s="79"/>
+      <c r="E7" s="94"/>
+      <c r="F7" s="16">
+        <v>45</v>
+      </c>
+      <c r="G7" s="13">
+        <v>17</v>
+      </c>
+      <c r="H7" s="51"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="16">
+        <v>43</v>
+      </c>
+      <c r="M7" s="13">
+        <v>19</v>
+      </c>
+      <c r="N7" s="80">
+        <f>F7+J7+L7</f>
+        <v>88</v>
+      </c>
+      <c r="O7" s="14">
+        <f>COUNTIF(D7:L7,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="P7" s="81"/>
+      <c r="Q7" s="13">
+        <v>2</v>
+      </c>
+      <c r="R7" s="82">
+        <f>SUMIF(G7:M7, "&lt;30")+P7+Q7</f>
+        <v>38</v>
+      </c>
+      <c r="S7" s="37">
+        <f>R7/O7</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="11">
+        <v>22</v>
+      </c>
+      <c r="D8" s="79"/>
+      <c r="E8" s="94"/>
+      <c r="F8" s="15">
+        <v>59</v>
+      </c>
+      <c r="G8" s="13">
+        <v>17</v>
+      </c>
+      <c r="H8" s="51"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="80">
+        <f>F8+J8+L8</f>
+        <v>59</v>
+      </c>
+      <c r="O8" s="14">
+        <f>COUNTIF(D8:L8,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P8" s="81"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="82">
+        <f>SUMIF(G8:M8, "&lt;30")+P8+Q8</f>
+        <v>17</v>
+      </c>
+      <c r="S8" s="37">
+        <f>R8/O8</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="11">
+        <v>15</v>
+      </c>
+      <c r="D9" s="79"/>
+      <c r="E9" s="94"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="15">
+        <v>52</v>
+      </c>
+      <c r="K9" s="13">
+        <v>17</v>
+      </c>
+      <c r="L9" s="15"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="80">
+        <f>F9+J9+L9</f>
+        <v>52</v>
+      </c>
+      <c r="O9" s="14">
+        <f>COUNTIF(D9:L9,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P9" s="81"/>
+      <c r="Q9" s="13"/>
+      <c r="R9" s="82">
+        <f>SUMIF(G9:M9, "&lt;30")+P9+Q9</f>
+        <v>17</v>
+      </c>
+      <c r="S9" s="37">
+        <f>R9/O9</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="11">
+        <v>21</v>
+      </c>
+      <c r="D10" s="79"/>
+      <c r="E10" s="94"/>
+      <c r="F10" s="17">
+        <v>61</v>
+      </c>
+      <c r="G10" s="13">
+        <v>14</v>
+      </c>
+      <c r="H10" s="51"/>
+      <c r="I10" s="52"/>
+      <c r="J10" s="17">
+        <v>56</v>
+      </c>
+      <c r="K10" s="13">
+        <v>19</v>
+      </c>
+      <c r="L10" s="83">
+        <v>60</v>
+      </c>
+      <c r="M10" s="13">
+        <v>15</v>
+      </c>
+      <c r="N10" s="80">
+        <f>F10+J10+L10</f>
+        <v>177</v>
+      </c>
+      <c r="O10" s="14">
+        <f>COUNTIF(D10:L10,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="P10" s="81">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="82">
+        <f>SUMIF(G10:M10, "&lt;30")+P10+Q10</f>
+        <v>50</v>
+      </c>
+      <c r="S10" s="37">
+        <f>R10/O10</f>
+        <v>16.666666666666668</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="11">
+        <v>18</v>
+      </c>
+      <c r="D11" s="79"/>
+      <c r="E11" s="94"/>
+      <c r="F11" s="15">
+        <v>56</v>
+      </c>
+      <c r="G11" s="13">
+        <v>16</v>
+      </c>
+      <c r="H11" s="51"/>
+      <c r="I11" s="52"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="80">
+        <f>F11+J11+L11</f>
+        <v>56</v>
+      </c>
+      <c r="O11" s="14">
+        <f>COUNTIF(D11:L11,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P11" s="81"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="82">
+        <f>SUMIF(G11:M11, "&lt;30")+P11+Q11</f>
+        <v>16</v>
+      </c>
+      <c r="S11" s="37">
+        <f>R11/O11</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="11">
+        <v>8</v>
+      </c>
+      <c r="D12" s="79"/>
+      <c r="E12" s="94"/>
+      <c r="F12" s="15">
+        <v>46</v>
+      </c>
+      <c r="G12" s="13">
+        <v>16</v>
+      </c>
+      <c r="H12" s="51"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="80">
+        <f>F12+J12+L12</f>
+        <v>46</v>
+      </c>
+      <c r="O12" s="14">
+        <f>COUNTIF(D12:L12,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P12" s="81"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="82">
+        <f>SUMIF(G12:M12, "&lt;30")+P12+Q12</f>
+        <v>16</v>
+      </c>
+      <c r="S12" s="37">
+        <f>R12/O12</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="11">
+        <v>17</v>
+      </c>
+      <c r="D13" s="79"/>
+      <c r="E13" s="94"/>
+      <c r="F13" s="15">
+        <v>55</v>
+      </c>
+      <c r="G13" s="13">
+        <v>16</v>
+      </c>
+      <c r="H13" s="51"/>
+      <c r="I13" s="52"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="15">
+        <v>56</v>
+      </c>
+      <c r="M13" s="13">
+        <v>15</v>
+      </c>
+      <c r="N13" s="80">
+        <f>F13+J13+L13</f>
+        <v>111</v>
+      </c>
+      <c r="O13" s="14">
+        <f>COUNTIF(D13:L13,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="P13" s="81"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="82">
+        <f>SUMIF(G13:M13, "&lt;30")+P13+Q13</f>
+        <v>31</v>
+      </c>
+      <c r="S13" s="37">
+        <f>R13/O13</f>
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="79"/>
+      <c r="E14" s="94"/>
+      <c r="F14" s="15">
+        <v>46</v>
+      </c>
+      <c r="G14" s="13"/>
+      <c r="H14" s="51"/>
+      <c r="I14" s="52"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="15">
+        <v>46</v>
+      </c>
+      <c r="M14" s="13"/>
+      <c r="N14" s="80">
+        <f>F14+J14+L14</f>
+        <v>92</v>
+      </c>
+      <c r="O14" s="14">
+        <f>COUNTIF(D14:L14,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="P14" s="85"/>
+      <c r="Q14" s="38"/>
+      <c r="R14" s="82">
+        <f>SUMIF(G14:M14, "&lt;30")+P14+Q14</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="37"/>
+    </row>
+    <row r="15" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="79"/>
+      <c r="E15" s="94"/>
+      <c r="F15" s="15">
+        <v>51</v>
+      </c>
+      <c r="G15" s="13"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="52"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="80">
+        <f>F15+J15+L15</f>
+        <v>51</v>
+      </c>
+      <c r="O15" s="14">
+        <f>COUNTIF(D15:L15,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P15" s="81"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="82">
+        <f>SUMIF(G15:M15, "&lt;30")+P15+Q15</f>
+        <v>0</v>
+      </c>
+      <c r="S15" s="37"/>
+    </row>
+    <row r="16" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="79"/>
+      <c r="E16" s="94"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="51"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="84">
+        <v>50</v>
+      </c>
+      <c r="M16" s="13"/>
+      <c r="N16" s="80">
+        <f>F16+J16+L16</f>
+        <v>50</v>
+      </c>
+      <c r="O16" s="14">
+        <f>COUNTIF(D16:L16,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P16" s="81"/>
+      <c r="Q16" s="13"/>
+      <c r="R16" s="82">
+        <f>SUMIF(G16:M16, "&lt;30")+P16+Q16</f>
+        <v>0</v>
+      </c>
+      <c r="S16" s="37"/>
+    </row>
+    <row r="17" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="Q4" s="40">
-        <f t="shared" ref="Q4:Q13" si="2">P4/M4</f>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="B17" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="79"/>
+      <c r="E17" s="94"/>
+      <c r="F17" s="15">
+        <v>41</v>
+      </c>
+      <c r="G17" s="13"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="52"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="80">
+        <f>F17+J17+L17</f>
+        <v>41</v>
+      </c>
+      <c r="O17" s="14">
+        <f>COUNTIF(D17:L17,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="P17" s="81"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="82">
+        <f>SUMIF(G17:M17, "&lt;30")+P17+Q17</f>
+        <v>0</v>
+      </c>
+      <c r="S17" s="37"/>
+    </row>
+    <row r="18" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="11">
+        <v>13</v>
+      </c>
+      <c r="D18" s="79"/>
+      <c r="E18" s="94"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="52"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="80"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="81"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="82"/>
+      <c r="S18" s="37"/>
+    </row>
+    <row r="19" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="11">
+        <v>2</v>
+      </c>
+      <c r="D19" s="79"/>
+      <c r="E19" s="94"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="52"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="80"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="81"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="82"/>
+      <c r="S19" s="37"/>
+    </row>
+    <row r="20" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="11">
         <v>15</v>
       </c>
-      <c r="C5" s="12">
-        <v>13</v>
-      </c>
-      <c r="D5" s="53"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="83">
-        <v>42</v>
-      </c>
-      <c r="G5" s="14">
-        <v>25</v>
-      </c>
-      <c r="H5" s="53"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="15">
-        <f t="shared" si="0"/>
-        <v>42</v>
-      </c>
-      <c r="M5" s="48">
-        <v>1</v>
-      </c>
-      <c r="N5" s="16">
-        <v>1</v>
-      </c>
-      <c r="O5" s="14"/>
-      <c r="P5" s="15">
-        <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-      <c r="Q5" s="41">
-        <f t="shared" si="2"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="12">
-        <v>22</v>
-      </c>
-      <c r="D6" s="53"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="17">
+      <c r="D20" s="79"/>
+      <c r="E20" s="94"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="51"/>
+      <c r="I20" s="52"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="80"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="81"/>
+      <c r="Q20" s="13"/>
+      <c r="R20" s="82"/>
+      <c r="S20" s="37"/>
+    </row>
+    <row r="21" spans="1:19" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="22">
+        <v>11</v>
+      </c>
+      <c r="D21" s="86"/>
+      <c r="E21" s="95"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="53"/>
+      <c r="I21" s="54"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="87"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="88"/>
+      <c r="Q21" s="24"/>
+      <c r="R21" s="89"/>
+      <c r="S21" s="39"/>
+    </row>
+    <row r="22" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="40"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42">
+        <f>AVERAGEIF(F4:F21,"&gt;0")</f>
+        <v>49.75</v>
+      </c>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42">
+        <f>AVERAGEIF(J4:J21,"&gt;0")</f>
+        <v>54</v>
+      </c>
+      <c r="K22" s="42"/>
+      <c r="L22" s="42">
+        <f>AVERAGEIF(L4:L21,"&gt;0")</f>
+        <v>51.428571428571431</v>
+      </c>
+      <c r="M22" s="42"/>
+      <c r="N22" s="43"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="26"/>
+      <c r="Q22" s="26"/>
+      <c r="R22" s="26"/>
+      <c r="S22" s="26"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="C23" s="27"/>
+      <c r="N23" s="28"/>
+      <c r="O23" s="28"/>
+      <c r="P23" s="29"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="30"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="C24" s="90" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="14">
-        <v>23</v>
-      </c>
-      <c r="H6" s="53"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="15">
-        <f t="shared" si="0"/>
-        <v>53</v>
-      </c>
-      <c r="M6" s="48">
-        <v>1</v>
-      </c>
-      <c r="N6" s="16"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="15">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-      <c r="Q6" s="41">
-        <f t="shared" si="2"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="12">
-        <v>8</v>
-      </c>
-      <c r="D7" s="53"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="18">
-        <v>45</v>
-      </c>
-      <c r="G7" s="14">
-        <v>17</v>
-      </c>
-      <c r="H7" s="53"/>
-      <c r="I7" s="54"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="15">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-      <c r="M7" s="48">
-        <v>1</v>
-      </c>
-      <c r="N7" s="16"/>
-      <c r="O7" s="14">
-        <v>1</v>
-      </c>
-      <c r="P7" s="15">
-        <f t="shared" si="1"/>
-        <v>18</v>
-      </c>
-      <c r="Q7" s="41">
-        <f t="shared" si="2"/>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="12">
-        <v>21</v>
-      </c>
-      <c r="D8" s="53"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="19">
-        <v>61</v>
-      </c>
-      <c r="G8" s="14">
-        <v>14</v>
-      </c>
-      <c r="H8" s="53"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="19">
-        <v>56</v>
-      </c>
-      <c r="K8" s="14">
-        <v>19</v>
-      </c>
-      <c r="L8" s="15">
-        <f t="shared" si="0"/>
-        <v>117</v>
-      </c>
-      <c r="M8" s="48">
-        <v>2</v>
-      </c>
-      <c r="N8" s="16">
-        <v>2</v>
-      </c>
-      <c r="O8" s="14"/>
-      <c r="P8" s="15">
-        <f t="shared" si="1"/>
-        <v>35</v>
-      </c>
-      <c r="Q8" s="41">
-        <f t="shared" si="2"/>
-        <v>17.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="12">
-        <v>22</v>
-      </c>
-      <c r="D9" s="53"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="17">
-        <v>59</v>
-      </c>
-      <c r="G9" s="14">
-        <v>17</v>
-      </c>
-      <c r="H9" s="53"/>
-      <c r="I9" s="54"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="15">
-        <f t="shared" si="0"/>
-        <v>59</v>
-      </c>
-      <c r="M9" s="48">
-        <v>1</v>
-      </c>
-      <c r="N9" s="16"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="15">
-        <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-      <c r="Q9" s="41">
-        <f t="shared" si="2"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="12">
-        <v>15</v>
-      </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="53"/>
-      <c r="I10" s="54"/>
-      <c r="J10" s="17">
-        <v>52</v>
-      </c>
-      <c r="K10" s="14">
-        <v>17</v>
-      </c>
-      <c r="L10" s="15">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="M10" s="48">
-        <v>1</v>
-      </c>
-      <c r="N10" s="16"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="15">
-        <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-      <c r="Q10" s="41">
-        <f t="shared" si="2"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="12">
-        <v>18</v>
-      </c>
-      <c r="D11" s="53"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="17">
-        <v>56</v>
-      </c>
-      <c r="G11" s="14">
-        <v>16</v>
-      </c>
-      <c r="H11" s="53"/>
-      <c r="I11" s="54"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="15">
-        <f t="shared" si="0"/>
-        <v>56</v>
-      </c>
-      <c r="M11" s="48">
-        <v>1</v>
-      </c>
-      <c r="N11" s="16"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="15">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="Q11" s="41">
-        <f t="shared" si="2"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="12">
-        <v>8</v>
-      </c>
-      <c r="D12" s="53"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="17">
-        <v>46</v>
-      </c>
-      <c r="G12" s="14">
-        <v>16</v>
-      </c>
-      <c r="H12" s="53"/>
-      <c r="I12" s="54"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="15">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-      <c r="M12" s="48">
-        <v>1</v>
-      </c>
-      <c r="N12" s="16"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="15">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="Q12" s="41">
-        <f t="shared" si="2"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="12">
-        <v>17</v>
-      </c>
-      <c r="D13" s="53"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="17">
+      <c r="F24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="L24" s="31"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="C25" s="91" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="F25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="L25" s="32"/>
+      <c r="N25" s="33"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="C26" s="92" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="14">
-        <v>16</v>
-      </c>
-      <c r="H13" s="53"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="15">
-        <f t="shared" si="0"/>
-        <v>55</v>
-      </c>
-      <c r="M13" s="48">
-        <v>1</v>
-      </c>
-      <c r="N13" s="16"/>
-      <c r="O13" s="14"/>
-      <c r="P13" s="15">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="Q13" s="41">
-        <f t="shared" si="2"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="12">
-        <v>13</v>
-      </c>
-      <c r="D14" s="53"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="53"/>
-      <c r="I14" s="54"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="48"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="14"/>
-      <c r="P14" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q14" s="41"/>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="12">
-        <v>2</v>
-      </c>
-      <c r="D15" s="53"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="53"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="48"/>
-      <c r="N15" s="16"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="41"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A16" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="53"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="17">
-        <v>51</v>
-      </c>
-      <c r="G16" s="14"/>
-      <c r="H16" s="53"/>
-      <c r="I16" s="54"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="15">
-        <f>F16+J16</f>
-        <v>51</v>
-      </c>
-      <c r="M16" s="48">
-        <v>1</v>
-      </c>
-      <c r="N16" s="16"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q16" s="41"/>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A17" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="53"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="17">
-        <v>46</v>
-      </c>
-      <c r="G17" s="14"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="54"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="15">
-        <f>F17+J17</f>
-        <v>46</v>
-      </c>
-      <c r="M17" s="48">
-        <v>1</v>
-      </c>
-      <c r="N17" s="17"/>
-      <c r="O17" s="42"/>
-      <c r="P17" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="41"/>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A18" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="53"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="17">
-        <v>41</v>
-      </c>
-      <c r="G18" s="14"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="54"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="15">
-        <f>F18+J18</f>
-        <v>41</v>
-      </c>
-      <c r="M18" s="48">
-        <v>1</v>
-      </c>
-      <c r="N18" s="16"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="41"/>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="12">
-        <v>15</v>
-      </c>
-      <c r="D19" s="53"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="53"/>
-      <c r="I19" s="54"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="15"/>
-      <c r="M19" s="48"/>
-      <c r="N19" s="16"/>
-      <c r="O19" s="14"/>
-      <c r="P19" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q19" s="41"/>
-    </row>
-    <row r="20" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="24">
-        <v>11</v>
-      </c>
-      <c r="D20" s="55"/>
-      <c r="E20" s="56"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="55"/>
-      <c r="I20" s="56"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="26"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="49"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="27">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q20" s="43"/>
-    </row>
-    <row r="21" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="44"/>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="46">
-        <f>AVERAGEIF(F4:F20,"&gt;0")</f>
-        <v>49.75</v>
-      </c>
-      <c r="G21" s="46"/>
-      <c r="H21" s="46"/>
-      <c r="I21" s="46"/>
-      <c r="J21" s="46">
-        <f>AVERAGEIF(J4:J20,"&gt;0")</f>
-        <v>54</v>
-      </c>
-      <c r="K21" s="46"/>
-      <c r="L21" s="50"/>
-      <c r="M21" s="29"/>
-      <c r="N21" s="29"/>
-      <c r="O21" s="29"/>
-      <c r="P21" s="29"/>
-      <c r="Q21" s="29"/>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C22" s="30"/>
-      <c r="L22" s="31"/>
-      <c r="M22" s="31"/>
-      <c r="N22" s="32"/>
-      <c r="O22" s="32"/>
-      <c r="P22" s="31"/>
-      <c r="Q22" s="33"/>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C23" s="84" t="s">
-        <v>43</v>
-      </c>
-      <c r="F23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="35"/>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C24" s="85" t="s">
-        <v>44</v>
-      </c>
-      <c r="F24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="37"/>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C25" s="86" t="s">
-        <v>49</v>
-      </c>
-      <c r="E25" s="39"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="39"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="38"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="35"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="34"/>
+      <c r="M26" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="D4:E20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:S21">
+    <sortCondition descending="1" ref="S4:S21"/>
+    <sortCondition descending="1" ref="N4:N21"/>
+    <sortCondition ref="B4:B21"/>
+  </sortState>
+  <mergeCells count="20">
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:N3"/>
+    <mergeCell ref="O1:S1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="S2:S3"/>
+    <mergeCell ref="H4:I21"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="H4:I20"/>
-    <mergeCell ref="L1:L3"/>
-    <mergeCell ref="M1:Q1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
060525 - added Drew CTTP on hole 4 week 5
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE152A4-F732-8C46-9333-4E5C8BE3F51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8A3CA5-59AA-0B4D-8B9D-0BEE87613743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10760" yWindow="3400" windowWidth="27640" windowHeight="16940" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="58">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -205,13 +205,19 @@
   </si>
   <si>
     <t>BLUE</t>
+  </si>
+  <si>
+    <t>SECOND HALF (11 Rounds)</t>
+  </si>
+  <si>
+    <t>`</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -317,6 +323,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -338,7 +351,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -877,11 +890,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -994,11 +1020,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1009,6 +1071,48 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1051,104 +1155,51 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1484,106 +1535,134 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:X26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="7" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" customWidth="1"/>
+    <col min="4" max="4" width="7.5" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="1.1640625" hidden="1" customWidth="1"/>
     <col min="8" max="13" width="6.83203125" customWidth="1"/>
-    <col min="14" max="14" width="6.33203125" customWidth="1"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1"/>
+    <col min="14" max="15" width="6.6640625" customWidth="1"/>
     <col min="16" max="16" width="6" customWidth="1"/>
     <col min="17" max="17" width="5.6640625" customWidth="1"/>
-    <col min="18" max="18" width="5.83203125" customWidth="1"/>
+    <col min="18" max="18" width="6.33203125" customWidth="1"/>
     <col min="19" max="19" width="10.83203125" customWidth="1"/>
+    <col min="20" max="20" width="8.5" hidden="1" customWidth="1"/>
+    <col min="21" max="22" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="8.5" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="10.6640625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+    <row r="1" spans="1:24" s="92" customFormat="1" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="61" t="s">
+      <c r="B1" s="82"/>
+      <c r="C1" s="87" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="45"/>
-      <c r="F1" s="44" t="s">
+      <c r="E1" s="67"/>
+      <c r="F1" s="66" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="45"/>
-      <c r="H1" s="44" t="s">
+      <c r="G1" s="67"/>
+      <c r="H1" s="66" t="s">
         <v>47</v>
       </c>
-      <c r="I1" s="45"/>
-      <c r="J1" s="44" t="s">
+      <c r="I1" s="67"/>
+      <c r="J1" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="K1" s="45"/>
-      <c r="L1" s="44" t="s">
+      <c r="K1" s="67"/>
+      <c r="L1" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="M1" s="45"/>
-      <c r="N1" s="63" t="s">
+      <c r="M1" s="67"/>
+      <c r="N1" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="65" t="s">
+      <c r="O1" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="67"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="72"/>
+      <c r="T1" s="89" t="s">
+        <v>56</v>
+      </c>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="91"/>
     </row>
-    <row r="2" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="57"/>
-      <c r="B2" s="58"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="46">
+    <row r="2" spans="1:24" s="92" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="83"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="58">
         <v>45782</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="46">
+      <c r="E2" s="59"/>
+      <c r="F2" s="58">
         <v>45789</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="46">
+      <c r="G2" s="59"/>
+      <c r="H2" s="58">
         <v>45796</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="46">
+      <c r="I2" s="59"/>
+      <c r="J2" s="58">
         <v>45803</v>
       </c>
-      <c r="K2" s="47"/>
-      <c r="L2" s="46">
+      <c r="K2" s="59"/>
+      <c r="L2" s="58">
         <v>45810</v>
       </c>
-      <c r="M2" s="47"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="48" t="s">
+      <c r="M2" s="59"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="P2" s="68" t="s">
+      <c r="P2" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="Q2" s="70" t="s">
+      <c r="Q2" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="R2" s="48" t="s">
+      <c r="R2" s="60" t="s">
         <v>8</v>
       </c>
       <c r="S2" s="73" t="s">
         <v>9</v>
       </c>
+      <c r="T2" s="93" t="s">
+        <v>5</v>
+      </c>
+      <c r="U2" s="93" t="s">
+        <v>6</v>
+      </c>
+      <c r="V2" s="93" t="s">
+        <v>7</v>
+      </c>
+      <c r="W2" s="93" t="s">
+        <v>8</v>
+      </c>
+      <c r="X2" s="93" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="3" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59"/>
-      <c r="B3" s="60"/>
-      <c r="C3" s="62"/>
+    <row r="3" spans="1:24" s="92" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="85"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="88"/>
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1614,14 +1693,19 @@
       <c r="M3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N3" s="64"/>
-      <c r="O3" s="72"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="71"/>
-      <c r="R3" s="72"/>
+      <c r="N3" s="69"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="65"/>
+      <c r="R3" s="61"/>
       <c r="S3" s="74"/>
+      <c r="T3" s="94"/>
+      <c r="U3" s="94"/>
+      <c r="V3" s="94"/>
+      <c r="W3" s="94"/>
+      <c r="X3" s="94"/>
     </row>
-    <row r="4" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1631,23 +1715,25 @@
       <c r="C4" s="5">
         <v>22</v>
       </c>
-      <c r="D4" s="75"/>
-      <c r="E4" s="93"/>
+      <c r="D4" s="75" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="76"/>
       <c r="F4" s="6">
         <v>53</v>
       </c>
       <c r="G4" s="7">
         <v>23</v>
       </c>
-      <c r="H4" s="49" t="s">
+      <c r="H4" s="75" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="50"/>
+      <c r="I4" s="76"/>
       <c r="J4" s="6"/>
       <c r="K4" s="7"/>
       <c r="L4" s="6"/>
       <c r="M4" s="7"/>
-      <c r="N4" s="76">
+      <c r="N4" s="44">
         <f>F4+J4+L4</f>
         <v>53</v>
       </c>
@@ -1655,9 +1741,9 @@
         <f>COUNTIF(D4:L4,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P4" s="77"/>
+      <c r="P4" s="45"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="78">
+      <c r="R4" s="46">
         <f>SUMIF(G4:M4, "&lt;30")+P4+Q4</f>
         <v>23</v>
       </c>
@@ -1665,8 +1751,15 @@
         <f>R4/O4</f>
         <v>23</v>
       </c>
+      <c r="T4" s="95"/>
+      <c r="U4" s="46"/>
+      <c r="V4" s="46"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="96" t="s">
+        <v>57</v>
+      </c>
     </row>
-    <row r="5" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -1676,18 +1769,16 @@
       <c r="C5" s="11">
         <v>15</v>
       </c>
-      <c r="D5" s="79" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" s="94"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="78"/>
       <c r="F5" s="15">
         <v>42</v>
       </c>
       <c r="G5" s="13">
         <v>27</v>
       </c>
-      <c r="H5" s="51"/>
-      <c r="I5" s="52"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="78"/>
       <c r="J5" s="15"/>
       <c r="K5" s="13"/>
       <c r="L5" s="15">
@@ -1696,7 +1787,7 @@
       <c r="M5" s="13">
         <v>15</v>
       </c>
-      <c r="N5" s="80">
+      <c r="N5" s="47">
         <f>F5+J5+L5</f>
         <v>96</v>
       </c>
@@ -1704,9 +1795,9 @@
         <f>COUNTIF(D5:L5,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="P5" s="81"/>
+      <c r="P5" s="48"/>
       <c r="Q5" s="13"/>
-      <c r="R5" s="82">
+      <c r="R5" s="49">
         <f>SUMIF(G5:M5, "&lt;30")+P5+Q5</f>
         <v>42</v>
       </c>
@@ -1714,8 +1805,13 @@
         <f>R5/O5</f>
         <v>21</v>
       </c>
+      <c r="T5" s="97"/>
+      <c r="U5" s="49"/>
+      <c r="V5" s="49"/>
+      <c r="W5" s="14"/>
+      <c r="X5" s="98"/>
     </row>
-    <row r="6" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>14</v>
       </c>
@@ -1725,25 +1821,25 @@
       <c r="C6" s="11">
         <v>13</v>
       </c>
-      <c r="D6" s="79"/>
-      <c r="E6" s="94"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="78"/>
       <c r="F6" s="12">
         <v>42</v>
       </c>
       <c r="G6" s="13">
         <v>25</v>
       </c>
-      <c r="H6" s="51"/>
-      <c r="I6" s="52"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="78"/>
       <c r="J6" s="12"/>
       <c r="K6" s="13"/>
-      <c r="L6" s="83">
+      <c r="L6" s="50">
         <v>51</v>
       </c>
       <c r="M6" s="13">
         <v>16</v>
       </c>
-      <c r="N6" s="80">
+      <c r="N6" s="47">
         <f>F6+J6+L6</f>
         <v>93</v>
       </c>
@@ -1751,11 +1847,11 @@
         <f>COUNTIF(D6:L6,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="P6" s="81">
+      <c r="P6" s="48">
         <v>1</v>
       </c>
       <c r="Q6" s="13"/>
-      <c r="R6" s="82">
+      <c r="R6" s="49">
         <f>SUMIF(G6:M6, "&lt;30")+P6+Q6</f>
         <v>42</v>
       </c>
@@ -1763,8 +1859,13 @@
         <f>R6/O6</f>
         <v>21</v>
       </c>
+      <c r="T6" s="97"/>
+      <c r="U6" s="49"/>
+      <c r="V6" s="49"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="98"/>
     </row>
-    <row r="7" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>14</v>
       </c>
@@ -1774,16 +1875,16 @@
       <c r="C7" s="11">
         <v>8</v>
       </c>
-      <c r="D7" s="79"/>
-      <c r="E7" s="94"/>
+      <c r="D7" s="77"/>
+      <c r="E7" s="78"/>
       <c r="F7" s="16">
         <v>45</v>
       </c>
       <c r="G7" s="13">
         <v>17</v>
       </c>
-      <c r="H7" s="51"/>
-      <c r="I7" s="52"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="78"/>
       <c r="J7" s="16"/>
       <c r="K7" s="13"/>
       <c r="L7" s="16">
@@ -1792,7 +1893,7 @@
       <c r="M7" s="13">
         <v>19</v>
       </c>
-      <c r="N7" s="80">
+      <c r="N7" s="47">
         <f>F7+J7+L7</f>
         <v>88</v>
       </c>
@@ -1800,11 +1901,11 @@
         <f>COUNTIF(D7:L7,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="P7" s="81"/>
+      <c r="P7" s="48"/>
       <c r="Q7" s="13">
         <v>2</v>
       </c>
-      <c r="R7" s="82">
+      <c r="R7" s="49">
         <f>SUMIF(G7:M7, "&lt;30")+P7+Q7</f>
         <v>38</v>
       </c>
@@ -1812,8 +1913,13 @@
         <f>R7/O7</f>
         <v>19</v>
       </c>
+      <c r="T7" s="97"/>
+      <c r="U7" s="49"/>
+      <c r="V7" s="49"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="98"/>
     </row>
-    <row r="8" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>19</v>
       </c>
@@ -1823,21 +1929,21 @@
       <c r="C8" s="11">
         <v>22</v>
       </c>
-      <c r="D8" s="79"/>
-      <c r="E8" s="94"/>
+      <c r="D8" s="77"/>
+      <c r="E8" s="78"/>
       <c r="F8" s="15">
         <v>59</v>
       </c>
       <c r="G8" s="13">
         <v>17</v>
       </c>
-      <c r="H8" s="51"/>
-      <c r="I8" s="52"/>
+      <c r="H8" s="77"/>
+      <c r="I8" s="78"/>
       <c r="J8" s="15"/>
       <c r="K8" s="13"/>
       <c r="L8" s="15"/>
       <c r="M8" s="13"/>
-      <c r="N8" s="80">
+      <c r="N8" s="47">
         <f>F8+J8+L8</f>
         <v>59</v>
       </c>
@@ -1845,9 +1951,9 @@
         <f>COUNTIF(D8:L8,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P8" s="81"/>
+      <c r="P8" s="48"/>
       <c r="Q8" s="13"/>
-      <c r="R8" s="82">
+      <c r="R8" s="49">
         <f>SUMIF(G8:M8, "&lt;30")+P8+Q8</f>
         <v>17</v>
       </c>
@@ -1855,8 +1961,13 @@
         <f>R8/O8</f>
         <v>17</v>
       </c>
+      <c r="T8" s="99"/>
+      <c r="U8" s="49"/>
+      <c r="V8" s="49"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="98"/>
     </row>
-    <row r="9" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>41</v>
       </c>
@@ -1866,12 +1977,12 @@
       <c r="C9" s="11">
         <v>15</v>
       </c>
-      <c r="D9" s="79"/>
-      <c r="E9" s="94"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="78"/>
       <c r="F9" s="15"/>
       <c r="G9" s="13"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="52"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="78"/>
       <c r="J9" s="15">
         <v>52</v>
       </c>
@@ -1880,7 +1991,7 @@
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="13"/>
-      <c r="N9" s="80">
+      <c r="N9" s="47">
         <f>F9+J9+L9</f>
         <v>52</v>
       </c>
@@ -1888,9 +1999,9 @@
         <f>COUNTIF(D9:L9,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P9" s="81"/>
+      <c r="P9" s="48"/>
       <c r="Q9" s="13"/>
-      <c r="R9" s="82">
+      <c r="R9" s="49">
         <f>SUMIF(G9:M9, "&lt;30")+P9+Q9</f>
         <v>17</v>
       </c>
@@ -1898,8 +2009,13 @@
         <f>R9/O9</f>
         <v>17</v>
       </c>
+      <c r="T9" s="97"/>
+      <c r="U9" s="49"/>
+      <c r="V9" s="49"/>
+      <c r="W9" s="14"/>
+      <c r="X9" s="98"/>
     </row>
-    <row r="10" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>25</v>
       </c>
@@ -1909,29 +2025,29 @@
       <c r="C10" s="11">
         <v>21</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="94"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="78"/>
       <c r="F10" s="17">
         <v>61</v>
       </c>
       <c r="G10" s="13">
         <v>14</v>
       </c>
-      <c r="H10" s="51"/>
-      <c r="I10" s="52"/>
+      <c r="H10" s="77"/>
+      <c r="I10" s="78"/>
       <c r="J10" s="17">
         <v>56</v>
       </c>
       <c r="K10" s="13">
         <v>19</v>
       </c>
-      <c r="L10" s="83">
+      <c r="L10" s="50">
         <v>60</v>
       </c>
       <c r="M10" s="13">
         <v>15</v>
       </c>
-      <c r="N10" s="80">
+      <c r="N10" s="47">
         <f>F10+J10+L10</f>
         <v>177</v>
       </c>
@@ -1939,11 +2055,11 @@
         <f>COUNTIF(D10:L10,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="P10" s="81">
+      <c r="P10" s="48">
         <v>2</v>
       </c>
       <c r="Q10" s="13"/>
-      <c r="R10" s="82">
+      <c r="R10" s="49">
         <f>SUMIF(G10:M10, "&lt;30")+P10+Q10</f>
         <v>50</v>
       </c>
@@ -1951,8 +2067,13 @@
         <f>R10/O10</f>
         <v>16.666666666666668</v>
       </c>
+      <c r="T10" s="100"/>
+      <c r="U10" s="49"/>
+      <c r="V10" s="49"/>
+      <c r="W10" s="14"/>
+      <c r="X10" s="98"/>
     </row>
-    <row r="11" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>23</v>
       </c>
@@ -1962,21 +2083,21 @@
       <c r="C11" s="11">
         <v>18</v>
       </c>
-      <c r="D11" s="79"/>
-      <c r="E11" s="94"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="78"/>
       <c r="F11" s="15">
         <v>56</v>
       </c>
       <c r="G11" s="13">
         <v>16</v>
       </c>
-      <c r="H11" s="51"/>
-      <c r="I11" s="52"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="78"/>
       <c r="J11" s="15"/>
       <c r="K11" s="13"/>
       <c r="L11" s="15"/>
       <c r="M11" s="13"/>
-      <c r="N11" s="80">
+      <c r="N11" s="47">
         <f>F11+J11+L11</f>
         <v>56</v>
       </c>
@@ -1984,9 +2105,9 @@
         <f>COUNTIF(D11:L11,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P11" s="81"/>
+      <c r="P11" s="48"/>
       <c r="Q11" s="13"/>
-      <c r="R11" s="82">
+      <c r="R11" s="49">
         <f>SUMIF(G11:M11, "&lt;30")+P11+Q11</f>
         <v>16</v>
       </c>
@@ -1994,8 +2115,13 @@
         <f>R11/O11</f>
         <v>16</v>
       </c>
+      <c r="T11" s="101"/>
+      <c r="U11" s="49"/>
+      <c r="V11" s="49"/>
+      <c r="W11" s="14"/>
+      <c r="X11" s="98"/>
     </row>
-    <row r="12" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>20</v>
       </c>
@@ -2005,21 +2131,21 @@
       <c r="C12" s="11">
         <v>8</v>
       </c>
-      <c r="D12" s="79"/>
-      <c r="E12" s="94"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="78"/>
       <c r="F12" s="15">
         <v>46</v>
       </c>
       <c r="G12" s="13">
         <v>16</v>
       </c>
-      <c r="H12" s="51"/>
-      <c r="I12" s="52"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="78"/>
       <c r="J12" s="15"/>
       <c r="K12" s="13"/>
       <c r="L12" s="15"/>
       <c r="M12" s="13"/>
-      <c r="N12" s="80">
+      <c r="N12" s="47">
         <f>F12+J12+L12</f>
         <v>46</v>
       </c>
@@ -2027,9 +2153,9 @@
         <f>COUNTIF(D12:L12,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P12" s="81"/>
+      <c r="P12" s="48"/>
       <c r="Q12" s="13"/>
-      <c r="R12" s="82">
+      <c r="R12" s="49">
         <f>SUMIF(G12:M12, "&lt;30")+P12+Q12</f>
         <v>16</v>
       </c>
@@ -2037,8 +2163,13 @@
         <f>R12/O12</f>
         <v>16</v>
       </c>
+      <c r="T12" s="101"/>
+      <c r="U12" s="49"/>
+      <c r="V12" s="49"/>
+      <c r="W12" s="14"/>
+      <c r="X12" s="98"/>
     </row>
-    <row r="13" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>22</v>
       </c>
@@ -2048,16 +2179,16 @@
       <c r="C13" s="11">
         <v>17</v>
       </c>
-      <c r="D13" s="79"/>
-      <c r="E13" s="94"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="78"/>
       <c r="F13" s="15">
         <v>55</v>
       </c>
       <c r="G13" s="13">
         <v>16</v>
       </c>
-      <c r="H13" s="51"/>
-      <c r="I13" s="52"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="78"/>
       <c r="J13" s="15"/>
       <c r="K13" s="13"/>
       <c r="L13" s="15">
@@ -2066,7 +2197,7 @@
       <c r="M13" s="13">
         <v>15</v>
       </c>
-      <c r="N13" s="80">
+      <c r="N13" s="47">
         <f>F13+J13+L13</f>
         <v>111</v>
       </c>
@@ -2074,9 +2205,9 @@
         <f>COUNTIF(D13:L13,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="P13" s="81"/>
+      <c r="P13" s="48"/>
       <c r="Q13" s="13"/>
-      <c r="R13" s="82">
+      <c r="R13" s="49">
         <f>SUMIF(G13:M13, "&lt;30")+P13+Q13</f>
         <v>31</v>
       </c>
@@ -2084,124 +2215,146 @@
         <f>R13/O13</f>
         <v>15.5</v>
       </c>
+      <c r="T13" s="101"/>
+      <c r="U13" s="49"/>
+      <c r="V13" s="49"/>
+      <c r="W13" s="14"/>
+      <c r="X13" s="98"/>
     </row>
-    <row r="14" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="79"/>
-      <c r="E14" s="94"/>
-      <c r="F14" s="15">
-        <v>46</v>
-      </c>
+      <c r="D14" s="77"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="13"/>
-      <c r="H14" s="51"/>
-      <c r="I14" s="52"/>
-      <c r="J14" s="15"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="78"/>
+      <c r="J14" s="19"/>
       <c r="K14" s="13"/>
-      <c r="L14" s="15">
-        <v>46</v>
+      <c r="L14" s="102">
+        <v>50</v>
       </c>
       <c r="M14" s="13"/>
-      <c r="N14" s="80">
+      <c r="N14" s="47">
         <f>F14+J14+L14</f>
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="O14" s="14">
         <f>COUNTIF(D14:L14,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="P14" s="85"/>
-      <c r="Q14" s="38"/>
-      <c r="R14" s="82">
+        <v>1</v>
+      </c>
+      <c r="P14" s="48">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="49">
         <f>SUMIF(G14:M14, "&lt;30")+P14+Q14</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" s="37"/>
+      <c r="T14" s="97"/>
+      <c r="U14" s="49"/>
+      <c r="V14" s="49"/>
+      <c r="W14" s="14"/>
+      <c r="X14" s="98"/>
     </row>
-    <row r="15" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="79"/>
-      <c r="E15" s="94"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="78"/>
       <c r="F15" s="15">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G15" s="13"/>
-      <c r="H15" s="51"/>
-      <c r="I15" s="52"/>
+      <c r="H15" s="77"/>
+      <c r="I15" s="78"/>
       <c r="J15" s="15"/>
       <c r="K15" s="13"/>
-      <c r="L15" s="15"/>
+      <c r="L15" s="15">
+        <v>46</v>
+      </c>
       <c r="M15" s="13"/>
-      <c r="N15" s="80">
+      <c r="N15" s="47">
         <f>F15+J15+L15</f>
-        <v>51</v>
+        <v>92</v>
       </c>
       <c r="O15" s="14">
         <f>COUNTIF(D15:L15,"&gt;30")</f>
-        <v>1</v>
-      </c>
-      <c r="P15" s="81"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="82">
+        <v>2</v>
+      </c>
+      <c r="P15" s="51"/>
+      <c r="Q15" s="38"/>
+      <c r="R15" s="49">
         <f>SUMIF(G15:M15, "&lt;30")+P15+Q15</f>
         <v>0</v>
       </c>
       <c r="S15" s="37"/>
+      <c r="T15" s="101"/>
+      <c r="U15" s="14"/>
+      <c r="V15" s="14"/>
+      <c r="W15" s="14"/>
+      <c r="X15" s="98"/>
     </row>
-    <row r="16" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="79"/>
-      <c r="E16" s="94"/>
-      <c r="F16" s="19"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="78"/>
+      <c r="F16" s="15">
+        <v>51</v>
+      </c>
       <c r="G16" s="13"/>
-      <c r="H16" s="51"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="19"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="78"/>
+      <c r="J16" s="15"/>
       <c r="K16" s="13"/>
-      <c r="L16" s="84">
-        <v>50</v>
-      </c>
+      <c r="L16" s="15"/>
       <c r="M16" s="13"/>
-      <c r="N16" s="80">
+      <c r="N16" s="47">
         <f>F16+J16+L16</f>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O16" s="14">
         <f>COUNTIF(D16:L16,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P16" s="81"/>
+      <c r="P16" s="48"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="82">
+      <c r="R16" s="49">
         <f>SUMIF(G16:M16, "&lt;30")+P16+Q16</f>
         <v>0</v>
       </c>
       <c r="S16" s="37"/>
+      <c r="T16" s="101"/>
+      <c r="U16" s="49"/>
+      <c r="V16" s="49"/>
+      <c r="W16" s="14"/>
+      <c r="X16" s="98"/>
     </row>
-    <row r="17" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
         <v>27</v>
       </c>
@@ -2211,19 +2364,19 @@
       <c r="C17" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="79"/>
-      <c r="E17" s="94"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="78"/>
       <c r="F17" s="15">
         <v>41</v>
       </c>
       <c r="G17" s="13"/>
-      <c r="H17" s="51"/>
-      <c r="I17" s="52"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="78"/>
       <c r="J17" s="15"/>
       <c r="K17" s="13"/>
       <c r="L17" s="15"/>
       <c r="M17" s="13"/>
-      <c r="N17" s="80">
+      <c r="N17" s="47">
         <f>F17+J17+L17</f>
         <v>41</v>
       </c>
@@ -2231,15 +2384,20 @@
         <f>COUNTIF(D17:L17,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="P17" s="81"/>
+      <c r="P17" s="48"/>
       <c r="Q17" s="13"/>
-      <c r="R17" s="82">
+      <c r="R17" s="49">
         <f>SUMIF(G17:M17, "&lt;30")+P17+Q17</f>
         <v>0</v>
       </c>
       <c r="S17" s="37"/>
+      <c r="T17" s="101"/>
+      <c r="U17" s="49"/>
+      <c r="V17" s="49"/>
+      <c r="W17" s="14"/>
+      <c r="X17" s="98"/>
     </row>
-    <row r="18" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
         <v>34</v>
       </c>
@@ -2249,24 +2407,35 @@
       <c r="C18" s="11">
         <v>13</v>
       </c>
-      <c r="D18" s="79"/>
-      <c r="E18" s="94"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="78"/>
       <c r="F18" s="18"/>
       <c r="G18" s="13"/>
-      <c r="H18" s="51"/>
-      <c r="I18" s="52"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="78"/>
       <c r="J18" s="18"/>
       <c r="K18" s="13"/>
       <c r="L18" s="18"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="80"/>
+      <c r="N18" s="47">
+        <f>F18+J18+L18</f>
+        <v>0</v>
+      </c>
       <c r="O18" s="14"/>
-      <c r="P18" s="81"/>
+      <c r="P18" s="48"/>
       <c r="Q18" s="13"/>
-      <c r="R18" s="82"/>
+      <c r="R18" s="49">
+        <f>SUMIF(G18:M18, "&lt;30")+P18+Q18</f>
+        <v>0</v>
+      </c>
       <c r="S18" s="37"/>
+      <c r="T18" s="97"/>
+      <c r="U18" s="49"/>
+      <c r="V18" s="49"/>
+      <c r="W18" s="14"/>
+      <c r="X18" s="98"/>
     </row>
-    <row r="19" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
         <v>36</v>
       </c>
@@ -2276,24 +2445,35 @@
       <c r="C19" s="11">
         <v>2</v>
       </c>
-      <c r="D19" s="79"/>
-      <c r="E19" s="94"/>
+      <c r="D19" s="77"/>
+      <c r="E19" s="78"/>
       <c r="F19" s="19"/>
       <c r="G19" s="13"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="52"/>
+      <c r="H19" s="77"/>
+      <c r="I19" s="78"/>
       <c r="J19" s="19"/>
       <c r="K19" s="13"/>
       <c r="L19" s="19"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="80"/>
+      <c r="N19" s="47">
+        <f>F19+J19+L19</f>
+        <v>0</v>
+      </c>
       <c r="O19" s="14"/>
-      <c r="P19" s="81"/>
+      <c r="P19" s="48"/>
       <c r="Q19" s="13"/>
-      <c r="R19" s="82"/>
+      <c r="R19" s="49">
+        <f>SUMIF(G19:M19, "&lt;30")+P19+Q19</f>
+        <v>0</v>
+      </c>
       <c r="S19" s="37"/>
+      <c r="T19" s="97"/>
+      <c r="U19" s="49"/>
+      <c r="V19" s="49"/>
+      <c r="W19" s="14"/>
+      <c r="X19" s="98"/>
     </row>
-    <row r="20" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
         <v>38</v>
       </c>
@@ -2303,24 +2483,35 @@
       <c r="C20" s="11">
         <v>15</v>
       </c>
-      <c r="D20" s="79"/>
-      <c r="E20" s="94"/>
+      <c r="D20" s="77"/>
+      <c r="E20" s="78"/>
       <c r="F20" s="15"/>
       <c r="G20" s="13"/>
-      <c r="H20" s="51"/>
-      <c r="I20" s="52"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="78"/>
       <c r="J20" s="15"/>
       <c r="K20" s="13"/>
       <c r="L20" s="15"/>
       <c r="M20" s="13"/>
-      <c r="N20" s="80"/>
+      <c r="N20" s="47">
+        <f>F20+J20+L20</f>
+        <v>0</v>
+      </c>
       <c r="O20" s="14"/>
-      <c r="P20" s="81"/>
+      <c r="P20" s="48"/>
       <c r="Q20" s="13"/>
-      <c r="R20" s="82"/>
+      <c r="R20" s="49">
+        <f>SUMIF(G20:M20, "&lt;30")+P20+Q20</f>
+        <v>0</v>
+      </c>
       <c r="S20" s="37"/>
+      <c r="T20" s="101"/>
+      <c r="U20" s="49"/>
+      <c r="V20" s="49"/>
+      <c r="W20" s="14"/>
+      <c r="X20" s="98"/>
     </row>
-    <row r="21" spans="1:19" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
         <v>32</v>
       </c>
@@ -2330,24 +2521,32 @@
       <c r="C21" s="22">
         <v>11</v>
       </c>
-      <c r="D21" s="86"/>
-      <c r="E21" s="95"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="80"/>
       <c r="F21" s="23"/>
       <c r="G21" s="24"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="54"/>
+      <c r="H21" s="79"/>
+      <c r="I21" s="80"/>
       <c r="J21" s="23"/>
       <c r="K21" s="24"/>
       <c r="L21" s="23"/>
       <c r="M21" s="24"/>
-      <c r="N21" s="87"/>
+      <c r="N21" s="52"/>
       <c r="O21" s="25"/>
-      <c r="P21" s="88"/>
+      <c r="P21" s="53"/>
       <c r="Q21" s="24"/>
-      <c r="R21" s="89"/>
+      <c r="R21" s="54">
+        <f>SUMIF(G21:M21, "&lt;30")+P21+Q21</f>
+        <v>0</v>
+      </c>
       <c r="S21" s="39"/>
+      <c r="T21" s="103"/>
+      <c r="U21" s="54"/>
+      <c r="V21" s="54"/>
+      <c r="W21" s="25"/>
+      <c r="X21" s="104"/>
     </row>
-    <row r="22" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" s="26" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="40"/>
       <c r="B22" s="41"/>
       <c r="C22" s="41"/>
@@ -2371,13 +2570,8 @@
       </c>
       <c r="M22" s="42"/>
       <c r="N22" s="43"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="26"/>
-      <c r="Q22" s="26"/>
-      <c r="R22" s="26"/>
-      <c r="S22" s="26"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C23" s="27"/>
       <c r="N23" s="28"/>
       <c r="O23" s="28"/>
@@ -2386,8 +2580,8 @@
       <c r="R23" s="28"/>
       <c r="S23" s="30"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="C24" s="90" t="s">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="C24" s="55" t="s">
         <v>43</v>
       </c>
       <c r="D24" s="31" t="s">
@@ -2398,8 +2592,8 @@
       <c r="J24" s="31"/>
       <c r="L24" s="31"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="C25" s="91" t="s">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="C25" s="56" t="s">
         <v>44</v>
       </c>
       <c r="D25" s="32" t="s">
@@ -2411,8 +2605,8 @@
       <c r="L25" s="32"/>
       <c r="N25" s="33"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="C26" s="92" t="s">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="C26" s="57" t="s">
         <v>49</v>
       </c>
       <c r="D26" s="34" t="s">
@@ -2434,18 +2628,14 @@
     <sortCondition descending="1" ref="N4:N21"/>
     <sortCondition ref="B4:B21"/>
   </sortState>
-  <mergeCells count="20">
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="N1:N3"/>
-    <mergeCell ref="O1:S1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="S2:S3"/>
+  <mergeCells count="27">
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="T1:X1"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
     <mergeCell ref="H4:I21"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
@@ -2454,7 +2644,18 @@
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="D4:E21"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:N3"/>
+    <mergeCell ref="O1:S1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="S2:S3"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
061625 - updated results from last week and tee times
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE6D7ED-C1A2-B14E-A379-CDC667422EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{0AE6D7ED-C1A2-B14E-A379-CDC667422EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA5799C0-4AE0-4A80-A76B-DE3BFB79B359}"/>
   <bookViews>
-    <workbookView xWindow="41660" yWindow="2180" windowWidth="27640" windowHeight="16940" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="39180" yWindow="780" windowWidth="26730" windowHeight="18135" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="61">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -214,13 +214,19 @@
   </si>
   <si>
     <t>Johnson</t>
+  </si>
+  <si>
+    <t>SECOND HALF (11 Rounds)</t>
+  </si>
+  <si>
+    <t>`</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -326,6 +332,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -347,7 +360,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -809,19 +822,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -835,19 +835,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -861,24 +848,24 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -890,7 +877,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1000,34 +987,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1045,12 +1023,57 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1075,27 +1098,6 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1120,34 +1122,50 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1484,111 +1502,141 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:X27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Z27"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.75"/>
   <cols>
-    <col min="3" max="3" width="10.6640625" customWidth="1"/>
-    <col min="4" max="9" width="0" hidden="1" customWidth="1"/>
-    <col min="10" max="15" width="6.83203125" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" customWidth="1"/>
-    <col min="17" max="17" width="6.5" customWidth="1"/>
-    <col min="18" max="18" width="6.6640625" customWidth="1"/>
-    <col min="19" max="19" width="6.5" customWidth="1"/>
-    <col min="20" max="20" width="7.5" customWidth="1"/>
+    <col min="1" max="1" width="8.75" customWidth="1"/>
+    <col min="2" max="2" width="8.25" customWidth="1"/>
+    <col min="3" max="3" width="10.125" customWidth="1"/>
+    <col min="4" max="9" width="6.875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="6.875" customWidth="1"/>
+    <col min="11" max="15" width="6" customWidth="1"/>
+    <col min="16" max="16" width="7.625" customWidth="1"/>
+    <col min="17" max="17" width="6.875" customWidth="1"/>
+    <col min="18" max="18" width="5.25" customWidth="1"/>
+    <col min="19" max="19" width="5.75" customWidth="1"/>
+    <col min="20" max="20" width="5.5" customWidth="1"/>
+    <col min="21" max="21" width="9.5" customWidth="1"/>
+    <col min="22" max="22" width="7.375" hidden="1" customWidth="1"/>
+    <col min="23" max="24" width="6" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="7.375" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="9.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="60" t="s">
+    <row r="1" spans="1:26" s="91" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="66" t="s">
+      <c r="B1" s="73"/>
+      <c r="C1" s="78" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="59"/>
-      <c r="F1" s="58" t="s">
+      <c r="E1" s="66"/>
+      <c r="F1" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="59"/>
-      <c r="H1" s="58" t="s">
+      <c r="G1" s="66"/>
+      <c r="H1" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="59"/>
-      <c r="J1" s="58" t="s">
+      <c r="I1" s="66"/>
+      <c r="J1" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="59"/>
-      <c r="L1" s="58" t="s">
+      <c r="K1" s="66"/>
+      <c r="L1" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="M1" s="59"/>
-      <c r="N1" s="58" t="s">
+      <c r="M1" s="66"/>
+      <c r="N1" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="O1" s="59"/>
-      <c r="P1" s="70" t="s">
+      <c r="O1" s="66"/>
+      <c r="P1" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="72" t="s">
+      <c r="Q1" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="73"/>
-      <c r="U1" s="74"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="68"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="88" t="s">
+        <v>59</v>
+      </c>
+      <c r="W1" s="89"/>
+      <c r="X1" s="89"/>
+      <c r="Y1" s="89"/>
+      <c r="Z1" s="90"/>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="62"/>
-      <c r="B2" s="63"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68">
+    <row r="2" spans="1:26" s="91" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="74"/>
+      <c r="B2" s="75"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="70">
         <v>45782</v>
       </c>
-      <c r="E2" s="69"/>
-      <c r="F2" s="68">
+      <c r="E2" s="71"/>
+      <c r="F2" s="70">
         <v>45789</v>
       </c>
-      <c r="G2" s="69"/>
-      <c r="H2" s="68">
+      <c r="G2" s="71"/>
+      <c r="H2" s="70">
         <v>45796</v>
       </c>
-      <c r="I2" s="69"/>
-      <c r="J2" s="68">
+      <c r="I2" s="71"/>
+      <c r="J2" s="70">
         <v>45803</v>
       </c>
-      <c r="K2" s="69"/>
-      <c r="L2" s="68">
+      <c r="K2" s="71"/>
+      <c r="L2" s="70">
         <v>45810</v>
       </c>
-      <c r="M2" s="69"/>
-      <c r="N2" s="68">
+      <c r="M2" s="71"/>
+      <c r="N2" s="70">
         <v>45817</v>
       </c>
-      <c r="O2" s="69"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="70" t="s">
+      <c r="O2" s="71"/>
+      <c r="P2" s="64"/>
+      <c r="Q2" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="R2" s="79" t="s">
+      <c r="R2" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="S2" s="81" t="s">
+      <c r="S2" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="T2" s="75" t="s">
+      <c r="T2" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="U2" s="77" t="s">
+      <c r="U2" s="82" t="s">
         <v>8</v>
       </c>
+      <c r="V2" s="92" t="s">
+        <v>4</v>
+      </c>
+      <c r="W2" s="92" t="s">
+        <v>5</v>
+      </c>
+      <c r="X2" s="92" t="s">
+        <v>6</v>
+      </c>
+      <c r="Y2" s="92" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z2" s="92" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:21" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="64"/>
-      <c r="B3" s="65"/>
-      <c r="C3" s="67"/>
+    <row r="3" spans="1:26" s="91" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
+      <c r="A3" s="76"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="79"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1625,14 +1673,19 @@
       <c r="O3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="71"/>
-      <c r="Q3" s="71"/>
-      <c r="R3" s="80"/>
-      <c r="S3" s="82"/>
-      <c r="T3" s="76"/>
-      <c r="U3" s="78"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="85"/>
+      <c r="S3" s="87"/>
+      <c r="T3" s="81"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="93"/>
+      <c r="W3" s="93"/>
+      <c r="X3" s="93"/>
+      <c r="Y3" s="93"/>
+      <c r="Z3" s="93"/>
     </row>
-    <row r="4" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" ht="15.95" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -1642,20 +1695,20 @@
       <c r="C4" s="5">
         <v>22</v>
       </c>
-      <c r="D4" s="83" t="s">
+      <c r="D4" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="84"/>
+      <c r="E4" s="56"/>
       <c r="F4" s="6">
         <v>53</v>
       </c>
       <c r="G4" s="7">
         <v>23</v>
       </c>
-      <c r="H4" s="83" t="s">
+      <c r="H4" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="84"/>
+      <c r="I4" s="56"/>
       <c r="J4" s="6"/>
       <c r="K4" s="7"/>
       <c r="L4" s="6"/>
@@ -1666,7 +1719,7 @@
       <c r="O4" s="7">
         <v>19</v>
       </c>
-      <c r="P4" s="43">
+      <c r="P4" s="8">
         <f>F4+J4+L4+N4</f>
         <v>110</v>
       </c>
@@ -1674,9 +1727,9 @@
         <f>COUNTIF(D4:N4,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R4" s="44"/>
+      <c r="R4" s="43"/>
       <c r="S4" s="7"/>
-      <c r="T4" s="45">
+      <c r="T4" s="44">
         <f>SUMIF(G4:O4, "&lt;30")+R4+S4</f>
         <v>42</v>
       </c>
@@ -1684,8 +1737,15 @@
         <f>T4/Q4</f>
         <v>21</v>
       </c>
+      <c r="V4" s="94"/>
+      <c r="W4" s="44"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="8"/>
+      <c r="Z4" s="95" t="s">
+        <v>60</v>
+      </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26">
       <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
@@ -1695,16 +1755,16 @@
       <c r="C5" s="11">
         <v>15</v>
       </c>
-      <c r="D5" s="85"/>
-      <c r="E5" s="86"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="58"/>
       <c r="F5" s="15">
         <v>42</v>
       </c>
       <c r="G5" s="13">
         <v>27</v>
       </c>
-      <c r="H5" s="85"/>
-      <c r="I5" s="86"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="58"/>
       <c r="J5" s="15"/>
       <c r="K5" s="13"/>
       <c r="L5" s="15">
@@ -1715,7 +1775,7 @@
       </c>
       <c r="N5" s="15"/>
       <c r="O5" s="13"/>
-      <c r="P5" s="46">
+      <c r="P5" s="14">
         <f>F5+J5+L5+N5</f>
         <v>96</v>
       </c>
@@ -1723,9 +1783,9 @@
         <f>COUNTIF(D5:N5,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R5" s="47"/>
+      <c r="R5" s="45"/>
       <c r="S5" s="13"/>
-      <c r="T5" s="48">
+      <c r="T5" s="46">
         <f>SUMIF(G5:O5, "&lt;30")+R5+S5</f>
         <v>42</v>
       </c>
@@ -1733,8 +1793,13 @@
         <f>T5/Q5</f>
         <v>21</v>
       </c>
+      <c r="V5" s="96"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="46"/>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="97"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26">
       <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
@@ -1744,27 +1809,27 @@
       <c r="C6" s="11">
         <v>13</v>
       </c>
-      <c r="D6" s="85"/>
-      <c r="E6" s="86"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="58"/>
       <c r="F6" s="12">
         <v>42</v>
       </c>
       <c r="G6" s="13">
         <v>25</v>
       </c>
-      <c r="H6" s="85"/>
-      <c r="I6" s="86"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="58"/>
       <c r="J6" s="12"/>
       <c r="K6" s="13"/>
-      <c r="L6" s="49">
+      <c r="L6" s="47">
         <v>51</v>
       </c>
       <c r="M6" s="13">
         <v>16</v>
       </c>
-      <c r="N6" s="49"/>
+      <c r="N6" s="47"/>
       <c r="O6" s="13"/>
-      <c r="P6" s="46">
+      <c r="P6" s="14">
         <f>F6+J6+L6+N6</f>
         <v>93</v>
       </c>
@@ -1772,11 +1837,11 @@
         <f>COUNTIF(D6:N6,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R6" s="47">
+      <c r="R6" s="45">
         <v>1</v>
       </c>
       <c r="S6" s="13"/>
-      <c r="T6" s="48">
+      <c r="T6" s="46">
         <f>SUMIF(G6:O6, "&lt;30")+R6+S6</f>
         <v>42</v>
       </c>
@@ -1784,8 +1849,13 @@
         <f>T6/Q6</f>
         <v>21</v>
       </c>
+      <c r="V6" s="96"/>
+      <c r="W6" s="46"/>
+      <c r="X6" s="46"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="97"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -1795,16 +1865,16 @@
       <c r="C7" s="11">
         <v>8</v>
       </c>
-      <c r="D7" s="85"/>
-      <c r="E7" s="86"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="58"/>
       <c r="F7" s="16">
         <v>45</v>
       </c>
       <c r="G7" s="13">
         <v>17</v>
       </c>
-      <c r="H7" s="85"/>
-      <c r="I7" s="86"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="58"/>
       <c r="J7" s="16"/>
       <c r="K7" s="13"/>
       <c r="L7" s="16">
@@ -1813,13 +1883,13 @@
       <c r="M7" s="13">
         <v>19</v>
       </c>
-      <c r="N7" s="89">
+      <c r="N7" s="61">
         <v>41</v>
       </c>
       <c r="O7" s="13">
         <v>21</v>
       </c>
-      <c r="P7" s="46">
+      <c r="P7" s="14">
         <f>F7+J7+L7+N7</f>
         <v>129</v>
       </c>
@@ -1827,13 +1897,13 @@
         <f>COUNTIF(D7:N7,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="R7" s="47">
+      <c r="R7" s="45">
         <v>1</v>
       </c>
       <c r="S7" s="13">
         <v>3</v>
       </c>
-      <c r="T7" s="48">
+      <c r="T7" s="46">
         <f>SUMIF(G7:O7, "&lt;30")+R7+S7</f>
         <v>61</v>
       </c>
@@ -1841,8 +1911,13 @@
         <f>T7/Q7</f>
         <v>20.333333333333332</v>
       </c>
+      <c r="V7" s="96"/>
+      <c r="W7" s="46"/>
+      <c r="X7" s="46"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="97"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26">
       <c r="A8" s="9" t="s">
         <v>40</v>
       </c>
@@ -1852,12 +1927,12 @@
       <c r="C8" s="11">
         <v>15</v>
       </c>
-      <c r="D8" s="85"/>
-      <c r="E8" s="86"/>
+      <c r="D8" s="57"/>
+      <c r="E8" s="58"/>
       <c r="F8" s="15"/>
       <c r="G8" s="13"/>
-      <c r="H8" s="85"/>
-      <c r="I8" s="86"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="58"/>
       <c r="J8" s="15">
         <v>52</v>
       </c>
@@ -1872,7 +1947,7 @@
       <c r="O8" s="13">
         <v>23</v>
       </c>
-      <c r="P8" s="46">
+      <c r="P8" s="14">
         <f>F8+J8+L8+N8</f>
         <v>98</v>
       </c>
@@ -1880,9 +1955,9 @@
         <f>COUNTIF(D8:N8,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R8" s="47"/>
+      <c r="R8" s="45"/>
       <c r="S8" s="13"/>
-      <c r="T8" s="48">
+      <c r="T8" s="46">
         <f>SUMIF(G8:O8, "&lt;30")+R8+S8</f>
         <v>40</v>
       </c>
@@ -1890,8 +1965,13 @@
         <f>T8/Q8</f>
         <v>20</v>
       </c>
+      <c r="V8" s="98"/>
+      <c r="W8" s="46"/>
+      <c r="X8" s="46"/>
+      <c r="Y8" s="14"/>
+      <c r="Z8" s="97"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26">
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
@@ -1901,16 +1981,16 @@
       <c r="C9" s="11">
         <v>8</v>
       </c>
-      <c r="D9" s="85"/>
-      <c r="E9" s="86"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="58"/>
       <c r="F9" s="15">
         <v>46</v>
       </c>
       <c r="G9" s="13">
         <v>16</v>
       </c>
-      <c r="H9" s="85"/>
-      <c r="I9" s="86"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="58"/>
       <c r="J9" s="15"/>
       <c r="K9" s="13"/>
       <c r="L9" s="15"/>
@@ -1921,7 +2001,7 @@
       <c r="O9" s="13">
         <v>20</v>
       </c>
-      <c r="P9" s="46">
+      <c r="P9" s="14">
         <f>F9+J9+L9+N9</f>
         <v>88</v>
       </c>
@@ -1929,11 +2009,11 @@
         <f>COUNTIF(D9:N9,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R9" s="47"/>
+      <c r="R9" s="45"/>
       <c r="S9" s="13">
         <v>1</v>
       </c>
-      <c r="T9" s="48">
+      <c r="T9" s="46">
         <f>SUMIF(G9:O9, "&lt;30")+R9+S9</f>
         <v>37</v>
       </c>
@@ -1941,8 +2021,13 @@
         <f>T9/Q9</f>
         <v>18.5</v>
       </c>
+      <c r="V9" s="99"/>
+      <c r="W9" s="46"/>
+      <c r="X9" s="46"/>
+      <c r="Y9" s="14"/>
+      <c r="Z9" s="97"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26">
       <c r="A10" s="9" t="s">
         <v>29</v>
       </c>
@@ -1952,16 +2037,16 @@
       <c r="C10" s="11">
         <v>10</v>
       </c>
-      <c r="D10" s="85"/>
-      <c r="E10" s="86"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="58"/>
       <c r="F10" s="15">
         <v>46</v>
       </c>
       <c r="G10" s="13">
         <v>18</v>
       </c>
-      <c r="H10" s="85"/>
-      <c r="I10" s="86"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="58"/>
       <c r="J10" s="15"/>
       <c r="K10" s="13"/>
       <c r="L10" s="15">
@@ -1976,7 +2061,7 @@
       <c r="O10" s="13">
         <v>18</v>
       </c>
-      <c r="P10" s="46">
+      <c r="P10" s="14">
         <f>F10+J10+L10+N10</f>
         <v>138</v>
       </c>
@@ -1984,9 +2069,9 @@
         <f>COUNTIF(D10:N10,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="R10" s="50"/>
+      <c r="R10" s="48"/>
       <c r="S10" s="37"/>
-      <c r="T10" s="48">
+      <c r="T10" s="46">
         <f>SUMIF(G10:O10, "&lt;30")+R10+S10</f>
         <v>54</v>
       </c>
@@ -1994,8 +2079,13 @@
         <f>T10/Q10</f>
         <v>18</v>
       </c>
+      <c r="V10" s="100"/>
+      <c r="W10" s="14"/>
+      <c r="X10" s="14"/>
+      <c r="Y10" s="14"/>
+      <c r="Z10" s="97"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26">
       <c r="A11" s="9" t="s">
         <v>24</v>
       </c>
@@ -2005,35 +2095,35 @@
       <c r="C11" s="11">
         <v>21</v>
       </c>
-      <c r="D11" s="85"/>
-      <c r="E11" s="86"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="58"/>
       <c r="F11" s="17">
         <v>61</v>
       </c>
       <c r="G11" s="13">
         <v>14</v>
       </c>
-      <c r="H11" s="85"/>
-      <c r="I11" s="86"/>
+      <c r="H11" s="57"/>
+      <c r="I11" s="58"/>
       <c r="J11" s="17">
         <v>56</v>
       </c>
       <c r="K11" s="13">
         <v>19</v>
       </c>
-      <c r="L11" s="49">
+      <c r="L11" s="47">
         <v>60</v>
       </c>
       <c r="M11" s="13">
         <v>15</v>
       </c>
-      <c r="N11" s="49">
+      <c r="N11" s="47">
         <v>56</v>
       </c>
       <c r="O11" s="13">
         <v>19</v>
       </c>
-      <c r="P11" s="46">
+      <c r="P11" s="14">
         <f>F11+J11+L11+N11</f>
         <v>233</v>
       </c>
@@ -2041,11 +2131,11 @@
         <f>COUNTIF(D11:N11,"&gt;30")</f>
         <v>4</v>
       </c>
-      <c r="R11" s="47">
+      <c r="R11" s="45">
         <v>2</v>
       </c>
       <c r="S11" s="13"/>
-      <c r="T11" s="48">
+      <c r="T11" s="46">
         <f>SUMIF(G11:O11, "&lt;30")+R11+S11</f>
         <v>69</v>
       </c>
@@ -2053,8 +2143,13 @@
         <f>T11/Q11</f>
         <v>17.25</v>
       </c>
+      <c r="V11" s="96"/>
+      <c r="W11" s="46"/>
+      <c r="X11" s="46"/>
+      <c r="Y11" s="14"/>
+      <c r="Z11" s="97"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26">
       <c r="A12" s="9" t="s">
         <v>18</v>
       </c>
@@ -2064,23 +2159,23 @@
       <c r="C12" s="11">
         <v>22</v>
       </c>
-      <c r="D12" s="85"/>
-      <c r="E12" s="86"/>
+      <c r="D12" s="57"/>
+      <c r="E12" s="58"/>
       <c r="F12" s="15">
         <v>59</v>
       </c>
       <c r="G12" s="13">
         <v>17</v>
       </c>
-      <c r="H12" s="85"/>
-      <c r="I12" s="86"/>
+      <c r="H12" s="57"/>
+      <c r="I12" s="58"/>
       <c r="J12" s="15"/>
       <c r="K12" s="13"/>
       <c r="L12" s="15"/>
       <c r="M12" s="13"/>
       <c r="N12" s="15"/>
       <c r="O12" s="13"/>
-      <c r="P12" s="46">
+      <c r="P12" s="14">
         <f>F12+J12+L12+N12</f>
         <v>59</v>
       </c>
@@ -2088,9 +2183,9 @@
         <f>COUNTIF(D12:N12,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="R12" s="47"/>
+      <c r="R12" s="45"/>
       <c r="S12" s="13"/>
-      <c r="T12" s="48">
+      <c r="T12" s="46">
         <f>SUMIF(G12:O12, "&lt;30")+R12+S12</f>
         <v>17</v>
       </c>
@@ -2098,8 +2193,13 @@
         <f>T12/Q12</f>
         <v>17</v>
       </c>
+      <c r="V12" s="99"/>
+      <c r="W12" s="46"/>
+      <c r="X12" s="46"/>
+      <c r="Y12" s="14"/>
+      <c r="Z12" s="97"/>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26">
       <c r="A13" s="9" t="s">
         <v>22</v>
       </c>
@@ -2109,23 +2209,23 @@
       <c r="C13" s="11">
         <v>18</v>
       </c>
-      <c r="D13" s="85"/>
-      <c r="E13" s="86"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="58"/>
       <c r="F13" s="15">
         <v>56</v>
       </c>
       <c r="G13" s="13">
         <v>16</v>
       </c>
-      <c r="H13" s="85"/>
-      <c r="I13" s="86"/>
+      <c r="H13" s="57"/>
+      <c r="I13" s="58"/>
       <c r="J13" s="15"/>
       <c r="K13" s="13"/>
       <c r="L13" s="15"/>
       <c r="M13" s="13"/>
       <c r="N13" s="15"/>
       <c r="O13" s="13"/>
-      <c r="P13" s="46">
+      <c r="P13" s="14">
         <f>F13+J13+L13+N13</f>
         <v>56</v>
       </c>
@@ -2133,9 +2233,9 @@
         <f>COUNTIF(D13:N13,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="R13" s="47"/>
+      <c r="R13" s="45"/>
       <c r="S13" s="13"/>
-      <c r="T13" s="48">
+      <c r="T13" s="46">
         <f>SUMIF(G13:O13, "&lt;30")+R13+S13</f>
         <v>16</v>
       </c>
@@ -2143,8 +2243,13 @@
         <f>T13/Q13</f>
         <v>16</v>
       </c>
+      <c r="V13" s="99"/>
+      <c r="W13" s="46"/>
+      <c r="X13" s="46"/>
+      <c r="Y13" s="14"/>
+      <c r="Z13" s="97"/>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26">
       <c r="A14" s="9" t="s">
         <v>21</v>
       </c>
@@ -2154,16 +2259,16 @@
       <c r="C14" s="11">
         <v>17</v>
       </c>
-      <c r="D14" s="85"/>
-      <c r="E14" s="86"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="58"/>
       <c r="F14" s="15">
         <v>55</v>
       </c>
       <c r="G14" s="13">
         <v>16</v>
       </c>
-      <c r="H14" s="85"/>
-      <c r="I14" s="86"/>
+      <c r="H14" s="57"/>
+      <c r="I14" s="58"/>
       <c r="J14" s="15"/>
       <c r="K14" s="13"/>
       <c r="L14" s="15">
@@ -2178,7 +2283,7 @@
       <c r="O14" s="13">
         <v>14</v>
       </c>
-      <c r="P14" s="46">
+      <c r="P14" s="14">
         <f>F14+J14+L14+N14</f>
         <v>168</v>
       </c>
@@ -2186,9 +2291,9 @@
         <f>COUNTIF(D14:N14,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="R14" s="47"/>
+      <c r="R14" s="45"/>
       <c r="S14" s="13"/>
-      <c r="T14" s="48">
+      <c r="T14" s="46">
         <f>SUMIF(G14:O14, "&lt;30")+R14+S14</f>
         <v>45</v>
       </c>
@@ -2196,8 +2301,13 @@
         <f>T14/Q14</f>
         <v>15</v>
       </c>
+      <c r="V14" s="99"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="46"/>
+      <c r="Y14" s="14"/>
+      <c r="Z14" s="97"/>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26">
       <c r="A15" s="9" t="s">
         <v>26</v>
       </c>
@@ -2207,23 +2317,23 @@
       <c r="C15" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="85"/>
-      <c r="E15" s="86"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="58"/>
       <c r="F15" s="15">
         <v>41</v>
       </c>
       <c r="G15" s="13"/>
-      <c r="H15" s="85"/>
-      <c r="I15" s="86"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="58"/>
       <c r="J15" s="15"/>
       <c r="K15" s="13"/>
       <c r="L15" s="15"/>
       <c r="M15" s="13"/>
-      <c r="N15" s="90">
+      <c r="N15" s="62">
         <v>48</v>
       </c>
       <c r="O15" s="13"/>
-      <c r="P15" s="46">
+      <c r="P15" s="14">
         <f>F15+J15+L15+N15</f>
         <v>89</v>
       </c>
@@ -2231,17 +2341,22 @@
         <f>COUNTIF(D15:N15,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R15" s="47">
+      <c r="R15" s="45">
         <v>1</v>
       </c>
       <c r="S15" s="13"/>
-      <c r="T15" s="48">
+      <c r="T15" s="46">
         <f>SUMIF(G15:O15, "&lt;30")+R15+S15</f>
         <v>1</v>
       </c>
       <c r="U15" s="36"/>
+      <c r="V15" s="99"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="46"/>
+      <c r="Y15" s="14"/>
+      <c r="Z15" s="97"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26">
       <c r="A16" s="9" t="s">
         <v>50</v>
       </c>
@@ -2251,21 +2366,21 @@
       <c r="C16" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="85"/>
-      <c r="E16" s="86"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="58"/>
       <c r="F16" s="19"/>
       <c r="G16" s="13"/>
-      <c r="H16" s="85"/>
-      <c r="I16" s="86"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="58"/>
       <c r="J16" s="19"/>
       <c r="K16" s="13"/>
-      <c r="L16" s="57">
+      <c r="L16" s="54">
         <v>50</v>
       </c>
       <c r="M16" s="13"/>
-      <c r="N16" s="57"/>
+      <c r="N16" s="54"/>
       <c r="O16" s="13"/>
-      <c r="P16" s="46">
+      <c r="P16" s="14">
         <f>F16+J16+L16+N16</f>
         <v>50</v>
       </c>
@@ -2273,17 +2388,22 @@
         <f>COUNTIF(D16:N16,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="R16" s="47">
+      <c r="R16" s="45">
         <v>1</v>
       </c>
       <c r="S16" s="13"/>
-      <c r="T16" s="48">
+      <c r="T16" s="46">
         <f>SUMIF(G16:O16, "&lt;30")+R16+S16</f>
         <v>1</v>
       </c>
       <c r="U16" s="36"/>
+      <c r="V16" s="96"/>
+      <c r="W16" s="46"/>
+      <c r="X16" s="46"/>
+      <c r="Y16" s="14"/>
+      <c r="Z16" s="97"/>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26">
       <c r="A17" s="9" t="s">
         <v>31</v>
       </c>
@@ -2293,14 +2413,14 @@
       <c r="C17" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="85"/>
-      <c r="E17" s="86"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="58"/>
       <c r="F17" s="15">
         <v>51</v>
       </c>
       <c r="G17" s="13"/>
-      <c r="H17" s="85"/>
-      <c r="I17" s="86"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="58"/>
       <c r="J17" s="15"/>
       <c r="K17" s="13"/>
       <c r="L17" s="15"/>
@@ -2309,7 +2429,7 @@
         <v>51</v>
       </c>
       <c r="O17" s="13"/>
-      <c r="P17" s="46">
+      <c r="P17" s="14">
         <f>F17+J17+L17+N17</f>
         <v>102</v>
       </c>
@@ -2317,75 +2437,86 @@
         <f>COUNTIF(D17:N17,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="R17" s="47"/>
+      <c r="R17" s="45"/>
       <c r="S17" s="13"/>
-      <c r="T17" s="48">
+      <c r="T17" s="46">
         <f>SUMIF(G17:O17, "&lt;30")+R17+S17</f>
         <v>0</v>
       </c>
       <c r="U17" s="36"/>
+      <c r="V17" s="99"/>
+      <c r="W17" s="46"/>
+      <c r="X17" s="46"/>
+      <c r="Y17" s="14"/>
+      <c r="Z17" s="97"/>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:26">
       <c r="A18" s="9" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="11">
-        <v>13</v>
-      </c>
-      <c r="D18" s="85"/>
-      <c r="E18" s="86"/>
+        <v>58</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="57"/>
+      <c r="E18" s="58"/>
       <c r="F18" s="18"/>
       <c r="G18" s="13"/>
-      <c r="H18" s="85"/>
-      <c r="I18" s="86"/>
+      <c r="H18" s="57"/>
+      <c r="I18" s="58"/>
       <c r="J18" s="18"/>
       <c r="K18" s="13"/>
       <c r="L18" s="18"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="18"/>
+      <c r="N18" s="47">
+        <v>45</v>
+      </c>
       <c r="O18" s="13"/>
-      <c r="P18" s="46">
+      <c r="P18" s="14">
         <f>F18+J18+L18+N18</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="Q18" s="14">
         <f>COUNTIF(D18:N18,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="R18" s="45"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="46">
         <v>0</v>
       </c>
-      <c r="R18" s="47"/>
-      <c r="S18" s="13"/>
-      <c r="T18" s="48">
-        <f>SUMIF(G18:O18, "&lt;30")+R18+S18</f>
-        <v>0</v>
-      </c>
       <c r="U18" s="36"/>
+      <c r="V18" s="96"/>
+      <c r="W18" s="46"/>
+      <c r="X18" s="46"/>
+      <c r="Y18" s="14"/>
+      <c r="Z18" s="97"/>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26">
       <c r="A19" s="9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C19" s="11">
-        <v>2</v>
-      </c>
-      <c r="D19" s="85"/>
-      <c r="E19" s="86"/>
-      <c r="F19" s="19"/>
+        <v>13</v>
+      </c>
+      <c r="D19" s="57"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="18"/>
       <c r="G19" s="13"/>
-      <c r="H19" s="85"/>
-      <c r="I19" s="86"/>
-      <c r="J19" s="19"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="58"/>
+      <c r="J19" s="18"/>
       <c r="K19" s="13"/>
-      <c r="L19" s="19"/>
+      <c r="L19" s="18"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="19"/>
+      <c r="N19" s="18"/>
       <c r="O19" s="13"/>
-      <c r="P19" s="46">
+      <c r="P19" s="14">
         <f>F19+J19+L19+N19</f>
         <v>0</v>
       </c>
@@ -2393,37 +2524,42 @@
         <f>COUNTIF(D19:N19,"&gt;30")</f>
         <v>0</v>
       </c>
-      <c r="R19" s="47"/>
+      <c r="R19" s="45"/>
       <c r="S19" s="13"/>
-      <c r="T19" s="48">
+      <c r="T19" s="46">
         <f>SUMIF(G19:O19, "&lt;30")+R19+S19</f>
         <v>0</v>
       </c>
       <c r="U19" s="36"/>
+      <c r="V19" s="96"/>
+      <c r="W19" s="46"/>
+      <c r="X19" s="46"/>
+      <c r="Y19" s="14"/>
+      <c r="Z19" s="97"/>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:26">
       <c r="A20" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C20" s="11">
-        <v>15</v>
-      </c>
-      <c r="D20" s="85"/>
-      <c r="E20" s="86"/>
-      <c r="F20" s="15"/>
+        <v>2</v>
+      </c>
+      <c r="D20" s="57"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="19"/>
       <c r="G20" s="13"/>
-      <c r="H20" s="85"/>
-      <c r="I20" s="86"/>
-      <c r="J20" s="15"/>
+      <c r="H20" s="57"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="19"/>
       <c r="K20" s="13"/>
-      <c r="L20" s="15"/>
+      <c r="L20" s="19"/>
       <c r="M20" s="13"/>
-      <c r="N20" s="15"/>
+      <c r="N20" s="19"/>
       <c r="O20" s="13"/>
-      <c r="P20" s="46">
+      <c r="P20" s="14">
         <f>F20+J20+L20+N20</f>
         <v>0</v>
       </c>
@@ -2431,37 +2567,42 @@
         <f>COUNTIF(D20:N20,"&gt;30")</f>
         <v>0</v>
       </c>
-      <c r="R20" s="47"/>
+      <c r="R20" s="45"/>
       <c r="S20" s="13"/>
-      <c r="T20" s="48">
+      <c r="T20" s="46">
         <f>SUMIF(G20:O20, "&lt;30")+R20+S20</f>
         <v>0</v>
       </c>
       <c r="U20" s="36"/>
+      <c r="V20" s="96"/>
+      <c r="W20" s="46"/>
+      <c r="X20" s="46"/>
+      <c r="Y20" s="14"/>
+      <c r="Z20" s="97"/>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26">
       <c r="A21" s="9" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21" s="11">
-        <v>11</v>
-      </c>
-      <c r="D21" s="85"/>
-      <c r="E21" s="86"/>
+        <v>15</v>
+      </c>
+      <c r="D21" s="57"/>
+      <c r="E21" s="58"/>
       <c r="F21" s="15"/>
       <c r="G21" s="13"/>
-      <c r="H21" s="85"/>
-      <c r="I21" s="86"/>
+      <c r="H21" s="57"/>
+      <c r="I21" s="58"/>
       <c r="J21" s="15"/>
       <c r="K21" s="13"/>
       <c r="L21" s="15"/>
       <c r="M21" s="13"/>
       <c r="N21" s="15"/>
       <c r="O21" s="13"/>
-      <c r="P21" s="46">
+      <c r="P21" s="14">
         <f>F21+J21+L21+N21</f>
         <v>0</v>
       </c>
@@ -2469,46 +2610,63 @@
         <f>COUNTIF(D21:N21,"&gt;30")</f>
         <v>0</v>
       </c>
-      <c r="R21" s="47"/>
+      <c r="R21" s="45"/>
       <c r="S21" s="13"/>
-      <c r="T21" s="48">
+      <c r="T21" s="46">
         <f>SUMIF(G21:O21, "&lt;30")+R21+S21</f>
         <v>0</v>
       </c>
       <c r="U21" s="36"/>
+      <c r="V21" s="99"/>
+      <c r="W21" s="46"/>
+      <c r="X21" s="46"/>
+      <c r="Y21" s="14"/>
+      <c r="Z21" s="97"/>
     </row>
-    <row r="22" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="16.5" thickBot="1">
       <c r="A22" s="20" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="87"/>
-      <c r="E22" s="88"/>
-      <c r="F22" s="91"/>
+        <v>39</v>
+      </c>
+      <c r="C22" s="22">
+        <v>11</v>
+      </c>
+      <c r="D22" s="59"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="101"/>
       <c r="G22" s="23"/>
-      <c r="H22" s="87"/>
-      <c r="I22" s="88"/>
-      <c r="J22" s="91"/>
+      <c r="H22" s="59"/>
+      <c r="I22" s="60"/>
+      <c r="J22" s="101"/>
       <c r="K22" s="23"/>
-      <c r="L22" s="91"/>
+      <c r="L22" s="101"/>
       <c r="M22" s="23"/>
-      <c r="N22" s="92">
-        <v>45</v>
-      </c>
+      <c r="N22" s="101"/>
       <c r="O22" s="23"/>
-      <c r="P22" s="51"/>
-      <c r="Q22" s="24"/>
-      <c r="R22" s="52"/>
+      <c r="P22" s="24">
+        <f>F22+J22+L22+N22</f>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="24">
+        <f>COUNTIF(D22:N22,"&gt;30")</f>
+        <v>0</v>
+      </c>
+      <c r="R22" s="49"/>
       <c r="S22" s="23"/>
-      <c r="T22" s="53"/>
+      <c r="T22" s="50">
+        <f>SUMIF(G22:O22, "&lt;30")+R22+S22</f>
+        <v>0</v>
+      </c>
       <c r="U22" s="38"/>
+      <c r="V22" s="102"/>
+      <c r="W22" s="50"/>
+      <c r="X22" s="50"/>
+      <c r="Y22" s="24"/>
+      <c r="Z22" s="103"/>
     </row>
-    <row r="23" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" s="25" customFormat="1" ht="16.5" thickBot="1">
       <c r="A23" s="39"/>
       <c r="B23" s="40"/>
       <c r="C23" s="40"/>
@@ -2537,13 +2695,8 @@
       </c>
       <c r="O23" s="41"/>
       <c r="P23" s="42"/>
-      <c r="Q23" s="25"/>
-      <c r="R23" s="25"/>
-      <c r="S23" s="25"/>
-      <c r="T23" s="25"/>
-      <c r="U23" s="25"/>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:26">
       <c r="C24" s="26"/>
       <c r="P24" s="27"/>
       <c r="Q24" s="27"/>
@@ -2552,8 +2705,8 @@
       <c r="T24" s="27"/>
       <c r="U24" s="29"/>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="C25" s="54" t="s">
+    <row r="25" spans="1:26">
+      <c r="C25" s="51" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="30" t="s">
@@ -2565,8 +2718,8 @@
       <c r="L25" s="30"/>
       <c r="N25" s="30"/>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="C26" s="55" t="s">
+    <row r="26" spans="1:26">
+      <c r="C26" s="52" t="s">
         <v>43</v>
       </c>
       <c r="D26" s="31" t="s">
@@ -2579,8 +2732,8 @@
       <c r="N26" s="31"/>
       <c r="P26" s="32"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="C27" s="56" t="s">
+    <row r="27" spans="1:26">
+      <c r="C27" s="53" t="s">
         <v>48</v>
       </c>
       <c r="D27" s="33" t="s">
@@ -2599,18 +2752,13 @@
       <c r="O27" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="P1:P3"/>
-    <mergeCell ref="Q1:U1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
+  <mergeCells count="27">
+    <mergeCell ref="V1:Z1"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="Z2:Z3"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="J1:K1"/>
@@ -2621,6 +2769,17 @@
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="S2:S3"/>
     <mergeCell ref="J2:K2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="P1:P3"/>
+    <mergeCell ref="Q1:U1"/>
+    <mergeCell ref="N2:O2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
062025 - updated scores for week 7 (6/16/25)
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{0AE6D7ED-C1A2-B14E-A379-CDC667422EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA5799C0-4AE0-4A80-A76B-DE3BFB79B359}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{462BA0F8-5679-0A4A-BF76-1EA90FFAFD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39180" yWindow="780" windowWidth="26730" windowHeight="18135" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="44380" yWindow="1480" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -226,7 +226,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1047,18 +1047,118 @@
     <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1067,106 +1167,6 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1503,140 +1503,140 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
   <dimension ref="A1:Z27"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.75" customWidth="1"/>
-    <col min="2" max="2" width="8.25" customWidth="1"/>
-    <col min="3" max="3" width="10.125" customWidth="1"/>
-    <col min="4" max="9" width="6.875" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="6.875" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="8.1640625" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" customWidth="1"/>
+    <col min="4" max="9" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="6.83203125" customWidth="1"/>
     <col min="11" max="15" width="6" customWidth="1"/>
-    <col min="16" max="16" width="7.625" customWidth="1"/>
-    <col min="17" max="17" width="6.875" customWidth="1"/>
-    <col min="18" max="18" width="5.25" customWidth="1"/>
-    <col min="19" max="19" width="5.75" customWidth="1"/>
+    <col min="16" max="16" width="7.6640625" customWidth="1"/>
+    <col min="17" max="17" width="6.83203125" customWidth="1"/>
+    <col min="18" max="18" width="5.1640625" customWidth="1"/>
+    <col min="19" max="19" width="5.6640625" customWidth="1"/>
     <col min="20" max="20" width="5.5" customWidth="1"/>
     <col min="21" max="21" width="9.5" customWidth="1"/>
-    <col min="22" max="22" width="7.375" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="7.33203125" hidden="1" customWidth="1"/>
     <col min="23" max="24" width="6" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="7.375" hidden="1" customWidth="1"/>
-    <col min="26" max="26" width="9.375" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="91" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="72" t="s">
+    <row r="1" spans="1:26" s="63" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="78" t="s">
+      <c r="B1" s="92"/>
+      <c r="C1" s="97" t="s">
         <v>55</v>
       </c>
-      <c r="D1" s="65" t="s">
+      <c r="D1" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="66"/>
-      <c r="F1" s="65" t="s">
+      <c r="E1" s="80"/>
+      <c r="F1" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="66"/>
-      <c r="H1" s="65" t="s">
+      <c r="G1" s="80"/>
+      <c r="H1" s="79" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="66"/>
-      <c r="J1" s="65" t="s">
+      <c r="I1" s="80"/>
+      <c r="J1" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="66"/>
-      <c r="L1" s="65" t="s">
+      <c r="K1" s="80"/>
+      <c r="L1" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="M1" s="66"/>
-      <c r="N1" s="65" t="s">
+      <c r="M1" s="80"/>
+      <c r="N1" s="79" t="s">
         <v>56</v>
       </c>
-      <c r="O1" s="66"/>
-      <c r="P1" s="63" t="s">
+      <c r="O1" s="80"/>
+      <c r="P1" s="99" t="s">
         <v>2</v>
       </c>
-      <c r="Q1" s="67" t="s">
+      <c r="Q1" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="69"/>
-      <c r="V1" s="88" t="s">
+      <c r="R1" s="102"/>
+      <c r="S1" s="102"/>
+      <c r="T1" s="102"/>
+      <c r="U1" s="103"/>
+      <c r="V1" s="74" t="s">
         <v>59</v>
       </c>
-      <c r="W1" s="89"/>
-      <c r="X1" s="89"/>
-      <c r="Y1" s="89"/>
-      <c r="Z1" s="90"/>
+      <c r="W1" s="75"/>
+      <c r="X1" s="75"/>
+      <c r="Y1" s="75"/>
+      <c r="Z1" s="76"/>
     </row>
-    <row r="2" spans="1:26" s="91" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="74"/>
-      <c r="B2" s="75"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="70">
+    <row r="2" spans="1:26" s="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="93"/>
+      <c r="B2" s="94"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="81">
         <v>45782</v>
       </c>
-      <c r="E2" s="71"/>
-      <c r="F2" s="70">
+      <c r="E2" s="82"/>
+      <c r="F2" s="81">
         <v>45789</v>
       </c>
-      <c r="G2" s="71"/>
-      <c r="H2" s="70">
+      <c r="G2" s="82"/>
+      <c r="H2" s="81">
         <v>45796</v>
       </c>
-      <c r="I2" s="71"/>
-      <c r="J2" s="70">
+      <c r="I2" s="82"/>
+      <c r="J2" s="81">
         <v>45803</v>
       </c>
-      <c r="K2" s="71"/>
-      <c r="L2" s="70">
+      <c r="K2" s="82"/>
+      <c r="L2" s="81">
         <v>45810</v>
       </c>
-      <c r="M2" s="71"/>
-      <c r="N2" s="70">
+      <c r="M2" s="82"/>
+      <c r="N2" s="81">
         <v>45817</v>
       </c>
-      <c r="O2" s="71"/>
-      <c r="P2" s="64"/>
-      <c r="Q2" s="63" t="s">
+      <c r="O2" s="82"/>
+      <c r="P2" s="100"/>
+      <c r="Q2" s="99" t="s">
         <v>4</v>
       </c>
-      <c r="R2" s="84" t="s">
+      <c r="R2" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="S2" s="86" t="s">
+      <c r="S2" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="T2" s="80" t="s">
+      <c r="T2" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="U2" s="82" t="s">
+      <c r="U2" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="92" t="s">
+      <c r="V2" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="W2" s="92" t="s">
+      <c r="W2" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="X2" s="92" t="s">
+      <c r="X2" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="Y2" s="92" t="s">
+      <c r="Y2" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="Z2" s="92" t="s">
+      <c r="Z2" s="77" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:26" s="91" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
-      <c r="A3" s="76"/>
-      <c r="B3" s="77"/>
-      <c r="C3" s="79"/>
+    <row r="3" spans="1:26" s="63" customFormat="1" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="95"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="98"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1673,19 +1673,19 @@
       <c r="O3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="85"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="81"/>
-      <c r="U3" s="83"/>
-      <c r="V3" s="93"/>
-      <c r="W3" s="93"/>
-      <c r="X3" s="93"/>
-      <c r="Y3" s="93"/>
-      <c r="Z3" s="93"/>
+      <c r="P3" s="100"/>
+      <c r="Q3" s="100"/>
+      <c r="R3" s="88"/>
+      <c r="S3" s="90"/>
+      <c r="T3" s="84"/>
+      <c r="U3" s="86"/>
+      <c r="V3" s="78"/>
+      <c r="W3" s="78"/>
+      <c r="X3" s="78"/>
+      <c r="Y3" s="78"/>
+      <c r="Z3" s="78"/>
     </row>
-    <row r="4" spans="1:26" ht="15.95" customHeight="1">
+    <row r="4" spans="1:26" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -1720,32 +1720,32 @@
         <v>19</v>
       </c>
       <c r="P4" s="8">
-        <f>F4+J4+L4+N4</f>
+        <f t="shared" ref="P4:P22" si="0">F4+J4+L4+N4</f>
         <v>110</v>
       </c>
       <c r="Q4" s="8">
-        <f>COUNTIF(D4:N4,"&gt;30")</f>
+        <f t="shared" ref="Q4:Q22" si="1">COUNTIF(D4:N4,"&gt;30")</f>
         <v>2</v>
       </c>
       <c r="R4" s="43"/>
       <c r="S4" s="7"/>
       <c r="T4" s="44">
-        <f>SUMIF(G4:O4, "&lt;30")+R4+S4</f>
+        <f t="shared" ref="T4:T17" si="2">SUMIF(G4:O4, "&lt;30")+R4+S4</f>
         <v>42</v>
       </c>
       <c r="U4" s="35">
-        <f>T4/Q4</f>
+        <f t="shared" ref="U4:U14" si="3">T4/Q4</f>
         <v>21</v>
       </c>
-      <c r="V4" s="94"/>
+      <c r="V4" s="64"/>
       <c r="W4" s="44"/>
       <c r="X4" s="44"/>
       <c r="Y4" s="8"/>
-      <c r="Z4" s="95" t="s">
+      <c r="Z4" s="65" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
@@ -1776,30 +1776,30 @@
       <c r="N5" s="15"/>
       <c r="O5" s="13"/>
       <c r="P5" s="14">
-        <f>F5+J5+L5+N5</f>
+        <f t="shared" si="0"/>
         <v>96</v>
       </c>
       <c r="Q5" s="14">
-        <f>COUNTIF(D5:N5,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="R5" s="45"/>
       <c r="S5" s="13"/>
       <c r="T5" s="46">
-        <f>SUMIF(G5:O5, "&lt;30")+R5+S5</f>
+        <f t="shared" si="2"/>
         <v>42</v>
       </c>
       <c r="U5" s="36">
-        <f>T5/Q5</f>
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
-      <c r="V5" s="96"/>
+      <c r="V5" s="66"/>
       <c r="W5" s="46"/>
       <c r="X5" s="46"/>
       <c r="Y5" s="14"/>
-      <c r="Z5" s="97"/>
+      <c r="Z5" s="67"/>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
@@ -1830,11 +1830,11 @@
       <c r="N6" s="47"/>
       <c r="O6" s="13"/>
       <c r="P6" s="14">
-        <f>F6+J6+L6+N6</f>
+        <f t="shared" si="0"/>
         <v>93</v>
       </c>
       <c r="Q6" s="14">
-        <f>COUNTIF(D6:N6,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="R6" s="45">
@@ -1842,20 +1842,20 @@
       </c>
       <c r="S6" s="13"/>
       <c r="T6" s="46">
-        <f>SUMIF(G6:O6, "&lt;30")+R6+S6</f>
+        <f t="shared" si="2"/>
         <v>42</v>
       </c>
       <c r="U6" s="36">
-        <f>T6/Q6</f>
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
-      <c r="V6" s="96"/>
+      <c r="V6" s="66"/>
       <c r="W6" s="46"/>
       <c r="X6" s="46"/>
       <c r="Y6" s="14"/>
-      <c r="Z6" s="97"/>
+      <c r="Z6" s="67"/>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -1890,11 +1890,11 @@
         <v>21</v>
       </c>
       <c r="P7" s="14">
-        <f>F7+J7+L7+N7</f>
+        <f t="shared" si="0"/>
         <v>129</v>
       </c>
       <c r="Q7" s="14">
-        <f>COUNTIF(D7:N7,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="R7" s="45">
@@ -1904,20 +1904,20 @@
         <v>3</v>
       </c>
       <c r="T7" s="46">
-        <f>SUMIF(G7:O7, "&lt;30")+R7+S7</f>
+        <f t="shared" si="2"/>
         <v>61</v>
       </c>
       <c r="U7" s="36">
-        <f>T7/Q7</f>
+        <f t="shared" si="3"/>
         <v>20.333333333333332</v>
       </c>
-      <c r="V7" s="96"/>
+      <c r="V7" s="66"/>
       <c r="W7" s="46"/>
       <c r="X7" s="46"/>
       <c r="Y7" s="14"/>
-      <c r="Z7" s="97"/>
+      <c r="Z7" s="67"/>
     </row>
-    <row r="8" spans="1:26">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>40</v>
       </c>
@@ -1948,30 +1948,30 @@
         <v>23</v>
       </c>
       <c r="P8" s="14">
-        <f>F8+J8+L8+N8</f>
+        <f t="shared" si="0"/>
         <v>98</v>
       </c>
       <c r="Q8" s="14">
-        <f>COUNTIF(D8:N8,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="R8" s="45"/>
       <c r="S8" s="13"/>
       <c r="T8" s="46">
-        <f>SUMIF(G8:O8, "&lt;30")+R8+S8</f>
+        <f t="shared" si="2"/>
         <v>40</v>
       </c>
       <c r="U8" s="36">
-        <f>T8/Q8</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="V8" s="98"/>
+      <c r="V8" s="68"/>
       <c r="W8" s="46"/>
       <c r="X8" s="46"/>
       <c r="Y8" s="14"/>
-      <c r="Z8" s="97"/>
+      <c r="Z8" s="67"/>
     </row>
-    <row r="9" spans="1:26">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
@@ -2002,11 +2002,11 @@
         <v>20</v>
       </c>
       <c r="P9" s="14">
-        <f>F9+J9+L9+N9</f>
+        <f t="shared" si="0"/>
         <v>88</v>
       </c>
       <c r="Q9" s="14">
-        <f>COUNTIF(D9:N9,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="R9" s="45"/>
@@ -2014,20 +2014,20 @@
         <v>1</v>
       </c>
       <c r="T9" s="46">
-        <f>SUMIF(G9:O9, "&lt;30")+R9+S9</f>
+        <f t="shared" si="2"/>
         <v>37</v>
       </c>
       <c r="U9" s="36">
-        <f>T9/Q9</f>
+        <f t="shared" si="3"/>
         <v>18.5</v>
       </c>
-      <c r="V9" s="99"/>
+      <c r="V9" s="69"/>
       <c r="W9" s="46"/>
       <c r="X9" s="46"/>
       <c r="Y9" s="14"/>
-      <c r="Z9" s="97"/>
+      <c r="Z9" s="67"/>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>29</v>
       </c>
@@ -2062,30 +2062,30 @@
         <v>18</v>
       </c>
       <c r="P10" s="14">
-        <f>F10+J10+L10+N10</f>
+        <f t="shared" si="0"/>
         <v>138</v>
       </c>
       <c r="Q10" s="14">
-        <f>COUNTIF(D10:N10,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="R10" s="48"/>
       <c r="S10" s="37"/>
       <c r="T10" s="46">
-        <f>SUMIF(G10:O10, "&lt;30")+R10+S10</f>
+        <f t="shared" si="2"/>
         <v>54</v>
       </c>
       <c r="U10" s="36">
-        <f>T10/Q10</f>
+        <f t="shared" si="3"/>
         <v>18</v>
       </c>
-      <c r="V10" s="100"/>
+      <c r="V10" s="70"/>
       <c r="W10" s="14"/>
       <c r="X10" s="14"/>
       <c r="Y10" s="14"/>
-      <c r="Z10" s="97"/>
+      <c r="Z10" s="67"/>
     </row>
-    <row r="11" spans="1:26">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>24</v>
       </c>
@@ -2124,11 +2124,11 @@
         <v>19</v>
       </c>
       <c r="P11" s="14">
-        <f>F11+J11+L11+N11</f>
+        <f t="shared" si="0"/>
         <v>233</v>
       </c>
       <c r="Q11" s="14">
-        <f>COUNTIF(D11:N11,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="R11" s="45">
@@ -2136,20 +2136,20 @@
       </c>
       <c r="S11" s="13"/>
       <c r="T11" s="46">
-        <f>SUMIF(G11:O11, "&lt;30")+R11+S11</f>
+        <f t="shared" si="2"/>
         <v>69</v>
       </c>
       <c r="U11" s="36">
-        <f>T11/Q11</f>
+        <f t="shared" si="3"/>
         <v>17.25</v>
       </c>
-      <c r="V11" s="96"/>
+      <c r="V11" s="66"/>
       <c r="W11" s="46"/>
       <c r="X11" s="46"/>
       <c r="Y11" s="14"/>
-      <c r="Z11" s="97"/>
+      <c r="Z11" s="67"/>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>18</v>
       </c>
@@ -2176,30 +2176,30 @@
       <c r="N12" s="15"/>
       <c r="O12" s="13"/>
       <c r="P12" s="14">
-        <f>F12+J12+L12+N12</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
       <c r="Q12" s="14">
-        <f>COUNTIF(D12:N12,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="R12" s="45"/>
       <c r="S12" s="13"/>
       <c r="T12" s="46">
-        <f>SUMIF(G12:O12, "&lt;30")+R12+S12</f>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
       <c r="U12" s="36">
-        <f>T12/Q12</f>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="V12" s="99"/>
+      <c r="V12" s="69"/>
       <c r="W12" s="46"/>
       <c r="X12" s="46"/>
       <c r="Y12" s="14"/>
-      <c r="Z12" s="97"/>
+      <c r="Z12" s="67"/>
     </row>
-    <row r="13" spans="1:26">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>22</v>
       </c>
@@ -2226,30 +2226,30 @@
       <c r="N13" s="15"/>
       <c r="O13" s="13"/>
       <c r="P13" s="14">
-        <f>F13+J13+L13+N13</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
       <c r="Q13" s="14">
-        <f>COUNTIF(D13:N13,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="R13" s="45"/>
       <c r="S13" s="13"/>
       <c r="T13" s="46">
-        <f>SUMIF(G13:O13, "&lt;30")+R13+S13</f>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="U13" s="36">
-        <f>T13/Q13</f>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="V13" s="99"/>
+      <c r="V13" s="69"/>
       <c r="W13" s="46"/>
       <c r="X13" s="46"/>
       <c r="Y13" s="14"/>
-      <c r="Z13" s="97"/>
+      <c r="Z13" s="67"/>
     </row>
-    <row r="14" spans="1:26">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>21</v>
       </c>
@@ -2284,30 +2284,30 @@
         <v>14</v>
       </c>
       <c r="P14" s="14">
-        <f>F14+J14+L14+N14</f>
+        <f t="shared" si="0"/>
         <v>168</v>
       </c>
       <c r="Q14" s="14">
-        <f>COUNTIF(D14:N14,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="R14" s="45"/>
       <c r="S14" s="13"/>
       <c r="T14" s="46">
-        <f>SUMIF(G14:O14, "&lt;30")+R14+S14</f>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="U14" s="36">
-        <f>T14/Q14</f>
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="V14" s="99"/>
+      <c r="V14" s="69"/>
       <c r="W14" s="46"/>
       <c r="X14" s="46"/>
       <c r="Y14" s="14"/>
-      <c r="Z14" s="97"/>
+      <c r="Z14" s="67"/>
     </row>
-    <row r="15" spans="1:26">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>26</v>
       </c>
@@ -2334,11 +2334,11 @@
       </c>
       <c r="O15" s="13"/>
       <c r="P15" s="14">
-        <f>F15+J15+L15+N15</f>
+        <f t="shared" si="0"/>
         <v>89</v>
       </c>
       <c r="Q15" s="14">
-        <f>COUNTIF(D15:N15,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="R15" s="45">
@@ -2346,17 +2346,17 @@
       </c>
       <c r="S15" s="13"/>
       <c r="T15" s="46">
-        <f>SUMIF(G15:O15, "&lt;30")+R15+S15</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="U15" s="36"/>
-      <c r="V15" s="99"/>
+      <c r="V15" s="69"/>
       <c r="W15" s="46"/>
       <c r="X15" s="46"/>
       <c r="Y15" s="14"/>
-      <c r="Z15" s="97"/>
+      <c r="Z15" s="67"/>
     </row>
-    <row r="16" spans="1:26">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>50</v>
       </c>
@@ -2381,11 +2381,11 @@
       <c r="N16" s="54"/>
       <c r="O16" s="13"/>
       <c r="P16" s="14">
-        <f>F16+J16+L16+N16</f>
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="Q16" s="14">
-        <f>COUNTIF(D16:N16,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="R16" s="45">
@@ -2393,17 +2393,17 @@
       </c>
       <c r="S16" s="13"/>
       <c r="T16" s="46">
-        <f>SUMIF(G16:O16, "&lt;30")+R16+S16</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="U16" s="36"/>
-      <c r="V16" s="96"/>
+      <c r="V16" s="66"/>
       <c r="W16" s="46"/>
       <c r="X16" s="46"/>
       <c r="Y16" s="14"/>
-      <c r="Z16" s="97"/>
+      <c r="Z16" s="67"/>
     </row>
-    <row r="17" spans="1:26">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
         <v>31</v>
       </c>
@@ -2430,27 +2430,27 @@
       </c>
       <c r="O17" s="13"/>
       <c r="P17" s="14">
-        <f>F17+J17+L17+N17</f>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
       <c r="Q17" s="14">
-        <f>COUNTIF(D17:N17,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="R17" s="45"/>
       <c r="S17" s="13"/>
       <c r="T17" s="46">
-        <f>SUMIF(G17:O17, "&lt;30")+R17+S17</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U17" s="36"/>
-      <c r="V17" s="99"/>
+      <c r="V17" s="69"/>
       <c r="W17" s="46"/>
       <c r="X17" s="46"/>
       <c r="Y17" s="14"/>
-      <c r="Z17" s="97"/>
+      <c r="Z17" s="67"/>
     </row>
-    <row r="18" spans="1:26">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
         <v>57</v>
       </c>
@@ -2475,11 +2475,11 @@
       </c>
       <c r="O18" s="13"/>
       <c r="P18" s="14">
-        <f>F18+J18+L18+N18</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="Q18" s="14">
-        <f>COUNTIF(D18:N18,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="R18" s="45"/>
@@ -2488,13 +2488,13 @@
         <v>0</v>
       </c>
       <c r="U18" s="36"/>
-      <c r="V18" s="96"/>
+      <c r="V18" s="66"/>
       <c r="W18" s="46"/>
       <c r="X18" s="46"/>
       <c r="Y18" s="14"/>
-      <c r="Z18" s="97"/>
+      <c r="Z18" s="67"/>
     </row>
-    <row r="19" spans="1:26">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
         <v>33</v>
       </c>
@@ -2517,11 +2517,11 @@
       <c r="N19" s="18"/>
       <c r="O19" s="13"/>
       <c r="P19" s="14">
-        <f>F19+J19+L19+N19</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q19" s="14">
-        <f>COUNTIF(D19:N19,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R19" s="45"/>
@@ -2531,13 +2531,13 @@
         <v>0</v>
       </c>
       <c r="U19" s="36"/>
-      <c r="V19" s="96"/>
+      <c r="V19" s="66"/>
       <c r="W19" s="46"/>
       <c r="X19" s="46"/>
       <c r="Y19" s="14"/>
-      <c r="Z19" s="97"/>
+      <c r="Z19" s="67"/>
     </row>
-    <row r="20" spans="1:26">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
         <v>35</v>
       </c>
@@ -2560,11 +2560,11 @@
       <c r="N20" s="19"/>
       <c r="O20" s="13"/>
       <c r="P20" s="14">
-        <f>F20+J20+L20+N20</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q20" s="14">
-        <f>COUNTIF(D20:N20,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R20" s="45"/>
@@ -2574,13 +2574,13 @@
         <v>0</v>
       </c>
       <c r="U20" s="36"/>
-      <c r="V20" s="96"/>
+      <c r="V20" s="66"/>
       <c r="W20" s="46"/>
       <c r="X20" s="46"/>
       <c r="Y20" s="14"/>
-      <c r="Z20" s="97"/>
+      <c r="Z20" s="67"/>
     </row>
-    <row r="21" spans="1:26">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
         <v>37</v>
       </c>
@@ -2603,11 +2603,11 @@
       <c r="N21" s="15"/>
       <c r="O21" s="13"/>
       <c r="P21" s="14">
-        <f>F21+J21+L21+N21</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q21" s="14">
-        <f>COUNTIF(D21:N21,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R21" s="45"/>
@@ -2617,13 +2617,13 @@
         <v>0</v>
       </c>
       <c r="U21" s="36"/>
-      <c r="V21" s="99"/>
+      <c r="V21" s="69"/>
       <c r="W21" s="46"/>
       <c r="X21" s="46"/>
       <c r="Y21" s="14"/>
-      <c r="Z21" s="97"/>
+      <c r="Z21" s="67"/>
     </row>
-    <row r="22" spans="1:26" ht="16.5" thickBot="1">
+    <row r="22" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>31</v>
       </c>
@@ -2635,22 +2635,22 @@
       </c>
       <c r="D22" s="59"/>
       <c r="E22" s="60"/>
-      <c r="F22" s="101"/>
+      <c r="F22" s="71"/>
       <c r="G22" s="23"/>
       <c r="H22" s="59"/>
       <c r="I22" s="60"/>
-      <c r="J22" s="101"/>
+      <c r="J22" s="71"/>
       <c r="K22" s="23"/>
-      <c r="L22" s="101"/>
+      <c r="L22" s="71"/>
       <c r="M22" s="23"/>
-      <c r="N22" s="101"/>
+      <c r="N22" s="71"/>
       <c r="O22" s="23"/>
       <c r="P22" s="24">
-        <f>F22+J22+L22+N22</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q22" s="24">
-        <f>COUNTIF(D22:N22,"&gt;30")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R22" s="49"/>
@@ -2660,13 +2660,13 @@
         <v>0</v>
       </c>
       <c r="U22" s="38"/>
-      <c r="V22" s="102"/>
+      <c r="V22" s="72"/>
       <c r="W22" s="50"/>
       <c r="X22" s="50"/>
       <c r="Y22" s="24"/>
-      <c r="Z22" s="103"/>
+      <c r="Z22" s="73"/>
     </row>
-    <row r="23" spans="1:26" s="25" customFormat="1" ht="16.5" thickBot="1">
+    <row r="23" spans="1:26" s="25" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="39"/>
       <c r="B23" s="40"/>
       <c r="C23" s="40"/>
@@ -2696,7 +2696,7 @@
       <c r="O23" s="41"/>
       <c r="P23" s="42"/>
     </row>
-    <row r="24" spans="1:26">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
       <c r="C24" s="26"/>
       <c r="P24" s="27"/>
       <c r="Q24" s="27"/>
@@ -2705,7 +2705,7 @@
       <c r="T24" s="27"/>
       <c r="U24" s="29"/>
     </row>
-    <row r="25" spans="1:26">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
       <c r="C25" s="51" t="s">
         <v>42</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="L25" s="30"/>
       <c r="N25" s="30"/>
     </row>
-    <row r="26" spans="1:26">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
       <c r="C26" s="52" t="s">
         <v>43</v>
       </c>
@@ -2732,7 +2732,7 @@
       <c r="N26" s="31"/>
       <c r="P26" s="32"/>
     </row>
-    <row r="27" spans="1:26">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
       <c r="C27" s="53" t="s">
         <v>48</v>
       </c>
@@ -2753,12 +2753,12 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="V1:Z1"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="J1:K1"/>
@@ -2769,17 +2769,17 @@
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="S2:S3"/>
     <mergeCell ref="J2:K2"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="N1:O1"/>
     <mergeCell ref="P1:P3"/>
     <mergeCell ref="Q1:U1"/>
     <mergeCell ref="N2:O2"/>
+    <mergeCell ref="V1:Z1"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="Z2:Z3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
062625 - updated scores for week 8 (6/23/25)
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20929D6-00F3-5A48-AA0D-F168C0088495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC0AC718-2FCF-9B46-BFF4-9C25FF493A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44380" yWindow="1480" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="62">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -220,13 +220,16 @@
   </si>
   <si>
     <t>WEEK 7</t>
+  </si>
+  <si>
+    <t>WEEK 8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +342,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1065,9 +1075,6 @@
     <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1093,6 +1100,96 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1117,113 +1214,26 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1559,7 +1569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AD27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1567,141 +1577,150 @@
     <col min="3" max="3" width="10.1640625" customWidth="1"/>
     <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="17" width="6.33203125" customWidth="1"/>
-    <col min="18" max="18" width="6.83203125" customWidth="1"/>
-    <col min="19" max="19" width="6.1640625" customWidth="1"/>
-    <col min="20" max="20" width="5.83203125" customWidth="1"/>
-    <col min="21" max="21" width="5.6640625" customWidth="1"/>
-    <col min="22" max="22" width="5.5" customWidth="1"/>
-    <col min="23" max="23" width="8" customWidth="1"/>
-    <col min="24" max="24" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="25" max="26" width="6" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="13" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="14" max="19" width="6.33203125" customWidth="1"/>
+    <col min="20" max="20" width="6.83203125" customWidth="1"/>
+    <col min="21" max="21" width="6.1640625" customWidth="1"/>
+    <col min="22" max="22" width="5.83203125" customWidth="1"/>
+    <col min="23" max="23" width="5.6640625" customWidth="1"/>
+    <col min="24" max="24" width="5.5" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="26" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="27" max="28" width="6" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="58" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="66" t="s">
+    <row r="1" spans="1:30" s="57" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="95" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="72" t="s">
+      <c r="B1" s="96"/>
+      <c r="C1" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="74" t="s">
+      <c r="D1" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="75"/>
-      <c r="F1" s="74" t="s">
+      <c r="E1" s="81"/>
+      <c r="F1" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="75"/>
-      <c r="H1" s="74" t="s">
+      <c r="G1" s="81"/>
+      <c r="H1" s="80" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="75"/>
-      <c r="J1" s="74" t="s">
+      <c r="I1" s="81"/>
+      <c r="J1" s="80" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="75"/>
-      <c r="L1" s="74" t="s">
+      <c r="K1" s="81"/>
+      <c r="L1" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="75"/>
-      <c r="N1" s="74" t="s">
+      <c r="M1" s="81"/>
+      <c r="N1" s="80" t="s">
         <v>55</v>
       </c>
-      <c r="O1" s="75"/>
-      <c r="P1" s="74" t="s">
+      <c r="O1" s="81"/>
+      <c r="P1" s="80" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="86" t="s">
+      <c r="Q1" s="81"/>
+      <c r="R1" s="80" t="s">
+        <v>61</v>
+      </c>
+      <c r="S1" s="81"/>
+      <c r="T1" s="90" t="s">
         <v>2</v>
       </c>
-      <c r="S1" s="88" t="s">
+      <c r="U1" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="89"/>
-      <c r="U1" s="89"/>
-      <c r="V1" s="89"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="91" t="s">
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
+      <c r="X1" s="93"/>
+      <c r="Y1" s="94"/>
+      <c r="Z1" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="Y1" s="92"/>
-      <c r="Z1" s="92"/>
-      <c r="AA1" s="92"/>
-      <c r="AB1" s="93"/>
+      <c r="AA1" s="76"/>
+      <c r="AB1" s="76"/>
+      <c r="AC1" s="76"/>
+      <c r="AD1" s="77"/>
     </row>
-    <row r="2" spans="1:28" s="58" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="68"/>
-      <c r="B2" s="69"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="76">
+    <row r="2" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="97"/>
+      <c r="B2" s="98"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="73">
         <v>45782</v>
       </c>
-      <c r="E2" s="77"/>
-      <c r="F2" s="76">
+      <c r="E2" s="74"/>
+      <c r="F2" s="73">
         <v>45789</v>
       </c>
-      <c r="G2" s="77"/>
-      <c r="H2" s="76">
+      <c r="G2" s="74"/>
+      <c r="H2" s="73">
         <v>45796</v>
       </c>
-      <c r="I2" s="77"/>
-      <c r="J2" s="76">
+      <c r="I2" s="74"/>
+      <c r="J2" s="73">
         <v>45803</v>
       </c>
-      <c r="K2" s="77"/>
-      <c r="L2" s="76">
+      <c r="K2" s="74"/>
+      <c r="L2" s="73">
         <v>45810</v>
       </c>
-      <c r="M2" s="77"/>
-      <c r="N2" s="76">
+      <c r="M2" s="74"/>
+      <c r="N2" s="73">
         <v>45817</v>
       </c>
-      <c r="O2" s="77"/>
-      <c r="P2" s="76">
+      <c r="O2" s="74"/>
+      <c r="P2" s="73">
         <v>45824</v>
       </c>
-      <c r="Q2" s="77"/>
-      <c r="R2" s="87"/>
-      <c r="S2" s="86" t="s">
+      <c r="Q2" s="74"/>
+      <c r="R2" s="73">
+        <v>45831</v>
+      </c>
+      <c r="S2" s="74"/>
+      <c r="T2" s="91"/>
+      <c r="U2" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="T2" s="82" t="s">
+      <c r="V2" s="86" t="s">
         <v>5</v>
       </c>
-      <c r="U2" s="84" t="s">
+      <c r="W2" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="V2" s="78" t="s">
+      <c r="X2" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="W2" s="80" t="s">
+      <c r="Y2" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="X2" s="94" t="s">
+      <c r="Z2" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="Y2" s="94" t="s">
+      <c r="AA2" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="Z2" s="94" t="s">
+      <c r="AB2" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="AA2" s="94" t="s">
+      <c r="AC2" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="94" t="s">
+      <c r="AD2" s="78" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:28" s="58" customFormat="1" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="71"/>
-      <c r="C3" s="73"/>
+    <row r="3" spans="1:30" s="57" customFormat="1" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="99"/>
+      <c r="B3" s="100"/>
+      <c r="C3" s="102"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1744,19 +1763,25 @@
       <c r="Q3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="R3" s="87"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="83"/>
-      <c r="U3" s="85"/>
-      <c r="V3" s="79"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="95"/>
-      <c r="Y3" s="95"/>
-      <c r="Z3" s="95"/>
-      <c r="AA3" s="95"/>
-      <c r="AB3" s="95"/>
+      <c r="R3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="T3" s="91"/>
+      <c r="U3" s="91"/>
+      <c r="V3" s="87"/>
+      <c r="W3" s="89"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="85"/>
+      <c r="Z3" s="79"/>
+      <c r="AA3" s="79"/>
+      <c r="AB3" s="79"/>
+      <c r="AC3" s="79"/>
+      <c r="AD3" s="79"/>
     </row>
-    <row r="4" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
@@ -1784,770 +1809,840 @@
       <c r="Q4" s="7">
         <v>26</v>
       </c>
-      <c r="R4" s="96">
-        <f>F4+J4+L4+N4+P4</f>
-        <v>43</v>
-      </c>
-      <c r="S4" s="8">
-        <f>COUNTIF(D4:P4,"&gt;30")</f>
+      <c r="R4" s="106">
+        <v>45</v>
+      </c>
+      <c r="S4" s="7">
+        <v>24</v>
+      </c>
+      <c r="T4" s="65">
+        <f>F4+J4+L4+N4+P4+R4</f>
+        <v>88</v>
+      </c>
+      <c r="U4" s="8">
+        <f>COUNTIF(D4:R4,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="V4" s="38">
         <v>1</v>
       </c>
-      <c r="T4" s="38"/>
-      <c r="U4" s="7">
+      <c r="W4" s="7">
         <v>1</v>
       </c>
-      <c r="V4" s="100">
-        <f>SUMIF(G4:Q4, "&lt;30")+T4+U4</f>
-        <v>27</v>
-      </c>
-      <c r="W4" s="59">
-        <f>V4/S4</f>
-        <v>27</v>
-      </c>
-      <c r="X4" s="108"/>
-      <c r="Y4" s="39"/>
-      <c r="Z4" s="39"/>
-      <c r="AA4" s="8"/>
-      <c r="AB4" s="59"/>
+      <c r="X4" s="39">
+        <f>SUMIF(G4:S4, "&lt;30")+V4+W4</f>
+        <v>52</v>
+      </c>
+      <c r="Y4" s="103">
+        <f>X4/U4</f>
+        <v>26</v>
+      </c>
+      <c r="Z4" s="72"/>
+      <c r="AA4" s="39"/>
+      <c r="AB4" s="39"/>
+      <c r="AC4" s="8"/>
+      <c r="AD4" s="58"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C5" s="11">
-        <v>15</v>
+        <f>(T5-(36*U5))/U5</f>
+        <v>17.333333333333332</v>
       </c>
       <c r="D5" s="52"/>
       <c r="E5" s="53"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="12"/>
+      <c r="F5" s="14">
+        <v>53</v>
+      </c>
+      <c r="G5" s="12">
+        <v>23</v>
+      </c>
       <c r="H5" s="52"/>
       <c r="I5" s="53"/>
-      <c r="J5" s="14">
-        <v>52</v>
-      </c>
-      <c r="K5" s="12">
-        <v>17</v>
-      </c>
+      <c r="J5" s="14"/>
+      <c r="K5" s="12"/>
       <c r="L5" s="14"/>
       <c r="M5" s="12"/>
       <c r="N5" s="14">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="O5" s="12">
-        <v>23</v>
-      </c>
-      <c r="P5" s="14">
-        <v>46</v>
-      </c>
-      <c r="Q5" s="12">
-        <v>23</v>
-      </c>
-      <c r="R5" s="97">
-        <f>F5+J5+L5+N5+P5</f>
-        <v>144</v>
-      </c>
-      <c r="S5" s="13">
-        <f>COUNTIF(D5:P5,"&gt;30")</f>
+        <v>19</v>
+      </c>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="14">
+        <v>50</v>
+      </c>
+      <c r="S5" s="12">
+        <v>26</v>
+      </c>
+      <c r="T5" s="66">
+        <f>F5+J5+L5+N5+P5+R5</f>
+        <v>160</v>
+      </c>
+      <c r="U5" s="13">
+        <f>COUNTIF(D5:R5,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="T5" s="40"/>
-      <c r="U5" s="12"/>
-      <c r="V5" s="101">
-        <f>SUMIF(G5:Q5, "&lt;30")+T5+U5</f>
-        <v>63</v>
-      </c>
-      <c r="W5" s="61">
-        <f>V5/S5</f>
-        <v>21</v>
-      </c>
-      <c r="X5" s="60"/>
-      <c r="Y5" s="41"/>
-      <c r="Z5" s="41"/>
-      <c r="AA5" s="13"/>
-      <c r="AB5" s="61"/>
+      <c r="V5" s="40"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="41">
+        <f>SUMIF(G5:S5, "&lt;30")+V5+W5</f>
+        <v>68</v>
+      </c>
+      <c r="Y5" s="104">
+        <f>X5/U5</f>
+        <v>22.666666666666668</v>
+      </c>
+      <c r="Z5" s="59"/>
+      <c r="AA5" s="41"/>
+      <c r="AB5" s="41"/>
+      <c r="AC5" s="13"/>
+      <c r="AD5" s="60" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" s="11">
-        <v>22</v>
+        <f>(T6-(36*U6))/U6</f>
+        <v>11</v>
       </c>
       <c r="D6" s="52"/>
       <c r="E6" s="53"/>
-      <c r="F6" s="14">
-        <v>53</v>
+      <c r="F6" s="107">
+        <v>42</v>
       </c>
       <c r="G6" s="12">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H6" s="52"/>
       <c r="I6" s="53"/>
-      <c r="J6" s="14"/>
+      <c r="J6" s="107"/>
       <c r="K6" s="12"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="14">
-        <v>57</v>
-      </c>
-      <c r="O6" s="12">
-        <v>19</v>
-      </c>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="97">
-        <f>F6+J6+L6+N6+P6</f>
-        <v>110</v>
-      </c>
-      <c r="S6" s="13">
-        <f>COUNTIF(D6:P6,"&gt;30")</f>
+      <c r="L6" s="42">
+        <v>51</v>
+      </c>
+      <c r="M6" s="12">
+        <v>16</v>
+      </c>
+      <c r="N6" s="42"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="15">
+        <v>49</v>
+      </c>
+      <c r="Q6" s="12">
+        <v>18</v>
+      </c>
+      <c r="R6" s="42">
+        <v>46</v>
+      </c>
+      <c r="S6" s="12">
+        <v>21</v>
+      </c>
+      <c r="T6" s="66">
+        <f>F6+J6+L6+N6+P6+R6</f>
+        <v>188</v>
+      </c>
+      <c r="U6" s="13">
+        <f>COUNTIF(D6:R6,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="V6" s="40">
         <v>2</v>
       </c>
-      <c r="T6" s="40"/>
-      <c r="U6" s="12"/>
-      <c r="V6" s="101">
-        <f>SUMIF(G6:Q6, "&lt;30")+T6+U6</f>
-        <v>42</v>
-      </c>
-      <c r="W6" s="61">
-        <f>V6/S6</f>
-        <v>21</v>
-      </c>
-      <c r="X6" s="60"/>
-      <c r="Y6" s="41"/>
-      <c r="Z6" s="41"/>
-      <c r="AA6" s="13"/>
-      <c r="AB6" s="61" t="s">
-        <v>59</v>
-      </c>
+      <c r="W6" s="12"/>
+      <c r="X6" s="41">
+        <f>SUMIF(G6:S6, "&lt;30")+V6+W6</f>
+        <v>82</v>
+      </c>
+      <c r="Y6" s="104">
+        <f>X6/U6</f>
+        <v>20.5</v>
+      </c>
+      <c r="Z6" s="59"/>
+      <c r="AA6" s="41"/>
+      <c r="AB6" s="41"/>
+      <c r="AC6" s="13"/>
+      <c r="AD6" s="60"/>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="C7" s="11">
-        <v>13</v>
+        <f>(T7-(36*U7))/U7</f>
+        <v>13.5</v>
       </c>
       <c r="D7" s="52"/>
       <c r="E7" s="53"/>
-      <c r="F7" s="106">
-        <v>42</v>
-      </c>
-      <c r="G7" s="12">
-        <v>25</v>
-      </c>
+      <c r="F7" s="108"/>
+      <c r="G7" s="12"/>
       <c r="H7" s="52"/>
       <c r="I7" s="53"/>
-      <c r="J7" s="106"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="103">
-        <v>51</v>
-      </c>
-      <c r="M7" s="12">
+      <c r="J7" s="108">
+        <v>52</v>
+      </c>
+      <c r="K7" s="12">
+        <v>17</v>
+      </c>
+      <c r="L7" s="108"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="108">
+        <v>46</v>
+      </c>
+      <c r="O7" s="12">
+        <v>23</v>
+      </c>
+      <c r="P7" s="108">
+        <v>46</v>
+      </c>
+      <c r="Q7" s="12">
+        <v>23</v>
+      </c>
+      <c r="R7" s="108">
+        <v>54</v>
+      </c>
+      <c r="S7" s="12">
         <v>16</v>
       </c>
-      <c r="N7" s="103"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="56">
-        <v>49</v>
-      </c>
-      <c r="Q7" s="12">
-        <v>18</v>
-      </c>
-      <c r="R7" s="97">
-        <f>F7+J7+L7+N7+P7</f>
-        <v>142</v>
-      </c>
-      <c r="S7" s="13">
-        <f>COUNTIF(D7:P7,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="T7" s="40">
-        <v>2</v>
-      </c>
-      <c r="U7" s="12"/>
-      <c r="V7" s="101">
-        <f>SUMIF(G7:Q7, "&lt;30")+T7+U7</f>
-        <v>61</v>
-      </c>
-      <c r="W7" s="61">
-        <f>V7/S7</f>
-        <v>20.333333333333332</v>
-      </c>
-      <c r="X7" s="60"/>
-      <c r="Y7" s="41"/>
-      <c r="Z7" s="41"/>
-      <c r="AA7" s="13"/>
-      <c r="AB7" s="61"/>
+      <c r="T7" s="66">
+        <f>F7+J7+L7+N7+P7+R7</f>
+        <v>198</v>
+      </c>
+      <c r="U7" s="13">
+        <f>COUNTIF(D7:R7,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="V7" s="40"/>
+      <c r="W7" s="12"/>
+      <c r="X7" s="41">
+        <f>SUMIF(G7:S7, "&lt;30")+V7+W7</f>
+        <v>79</v>
+      </c>
+      <c r="Y7" s="104">
+        <f>X7/U7</f>
+        <v>19.75</v>
+      </c>
+      <c r="Z7" s="59"/>
+      <c r="AA7" s="41"/>
+      <c r="AB7" s="41"/>
+      <c r="AC7" s="13"/>
+      <c r="AD7" s="60"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C8" s="11">
-        <v>13</v>
+        <f>(T8-(36*U8))/U8</f>
+        <v>7.6</v>
       </c>
       <c r="D8" s="52"/>
       <c r="E8" s="53"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="12"/>
+      <c r="F8" s="70">
+        <v>45</v>
+      </c>
+      <c r="G8" s="12">
+        <v>17</v>
+      </c>
       <c r="H8" s="52"/>
       <c r="I8" s="53"/>
-      <c r="J8" s="16"/>
+      <c r="J8" s="70"/>
       <c r="K8" s="12"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="12"/>
+      <c r="L8" s="70">
+        <v>43</v>
+      </c>
+      <c r="M8" s="12">
+        <v>19</v>
+      </c>
+      <c r="N8" s="15">
+        <v>41</v>
+      </c>
+      <c r="O8" s="12">
+        <v>21</v>
+      </c>
       <c r="P8" s="42">
         <v>47</v>
       </c>
       <c r="Q8" s="12">
+        <v>15</v>
+      </c>
+      <c r="R8" s="42">
+        <v>42</v>
+      </c>
+      <c r="S8" s="12">
         <v>20</v>
       </c>
-      <c r="R8" s="97">
-        <f>F8+J8+L8+N8+P8</f>
-        <v>47</v>
-      </c>
-      <c r="S8" s="13">
-        <f>COUNTIF(D8:P8,"&gt;30")</f>
+      <c r="T8" s="66">
+        <f>F8+J8+L8+N8+P8+R8</f>
+        <v>218</v>
+      </c>
+      <c r="U8" s="13">
+        <f>COUNTIF(D8:R8,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="V8" s="40">
         <v>1</v>
       </c>
-      <c r="T8" s="40"/>
-      <c r="U8" s="12"/>
-      <c r="V8" s="101">
-        <f>SUMIF(G8:Q8, "&lt;30")+T8+U8</f>
-        <v>20</v>
-      </c>
-      <c r="W8" s="61">
-        <f>V8/S8</f>
-        <v>20</v>
-      </c>
-      <c r="X8" s="62"/>
-      <c r="Y8" s="41"/>
-      <c r="Z8" s="41"/>
-      <c r="AA8" s="13"/>
-      <c r="AB8" s="61"/>
+      <c r="W8" s="12">
+        <v>3</v>
+      </c>
+      <c r="X8" s="41">
+        <f>SUMIF(G8:S8, "&lt;30")+V8+W8</f>
+        <v>96</v>
+      </c>
+      <c r="Y8" s="104">
+        <f>X8/U8</f>
+        <v>19.2</v>
+      </c>
+      <c r="Z8" s="61"/>
+      <c r="AA8" s="41"/>
+      <c r="AB8" s="41"/>
+      <c r="AC8" s="13"/>
+      <c r="AD8" s="60"/>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="11">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="53"/>
       <c r="F9" s="14">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="G9" s="12">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H9" s="52"/>
       <c r="I9" s="53"/>
       <c r="J9" s="14"/>
       <c r="K9" s="12"/>
-      <c r="L9" s="14">
-        <v>54</v>
-      </c>
-      <c r="M9" s="12">
-        <v>15</v>
-      </c>
+      <c r="L9" s="14"/>
+      <c r="M9" s="12"/>
       <c r="N9" s="14"/>
       <c r="O9" s="12"/>
-      <c r="P9" s="14">
-        <v>54</v>
-      </c>
-      <c r="Q9" s="12">
-        <v>16</v>
-      </c>
-      <c r="R9" s="97">
-        <f>F9+J9+L9+N9+P9</f>
-        <v>150</v>
-      </c>
-      <c r="S9" s="13">
-        <f>COUNTIF(D9:P9,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="T9" s="40"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="101">
-        <f>SUMIF(G9:Q9, "&lt;30")+T9+U9</f>
-        <v>58</v>
-      </c>
-      <c r="W9" s="61">
-        <f>V9/S9</f>
-        <v>19.333333333333332</v>
-      </c>
-      <c r="X9" s="60"/>
-      <c r="Y9" s="41"/>
-      <c r="Z9" s="41"/>
-      <c r="AA9" s="13"/>
-      <c r="AB9" s="61"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="14">
+        <v>55</v>
+      </c>
+      <c r="S9" s="12">
+        <v>21</v>
+      </c>
+      <c r="T9" s="66">
+        <f>F9+J9+L9+N9+P9+R9</f>
+        <v>114</v>
+      </c>
+      <c r="U9" s="13">
+        <f>COUNTIF(D9:R9,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="V9" s="40"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="41">
+        <f>SUMIF(G9:S9, "&lt;30")+V9+W9</f>
+        <v>38</v>
+      </c>
+      <c r="Y9" s="104">
+        <f>X9/U9</f>
+        <v>19</v>
+      </c>
+      <c r="Z9" s="62"/>
+      <c r="AA9" s="41"/>
+      <c r="AB9" s="41"/>
+      <c r="AC9" s="13"/>
+      <c r="AD9" s="60"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C10" s="11">
-        <v>8</v>
+        <f>(T10-(36*U10))/U10</f>
+        <v>7.666666666666667</v>
       </c>
       <c r="D10" s="52"/>
       <c r="E10" s="53"/>
-      <c r="F10" s="105">
-        <v>45</v>
+      <c r="F10" s="14">
+        <v>46</v>
       </c>
       <c r="G10" s="12">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H10" s="52"/>
       <c r="I10" s="53"/>
-      <c r="J10" s="105"/>
+      <c r="J10" s="14"/>
       <c r="K10" s="12"/>
-      <c r="L10" s="105">
+      <c r="L10" s="14"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="14">
+        <v>42</v>
+      </c>
+      <c r="O10" s="12">
+        <v>20</v>
+      </c>
+      <c r="P10" s="14">
         <v>43</v>
       </c>
-      <c r="M10" s="12">
+      <c r="Q10" s="12">
         <v>19</v>
       </c>
-      <c r="N10" s="15">
-        <v>41</v>
-      </c>
-      <c r="O10" s="12">
-        <v>21</v>
-      </c>
-      <c r="P10" s="42">
-        <v>47</v>
-      </c>
-      <c r="Q10" s="12">
-        <v>15</v>
-      </c>
-      <c r="R10" s="97">
-        <f>F10+J10+L10+N10+P10</f>
-        <v>176</v>
-      </c>
-      <c r="S10" s="13">
-        <f>COUNTIF(D10:P10,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="T10" s="40">
+      <c r="R10" s="14"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="66">
+        <f>F10+J10+L10+N10+P10+R10</f>
+        <v>131</v>
+      </c>
+      <c r="U10" s="13">
+        <f>COUNTIF(D10:R10,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="V10" s="40"/>
+      <c r="W10" s="12">
         <v>1</v>
       </c>
-      <c r="U10" s="12">
-        <v>3</v>
-      </c>
-      <c r="V10" s="101">
-        <f>SUMIF(G10:Q10, "&lt;30")+T10+U10</f>
-        <v>76</v>
-      </c>
-      <c r="W10" s="61">
-        <f>V10/S10</f>
-        <v>19</v>
-      </c>
-      <c r="X10" s="109"/>
-      <c r="Y10" s="41"/>
-      <c r="Z10" s="41"/>
-      <c r="AA10" s="13"/>
-      <c r="AB10" s="61"/>
+      <c r="X10" s="41">
+        <f>SUMIF(G10:S10, "&lt;30")+V10+W10</f>
+        <v>56</v>
+      </c>
+      <c r="Y10" s="104">
+        <f>X10/U10</f>
+        <v>18.666666666666668</v>
+      </c>
+      <c r="Z10" s="109"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="60"/>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C11" s="11">
-        <v>8</v>
+        <f>(T11-(36*U11))/U11</f>
+        <v>14.75</v>
       </c>
       <c r="D11" s="52"/>
       <c r="E11" s="53"/>
       <c r="F11" s="14">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G11" s="12">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="H11" s="52"/>
       <c r="I11" s="53"/>
       <c r="J11" s="14"/>
       <c r="K11" s="12"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="14">
-        <v>42</v>
-      </c>
-      <c r="O11" s="12">
-        <v>20</v>
-      </c>
+      <c r="L11" s="14">
+        <v>54</v>
+      </c>
+      <c r="M11" s="12">
+        <v>15</v>
+      </c>
+      <c r="N11" s="14"/>
+      <c r="O11" s="12"/>
       <c r="P11" s="14">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="12">
-        <v>19</v>
-      </c>
-      <c r="R11" s="97">
-        <f>F11+J11+L11+N11+P11</f>
-        <v>131</v>
-      </c>
-      <c r="S11" s="13">
-        <f>COUNTIF(D11:P11,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="T11" s="40"/>
-      <c r="U11" s="12">
-        <v>1</v>
-      </c>
-      <c r="V11" s="101">
-        <f>SUMIF(G11:Q11, "&lt;30")+T11+U11</f>
-        <v>56</v>
-      </c>
-      <c r="W11" s="61">
-        <f>V11/S11</f>
-        <v>18.666666666666668</v>
-      </c>
-      <c r="X11" s="63"/>
-      <c r="Y11" s="41"/>
-      <c r="Z11" s="41"/>
-      <c r="AA11" s="13"/>
-      <c r="AB11" s="61"/>
+        <v>16</v>
+      </c>
+      <c r="R11" s="14">
+        <v>53</v>
+      </c>
+      <c r="S11" s="12">
+        <v>16</v>
+      </c>
+      <c r="T11" s="66">
+        <f>F11+J11+L11+N11+P11+R11</f>
+        <v>203</v>
+      </c>
+      <c r="U11" s="13">
+        <f>COUNTIF(D11:R11,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="V11" s="40"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="41">
+        <f>SUMIF(G11:S11, "&lt;30")+V11+W11</f>
+        <v>74</v>
+      </c>
+      <c r="Y11" s="104">
+        <f>X11/U11</f>
+        <v>18.5</v>
+      </c>
+      <c r="Z11" s="59"/>
+      <c r="AA11" s="41"/>
+      <c r="AB11" s="41"/>
+      <c r="AC11" s="13"/>
+      <c r="AD11" s="60"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C12" s="11">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D12" s="52"/>
       <c r="E12" s="53"/>
-      <c r="F12" s="15">
-        <v>61</v>
-      </c>
-      <c r="G12" s="12">
-        <v>14</v>
-      </c>
+      <c r="F12" s="16"/>
+      <c r="G12" s="12"/>
       <c r="H12" s="52"/>
       <c r="I12" s="53"/>
-      <c r="J12" s="15">
-        <v>56</v>
-      </c>
-      <c r="K12" s="12">
-        <v>19</v>
-      </c>
-      <c r="L12" s="42">
-        <v>60</v>
-      </c>
-      <c r="M12" s="12">
-        <v>15</v>
-      </c>
-      <c r="N12" s="42">
-        <v>56</v>
-      </c>
-      <c r="O12" s="12">
+      <c r="J12" s="16"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="42">
+        <v>47</v>
+      </c>
+      <c r="Q12" s="12">
         <v>20</v>
       </c>
-      <c r="P12" s="42">
-        <v>54</v>
-      </c>
-      <c r="Q12" s="12">
-        <v>22</v>
-      </c>
-      <c r="R12" s="97">
-        <f>F12+J12+L12+N12+P12</f>
-        <v>287</v>
-      </c>
-      <c r="S12" s="13">
-        <f>COUNTIF(D12:P12,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="T12" s="40">
+      <c r="R12" s="42">
+        <v>50</v>
+      </c>
+      <c r="S12" s="12">
+        <v>17</v>
+      </c>
+      <c r="T12" s="66">
+        <f>F12+J12+L12+N12+P12+R12</f>
+        <v>97</v>
+      </c>
+      <c r="U12" s="13">
+        <f>COUNTIF(D12:R12,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="U12" s="12"/>
-      <c r="V12" s="101">
-        <f>SUMIF(G12:Q12, "&lt;30")+T12+U12</f>
-        <v>92</v>
-      </c>
-      <c r="W12" s="61">
-        <f>V12/S12</f>
-        <v>18.399999999999999</v>
-      </c>
-      <c r="X12" s="60"/>
-      <c r="Y12" s="41"/>
-      <c r="Z12" s="41"/>
-      <c r="AA12" s="13"/>
-      <c r="AB12" s="61"/>
+      <c r="V12" s="40"/>
+      <c r="W12" s="12"/>
+      <c r="X12" s="41">
+        <f>SUMIF(G12:S12, "&lt;30")+V12+W12</f>
+        <v>37</v>
+      </c>
+      <c r="Y12" s="104">
+        <f>X12/U12</f>
+        <v>18.5</v>
+      </c>
+      <c r="Z12" s="59"/>
+      <c r="AA12" s="41"/>
+      <c r="AB12" s="41"/>
+      <c r="AC12" s="13"/>
+      <c r="AD12" s="60"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C13" s="11">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D13" s="52"/>
       <c r="E13" s="53"/>
-      <c r="F13" s="14">
-        <v>46</v>
-      </c>
-      <c r="G13" s="12">
-        <v>18</v>
-      </c>
+      <c r="F13" s="17"/>
+      <c r="G13" s="12"/>
       <c r="H13" s="52"/>
       <c r="I13" s="53"/>
-      <c r="J13" s="14"/>
+      <c r="J13" s="17"/>
       <c r="K13" s="12"/>
-      <c r="L13" s="14">
-        <v>46</v>
-      </c>
-      <c r="M13" s="12">
+      <c r="L13" s="17"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="68">
+        <v>39</v>
+      </c>
+      <c r="Q13" s="12">
+        <v>17</v>
+      </c>
+      <c r="R13" s="68">
+        <v>38</v>
+      </c>
+      <c r="S13" s="12">
         <v>18</v>
       </c>
-      <c r="N13" s="14">
-        <v>46</v>
-      </c>
-      <c r="O13" s="12">
-        <v>18</v>
-      </c>
-      <c r="P13" s="14">
-        <v>46</v>
-      </c>
-      <c r="Q13" s="12">
-        <v>18</v>
-      </c>
-      <c r="R13" s="97">
-        <f>F13+J13+L13+N13+P13</f>
-        <v>184</v>
-      </c>
-      <c r="S13" s="13">
-        <f>COUNTIF(D13:P13,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="T13" s="43"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="101">
-        <f>SUMIF(G13:Q13, "&lt;30")+T13+U13</f>
-        <v>72</v>
-      </c>
-      <c r="W13" s="61">
-        <f>V13/S13</f>
-        <v>18</v>
-      </c>
-      <c r="X13" s="63"/>
-      <c r="Y13" s="13"/>
-      <c r="Z13" s="13"/>
-      <c r="AA13" s="13"/>
-      <c r="AB13" s="61"/>
+      <c r="T13" s="66">
+        <f>F13+J13+L13+N13+P13+R13</f>
+        <v>77</v>
+      </c>
+      <c r="U13" s="13">
+        <f>COUNTIF(D13:R13,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="V13" s="40"/>
+      <c r="W13" s="12">
+        <v>2</v>
+      </c>
+      <c r="X13" s="41">
+        <f>SUMIF(G13:S13, "&lt;30")+V13+W13</f>
+        <v>37</v>
+      </c>
+      <c r="Y13" s="104">
+        <f>X13/U13</f>
+        <v>18.5</v>
+      </c>
+      <c r="Z13" s="59"/>
+      <c r="AA13" s="41"/>
+      <c r="AB13" s="41"/>
+      <c r="AC13" s="13"/>
+      <c r="AD13" s="60"/>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C14" s="11">
-        <v>8</v>
+        <f>(T14-(36*U14))/U14</f>
+        <v>21.4</v>
       </c>
       <c r="D14" s="52"/>
       <c r="E14" s="53"/>
-      <c r="F14" s="14">
-        <v>41</v>
+      <c r="F14" s="15">
+        <v>61</v>
       </c>
       <c r="G14" s="12">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H14" s="52"/>
       <c r="I14" s="53"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="57">
-        <v>48</v>
+      <c r="J14" s="15">
+        <v>56</v>
+      </c>
+      <c r="K14" s="12">
+        <v>19</v>
+      </c>
+      <c r="L14" s="42">
+        <v>60</v>
+      </c>
+      <c r="M14" s="12">
+        <v>15</v>
+      </c>
+      <c r="N14" s="42">
+        <v>56</v>
       </c>
       <c r="O14" s="12">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="P14" s="42">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="Q14" s="12">
-        <v>18</v>
-      </c>
-      <c r="R14" s="97">
-        <f>F14+J14+L14+N14+P14</f>
-        <v>133</v>
-      </c>
-      <c r="S14" s="13">
-        <f>COUNTIF(D14:P14,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="T14" s="40">
-        <v>1</v>
-      </c>
-      <c r="U14" s="12"/>
-      <c r="V14" s="101">
-        <f>SUMIF(G14:Q14, "&lt;30")+T14+U14</f>
-        <v>54</v>
-      </c>
-      <c r="W14" s="61">
-        <f>V14/S14</f>
-        <v>18</v>
-      </c>
-      <c r="X14" s="63"/>
-      <c r="Y14" s="41"/>
-      <c r="Z14" s="41"/>
-      <c r="AA14" s="13"/>
-      <c r="AB14" s="61"/>
+        <v>22</v>
+      </c>
+      <c r="R14" s="42"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="66">
+        <f>F14+J14+L14+N14+P14+R14</f>
+        <v>287</v>
+      </c>
+      <c r="U14" s="13">
+        <f>COUNTIF(D14:R14,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="V14" s="40">
+        <v>2</v>
+      </c>
+      <c r="W14" s="12"/>
+      <c r="X14" s="41">
+        <f>SUMIF(G14:S14, "&lt;30")+V14+W14</f>
+        <v>92</v>
+      </c>
+      <c r="Y14" s="104">
+        <f>X14/U14</f>
+        <v>18.399999999999999</v>
+      </c>
+      <c r="Z14" s="59"/>
+      <c r="AA14" s="41"/>
+      <c r="AB14" s="41"/>
+      <c r="AC14" s="13"/>
+      <c r="AD14" s="60"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C15" s="11">
-        <v>11</v>
+        <f>(T15-(36*U15))/U15</f>
+        <v>8.3333333333333339</v>
       </c>
       <c r="D15" s="52"/>
       <c r="E15" s="53"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="12"/>
+      <c r="F15" s="14">
+        <v>41</v>
+      </c>
+      <c r="G15" s="12">
+        <v>21</v>
+      </c>
       <c r="H15" s="52"/>
       <c r="I15" s="53"/>
       <c r="J15" s="14"/>
       <c r="K15" s="12"/>
       <c r="L15" s="14"/>
       <c r="M15" s="12"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="12"/>
-      <c r="P15" s="14">
+      <c r="N15" s="56">
         <v>48</v>
+      </c>
+      <c r="O15" s="12">
+        <v>14</v>
+      </c>
+      <c r="P15" s="42">
+        <v>44</v>
       </c>
       <c r="Q15" s="12">
         <v>18</v>
       </c>
-      <c r="R15" s="97">
-        <f>F15+J15+L15+N15+P15</f>
-        <v>48</v>
-      </c>
-      <c r="S15" s="13">
-        <f>COUNTIF(D15:P15,"&gt;30")</f>
+      <c r="R15" s="42"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="66">
+        <f>F15+J15+L15+N15+P15+R15</f>
+        <v>133</v>
+      </c>
+      <c r="U15" s="13">
+        <f>COUNTIF(D15:R15,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="V15" s="40">
         <v>1</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="12"/>
-      <c r="V15" s="101">
-        <f>SUMIF(G15:Q15, "&lt;30")+T15+U15</f>
+      <c r="W15" s="12"/>
+      <c r="X15" s="41">
+        <f>SUMIF(G15:S15, "&lt;30")+V15+W15</f>
+        <v>54</v>
+      </c>
+      <c r="Y15" s="104">
+        <f>X15/U15</f>
         <v>18</v>
       </c>
-      <c r="W15" s="61">
-        <f>V15/S15</f>
-        <v>18</v>
-      </c>
-      <c r="X15" s="60"/>
-      <c r="Y15" s="41"/>
-      <c r="Z15" s="41"/>
-      <c r="AA15" s="13"/>
-      <c r="AB15" s="61"/>
+      <c r="Z15" s="62"/>
+      <c r="AA15" s="41"/>
+      <c r="AB15" s="41"/>
+      <c r="AC15" s="13"/>
+      <c r="AD15" s="60"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C16" s="11">
-        <v>2</v>
+        <f>(T16-(36*U16))/U16</f>
+        <v>15.333333333333334</v>
       </c>
       <c r="D16" s="52"/>
       <c r="E16" s="53"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="12"/>
+      <c r="F16" s="14">
+        <v>51</v>
+      </c>
+      <c r="G16" s="12">
+        <v>18</v>
+      </c>
       <c r="H16" s="52"/>
       <c r="I16" s="53"/>
-      <c r="J16" s="17"/>
+      <c r="J16" s="14"/>
       <c r="K16" s="12"/>
-      <c r="L16" s="17"/>
+      <c r="L16" s="14"/>
       <c r="M16" s="12"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="12"/>
-      <c r="P16" s="99">
-        <v>39</v>
+      <c r="N16" s="14">
+        <v>51</v>
+      </c>
+      <c r="O16" s="12">
+        <v>18</v>
+      </c>
+      <c r="P16" s="14">
+        <v>52</v>
       </c>
       <c r="Q16" s="12">
         <v>17</v>
       </c>
-      <c r="R16" s="97">
-        <f>F16+J16+L16+N16+P16</f>
-        <v>39</v>
-      </c>
-      <c r="S16" s="13">
-        <f>COUNTIF(D16:P16,"&gt;30")</f>
-        <v>1</v>
-      </c>
-      <c r="T16" s="40"/>
-      <c r="U16" s="12">
-        <v>1</v>
-      </c>
-      <c r="V16" s="101">
-        <f>SUMIF(G16:Q16, "&lt;30")+T16+U16</f>
-        <v>18</v>
-      </c>
-      <c r="W16" s="61">
-        <f>V16/S16</f>
-        <v>18</v>
-      </c>
-      <c r="X16" s="60"/>
-      <c r="Y16" s="41"/>
-      <c r="Z16" s="41"/>
-      <c r="AA16" s="13"/>
-      <c r="AB16" s="61"/>
+      <c r="R16" s="14"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="66">
+        <f>F16+J16+L16+N16+P16+R16</f>
+        <v>154</v>
+      </c>
+      <c r="U16" s="13">
+        <f>COUNTIF(D16:R16,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="V16" s="40"/>
+      <c r="W16" s="12"/>
+      <c r="X16" s="41">
+        <f>SUMIF(G16:S16, "&lt;30")+V16+W16</f>
+        <v>53</v>
+      </c>
+      <c r="Y16" s="104">
+        <f>X16/U16</f>
+        <v>17.666666666666668</v>
+      </c>
+      <c r="Z16" s="62"/>
+      <c r="AA16" s="41"/>
+      <c r="AB16" s="41"/>
+      <c r="AC16" s="13"/>
+      <c r="AD16" s="60"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C17" s="11">
-        <v>15</v>
+        <f>(T17-(36*U17))/U17</f>
+        <v>10.199999999999999</v>
       </c>
       <c r="D17" s="52"/>
       <c r="E17" s="53"/>
       <c r="F17" s="14">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G17" s="12">
         <v>18</v>
@@ -2556,62 +2651,68 @@
       <c r="I17" s="53"/>
       <c r="J17" s="14"/>
       <c r="K17" s="12"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="12"/>
+      <c r="L17" s="14">
+        <v>46</v>
+      </c>
+      <c r="M17" s="12">
+        <v>18</v>
+      </c>
       <c r="N17" s="14">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="O17" s="12">
         <v>18</v>
       </c>
       <c r="P17" s="14">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="Q17" s="12">
-        <v>17</v>
-      </c>
-      <c r="R17" s="97">
-        <f>F17+J17+L17+N17+P17</f>
-        <v>154</v>
-      </c>
-      <c r="S17" s="13">
-        <f>COUNTIF(D17:P17,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="T17" s="40"/>
-      <c r="U17" s="12"/>
-      <c r="V17" s="101">
-        <f>SUMIF(G17:Q17, "&lt;30")+T17+U17</f>
-        <v>53</v>
-      </c>
-      <c r="W17" s="61">
-        <f>V17/S17</f>
-        <v>17.666666666666668</v>
-      </c>
-      <c r="X17" s="63"/>
-      <c r="Y17" s="41"/>
-      <c r="Z17" s="41"/>
+        <v>18</v>
+      </c>
+      <c r="R17" s="14">
+        <v>47</v>
+      </c>
+      <c r="S17" s="12">
+        <v>14</v>
+      </c>
+      <c r="T17" s="66">
+        <f>F17+J17+L17+N17+P17+R17</f>
+        <v>231</v>
+      </c>
+      <c r="U17" s="13">
+        <f>COUNTIF(D17:R17,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="V17" s="43"/>
+      <c r="W17" s="33"/>
+      <c r="X17" s="41">
+        <f>SUMIF(G17:S17, "&lt;30")+V17+W17</f>
+        <v>86</v>
+      </c>
+      <c r="Y17" s="104">
+        <f>X17/U17</f>
+        <v>17.2</v>
+      </c>
+      <c r="Z17" s="62"/>
       <c r="AA17" s="13"/>
-      <c r="AB17" s="61"/>
+      <c r="AB17" s="13"/>
+      <c r="AC17" s="13"/>
+      <c r="AD17" s="60"/>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C18" s="11">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D18" s="52"/>
       <c r="E18" s="53"/>
-      <c r="F18" s="14">
-        <v>59</v>
-      </c>
-      <c r="G18" s="12">
-        <v>17</v>
-      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="12"/>
       <c r="H18" s="52"/>
       <c r="I18" s="53"/>
       <c r="J18" s="14"/>
@@ -2620,33 +2721,43 @@
       <c r="M18" s="12"/>
       <c r="N18" s="14"/>
       <c r="O18" s="12"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="97">
-        <f>F18+J18+L18+N18+P18</f>
-        <v>59</v>
-      </c>
-      <c r="S18" s="13">
-        <f>COUNTIF(D18:P18,"&gt;30")</f>
-        <v>1</v>
-      </c>
-      <c r="T18" s="40"/>
-      <c r="U18" s="12"/>
-      <c r="V18" s="101">
-        <f>SUMIF(G18:Q18, "&lt;30")+T18+U18</f>
-        <v>17</v>
-      </c>
-      <c r="W18" s="61">
-        <f>V18/S18</f>
-        <v>17</v>
-      </c>
-      <c r="X18" s="63"/>
-      <c r="Y18" s="41"/>
-      <c r="Z18" s="41"/>
-      <c r="AA18" s="13"/>
-      <c r="AB18" s="61"/>
+      <c r="P18" s="14">
+        <v>48</v>
+      </c>
+      <c r="Q18" s="12">
+        <v>18</v>
+      </c>
+      <c r="R18" s="14">
+        <v>51</v>
+      </c>
+      <c r="S18" s="12">
+        <v>14</v>
+      </c>
+      <c r="T18" s="66">
+        <f>F18+J18+L18+N18+P18+R18</f>
+        <v>99</v>
+      </c>
+      <c r="U18" s="13">
+        <f>COUNTIF(D18:R18,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="V18" s="40"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="41">
+        <f>SUMIF(G18:S18, "&lt;30")+V18+W18</f>
+        <v>32</v>
+      </c>
+      <c r="Y18" s="104">
+        <f>X18/U18</f>
+        <v>16</v>
+      </c>
+      <c r="Z18" s="59"/>
+      <c r="AA18" s="41"/>
+      <c r="AB18" s="41"/>
+      <c r="AC18" s="13"/>
+      <c r="AD18" s="60"/>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
         <v>22</v>
       </c>
@@ -2674,31 +2785,33 @@
       <c r="O19" s="12"/>
       <c r="P19" s="14"/>
       <c r="Q19" s="12"/>
-      <c r="R19" s="97">
-        <f>F19+J19+L19+N19+P19</f>
+      <c r="R19" s="14"/>
+      <c r="S19" s="12"/>
+      <c r="T19" s="66">
+        <f>F19+J19+L19+N19+P19+R19</f>
         <v>56</v>
       </c>
-      <c r="S19" s="13">
-        <f>COUNTIF(D19:P19,"&gt;30")</f>
+      <c r="U19" s="13">
+        <f>COUNTIF(D19:R19,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="T19" s="40"/>
-      <c r="U19" s="12"/>
-      <c r="V19" s="101">
-        <f>SUMIF(G19:Q19, "&lt;30")+T19+U19</f>
+      <c r="V19" s="40"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="41">
+        <f>SUMIF(G19:S19, "&lt;30")+V19+W19</f>
         <v>16</v>
       </c>
-      <c r="W19" s="61">
-        <f>V19/S19</f>
+      <c r="Y19" s="104">
+        <f>X19/U19</f>
         <v>16</v>
       </c>
-      <c r="X19" s="63"/>
-      <c r="Y19" s="41"/>
-      <c r="Z19" s="41"/>
-      <c r="AA19" s="13"/>
-      <c r="AB19" s="61"/>
+      <c r="Z19" s="62"/>
+      <c r="AA19" s="41"/>
+      <c r="AB19" s="41"/>
+      <c r="AC19" s="13"/>
+      <c r="AD19" s="60"/>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
         <v>21</v>
       </c>
@@ -2706,7 +2819,8 @@
         <v>16</v>
       </c>
       <c r="C20" s="11">
-        <v>17</v>
+        <f>(T20-(36*U20))/U20</f>
+        <v>20</v>
       </c>
       <c r="D20" s="52"/>
       <c r="E20" s="53"/>
@@ -2734,31 +2848,33 @@
       </c>
       <c r="P20" s="14"/>
       <c r="Q20" s="12"/>
-      <c r="R20" s="97">
-        <f>F20+J20+L20+N20+P20</f>
+      <c r="R20" s="14"/>
+      <c r="S20" s="12"/>
+      <c r="T20" s="66">
+        <f>F20+J20+L20+N20+P20+R20</f>
         <v>168</v>
       </c>
-      <c r="S20" s="13">
-        <f>COUNTIF(D20:P20,"&gt;30")</f>
+      <c r="U20" s="13">
+        <f>COUNTIF(D20:R20,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="T20" s="40"/>
-      <c r="U20" s="12"/>
-      <c r="V20" s="101">
-        <f>SUMIF(G20:Q20, "&lt;30")+T20+U20</f>
+      <c r="V20" s="40"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="41">
+        <f>SUMIF(G20:S20, "&lt;30")+V20+W20</f>
         <v>45</v>
       </c>
-      <c r="W20" s="61">
-        <f>V20/S20</f>
+      <c r="Y20" s="104">
+        <f>X20/U20</f>
         <v>15</v>
       </c>
-      <c r="X20" s="63"/>
-      <c r="Y20" s="41"/>
-      <c r="Z20" s="41"/>
-      <c r="AA20" s="13"/>
-      <c r="AB20" s="61"/>
+      <c r="Z20" s="62"/>
+      <c r="AA20" s="41"/>
+      <c r="AB20" s="41"/>
+      <c r="AC20" s="13"/>
+      <c r="AD20" s="60"/>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
         <v>49</v>
       </c>
@@ -2784,33 +2900,35 @@
       <c r="O21" s="12"/>
       <c r="P21" s="49"/>
       <c r="Q21" s="12"/>
-      <c r="R21" s="97">
-        <f>F21+J21+L21+N21+P21</f>
+      <c r="R21" s="49"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="66">
+        <f>F21+J21+L21+N21+P21+R21</f>
         <v>50</v>
       </c>
-      <c r="S21" s="13">
-        <f>COUNTIF(D21:P21,"&gt;30")</f>
+      <c r="U21" s="13">
+        <f>COUNTIF(D21:R21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="T21" s="40">
+      <c r="V21" s="40">
         <v>1</v>
       </c>
-      <c r="U21" s="12"/>
-      <c r="V21" s="101">
-        <f>SUMIF(G21:Q21, "&lt;30")+T21+U21</f>
+      <c r="W21" s="12"/>
+      <c r="X21" s="41">
+        <f>SUMIF(G21:S21, "&lt;30")+V21+W21</f>
         <v>1</v>
       </c>
-      <c r="W21" s="61">
-        <f>V21/S21</f>
+      <c r="Y21" s="104">
+        <f>X21/U21</f>
         <v>1</v>
       </c>
-      <c r="X21" s="60"/>
-      <c r="Y21" s="41"/>
-      <c r="Z21" s="41"/>
-      <c r="AA21" s="13"/>
-      <c r="AB21" s="61"/>
+      <c r="Z21" s="59"/>
+      <c r="AA21" s="41"/>
+      <c r="AB21" s="41"/>
+      <c r="AC21" s="13"/>
+      <c r="AD21" s="60"/>
     </row>
-    <row r="22" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
         <v>56</v>
       </c>
@@ -2822,47 +2940,49 @@
       </c>
       <c r="D22" s="54"/>
       <c r="E22" s="55"/>
-      <c r="F22" s="104"/>
+      <c r="F22" s="69"/>
       <c r="G22" s="21"/>
       <c r="H22" s="54"/>
       <c r="I22" s="55"/>
-      <c r="J22" s="104"/>
+      <c r="J22" s="69"/>
       <c r="K22" s="21"/>
-      <c r="L22" s="104"/>
+      <c r="L22" s="69"/>
       <c r="M22" s="21"/>
-      <c r="N22" s="107">
+      <c r="N22" s="71">
         <v>45</v>
       </c>
       <c r="O22" s="21"/>
-      <c r="P22" s="107">
+      <c r="P22" s="71">
         <v>43</v>
       </c>
       <c r="Q22" s="21"/>
-      <c r="R22" s="98">
-        <f>F22+J22+L22+N22+P22</f>
+      <c r="R22" s="71"/>
+      <c r="S22" s="21"/>
+      <c r="T22" s="67">
+        <f>F22+J22+L22+N22+P22+R22</f>
         <v>88</v>
       </c>
-      <c r="S22" s="22">
-        <f>COUNTIF(D22:P22,"&gt;30")</f>
+      <c r="U22" s="22">
+        <f>COUNTIF(D22:R22,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="T22" s="44"/>
-      <c r="U22" s="21"/>
-      <c r="V22" s="102">
-        <f>SUMIF(G22:Q22, "&lt;30")+T22+U22</f>
+      <c r="V22" s="44"/>
+      <c r="W22" s="21"/>
+      <c r="X22" s="45">
+        <f>SUMIF(G22:S22, "&lt;30")+V22+W22</f>
         <v>0</v>
       </c>
-      <c r="W22" s="65">
-        <f>V22/S22</f>
+      <c r="Y22" s="105">
+        <f>X22/U22</f>
         <v>0</v>
       </c>
-      <c r="X22" s="64"/>
-      <c r="Y22" s="45"/>
-      <c r="Z22" s="45"/>
-      <c r="AA22" s="22"/>
-      <c r="AB22" s="65"/>
+      <c r="Z22" s="63"/>
+      <c r="AA22" s="45"/>
+      <c r="AB22" s="45"/>
+      <c r="AC22" s="22"/>
+      <c r="AD22" s="64"/>
     </row>
-    <row r="23" spans="1:28" s="23" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" s="23" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="34"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -2895,18 +3015,23 @@
         <v>46.785714285714285</v>
       </c>
       <c r="Q23" s="36"/>
-      <c r="R23" s="37"/>
+      <c r="R23" s="36">
+        <f>AVERAGEIF(R4:R22,"&gt;0")</f>
+        <v>48.272727272727273</v>
+      </c>
+      <c r="S23" s="36"/>
+      <c r="T23" s="37"/>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
       <c r="C24" s="24"/>
-      <c r="R24" s="25"/>
-      <c r="S24" s="25"/>
-      <c r="T24" s="26"/>
-      <c r="U24" s="26"/>
-      <c r="V24" s="25"/>
-      <c r="W24" s="27"/>
+      <c r="T24" s="25"/>
+      <c r="U24" s="25"/>
+      <c r="V24" s="26"/>
+      <c r="W24" s="26"/>
+      <c r="X24" s="25"/>
+      <c r="Y24" s="27"/>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
       <c r="C25" s="46" t="s">
         <v>42</v>
       </c>
@@ -2919,8 +3044,9 @@
       <c r="L25" s="28"/>
       <c r="N25" s="28"/>
       <c r="P25" s="28"/>
+      <c r="R25" s="28"/>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
       <c r="C26" s="47" t="s">
         <v>43</v>
       </c>
@@ -2933,9 +3059,10 @@
       <c r="L26" s="29"/>
       <c r="N26" s="29"/>
       <c r="P26" s="29"/>
-      <c r="R26" s="30"/>
+      <c r="R26" s="29"/>
+      <c r="T26" s="30"/>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
       <c r="C27" s="48" t="s">
         <v>47</v>
       </c>
@@ -2955,42 +3082,46 @@
       <c r="O27" s="32"/>
       <c r="P27" s="31"/>
       <c r="Q27" s="32"/>
+      <c r="R27" s="31"/>
+      <c r="S27" s="32"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AB22">
-    <sortCondition descending="1" ref="W4:W22"/>
-    <sortCondition descending="1" ref="R4:R22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AD22">
+    <sortCondition descending="1" ref="Y4:Y22"/>
+    <sortCondition descending="1" ref="T4:T22"/>
   </sortState>
-  <mergeCells count="29">
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="X1:AB1"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="S2:S3"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="R1:R3"/>
-    <mergeCell ref="S1:W1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
+  <mergeCells count="31">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="T1:T3"/>
+    <mergeCell ref="U1:Y1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="Z1:AD1"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
070325 - updated scores and skins from 6/30.  cleared tee times table
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC0AC718-2FCF-9B46-BFF4-9C25FF493A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC66D5BD-DA05-4449-B3BD-0984F6BD15D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44380" yWindow="1480" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="63">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -223,13 +223,16 @@
   </si>
   <si>
     <t>WEEK 8</t>
+  </si>
+  <si>
+    <t>WEEK 9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -349,6 +352,11 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -926,7 +934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1124,11 +1132,95 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1145,95 +1237,20 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1569,158 +1586,166 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AD27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AF27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
     <col min="2" max="2" width="8.1640625" customWidth="1"/>
     <col min="3" max="3" width="10.1640625" customWidth="1"/>
     <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="13" width="6.33203125" hidden="1" customWidth="1"/>
-    <col min="14" max="19" width="6.33203125" customWidth="1"/>
-    <col min="20" max="20" width="6.83203125" customWidth="1"/>
-    <col min="21" max="21" width="6.1640625" customWidth="1"/>
-    <col min="22" max="22" width="5.83203125" customWidth="1"/>
-    <col min="23" max="23" width="5.6640625" customWidth="1"/>
-    <col min="24" max="24" width="5.5" customWidth="1"/>
-    <col min="25" max="25" width="8" customWidth="1"/>
-    <col min="26" max="26" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="27" max="28" width="6" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="15" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="16" max="21" width="6.33203125" customWidth="1"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1"/>
+    <col min="23" max="23" width="6.1640625" customWidth="1"/>
+    <col min="24" max="24" width="5.83203125" customWidth="1"/>
+    <col min="25" max="25" width="5.6640625" customWidth="1"/>
+    <col min="26" max="26" width="5.5" customWidth="1"/>
+    <col min="27" max="27" width="8" customWidth="1"/>
+    <col min="28" max="28" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="29" max="30" width="6" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="57" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="95" t="s">
+    <row r="1" spans="1:32" s="57" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="101" t="s">
+      <c r="B1" s="79"/>
+      <c r="C1" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="80" t="s">
+      <c r="D1" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="81"/>
-      <c r="F1" s="80" t="s">
+      <c r="E1" s="87"/>
+      <c r="F1" s="86" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="81"/>
-      <c r="H1" s="80" t="s">
+      <c r="G1" s="87"/>
+      <c r="H1" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="81"/>
-      <c r="J1" s="80" t="s">
+      <c r="I1" s="87"/>
+      <c r="J1" s="86" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="81"/>
-      <c r="L1" s="80" t="s">
+      <c r="K1" s="87"/>
+      <c r="L1" s="86" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="81"/>
-      <c r="N1" s="80" t="s">
+      <c r="M1" s="87"/>
+      <c r="N1" s="86" t="s">
         <v>55</v>
       </c>
-      <c r="O1" s="81"/>
-      <c r="P1" s="80" t="s">
+      <c r="O1" s="87"/>
+      <c r="P1" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="81"/>
-      <c r="R1" s="80" t="s">
+      <c r="Q1" s="87"/>
+      <c r="R1" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="81"/>
-      <c r="T1" s="90" t="s">
+      <c r="S1" s="87"/>
+      <c r="T1" s="86" t="s">
+        <v>62</v>
+      </c>
+      <c r="U1" s="87"/>
+      <c r="V1" s="98" t="s">
         <v>2</v>
       </c>
-      <c r="U1" s="92" t="s">
+      <c r="W1" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="V1" s="93"/>
-      <c r="W1" s="93"/>
-      <c r="X1" s="93"/>
-      <c r="Y1" s="94"/>
-      <c r="Z1" s="75" t="s">
+      <c r="X1" s="101"/>
+      <c r="Y1" s="101"/>
+      <c r="Z1" s="101"/>
+      <c r="AA1" s="102"/>
+      <c r="AB1" s="103" t="s">
         <v>58</v>
       </c>
-      <c r="AA1" s="76"/>
-      <c r="AB1" s="76"/>
-      <c r="AC1" s="76"/>
-      <c r="AD1" s="77"/>
+      <c r="AC1" s="104"/>
+      <c r="AD1" s="104"/>
+      <c r="AE1" s="104"/>
+      <c r="AF1" s="105"/>
     </row>
-    <row r="2" spans="1:30" s="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="97"/>
-      <c r="B2" s="98"/>
-      <c r="C2" s="102"/>
-      <c r="D2" s="73">
+    <row r="2" spans="1:32" s="57" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="80"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="88">
         <v>45782</v>
       </c>
-      <c r="E2" s="74"/>
-      <c r="F2" s="73">
+      <c r="E2" s="89"/>
+      <c r="F2" s="88">
         <v>45789</v>
       </c>
-      <c r="G2" s="74"/>
-      <c r="H2" s="73">
+      <c r="G2" s="89"/>
+      <c r="H2" s="88">
         <v>45796</v>
       </c>
-      <c r="I2" s="74"/>
-      <c r="J2" s="73">
+      <c r="I2" s="89"/>
+      <c r="J2" s="88">
         <v>45803</v>
       </c>
-      <c r="K2" s="74"/>
-      <c r="L2" s="73">
+      <c r="K2" s="89"/>
+      <c r="L2" s="88">
         <v>45810</v>
       </c>
-      <c r="M2" s="74"/>
-      <c r="N2" s="73">
+      <c r="M2" s="89"/>
+      <c r="N2" s="88">
         <v>45817</v>
       </c>
-      <c r="O2" s="74"/>
-      <c r="P2" s="73">
+      <c r="O2" s="89"/>
+      <c r="P2" s="88">
         <v>45824</v>
       </c>
-      <c r="Q2" s="74"/>
-      <c r="R2" s="73">
+      <c r="Q2" s="89"/>
+      <c r="R2" s="88">
         <v>45831</v>
       </c>
-      <c r="S2" s="74"/>
-      <c r="T2" s="91"/>
-      <c r="U2" s="90" t="s">
+      <c r="S2" s="89"/>
+      <c r="T2" s="88">
+        <v>45838</v>
+      </c>
+      <c r="U2" s="89"/>
+      <c r="V2" s="99"/>
+      <c r="W2" s="98" t="s">
         <v>4</v>
       </c>
-      <c r="V2" s="86" t="s">
+      <c r="X2" s="94" t="s">
         <v>5</v>
       </c>
-      <c r="W2" s="88" t="s">
+      <c r="Y2" s="96" t="s">
         <v>6</v>
       </c>
-      <c r="X2" s="82" t="s">
+      <c r="Z2" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="Y2" s="84" t="s">
+      <c r="AA2" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="Z2" s="78" t="s">
+      <c r="AB2" s="106" t="s">
         <v>4</v>
       </c>
-      <c r="AA2" s="78" t="s">
+      <c r="AC2" s="106" t="s">
         <v>5</v>
       </c>
-      <c r="AB2" s="78" t="s">
+      <c r="AD2" s="106" t="s">
         <v>6</v>
       </c>
-      <c r="AC2" s="78" t="s">
+      <c r="AE2" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="AD2" s="78" t="s">
+      <c r="AF2" s="106" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="57" customFormat="1" ht="29" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="99"/>
-      <c r="B3" s="100"/>
-      <c r="C3" s="102"/>
+    <row r="3" spans="1:32" s="57" customFormat="1" ht="29" customHeight="1" thickBot="1">
+      <c r="A3" s="82"/>
+      <c r="B3" s="83"/>
+      <c r="C3" s="85"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1769,19 +1794,25 @@
       <c r="S3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="T3" s="91"/>
-      <c r="U3" s="91"/>
-      <c r="V3" s="87"/>
-      <c r="W3" s="89"/>
-      <c r="X3" s="83"/>
-      <c r="Y3" s="85"/>
-      <c r="Z3" s="79"/>
-      <c r="AA3" s="79"/>
-      <c r="AB3" s="79"/>
-      <c r="AC3" s="79"/>
-      <c r="AD3" s="79"/>
+      <c r="T3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="95"/>
+      <c r="Y3" s="97"/>
+      <c r="Z3" s="91"/>
+      <c r="AA3" s="93"/>
+      <c r="AB3" s="107"/>
+      <c r="AC3" s="107"/>
+      <c r="AD3" s="107"/>
+      <c r="AE3" s="107"/>
+      <c r="AF3" s="107"/>
     </row>
-    <row r="4" spans="1:30" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:32" ht="16" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
@@ -1809,41 +1840,43 @@
       <c r="Q4" s="7">
         <v>26</v>
       </c>
-      <c r="R4" s="106">
+      <c r="R4" s="76">
         <v>45</v>
       </c>
       <c r="S4" s="7">
         <v>24</v>
       </c>
-      <c r="T4" s="65">
-        <f>F4+J4+L4+N4+P4+R4</f>
+      <c r="T4" s="108"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="65">
+        <f>F4+J4+L4+N4+P4+R4+T4</f>
         <v>88</v>
       </c>
-      <c r="U4" s="8">
-        <f>COUNTIF(D4:R4,"&gt;30")</f>
+      <c r="W4" s="8">
+        <f>COUNTIF(D4:T4,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="V4" s="38">
+      <c r="X4" s="38">
         <v>1</v>
       </c>
-      <c r="W4" s="7">
+      <c r="Y4" s="7">
         <v>1</v>
       </c>
-      <c r="X4" s="39">
-        <f>SUMIF(G4:S4, "&lt;30")+V4+W4</f>
+      <c r="Z4" s="39">
+        <f>SUMIF(G4:U4, "&lt;30")+X4+Y4</f>
         <v>52</v>
       </c>
-      <c r="Y4" s="103">
-        <f>X4/U4</f>
+      <c r="AA4" s="73">
+        <f>Z4/W4</f>
         <v>26</v>
       </c>
-      <c r="Z4" s="72"/>
-      <c r="AA4" s="39"/>
-      <c r="AB4" s="39"/>
-      <c r="AC4" s="8"/>
-      <c r="AD4" s="58"/>
+      <c r="AB4" s="72"/>
+      <c r="AC4" s="39"/>
+      <c r="AD4" s="39"/>
+      <c r="AE4" s="8"/>
+      <c r="AF4" s="58"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:32">
       <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
@@ -1851,8 +1884,8 @@
         <v>16</v>
       </c>
       <c r="C5" s="11">
-        <f>(T5-(36*U5))/U5</f>
-        <v>17.333333333333332</v>
+        <f>ROUND((V5-(36*W5))/W5,0)</f>
+        <v>18</v>
       </c>
       <c r="D5" s="52"/>
       <c r="E5" s="53"/>
@@ -1882,319 +1915,349 @@
       <c r="S5" s="12">
         <v>26</v>
       </c>
-      <c r="T5" s="66">
-        <f>F5+J5+L5+N5+P5+R5</f>
-        <v>160</v>
-      </c>
-      <c r="U5" s="13">
-        <f>COUNTIF(D5:R5,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="V5" s="40"/>
-      <c r="W5" s="12"/>
-      <c r="X5" s="41">
-        <f>SUMIF(G5:S5, "&lt;30")+V5+W5</f>
-        <v>68</v>
-      </c>
-      <c r="Y5" s="104">
-        <f>X5/U5</f>
-        <v>22.666666666666668</v>
-      </c>
-      <c r="Z5" s="59"/>
-      <c r="AA5" s="41"/>
-      <c r="AB5" s="41"/>
-      <c r="AC5" s="13"/>
-      <c r="AD5" s="60" t="s">
+      <c r="T5" s="14">
+        <v>56</v>
+      </c>
+      <c r="U5" s="12">
+        <v>15</v>
+      </c>
+      <c r="V5" s="66">
+        <f>F5+J5+L5+N5+P5+R5+T5</f>
+        <v>216</v>
+      </c>
+      <c r="W5" s="13">
+        <f>COUNTIF(D5:T5,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="X5" s="40"/>
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="41">
+        <f>SUMIF(G5:U5, "&lt;30")+X5+Y5</f>
+        <v>83</v>
+      </c>
+      <c r="AA5" s="74">
+        <f>Z5/W5</f>
+        <v>20.75</v>
+      </c>
+      <c r="AB5" s="59"/>
+      <c r="AC5" s="41"/>
+      <c r="AD5" s="41"/>
+      <c r="AE5" s="13"/>
+      <c r="AF5" s="60" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:32">
       <c r="A6" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="11">
+        <f>ROUND((V6-(36*W6))/W6,0)</f>
         <v>13</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="11">
-        <f>(T6-(36*U6))/U6</f>
-        <v>11</v>
       </c>
       <c r="D6" s="52"/>
       <c r="E6" s="53"/>
-      <c r="F6" s="107">
-        <v>42</v>
-      </c>
-      <c r="G6" s="12">
-        <v>25</v>
-      </c>
+      <c r="F6" s="14"/>
+      <c r="G6" s="12"/>
       <c r="H6" s="52"/>
       <c r="I6" s="53"/>
-      <c r="J6" s="107"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="42">
-        <v>51</v>
-      </c>
-      <c r="M6" s="12">
+      <c r="J6" s="14">
+        <v>52</v>
+      </c>
+      <c r="K6" s="12">
+        <v>17</v>
+      </c>
+      <c r="L6" s="14"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="14">
+        <v>46</v>
+      </c>
+      <c r="O6" s="12">
+        <v>23</v>
+      </c>
+      <c r="P6" s="14">
+        <v>46</v>
+      </c>
+      <c r="Q6" s="12">
+        <v>23</v>
+      </c>
+      <c r="R6" s="14">
+        <v>54</v>
+      </c>
+      <c r="S6" s="12">
         <v>16</v>
       </c>
-      <c r="N6" s="42"/>
-      <c r="O6" s="12"/>
-      <c r="P6" s="15">
-        <v>49</v>
-      </c>
-      <c r="Q6" s="12">
-        <v>18</v>
-      </c>
-      <c r="R6" s="42">
-        <v>46</v>
-      </c>
-      <c r="S6" s="12">
-        <v>21</v>
-      </c>
-      <c r="T6" s="66">
-        <f>F6+J6+L6+N6+P6+R6</f>
-        <v>188</v>
-      </c>
-      <c r="U6" s="13">
-        <f>COUNTIF(D6:R6,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="V6" s="40">
-        <v>2</v>
-      </c>
-      <c r="W6" s="12"/>
-      <c r="X6" s="41">
-        <f>SUMIF(G6:S6, "&lt;30")+V6+W6</f>
-        <v>82</v>
-      </c>
-      <c r="Y6" s="104">
-        <f>X6/U6</f>
-        <v>20.5</v>
-      </c>
-      <c r="Z6" s="59"/>
-      <c r="AA6" s="41"/>
-      <c r="AB6" s="41"/>
-      <c r="AC6" s="13"/>
-      <c r="AD6" s="60"/>
+      <c r="T6" s="14">
+        <v>45</v>
+      </c>
+      <c r="U6" s="12">
+        <v>23</v>
+      </c>
+      <c r="V6" s="66">
+        <f>F6+J6+L6+N6+P6+R6+T6</f>
+        <v>243</v>
+      </c>
+      <c r="W6" s="13">
+        <f>COUNTIF(D6:T6,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="X6" s="40"/>
+      <c r="Y6" s="12"/>
+      <c r="Z6" s="41">
+        <f>SUMIF(G6:U6, "&lt;30")+X6+Y6</f>
+        <v>102</v>
+      </c>
+      <c r="AA6" s="74">
+        <f>Z6/W6</f>
+        <v>20.399999999999999</v>
+      </c>
+      <c r="AB6" s="59"/>
+      <c r="AC6" s="41"/>
+      <c r="AD6" s="41"/>
+      <c r="AE6" s="13"/>
+      <c r="AF6" s="60"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:32">
       <c r="A7" s="9" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="C7" s="11">
-        <f>(T7-(36*U7))/U7</f>
-        <v>13.5</v>
+        <f>ROUND((V7-(36*W7))/W7,0)</f>
+        <v>11</v>
       </c>
       <c r="D7" s="52"/>
       <c r="E7" s="53"/>
-      <c r="F7" s="108"/>
-      <c r="G7" s="12"/>
+      <c r="F7" s="110">
+        <v>42</v>
+      </c>
+      <c r="G7" s="12">
+        <v>25</v>
+      </c>
       <c r="H7" s="52"/>
       <c r="I7" s="53"/>
-      <c r="J7" s="108">
-        <v>52</v>
-      </c>
-      <c r="K7" s="12">
-        <v>17</v>
-      </c>
-      <c r="L7" s="108"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="108">
+      <c r="J7" s="110"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="111">
+        <v>51</v>
+      </c>
+      <c r="M7" s="12">
+        <v>16</v>
+      </c>
+      <c r="N7" s="111"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="112">
+        <v>49</v>
+      </c>
+      <c r="Q7" s="12">
+        <v>18</v>
+      </c>
+      <c r="R7" s="111">
         <v>46</v>
       </c>
-      <c r="O7" s="12">
-        <v>23</v>
-      </c>
-      <c r="P7" s="108">
-        <v>46</v>
-      </c>
-      <c r="Q7" s="12">
-        <v>23</v>
-      </c>
-      <c r="R7" s="108">
-        <v>54</v>
-      </c>
       <c r="S7" s="12">
-        <v>16</v>
-      </c>
-      <c r="T7" s="66">
-        <f>F7+J7+L7+N7+P7+R7</f>
-        <v>198</v>
-      </c>
-      <c r="U7" s="13">
-        <f>COUNTIF(D7:R7,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="V7" s="40"/>
-      <c r="W7" s="12"/>
-      <c r="X7" s="41">
-        <f>SUMIF(G7:S7, "&lt;30")+V7+W7</f>
-        <v>79</v>
-      </c>
-      <c r="Y7" s="104">
-        <f>X7/U7</f>
-        <v>19.75</v>
-      </c>
-      <c r="Z7" s="59"/>
-      <c r="AA7" s="41"/>
-      <c r="AB7" s="41"/>
-      <c r="AC7" s="13"/>
-      <c r="AD7" s="60"/>
+        <v>21</v>
+      </c>
+      <c r="T7" s="111">
+        <v>45</v>
+      </c>
+      <c r="U7" s="12">
+        <v>20</v>
+      </c>
+      <c r="V7" s="66">
+        <f>F7+J7+L7+N7+P7+R7+T7</f>
+        <v>233</v>
+      </c>
+      <c r="W7" s="13">
+        <f>COUNTIF(D7:T7,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="X7" s="40">
+        <v>2</v>
+      </c>
+      <c r="Y7" s="12"/>
+      <c r="Z7" s="41">
+        <f>SUMIF(G7:U7, "&lt;30")+X7+Y7</f>
+        <v>102</v>
+      </c>
+      <c r="AA7" s="74">
+        <f>Z7/W7</f>
+        <v>20.399999999999999</v>
+      </c>
+      <c r="AB7" s="59"/>
+      <c r="AC7" s="41"/>
+      <c r="AD7" s="41"/>
+      <c r="AE7" s="13"/>
+      <c r="AF7" s="60"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:32">
       <c r="A8" s="9" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C8" s="11">
-        <f>(T8-(36*U8))/U8</f>
-        <v>7.6</v>
+        <f>ROUND((V8-(36*W8))/W8,0)</f>
+        <v>12</v>
       </c>
       <c r="D8" s="52"/>
       <c r="E8" s="53"/>
-      <c r="F8" s="70">
-        <v>45</v>
-      </c>
-      <c r="G8" s="12">
-        <v>17</v>
-      </c>
+      <c r="F8" s="16"/>
+      <c r="G8" s="12"/>
       <c r="H8" s="52"/>
       <c r="I8" s="53"/>
-      <c r="J8" s="70"/>
+      <c r="J8" s="16"/>
       <c r="K8" s="12"/>
-      <c r="L8" s="70">
-        <v>43</v>
-      </c>
-      <c r="M8" s="12">
-        <v>19</v>
-      </c>
-      <c r="N8" s="15">
-        <v>41</v>
-      </c>
-      <c r="O8" s="12">
-        <v>21</v>
-      </c>
+      <c r="L8" s="16"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="12"/>
       <c r="P8" s="42">
         <v>47</v>
       </c>
       <c r="Q8" s="12">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R8" s="42">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="S8" s="12">
-        <v>20</v>
-      </c>
-      <c r="T8" s="66">
-        <f>F8+J8+L8+N8+P8+R8</f>
-        <v>218</v>
-      </c>
-      <c r="U8" s="13">
-        <f>COUNTIF(D8:R8,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="V8" s="40">
-        <v>1</v>
-      </c>
-      <c r="W8" s="12">
+        <v>17</v>
+      </c>
+      <c r="T8" s="42">
+        <v>46</v>
+      </c>
+      <c r="U8" s="12">
+        <v>21</v>
+      </c>
+      <c r="V8" s="66">
+        <f>F8+J8+L8+N8+P8+R8+T8</f>
+        <v>143</v>
+      </c>
+      <c r="W8" s="13">
+        <f>COUNTIF(D8:T8,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="X8" s="41">
-        <f>SUMIF(G8:S8, "&lt;30")+V8+W8</f>
-        <v>96</v>
-      </c>
-      <c r="Y8" s="104">
-        <f>X8/U8</f>
-        <v>19.2</v>
-      </c>
-      <c r="Z8" s="61"/>
-      <c r="AA8" s="41"/>
-      <c r="AB8" s="41"/>
-      <c r="AC8" s="13"/>
-      <c r="AD8" s="60"/>
+      <c r="X8" s="40"/>
+      <c r="Y8" s="12"/>
+      <c r="Z8" s="41">
+        <f>SUMIF(G8:U8, "&lt;30")+X8+Y8</f>
+        <v>58</v>
+      </c>
+      <c r="AA8" s="74">
+        <f>Z8/W8</f>
+        <v>19.333333333333332</v>
+      </c>
+      <c r="AB8" s="61"/>
+      <c r="AC8" s="41"/>
+      <c r="AD8" s="41"/>
+      <c r="AE8" s="13"/>
+      <c r="AF8" s="60"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:32">
       <c r="A9" s="9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C9" s="11">
-        <v>22</v>
+        <f>ROUND((V9-(36*W9))/W9,0)</f>
+        <v>8</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="53"/>
-      <c r="F9" s="14">
-        <v>59</v>
+      <c r="F9" s="70">
+        <v>45</v>
       </c>
       <c r="G9" s="12">
         <v>17</v>
       </c>
       <c r="H9" s="52"/>
       <c r="I9" s="53"/>
-      <c r="J9" s="14"/>
+      <c r="J9" s="70"/>
       <c r="K9" s="12"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="14">
-        <v>55</v>
+      <c r="L9" s="70">
+        <v>43</v>
+      </c>
+      <c r="M9" s="12">
+        <v>19</v>
+      </c>
+      <c r="N9" s="15">
+        <v>41</v>
+      </c>
+      <c r="O9" s="12">
+        <v>21</v>
+      </c>
+      <c r="P9" s="42">
+        <v>47</v>
+      </c>
+      <c r="Q9" s="12">
+        <v>15</v>
+      </c>
+      <c r="R9" s="42">
+        <v>42</v>
       </c>
       <c r="S9" s="12">
-        <v>21</v>
-      </c>
-      <c r="T9" s="66">
-        <f>F9+J9+L9+N9+P9+R9</f>
-        <v>114</v>
-      </c>
-      <c r="U9" s="13">
-        <f>COUNTIF(D9:R9,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="V9" s="40"/>
-      <c r="W9" s="12"/>
-      <c r="X9" s="41">
-        <f>SUMIF(G9:S9, "&lt;30")+V9+W9</f>
-        <v>38</v>
-      </c>
-      <c r="Y9" s="104">
-        <f>X9/U9</f>
+        <v>20</v>
+      </c>
+      <c r="T9" s="42">
+        <v>43</v>
+      </c>
+      <c r="U9" s="12">
         <v>19</v>
       </c>
-      <c r="Z9" s="62"/>
-      <c r="AA9" s="41"/>
-      <c r="AB9" s="41"/>
-      <c r="AC9" s="13"/>
-      <c r="AD9" s="60"/>
+      <c r="V9" s="66">
+        <f>F9+J9+L9+N9+P9+R9+T9</f>
+        <v>261</v>
+      </c>
+      <c r="W9" s="13">
+        <f>COUNTIF(D9:T9,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="X9" s="40">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="12">
+        <v>3</v>
+      </c>
+      <c r="Z9" s="41">
+        <f>SUMIF(G9:U9, "&lt;30")+X9+Y9</f>
+        <v>115</v>
+      </c>
+      <c r="AA9" s="74">
+        <f>Z9/W9</f>
+        <v>19.166666666666668</v>
+      </c>
+      <c r="AB9" s="59"/>
+      <c r="AC9" s="41"/>
+      <c r="AD9" s="41"/>
+      <c r="AE9" s="13"/>
+      <c r="AF9" s="60"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:32">
       <c r="A10" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C10" s="11">
-        <f>(T10-(36*U10))/U10</f>
-        <v>7.666666666666667</v>
+        <v>22</v>
       </c>
       <c r="D10" s="52"/>
       <c r="E10" s="53"/>
       <c r="F10" s="14">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="G10" s="12">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H10" s="52"/>
       <c r="I10" s="53"/>
@@ -2202,172 +2265,179 @@
       <c r="K10" s="12"/>
       <c r="L10" s="14"/>
       <c r="M10" s="12"/>
-      <c r="N10" s="14">
-        <v>42</v>
-      </c>
-      <c r="O10" s="12">
+      <c r="N10" s="14"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="14">
+        <v>55</v>
+      </c>
+      <c r="S10" s="12">
+        <v>21</v>
+      </c>
+      <c r="T10" s="14"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="66">
+        <f>F10+J10+L10+N10+P10+R10+T10</f>
+        <v>114</v>
+      </c>
+      <c r="W10" s="13">
+        <f>COUNTIF(D10:T10,"&gt;30")</f>
+        <v>2</v>
+      </c>
+      <c r="X10" s="40"/>
+      <c r="Y10" s="12"/>
+      <c r="Z10" s="41">
+        <f>SUMIF(G10:U10, "&lt;30")+X10+Y10</f>
+        <v>38</v>
+      </c>
+      <c r="AA10" s="74">
+        <f>Z10/W10</f>
+        <v>19</v>
+      </c>
+      <c r="AB10" s="77"/>
+      <c r="AC10" s="41"/>
+      <c r="AD10" s="41"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="60"/>
+    </row>
+    <row r="11" spans="1:32">
+      <c r="A11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="P10" s="14">
-        <v>43</v>
-      </c>
-      <c r="Q10" s="12">
-        <v>19</v>
-      </c>
-      <c r="R10" s="14"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="66">
-        <f>F10+J10+L10+N10+P10+R10</f>
-        <v>131</v>
-      </c>
-      <c r="U10" s="13">
-        <f>COUNTIF(D10:R10,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="V10" s="40"/>
-      <c r="W10" s="12">
-        <v>1</v>
-      </c>
-      <c r="X10" s="41">
-        <f>SUMIF(G10:S10, "&lt;30")+V10+W10</f>
-        <v>56</v>
-      </c>
-      <c r="Y10" s="104">
-        <f>X10/U10</f>
-        <v>18.666666666666668</v>
-      </c>
-      <c r="Z10" s="109"/>
-      <c r="AA10" s="41"/>
-      <c r="AB10" s="41"/>
-      <c r="AC10" s="13"/>
-      <c r="AD10" s="60"/>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A11" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>12</v>
-      </c>
       <c r="C11" s="11">
-        <f>(T11-(36*U11))/U11</f>
-        <v>14.75</v>
+        <f>ROUND((V11-(36*W11))/W11,0)</f>
+        <v>8</v>
       </c>
       <c r="D11" s="52"/>
       <c r="E11" s="53"/>
       <c r="F11" s="14">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G11" s="12">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H11" s="52"/>
       <c r="I11" s="53"/>
       <c r="J11" s="14"/>
       <c r="K11" s="12"/>
-      <c r="L11" s="14">
-        <v>54</v>
-      </c>
-      <c r="M11" s="12">
+      <c r="L11" s="14"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="14">
+        <v>42</v>
+      </c>
+      <c r="O11" s="12">
+        <v>20</v>
+      </c>
+      <c r="P11" s="14">
+        <v>43</v>
+      </c>
+      <c r="Q11" s="12">
+        <v>19</v>
+      </c>
+      <c r="R11" s="14"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="12"/>
+      <c r="V11" s="66">
+        <f>F11+J11+L11+N11+P11+R11+T11</f>
+        <v>131</v>
+      </c>
+      <c r="W11" s="13">
+        <f>COUNTIF(D11:T11,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="X11" s="40"/>
+      <c r="Y11" s="12">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="41">
+        <f>SUMIF(G11:U11, "&lt;30")+X11+Y11</f>
+        <v>56</v>
+      </c>
+      <c r="AA11" s="74">
+        <f>Z11/W11</f>
+        <v>18.666666666666668</v>
+      </c>
+      <c r="AB11" s="62"/>
+      <c r="AC11" s="41"/>
+      <c r="AD11" s="41"/>
+      <c r="AE11" s="13"/>
+      <c r="AF11" s="60"/>
+    </row>
+    <row r="12" spans="1:32">
+      <c r="A12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="11">
+        <f>ROUND((V12-(36*W12))/W12,0)</f>
         <v>15</v>
-      </c>
-      <c r="N11" s="14"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="14">
-        <v>54</v>
-      </c>
-      <c r="Q11" s="12">
-        <v>16</v>
-      </c>
-      <c r="R11" s="14">
-        <v>53</v>
-      </c>
-      <c r="S11" s="12">
-        <v>16</v>
-      </c>
-      <c r="T11" s="66">
-        <f>F11+J11+L11+N11+P11+R11</f>
-        <v>203</v>
-      </c>
-      <c r="U11" s="13">
-        <f>COUNTIF(D11:R11,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="V11" s="40"/>
-      <c r="W11" s="12"/>
-      <c r="X11" s="41">
-        <f>SUMIF(G11:S11, "&lt;30")+V11+W11</f>
-        <v>74</v>
-      </c>
-      <c r="Y11" s="104">
-        <f>X11/U11</f>
-        <v>18.5</v>
-      </c>
-      <c r="Z11" s="59"/>
-      <c r="AA11" s="41"/>
-      <c r="AB11" s="41"/>
-      <c r="AC11" s="13"/>
-      <c r="AD11" s="60"/>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="11">
-        <v>13</v>
       </c>
       <c r="D12" s="52"/>
       <c r="E12" s="53"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="12"/>
+      <c r="F12" s="14">
+        <v>42</v>
+      </c>
+      <c r="G12" s="12">
+        <v>27</v>
+      </c>
       <c r="H12" s="52"/>
       <c r="I12" s="53"/>
-      <c r="J12" s="16"/>
+      <c r="J12" s="14"/>
       <c r="K12" s="12"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="16"/>
+      <c r="L12" s="14">
+        <v>54</v>
+      </c>
+      <c r="M12" s="12">
+        <v>15</v>
+      </c>
+      <c r="N12" s="14"/>
       <c r="O12" s="12"/>
-      <c r="P12" s="42">
-        <v>47</v>
+      <c r="P12" s="14">
+        <v>54</v>
       </c>
       <c r="Q12" s="12">
-        <v>20</v>
-      </c>
-      <c r="R12" s="42">
-        <v>50</v>
+        <v>16</v>
+      </c>
+      <c r="R12" s="14">
+        <v>53</v>
       </c>
       <c r="S12" s="12">
-        <v>17</v>
-      </c>
-      <c r="T12" s="66">
-        <f>F12+J12+L12+N12+P12+R12</f>
-        <v>97</v>
-      </c>
-      <c r="U12" s="13">
-        <f>COUNTIF(D12:R12,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="V12" s="40"/>
-      <c r="W12" s="12"/>
-      <c r="X12" s="41">
-        <f>SUMIF(G12:S12, "&lt;30")+V12+W12</f>
-        <v>37</v>
-      </c>
-      <c r="Y12" s="104">
-        <f>X12/U12</f>
+        <v>16</v>
+      </c>
+      <c r="T12" s="14"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="66">
+        <f>F12+J12+L12+N12+P12+R12+T12</f>
+        <v>203</v>
+      </c>
+      <c r="W12" s="13">
+        <f>COUNTIF(D12:T12,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="X12" s="40"/>
+      <c r="Y12" s="12"/>
+      <c r="Z12" s="41">
+        <f>SUMIF(G12:U12, "&lt;30")+X12+Y12</f>
+        <v>74</v>
+      </c>
+      <c r="AA12" s="74">
+        <f>Z12/W12</f>
         <v>18.5</v>
       </c>
-      <c r="Z12" s="59"/>
-      <c r="AA12" s="41"/>
-      <c r="AB12" s="41"/>
-      <c r="AC12" s="13"/>
-      <c r="AD12" s="60"/>
+      <c r="AB12" s="59"/>
+      <c r="AC12" s="41"/>
+      <c r="AD12" s="41"/>
+      <c r="AE12" s="13"/>
+      <c r="AF12" s="60"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:32">
       <c r="A13" s="9" t="s">
         <v>35</v>
       </c>
@@ -2401,123 +2471,119 @@
       <c r="S13" s="12">
         <v>18</v>
       </c>
-      <c r="T13" s="66">
-        <f>F13+J13+L13+N13+P13+R13</f>
+      <c r="T13" s="68"/>
+      <c r="U13" s="12"/>
+      <c r="V13" s="66">
+        <f>F13+J13+L13+N13+P13+R13+T13</f>
         <v>77</v>
       </c>
-      <c r="U13" s="13">
-        <f>COUNTIF(D13:R13,"&gt;30")</f>
+      <c r="W13" s="13">
+        <f>COUNTIF(D13:T13,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="V13" s="40"/>
-      <c r="W13" s="12">
+      <c r="X13" s="40"/>
+      <c r="Y13" s="12">
         <v>2</v>
       </c>
-      <c r="X13" s="41">
-        <f>SUMIF(G13:S13, "&lt;30")+V13+W13</f>
+      <c r="Z13" s="41">
+        <f>SUMIF(G13:U13, "&lt;30")+X13+Y13</f>
         <v>37</v>
       </c>
-      <c r="Y13" s="104">
-        <f>X13/U13</f>
+      <c r="AA13" s="74">
+        <f>Z13/W13</f>
         <v>18.5</v>
       </c>
-      <c r="Z13" s="59"/>
-      <c r="AA13" s="41"/>
-      <c r="AB13" s="41"/>
-      <c r="AC13" s="13"/>
-      <c r="AD13" s="60"/>
+      <c r="AB13" s="59"/>
+      <c r="AC13" s="41"/>
+      <c r="AD13" s="41"/>
+      <c r="AE13" s="13"/>
+      <c r="AF13" s="60"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:32">
       <c r="A14" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" s="11">
-        <f>(T14-(36*U14))/U14</f>
-        <v>21.4</v>
+        <f>ROUND((V14-(36*W14))/W14,0)</f>
+        <v>8</v>
       </c>
       <c r="D14" s="52"/>
       <c r="E14" s="53"/>
-      <c r="F14" s="15">
-        <v>61</v>
+      <c r="F14" s="14">
+        <v>41</v>
       </c>
       <c r="G14" s="12">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H14" s="52"/>
       <c r="I14" s="53"/>
-      <c r="J14" s="15">
-        <v>56</v>
-      </c>
-      <c r="K14" s="12">
-        <v>19</v>
-      </c>
-      <c r="L14" s="42">
-        <v>60</v>
-      </c>
-      <c r="M14" s="12">
-        <v>15</v>
-      </c>
-      <c r="N14" s="42">
-        <v>56</v>
+      <c r="J14" s="14"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="56">
+        <v>48</v>
       </c>
       <c r="O14" s="12">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="P14" s="42">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="Q14" s="12">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="R14" s="42"/>
       <c r="S14" s="12"/>
-      <c r="T14" s="66">
-        <f>F14+J14+L14+N14+P14+R14</f>
-        <v>287</v>
-      </c>
-      <c r="U14" s="13">
-        <f>COUNTIF(D14:R14,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="V14" s="40">
-        <v>2</v>
-      </c>
-      <c r="W14" s="12"/>
-      <c r="X14" s="41">
-        <f>SUMIF(G14:S14, "&lt;30")+V14+W14</f>
-        <v>92</v>
-      </c>
-      <c r="Y14" s="104">
-        <f>X14/U14</f>
-        <v>18.399999999999999</v>
-      </c>
-      <c r="Z14" s="59"/>
-      <c r="AA14" s="41"/>
-      <c r="AB14" s="41"/>
-      <c r="AC14" s="13"/>
-      <c r="AD14" s="60"/>
+      <c r="T14" s="42"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="66">
+        <f>F14+J14+L14+N14+P14+R14+T14</f>
+        <v>133</v>
+      </c>
+      <c r="W14" s="13">
+        <f>COUNTIF(D14:T14,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="X14" s="40">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="41">
+        <f>SUMIF(G14:U14, "&lt;30")+X14+Y14</f>
+        <v>54</v>
+      </c>
+      <c r="AA14" s="74">
+        <f>Z14/W14</f>
+        <v>18</v>
+      </c>
+      <c r="AB14" s="62"/>
+      <c r="AC14" s="41"/>
+      <c r="AD14" s="41"/>
+      <c r="AE14" s="13"/>
+      <c r="AF14" s="60"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:32">
       <c r="A15" s="9" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C15" s="11">
-        <f>(T15-(36*U15))/U15</f>
-        <v>8.3333333333333339</v>
+        <f>ROUND((V15-(36*W15))/W15,0)</f>
+        <v>15</v>
       </c>
       <c r="D15" s="52"/>
       <c r="E15" s="53"/>
       <c r="F15" s="14">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="G15" s="12">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H15" s="52"/>
       <c r="I15" s="53"/>
@@ -2525,239 +2591,274 @@
       <c r="K15" s="12"/>
       <c r="L15" s="14"/>
       <c r="M15" s="12"/>
-      <c r="N15" s="56">
-        <v>48</v>
+      <c r="N15" s="14">
+        <v>51</v>
       </c>
       <c r="O15" s="12">
-        <v>14</v>
-      </c>
-      <c r="P15" s="42">
-        <v>44</v>
+        <v>18</v>
+      </c>
+      <c r="P15" s="14">
+        <v>52</v>
       </c>
       <c r="Q15" s="12">
+        <v>17</v>
+      </c>
+      <c r="R15" s="14"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="12"/>
+      <c r="V15" s="66">
+        <f>F15+J15+L15+N15+P15+R15+T15</f>
+        <v>154</v>
+      </c>
+      <c r="W15" s="13">
+        <f>COUNTIF(D15:T15,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="X15" s="40"/>
+      <c r="Y15" s="12"/>
+      <c r="Z15" s="41">
+        <f>SUMIF(G15:U15, "&lt;30")+X15+Y15</f>
+        <v>53</v>
+      </c>
+      <c r="AA15" s="74">
+        <f>Z15/W15</f>
+        <v>17.666666666666668</v>
+      </c>
+      <c r="AB15" s="62"/>
+      <c r="AC15" s="41"/>
+      <c r="AD15" s="41"/>
+      <c r="AE15" s="13"/>
+      <c r="AF15" s="60"/>
+    </row>
+    <row r="16" spans="1:32">
+      <c r="A16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="11">
+        <f>ROUND((V16-(36*W16))/W16,0)</f>
         <v>18</v>
-      </c>
-      <c r="R15" s="42"/>
-      <c r="S15" s="12"/>
-      <c r="T15" s="66">
-        <f>F15+J15+L15+N15+P15+R15</f>
-        <v>133</v>
-      </c>
-      <c r="U15" s="13">
-        <f>COUNTIF(D15:R15,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="V15" s="40">
-        <v>1</v>
-      </c>
-      <c r="W15" s="12"/>
-      <c r="X15" s="41">
-        <f>SUMIF(G15:S15, "&lt;30")+V15+W15</f>
-        <v>54</v>
-      </c>
-      <c r="Y15" s="104">
-        <f>X15/U15</f>
-        <v>18</v>
-      </c>
-      <c r="Z15" s="62"/>
-      <c r="AA15" s="41"/>
-      <c r="AB15" s="41"/>
-      <c r="AC15" s="13"/>
-      <c r="AD15" s="60"/>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A16" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="11">
-        <f>(T16-(36*U16))/U16</f>
-        <v>15.333333333333334</v>
       </c>
       <c r="D16" s="52"/>
       <c r="E16" s="53"/>
       <c r="F16" s="14">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G16" s="12">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H16" s="52"/>
       <c r="I16" s="53"/>
       <c r="J16" s="14"/>
       <c r="K16" s="12"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="12"/>
+      <c r="L16" s="14">
+        <v>56</v>
+      </c>
+      <c r="M16" s="12">
+        <v>15</v>
+      </c>
       <c r="N16" s="14">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="O16" s="12">
-        <v>18</v>
-      </c>
-      <c r="P16" s="14">
-        <v>52</v>
-      </c>
-      <c r="Q16" s="12">
-        <v>17</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="12"/>
       <c r="R16" s="14"/>
       <c r="S16" s="12"/>
-      <c r="T16" s="66">
-        <f>F16+J16+L16+N16+P16+R16</f>
-        <v>154</v>
-      </c>
-      <c r="U16" s="13">
-        <f>COUNTIF(D16:R16,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="V16" s="40"/>
-      <c r="W16" s="12"/>
-      <c r="X16" s="41">
-        <f>SUMIF(G16:S16, "&lt;30")+V16+W16</f>
-        <v>53</v>
-      </c>
-      <c r="Y16" s="104">
-        <f>X16/U16</f>
-        <v>17.666666666666668</v>
-      </c>
-      <c r="Z16" s="62"/>
-      <c r="AA16" s="41"/>
-      <c r="AB16" s="41"/>
-      <c r="AC16" s="13"/>
-      <c r="AD16" s="60"/>
+      <c r="T16" s="109">
+        <v>49</v>
+      </c>
+      <c r="U16" s="12">
+        <v>22</v>
+      </c>
+      <c r="V16" s="66">
+        <f>F16+J16+L16+N16+P16+R16+T16</f>
+        <v>217</v>
+      </c>
+      <c r="W16" s="13">
+        <f>COUNTIF(D16:T16,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="X16" s="40">
+        <v>1</v>
+      </c>
+      <c r="Y16" s="12"/>
+      <c r="Z16" s="41">
+        <f>SUMIF(G16:U16, "&lt;30")+X16+Y16</f>
+        <v>68</v>
+      </c>
+      <c r="AA16" s="74">
+        <f>Z16/W16</f>
+        <v>17</v>
+      </c>
+      <c r="AB16" s="62"/>
+      <c r="AC16" s="41"/>
+      <c r="AD16" s="41"/>
+      <c r="AE16" s="13"/>
+      <c r="AF16" s="60"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:32">
       <c r="A17" s="9" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C17" s="11">
-        <f>(T17-(36*U17))/U17</f>
-        <v>10.199999999999999</v>
+        <f>ROUND((V17-(36*W17))/W17,0)</f>
+        <v>23</v>
       </c>
       <c r="D17" s="52"/>
       <c r="E17" s="53"/>
-      <c r="F17" s="14">
-        <v>46</v>
+      <c r="F17" s="15">
+        <v>61</v>
       </c>
       <c r="G17" s="12">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H17" s="52"/>
       <c r="I17" s="53"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="14">
-        <v>46</v>
+      <c r="J17" s="15">
+        <v>56</v>
+      </c>
+      <c r="K17" s="12">
+        <v>19</v>
+      </c>
+      <c r="L17" s="42">
+        <v>60</v>
       </c>
       <c r="M17" s="12">
-        <v>18</v>
-      </c>
-      <c r="N17" s="14">
-        <v>46</v>
+        <v>15</v>
+      </c>
+      <c r="N17" s="42">
+        <v>56</v>
       </c>
       <c r="O17" s="12">
-        <v>18</v>
-      </c>
-      <c r="P17" s="14">
-        <v>46</v>
+        <v>20</v>
+      </c>
+      <c r="P17" s="42">
+        <v>54</v>
       </c>
       <c r="Q17" s="12">
-        <v>18</v>
-      </c>
-      <c r="R17" s="14">
-        <v>47</v>
-      </c>
-      <c r="S17" s="12">
-        <v>14</v>
-      </c>
-      <c r="T17" s="66">
-        <f>F17+J17+L17+N17+P17+R17</f>
-        <v>231</v>
-      </c>
-      <c r="U17" s="13">
-        <f>COUNTIF(D17:R17,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="V17" s="43"/>
-      <c r="W17" s="33"/>
-      <c r="X17" s="41">
-        <f>SUMIF(G17:S17, "&lt;30")+V17+W17</f>
-        <v>86</v>
-      </c>
-      <c r="Y17" s="104">
-        <f>X17/U17</f>
-        <v>17.2</v>
-      </c>
-      <c r="Z17" s="62"/>
-      <c r="AA17" s="13"/>
-      <c r="AB17" s="13"/>
-      <c r="AC17" s="13"/>
-      <c r="AD17" s="60"/>
+        <v>22</v>
+      </c>
+      <c r="R17" s="42"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="42">
+        <v>66</v>
+      </c>
+      <c r="U17" s="12">
+        <v>9</v>
+      </c>
+      <c r="V17" s="66">
+        <f>F17+J17+L17+N17+P17+R17+T17</f>
+        <v>353</v>
+      </c>
+      <c r="W17" s="13">
+        <f>COUNTIF(D17:T17,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="X17" s="40">
+        <v>2</v>
+      </c>
+      <c r="Y17" s="12"/>
+      <c r="Z17" s="41">
+        <f>SUMIF(G17:U17, "&lt;30")+X17+Y17</f>
+        <v>101</v>
+      </c>
+      <c r="AA17" s="74">
+        <f>Z17/W17</f>
+        <v>16.833333333333332</v>
+      </c>
+      <c r="AB17" s="59"/>
+      <c r="AC17" s="41"/>
+      <c r="AD17" s="41"/>
+      <c r="AE17" s="13"/>
+      <c r="AF17" s="60"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:32">
       <c r="A18" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C18" s="11">
+        <f>ROUND((V18-(36*W18))/W18,0)</f>
         <v>11</v>
       </c>
       <c r="D18" s="52"/>
       <c r="E18" s="53"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="12"/>
+      <c r="F18" s="14">
+        <v>46</v>
+      </c>
+      <c r="G18" s="12">
+        <v>18</v>
+      </c>
       <c r="H18" s="52"/>
       <c r="I18" s="53"/>
       <c r="J18" s="14"/>
       <c r="K18" s="12"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="12"/>
+      <c r="L18" s="14">
+        <v>46</v>
+      </c>
+      <c r="M18" s="12">
+        <v>18</v>
+      </c>
+      <c r="N18" s="14">
+        <v>46</v>
+      </c>
+      <c r="O18" s="12">
+        <v>18</v>
+      </c>
       <c r="P18" s="14">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="Q18" s="12">
         <v>18</v>
       </c>
       <c r="R18" s="14">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="S18" s="12">
         <v>14</v>
       </c>
-      <c r="T18" s="66">
-        <f>F18+J18+L18+N18+P18+R18</f>
+      <c r="T18" s="14">
+        <v>52</v>
+      </c>
+      <c r="U18" s="12">
+        <v>13</v>
+      </c>
+      <c r="V18" s="66">
+        <f>F18+J18+L18+N18+P18+R18+T18</f>
+        <v>283</v>
+      </c>
+      <c r="W18" s="13">
+        <f>COUNTIF(D18:T18,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="X18" s="43"/>
+      <c r="Y18" s="33"/>
+      <c r="Z18" s="41">
+        <f>SUMIF(G18:U18, "&lt;30")+X18+Y18</f>
         <v>99</v>
       </c>
-      <c r="U18" s="13">
-        <f>COUNTIF(D18:R18,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="V18" s="40"/>
-      <c r="W18" s="12"/>
-      <c r="X18" s="41">
-        <f>SUMIF(G18:S18, "&lt;30")+V18+W18</f>
-        <v>32</v>
-      </c>
-      <c r="Y18" s="104">
-        <f>X18/U18</f>
-        <v>16</v>
-      </c>
-      <c r="Z18" s="59"/>
-      <c r="AA18" s="41"/>
-      <c r="AB18" s="41"/>
+      <c r="AA18" s="74">
+        <f>Z18/W18</f>
+        <v>16.5</v>
+      </c>
+      <c r="AB18" s="62"/>
       <c r="AC18" s="13"/>
-      <c r="AD18" s="60"/>
+      <c r="AD18" s="13"/>
+      <c r="AE18" s="13"/>
+      <c r="AF18" s="60"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:32">
       <c r="A19" s="9" t="s">
         <v>22</v>
       </c>
@@ -2787,94 +2888,98 @@
       <c r="Q19" s="12"/>
       <c r="R19" s="14"/>
       <c r="S19" s="12"/>
-      <c r="T19" s="66">
-        <f>F19+J19+L19+N19+P19+R19</f>
+      <c r="T19" s="14"/>
+      <c r="U19" s="12"/>
+      <c r="V19" s="66">
+        <f>F19+J19+L19+N19+P19+R19+T19</f>
         <v>56</v>
       </c>
-      <c r="U19" s="13">
-        <f>COUNTIF(D19:R19,"&gt;30")</f>
+      <c r="W19" s="13">
+        <f>COUNTIF(D19:T19,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="V19" s="40"/>
-      <c r="W19" s="12"/>
-      <c r="X19" s="41">
-        <f>SUMIF(G19:S19, "&lt;30")+V19+W19</f>
+      <c r="X19" s="40"/>
+      <c r="Y19" s="12"/>
+      <c r="Z19" s="41">
+        <f>SUMIF(G19:U19, "&lt;30")+X19+Y19</f>
         <v>16</v>
       </c>
-      <c r="Y19" s="104">
-        <f>X19/U19</f>
+      <c r="AA19" s="74">
+        <f>Z19/W19</f>
         <v>16</v>
       </c>
-      <c r="Z19" s="62"/>
-      <c r="AA19" s="41"/>
-      <c r="AB19" s="41"/>
-      <c r="AC19" s="13"/>
-      <c r="AD19" s="60"/>
+      <c r="AB19" s="62"/>
+      <c r="AC19" s="41"/>
+      <c r="AD19" s="41"/>
+      <c r="AE19" s="13"/>
+      <c r="AF19" s="60"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:32">
       <c r="A20" s="9" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="C20" s="11">
-        <f>(T20-(36*U20))/U20</f>
-        <v>20</v>
+        <f>ROUND((V20-(36*W20))/W20,0)</f>
+        <v>14</v>
       </c>
       <c r="D20" s="52"/>
       <c r="E20" s="53"/>
-      <c r="F20" s="14">
-        <v>55</v>
-      </c>
-      <c r="G20" s="12">
-        <v>16</v>
-      </c>
+      <c r="F20" s="14"/>
+      <c r="G20" s="12"/>
       <c r="H20" s="52"/>
       <c r="I20" s="53"/>
       <c r="J20" s="14"/>
       <c r="K20" s="12"/>
-      <c r="L20" s="14">
-        <v>56</v>
-      </c>
-      <c r="M20" s="12">
-        <v>15</v>
-      </c>
-      <c r="N20" s="14">
-        <v>57</v>
-      </c>
-      <c r="O20" s="12">
+      <c r="L20" s="14"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="14">
+        <v>48</v>
+      </c>
+      <c r="Q20" s="12">
+        <v>18</v>
+      </c>
+      <c r="R20" s="14">
+        <v>51</v>
+      </c>
+      <c r="S20" s="12">
         <v>14</v>
       </c>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="12"/>
-      <c r="R20" s="14"/>
-      <c r="S20" s="12"/>
-      <c r="T20" s="66">
-        <f>F20+J20+L20+N20+P20+R20</f>
-        <v>168</v>
-      </c>
-      <c r="U20" s="13">
-        <f>COUNTIF(D20:R20,"&gt;30")</f>
+      <c r="T20" s="14">
+        <v>51</v>
+      </c>
+      <c r="U20" s="12">
+        <v>14</v>
+      </c>
+      <c r="V20" s="66">
+        <f>F20+J20+L20+N20+P20+R20+T20</f>
+        <v>150</v>
+      </c>
+      <c r="W20" s="13">
+        <f>COUNTIF(D20:T20,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="V20" s="40"/>
-      <c r="W20" s="12"/>
-      <c r="X20" s="41">
-        <f>SUMIF(G20:S20, "&lt;30")+V20+W20</f>
-        <v>45</v>
-      </c>
-      <c r="Y20" s="104">
-        <f>X20/U20</f>
-        <v>15</v>
-      </c>
-      <c r="Z20" s="62"/>
-      <c r="AA20" s="41"/>
-      <c r="AB20" s="41"/>
-      <c r="AC20" s="13"/>
-      <c r="AD20" s="60"/>
+      <c r="X20" s="40"/>
+      <c r="Y20" s="12"/>
+      <c r="Z20" s="41">
+        <f>SUMIF(G20:U20, "&lt;30")+X20+Y20</f>
+        <v>46</v>
+      </c>
+      <c r="AA20" s="74">
+        <f>Z20/W20</f>
+        <v>15.333333333333334</v>
+      </c>
+      <c r="AB20" s="59"/>
+      <c r="AC20" s="41"/>
+      <c r="AD20" s="41"/>
+      <c r="AE20" s="13"/>
+      <c r="AF20" s="60"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:32">
       <c r="A21" s="9" t="s">
         <v>49</v>
       </c>
@@ -2902,33 +3007,35 @@
       <c r="Q21" s="12"/>
       <c r="R21" s="49"/>
       <c r="S21" s="12"/>
-      <c r="T21" s="66">
-        <f>F21+J21+L21+N21+P21+R21</f>
+      <c r="T21" s="49"/>
+      <c r="U21" s="12"/>
+      <c r="V21" s="66">
+        <f>F21+J21+L21+N21+P21+R21+T21</f>
         <v>50</v>
       </c>
-      <c r="U21" s="13">
-        <f>COUNTIF(D21:R21,"&gt;30")</f>
+      <c r="W21" s="13">
+        <f>COUNTIF(D21:T21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="V21" s="40">
+      <c r="X21" s="40">
         <v>1</v>
       </c>
-      <c r="W21" s="12"/>
-      <c r="X21" s="41">
-        <f>SUMIF(G21:S21, "&lt;30")+V21+W21</f>
+      <c r="Y21" s="12"/>
+      <c r="Z21" s="41">
+        <f>SUMIF(G21:U21, "&lt;30")+X21+Y21</f>
         <v>1</v>
       </c>
-      <c r="Y21" s="104">
-        <f>X21/U21</f>
+      <c r="AA21" s="74">
+        <f>Z21/W21</f>
         <v>1</v>
       </c>
-      <c r="Z21" s="59"/>
-      <c r="AA21" s="41"/>
-      <c r="AB21" s="41"/>
-      <c r="AC21" s="13"/>
-      <c r="AD21" s="60"/>
+      <c r="AB21" s="59"/>
+      <c r="AC21" s="41"/>
+      <c r="AD21" s="41"/>
+      <c r="AE21" s="13"/>
+      <c r="AF21" s="60"/>
     </row>
-    <row r="22" spans="1:30" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" ht="17" thickBot="1">
       <c r="A22" s="18" t="s">
         <v>56</v>
       </c>
@@ -2958,31 +3065,33 @@
       <c r="Q22" s="21"/>
       <c r="R22" s="71"/>
       <c r="S22" s="21"/>
-      <c r="T22" s="67">
-        <f>F22+J22+L22+N22+P22+R22</f>
+      <c r="T22" s="71"/>
+      <c r="U22" s="21"/>
+      <c r="V22" s="67">
+        <f>F22+J22+L22+N22+P22+R22+T22</f>
         <v>88</v>
       </c>
-      <c r="U22" s="22">
-        <f>COUNTIF(D22:R22,"&gt;30")</f>
+      <c r="W22" s="22">
+        <f>COUNTIF(D22:T22,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="V22" s="44"/>
-      <c r="W22" s="21"/>
-      <c r="X22" s="45">
-        <f>SUMIF(G22:S22, "&lt;30")+V22+W22</f>
+      <c r="X22" s="44"/>
+      <c r="Y22" s="21"/>
+      <c r="Z22" s="45">
+        <f>SUMIF(G22:S22, "&lt;30")+X22+Y22</f>
         <v>0</v>
       </c>
-      <c r="Y22" s="105">
-        <f>X22/U22</f>
+      <c r="AA22" s="75">
+        <f>Z22/W22</f>
         <v>0</v>
       </c>
-      <c r="Z22" s="63"/>
-      <c r="AA22" s="45"/>
-      <c r="AB22" s="45"/>
-      <c r="AC22" s="22"/>
-      <c r="AD22" s="64"/>
+      <c r="AB22" s="63"/>
+      <c r="AC22" s="45"/>
+      <c r="AD22" s="45"/>
+      <c r="AE22" s="22"/>
+      <c r="AF22" s="64"/>
     </row>
-    <row r="23" spans="1:30" s="23" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" s="23" customFormat="1" ht="17" thickBot="1">
       <c r="A23" s="34"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -3020,18 +3129,23 @@
         <v>48.272727272727273</v>
       </c>
       <c r="S23" s="36"/>
-      <c r="T23" s="37"/>
+      <c r="T23" s="36">
+        <f>AVERAGEIF(T4:T22,"&gt;0")</f>
+        <v>50.333333333333336</v>
+      </c>
+      <c r="U23" s="36"/>
+      <c r="V23" s="37"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:32">
       <c r="C24" s="24"/>
-      <c r="T24" s="25"/>
-      <c r="U24" s="25"/>
-      <c r="V24" s="26"/>
-      <c r="W24" s="26"/>
-      <c r="X24" s="25"/>
-      <c r="Y24" s="27"/>
+      <c r="V24" s="25"/>
+      <c r="W24" s="25"/>
+      <c r="X24" s="26"/>
+      <c r="Y24" s="26"/>
+      <c r="Z24" s="25"/>
+      <c r="AA24" s="27"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:32">
       <c r="C25" s="46" t="s">
         <v>42</v>
       </c>
@@ -3045,8 +3159,9 @@
       <c r="N25" s="28"/>
       <c r="P25" s="28"/>
       <c r="R25" s="28"/>
+      <c r="T25" s="28"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:32">
       <c r="C26" s="47" t="s">
         <v>43</v>
       </c>
@@ -3060,9 +3175,10 @@
       <c r="N26" s="29"/>
       <c r="P26" s="29"/>
       <c r="R26" s="29"/>
-      <c r="T26" s="30"/>
+      <c r="T26" s="29"/>
+      <c r="V26" s="30"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:32">
       <c r="C27" s="48" t="s">
         <v>47</v>
       </c>
@@ -3084,44 +3200,48 @@
       <c r="Q27" s="32"/>
       <c r="R27" s="31"/>
       <c r="S27" s="32"/>
+      <c r="T27" s="31"/>
+      <c r="U27" s="32"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AD22">
-    <sortCondition descending="1" ref="Y4:Y22"/>
-    <sortCondition descending="1" ref="T4:T22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AF22">
+    <sortCondition descending="1" ref="AA4:AA22"/>
+    <sortCondition descending="1" ref="V4:V22"/>
   </sortState>
-  <mergeCells count="31">
+  <mergeCells count="33">
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="AB1:AF1"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="V1:V3"/>
+    <mergeCell ref="W1:AA1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="T1:T3"/>
-    <mergeCell ref="U1:Y1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="Z1:AD1"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R2:S2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
070825 - updated scores/handicaps/tee times
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC66D5BD-DA05-4449-B3BD-0984F6BD15D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A08374-C824-1D4B-B357-6065B8F394EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44380" yWindow="1480" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="64">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>WEEK 9</t>
+  </si>
+  <si>
+    <t>WEEK 10</t>
   </si>
 </sst>
 </file>
@@ -934,7 +937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1144,7 +1147,85 @@
     <xf numFmtId="1" fontId="16" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1171,85 +1252,10 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1586,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AF27"/>
+  <dimension ref="A1:AH27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1594,158 +1600,166 @@
     <col min="3" max="3" width="10.1640625" customWidth="1"/>
     <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="15" width="6.33203125" hidden="1" customWidth="1"/>
-    <col min="16" max="21" width="6.33203125" customWidth="1"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1"/>
-    <col min="23" max="23" width="6.1640625" customWidth="1"/>
-    <col min="24" max="24" width="5.83203125" customWidth="1"/>
-    <col min="25" max="25" width="5.6640625" customWidth="1"/>
-    <col min="26" max="26" width="5.5" customWidth="1"/>
-    <col min="27" max="27" width="8" customWidth="1"/>
-    <col min="28" max="28" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="29" max="30" width="6" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="32" max="32" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="17" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="18" max="23" width="6.33203125" customWidth="1"/>
+    <col min="24" max="24" width="8.83203125" customWidth="1"/>
+    <col min="25" max="25" width="6.1640625" customWidth="1"/>
+    <col min="26" max="26" width="5.83203125" customWidth="1"/>
+    <col min="27" max="27" width="5.6640625" customWidth="1"/>
+    <col min="28" max="28" width="5.5" customWidth="1"/>
+    <col min="29" max="29" width="8" customWidth="1"/>
+    <col min="30" max="30" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="31" max="32" width="6" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="34" max="34" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="57" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="78" t="s">
+    <row r="1" spans="1:34" s="57" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="84" t="s">
+      <c r="B1" s="105"/>
+      <c r="C1" s="110" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="86" t="s">
+      <c r="D1" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="87"/>
-      <c r="F1" s="86" t="s">
+      <c r="E1" s="90"/>
+      <c r="F1" s="89" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="87"/>
-      <c r="H1" s="86" t="s">
+      <c r="G1" s="90"/>
+      <c r="H1" s="89" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="87"/>
-      <c r="J1" s="86" t="s">
+      <c r="I1" s="90"/>
+      <c r="J1" s="89" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="87"/>
-      <c r="L1" s="86" t="s">
+      <c r="K1" s="90"/>
+      <c r="L1" s="89" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="87"/>
-      <c r="N1" s="86" t="s">
+      <c r="M1" s="90"/>
+      <c r="N1" s="89" t="s">
         <v>55</v>
       </c>
-      <c r="O1" s="87"/>
-      <c r="P1" s="86" t="s">
+      <c r="O1" s="90"/>
+      <c r="P1" s="89" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="87"/>
-      <c r="R1" s="86" t="s">
+      <c r="Q1" s="90"/>
+      <c r="R1" s="89" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="87"/>
-      <c r="T1" s="86" t="s">
+      <c r="S1" s="90"/>
+      <c r="T1" s="89" t="s">
         <v>62</v>
       </c>
-      <c r="U1" s="87"/>
-      <c r="V1" s="98" t="s">
+      <c r="U1" s="90"/>
+      <c r="V1" s="89" t="s">
+        <v>63</v>
+      </c>
+      <c r="W1" s="90"/>
+      <c r="X1" s="99" t="s">
         <v>2</v>
       </c>
-      <c r="W1" s="100" t="s">
+      <c r="Y1" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="X1" s="101"/>
-      <c r="Y1" s="101"/>
-      <c r="Z1" s="101"/>
+      <c r="Z1" s="102"/>
       <c r="AA1" s="102"/>
-      <c r="AB1" s="103" t="s">
+      <c r="AB1" s="102"/>
+      <c r="AC1" s="103"/>
+      <c r="AD1" s="84" t="s">
         <v>58</v>
       </c>
-      <c r="AC1" s="104"/>
-      <c r="AD1" s="104"/>
-      <c r="AE1" s="104"/>
-      <c r="AF1" s="105"/>
+      <c r="AE1" s="85"/>
+      <c r="AF1" s="85"/>
+      <c r="AG1" s="85"/>
+      <c r="AH1" s="86"/>
     </row>
-    <row r="2" spans="1:32" s="57" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="80"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="88">
+    <row r="2" spans="1:34" s="57" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="106"/>
+      <c r="B2" s="107"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="82">
         <v>45782</v>
       </c>
-      <c r="E2" s="89"/>
-      <c r="F2" s="88">
+      <c r="E2" s="83"/>
+      <c r="F2" s="82">
         <v>45789</v>
       </c>
-      <c r="G2" s="89"/>
-      <c r="H2" s="88">
+      <c r="G2" s="83"/>
+      <c r="H2" s="82">
         <v>45796</v>
       </c>
-      <c r="I2" s="89"/>
-      <c r="J2" s="88">
+      <c r="I2" s="83"/>
+      <c r="J2" s="82">
         <v>45803</v>
       </c>
-      <c r="K2" s="89"/>
-      <c r="L2" s="88">
+      <c r="K2" s="83"/>
+      <c r="L2" s="82">
         <v>45810</v>
       </c>
-      <c r="M2" s="89"/>
-      <c r="N2" s="88">
+      <c r="M2" s="83"/>
+      <c r="N2" s="82">
         <v>45817</v>
       </c>
-      <c r="O2" s="89"/>
-      <c r="P2" s="88">
+      <c r="O2" s="83"/>
+      <c r="P2" s="82">
         <v>45824</v>
       </c>
-      <c r="Q2" s="89"/>
-      <c r="R2" s="88">
+      <c r="Q2" s="83"/>
+      <c r="R2" s="82">
         <v>45831</v>
       </c>
-      <c r="S2" s="89"/>
-      <c r="T2" s="88">
+      <c r="S2" s="83"/>
+      <c r="T2" s="82">
         <v>45838</v>
       </c>
-      <c r="U2" s="89"/>
-      <c r="V2" s="99"/>
-      <c r="W2" s="98" t="s">
+      <c r="U2" s="83"/>
+      <c r="V2" s="82">
+        <v>45845</v>
+      </c>
+      <c r="W2" s="83"/>
+      <c r="X2" s="100"/>
+      <c r="Y2" s="99" t="s">
         <v>4</v>
       </c>
-      <c r="X2" s="94" t="s">
+      <c r="Z2" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="Y2" s="96" t="s">
+      <c r="AA2" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="Z2" s="90" t="s">
+      <c r="AB2" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="AA2" s="92" t="s">
+      <c r="AC2" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="AB2" s="106" t="s">
+      <c r="AD2" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="AC2" s="106" t="s">
+      <c r="AE2" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="AD2" s="106" t="s">
+      <c r="AF2" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="AE2" s="106" t="s">
+      <c r="AG2" s="87" t="s">
         <v>7</v>
       </c>
-      <c r="AF2" s="106" t="s">
+      <c r="AH2" s="87" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:32" s="57" customFormat="1" ht="29" customHeight="1" thickBot="1">
-      <c r="A3" s="82"/>
-      <c r="B3" s="83"/>
-      <c r="C3" s="85"/>
+    <row r="3" spans="1:34" s="57" customFormat="1" ht="29" customHeight="1" thickBot="1">
+      <c r="A3" s="108"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="111"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1800,19 +1814,25 @@
       <c r="U3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="V3" s="99"/>
-      <c r="W3" s="99"/>
-      <c r="X3" s="95"/>
-      <c r="Y3" s="97"/>
-      <c r="Z3" s="91"/>
-      <c r="AA3" s="93"/>
-      <c r="AB3" s="107"/>
-      <c r="AC3" s="107"/>
-      <c r="AD3" s="107"/>
-      <c r="AE3" s="107"/>
-      <c r="AF3" s="107"/>
+      <c r="V3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="X3" s="100"/>
+      <c r="Y3" s="100"/>
+      <c r="Z3" s="96"/>
+      <c r="AA3" s="98"/>
+      <c r="AB3" s="92"/>
+      <c r="AC3" s="94"/>
+      <c r="AD3" s="88"/>
+      <c r="AE3" s="88"/>
+      <c r="AF3" s="88"/>
+      <c r="AG3" s="88"/>
+      <c r="AH3" s="88"/>
     </row>
-    <row r="4" spans="1:32" ht="16" customHeight="1">
+    <row r="4" spans="1:34" ht="16" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
@@ -1820,7 +1840,8 @@
         <v>38</v>
       </c>
       <c r="C4" s="5">
-        <v>15</v>
+        <f>ROUND((X4-(36*Y4))/Y4,0)</f>
+        <v>10</v>
       </c>
       <c r="D4" s="50"/>
       <c r="E4" s="51"/>
@@ -1846,37 +1867,43 @@
       <c r="S4" s="7">
         <v>24</v>
       </c>
-      <c r="T4" s="108"/>
+      <c r="T4" s="77"/>
       <c r="U4" s="7"/>
-      <c r="V4" s="65">
-        <f>F4+J4+L4+N4+P4+R4+T4</f>
-        <v>88</v>
-      </c>
-      <c r="W4" s="8">
-        <f>COUNTIF(D4:T4,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="X4" s="38">
+      <c r="V4" s="77">
+        <v>50</v>
+      </c>
+      <c r="W4" s="7">
+        <v>19</v>
+      </c>
+      <c r="X4" s="65">
+        <f>F4+J4+L4+N4+P4+R4+T4+V4</f>
+        <v>138</v>
+      </c>
+      <c r="Y4" s="8">
+        <f>COUNTIF(D4:V4,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="Z4" s="38">
         <v>1</v>
       </c>
-      <c r="Y4" s="7">
+      <c r="AA4" s="7">
         <v>1</v>
       </c>
-      <c r="Z4" s="39">
-        <f>SUMIF(G4:U4, "&lt;30")+X4+Y4</f>
-        <v>52</v>
-      </c>
-      <c r="AA4" s="73">
-        <f>Z4/W4</f>
-        <v>26</v>
-      </c>
-      <c r="AB4" s="72"/>
-      <c r="AC4" s="39"/>
-      <c r="AD4" s="39"/>
-      <c r="AE4" s="8"/>
-      <c r="AF4" s="58"/>
+      <c r="AB4" s="39">
+        <f>SUMIF(G4:W4, "&lt;30")+Z4+AA4</f>
+        <v>71</v>
+      </c>
+      <c r="AC4" s="73">
+        <f>AB4/Y4</f>
+        <v>23.666666666666668</v>
+      </c>
+      <c r="AD4" s="72"/>
+      <c r="AE4" s="39"/>
+      <c r="AF4" s="39"/>
+      <c r="AG4" s="8"/>
+      <c r="AH4" s="58"/>
     </row>
-    <row r="5" spans="1:32">
+    <row r="5" spans="1:34">
       <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
@@ -1884,7 +1911,7 @@
         <v>16</v>
       </c>
       <c r="C5" s="11">
-        <f>ROUND((V5-(36*W5))/W5,0)</f>
+        <f>ROUND((X5-(36*Y5))/Y5,0)</f>
         <v>18</v>
       </c>
       <c r="D5" s="52"/>
@@ -1921,33 +1948,35 @@
       <c r="U5" s="12">
         <v>15</v>
       </c>
-      <c r="V5" s="66">
-        <f>F5+J5+L5+N5+P5+R5+T5</f>
+      <c r="V5" s="14"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="66">
+        <f>F5+J5+L5+N5+P5+R5+T5+V5</f>
         <v>216</v>
       </c>
-      <c r="W5" s="13">
-        <f>COUNTIF(D5:T5,"&gt;30")</f>
+      <c r="Y5" s="13">
+        <f>COUNTIF(D5:V5,"&gt;30")</f>
         <v>4</v>
       </c>
-      <c r="X5" s="40"/>
-      <c r="Y5" s="12"/>
-      <c r="Z5" s="41">
-        <f>SUMIF(G5:U5, "&lt;30")+X5+Y5</f>
+      <c r="Z5" s="40"/>
+      <c r="AA5" s="12"/>
+      <c r="AB5" s="41">
+        <f>SUMIF(G5:W5, "&lt;30")+Z5+AA5</f>
         <v>83</v>
       </c>
-      <c r="AA5" s="74">
-        <f>Z5/W5</f>
+      <c r="AC5" s="74">
+        <f>AB5/Y5</f>
         <v>20.75</v>
       </c>
-      <c r="AB5" s="59"/>
-      <c r="AC5" s="41"/>
-      <c r="AD5" s="41"/>
-      <c r="AE5" s="13"/>
-      <c r="AF5" s="60" t="s">
+      <c r="AD5" s="59"/>
+      <c r="AE5" s="41"/>
+      <c r="AF5" s="41"/>
+      <c r="AG5" s="13"/>
+      <c r="AH5" s="60" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:32">
+    <row r="6" spans="1:34">
       <c r="A6" s="9" t="s">
         <v>40</v>
       </c>
@@ -1955,7 +1984,7 @@
         <v>41</v>
       </c>
       <c r="C6" s="11">
-        <f>ROUND((V6-(36*W6))/W6,0)</f>
+        <f>ROUND((X6-(36*Y6))/Y6,0)</f>
         <v>13</v>
       </c>
       <c r="D6" s="52"/>
@@ -1996,31 +2025,37 @@
       <c r="U6" s="12">
         <v>23</v>
       </c>
-      <c r="V6" s="66">
-        <f>F6+J6+L6+N6+P6+R6+T6</f>
-        <v>243</v>
-      </c>
-      <c r="W6" s="13">
-        <f>COUNTIF(D6:T6,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="X6" s="40"/>
-      <c r="Y6" s="12"/>
-      <c r="Z6" s="41">
-        <f>SUMIF(G6:U6, "&lt;30")+X6+Y6</f>
-        <v>102</v>
-      </c>
-      <c r="AA6" s="74">
-        <f>Z6/W6</f>
-        <v>20.399999999999999</v>
-      </c>
-      <c r="AB6" s="59"/>
-      <c r="AC6" s="41"/>
-      <c r="AD6" s="41"/>
-      <c r="AE6" s="13"/>
-      <c r="AF6" s="60"/>
+      <c r="V6" s="14">
+        <v>48</v>
+      </c>
+      <c r="W6" s="12">
+        <v>19</v>
+      </c>
+      <c r="X6" s="66">
+        <f>F6+J6+L6+N6+P6+R6+T6+V6</f>
+        <v>291</v>
+      </c>
+      <c r="Y6" s="13">
+        <f>COUNTIF(D6:V6,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="Z6" s="40"/>
+      <c r="AA6" s="12"/>
+      <c r="AB6" s="41">
+        <f>SUMIF(G6:W6, "&lt;30")+Z6+AA6</f>
+        <v>121</v>
+      </c>
+      <c r="AC6" s="74">
+        <f>AB6/Y6</f>
+        <v>20.166666666666668</v>
+      </c>
+      <c r="AD6" s="59"/>
+      <c r="AE6" s="41"/>
+      <c r="AF6" s="41"/>
+      <c r="AG6" s="13"/>
+      <c r="AH6" s="60"/>
     </row>
-    <row r="7" spans="1:32">
+    <row r="7" spans="1:34">
       <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
@@ -2028,12 +2063,12 @@
         <v>14</v>
       </c>
       <c r="C7" s="11">
-        <f>ROUND((V7-(36*W7))/W7,0)</f>
+        <f>ROUND((X7-(36*Y7))/Y7,0)</f>
         <v>11</v>
       </c>
       <c r="D7" s="52"/>
       <c r="E7" s="53"/>
-      <c r="F7" s="110">
+      <c r="F7" s="79">
         <v>42</v>
       </c>
       <c r="G7" s="12">
@@ -2041,465 +2076,507 @@
       </c>
       <c r="H7" s="52"/>
       <c r="I7" s="53"/>
-      <c r="J7" s="110"/>
+      <c r="J7" s="79"/>
       <c r="K7" s="12"/>
-      <c r="L7" s="111">
+      <c r="L7" s="80">
         <v>51</v>
       </c>
       <c r="M7" s="12">
         <v>16</v>
       </c>
-      <c r="N7" s="111"/>
+      <c r="N7" s="80"/>
       <c r="O7" s="12"/>
-      <c r="P7" s="112">
+      <c r="P7" s="81">
         <v>49</v>
       </c>
       <c r="Q7" s="12">
         <v>18</v>
       </c>
-      <c r="R7" s="111">
+      <c r="R7" s="80">
         <v>46</v>
       </c>
       <c r="S7" s="12">
         <v>21</v>
       </c>
-      <c r="T7" s="111">
+      <c r="T7" s="80">
         <v>45</v>
       </c>
       <c r="U7" s="12">
         <v>20</v>
       </c>
-      <c r="V7" s="66">
-        <f>F7+J7+L7+N7+P7+R7+T7</f>
-        <v>233</v>
-      </c>
-      <c r="W7" s="13">
-        <f>COUNTIF(D7:T7,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="X7" s="40">
+      <c r="V7" s="80">
+        <v>46</v>
+      </c>
+      <c r="W7" s="12">
+        <v>19</v>
+      </c>
+      <c r="X7" s="66">
+        <f>F7+J7+L7+N7+P7+R7+T7+V7</f>
+        <v>279</v>
+      </c>
+      <c r="Y7" s="13">
+        <f>COUNTIF(D7:V7,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="Z7" s="40">
         <v>2</v>
       </c>
-      <c r="Y7" s="12"/>
-      <c r="Z7" s="41">
-        <f>SUMIF(G7:U7, "&lt;30")+X7+Y7</f>
-        <v>102</v>
-      </c>
-      <c r="AA7" s="74">
-        <f>Z7/W7</f>
-        <v>20.399999999999999</v>
-      </c>
-      <c r="AB7" s="59"/>
-      <c r="AC7" s="41"/>
-      <c r="AD7" s="41"/>
-      <c r="AE7" s="13"/>
-      <c r="AF7" s="60"/>
+      <c r="AA7" s="12"/>
+      <c r="AB7" s="41">
+        <f>SUMIF(G7:W7, "&lt;30")+Z7+AA7</f>
+        <v>121</v>
+      </c>
+      <c r="AC7" s="74">
+        <f>AB7/Y7</f>
+        <v>20.166666666666668</v>
+      </c>
+      <c r="AD7" s="59"/>
+      <c r="AE7" s="41"/>
+      <c r="AF7" s="41"/>
+      <c r="AG7" s="13"/>
+      <c r="AH7" s="60"/>
     </row>
-    <row r="8" spans="1:32">
+    <row r="8" spans="1:34">
       <c r="A8" s="9" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="C8" s="11">
-        <f>ROUND((V8-(36*W8))/W8,0)</f>
-        <v>12</v>
+        <f>ROUND((X8-(36*Y8))/Y8,0)</f>
+        <v>14</v>
       </c>
       <c r="D8" s="52"/>
       <c r="E8" s="53"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="12"/>
+      <c r="F8" s="14">
+        <v>42</v>
+      </c>
+      <c r="G8" s="12">
+        <v>27</v>
+      </c>
       <c r="H8" s="52"/>
       <c r="I8" s="53"/>
-      <c r="J8" s="16"/>
+      <c r="J8" s="14"/>
       <c r="K8" s="12"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="16"/>
+      <c r="L8" s="14">
+        <v>54</v>
+      </c>
+      <c r="M8" s="12">
+        <v>15</v>
+      </c>
+      <c r="N8" s="14"/>
       <c r="O8" s="12"/>
-      <c r="P8" s="42">
-        <v>47</v>
+      <c r="P8" s="14">
+        <v>54</v>
       </c>
       <c r="Q8" s="12">
-        <v>20</v>
-      </c>
-      <c r="R8" s="42">
-        <v>50</v>
+        <v>16</v>
+      </c>
+      <c r="R8" s="14">
+        <v>53</v>
       </c>
       <c r="S8" s="12">
-        <v>17</v>
-      </c>
-      <c r="T8" s="42">
+        <v>16</v>
+      </c>
+      <c r="T8" s="14"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="78">
         <v>46</v>
       </c>
-      <c r="U8" s="12">
-        <v>21</v>
-      </c>
-      <c r="V8" s="66">
-        <f>F8+J8+L8+N8+P8+R8+T8</f>
-        <v>143</v>
-      </c>
-      <c r="W8" s="13">
-        <f>COUNTIF(D8:T8,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="X8" s="40"/>
-      <c r="Y8" s="12"/>
-      <c r="Z8" s="41">
-        <f>SUMIF(G8:U8, "&lt;30")+X8+Y8</f>
-        <v>58</v>
-      </c>
-      <c r="AA8" s="74">
-        <f>Z8/W8</f>
-        <v>19.333333333333332</v>
-      </c>
-      <c r="AB8" s="61"/>
-      <c r="AC8" s="41"/>
-      <c r="AD8" s="41"/>
-      <c r="AE8" s="13"/>
-      <c r="AF8" s="60"/>
+      <c r="W8" s="12">
+        <v>23</v>
+      </c>
+      <c r="X8" s="66">
+        <f>F8+J8+L8+N8+P8+R8+T8+V8</f>
+        <v>249</v>
+      </c>
+      <c r="Y8" s="13">
+        <f>COUNTIF(D8:V8,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="Z8" s="40">
+        <v>1</v>
+      </c>
+      <c r="AA8" s="12"/>
+      <c r="AB8" s="41">
+        <f>SUMIF(G8:W8, "&lt;30")+Z8+AA8</f>
+        <v>98</v>
+      </c>
+      <c r="AC8" s="74">
+        <f>AB8/Y8</f>
+        <v>19.600000000000001</v>
+      </c>
+      <c r="AD8" s="61"/>
+      <c r="AE8" s="41"/>
+      <c r="AF8" s="41"/>
+      <c r="AG8" s="13"/>
+      <c r="AH8" s="60"/>
     </row>
-    <row r="9" spans="1:32">
+    <row r="9" spans="1:34">
       <c r="A9" s="9" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C9" s="11">
-        <f>ROUND((V9-(36*W9))/W9,0)</f>
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="53"/>
-      <c r="F9" s="70">
-        <v>45</v>
-      </c>
-      <c r="G9" s="12">
-        <v>17</v>
-      </c>
+      <c r="F9" s="17"/>
+      <c r="G9" s="12"/>
       <c r="H9" s="52"/>
       <c r="I9" s="53"/>
-      <c r="J9" s="70"/>
+      <c r="J9" s="17"/>
       <c r="K9" s="12"/>
-      <c r="L9" s="70">
-        <v>43</v>
-      </c>
-      <c r="M9" s="12">
+      <c r="L9" s="17"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="68">
+        <v>39</v>
+      </c>
+      <c r="Q9" s="12">
+        <v>17</v>
+      </c>
+      <c r="R9" s="68">
+        <v>38</v>
+      </c>
+      <c r="S9" s="12">
+        <v>18</v>
+      </c>
+      <c r="T9" s="68"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="112">
+        <v>37</v>
+      </c>
+      <c r="W9" s="12">
         <v>19</v>
       </c>
-      <c r="N9" s="15">
-        <v>41</v>
-      </c>
-      <c r="O9" s="12">
-        <v>21</v>
-      </c>
-      <c r="P9" s="42">
-        <v>47</v>
-      </c>
-      <c r="Q9" s="12">
-        <v>15</v>
-      </c>
-      <c r="R9" s="42">
-        <v>42</v>
-      </c>
-      <c r="S9" s="12">
-        <v>20</v>
-      </c>
-      <c r="T9" s="42">
-        <v>43</v>
-      </c>
-      <c r="U9" s="12">
-        <v>19</v>
-      </c>
-      <c r="V9" s="66">
-        <f>F9+J9+L9+N9+P9+R9+T9</f>
-        <v>261</v>
-      </c>
-      <c r="W9" s="13">
-        <f>COUNTIF(D9:T9,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="X9" s="40">
+      <c r="X9" s="66">
+        <f>F9+J9+L9+N9+P9+R9+T9+V9</f>
+        <v>114</v>
+      </c>
+      <c r="Y9" s="13">
+        <f>COUNTIF(D9:V9,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="Z9" s="40">
         <v>1</v>
       </c>
-      <c r="Y9" s="12">
+      <c r="AA9" s="12">
         <v>3</v>
       </c>
-      <c r="Z9" s="41">
-        <f>SUMIF(G9:U9, "&lt;30")+X9+Y9</f>
-        <v>115</v>
-      </c>
-      <c r="AA9" s="74">
-        <f>Z9/W9</f>
-        <v>19.166666666666668</v>
-      </c>
-      <c r="AB9" s="59"/>
-      <c r="AC9" s="41"/>
-      <c r="AD9" s="41"/>
-      <c r="AE9" s="13"/>
-      <c r="AF9" s="60"/>
+      <c r="AB9" s="41">
+        <f>SUMIF(G9:W9, "&lt;30")+Z9+AA9</f>
+        <v>58</v>
+      </c>
+      <c r="AC9" s="74">
+        <f>AB9/Y9</f>
+        <v>19.333333333333332</v>
+      </c>
+      <c r="AD9" s="59"/>
+      <c r="AE9" s="41"/>
+      <c r="AF9" s="41"/>
+      <c r="AG9" s="13"/>
+      <c r="AH9" s="60"/>
     </row>
-    <row r="10" spans="1:32">
+    <row r="10" spans="1:34">
       <c r="A10" s="9" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="11">
+        <f>ROUND((X10-(36*Y10))/Y10,0)</f>
         <v>12</v>
-      </c>
-      <c r="C10" s="11">
-        <v>22</v>
       </c>
       <c r="D10" s="52"/>
       <c r="E10" s="53"/>
-      <c r="F10" s="14">
-        <v>59</v>
-      </c>
-      <c r="G10" s="12">
-        <v>17</v>
-      </c>
+      <c r="F10" s="16"/>
+      <c r="G10" s="12"/>
       <c r="H10" s="52"/>
       <c r="I10" s="53"/>
-      <c r="J10" s="14"/>
+      <c r="J10" s="16"/>
       <c r="K10" s="12"/>
-      <c r="L10" s="14"/>
+      <c r="L10" s="16"/>
       <c r="M10" s="12"/>
-      <c r="N10" s="14"/>
+      <c r="N10" s="16"/>
       <c r="O10" s="12"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="14">
-        <v>55</v>
+      <c r="P10" s="42">
+        <v>47</v>
+      </c>
+      <c r="Q10" s="12">
+        <v>20</v>
+      </c>
+      <c r="R10" s="42">
+        <v>50</v>
       </c>
       <c r="S10" s="12">
+        <v>17</v>
+      </c>
+      <c r="T10" s="42">
+        <v>46</v>
+      </c>
+      <c r="U10" s="12">
         <v>21</v>
       </c>
-      <c r="T10" s="14"/>
-      <c r="U10" s="12"/>
-      <c r="V10" s="66">
-        <f>F10+J10+L10+N10+P10+R10+T10</f>
-        <v>114</v>
-      </c>
-      <c r="W10" s="13">
-        <f>COUNTIF(D10:T10,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="X10" s="40"/>
-      <c r="Y10" s="12"/>
-      <c r="Z10" s="41">
-        <f>SUMIF(G10:U10, "&lt;30")+X10+Y10</f>
-        <v>38</v>
-      </c>
-      <c r="AA10" s="74">
-        <f>Z10/W10</f>
+      <c r="V10" s="42">
+        <v>47</v>
+      </c>
+      <c r="W10" s="12">
         <v>19</v>
       </c>
-      <c r="AB10" s="77"/>
-      <c r="AC10" s="41"/>
-      <c r="AD10" s="41"/>
-      <c r="AE10" s="13"/>
-      <c r="AF10" s="60"/>
+      <c r="X10" s="66">
+        <f>F10+J10+L10+N10+P10+R10+T10+V10</f>
+        <v>190</v>
+      </c>
+      <c r="Y10" s="13">
+        <f>COUNTIF(D10:V10,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="Z10" s="40"/>
+      <c r="AA10" s="12"/>
+      <c r="AB10" s="41">
+        <f>SUMIF(G10:W10, "&lt;30")+Z10+AA10</f>
+        <v>77</v>
+      </c>
+      <c r="AC10" s="74">
+        <f>AB10/Y10</f>
+        <v>19.25</v>
+      </c>
+      <c r="AD10" s="113"/>
+      <c r="AE10" s="41"/>
+      <c r="AF10" s="41"/>
+      <c r="AG10" s="13"/>
+      <c r="AH10" s="60"/>
     </row>
-    <row r="11" spans="1:32">
+    <row r="11" spans="1:34">
       <c r="A11" s="9" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" s="11">
-        <f>ROUND((V11-(36*W11))/W11,0)</f>
+        <f>ROUND((X11-(36*Y11))/Y11,0)</f>
         <v>8</v>
       </c>
       <c r="D11" s="52"/>
       <c r="E11" s="53"/>
-      <c r="F11" s="14">
-        <v>46</v>
+      <c r="F11" s="70">
+        <v>45</v>
       </c>
       <c r="G11" s="12">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H11" s="52"/>
       <c r="I11" s="53"/>
-      <c r="J11" s="14"/>
+      <c r="J11" s="70"/>
       <c r="K11" s="12"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="14">
+      <c r="L11" s="70">
+        <v>43</v>
+      </c>
+      <c r="M11" s="12">
+        <v>19</v>
+      </c>
+      <c r="N11" s="15">
+        <v>41</v>
+      </c>
+      <c r="O11" s="12">
+        <v>21</v>
+      </c>
+      <c r="P11" s="42">
+        <v>47</v>
+      </c>
+      <c r="Q11" s="12">
+        <v>15</v>
+      </c>
+      <c r="R11" s="42">
         <v>42</v>
       </c>
-      <c r="O11" s="12">
+      <c r="S11" s="12">
         <v>20</v>
       </c>
-      <c r="P11" s="14">
+      <c r="T11" s="42">
         <v>43</v>
       </c>
-      <c r="Q11" s="12">
+      <c r="U11" s="12">
         <v>19</v>
       </c>
-      <c r="R11" s="14"/>
-      <c r="S11" s="12"/>
-      <c r="T11" s="14"/>
-      <c r="U11" s="12"/>
-      <c r="V11" s="66">
-        <f>F11+J11+L11+N11+P11+R11+T11</f>
-        <v>131</v>
-      </c>
-      <c r="W11" s="13">
-        <f>COUNTIF(D11:T11,"&gt;30")</f>
+      <c r="V11" s="42">
+        <v>44</v>
+      </c>
+      <c r="W11" s="12">
+        <v>18</v>
+      </c>
+      <c r="X11" s="66">
+        <f>F11+J11+L11+N11+P11+R11+T11+V11</f>
+        <v>305</v>
+      </c>
+      <c r="Y11" s="13">
+        <f>COUNTIF(D11:V11,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="Z11" s="40">
+        <v>1</v>
+      </c>
+      <c r="AA11" s="12">
         <v>3</v>
       </c>
-      <c r="X11" s="40"/>
-      <c r="Y11" s="12">
-        <v>1</v>
-      </c>
-      <c r="Z11" s="41">
-        <f>SUMIF(G11:U11, "&lt;30")+X11+Y11</f>
-        <v>56</v>
-      </c>
-      <c r="AA11" s="74">
-        <f>Z11/W11</f>
-        <v>18.666666666666668</v>
-      </c>
-      <c r="AB11" s="62"/>
-      <c r="AC11" s="41"/>
-      <c r="AD11" s="41"/>
-      <c r="AE11" s="13"/>
-      <c r="AF11" s="60"/>
+      <c r="AB11" s="41">
+        <f>SUMIF(G11:W11, "&lt;30")+Z11+AA11</f>
+        <v>133</v>
+      </c>
+      <c r="AC11" s="74">
+        <f>AB11/Y11</f>
+        <v>19</v>
+      </c>
+      <c r="AD11" s="59"/>
+      <c r="AE11" s="41"/>
+      <c r="AF11" s="41"/>
+      <c r="AG11" s="13"/>
+      <c r="AH11" s="60"/>
     </row>
-    <row r="12" spans="1:32">
+    <row r="12" spans="1:34">
       <c r="A12" s="9" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C12" s="11">
-        <f>ROUND((V12-(36*W12))/W12,0)</f>
-        <v>15</v>
+        <f>ROUND((X12-(36*Y12))/Y12,0)</f>
+        <v>8</v>
       </c>
       <c r="D12" s="52"/>
       <c r="E12" s="53"/>
       <c r="F12" s="14">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G12" s="12">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H12" s="52"/>
       <c r="I12" s="53"/>
       <c r="J12" s="14"/>
       <c r="K12" s="12"/>
-      <c r="L12" s="14">
-        <v>54</v>
-      </c>
-      <c r="M12" s="12">
-        <v>15</v>
-      </c>
-      <c r="N12" s="14"/>
-      <c r="O12" s="12"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="14">
+        <v>42</v>
+      </c>
+      <c r="O12" s="12">
+        <v>20</v>
+      </c>
       <c r="P12" s="14">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="Q12" s="12">
-        <v>16</v>
-      </c>
-      <c r="R12" s="14">
-        <v>53</v>
-      </c>
-      <c r="S12" s="12">
-        <v>16</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="R12" s="14"/>
+      <c r="S12" s="12"/>
       <c r="T12" s="14"/>
       <c r="U12" s="12"/>
-      <c r="V12" s="66">
-        <f>F12+J12+L12+N12+P12+R12+T12</f>
-        <v>203</v>
-      </c>
-      <c r="W12" s="13">
-        <f>COUNTIF(D12:T12,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="X12" s="40"/>
-      <c r="Y12" s="12"/>
-      <c r="Z12" s="41">
-        <f>SUMIF(G12:U12, "&lt;30")+X12+Y12</f>
-        <v>74</v>
-      </c>
-      <c r="AA12" s="74">
-        <f>Z12/W12</f>
-        <v>18.5</v>
-      </c>
-      <c r="AB12" s="59"/>
-      <c r="AC12" s="41"/>
-      <c r="AD12" s="41"/>
-      <c r="AE12" s="13"/>
-      <c r="AF12" s="60"/>
+      <c r="V12" s="14"/>
+      <c r="W12" s="12"/>
+      <c r="X12" s="66">
+        <f>F12+J12+L12+N12+P12+R12+T12+V12</f>
+        <v>131</v>
+      </c>
+      <c r="Y12" s="13">
+        <f>COUNTIF(D12:V12,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="Z12" s="40"/>
+      <c r="AA12" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="41">
+        <f>SUMIF(G12:W12, "&lt;30")+Z12+AA12</f>
+        <v>56</v>
+      </c>
+      <c r="AC12" s="74">
+        <f>AB12/Y12</f>
+        <v>18.666666666666668</v>
+      </c>
+      <c r="AD12" s="62"/>
+      <c r="AE12" s="41"/>
+      <c r="AF12" s="41"/>
+      <c r="AG12" s="13"/>
+      <c r="AH12" s="60"/>
     </row>
-    <row r="13" spans="1:32">
+    <row r="13" spans="1:34">
       <c r="A13" s="9" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="C13" s="11">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D13" s="52"/>
       <c r="E13" s="53"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="12"/>
+      <c r="F13" s="14">
+        <v>59</v>
+      </c>
+      <c r="G13" s="12">
+        <v>17</v>
+      </c>
       <c r="H13" s="52"/>
       <c r="I13" s="53"/>
-      <c r="J13" s="17"/>
+      <c r="J13" s="14"/>
       <c r="K13" s="12"/>
-      <c r="L13" s="17"/>
+      <c r="L13" s="14"/>
       <c r="M13" s="12"/>
-      <c r="N13" s="17"/>
+      <c r="N13" s="14"/>
       <c r="O13" s="12"/>
-      <c r="P13" s="68">
-        <v>39</v>
-      </c>
-      <c r="Q13" s="12">
+      <c r="P13" s="14"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="14">
+        <v>55</v>
+      </c>
+      <c r="S13" s="12">
+        <v>21</v>
+      </c>
+      <c r="T13" s="14"/>
+      <c r="U13" s="12"/>
+      <c r="V13" s="14">
+        <v>59</v>
+      </c>
+      <c r="W13" s="12">
         <v>17</v>
       </c>
-      <c r="R13" s="68">
-        <v>38</v>
-      </c>
-      <c r="S13" s="12">
-        <v>18</v>
-      </c>
-      <c r="T13" s="68"/>
-      <c r="U13" s="12"/>
-      <c r="V13" s="66">
-        <f>F13+J13+L13+N13+P13+R13+T13</f>
-        <v>77</v>
-      </c>
-      <c r="W13" s="13">
-        <f>COUNTIF(D13:T13,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="X13" s="40"/>
-      <c r="Y13" s="12">
-        <v>2</v>
-      </c>
-      <c r="Z13" s="41">
-        <f>SUMIF(G13:U13, "&lt;30")+X13+Y13</f>
-        <v>37</v>
-      </c>
-      <c r="AA13" s="74">
-        <f>Z13/W13</f>
-        <v>18.5</v>
-      </c>
-      <c r="AB13" s="59"/>
-      <c r="AC13" s="41"/>
-      <c r="AD13" s="41"/>
-      <c r="AE13" s="13"/>
-      <c r="AF13" s="60"/>
+      <c r="X13" s="66">
+        <f>F13+J13+L13+N13+P13+R13+T13+V13</f>
+        <v>173</v>
+      </c>
+      <c r="Y13" s="13">
+        <f>COUNTIF(D13:V13,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="Z13" s="40"/>
+      <c r="AA13" s="12"/>
+      <c r="AB13" s="41">
+        <f>SUMIF(G13:W13, "&lt;30")+Z13+AA13</f>
+        <v>55</v>
+      </c>
+      <c r="AC13" s="74">
+        <f>AB13/Y13</f>
+        <v>18.333333333333332</v>
+      </c>
+      <c r="AD13" s="62"/>
+      <c r="AE13" s="41"/>
+      <c r="AF13" s="41"/>
+      <c r="AG13" s="13"/>
+      <c r="AH13" s="60"/>
     </row>
-    <row r="14" spans="1:32">
+    <row r="14" spans="1:34">
       <c r="A14" s="9" t="s">
         <v>26</v>
       </c>
@@ -2507,7 +2584,7 @@
         <v>27</v>
       </c>
       <c r="C14" s="11">
-        <f>ROUND((V14-(36*W14))/W14,0)</f>
+        <f>ROUND((X14-(36*Y14))/Y14,0)</f>
         <v>8</v>
       </c>
       <c r="D14" s="52"/>
@@ -2540,33 +2617,35 @@
       <c r="S14" s="12"/>
       <c r="T14" s="42"/>
       <c r="U14" s="12"/>
-      <c r="V14" s="66">
-        <f>F14+J14+L14+N14+P14+R14+T14</f>
+      <c r="V14" s="42"/>
+      <c r="W14" s="12"/>
+      <c r="X14" s="66">
+        <f>F14+J14+L14+N14+P14+R14+T14+V14</f>
         <v>133</v>
       </c>
-      <c r="W14" s="13">
-        <f>COUNTIF(D14:T14,"&gt;30")</f>
+      <c r="Y14" s="13">
+        <f>COUNTIF(D14:V14,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="X14" s="40">
+      <c r="Z14" s="40">
         <v>1</v>
       </c>
-      <c r="Y14" s="12"/>
-      <c r="Z14" s="41">
-        <f>SUMIF(G14:U14, "&lt;30")+X14+Y14</f>
+      <c r="AA14" s="12"/>
+      <c r="AB14" s="41">
+        <f>SUMIF(G14:W14, "&lt;30")+Z14+AA14</f>
         <v>54</v>
       </c>
-      <c r="AA14" s="74">
-        <f>Z14/W14</f>
+      <c r="AC14" s="74">
+        <f>AB14/Y14</f>
         <v>18</v>
       </c>
-      <c r="AB14" s="62"/>
-      <c r="AC14" s="41"/>
-      <c r="AD14" s="41"/>
-      <c r="AE14" s="13"/>
-      <c r="AF14" s="60"/>
+      <c r="AD14" s="62"/>
+      <c r="AE14" s="41"/>
+      <c r="AF14" s="41"/>
+      <c r="AG14" s="13"/>
+      <c r="AH14" s="60"/>
     </row>
-    <row r="15" spans="1:32">
+    <row r="15" spans="1:34">
       <c r="A15" s="9" t="s">
         <v>31</v>
       </c>
@@ -2574,7 +2653,7 @@
         <v>32</v>
       </c>
       <c r="C15" s="11">
-        <f>ROUND((V15-(36*W15))/W15,0)</f>
+        <f>ROUND((X15-(36*Y15))/Y15,0)</f>
         <v>15</v>
       </c>
       <c r="D15" s="52"/>
@@ -2607,258 +2686,274 @@
       <c r="S15" s="12"/>
       <c r="T15" s="14"/>
       <c r="U15" s="12"/>
-      <c r="V15" s="66">
-        <f>F15+J15+L15+N15+P15+R15+T15</f>
+      <c r="V15" s="14"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="66">
+        <f>F15+J15+L15+N15+P15+R15+T15+V15</f>
         <v>154</v>
       </c>
-      <c r="W15" s="13">
-        <f>COUNTIF(D15:T15,"&gt;30")</f>
+      <c r="Y15" s="13">
+        <f>COUNTIF(D15:V15,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="X15" s="40"/>
-      <c r="Y15" s="12"/>
-      <c r="Z15" s="41">
-        <f>SUMIF(G15:U15, "&lt;30")+X15+Y15</f>
+      <c r="Z15" s="40"/>
+      <c r="AA15" s="12"/>
+      <c r="AB15" s="41">
+        <f>SUMIF(G15:W15, "&lt;30")+Z15+AA15</f>
         <v>53</v>
       </c>
-      <c r="AA15" s="74">
-        <f>Z15/W15</f>
+      <c r="AC15" s="74">
+        <f>AB15/Y15</f>
         <v>17.666666666666668</v>
       </c>
-      <c r="AB15" s="62"/>
-      <c r="AC15" s="41"/>
-      <c r="AD15" s="41"/>
-      <c r="AE15" s="13"/>
-      <c r="AF15" s="60"/>
+      <c r="AD15" s="62"/>
+      <c r="AE15" s="41"/>
+      <c r="AF15" s="41"/>
+      <c r="AG15" s="13"/>
+      <c r="AH15" s="60"/>
     </row>
-    <row r="16" spans="1:32">
+    <row r="16" spans="1:34">
       <c r="A16" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C16" s="11">
-        <f>ROUND((V16-(36*W16))/W16,0)</f>
-        <v>18</v>
+        <f>ROUND((X16-(36*Y16))/Y16,0)</f>
+        <v>22</v>
       </c>
       <c r="D16" s="52"/>
       <c r="E16" s="53"/>
-      <c r="F16" s="14">
-        <v>55</v>
+      <c r="F16" s="15">
+        <v>61</v>
       </c>
       <c r="G16" s="12">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H16" s="52"/>
       <c r="I16" s="53"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="14">
+      <c r="J16" s="15">
         <v>56</v>
+      </c>
+      <c r="K16" s="12">
+        <v>19</v>
+      </c>
+      <c r="L16" s="42">
+        <v>60</v>
       </c>
       <c r="M16" s="12">
         <v>15</v>
       </c>
-      <c r="N16" s="14">
-        <v>57</v>
+      <c r="N16" s="42">
+        <v>56</v>
       </c>
       <c r="O16" s="12">
-        <v>14</v>
-      </c>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="12"/>
-      <c r="R16" s="14"/>
+        <v>20</v>
+      </c>
+      <c r="P16" s="42">
+        <v>54</v>
+      </c>
+      <c r="Q16" s="12">
+        <v>22</v>
+      </c>
+      <c r="R16" s="42"/>
       <c r="S16" s="12"/>
-      <c r="T16" s="109">
-        <v>49</v>
+      <c r="T16" s="42">
+        <v>66</v>
       </c>
       <c r="U16" s="12">
+        <v>9</v>
+      </c>
+      <c r="V16" s="42">
+        <v>55</v>
+      </c>
+      <c r="W16" s="12">
         <v>22</v>
       </c>
-      <c r="V16" s="66">
-        <f>F16+J16+L16+N16+P16+R16+T16</f>
-        <v>217</v>
-      </c>
-      <c r="W16" s="13">
-        <f>COUNTIF(D16:T16,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="X16" s="40">
-        <v>1</v>
-      </c>
-      <c r="Y16" s="12"/>
-      <c r="Z16" s="41">
-        <f>SUMIF(G16:U16, "&lt;30")+X16+Y16</f>
-        <v>68</v>
-      </c>
-      <c r="AA16" s="74">
-        <f>Z16/W16</f>
-        <v>17</v>
-      </c>
-      <c r="AB16" s="62"/>
-      <c r="AC16" s="41"/>
-      <c r="AD16" s="41"/>
-      <c r="AE16" s="13"/>
-      <c r="AF16" s="60"/>
+      <c r="X16" s="66">
+        <f>F16+J16+L16+N16+P16+R16+T16+V16</f>
+        <v>408</v>
+      </c>
+      <c r="Y16" s="13">
+        <f>COUNTIF(D16:V16,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="Z16" s="40">
+        <v>2</v>
+      </c>
+      <c r="AA16" s="12"/>
+      <c r="AB16" s="41">
+        <f>SUMIF(G16:W16, "&lt;30")+Z16+AA16</f>
+        <v>123</v>
+      </c>
+      <c r="AC16" s="74">
+        <f>AB16/Y16</f>
+        <v>17.571428571428573</v>
+      </c>
+      <c r="AD16" s="59"/>
+      <c r="AE16" s="41"/>
+      <c r="AF16" s="41"/>
+      <c r="AG16" s="13"/>
+      <c r="AH16" s="60"/>
     </row>
-    <row r="17" spans="1:32">
+    <row r="17" spans="1:34">
       <c r="A17" s="9" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C17" s="11">
-        <f>ROUND((V17-(36*W17))/W17,0)</f>
-        <v>23</v>
+        <f>ROUND((X17-(36*Y17))/Y17,0)</f>
+        <v>11</v>
       </c>
       <c r="D17" s="52"/>
       <c r="E17" s="53"/>
-      <c r="F17" s="15">
-        <v>61</v>
+      <c r="F17" s="14">
+        <v>46</v>
       </c>
       <c r="G17" s="12">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H17" s="52"/>
       <c r="I17" s="53"/>
-      <c r="J17" s="15">
-        <v>56</v>
-      </c>
-      <c r="K17" s="12">
+      <c r="J17" s="14"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="14">
+        <v>46</v>
+      </c>
+      <c r="M17" s="12">
+        <v>18</v>
+      </c>
+      <c r="N17" s="14">
+        <v>46</v>
+      </c>
+      <c r="O17" s="12">
+        <v>18</v>
+      </c>
+      <c r="P17" s="14">
+        <v>46</v>
+      </c>
+      <c r="Q17" s="12">
+        <v>18</v>
+      </c>
+      <c r="R17" s="14">
+        <v>47</v>
+      </c>
+      <c r="S17" s="12">
+        <v>14</v>
+      </c>
+      <c r="T17" s="14">
+        <v>52</v>
+      </c>
+      <c r="U17" s="12">
+        <v>13</v>
+      </c>
+      <c r="V17" s="14"/>
+      <c r="W17" s="12"/>
+      <c r="X17" s="66">
+        <f>F17+J17+L17+N17+P17+R17+T17+V17</f>
+        <v>283</v>
+      </c>
+      <c r="Y17" s="13">
+        <f>COUNTIF(D17:V17,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="Z17" s="43"/>
+      <c r="AA17" s="33"/>
+      <c r="AB17" s="41">
+        <f>SUMIF(G17:W17, "&lt;30")+Z17+AA17</f>
+        <v>99</v>
+      </c>
+      <c r="AC17" s="74">
+        <f>AB17/Y17</f>
+        <v>16.5</v>
+      </c>
+      <c r="AD17" s="62"/>
+      <c r="AE17" s="13"/>
+      <c r="AF17" s="13"/>
+      <c r="AG17" s="13"/>
+      <c r="AH17" s="60"/>
+    </row>
+    <row r="18" spans="1:34">
+      <c r="A18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="11">
+        <f>ROUND((X18-(36*Y18))/Y18,0)</f>
         <v>19</v>
-      </c>
-      <c r="L17" s="42">
-        <v>60</v>
-      </c>
-      <c r="M17" s="12">
-        <v>15</v>
-      </c>
-      <c r="N17" s="42">
-        <v>56</v>
-      </c>
-      <c r="O17" s="12">
-        <v>20</v>
-      </c>
-      <c r="P17" s="42">
-        <v>54</v>
-      </c>
-      <c r="Q17" s="12">
-        <v>22</v>
-      </c>
-      <c r="R17" s="42"/>
-      <c r="S17" s="12"/>
-      <c r="T17" s="42">
-        <v>66</v>
-      </c>
-      <c r="U17" s="12">
-        <v>9</v>
-      </c>
-      <c r="V17" s="66">
-        <f>F17+J17+L17+N17+P17+R17+T17</f>
-        <v>353</v>
-      </c>
-      <c r="W17" s="13">
-        <f>COUNTIF(D17:T17,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="X17" s="40">
-        <v>2</v>
-      </c>
-      <c r="Y17" s="12"/>
-      <c r="Z17" s="41">
-        <f>SUMIF(G17:U17, "&lt;30")+X17+Y17</f>
-        <v>101</v>
-      </c>
-      <c r="AA17" s="74">
-        <f>Z17/W17</f>
-        <v>16.833333333333332</v>
-      </c>
-      <c r="AB17" s="59"/>
-      <c r="AC17" s="41"/>
-      <c r="AD17" s="41"/>
-      <c r="AE17" s="13"/>
-      <c r="AF17" s="60"/>
-    </row>
-    <row r="18" spans="1:32">
-      <c r="A18" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="11">
-        <f>ROUND((V18-(36*W18))/W18,0)</f>
-        <v>11</v>
       </c>
       <c r="D18" s="52"/>
       <c r="E18" s="53"/>
       <c r="F18" s="14">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G18" s="12">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H18" s="52"/>
       <c r="I18" s="53"/>
       <c r="J18" s="14"/>
       <c r="K18" s="12"/>
       <c r="L18" s="14">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="M18" s="12">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="N18" s="14">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="O18" s="12">
-        <v>18</v>
-      </c>
-      <c r="P18" s="14">
-        <v>46</v>
-      </c>
-      <c r="Q18" s="12">
-        <v>18</v>
-      </c>
-      <c r="R18" s="14">
-        <v>47</v>
-      </c>
-      <c r="S18" s="12">
         <v>14</v>
       </c>
-      <c r="T18" s="14">
-        <v>52</v>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="78">
+        <v>49</v>
       </c>
       <c r="U18" s="12">
-        <v>13</v>
-      </c>
-      <c r="V18" s="66">
-        <f>F18+J18+L18+N18+P18+R18+T18</f>
-        <v>283</v>
-      </c>
-      <c r="W18" s="13">
-        <f>COUNTIF(D18:T18,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="X18" s="43"/>
-      <c r="Y18" s="33"/>
-      <c r="Z18" s="41">
-        <f>SUMIF(G18:U18, "&lt;30")+X18+Y18</f>
-        <v>99</v>
-      </c>
-      <c r="AA18" s="74">
-        <f>Z18/W18</f>
-        <v>16.5</v>
-      </c>
-      <c r="AB18" s="62"/>
-      <c r="AC18" s="13"/>
-      <c r="AD18" s="13"/>
-      <c r="AE18" s="13"/>
-      <c r="AF18" s="60"/>
+        <v>22</v>
+      </c>
+      <c r="V18" s="78">
+        <v>58</v>
+      </c>
+      <c r="W18" s="12">
+        <v>14</v>
+      </c>
+      <c r="X18" s="66">
+        <f>F18+J18+L18+N18+P18+R18+T18+V18</f>
+        <v>275</v>
+      </c>
+      <c r="Y18" s="13">
+        <f>COUNTIF(D18:V18,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="Z18" s="40">
+        <v>1</v>
+      </c>
+      <c r="AA18" s="12"/>
+      <c r="AB18" s="41">
+        <f>SUMIF(G18:W18, "&lt;30")+Z18+AA18</f>
+        <v>82</v>
+      </c>
+      <c r="AC18" s="74">
+        <f>AB18/Y18</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="AD18" s="62"/>
+      <c r="AE18" s="41"/>
+      <c r="AF18" s="41"/>
+      <c r="AG18" s="13"/>
+      <c r="AH18" s="60"/>
     </row>
-    <row r="19" spans="1:32">
+    <row r="19" spans="1:34">
       <c r="A19" s="9" t="s">
         <v>22</v>
       </c>
@@ -2890,31 +2985,33 @@
       <c r="S19" s="12"/>
       <c r="T19" s="14"/>
       <c r="U19" s="12"/>
-      <c r="V19" s="66">
-        <f>F19+J19+L19+N19+P19+R19+T19</f>
+      <c r="V19" s="14"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="66">
+        <f>F19+J19+L19+N19+P19+R19+T19+V19</f>
         <v>56</v>
       </c>
-      <c r="W19" s="13">
-        <f>COUNTIF(D19:T19,"&gt;30")</f>
+      <c r="Y19" s="13">
+        <f>COUNTIF(D19:V19,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="X19" s="40"/>
-      <c r="Y19" s="12"/>
-      <c r="Z19" s="41">
-        <f>SUMIF(G19:U19, "&lt;30")+X19+Y19</f>
+      <c r="Z19" s="40"/>
+      <c r="AA19" s="12"/>
+      <c r="AB19" s="41">
+        <f>SUMIF(G19:W19, "&lt;30")+Z19+AA19</f>
         <v>16</v>
       </c>
-      <c r="AA19" s="74">
-        <f>Z19/W19</f>
+      <c r="AC19" s="74">
+        <f>AB19/Y19</f>
         <v>16</v>
       </c>
-      <c r="AB19" s="62"/>
-      <c r="AC19" s="41"/>
-      <c r="AD19" s="41"/>
-      <c r="AE19" s="13"/>
-      <c r="AF19" s="60"/>
+      <c r="AD19" s="62"/>
+      <c r="AE19" s="41"/>
+      <c r="AF19" s="41"/>
+      <c r="AG19" s="13"/>
+      <c r="AH19" s="60"/>
     </row>
-    <row r="20" spans="1:32">
+    <row r="20" spans="1:34">
       <c r="A20" s="9" t="s">
         <v>31</v>
       </c>
@@ -2922,7 +3019,7 @@
         <v>39</v>
       </c>
       <c r="C20" s="11">
-        <f>ROUND((V20-(36*W20))/W20,0)</f>
+        <f>ROUND((X20-(36*Y20))/Y20,0)</f>
         <v>14</v>
       </c>
       <c r="D20" s="52"/>
@@ -2955,31 +3052,33 @@
       <c r="U20" s="12">
         <v>14</v>
       </c>
-      <c r="V20" s="66">
-        <f>F20+J20+L20+N20+P20+R20+T20</f>
+      <c r="V20" s="14"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="66">
+        <f>F20+J20+L20+N20+P20+R20+T20+V20</f>
         <v>150</v>
       </c>
-      <c r="W20" s="13">
-        <f>COUNTIF(D20:T20,"&gt;30")</f>
+      <c r="Y20" s="13">
+        <f>COUNTIF(D20:V20,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="X20" s="40"/>
-      <c r="Y20" s="12"/>
-      <c r="Z20" s="41">
-        <f>SUMIF(G20:U20, "&lt;30")+X20+Y20</f>
+      <c r="Z20" s="40"/>
+      <c r="AA20" s="12"/>
+      <c r="AB20" s="41">
+        <f>SUMIF(G20:W20, "&lt;30")+Z20+AA20</f>
         <v>46</v>
       </c>
-      <c r="AA20" s="74">
-        <f>Z20/W20</f>
+      <c r="AC20" s="74">
+        <f>AB20/Y20</f>
         <v>15.333333333333334</v>
       </c>
-      <c r="AB20" s="59"/>
-      <c r="AC20" s="41"/>
-      <c r="AD20" s="41"/>
-      <c r="AE20" s="13"/>
-      <c r="AF20" s="60"/>
+      <c r="AD20" s="59"/>
+      <c r="AE20" s="41"/>
+      <c r="AF20" s="41"/>
+      <c r="AG20" s="13"/>
+      <c r="AH20" s="60"/>
     </row>
-    <row r="21" spans="1:32">
+    <row r="21" spans="1:34">
       <c r="A21" s="9" t="s">
         <v>49</v>
       </c>
@@ -3009,33 +3108,35 @@
       <c r="S21" s="12"/>
       <c r="T21" s="49"/>
       <c r="U21" s="12"/>
-      <c r="V21" s="66">
-        <f>F21+J21+L21+N21+P21+R21+T21</f>
+      <c r="V21" s="49"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="66">
+        <f>F21+J21+L21+N21+P21+R21+T21+V21</f>
         <v>50</v>
       </c>
-      <c r="W21" s="13">
-        <f>COUNTIF(D21:T21,"&gt;30")</f>
+      <c r="Y21" s="13">
+        <f>COUNTIF(D21:V21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="X21" s="40">
+      <c r="Z21" s="40">
         <v>1</v>
       </c>
-      <c r="Y21" s="12"/>
-      <c r="Z21" s="41">
-        <f>SUMIF(G21:U21, "&lt;30")+X21+Y21</f>
+      <c r="AA21" s="12"/>
+      <c r="AB21" s="41">
+        <f>SUMIF(G21:W21, "&lt;30")+Z21+AA21</f>
         <v>1</v>
       </c>
-      <c r="AA21" s="74">
-        <f>Z21/W21</f>
+      <c r="AC21" s="74">
+        <f>AB21/Y21</f>
         <v>1</v>
       </c>
-      <c r="AB21" s="59"/>
-      <c r="AC21" s="41"/>
-      <c r="AD21" s="41"/>
-      <c r="AE21" s="13"/>
-      <c r="AF21" s="60"/>
+      <c r="AD21" s="59"/>
+      <c r="AE21" s="41"/>
+      <c r="AF21" s="41"/>
+      <c r="AG21" s="13"/>
+      <c r="AH21" s="60"/>
     </row>
-    <row r="22" spans="1:32" ht="17" thickBot="1">
+    <row r="22" spans="1:34" ht="17" thickBot="1">
       <c r="A22" s="18" t="s">
         <v>56</v>
       </c>
@@ -3067,31 +3168,33 @@
       <c r="S22" s="21"/>
       <c r="T22" s="71"/>
       <c r="U22" s="21"/>
-      <c r="V22" s="67">
-        <f>F22+J22+L22+N22+P22+R22+T22</f>
+      <c r="V22" s="71"/>
+      <c r="W22" s="21"/>
+      <c r="X22" s="67">
+        <f>F22+J22+L22+N22+P22+R22+T22+V22</f>
         <v>88</v>
       </c>
-      <c r="W22" s="22">
-        <f>COUNTIF(D22:T22,"&gt;30")</f>
+      <c r="Y22" s="22">
+        <f>COUNTIF(D22:V22,"&gt;30")</f>
         <v>2</v>
       </c>
-      <c r="X22" s="44"/>
-      <c r="Y22" s="21"/>
-      <c r="Z22" s="45">
-        <f>SUMIF(G22:S22, "&lt;30")+X22+Y22</f>
+      <c r="Z22" s="44"/>
+      <c r="AA22" s="21"/>
+      <c r="AB22" s="45">
+        <f>SUMIF(G22:W22, "&lt;30")+Z22+AA22</f>
         <v>0</v>
       </c>
-      <c r="AA22" s="75">
-        <f>Z22/W22</f>
+      <c r="AC22" s="75">
+        <f>AB22/Y22</f>
         <v>0</v>
       </c>
-      <c r="AB22" s="63"/>
-      <c r="AC22" s="45"/>
-      <c r="AD22" s="45"/>
-      <c r="AE22" s="22"/>
-      <c r="AF22" s="64"/>
+      <c r="AD22" s="63"/>
+      <c r="AE22" s="45"/>
+      <c r="AF22" s="45"/>
+      <c r="AG22" s="22"/>
+      <c r="AH22" s="64"/>
     </row>
-    <row r="23" spans="1:32" s="23" customFormat="1" ht="17" thickBot="1">
+    <row r="23" spans="1:34" s="23" customFormat="1" ht="17" thickBot="1">
       <c r="A23" s="34"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -3134,18 +3237,23 @@
         <v>50.333333333333336</v>
       </c>
       <c r="U23" s="36"/>
-      <c r="V23" s="37"/>
+      <c r="V23" s="36">
+        <f>AVERAGEIF(V4:V22,"&gt;0")</f>
+        <v>49</v>
+      </c>
+      <c r="W23" s="36"/>
+      <c r="X23" s="37"/>
     </row>
-    <row r="24" spans="1:32">
+    <row r="24" spans="1:34">
       <c r="C24" s="24"/>
-      <c r="V24" s="25"/>
-      <c r="W24" s="25"/>
-      <c r="X24" s="26"/>
-      <c r="Y24" s="26"/>
-      <c r="Z24" s="25"/>
-      <c r="AA24" s="27"/>
+      <c r="X24" s="25"/>
+      <c r="Y24" s="25"/>
+      <c r="Z24" s="26"/>
+      <c r="AA24" s="26"/>
+      <c r="AB24" s="25"/>
+      <c r="AC24" s="27"/>
     </row>
-    <row r="25" spans="1:32">
+    <row r="25" spans="1:34">
       <c r="C25" s="46" t="s">
         <v>42</v>
       </c>
@@ -3160,8 +3268,9 @@
       <c r="P25" s="28"/>
       <c r="R25" s="28"/>
       <c r="T25" s="28"/>
+      <c r="V25" s="28"/>
     </row>
-    <row r="26" spans="1:32">
+    <row r="26" spans="1:34">
       <c r="C26" s="47" t="s">
         <v>43</v>
       </c>
@@ -3176,9 +3285,10 @@
       <c r="P26" s="29"/>
       <c r="R26" s="29"/>
       <c r="T26" s="29"/>
-      <c r="V26" s="30"/>
+      <c r="V26" s="29"/>
+      <c r="X26" s="30"/>
     </row>
-    <row r="27" spans="1:32">
+    <row r="27" spans="1:34">
       <c r="C27" s="48" t="s">
         <v>47</v>
       </c>
@@ -3202,46 +3312,50 @@
       <c r="S27" s="32"/>
       <c r="T27" s="31"/>
       <c r="U27" s="32"/>
+      <c r="V27" s="31"/>
+      <c r="W27" s="32"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AF22">
-    <sortCondition descending="1" ref="AA4:AA22"/>
-    <sortCondition descending="1" ref="V4:V22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AH24">
+    <sortCondition descending="1" ref="AC4:AC24"/>
+    <sortCondition descending="1" ref="X4:X24"/>
   </sortState>
-  <mergeCells count="33">
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="AB1:AF1"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="V1:V3"/>
-    <mergeCell ref="W1:AA1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
+  <mergeCells count="35">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="X1:X3"/>
+    <mergeCell ref="Y1:AC1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="AD1:AH1"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="AH2:AH3"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="V2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
072125 - updated scores from last week
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A08374-C824-1D4B-B357-6065B8F394EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB35BD0-4E70-974C-9F08-797ACED9DD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44380" yWindow="1480" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="42340" yWindow="1300" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="65">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -229,6 +229,9 @@
   </si>
   <si>
     <t>WEEK 10</t>
+  </si>
+  <si>
+    <t>WEEK 11</t>
   </si>
 </sst>
 </file>
@@ -937,7 +940,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1065,9 +1068,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90"/>
     </xf>
@@ -1123,13 +1123,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1153,20 +1147,83 @@
     <xf numFmtId="1" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1183,80 +1240,23 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1592,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AH27"/>
+  <dimension ref="A1:AJ27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1600,166 +1600,176 @@
     <col min="3" max="3" width="10.1640625" customWidth="1"/>
     <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="17" width="6.33203125" hidden="1" customWidth="1"/>
-    <col min="18" max="23" width="6.33203125" customWidth="1"/>
-    <col min="24" max="24" width="8.83203125" customWidth="1"/>
-    <col min="25" max="25" width="6.1640625" customWidth="1"/>
-    <col min="26" max="26" width="5.83203125" customWidth="1"/>
-    <col min="27" max="27" width="5.6640625" customWidth="1"/>
-    <col min="28" max="28" width="5.5" customWidth="1"/>
-    <col min="29" max="29" width="8" customWidth="1"/>
-    <col min="30" max="30" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="31" max="32" width="6" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="19" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="20" max="23" width="6.33203125" customWidth="1"/>
+    <col min="24" max="24" width="6" customWidth="1"/>
+    <col min="25" max="25" width="6.33203125" customWidth="1"/>
+    <col min="26" max="26" width="8.83203125" customWidth="1"/>
+    <col min="27" max="27" width="6.1640625" customWidth="1"/>
+    <col min="28" max="28" width="5.83203125" customWidth="1"/>
+    <col min="29" max="29" width="5.6640625" customWidth="1"/>
+    <col min="30" max="30" width="5.5" customWidth="1"/>
+    <col min="31" max="31" width="8" customWidth="1"/>
+    <col min="32" max="32" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="33" max="34" width="6" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="57" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="104" t="s">
+    <row r="1" spans="1:36" s="56" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="105"/>
-      <c r="C1" s="110" t="s">
+      <c r="B1" s="78"/>
+      <c r="C1" s="83" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="89" t="s">
+      <c r="D1" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="90"/>
-      <c r="F1" s="89" t="s">
+      <c r="E1" s="86"/>
+      <c r="F1" s="85" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="90"/>
-      <c r="H1" s="89" t="s">
+      <c r="G1" s="86"/>
+      <c r="H1" s="85" t="s">
         <v>45</v>
       </c>
-      <c r="I1" s="90"/>
-      <c r="J1" s="89" t="s">
+      <c r="I1" s="86"/>
+      <c r="J1" s="85" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="90"/>
-      <c r="L1" s="89" t="s">
+      <c r="K1" s="86"/>
+      <c r="L1" s="85" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="90"/>
-      <c r="N1" s="89" t="s">
+      <c r="M1" s="86"/>
+      <c r="N1" s="85" t="s">
         <v>55</v>
       </c>
-      <c r="O1" s="90"/>
-      <c r="P1" s="89" t="s">
+      <c r="O1" s="86"/>
+      <c r="P1" s="85" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="89" t="s">
+      <c r="Q1" s="86"/>
+      <c r="R1" s="85" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="90"/>
-      <c r="T1" s="89" t="s">
+      <c r="S1" s="86"/>
+      <c r="T1" s="85" t="s">
         <v>62</v>
       </c>
-      <c r="U1" s="90"/>
-      <c r="V1" s="89" t="s">
+      <c r="U1" s="86"/>
+      <c r="V1" s="85" t="s">
         <v>63</v>
       </c>
-      <c r="W1" s="90"/>
-      <c r="X1" s="99" t="s">
+      <c r="W1" s="86"/>
+      <c r="X1" s="85" t="s">
+        <v>64</v>
+      </c>
+      <c r="Y1" s="86"/>
+      <c r="Z1" s="97" t="s">
         <v>2</v>
       </c>
-      <c r="Y1" s="101" t="s">
+      <c r="AA1" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="Z1" s="102"/>
-      <c r="AA1" s="102"/>
-      <c r="AB1" s="102"/>
-      <c r="AC1" s="103"/>
-      <c r="AD1" s="84" t="s">
+      <c r="AB1" s="100"/>
+      <c r="AC1" s="100"/>
+      <c r="AD1" s="100"/>
+      <c r="AE1" s="101"/>
+      <c r="AF1" s="102" t="s">
         <v>58</v>
       </c>
-      <c r="AE1" s="85"/>
-      <c r="AF1" s="85"/>
-      <c r="AG1" s="85"/>
-      <c r="AH1" s="86"/>
+      <c r="AG1" s="103"/>
+      <c r="AH1" s="103"/>
+      <c r="AI1" s="103"/>
+      <c r="AJ1" s="104"/>
     </row>
-    <row r="2" spans="1:34" s="57" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="106"/>
-      <c r="B2" s="107"/>
-      <c r="C2" s="111"/>
-      <c r="D2" s="82">
+    <row r="2" spans="1:36" s="56" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="79"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="87">
         <v>45782</v>
       </c>
-      <c r="E2" s="83"/>
-      <c r="F2" s="82">
+      <c r="E2" s="88"/>
+      <c r="F2" s="87">
         <v>45789</v>
       </c>
-      <c r="G2" s="83"/>
-      <c r="H2" s="82">
+      <c r="G2" s="88"/>
+      <c r="H2" s="87">
         <v>45796</v>
       </c>
-      <c r="I2" s="83"/>
-      <c r="J2" s="82">
+      <c r="I2" s="88"/>
+      <c r="J2" s="87">
         <v>45803</v>
       </c>
-      <c r="K2" s="83"/>
-      <c r="L2" s="82">
+      <c r="K2" s="88"/>
+      <c r="L2" s="87">
         <v>45810</v>
       </c>
-      <c r="M2" s="83"/>
-      <c r="N2" s="82">
+      <c r="M2" s="88"/>
+      <c r="N2" s="87">
         <v>45817</v>
       </c>
-      <c r="O2" s="83"/>
-      <c r="P2" s="82">
+      <c r="O2" s="88"/>
+      <c r="P2" s="87">
         <v>45824</v>
       </c>
-      <c r="Q2" s="83"/>
-      <c r="R2" s="82">
+      <c r="Q2" s="88"/>
+      <c r="R2" s="87">
         <v>45831</v>
       </c>
-      <c r="S2" s="83"/>
-      <c r="T2" s="82">
+      <c r="S2" s="88"/>
+      <c r="T2" s="87">
         <v>45838</v>
       </c>
-      <c r="U2" s="83"/>
-      <c r="V2" s="82">
+      <c r="U2" s="88"/>
+      <c r="V2" s="87">
         <v>45845</v>
       </c>
-      <c r="W2" s="83"/>
-      <c r="X2" s="100"/>
-      <c r="Y2" s="99" t="s">
+      <c r="W2" s="88"/>
+      <c r="X2" s="87">
+        <v>45852</v>
+      </c>
+      <c r="Y2" s="88"/>
+      <c r="Z2" s="98"/>
+      <c r="AA2" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="Z2" s="95" t="s">
+      <c r="AB2" s="93" t="s">
         <v>5</v>
       </c>
-      <c r="AA2" s="97" t="s">
+      <c r="AC2" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="AB2" s="91" t="s">
+      <c r="AD2" s="89" t="s">
         <v>7</v>
       </c>
-      <c r="AC2" s="93" t="s">
+      <c r="AE2" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="AD2" s="87" t="s">
+      <c r="AF2" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="AE2" s="87" t="s">
+      <c r="AG2" s="105" t="s">
         <v>5</v>
       </c>
-      <c r="AF2" s="87" t="s">
+      <c r="AH2" s="105" t="s">
         <v>6</v>
       </c>
-      <c r="AG2" s="87" t="s">
+      <c r="AI2" s="105" t="s">
         <v>7</v>
       </c>
-      <c r="AH2" s="87" t="s">
+      <c r="AJ2" s="105" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:34" s="57" customFormat="1" ht="29" customHeight="1" thickBot="1">
-      <c r="A3" s="108"/>
-      <c r="B3" s="109"/>
-      <c r="C3" s="111"/>
+    <row r="3" spans="1:36" s="56" customFormat="1" ht="29" customHeight="1" thickBot="1">
+      <c r="A3" s="81"/>
+      <c r="B3" s="82"/>
+      <c r="C3" s="84"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1820,19 +1830,25 @@
       <c r="W3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="X3" s="100"/>
-      <c r="Y3" s="100"/>
-      <c r="Z3" s="96"/>
+      <c r="X3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="Z3" s="98"/>
       <c r="AA3" s="98"/>
-      <c r="AB3" s="92"/>
-      <c r="AC3" s="94"/>
-      <c r="AD3" s="88"/>
-      <c r="AE3" s="88"/>
-      <c r="AF3" s="88"/>
-      <c r="AG3" s="88"/>
-      <c r="AH3" s="88"/>
+      <c r="AB3" s="94"/>
+      <c r="AC3" s="96"/>
+      <c r="AD3" s="90"/>
+      <c r="AE3" s="92"/>
+      <c r="AF3" s="106"/>
+      <c r="AG3" s="106"/>
+      <c r="AH3" s="106"/>
+      <c r="AI3" s="106"/>
+      <c r="AJ3" s="106"/>
     </row>
-    <row r="4" spans="1:34" ht="16" customHeight="1">
+    <row r="4" spans="1:36" ht="16" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
@@ -1840,15 +1856,15 @@
         <v>38</v>
       </c>
       <c r="C4" s="5">
-        <f>ROUND((X4-(36*Y4))/Y4,0)</f>
+        <f>ROUND((Z4-(36*AA4))/AA4,0)</f>
         <v>10</v>
       </c>
-      <c r="D4" s="50"/>
-      <c r="E4" s="51"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="50"/>
       <c r="F4" s="6"/>
       <c r="G4" s="7"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="51"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="50"/>
       <c r="J4" s="6"/>
       <c r="K4" s="7"/>
       <c r="L4" s="6"/>
@@ -1861,49 +1877,55 @@
       <c r="Q4" s="7">
         <v>26</v>
       </c>
-      <c r="R4" s="76">
+      <c r="R4" s="73">
         <v>45</v>
       </c>
       <c r="S4" s="7">
         <v>24</v>
       </c>
-      <c r="T4" s="77"/>
+      <c r="T4" s="74"/>
       <c r="U4" s="7"/>
-      <c r="V4" s="77">
+      <c r="V4" s="74">
         <v>50</v>
       </c>
       <c r="W4" s="7">
         <v>19</v>
       </c>
-      <c r="X4" s="65">
-        <f>F4+J4+L4+N4+P4+R4+T4+V4</f>
-        <v>138</v>
-      </c>
-      <c r="Y4" s="8">
-        <f>COUNTIF(D4:V4,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="Z4" s="38">
+      <c r="X4" s="74">
+        <v>44</v>
+      </c>
+      <c r="Y4" s="7">
+        <v>20</v>
+      </c>
+      <c r="Z4" s="64">
+        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4</f>
+        <v>182</v>
+      </c>
+      <c r="AA4" s="8">
+        <f>COUNTIF(D4:X4,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AB4" s="38">
         <v>1</v>
       </c>
-      <c r="AA4" s="7">
+      <c r="AC4" s="7">
         <v>1</v>
       </c>
-      <c r="AB4" s="39">
-        <f>SUMIF(G4:W4, "&lt;30")+Z4+AA4</f>
-        <v>71</v>
-      </c>
-      <c r="AC4" s="73">
-        <f>AB4/Y4</f>
-        <v>23.666666666666668</v>
-      </c>
-      <c r="AD4" s="72"/>
-      <c r="AE4" s="39"/>
-      <c r="AF4" s="39"/>
-      <c r="AG4" s="8"/>
-      <c r="AH4" s="58"/>
+      <c r="AD4" s="39">
+        <f>SUMIF(G4:Y4, "&lt;30")+AB4+AC4</f>
+        <v>91</v>
+      </c>
+      <c r="AE4" s="70">
+        <f>AD4/AA4</f>
+        <v>22.75</v>
+      </c>
+      <c r="AF4" s="69"/>
+      <c r="AG4" s="39"/>
+      <c r="AH4" s="39"/>
+      <c r="AI4" s="8"/>
+      <c r="AJ4" s="57"/>
     </row>
-    <row r="5" spans="1:34">
+    <row r="5" spans="1:36">
       <c r="A5" s="9" t="s">
         <v>15</v>
       </c>
@@ -1911,19 +1933,19 @@
         <v>16</v>
       </c>
       <c r="C5" s="11">
-        <f>ROUND((X5-(36*Y5))/Y5,0)</f>
+        <f>ROUND((Z5-(36*AA5))/AA5,0)</f>
         <v>18</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="53"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="52"/>
       <c r="F5" s="14">
         <v>53</v>
       </c>
       <c r="G5" s="12">
         <v>23</v>
       </c>
-      <c r="H5" s="52"/>
-      <c r="I5" s="53"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="52"/>
       <c r="J5" s="14"/>
       <c r="K5" s="12"/>
       <c r="L5" s="14"/>
@@ -1950,737 +1972,791 @@
       </c>
       <c r="V5" s="14"/>
       <c r="W5" s="12"/>
-      <c r="X5" s="66">
-        <f>F5+J5+L5+N5+P5+R5+T5+V5</f>
+      <c r="X5" s="14"/>
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="65">
+        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5</f>
         <v>216</v>
       </c>
-      <c r="Y5" s="13">
-        <f>COUNTIF(D5:V5,"&gt;30")</f>
+      <c r="AA5" s="13">
+        <f>COUNTIF(D5:X5,"&gt;30")</f>
         <v>4</v>
       </c>
-      <c r="Z5" s="40"/>
-      <c r="AA5" s="12"/>
-      <c r="AB5" s="41">
-        <f>SUMIF(G5:W5, "&lt;30")+Z5+AA5</f>
+      <c r="AB5" s="40"/>
+      <c r="AC5" s="12"/>
+      <c r="AD5" s="41">
+        <f>SUMIF(G5:Y5, "&lt;30")+AB5+AC5</f>
         <v>83</v>
       </c>
-      <c r="AC5" s="74">
-        <f>AB5/Y5</f>
+      <c r="AE5" s="71">
+        <f>AD5/AA5</f>
         <v>20.75</v>
       </c>
-      <c r="AD5" s="59"/>
-      <c r="AE5" s="41"/>
-      <c r="AF5" s="41"/>
-      <c r="AG5" s="13"/>
-      <c r="AH5" s="60" t="s">
+      <c r="AF5" s="58"/>
+      <c r="AG5" s="41"/>
+      <c r="AH5" s="41"/>
+      <c r="AI5" s="13"/>
+      <c r="AJ5" s="59" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:34">
+    <row r="6" spans="1:36">
       <c r="A6" s="9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C6" s="11">
-        <f>ROUND((X6-(36*Y6))/Y6,0)</f>
-        <v>13</v>
-      </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="14"/>
+        <v>2</v>
+      </c>
+      <c r="D6" s="51"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="17"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="14">
-        <v>52</v>
-      </c>
-      <c r="K6" s="12">
+      <c r="H6" s="51"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="67">
+        <v>39</v>
+      </c>
+      <c r="Q6" s="12">
         <v>17</v>
       </c>
-      <c r="L6" s="14"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="14">
-        <v>46</v>
-      </c>
-      <c r="O6" s="12">
-        <v>23</v>
-      </c>
-      <c r="P6" s="14">
-        <v>46</v>
-      </c>
-      <c r="Q6" s="12">
-        <v>23</v>
-      </c>
-      <c r="R6" s="14">
-        <v>54</v>
+      <c r="R6" s="67">
+        <v>38</v>
       </c>
       <c r="S6" s="12">
-        <v>16</v>
-      </c>
-      <c r="T6" s="14">
-        <v>45</v>
-      </c>
-      <c r="U6" s="12">
-        <v>23</v>
-      </c>
-      <c r="V6" s="14">
-        <v>48</v>
+        <v>18</v>
+      </c>
+      <c r="T6" s="67"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="76">
+        <v>37</v>
       </c>
       <c r="W6" s="12">
         <v>19</v>
       </c>
-      <c r="X6" s="66">
-        <f>F6+J6+L6+N6+P6+R6+T6+V6</f>
-        <v>291</v>
-      </c>
-      <c r="Y6" s="13">
-        <f>COUNTIF(D6:V6,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="Z6" s="40"/>
-      <c r="AA6" s="12"/>
-      <c r="AB6" s="41">
-        <f>SUMIF(G6:W6, "&lt;30")+Z6+AA6</f>
-        <v>121</v>
-      </c>
-      <c r="AC6" s="74">
-        <f>AB6/Y6</f>
-        <v>20.166666666666668</v>
-      </c>
-      <c r="AD6" s="59"/>
-      <c r="AE6" s="41"/>
-      <c r="AF6" s="41"/>
-      <c r="AG6" s="13"/>
-      <c r="AH6" s="60"/>
+      <c r="X6" s="76">
+        <v>36</v>
+      </c>
+      <c r="Y6" s="12">
+        <v>20</v>
+      </c>
+      <c r="Z6" s="65">
+        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6</f>
+        <v>150</v>
+      </c>
+      <c r="AA6" s="13">
+        <f>COUNTIF(D6:X6,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AB6" s="40">
+        <v>2</v>
+      </c>
+      <c r="AC6" s="12">
+        <v>5</v>
+      </c>
+      <c r="AD6" s="41">
+        <f>SUMIF(G6:Y6, "&lt;30")+AB6+AC6</f>
+        <v>81</v>
+      </c>
+      <c r="AE6" s="71">
+        <f>AD6/AA6</f>
+        <v>20.25</v>
+      </c>
+      <c r="AF6" s="58"/>
+      <c r="AG6" s="41"/>
+      <c r="AH6" s="41"/>
+      <c r="AI6" s="13"/>
+      <c r="AJ6" s="59"/>
     </row>
-    <row r="7" spans="1:34">
+    <row r="7" spans="1:36">
       <c r="A7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="11">
+        <f>ROUND((Z7-(36*AA7))/AA7,0)</f>
         <v>13</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="11">
-        <f>ROUND((X7-(36*Y7))/Y7,0)</f>
-        <v>11</v>
-      </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="79">
-        <v>42</v>
-      </c>
-      <c r="G7" s="12">
-        <v>25</v>
-      </c>
-      <c r="H7" s="52"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="79"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="80">
-        <v>51</v>
-      </c>
-      <c r="M7" s="12">
+      <c r="D7" s="51"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="109"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="51"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="109">
+        <v>52</v>
+      </c>
+      <c r="K7" s="12">
+        <v>17</v>
+      </c>
+      <c r="L7" s="109"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="109">
+        <v>46</v>
+      </c>
+      <c r="O7" s="12">
+        <v>23</v>
+      </c>
+      <c r="P7" s="109">
+        <v>46</v>
+      </c>
+      <c r="Q7" s="12">
+        <v>23</v>
+      </c>
+      <c r="R7" s="109">
+        <v>54</v>
+      </c>
+      <c r="S7" s="12">
         <v>16</v>
       </c>
-      <c r="N7" s="80"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="81">
-        <v>49</v>
-      </c>
-      <c r="Q7" s="12">
-        <v>18</v>
-      </c>
-      <c r="R7" s="80">
-        <v>46</v>
-      </c>
-      <c r="S7" s="12">
-        <v>21</v>
-      </c>
-      <c r="T7" s="80">
+      <c r="T7" s="109">
         <v>45</v>
       </c>
       <c r="U7" s="12">
-        <v>20</v>
-      </c>
-      <c r="V7" s="80">
-        <v>46</v>
+        <v>23</v>
+      </c>
+      <c r="V7" s="109">
+        <v>48</v>
       </c>
       <c r="W7" s="12">
         <v>19</v>
       </c>
-      <c r="X7" s="66">
-        <f>F7+J7+L7+N7+P7+R7+T7+V7</f>
-        <v>279</v>
-      </c>
-      <c r="Y7" s="13">
-        <f>COUNTIF(D7:V7,"&gt;30")</f>
+      <c r="X7" s="109">
+        <v>49</v>
+      </c>
+      <c r="Y7" s="12">
+        <v>18</v>
+      </c>
+      <c r="Z7" s="65">
+        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7</f>
+        <v>340</v>
+      </c>
+      <c r="AA7" s="13">
+        <f>COUNTIF(D7:X7,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AB7" s="40"/>
+      <c r="AC7" s="12"/>
+      <c r="AD7" s="41">
+        <f>SUMIF(G7:Y7, "&lt;30")+AB7+AC7</f>
+        <v>139</v>
+      </c>
+      <c r="AE7" s="71">
+        <f>AD7/AA7</f>
+        <v>19.857142857142858</v>
+      </c>
+      <c r="AF7" s="58"/>
+      <c r="AG7" s="41"/>
+      <c r="AH7" s="41"/>
+      <c r="AI7" s="13"/>
+      <c r="AJ7" s="59"/>
+    </row>
+    <row r="8" spans="1:36">
+      <c r="A8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="11">
+        <f>ROUND((Z8-(36*AA8))/AA8,0)</f>
+        <v>11</v>
+      </c>
+      <c r="D8" s="51"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="42">
+        <v>47</v>
+      </c>
+      <c r="Q8" s="12">
+        <v>20</v>
+      </c>
+      <c r="R8" s="42">
+        <v>50</v>
+      </c>
+      <c r="S8" s="12">
+        <v>17</v>
+      </c>
+      <c r="T8" s="42">
+        <v>46</v>
+      </c>
+      <c r="U8" s="12">
+        <v>21</v>
+      </c>
+      <c r="V8" s="42">
+        <v>47</v>
+      </c>
+      <c r="W8" s="12">
+        <v>19</v>
+      </c>
+      <c r="X8" s="42">
+        <v>44</v>
+      </c>
+      <c r="Y8" s="12">
+        <v>22</v>
+      </c>
+      <c r="Z8" s="65">
+        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8</f>
+        <v>234</v>
+      </c>
+      <c r="AA8" s="13">
+        <f>COUNTIF(D8:X8,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AB8" s="40"/>
+      <c r="AC8" s="12"/>
+      <c r="AD8" s="41">
+        <f>SUMIF(G8:Y8, "&lt;30")+AB8+AC8</f>
+        <v>99</v>
+      </c>
+      <c r="AE8" s="71">
+        <f>AD8/AA8</f>
+        <v>19.8</v>
+      </c>
+      <c r="AF8" s="60"/>
+      <c r="AG8" s="41"/>
+      <c r="AH8" s="41"/>
+      <c r="AI8" s="13"/>
+      <c r="AJ8" s="59"/>
+    </row>
+    <row r="9" spans="1:36">
+      <c r="A9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="11">
+        <f>ROUND((Z9-(36*AA9))/AA9,0)</f>
+        <v>14</v>
+      </c>
+      <c r="D9" s="51"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="14">
+        <v>42</v>
+      </c>
+      <c r="G9" s="12">
+        <v>27</v>
+      </c>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="14">
+        <v>54</v>
+      </c>
+      <c r="M9" s="12">
+        <v>15</v>
+      </c>
+      <c r="N9" s="14"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="14">
+        <v>54</v>
+      </c>
+      <c r="Q9" s="12">
+        <v>16</v>
+      </c>
+      <c r="R9" s="14">
+        <v>53</v>
+      </c>
+      <c r="S9" s="12">
+        <v>16</v>
+      </c>
+      <c r="T9" s="14"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="75">
+        <v>46</v>
+      </c>
+      <c r="W9" s="12">
+        <v>23</v>
+      </c>
+      <c r="X9" s="107">
+        <v>49</v>
+      </c>
+      <c r="Y9" s="12">
+        <v>19</v>
+      </c>
+      <c r="Z9" s="65">
+        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9</f>
+        <v>298</v>
+      </c>
+      <c r="AA9" s="13">
+        <f>COUNTIF(D9:X9,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="Z7" s="40">
-        <v>2</v>
-      </c>
-      <c r="AA7" s="12"/>
-      <c r="AB7" s="41">
-        <f>SUMIF(G7:W7, "&lt;30")+Z7+AA7</f>
-        <v>121</v>
-      </c>
-      <c r="AC7" s="74">
-        <f>AB7/Y7</f>
-        <v>20.166666666666668</v>
-      </c>
-      <c r="AD7" s="59"/>
-      <c r="AE7" s="41"/>
-      <c r="AF7" s="41"/>
-      <c r="AG7" s="13"/>
-      <c r="AH7" s="60"/>
+      <c r="AB9" s="40">
+        <v>1</v>
+      </c>
+      <c r="AC9" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD9" s="41">
+        <f>SUMIF(G9:Y9, "&lt;30")+AB9+AC9</f>
+        <v>118</v>
+      </c>
+      <c r="AE9" s="71">
+        <f>AD9/AA9</f>
+        <v>19.666666666666668</v>
+      </c>
+      <c r="AF9" s="58"/>
+      <c r="AG9" s="41"/>
+      <c r="AH9" s="41"/>
+      <c r="AI9" s="13"/>
+      <c r="AJ9" s="59"/>
     </row>
-    <row r="8" spans="1:34">
-      <c r="A8" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="11">
-        <f>ROUND((X8-(36*Y8))/Y8,0)</f>
+    <row r="10" spans="1:36">
+      <c r="A10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="11">
+        <f>ROUND((Z10-(36*AA10))/AA10,0)</f>
+        <v>7</v>
+      </c>
+      <c r="D10" s="51"/>
+      <c r="E10" s="52"/>
+      <c r="F10" s="14">
+        <v>41</v>
+      </c>
+      <c r="G10" s="12">
+        <v>21</v>
+      </c>
+      <c r="H10" s="51"/>
+      <c r="I10" s="52"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="55">
+        <v>48</v>
+      </c>
+      <c r="O10" s="12">
         <v>14</v>
       </c>
-      <c r="D8" s="52"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="14">
-        <v>42</v>
-      </c>
-      <c r="G8" s="12">
-        <v>27</v>
-      </c>
-      <c r="H8" s="52"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="14">
-        <v>54</v>
-      </c>
-      <c r="M8" s="12">
-        <v>15</v>
-      </c>
-      <c r="N8" s="14"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="14">
-        <v>54</v>
-      </c>
-      <c r="Q8" s="12">
-        <v>16</v>
-      </c>
-      <c r="R8" s="14">
-        <v>53</v>
-      </c>
-      <c r="S8" s="12">
-        <v>16</v>
-      </c>
-      <c r="T8" s="14"/>
-      <c r="U8" s="12"/>
-      <c r="V8" s="78">
-        <v>46</v>
-      </c>
-      <c r="W8" s="12">
-        <v>23</v>
-      </c>
-      <c r="X8" s="66">
-        <f>F8+J8+L8+N8+P8+R8+T8+V8</f>
-        <v>249</v>
-      </c>
-      <c r="Y8" s="13">
-        <f>COUNTIF(D8:V8,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="Z8" s="40">
+      <c r="P10" s="42">
+        <v>44</v>
+      </c>
+      <c r="Q10" s="12">
+        <v>18</v>
+      </c>
+      <c r="R10" s="42"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="42"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="42"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="15">
+        <v>40</v>
+      </c>
+      <c r="Y10" s="12">
+        <v>22</v>
+      </c>
+      <c r="Z10" s="65">
+        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10</f>
+        <v>173</v>
+      </c>
+      <c r="AA10" s="13">
+        <f>COUNTIF(D10:X10,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AB10" s="40">
         <v>1</v>
       </c>
-      <c r="AA8" s="12"/>
-      <c r="AB8" s="41">
-        <f>SUMIF(G8:W8, "&lt;30")+Z8+AA8</f>
-        <v>98</v>
-      </c>
-      <c r="AC8" s="74">
-        <f>AB8/Y8</f>
-        <v>19.600000000000001</v>
-      </c>
-      <c r="AD8" s="61"/>
-      <c r="AE8" s="41"/>
-      <c r="AF8" s="41"/>
-      <c r="AG8" s="13"/>
-      <c r="AH8" s="60"/>
+      <c r="AC10" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD10" s="41">
+        <f>SUMIF(G10:Y10, "&lt;30")+AB10+AC10</f>
+        <v>77</v>
+      </c>
+      <c r="AE10" s="71">
+        <f>AD10/AA10</f>
+        <v>19.25</v>
+      </c>
+      <c r="AF10" s="112"/>
+      <c r="AG10" s="41"/>
+      <c r="AH10" s="41"/>
+      <c r="AI10" s="13"/>
+      <c r="AJ10" s="59"/>
     </row>
-    <row r="9" spans="1:34">
-      <c r="A9" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="11">
-        <v>2</v>
-      </c>
-      <c r="D9" s="52"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="53"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="68">
-        <v>39</v>
-      </c>
-      <c r="Q9" s="12">
-        <v>17</v>
-      </c>
-      <c r="R9" s="68">
-        <v>38</v>
-      </c>
-      <c r="S9" s="12">
-        <v>18</v>
-      </c>
-      <c r="T9" s="68"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="112">
-        <v>37</v>
-      </c>
-      <c r="W9" s="12">
-        <v>19</v>
-      </c>
-      <c r="X9" s="66">
-        <f>F9+J9+L9+N9+P9+R9+T9+V9</f>
-        <v>114</v>
-      </c>
-      <c r="Y9" s="13">
-        <f>COUNTIF(D9:V9,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="Z9" s="40">
-        <v>1</v>
-      </c>
-      <c r="AA9" s="12">
-        <v>3</v>
-      </c>
-      <c r="AB9" s="41">
-        <f>SUMIF(G9:W9, "&lt;30")+Z9+AA9</f>
-        <v>58</v>
-      </c>
-      <c r="AC9" s="74">
-        <f>AB9/Y9</f>
-        <v>19.333333333333332</v>
-      </c>
-      <c r="AD9" s="59"/>
-      <c r="AE9" s="41"/>
-      <c r="AF9" s="41"/>
-      <c r="AG9" s="13"/>
-      <c r="AH9" s="60"/>
-    </row>
-    <row r="10" spans="1:34">
-      <c r="A10" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="11">
-        <f>ROUND((X10-(36*Y10))/Y10,0)</f>
-        <v>12</v>
-      </c>
-      <c r="D10" s="52"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="52"/>
-      <c r="I10" s="53"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="42">
-        <v>47</v>
-      </c>
-      <c r="Q10" s="12">
-        <v>20</v>
-      </c>
-      <c r="R10" s="42">
-        <v>50</v>
-      </c>
-      <c r="S10" s="12">
-        <v>17</v>
-      </c>
-      <c r="T10" s="42">
-        <v>46</v>
-      </c>
-      <c r="U10" s="12">
-        <v>21</v>
-      </c>
-      <c r="V10" s="42">
-        <v>47</v>
-      </c>
-      <c r="W10" s="12">
-        <v>19</v>
-      </c>
-      <c r="X10" s="66">
-        <f>F10+J10+L10+N10+P10+R10+T10+V10</f>
-        <v>190</v>
-      </c>
-      <c r="Y10" s="13">
-        <f>COUNTIF(D10:V10,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="Z10" s="40"/>
-      <c r="AA10" s="12"/>
-      <c r="AB10" s="41">
-        <f>SUMIF(G10:W10, "&lt;30")+Z10+AA10</f>
-        <v>77</v>
-      </c>
-      <c r="AC10" s="74">
-        <f>AB10/Y10</f>
-        <v>19.25</v>
-      </c>
-      <c r="AD10" s="113"/>
-      <c r="AE10" s="41"/>
-      <c r="AF10" s="41"/>
-      <c r="AG10" s="13"/>
-      <c r="AH10" s="60"/>
-    </row>
-    <row r="11" spans="1:34">
+    <row r="11" spans="1:36">
       <c r="A11" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="11">
+        <f>ROUND((Z11-(36*AA11))/AA11,0)</f>
+        <v>11</v>
+      </c>
+      <c r="D11" s="51"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="108">
+        <v>42</v>
+      </c>
+      <c r="G11" s="12">
+        <v>25</v>
+      </c>
+      <c r="H11" s="51"/>
+      <c r="I11" s="52"/>
+      <c r="J11" s="108"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="42">
+        <v>51</v>
+      </c>
+      <c r="M11" s="12">
+        <v>16</v>
+      </c>
+      <c r="N11" s="42"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="15">
+        <v>49</v>
+      </c>
+      <c r="Q11" s="12">
+        <v>18</v>
+      </c>
+      <c r="R11" s="42">
+        <v>46</v>
+      </c>
+      <c r="S11" s="12">
+        <v>21</v>
+      </c>
+      <c r="T11" s="42">
+        <v>45</v>
+      </c>
+      <c r="U11" s="12">
+        <v>20</v>
+      </c>
+      <c r="V11" s="42">
+        <v>46</v>
+      </c>
+      <c r="W11" s="12">
+        <v>19</v>
+      </c>
+      <c r="X11" s="42">
+        <v>53</v>
+      </c>
+      <c r="Y11" s="12">
+        <v>13</v>
+      </c>
+      <c r="Z11" s="65">
+        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11</f>
+        <v>332</v>
+      </c>
+      <c r="AA11" s="13">
+        <f>COUNTIF(D11:X11,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AB11" s="40">
+        <v>2</v>
+      </c>
+      <c r="AC11" s="12"/>
+      <c r="AD11" s="41">
+        <f>SUMIF(G11:Y11, "&lt;30")+AB11+AC11</f>
+        <v>134</v>
+      </c>
+      <c r="AE11" s="71">
+        <f>AD11/AA11</f>
+        <v>19.142857142857142</v>
+      </c>
+      <c r="AF11" s="58"/>
+      <c r="AG11" s="41"/>
+      <c r="AH11" s="41"/>
+      <c r="AI11" s="13"/>
+      <c r="AJ11" s="59"/>
+    </row>
+    <row r="12" spans="1:36">
+      <c r="A12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="11">
-        <f>ROUND((X11-(36*Y11))/Y11,0)</f>
+      <c r="C12" s="11">
+        <f>ROUND((Z12-(36*AA12))/AA12,0)</f>
         <v>8</v>
       </c>
-      <c r="D11" s="52"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="70">
+      <c r="D12" s="51"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="68">
         <v>45</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G12" s="12">
         <v>17</v>
       </c>
-      <c r="H11" s="52"/>
-      <c r="I11" s="53"/>
-      <c r="J11" s="70"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="70">
+      <c r="H12" s="51"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="68"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="68">
         <v>43</v>
       </c>
-      <c r="M11" s="12">
+      <c r="M12" s="12">
         <v>19</v>
       </c>
-      <c r="N11" s="15">
+      <c r="N12" s="15">
         <v>41</v>
       </c>
-      <c r="O11" s="12">
+      <c r="O12" s="12">
         <v>21</v>
       </c>
-      <c r="P11" s="42">
+      <c r="P12" s="42">
         <v>47</v>
       </c>
-      <c r="Q11" s="12">
+      <c r="Q12" s="12">
         <v>15</v>
       </c>
-      <c r="R11" s="42">
+      <c r="R12" s="42">
         <v>42</v>
       </c>
-      <c r="S11" s="12">
+      <c r="S12" s="12">
         <v>20</v>
       </c>
-      <c r="T11" s="42">
+      <c r="T12" s="42">
         <v>43</v>
       </c>
-      <c r="U11" s="12">
+      <c r="U12" s="12">
         <v>19</v>
       </c>
-      <c r="V11" s="42">
+      <c r="V12" s="42">
         <v>44</v>
       </c>
-      <c r="W11" s="12">
+      <c r="W12" s="12">
         <v>18</v>
       </c>
-      <c r="X11" s="66">
-        <f>F11+J11+L11+N11+P11+R11+T11+V11</f>
-        <v>305</v>
-      </c>
-      <c r="Y11" s="13">
-        <f>COUNTIF(D11:V11,"&gt;30")</f>
-        <v>7</v>
-      </c>
-      <c r="Z11" s="40">
+      <c r="X12" s="42">
+        <v>48</v>
+      </c>
+      <c r="Y12" s="12">
+        <v>16</v>
+      </c>
+      <c r="Z12" s="65">
+        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12</f>
+        <v>353</v>
+      </c>
+      <c r="AA12" s="13">
+        <f>COUNTIF(D12:X12,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AB12" s="40">
         <v>1</v>
       </c>
-      <c r="AA11" s="12">
-        <v>3</v>
-      </c>
-      <c r="AB11" s="41">
-        <f>SUMIF(G11:W11, "&lt;30")+Z11+AA11</f>
-        <v>133</v>
-      </c>
-      <c r="AC11" s="74">
-        <f>AB11/Y11</f>
-        <v>19</v>
-      </c>
-      <c r="AD11" s="59"/>
-      <c r="AE11" s="41"/>
-      <c r="AF11" s="41"/>
-      <c r="AG11" s="13"/>
-      <c r="AH11" s="60"/>
+      <c r="AC12" s="12">
+        <v>4</v>
+      </c>
+      <c r="AD12" s="41">
+        <f>SUMIF(G12:Y12, "&lt;30")+AB12+AC12</f>
+        <v>150</v>
+      </c>
+      <c r="AE12" s="71">
+        <f>AD12/AA12</f>
+        <v>18.75</v>
+      </c>
+      <c r="AF12" s="58"/>
+      <c r="AG12" s="41"/>
+      <c r="AH12" s="41"/>
+      <c r="AI12" s="13"/>
+      <c r="AJ12" s="59"/>
     </row>
-    <row r="12" spans="1:34">
-      <c r="A12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="11">
-        <f>ROUND((X12-(36*Y12))/Y12,0)</f>
-        <v>8</v>
-      </c>
-      <c r="D12" s="52"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="14">
-        <v>46</v>
-      </c>
-      <c r="G12" s="12">
-        <v>16</v>
-      </c>
-      <c r="H12" s="52"/>
-      <c r="I12" s="53"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="14">
-        <v>42</v>
-      </c>
-      <c r="O12" s="12">
-        <v>20</v>
-      </c>
-      <c r="P12" s="14">
-        <v>43</v>
-      </c>
-      <c r="Q12" s="12">
-        <v>19</v>
-      </c>
-      <c r="R12" s="14"/>
-      <c r="S12" s="12"/>
-      <c r="T12" s="14"/>
-      <c r="U12" s="12"/>
-      <c r="V12" s="14"/>
-      <c r="W12" s="12"/>
-      <c r="X12" s="66">
-        <f>F12+J12+L12+N12+P12+R12+T12+V12</f>
-        <v>131</v>
-      </c>
-      <c r="Y12" s="13">
-        <f>COUNTIF(D12:V12,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="Z12" s="40"/>
-      <c r="AA12" s="12">
-        <v>1</v>
-      </c>
-      <c r="AB12" s="41">
-        <f>SUMIF(G12:W12, "&lt;30")+Z12+AA12</f>
-        <v>56</v>
-      </c>
-      <c r="AC12" s="74">
-        <f>AB12/Y12</f>
-        <v>18.666666666666668</v>
-      </c>
-      <c r="AD12" s="62"/>
-      <c r="AE12" s="41"/>
-      <c r="AF12" s="41"/>
-      <c r="AG12" s="13"/>
-      <c r="AH12" s="60"/>
-    </row>
-    <row r="13" spans="1:34">
+    <row r="13" spans="1:36">
       <c r="A13" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="11">
+        <f>ROUND((Z13-(36*AA13))/AA13,0)</f>
+        <v>15</v>
+      </c>
+      <c r="D13" s="51"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="14">
+        <v>51</v>
+      </c>
+      <c r="G13" s="12">
         <v>18</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="11">
-        <v>22</v>
-      </c>
-      <c r="D13" s="52"/>
-      <c r="E13" s="53"/>
-      <c r="F13" s="14">
-        <v>59</v>
-      </c>
-      <c r="G13" s="12">
-        <v>17</v>
-      </c>
-      <c r="H13" s="52"/>
-      <c r="I13" s="53"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="52"/>
       <c r="J13" s="14"/>
       <c r="K13" s="12"/>
       <c r="L13" s="14"/>
       <c r="M13" s="12"/>
-      <c r="N13" s="14"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="14"/>
-      <c r="Q13" s="12"/>
-      <c r="R13" s="14">
-        <v>55</v>
-      </c>
-      <c r="S13" s="12">
-        <v>21</v>
-      </c>
+      <c r="N13" s="14">
+        <v>51</v>
+      </c>
+      <c r="O13" s="12">
+        <v>18</v>
+      </c>
+      <c r="P13" s="14">
+        <v>52</v>
+      </c>
+      <c r="Q13" s="12">
+        <v>17</v>
+      </c>
+      <c r="R13" s="14"/>
+      <c r="S13" s="12"/>
       <c r="T13" s="14"/>
       <c r="U13" s="12"/>
-      <c r="V13" s="14">
+      <c r="V13" s="14"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="14">
+        <v>48</v>
+      </c>
+      <c r="Y13" s="12">
+        <v>21</v>
+      </c>
+      <c r="Z13" s="65">
+        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13</f>
+        <v>202</v>
+      </c>
+      <c r="AA13" s="13">
+        <f>COUNTIF(D13:X13,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AB13" s="40"/>
+      <c r="AC13" s="12"/>
+      <c r="AD13" s="41">
+        <f>SUMIF(G13:Y13, "&lt;30")+AB13+AC13</f>
+        <v>74</v>
+      </c>
+      <c r="AE13" s="71">
+        <f>AD13/AA13</f>
+        <v>18.5</v>
+      </c>
+      <c r="AF13" s="61"/>
+      <c r="AG13" s="41"/>
+      <c r="AH13" s="41"/>
+      <c r="AI13" s="13"/>
+      <c r="AJ13" s="59"/>
+    </row>
+    <row r="14" spans="1:36">
+      <c r="A14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="11">
+        <v>22</v>
+      </c>
+      <c r="D14" s="51"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="14">
         <v>59</v>
       </c>
-      <c r="W13" s="12">
+      <c r="G14" s="12">
         <v>17</v>
       </c>
-      <c r="X13" s="66">
-        <f>F13+J13+L13+N13+P13+R13+T13+V13</f>
-        <v>173</v>
-      </c>
-      <c r="Y13" s="13">
-        <f>COUNTIF(D13:V13,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="Z13" s="40"/>
-      <c r="AA13" s="12"/>
-      <c r="AB13" s="41">
-        <f>SUMIF(G13:W13, "&lt;30")+Z13+AA13</f>
-        <v>55</v>
-      </c>
-      <c r="AC13" s="74">
-        <f>AB13/Y13</f>
-        <v>18.333333333333332</v>
-      </c>
-      <c r="AD13" s="62"/>
-      <c r="AE13" s="41"/>
-      <c r="AF13" s="41"/>
-      <c r="AG13" s="13"/>
-      <c r="AH13" s="60"/>
-    </row>
-    <row r="14" spans="1:34">
-      <c r="A14" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="11">
-        <f>ROUND((X14-(36*Y14))/Y14,0)</f>
-        <v>8</v>
-      </c>
-      <c r="D14" s="52"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="14">
-        <v>41</v>
-      </c>
-      <c r="G14" s="12">
-        <v>21</v>
-      </c>
-      <c r="H14" s="52"/>
-      <c r="I14" s="53"/>
+      <c r="H14" s="51"/>
+      <c r="I14" s="52"/>
       <c r="J14" s="14"/>
       <c r="K14" s="12"/>
       <c r="L14" s="14"/>
       <c r="M14" s="12"/>
-      <c r="N14" s="56">
-        <v>48</v>
-      </c>
-      <c r="O14" s="12">
-        <v>14</v>
-      </c>
-      <c r="P14" s="42">
-        <v>44</v>
-      </c>
-      <c r="Q14" s="12">
-        <v>18</v>
-      </c>
-      <c r="R14" s="42"/>
-      <c r="S14" s="12"/>
-      <c r="T14" s="42"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="14"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="14">
+        <v>55</v>
+      </c>
+      <c r="S14" s="12">
+        <v>21</v>
+      </c>
+      <c r="T14" s="14"/>
       <c r="U14" s="12"/>
-      <c r="V14" s="42"/>
-      <c r="W14" s="12"/>
-      <c r="X14" s="66">
-        <f>F14+J14+L14+N14+P14+R14+T14+V14</f>
-        <v>133</v>
-      </c>
-      <c r="Y14" s="13">
-        <f>COUNTIF(D14:V14,"&gt;30")</f>
+      <c r="V14" s="14">
+        <v>59</v>
+      </c>
+      <c r="W14" s="12">
+        <v>17</v>
+      </c>
+      <c r="X14" s="14"/>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="65">
+        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14</f>
+        <v>173</v>
+      </c>
+      <c r="AA14" s="13">
+        <f>COUNTIF(D14:X14,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="Z14" s="40">
-        <v>1</v>
-      </c>
-      <c r="AA14" s="12"/>
-      <c r="AB14" s="41">
-        <f>SUMIF(G14:W14, "&lt;30")+Z14+AA14</f>
-        <v>54</v>
-      </c>
-      <c r="AC14" s="74">
-        <f>AB14/Y14</f>
-        <v>18</v>
-      </c>
-      <c r="AD14" s="62"/>
-      <c r="AE14" s="41"/>
-      <c r="AF14" s="41"/>
-      <c r="AG14" s="13"/>
-      <c r="AH14" s="60"/>
+      <c r="AB14" s="40"/>
+      <c r="AC14" s="12"/>
+      <c r="AD14" s="41">
+        <f>SUMIF(G14:Y14, "&lt;30")+AB14+AC14</f>
+        <v>55</v>
+      </c>
+      <c r="AE14" s="71">
+        <f>AD14/AA14</f>
+        <v>18.333333333333332</v>
+      </c>
+      <c r="AF14" s="61"/>
+      <c r="AG14" s="41"/>
+      <c r="AH14" s="41"/>
+      <c r="AI14" s="13"/>
+      <c r="AJ14" s="59"/>
     </row>
-    <row r="15" spans="1:34">
+    <row r="15" spans="1:36">
       <c r="A15" s="9" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C15" s="11">
-        <f>ROUND((X15-(36*Y15))/Y15,0)</f>
-        <v>15</v>
-      </c>
-      <c r="D15" s="52"/>
-      <c r="E15" s="53"/>
+        <f>ROUND((Z15-(36*AA15))/AA15,0)</f>
+        <v>9</v>
+      </c>
+      <c r="D15" s="51"/>
+      <c r="E15" s="52"/>
       <c r="F15" s="14">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G15" s="12">
-        <v>18</v>
-      </c>
-      <c r="H15" s="52"/>
-      <c r="I15" s="53"/>
+        <v>16</v>
+      </c>
+      <c r="H15" s="51"/>
+      <c r="I15" s="52"/>
       <c r="J15" s="14"/>
       <c r="K15" s="12"/>
       <c r="L15" s="14"/>
       <c r="M15" s="12"/>
       <c r="N15" s="14">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="O15" s="12">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="P15" s="14">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="Q15" s="12">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="R15" s="14"/>
       <c r="S15" s="12"/>
@@ -2688,195 +2764,196 @@
       <c r="U15" s="12"/>
       <c r="V15" s="14"/>
       <c r="W15" s="12"/>
-      <c r="X15" s="66">
-        <f>F15+J15+L15+N15+P15+R15+T15+V15</f>
-        <v>154</v>
-      </c>
-      <c r="Y15" s="13">
-        <f>COUNTIF(D15:V15,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="Z15" s="40"/>
-      <c r="AA15" s="12"/>
-      <c r="AB15" s="41">
-        <f>SUMIF(G15:W15, "&lt;30")+Z15+AA15</f>
-        <v>53</v>
-      </c>
-      <c r="AC15" s="74">
-        <f>AB15/Y15</f>
-        <v>17.666666666666668</v>
-      </c>
-      <c r="AD15" s="62"/>
-      <c r="AE15" s="41"/>
-      <c r="AF15" s="41"/>
-      <c r="AG15" s="13"/>
-      <c r="AH15" s="60"/>
+      <c r="X15" s="14">
+        <v>47</v>
+      </c>
+      <c r="Y15" s="12">
+        <v>16</v>
+      </c>
+      <c r="Z15" s="65">
+        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15</f>
+        <v>178</v>
+      </c>
+      <c r="AA15" s="13">
+        <f>COUNTIF(D15:X15,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AB15" s="40"/>
+      <c r="AC15" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD15" s="41">
+        <f>SUMIF(G15:Y15, "&lt;30")+AB15+AC15</f>
+        <v>72</v>
+      </c>
+      <c r="AE15" s="71">
+        <f>AD15/AA15</f>
+        <v>18</v>
+      </c>
+      <c r="AF15" s="61"/>
+      <c r="AG15" s="41"/>
+      <c r="AH15" s="41"/>
+      <c r="AI15" s="13"/>
+      <c r="AJ15" s="59"/>
     </row>
-    <row r="16" spans="1:34">
+    <row r="16" spans="1:36">
       <c r="A16" s="9" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="C16" s="11">
-        <f>ROUND((X16-(36*Y16))/Y16,0)</f>
-        <v>22</v>
-      </c>
-      <c r="D16" s="52"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="15">
-        <v>61</v>
-      </c>
-      <c r="G16" s="12">
-        <v>14</v>
-      </c>
-      <c r="H16" s="52"/>
-      <c r="I16" s="53"/>
-      <c r="J16" s="15">
-        <v>56</v>
-      </c>
-      <c r="K16" s="12">
-        <v>19</v>
-      </c>
-      <c r="L16" s="42">
-        <v>60</v>
-      </c>
-      <c r="M16" s="12">
-        <v>15</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="D16" s="51"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="51"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="12"/>
       <c r="N16" s="42">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="O16" s="12">
+        <v>18</v>
+      </c>
+      <c r="P16" s="42">
+        <v>43</v>
+      </c>
+      <c r="Q16" s="12">
         <v>20</v>
-      </c>
-      <c r="P16" s="42">
-        <v>54</v>
-      </c>
-      <c r="Q16" s="12">
-        <v>22</v>
       </c>
       <c r="R16" s="42"/>
       <c r="S16" s="12"/>
-      <c r="T16" s="42">
+      <c r="T16" s="42"/>
+      <c r="U16" s="12"/>
+      <c r="V16" s="42"/>
+      <c r="W16" s="12"/>
+      <c r="X16" s="42">
+        <v>48</v>
+      </c>
+      <c r="Y16" s="12">
+        <v>15</v>
+      </c>
+      <c r="Z16" s="65">
+        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16</f>
+        <v>136</v>
+      </c>
+      <c r="AA16" s="13">
+        <f>COUNTIF(D16:X16,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="AB16" s="40"/>
+      <c r="AC16" s="12">
+        <v>1</v>
+      </c>
+      <c r="AD16" s="41">
+        <f>SUMIF(G16:Y16, "&lt;30")+AB16+AC16</f>
+        <v>54</v>
+      </c>
+      <c r="AE16" s="71">
+        <f>AD16/AA16</f>
+        <v>18</v>
+      </c>
+      <c r="AF16" s="58"/>
+      <c r="AG16" s="41"/>
+      <c r="AH16" s="41"/>
+      <c r="AI16" s="13"/>
+      <c r="AJ16" s="59"/>
+    </row>
+    <row r="17" spans="1:36">
+      <c r="A17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="11">
+        <f>ROUND((Z17-(36*AA17))/AA17,0)</f>
+        <v>22</v>
+      </c>
+      <c r="D17" s="51"/>
+      <c r="E17" s="52"/>
+      <c r="F17" s="15">
+        <v>61</v>
+      </c>
+      <c r="G17" s="12">
+        <v>14</v>
+      </c>
+      <c r="H17" s="51"/>
+      <c r="I17" s="52"/>
+      <c r="J17" s="15">
+        <v>56</v>
+      </c>
+      <c r="K17" s="12">
+        <v>19</v>
+      </c>
+      <c r="L17" s="42">
+        <v>60</v>
+      </c>
+      <c r="M17" s="12">
+        <v>15</v>
+      </c>
+      <c r="N17" s="42">
+        <v>56</v>
+      </c>
+      <c r="O17" s="12">
+        <v>20</v>
+      </c>
+      <c r="P17" s="42">
+        <v>54</v>
+      </c>
+      <c r="Q17" s="12">
+        <v>22</v>
+      </c>
+      <c r="R17" s="42"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="42">
         <v>66</v>
       </c>
-      <c r="U16" s="12">
+      <c r="U17" s="12">
         <v>9</v>
       </c>
-      <c r="V16" s="42">
+      <c r="V17" s="42">
         <v>55</v>
       </c>
-      <c r="W16" s="12">
+      <c r="W17" s="12">
         <v>22</v>
       </c>
-      <c r="X16" s="66">
-        <f>F16+J16+L16+N16+P16+R16+T16+V16</f>
+      <c r="X17" s="42"/>
+      <c r="Y17" s="12"/>
+      <c r="Z17" s="65">
+        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17</f>
         <v>408</v>
       </c>
-      <c r="Y16" s="13">
-        <f>COUNTIF(D16:V16,"&gt;30")</f>
+      <c r="AA17" s="13">
+        <f>COUNTIF(D17:X17,"&gt;30")</f>
         <v>7</v>
       </c>
-      <c r="Z16" s="40">
+      <c r="AB17" s="40">
         <v>2</v>
       </c>
-      <c r="AA16" s="12"/>
-      <c r="AB16" s="41">
-        <f>SUMIF(G16:W16, "&lt;30")+Z16+AA16</f>
+      <c r="AC17" s="12"/>
+      <c r="AD17" s="41">
+        <f>SUMIF(G17:Y17, "&lt;30")+AB17+AC17</f>
         <v>123</v>
       </c>
-      <c r="AC16" s="74">
-        <f>AB16/Y16</f>
+      <c r="AE17" s="71">
+        <f>AD17/AA17</f>
         <v>17.571428571428573</v>
       </c>
-      <c r="AD16" s="59"/>
-      <c r="AE16" s="41"/>
-      <c r="AF16" s="41"/>
-      <c r="AG16" s="13"/>
-      <c r="AH16" s="60"/>
+      <c r="AF17" s="58"/>
+      <c r="AG17" s="41"/>
+      <c r="AH17" s="41"/>
+      <c r="AI17" s="13"/>
+      <c r="AJ17" s="59"/>
     </row>
-    <row r="17" spans="1:34">
-      <c r="A17" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="11">
-        <f>ROUND((X17-(36*Y17))/Y17,0)</f>
-        <v>11</v>
-      </c>
-      <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="14">
-        <v>46</v>
-      </c>
-      <c r="G17" s="12">
-        <v>18</v>
-      </c>
-      <c r="H17" s="52"/>
-      <c r="I17" s="53"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="14">
-        <v>46</v>
-      </c>
-      <c r="M17" s="12">
-        <v>18</v>
-      </c>
-      <c r="N17" s="14">
-        <v>46</v>
-      </c>
-      <c r="O17" s="12">
-        <v>18</v>
-      </c>
-      <c r="P17" s="14">
-        <v>46</v>
-      </c>
-      <c r="Q17" s="12">
-        <v>18</v>
-      </c>
-      <c r="R17" s="14">
-        <v>47</v>
-      </c>
-      <c r="S17" s="12">
-        <v>14</v>
-      </c>
-      <c r="T17" s="14">
-        <v>52</v>
-      </c>
-      <c r="U17" s="12">
-        <v>13</v>
-      </c>
-      <c r="V17" s="14"/>
-      <c r="W17" s="12"/>
-      <c r="X17" s="66">
-        <f>F17+J17+L17+N17+P17+R17+T17+V17</f>
-        <v>283</v>
-      </c>
-      <c r="Y17" s="13">
-        <f>COUNTIF(D17:V17,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="Z17" s="43"/>
-      <c r="AA17" s="33"/>
-      <c r="AB17" s="41">
-        <f>SUMIF(G17:W17, "&lt;30")+Z17+AA17</f>
-        <v>99</v>
-      </c>
-      <c r="AC17" s="74">
-        <f>AB17/Y17</f>
-        <v>16.5</v>
-      </c>
-      <c r="AD17" s="62"/>
-      <c r="AE17" s="13"/>
-      <c r="AF17" s="13"/>
-      <c r="AG17" s="13"/>
-      <c r="AH17" s="60"/>
-    </row>
-    <row r="18" spans="1:34">
+    <row r="18" spans="1:36">
       <c r="A18" s="9" t="s">
         <v>21</v>
       </c>
@@ -2884,19 +2961,19 @@
         <v>16</v>
       </c>
       <c r="C18" s="11">
-        <f>ROUND((X18-(36*Y18))/Y18,0)</f>
-        <v>19</v>
-      </c>
-      <c r="D18" s="52"/>
-      <c r="E18" s="53"/>
+        <f>ROUND((Z18-(36*AA18))/AA18,0)</f>
+        <v>18</v>
+      </c>
+      <c r="D18" s="51"/>
+      <c r="E18" s="52"/>
       <c r="F18" s="14">
         <v>55</v>
       </c>
       <c r="G18" s="12">
         <v>16</v>
       </c>
-      <c r="H18" s="52"/>
-      <c r="I18" s="53"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="52"/>
       <c r="J18" s="14"/>
       <c r="K18" s="12"/>
       <c r="L18" s="14">
@@ -2915,103 +2992,132 @@
       <c r="Q18" s="12"/>
       <c r="R18" s="14"/>
       <c r="S18" s="12"/>
-      <c r="T18" s="78">
+      <c r="T18" s="75">
         <v>49</v>
       </c>
       <c r="U18" s="12">
         <v>22</v>
       </c>
-      <c r="V18" s="78">
+      <c r="V18" s="75">
         <v>58</v>
       </c>
       <c r="W18" s="12">
         <v>14</v>
       </c>
-      <c r="X18" s="66">
-        <f>F18+J18+L18+N18+P18+R18+T18+V18</f>
-        <v>275</v>
-      </c>
-      <c r="Y18" s="13">
-        <f>COUNTIF(D18:V18,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="Z18" s="40">
+      <c r="X18" s="107">
+        <v>50</v>
+      </c>
+      <c r="Y18" s="12">
+        <v>23</v>
+      </c>
+      <c r="Z18" s="65">
+        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18</f>
+        <v>325</v>
+      </c>
+      <c r="AA18" s="13">
+        <f>COUNTIF(D18:X18,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AB18" s="40">
         <v>1</v>
       </c>
-      <c r="AA18" s="12"/>
-      <c r="AB18" s="41">
-        <f>SUMIF(G18:W18, "&lt;30")+Z18+AA18</f>
-        <v>82</v>
-      </c>
-      <c r="AC18" s="74">
-        <f>AB18/Y18</f>
-        <v>16.399999999999999</v>
-      </c>
-      <c r="AD18" s="62"/>
-      <c r="AE18" s="41"/>
-      <c r="AF18" s="41"/>
-      <c r="AG18" s="13"/>
-      <c r="AH18" s="60"/>
+      <c r="AC18" s="12"/>
+      <c r="AD18" s="41">
+        <f>SUMIF(G18:Y18, "&lt;30")+AB18+AC18</f>
+        <v>105</v>
+      </c>
+      <c r="AE18" s="71">
+        <f>AD18/AA18</f>
+        <v>17.5</v>
+      </c>
+      <c r="AF18" s="61"/>
+      <c r="AG18" s="41"/>
+      <c r="AH18" s="41"/>
+      <c r="AI18" s="13"/>
+      <c r="AJ18" s="59"/>
     </row>
-    <row r="19" spans="1:34">
+    <row r="19" spans="1:36">
       <c r="A19" s="9" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C19" s="11">
+        <f>ROUND((Z19-(36*AA19))/AA19,0)</f>
+        <v>11</v>
+      </c>
+      <c r="D19" s="51"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="14">
+        <v>46</v>
+      </c>
+      <c r="G19" s="12">
         <v>18</v>
       </c>
-      <c r="D19" s="52"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="14">
-        <v>56</v>
-      </c>
-      <c r="G19" s="12">
-        <v>16</v>
-      </c>
-      <c r="H19" s="52"/>
-      <c r="I19" s="53"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="52"/>
       <c r="J19" s="14"/>
       <c r="K19" s="12"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="12"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="12"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="12"/>
-      <c r="R19" s="14"/>
-      <c r="S19" s="12"/>
-      <c r="T19" s="14"/>
-      <c r="U19" s="12"/>
+      <c r="L19" s="14">
+        <v>46</v>
+      </c>
+      <c r="M19" s="12">
+        <v>18</v>
+      </c>
+      <c r="N19" s="14">
+        <v>46</v>
+      </c>
+      <c r="O19" s="12">
+        <v>18</v>
+      </c>
+      <c r="P19" s="14">
+        <v>46</v>
+      </c>
+      <c r="Q19" s="12">
+        <v>18</v>
+      </c>
+      <c r="R19" s="14">
+        <v>47</v>
+      </c>
+      <c r="S19" s="12">
+        <v>14</v>
+      </c>
+      <c r="T19" s="14">
+        <v>52</v>
+      </c>
+      <c r="U19" s="12">
+        <v>13</v>
+      </c>
       <c r="V19" s="14"/>
       <c r="W19" s="12"/>
-      <c r="X19" s="66">
-        <f>F19+J19+L19+N19+P19+R19+T19+V19</f>
-        <v>56</v>
-      </c>
-      <c r="Y19" s="13">
-        <f>COUNTIF(D19:V19,"&gt;30")</f>
-        <v>1</v>
-      </c>
-      <c r="Z19" s="40"/>
-      <c r="AA19" s="12"/>
-      <c r="AB19" s="41">
-        <f>SUMIF(G19:W19, "&lt;30")+Z19+AA19</f>
-        <v>16</v>
-      </c>
-      <c r="AC19" s="74">
-        <f>AB19/Y19</f>
-        <v>16</v>
-      </c>
-      <c r="AD19" s="62"/>
-      <c r="AE19" s="41"/>
-      <c r="AF19" s="41"/>
+      <c r="X19" s="14"/>
+      <c r="Y19" s="12"/>
+      <c r="Z19" s="65">
+        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19</f>
+        <v>283</v>
+      </c>
+      <c r="AA19" s="13">
+        <f>COUNTIF(D19:X19,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AB19" s="43"/>
+      <c r="AC19" s="33"/>
+      <c r="AD19" s="41">
+        <f>SUMIF(G19:Y19, "&lt;30")+AB19+AC19</f>
+        <v>99</v>
+      </c>
+      <c r="AE19" s="71">
+        <f>AD19/AA19</f>
+        <v>16.5</v>
+      </c>
+      <c r="AF19" s="61"/>
       <c r="AG19" s="13"/>
-      <c r="AH19" s="60"/>
+      <c r="AH19" s="13"/>
+      <c r="AI19" s="13"/>
+      <c r="AJ19" s="59"/>
     </row>
-    <row r="20" spans="1:34">
+    <row r="20" spans="1:36">
       <c r="A20" s="9" t="s">
         <v>31</v>
       </c>
@@ -3019,15 +3125,15 @@
         <v>39</v>
       </c>
       <c r="C20" s="11">
-        <f>ROUND((X20-(36*Y20))/Y20,0)</f>
+        <f>ROUND((Z20-(36*AA20))/AA20,0)</f>
         <v>14</v>
       </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="53"/>
+      <c r="D20" s="51"/>
+      <c r="E20" s="52"/>
       <c r="F20" s="14"/>
       <c r="G20" s="12"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="53"/>
+      <c r="H20" s="51"/>
+      <c r="I20" s="52"/>
       <c r="J20" s="14"/>
       <c r="K20" s="12"/>
       <c r="L20" s="14"/>
@@ -3054,147 +3160,157 @@
       </c>
       <c r="V20" s="14"/>
       <c r="W20" s="12"/>
-      <c r="X20" s="66">
-        <f>F20+J20+L20+N20+P20+R20+T20+V20</f>
-        <v>150</v>
-      </c>
-      <c r="Y20" s="13">
-        <f>COUNTIF(D20:V20,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="Z20" s="40"/>
-      <c r="AA20" s="12"/>
-      <c r="AB20" s="41">
-        <f>SUMIF(G20:W20, "&lt;30")+Z20+AA20</f>
-        <v>46</v>
-      </c>
-      <c r="AC20" s="74">
-        <f>AB20/Y20</f>
-        <v>15.333333333333334</v>
-      </c>
-      <c r="AD20" s="59"/>
-      <c r="AE20" s="41"/>
-      <c r="AF20" s="41"/>
-      <c r="AG20" s="13"/>
-      <c r="AH20" s="60"/>
+      <c r="X20" s="14">
+        <v>48</v>
+      </c>
+      <c r="Y20" s="12">
+        <v>20</v>
+      </c>
+      <c r="Z20" s="65">
+        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20</f>
+        <v>198</v>
+      </c>
+      <c r="AA20" s="13">
+        <f>COUNTIF(D20:X20,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AB20" s="40"/>
+      <c r="AC20" s="12"/>
+      <c r="AD20" s="41">
+        <f>SUMIF(G20:Y20, "&lt;30")+AB20+AC20</f>
+        <v>66</v>
+      </c>
+      <c r="AE20" s="71">
+        <f>AD20/AA20</f>
+        <v>16.5</v>
+      </c>
+      <c r="AF20" s="58"/>
+      <c r="AG20" s="41"/>
+      <c r="AH20" s="41"/>
+      <c r="AI20" s="13"/>
+      <c r="AJ20" s="59"/>
     </row>
-    <row r="21" spans="1:34">
+    <row r="21" spans="1:36">
       <c r="A21" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="11">
+        <v>18</v>
+      </c>
+      <c r="D21" s="51"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="14">
+        <v>56</v>
+      </c>
+      <c r="G21" s="12">
+        <v>16</v>
+      </c>
+      <c r="H21" s="51"/>
+      <c r="I21" s="52"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="14"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="14"/>
+      <c r="U21" s="12"/>
+      <c r="V21" s="14"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="14"/>
+      <c r="Y21" s="12"/>
+      <c r="Z21" s="65">
+        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21</f>
+        <v>56</v>
+      </c>
+      <c r="AA21" s="13">
+        <f>COUNTIF(D21:X21,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="AB21" s="40"/>
+      <c r="AC21" s="12"/>
+      <c r="AD21" s="41">
+        <f>SUMIF(G21:Y21, "&lt;30")+AB21+AC21</f>
+        <v>16</v>
+      </c>
+      <c r="AE21" s="71">
+        <f>AD21/AA21</f>
+        <v>16</v>
+      </c>
+      <c r="AF21" s="61"/>
+      <c r="AG21" s="41"/>
+      <c r="AH21" s="41"/>
+      <c r="AI21" s="13"/>
+      <c r="AJ21" s="59"/>
+    </row>
+    <row r="22" spans="1:36" ht="17" thickBot="1">
+      <c r="A22" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B22" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="52"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="49">
-        <v>50</v>
-      </c>
-      <c r="M21" s="12"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="12"/>
-      <c r="P21" s="49"/>
-      <c r="Q21" s="12"/>
-      <c r="R21" s="49"/>
-      <c r="S21" s="12"/>
-      <c r="T21" s="49"/>
-      <c r="U21" s="12"/>
-      <c r="V21" s="49"/>
-      <c r="W21" s="12"/>
-      <c r="X21" s="66">
-        <f>F21+J21+L21+N21+P21+R21+T21+V21</f>
-        <v>50</v>
-      </c>
-      <c r="Y21" s="13">
-        <f>COUNTIF(D21:V21,"&gt;30")</f>
-        <v>1</v>
-      </c>
-      <c r="Z21" s="40">
-        <v>1</v>
-      </c>
-      <c r="AA21" s="12"/>
-      <c r="AB21" s="41">
-        <f>SUMIF(G21:W21, "&lt;30")+Z21+AA21</f>
-        <v>1</v>
-      </c>
-      <c r="AC21" s="74">
-        <f>AB21/Y21</f>
-        <v>1</v>
-      </c>
-      <c r="AD21" s="59"/>
-      <c r="AE21" s="41"/>
-      <c r="AF21" s="41"/>
-      <c r="AG21" s="13"/>
-      <c r="AH21" s="60"/>
-    </row>
-    <row r="22" spans="1:34" ht="17" thickBot="1">
-      <c r="A22" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>57</v>
       </c>
       <c r="C22" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="54"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="69"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="110"/>
       <c r="G22" s="21"/>
-      <c r="H22" s="54"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="69"/>
+      <c r="H22" s="53"/>
+      <c r="I22" s="54"/>
+      <c r="J22" s="110"/>
       <c r="K22" s="21"/>
-      <c r="L22" s="69"/>
+      <c r="L22" s="111">
+        <v>50</v>
+      </c>
       <c r="M22" s="21"/>
-      <c r="N22" s="71">
-        <v>45</v>
-      </c>
+      <c r="N22" s="111"/>
       <c r="O22" s="21"/>
-      <c r="P22" s="71">
-        <v>43</v>
-      </c>
+      <c r="P22" s="111"/>
       <c r="Q22" s="21"/>
-      <c r="R22" s="71"/>
+      <c r="R22" s="111"/>
       <c r="S22" s="21"/>
-      <c r="T22" s="71"/>
+      <c r="T22" s="111"/>
       <c r="U22" s="21"/>
-      <c r="V22" s="71"/>
+      <c r="V22" s="111"/>
       <c r="W22" s="21"/>
-      <c r="X22" s="67">
-        <f>F22+J22+L22+N22+P22+R22+T22+V22</f>
-        <v>88</v>
-      </c>
-      <c r="Y22" s="22">
-        <f>COUNTIF(D22:V22,"&gt;30")</f>
-        <v>2</v>
-      </c>
-      <c r="Z22" s="44"/>
-      <c r="AA22" s="21"/>
-      <c r="AB22" s="45">
-        <f>SUMIF(G22:W22, "&lt;30")+Z22+AA22</f>
-        <v>0</v>
-      </c>
-      <c r="AC22" s="75">
-        <f>AB22/Y22</f>
-        <v>0</v>
-      </c>
-      <c r="AD22" s="63"/>
-      <c r="AE22" s="45"/>
-      <c r="AF22" s="45"/>
-      <c r="AG22" s="22"/>
-      <c r="AH22" s="64"/>
+      <c r="X22" s="111"/>
+      <c r="Y22" s="21"/>
+      <c r="Z22" s="66">
+        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22</f>
+        <v>50</v>
+      </c>
+      <c r="AA22" s="22">
+        <f>COUNTIF(D22:X22,"&gt;30")</f>
+        <v>1</v>
+      </c>
+      <c r="AB22" s="44">
+        <v>1</v>
+      </c>
+      <c r="AC22" s="21"/>
+      <c r="AD22" s="45">
+        <f>SUMIF(G22:Y22, "&lt;30")+AB22+AC22</f>
+        <v>1</v>
+      </c>
+      <c r="AE22" s="72">
+        <f>AD22/AA22</f>
+        <v>1</v>
+      </c>
+      <c r="AF22" s="62"/>
+      <c r="AG22" s="45"/>
+      <c r="AH22" s="45"/>
+      <c r="AI22" s="22"/>
+      <c r="AJ22" s="63"/>
     </row>
-    <row r="23" spans="1:34" s="23" customFormat="1" ht="17" thickBot="1">
+    <row r="23" spans="1:36" s="23" customFormat="1" ht="17" thickBot="1">
       <c r="A23" s="34"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -3242,18 +3358,23 @@
         <v>49</v>
       </c>
       <c r="W23" s="36"/>
-      <c r="X23" s="37"/>
+      <c r="X23" s="36">
+        <f>AVERAGEIF(X4:X22,"&gt;0")</f>
+        <v>46.46153846153846</v>
+      </c>
+      <c r="Y23" s="36"/>
+      <c r="Z23" s="37"/>
     </row>
-    <row r="24" spans="1:34">
+    <row r="24" spans="1:36">
       <c r="C24" s="24"/>
-      <c r="X24" s="25"/>
-      <c r="Y24" s="25"/>
-      <c r="Z24" s="26"/>
-      <c r="AA24" s="26"/>
-      <c r="AB24" s="25"/>
-      <c r="AC24" s="27"/>
+      <c r="Z24" s="25"/>
+      <c r="AA24" s="25"/>
+      <c r="AB24" s="26"/>
+      <c r="AC24" s="26"/>
+      <c r="AD24" s="25"/>
+      <c r="AE24" s="27"/>
     </row>
-    <row r="25" spans="1:34">
+    <row r="25" spans="1:36">
       <c r="C25" s="46" t="s">
         <v>42</v>
       </c>
@@ -3269,8 +3390,9 @@
       <c r="R25" s="28"/>
       <c r="T25" s="28"/>
       <c r="V25" s="28"/>
+      <c r="X25" s="28"/>
     </row>
-    <row r="26" spans="1:34">
+    <row r="26" spans="1:36">
       <c r="C26" s="47" t="s">
         <v>43</v>
       </c>
@@ -3286,9 +3408,10 @@
       <c r="R26" s="29"/>
       <c r="T26" s="29"/>
       <c r="V26" s="29"/>
-      <c r="X26" s="30"/>
+      <c r="X26" s="29"/>
+      <c r="Z26" s="30"/>
     </row>
-    <row r="27" spans="1:34">
+    <row r="27" spans="1:36">
       <c r="C27" s="48" t="s">
         <v>47</v>
       </c>
@@ -3314,48 +3437,52 @@
       <c r="U27" s="32"/>
       <c r="V27" s="31"/>
       <c r="W27" s="32"/>
+      <c r="X27" s="31"/>
+      <c r="Y27" s="32"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AH24">
-    <sortCondition descending="1" ref="AC4:AC24"/>
-    <sortCondition descending="1" ref="X4:X24"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AJ22">
+    <sortCondition descending="1" ref="AE4:AE22"/>
+    <sortCondition descending="1" ref="Z4:Z22"/>
   </sortState>
-  <mergeCells count="35">
+  <mergeCells count="37">
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="AF1:AJ1"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="AH2:AH3"/>
+    <mergeCell ref="AI2:AI3"/>
+    <mergeCell ref="AJ2:AJ3"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="AB2:AB3"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="Z1:Z3"/>
+    <mergeCell ref="AA1:AE1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="X1:X3"/>
-    <mergeCell ref="Y1:AC1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="AD1:AH1"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="AH2:AH3"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="V2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
072225 - updated scores for week 12
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB35BD0-4E70-974C-9F08-797ACED9DD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CAE5E90-48E5-B34A-9959-1B4C679045F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42340" yWindow="1300" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="42640" yWindow="1260" windowWidth="26740" windowHeight="18140" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="66">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>Total Strokes</t>
-  </si>
-  <si>
-    <t>FIRST HALF (11 Rounds)</t>
   </si>
   <si>
     <t>Rounds Played</t>
@@ -232,6 +229,12 @@
   </si>
   <si>
     <t>WEEK 11</t>
+  </si>
+  <si>
+    <t>WEEK 12</t>
+  </si>
+  <si>
+    <t>OVERALL</t>
   </si>
 </sst>
 </file>
@@ -940,7 +943,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1150,6 +1153,90 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1174,89 +1261,14 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1592,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AJ27"/>
+  <dimension ref="A1:AL27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1600,263 +1612,279 @@
     <col min="3" max="3" width="10.1640625" customWidth="1"/>
     <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="19" width="6.33203125" hidden="1" customWidth="1"/>
-    <col min="20" max="23" width="6.33203125" customWidth="1"/>
+    <col min="12" max="21" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="22" max="23" width="6.33203125" customWidth="1"/>
     <col min="24" max="24" width="6" customWidth="1"/>
     <col min="25" max="25" width="6.33203125" customWidth="1"/>
-    <col min="26" max="26" width="8.83203125" customWidth="1"/>
-    <col min="27" max="27" width="6.1640625" customWidth="1"/>
-    <col min="28" max="28" width="5.83203125" customWidth="1"/>
-    <col min="29" max="29" width="5.6640625" customWidth="1"/>
-    <col min="30" max="30" width="5.5" customWidth="1"/>
-    <col min="31" max="31" width="8" customWidth="1"/>
-    <col min="32" max="32" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="33" max="34" width="6" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="36" max="36" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="6" customWidth="1"/>
+    <col min="27" max="27" width="6.33203125" customWidth="1"/>
+    <col min="28" max="28" width="8.83203125" customWidth="1"/>
+    <col min="29" max="29" width="6.1640625" customWidth="1"/>
+    <col min="30" max="30" width="5.83203125" customWidth="1"/>
+    <col min="31" max="31" width="5.6640625" customWidth="1"/>
+    <col min="32" max="32" width="5.5" customWidth="1"/>
+    <col min="33" max="33" width="8" customWidth="1"/>
+    <col min="34" max="34" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="35" max="36" width="6" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="38" max="38" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="56" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="77" t="s">
+    <row r="1" spans="1:38" s="56" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="83" t="s">
+      <c r="B1" s="106"/>
+      <c r="C1" s="111" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="90" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="91"/>
+      <c r="F1" s="90" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="91"/>
+      <c r="H1" s="90" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="91"/>
+      <c r="J1" s="90" t="s">
+        <v>45</v>
+      </c>
+      <c r="K1" s="91"/>
+      <c r="L1" s="90" t="s">
+        <v>47</v>
+      </c>
+      <c r="M1" s="91"/>
+      <c r="N1" s="90" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="85" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="86"/>
-      <c r="F1" s="85" t="s">
-        <v>44</v>
-      </c>
-      <c r="G1" s="86"/>
-      <c r="H1" s="85" t="s">
-        <v>45</v>
-      </c>
-      <c r="I1" s="86"/>
-      <c r="J1" s="85" t="s">
-        <v>46</v>
-      </c>
-      <c r="K1" s="86"/>
-      <c r="L1" s="85" t="s">
-        <v>48</v>
-      </c>
-      <c r="M1" s="86"/>
-      <c r="N1" s="85" t="s">
-        <v>55</v>
-      </c>
-      <c r="O1" s="86"/>
-      <c r="P1" s="85" t="s">
+      <c r="O1" s="91"/>
+      <c r="P1" s="90" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="90" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="86"/>
-      <c r="R1" s="85" t="s">
+      <c r="S1" s="91"/>
+      <c r="T1" s="90" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="86"/>
-      <c r="T1" s="85" t="s">
+      <c r="U1" s="91"/>
+      <c r="V1" s="90" t="s">
         <v>62</v>
       </c>
-      <c r="U1" s="86"/>
-      <c r="V1" s="85" t="s">
+      <c r="W1" s="91"/>
+      <c r="X1" s="90" t="s">
         <v>63</v>
       </c>
-      <c r="W1" s="86"/>
-      <c r="X1" s="85" t="s">
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="90" t="s">
         <v>64</v>
       </c>
-      <c r="Y1" s="86"/>
-      <c r="Z1" s="97" t="s">
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="AA1" s="99" t="s">
+      <c r="AC1" s="102" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD1" s="103"/>
+      <c r="AE1" s="103"/>
+      <c r="AF1" s="103"/>
+      <c r="AG1" s="104"/>
+      <c r="AH1" s="85" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI1" s="86"/>
+      <c r="AJ1" s="86"/>
+      <c r="AK1" s="86"/>
+      <c r="AL1" s="87"/>
+    </row>
+    <row r="2" spans="1:38" s="56" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="107"/>
+      <c r="B2" s="108"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="83">
+        <v>45782</v>
+      </c>
+      <c r="E2" s="84"/>
+      <c r="F2" s="83">
+        <v>45789</v>
+      </c>
+      <c r="G2" s="84"/>
+      <c r="H2" s="83">
+        <v>45796</v>
+      </c>
+      <c r="I2" s="84"/>
+      <c r="J2" s="83">
+        <v>45803</v>
+      </c>
+      <c r="K2" s="84"/>
+      <c r="L2" s="83">
+        <v>45810</v>
+      </c>
+      <c r="M2" s="84"/>
+      <c r="N2" s="83">
+        <v>45817</v>
+      </c>
+      <c r="O2" s="84"/>
+      <c r="P2" s="83">
+        <v>45824</v>
+      </c>
+      <c r="Q2" s="84"/>
+      <c r="R2" s="83">
+        <v>45831</v>
+      </c>
+      <c r="S2" s="84"/>
+      <c r="T2" s="83">
+        <v>45838</v>
+      </c>
+      <c r="U2" s="84"/>
+      <c r="V2" s="83">
+        <v>45845</v>
+      </c>
+      <c r="W2" s="84"/>
+      <c r="X2" s="83">
+        <v>45852</v>
+      </c>
+      <c r="Y2" s="84"/>
+      <c r="Z2" s="83">
+        <v>45859</v>
+      </c>
+      <c r="AA2" s="84"/>
+      <c r="AB2" s="101"/>
+      <c r="AC2" s="100" t="s">
         <v>3</v>
       </c>
-      <c r="AB1" s="100"/>
-      <c r="AC1" s="100"/>
-      <c r="AD1" s="100"/>
-      <c r="AE1" s="101"/>
-      <c r="AF1" s="102" t="s">
-        <v>58</v>
-      </c>
-      <c r="AG1" s="103"/>
-      <c r="AH1" s="103"/>
-      <c r="AI1" s="103"/>
-      <c r="AJ1" s="104"/>
+      <c r="AD2" s="96" t="s">
+        <v>4</v>
+      </c>
+      <c r="AE2" s="98" t="s">
+        <v>5</v>
+      </c>
+      <c r="AF2" s="92" t="s">
+        <v>6</v>
+      </c>
+      <c r="AG2" s="94" t="s">
+        <v>7</v>
+      </c>
+      <c r="AH2" s="88" t="s">
+        <v>3</v>
+      </c>
+      <c r="AI2" s="88" t="s">
+        <v>4</v>
+      </c>
+      <c r="AJ2" s="88" t="s">
+        <v>5</v>
+      </c>
+      <c r="AK2" s="88" t="s">
+        <v>6</v>
+      </c>
+      <c r="AL2" s="88" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:36" s="56" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="79"/>
-      <c r="B2" s="80"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="87">
-        <v>45782</v>
-      </c>
-      <c r="E2" s="88"/>
-      <c r="F2" s="87">
-        <v>45789</v>
-      </c>
-      <c r="G2" s="88"/>
-      <c r="H2" s="87">
-        <v>45796</v>
-      </c>
-      <c r="I2" s="88"/>
-      <c r="J2" s="87">
-        <v>45803</v>
-      </c>
-      <c r="K2" s="88"/>
-      <c r="L2" s="87">
-        <v>45810</v>
-      </c>
-      <c r="M2" s="88"/>
-      <c r="N2" s="87">
-        <v>45817</v>
-      </c>
-      <c r="O2" s="88"/>
-      <c r="P2" s="87">
-        <v>45824</v>
-      </c>
-      <c r="Q2" s="88"/>
-      <c r="R2" s="87">
-        <v>45831</v>
-      </c>
-      <c r="S2" s="88"/>
-      <c r="T2" s="87">
-        <v>45838</v>
-      </c>
-      <c r="U2" s="88"/>
-      <c r="V2" s="87">
-        <v>45845</v>
-      </c>
-      <c r="W2" s="88"/>
-      <c r="X2" s="87">
-        <v>45852</v>
-      </c>
-      <c r="Y2" s="88"/>
-      <c r="Z2" s="98"/>
-      <c r="AA2" s="97" t="s">
-        <v>4</v>
-      </c>
-      <c r="AB2" s="93" t="s">
-        <v>5</v>
-      </c>
-      <c r="AC2" s="95" t="s">
-        <v>6</v>
-      </c>
-      <c r="AD2" s="89" t="s">
-        <v>7</v>
-      </c>
-      <c r="AE2" s="91" t="s">
+    <row r="3" spans="1:38" s="56" customFormat="1" ht="29" customHeight="1" thickBot="1">
+      <c r="A3" s="109"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="AF2" s="105" t="s">
-        <v>4</v>
-      </c>
-      <c r="AG2" s="105" t="s">
-        <v>5</v>
-      </c>
-      <c r="AH2" s="105" t="s">
-        <v>6</v>
-      </c>
-      <c r="AI2" s="105" t="s">
-        <v>7</v>
-      </c>
-      <c r="AJ2" s="105" t="s">
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB3" s="101"/>
+      <c r="AC3" s="101"/>
+      <c r="AD3" s="97"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="93"/>
+      <c r="AG3" s="95"/>
+      <c r="AH3" s="89"/>
+      <c r="AI3" s="89"/>
+      <c r="AJ3" s="89"/>
+      <c r="AK3" s="89"/>
+      <c r="AL3" s="89"/>
     </row>
-    <row r="3" spans="1:36" s="56" customFormat="1" ht="29" customHeight="1" thickBot="1">
-      <c r="A3" s="81"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="84"/>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="Z3" s="98"/>
-      <c r="AA3" s="98"/>
-      <c r="AB3" s="94"/>
-      <c r="AC3" s="96"/>
-      <c r="AD3" s="90"/>
-      <c r="AE3" s="92"/>
-      <c r="AF3" s="106"/>
-      <c r="AG3" s="106"/>
-      <c r="AH3" s="106"/>
-      <c r="AI3" s="106"/>
-      <c r="AJ3" s="106"/>
-    </row>
-    <row r="4" spans="1:36" ht="16" customHeight="1">
+    <row r="4" spans="1:38" ht="16" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="C4" s="5">
-        <f>ROUND((Z4-(36*AA4))/AA4,0)</f>
+        <f>ROUND((AB4-(36*AC4))/AC4,0)</f>
         <v>10</v>
       </c>
       <c r="D4" s="49"/>
@@ -1897,43 +1925,45 @@
       <c r="Y4" s="7">
         <v>20</v>
       </c>
-      <c r="Z4" s="64">
-        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4</f>
+      <c r="Z4" s="74"/>
+      <c r="AA4" s="113"/>
+      <c r="AB4" s="64">
+        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4</f>
         <v>182</v>
       </c>
-      <c r="AA4" s="8">
-        <f>COUNTIF(D4:X4,"&gt;30")</f>
+      <c r="AC4" s="8">
+        <f>COUNTIF(D4:Z4,"&gt;30")</f>
         <v>4</v>
       </c>
-      <c r="AB4" s="38">
+      <c r="AD4" s="38">
         <v>1</v>
       </c>
-      <c r="AC4" s="7">
+      <c r="AE4" s="7">
         <v>1</v>
       </c>
-      <c r="AD4" s="39">
-        <f>SUMIF(G4:Y4, "&lt;30")+AB4+AC4</f>
+      <c r="AF4" s="39">
+        <f>SUMIF(G4:AA4, "&lt;30")+AD4+AE4</f>
         <v>91</v>
       </c>
-      <c r="AE4" s="70">
-        <f>AD4/AA4</f>
+      <c r="AG4" s="70">
+        <f>AF4/AC4</f>
         <v>22.75</v>
       </c>
-      <c r="AF4" s="69"/>
-      <c r="AG4" s="39"/>
-      <c r="AH4" s="39"/>
-      <c r="AI4" s="8"/>
-      <c r="AJ4" s="57"/>
+      <c r="AH4" s="69"/>
+      <c r="AI4" s="39"/>
+      <c r="AJ4" s="39"/>
+      <c r="AK4" s="8"/>
+      <c r="AL4" s="57"/>
     </row>
-    <row r="5" spans="1:36">
+    <row r="5" spans="1:38">
       <c r="A5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>16</v>
-      </c>
       <c r="C5" s="11">
-        <f>ROUND((Z5-(36*AA5))/AA5,0)</f>
+        <f>ROUND((AB5-(36*AC5))/AC5,0)</f>
         <v>18</v>
       </c>
       <c r="D5" s="51"/>
@@ -1974,38 +2004,44 @@
       <c r="W5" s="12"/>
       <c r="X5" s="14"/>
       <c r="Y5" s="12"/>
-      <c r="Z5" s="65">
-        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5</f>
-        <v>216</v>
-      </c>
-      <c r="AA5" s="13">
-        <f>COUNTIF(D5:X5,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="AB5" s="40"/>
-      <c r="AC5" s="12"/>
-      <c r="AD5" s="41">
-        <f>SUMIF(G5:Y5, "&lt;30")+AB5+AC5</f>
-        <v>83</v>
-      </c>
-      <c r="AE5" s="71">
-        <f>AD5/AA5</f>
-        <v>20.75</v>
-      </c>
-      <c r="AF5" s="58"/>
-      <c r="AG5" s="41"/>
-      <c r="AH5" s="41"/>
-      <c r="AI5" s="13"/>
-      <c r="AJ5" s="59" t="s">
-        <v>59</v>
+      <c r="Z5" s="77">
+        <v>54</v>
+      </c>
+      <c r="AA5" s="114">
+        <v>18</v>
+      </c>
+      <c r="AB5" s="65">
+        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5</f>
+        <v>270</v>
+      </c>
+      <c r="AC5" s="13">
+        <f>COUNTIF(D5:Z5,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AD5" s="40"/>
+      <c r="AE5" s="12"/>
+      <c r="AF5" s="41">
+        <f>SUMIF(G5:AA5, "&lt;30")+AD5+AE5</f>
+        <v>101</v>
+      </c>
+      <c r="AG5" s="71">
+        <f>AF5/AC5</f>
+        <v>20.2</v>
+      </c>
+      <c r="AH5" s="58"/>
+      <c r="AI5" s="41"/>
+      <c r="AJ5" s="41"/>
+      <c r="AK5" s="13"/>
+      <c r="AL5" s="59" t="s">
+        <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:36">
+    <row r="6" spans="1:38">
       <c r="A6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>35</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>36</v>
       </c>
       <c r="C6" s="11">
         <v>2</v>
@@ -2048,299 +2084,335 @@
       <c r="Y6" s="12">
         <v>20</v>
       </c>
-      <c r="Z6" s="65">
-        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6</f>
-        <v>150</v>
-      </c>
-      <c r="AA6" s="13">
-        <f>COUNTIF(D6:X6,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="AB6" s="40">
-        <v>2</v>
-      </c>
-      <c r="AC6" s="12">
+      <c r="Z6" s="76">
+        <v>38</v>
+      </c>
+      <c r="AA6" s="114">
+        <v>18</v>
+      </c>
+      <c r="AB6" s="65">
+        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6</f>
+        <v>188</v>
+      </c>
+      <c r="AC6" s="13">
+        <f>COUNTIF(D6:Z6,"&gt;30")</f>
         <v>5</v>
       </c>
-      <c r="AD6" s="41">
-        <f>SUMIF(G6:Y6, "&lt;30")+AB6+AC6</f>
-        <v>81</v>
-      </c>
-      <c r="AE6" s="71">
-        <f>AD6/AA6</f>
-        <v>20.25</v>
-      </c>
-      <c r="AF6" s="58"/>
-      <c r="AG6" s="41"/>
-      <c r="AH6" s="41"/>
-      <c r="AI6" s="13"/>
-      <c r="AJ6" s="59"/>
+      <c r="AD6" s="40">
+        <v>3</v>
+      </c>
+      <c r="AE6" s="12">
+        <v>5</v>
+      </c>
+      <c r="AF6" s="41">
+        <f>SUMIF(G6:AA6, "&lt;30")+AD6+AE6</f>
+        <v>100</v>
+      </c>
+      <c r="AG6" s="71">
+        <f>AF6/AC6</f>
+        <v>20</v>
+      </c>
+      <c r="AH6" s="58"/>
+      <c r="AI6" s="41"/>
+      <c r="AJ6" s="41"/>
+      <c r="AK6" s="13"/>
+      <c r="AL6" s="59"/>
     </row>
-    <row r="7" spans="1:36">
+    <row r="7" spans="1:38">
       <c r="A7" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>41</v>
-      </c>
       <c r="C7" s="11">
-        <f>ROUND((Z7-(36*AA7))/AA7,0)</f>
+        <f>ROUND((AB7-(36*AC7))/AC7,0)</f>
         <v>13</v>
       </c>
       <c r="D7" s="51"/>
       <c r="E7" s="52"/>
-      <c r="F7" s="109"/>
+      <c r="F7" s="79"/>
       <c r="G7" s="12"/>
       <c r="H7" s="51"/>
       <c r="I7" s="52"/>
-      <c r="J7" s="109">
+      <c r="J7" s="79">
         <v>52</v>
       </c>
       <c r="K7" s="12">
         <v>17</v>
       </c>
-      <c r="L7" s="109"/>
+      <c r="L7" s="79"/>
       <c r="M7" s="12"/>
-      <c r="N7" s="109">
+      <c r="N7" s="79">
         <v>46</v>
       </c>
       <c r="O7" s="12">
         <v>23</v>
       </c>
-      <c r="P7" s="109">
+      <c r="P7" s="79">
         <v>46</v>
       </c>
       <c r="Q7" s="12">
         <v>23</v>
       </c>
-      <c r="R7" s="109">
+      <c r="R7" s="79">
         <v>54</v>
       </c>
       <c r="S7" s="12">
         <v>16</v>
       </c>
-      <c r="T7" s="109">
+      <c r="T7" s="79">
         <v>45</v>
       </c>
       <c r="U7" s="12">
         <v>23</v>
       </c>
-      <c r="V7" s="109">
+      <c r="V7" s="79">
         <v>48</v>
       </c>
       <c r="W7" s="12">
         <v>19</v>
       </c>
-      <c r="X7" s="109">
+      <c r="X7" s="79">
         <v>49</v>
       </c>
       <c r="Y7" s="12">
         <v>18</v>
       </c>
-      <c r="Z7" s="65">
-        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7</f>
+      <c r="Z7" s="115"/>
+      <c r="AA7" s="114"/>
+      <c r="AB7" s="65">
+        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7</f>
         <v>340</v>
       </c>
-      <c r="AA7" s="13">
-        <f>COUNTIF(D7:X7,"&gt;30")</f>
+      <c r="AC7" s="13">
+        <f>COUNTIF(D7:Z7,"&gt;30")</f>
         <v>7</v>
       </c>
-      <c r="AB7" s="40"/>
-      <c r="AC7" s="12"/>
-      <c r="AD7" s="41">
-        <f>SUMIF(G7:Y7, "&lt;30")+AB7+AC7</f>
+      <c r="AD7" s="40"/>
+      <c r="AE7" s="12"/>
+      <c r="AF7" s="41">
+        <f>SUMIF(G7:AA7, "&lt;30")+AD7+AE7</f>
         <v>139</v>
       </c>
-      <c r="AE7" s="71">
-        <f>AD7/AA7</f>
+      <c r="AG7" s="71">
+        <f>AF7/AC7</f>
         <v>19.857142857142858</v>
       </c>
-      <c r="AF7" s="58"/>
-      <c r="AG7" s="41"/>
-      <c r="AH7" s="41"/>
-      <c r="AI7" s="13"/>
-      <c r="AJ7" s="59"/>
+      <c r="AH7" s="58"/>
+      <c r="AI7" s="41"/>
+      <c r="AJ7" s="41"/>
+      <c r="AK7" s="13"/>
+      <c r="AL7" s="59"/>
     </row>
-    <row r="8" spans="1:36">
+    <row r="8" spans="1:38">
       <c r="A8" s="9" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C8" s="11">
-        <f>ROUND((Z8-(36*AA8))/AA8,0)</f>
-        <v>11</v>
+        <f>ROUND((AB8-(36*AC8))/AC8,0)</f>
+        <v>14</v>
       </c>
       <c r="D8" s="51"/>
       <c r="E8" s="52"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="12"/>
+      <c r="F8" s="14">
+        <v>42</v>
+      </c>
+      <c r="G8" s="12">
+        <v>27</v>
+      </c>
       <c r="H8" s="51"/>
       <c r="I8" s="52"/>
-      <c r="J8" s="16"/>
+      <c r="J8" s="14"/>
       <c r="K8" s="12"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="16"/>
+      <c r="L8" s="14">
+        <v>54</v>
+      </c>
+      <c r="M8" s="12">
+        <v>15</v>
+      </c>
+      <c r="N8" s="14"/>
       <c r="O8" s="12"/>
-      <c r="P8" s="42">
-        <v>47</v>
+      <c r="P8" s="14">
+        <v>54</v>
       </c>
       <c r="Q8" s="12">
-        <v>20</v>
-      </c>
-      <c r="R8" s="42">
+        <v>16</v>
+      </c>
+      <c r="R8" s="14">
+        <v>53</v>
+      </c>
+      <c r="S8" s="12">
+        <v>16</v>
+      </c>
+      <c r="T8" s="14"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="75">
+        <v>46</v>
+      </c>
+      <c r="W8" s="12">
+        <v>23</v>
+      </c>
+      <c r="X8" s="77">
+        <v>49</v>
+      </c>
+      <c r="Y8" s="12">
+        <v>19</v>
+      </c>
+      <c r="Z8" s="77">
         <v>50</v>
       </c>
-      <c r="S8" s="12">
-        <v>17</v>
-      </c>
-      <c r="T8" s="42">
-        <v>46</v>
-      </c>
-      <c r="U8" s="12">
-        <v>21</v>
-      </c>
-      <c r="V8" s="42">
-        <v>47</v>
-      </c>
-      <c r="W8" s="12">
-        <v>19</v>
-      </c>
-      <c r="X8" s="42">
-        <v>44</v>
-      </c>
-      <c r="Y8" s="12">
-        <v>22</v>
-      </c>
-      <c r="Z8" s="65">
-        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8</f>
-        <v>234</v>
-      </c>
-      <c r="AA8" s="13">
-        <f>COUNTIF(D8:X8,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="AB8" s="40"/>
-      <c r="AC8" s="12"/>
-      <c r="AD8" s="41">
-        <f>SUMIF(G8:Y8, "&lt;30")+AB8+AC8</f>
-        <v>99</v>
-      </c>
-      <c r="AE8" s="71">
-        <f>AD8/AA8</f>
-        <v>19.8</v>
-      </c>
-      <c r="AF8" s="60"/>
-      <c r="AG8" s="41"/>
-      <c r="AH8" s="41"/>
-      <c r="AI8" s="13"/>
-      <c r="AJ8" s="59"/>
+      <c r="AA8" s="114">
+        <v>18</v>
+      </c>
+      <c r="AB8" s="65">
+        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8</f>
+        <v>348</v>
+      </c>
+      <c r="AC8" s="13">
+        <f>COUNTIF(D8:Z8,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AD8" s="40">
+        <v>1</v>
+      </c>
+      <c r="AE8" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF8" s="41">
+        <f>SUMIF(G8:AA8, "&lt;30")+AD8+AE8</f>
+        <v>136</v>
+      </c>
+      <c r="AG8" s="71">
+        <f>AF8/AC8</f>
+        <v>19.428571428571427</v>
+      </c>
+      <c r="AH8" s="60"/>
+      <c r="AI8" s="41"/>
+      <c r="AJ8" s="41"/>
+      <c r="AK8" s="13"/>
+      <c r="AL8" s="59"/>
     </row>
-    <row r="9" spans="1:36">
+    <row r="9" spans="1:38">
       <c r="A9" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C9" s="11">
-        <f>ROUND((Z9-(36*AA9))/AA9,0)</f>
-        <v>14</v>
+        <f>ROUND((AB9-(36*AC9))/AC9,0)</f>
+        <v>8</v>
       </c>
       <c r="D9" s="51"/>
       <c r="E9" s="52"/>
-      <c r="F9" s="14">
-        <v>42</v>
+      <c r="F9" s="68">
+        <v>45</v>
       </c>
       <c r="G9" s="12">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H9" s="51"/>
       <c r="I9" s="52"/>
-      <c r="J9" s="14"/>
+      <c r="J9" s="68"/>
       <c r="K9" s="12"/>
-      <c r="L9" s="14">
-        <v>54</v>
+      <c r="L9" s="68">
+        <v>43</v>
       </c>
       <c r="M9" s="12">
+        <v>19</v>
+      </c>
+      <c r="N9" s="15">
+        <v>41</v>
+      </c>
+      <c r="O9" s="12">
+        <v>21</v>
+      </c>
+      <c r="P9" s="42">
+        <v>47</v>
+      </c>
+      <c r="Q9" s="12">
         <v>15</v>
       </c>
-      <c r="N9" s="14"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="14">
-        <v>54</v>
-      </c>
-      <c r="Q9" s="12">
+      <c r="R9" s="42">
+        <v>42</v>
+      </c>
+      <c r="S9" s="12">
+        <v>20</v>
+      </c>
+      <c r="T9" s="42">
+        <v>43</v>
+      </c>
+      <c r="U9" s="12">
+        <v>19</v>
+      </c>
+      <c r="V9" s="42">
+        <v>44</v>
+      </c>
+      <c r="W9" s="12">
+        <v>18</v>
+      </c>
+      <c r="X9" s="42">
+        <v>48</v>
+      </c>
+      <c r="Y9" s="12">
         <v>16</v>
       </c>
-      <c r="R9" s="14">
-        <v>53</v>
-      </c>
-      <c r="S9" s="12">
-        <v>16</v>
-      </c>
-      <c r="T9" s="14"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="75">
-        <v>46</v>
-      </c>
-      <c r="W9" s="12">
-        <v>23</v>
-      </c>
-      <c r="X9" s="107">
-        <v>49</v>
-      </c>
-      <c r="Y9" s="12">
+      <c r="Z9" s="42">
+        <v>40</v>
+      </c>
+      <c r="AA9" s="114">
+        <v>22</v>
+      </c>
+      <c r="AB9" s="65">
+        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9</f>
+        <v>393</v>
+      </c>
+      <c r="AC9" s="13">
+        <f>COUNTIF(D9:Z9,"&gt;30")</f>
+        <v>9</v>
+      </c>
+      <c r="AD9" s="40">
+        <v>1</v>
+      </c>
+      <c r="AE9" s="12">
+        <v>4</v>
+      </c>
+      <c r="AF9" s="41">
+        <f>SUMIF(G9:AA9, "&lt;30")+AD9+AE9</f>
+        <v>172</v>
+      </c>
+      <c r="AG9" s="71">
+        <f>AF9/AC9</f>
+        <v>19.111111111111111</v>
+      </c>
+      <c r="AH9" s="58"/>
+      <c r="AI9" s="41"/>
+      <c r="AJ9" s="41"/>
+      <c r="AK9" s="13"/>
+      <c r="AL9" s="59"/>
+    </row>
+    <row r="10" spans="1:38">
+      <c r="A10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="Z9" s="65">
-        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9</f>
-        <v>298</v>
-      </c>
-      <c r="AA9" s="13">
-        <f>COUNTIF(D9:X9,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AB9" s="40">
-        <v>1</v>
-      </c>
-      <c r="AC9" s="12">
-        <v>1</v>
-      </c>
-      <c r="AD9" s="41">
-        <f>SUMIF(G9:Y9, "&lt;30")+AB9+AC9</f>
-        <v>118</v>
-      </c>
-      <c r="AE9" s="71">
-        <f>AD9/AA9</f>
-        <v>19.666666666666668</v>
-      </c>
-      <c r="AF9" s="58"/>
-      <c r="AG9" s="41"/>
-      <c r="AH9" s="41"/>
-      <c r="AI9" s="13"/>
-      <c r="AJ9" s="59"/>
-    </row>
-    <row r="10" spans="1:36">
-      <c r="A10" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>27</v>
-      </c>
       <c r="C10" s="11">
-        <f>ROUND((Z10-(36*AA10))/AA10,0)</f>
-        <v>7</v>
+        <f>ROUND((AB10-(36*AC10))/AC10,0)</f>
+        <v>8</v>
       </c>
       <c r="D10" s="51"/>
       <c r="E10" s="52"/>
       <c r="F10" s="14">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G10" s="12">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H10" s="51"/>
       <c r="I10" s="52"/>
@@ -2348,247 +2420,239 @@
       <c r="K10" s="12"/>
       <c r="L10" s="14"/>
       <c r="M10" s="12"/>
-      <c r="N10" s="55">
-        <v>48</v>
+      <c r="N10" s="14">
+        <v>42</v>
       </c>
       <c r="O10" s="12">
-        <v>14</v>
-      </c>
-      <c r="P10" s="42">
-        <v>44</v>
+        <v>20</v>
+      </c>
+      <c r="P10" s="14">
+        <v>43</v>
       </c>
       <c r="Q10" s="12">
-        <v>18</v>
-      </c>
-      <c r="R10" s="42"/>
+        <v>19</v>
+      </c>
+      <c r="R10" s="14"/>
       <c r="S10" s="12"/>
-      <c r="T10" s="42"/>
+      <c r="T10" s="14"/>
       <c r="U10" s="12"/>
-      <c r="V10" s="42"/>
+      <c r="V10" s="14"/>
       <c r="W10" s="12"/>
-      <c r="X10" s="15">
-        <v>40</v>
+      <c r="X10" s="14">
+        <v>47</v>
       </c>
       <c r="Y10" s="12">
+        <v>16</v>
+      </c>
+      <c r="Z10" s="75">
+        <v>41</v>
+      </c>
+      <c r="AA10" s="114">
         <v>22</v>
       </c>
-      <c r="Z10" s="65">
-        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10</f>
-        <v>173</v>
-      </c>
-      <c r="AA10" s="13">
-        <f>COUNTIF(D10:X10,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="AB10" s="40">
+      <c r="AB10" s="65">
+        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10</f>
+        <v>219</v>
+      </c>
+      <c r="AC10" s="13">
+        <f>COUNTIF(D10:Z10,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AD10" s="40">
         <v>1</v>
       </c>
-      <c r="AC10" s="12">
+      <c r="AE10" s="12">
         <v>1</v>
       </c>
-      <c r="AD10" s="41">
-        <f>SUMIF(G10:Y10, "&lt;30")+AB10+AC10</f>
-        <v>77</v>
-      </c>
-      <c r="AE10" s="71">
-        <f>AD10/AA10</f>
-        <v>19.25</v>
-      </c>
-      <c r="AF10" s="112"/>
-      <c r="AG10" s="41"/>
-      <c r="AH10" s="41"/>
-      <c r="AI10" s="13"/>
-      <c r="AJ10" s="59"/>
+      <c r="AF10" s="41">
+        <f>SUMIF(G10:AA10, "&lt;30")+AD10+AE10</f>
+        <v>95</v>
+      </c>
+      <c r="AG10" s="71">
+        <f>AF10/AC10</f>
+        <v>19</v>
+      </c>
+      <c r="AH10" s="82"/>
+      <c r="AI10" s="41"/>
+      <c r="AJ10" s="41"/>
+      <c r="AK10" s="13"/>
+      <c r="AL10" s="59"/>
     </row>
-    <row r="11" spans="1:36">
+    <row r="11" spans="1:38">
       <c r="A11" s="9" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="C11" s="11">
-        <f>ROUND((Z11-(36*AA11))/AA11,0)</f>
-        <v>11</v>
+        <f>ROUND((AB11-(36*AC11))/AC11,0)</f>
+        <v>12</v>
       </c>
       <c r="D11" s="51"/>
       <c r="E11" s="52"/>
-      <c r="F11" s="108">
-        <v>42</v>
-      </c>
-      <c r="G11" s="12">
-        <v>25</v>
-      </c>
+      <c r="F11" s="16"/>
+      <c r="G11" s="12"/>
       <c r="H11" s="51"/>
       <c r="I11" s="52"/>
-      <c r="J11" s="108"/>
+      <c r="J11" s="16"/>
       <c r="K11" s="12"/>
-      <c r="L11" s="42">
-        <v>51</v>
-      </c>
-      <c r="M11" s="12">
-        <v>16</v>
-      </c>
-      <c r="N11" s="42"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="16"/>
       <c r="O11" s="12"/>
-      <c r="P11" s="15">
-        <v>49</v>
+      <c r="P11" s="42">
+        <v>47</v>
       </c>
       <c r="Q11" s="12">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="R11" s="42">
+        <v>50</v>
+      </c>
+      <c r="S11" s="12">
+        <v>17</v>
+      </c>
+      <c r="T11" s="42">
         <v>46</v>
       </c>
-      <c r="S11" s="12">
+      <c r="U11" s="12">
         <v>21</v>
       </c>
-      <c r="T11" s="42">
-        <v>45</v>
-      </c>
-      <c r="U11" s="12">
-        <v>20</v>
-      </c>
       <c r="V11" s="42">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W11" s="12">
         <v>19</v>
       </c>
       <c r="X11" s="42">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="Y11" s="12">
-        <v>13</v>
-      </c>
-      <c r="Z11" s="65">
-        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11</f>
-        <v>332</v>
-      </c>
-      <c r="AA11" s="13">
-        <f>COUNTIF(D11:X11,"&gt;30")</f>
+        <v>22</v>
+      </c>
+      <c r="Z11" s="42">
+        <v>52</v>
+      </c>
+      <c r="AA11" s="114">
+        <v>14</v>
+      </c>
+      <c r="AB11" s="65">
+        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11</f>
+        <v>286</v>
+      </c>
+      <c r="AC11" s="13">
+        <f>COUNTIF(D11:Z11,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AD11" s="40"/>
+      <c r="AE11" s="12"/>
+      <c r="AF11" s="41">
+        <f>SUMIF(G11:AA11, "&lt;30")+AD11+AE11</f>
+        <v>113</v>
+      </c>
+      <c r="AG11" s="71">
+        <f>AF11/AC11</f>
+        <v>18.833333333333332</v>
+      </c>
+      <c r="AH11" s="58"/>
+      <c r="AI11" s="41"/>
+      <c r="AJ11" s="41"/>
+      <c r="AK11" s="13"/>
+      <c r="AL11" s="59"/>
+    </row>
+    <row r="12" spans="1:38">
+      <c r="A12" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="11">
+        <f>ROUND((AB12-(36*AC12))/AC12,0)</f>
         <v>7</v>
-      </c>
-      <c r="AB11" s="40">
-        <v>2</v>
-      </c>
-      <c r="AC11" s="12"/>
-      <c r="AD11" s="41">
-        <f>SUMIF(G11:Y11, "&lt;30")+AB11+AC11</f>
-        <v>134</v>
-      </c>
-      <c r="AE11" s="71">
-        <f>AD11/AA11</f>
-        <v>19.142857142857142</v>
-      </c>
-      <c r="AF11" s="58"/>
-      <c r="AG11" s="41"/>
-      <c r="AH11" s="41"/>
-      <c r="AI11" s="13"/>
-      <c r="AJ11" s="59"/>
-    </row>
-    <row r="12" spans="1:36">
-      <c r="A12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="11">
-        <f>ROUND((Z12-(36*AA12))/AA12,0)</f>
-        <v>8</v>
       </c>
       <c r="D12" s="51"/>
       <c r="E12" s="52"/>
-      <c r="F12" s="68">
-        <v>45</v>
+      <c r="F12" s="14">
+        <v>41</v>
       </c>
       <c r="G12" s="12">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H12" s="51"/>
       <c r="I12" s="52"/>
-      <c r="J12" s="68"/>
+      <c r="J12" s="14"/>
       <c r="K12" s="12"/>
-      <c r="L12" s="68">
-        <v>43</v>
-      </c>
-      <c r="M12" s="12">
-        <v>19</v>
-      </c>
-      <c r="N12" s="15">
-        <v>41</v>
+      <c r="L12" s="14"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="55">
+        <v>48</v>
       </c>
       <c r="O12" s="12">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P12" s="42">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Q12" s="12">
-        <v>15</v>
-      </c>
-      <c r="R12" s="42">
-        <v>42</v>
-      </c>
-      <c r="S12" s="12">
-        <v>20</v>
-      </c>
-      <c r="T12" s="42">
-        <v>43</v>
-      </c>
-      <c r="U12" s="12">
-        <v>19</v>
-      </c>
-      <c r="V12" s="42">
+        <v>18</v>
+      </c>
+      <c r="R12" s="42"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="42"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="42"/>
+      <c r="W12" s="12"/>
+      <c r="X12" s="15">
+        <v>40</v>
+      </c>
+      <c r="Y12" s="12">
+        <v>22</v>
+      </c>
+      <c r="Z12" s="42">
         <v>44</v>
       </c>
-      <c r="W12" s="12">
-        <v>18</v>
-      </c>
-      <c r="X12" s="42">
-        <v>48</v>
-      </c>
-      <c r="Y12" s="12">
-        <v>16</v>
-      </c>
-      <c r="Z12" s="65">
-        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12</f>
-        <v>353</v>
-      </c>
-      <c r="AA12" s="13">
-        <f>COUNTIF(D12:X12,"&gt;30")</f>
-        <v>8</v>
-      </c>
-      <c r="AB12" s="40">
+      <c r="AA12" s="114">
+        <v>17</v>
+      </c>
+      <c r="AB12" s="65">
+        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12</f>
+        <v>217</v>
+      </c>
+      <c r="AC12" s="13">
+        <f>COUNTIF(D12:Z12,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AD12" s="40">
         <v>1</v>
       </c>
-      <c r="AC12" s="12">
-        <v>4</v>
-      </c>
-      <c r="AD12" s="41">
-        <f>SUMIF(G12:Y12, "&lt;30")+AB12+AC12</f>
-        <v>150</v>
-      </c>
-      <c r="AE12" s="71">
-        <f>AD12/AA12</f>
-        <v>18.75</v>
-      </c>
-      <c r="AF12" s="58"/>
-      <c r="AG12" s="41"/>
-      <c r="AH12" s="41"/>
-      <c r="AI12" s="13"/>
-      <c r="AJ12" s="59"/>
+      <c r="AE12" s="12">
+        <v>1</v>
+      </c>
+      <c r="AF12" s="41">
+        <f>SUMIF(G12:AA12, "&lt;30")+AD12+AE12</f>
+        <v>94</v>
+      </c>
+      <c r="AG12" s="71">
+        <f>AF12/AC12</f>
+        <v>18.8</v>
+      </c>
+      <c r="AH12" s="61"/>
+      <c r="AI12" s="41"/>
+      <c r="AJ12" s="41"/>
+      <c r="AK12" s="13"/>
+      <c r="AL12" s="59"/>
     </row>
-    <row r="13" spans="1:36">
+    <row r="13" spans="1:38">
       <c r="A13" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="C13" s="11">
-        <f>ROUND((Z13-(36*AA13))/AA13,0)</f>
+        <f>ROUND((AB13-(36*AC13))/AC13,0)</f>
         <v>15</v>
       </c>
       <c r="D13" s="51"/>
@@ -2629,116 +2693,142 @@
       <c r="Y13" s="12">
         <v>21</v>
       </c>
-      <c r="Z13" s="65">
-        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13</f>
+      <c r="Z13" s="77"/>
+      <c r="AA13" s="114"/>
+      <c r="AB13" s="65">
+        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13</f>
         <v>202</v>
       </c>
-      <c r="AA13" s="13">
-        <f>COUNTIF(D13:X13,"&gt;30")</f>
+      <c r="AC13" s="13">
+        <f>COUNTIF(D13:Z13,"&gt;30")</f>
         <v>4</v>
       </c>
-      <c r="AB13" s="40"/>
-      <c r="AC13" s="12"/>
-      <c r="AD13" s="41">
-        <f>SUMIF(G13:Y13, "&lt;30")+AB13+AC13</f>
+      <c r="AD13" s="40"/>
+      <c r="AE13" s="12"/>
+      <c r="AF13" s="41">
+        <f>SUMIF(G13:AA13, "&lt;30")+AD13+AE13</f>
         <v>74</v>
       </c>
-      <c r="AE13" s="71">
-        <f>AD13/AA13</f>
+      <c r="AG13" s="71">
+        <f>AF13/AC13</f>
         <v>18.5</v>
       </c>
-      <c r="AF13" s="61"/>
-      <c r="AG13" s="41"/>
-      <c r="AH13" s="41"/>
-      <c r="AI13" s="13"/>
-      <c r="AJ13" s="59"/>
+      <c r="AH13" s="61"/>
+      <c r="AI13" s="41"/>
+      <c r="AJ13" s="41"/>
+      <c r="AK13" s="13"/>
+      <c r="AL13" s="59"/>
     </row>
-    <row r="14" spans="1:36">
+    <row r="14" spans="1:38">
       <c r="A14" s="9" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="11">
+        <f>ROUND((AB14-(36*AC14))/AC14,0)</f>
         <v>12</v>
-      </c>
-      <c r="C14" s="11">
-        <v>22</v>
       </c>
       <c r="D14" s="51"/>
       <c r="E14" s="52"/>
-      <c r="F14" s="14">
-        <v>59</v>
+      <c r="F14" s="78">
+        <v>42</v>
       </c>
       <c r="G14" s="12">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H14" s="51"/>
       <c r="I14" s="52"/>
-      <c r="J14" s="14"/>
+      <c r="J14" s="78"/>
       <c r="K14" s="12"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="14"/>
+      <c r="L14" s="42">
+        <v>51</v>
+      </c>
+      <c r="M14" s="12">
+        <v>16</v>
+      </c>
+      <c r="N14" s="42"/>
       <c r="O14" s="12"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="12"/>
-      <c r="R14" s="14">
-        <v>55</v>
+      <c r="P14" s="15">
+        <v>49</v>
+      </c>
+      <c r="Q14" s="12">
+        <v>18</v>
+      </c>
+      <c r="R14" s="42">
+        <v>46</v>
       </c>
       <c r="S14" s="12">
         <v>21</v>
       </c>
-      <c r="T14" s="14"/>
-      <c r="U14" s="12"/>
-      <c r="V14" s="14">
-        <v>59</v>
+      <c r="T14" s="42">
+        <v>45</v>
+      </c>
+      <c r="U14" s="12">
+        <v>20</v>
+      </c>
+      <c r="V14" s="42">
+        <v>46</v>
       </c>
       <c r="W14" s="12">
+        <v>19</v>
+      </c>
+      <c r="X14" s="42">
+        <v>53</v>
+      </c>
+      <c r="Y14" s="12">
+        <v>13</v>
+      </c>
+      <c r="Z14" s="42">
+        <v>52</v>
+      </c>
+      <c r="AA14" s="114">
+        <v>13</v>
+      </c>
+      <c r="AB14" s="65">
+        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14</f>
+        <v>384</v>
+      </c>
+      <c r="AC14" s="13">
+        <f>COUNTIF(D14:Z14,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AD14" s="40">
+        <v>2</v>
+      </c>
+      <c r="AE14" s="12"/>
+      <c r="AF14" s="41">
+        <f>SUMIF(G14:AA14, "&lt;30")+AD14+AE14</f>
+        <v>147</v>
+      </c>
+      <c r="AG14" s="71">
+        <f>AF14/AC14</f>
+        <v>18.375</v>
+      </c>
+      <c r="AH14" s="58"/>
+      <c r="AI14" s="41"/>
+      <c r="AJ14" s="41"/>
+      <c r="AK14" s="13"/>
+      <c r="AL14" s="59"/>
+    </row>
+    <row r="15" spans="1:38">
+      <c r="A15" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="X14" s="14"/>
-      <c r="Y14" s="12"/>
-      <c r="Z14" s="65">
-        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14</f>
-        <v>173</v>
-      </c>
-      <c r="AA14" s="13">
-        <f>COUNTIF(D14:X14,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="AB14" s="40"/>
-      <c r="AC14" s="12"/>
-      <c r="AD14" s="41">
-        <f>SUMIF(G14:Y14, "&lt;30")+AB14+AC14</f>
-        <v>55</v>
-      </c>
-      <c r="AE14" s="71">
-        <f>AD14/AA14</f>
-        <v>18.333333333333332</v>
-      </c>
-      <c r="AF14" s="61"/>
-      <c r="AG14" s="41"/>
-      <c r="AH14" s="41"/>
-      <c r="AI14" s="13"/>
-      <c r="AJ14" s="59"/>
-    </row>
-    <row r="15" spans="1:36">
-      <c r="A15" s="9" t="s">
-        <v>19</v>
-      </c>
       <c r="B15" s="10" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C15" s="11">
-        <f>ROUND((Z15-(36*AA15))/AA15,0)</f>
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="D15" s="51"/>
       <c r="E15" s="52"/>
       <c r="F15" s="14">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="G15" s="12">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H15" s="51"/>
       <c r="I15" s="52"/>
@@ -2746,62 +2836,58 @@
       <c r="K15" s="12"/>
       <c r="L15" s="14"/>
       <c r="M15" s="12"/>
-      <c r="N15" s="14">
-        <v>42</v>
-      </c>
-      <c r="O15" s="12">
-        <v>20</v>
-      </c>
-      <c r="P15" s="14">
-        <v>43</v>
-      </c>
-      <c r="Q15" s="12">
-        <v>19</v>
-      </c>
-      <c r="R15" s="14"/>
-      <c r="S15" s="12"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="14">
+        <v>55</v>
+      </c>
+      <c r="S15" s="12">
+        <v>21</v>
+      </c>
       <c r="T15" s="14"/>
       <c r="U15" s="12"/>
-      <c r="V15" s="14"/>
-      <c r="W15" s="12"/>
-      <c r="X15" s="14">
-        <v>47</v>
-      </c>
-      <c r="Y15" s="12">
-        <v>16</v>
-      </c>
-      <c r="Z15" s="65">
-        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15</f>
-        <v>178</v>
-      </c>
-      <c r="AA15" s="13">
-        <f>COUNTIF(D15:X15,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="AB15" s="40"/>
-      <c r="AC15" s="12">
-        <v>1</v>
-      </c>
-      <c r="AD15" s="41">
-        <f>SUMIF(G15:Y15, "&lt;30")+AB15+AC15</f>
-        <v>72</v>
-      </c>
-      <c r="AE15" s="71">
-        <f>AD15/AA15</f>
-        <v>18</v>
-      </c>
-      <c r="AF15" s="61"/>
-      <c r="AG15" s="41"/>
-      <c r="AH15" s="41"/>
-      <c r="AI15" s="13"/>
-      <c r="AJ15" s="59"/>
+      <c r="V15" s="14">
+        <v>59</v>
+      </c>
+      <c r="W15" s="12">
+        <v>17</v>
+      </c>
+      <c r="X15" s="14"/>
+      <c r="Y15" s="12"/>
+      <c r="Z15" s="77"/>
+      <c r="AA15" s="114"/>
+      <c r="AB15" s="65">
+        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15</f>
+        <v>173</v>
+      </c>
+      <c r="AC15" s="13">
+        <f>COUNTIF(D15:Z15,"&gt;30")</f>
+        <v>3</v>
+      </c>
+      <c r="AD15" s="40"/>
+      <c r="AE15" s="12"/>
+      <c r="AF15" s="41">
+        <f>SUMIF(G15:AA15, "&lt;30")+AD15+AE15</f>
+        <v>55</v>
+      </c>
+      <c r="AG15" s="71">
+        <f>AF15/AC15</f>
+        <v>18.333333333333332</v>
+      </c>
+      <c r="AH15" s="61"/>
+      <c r="AI15" s="41"/>
+      <c r="AJ15" s="41"/>
+      <c r="AK15" s="13"/>
+      <c r="AL15" s="59"/>
     </row>
-    <row r="16" spans="1:36">
+    <row r="16" spans="1:38">
       <c r="A16" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>57</v>
       </c>
       <c r="C16" s="11">
         <v>9</v>
@@ -2840,212 +2926,216 @@
       <c r="Y16" s="12">
         <v>15</v>
       </c>
-      <c r="Z16" s="65">
-        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16</f>
-        <v>136</v>
-      </c>
-      <c r="AA16" s="13">
-        <f>COUNTIF(D16:X16,"&gt;30")</f>
-        <v>3</v>
-      </c>
-      <c r="AB16" s="40"/>
-      <c r="AC16" s="12">
+      <c r="Z16" s="42">
+        <v>47</v>
+      </c>
+      <c r="AA16" s="114">
+        <v>16</v>
+      </c>
+      <c r="AB16" s="65">
+        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16</f>
+        <v>183</v>
+      </c>
+      <c r="AC16" s="13">
+        <f>COUNTIF(D16:Z16,"&gt;30")</f>
+        <v>4</v>
+      </c>
+      <c r="AD16" s="40"/>
+      <c r="AE16" s="12">
         <v>1</v>
       </c>
-      <c r="AD16" s="41">
-        <f>SUMIF(G16:Y16, "&lt;30")+AB16+AC16</f>
-        <v>54</v>
-      </c>
-      <c r="AE16" s="71">
-        <f>AD16/AA16</f>
+      <c r="AF16" s="41">
+        <f>SUMIF(G16:AA16, "&lt;30")+AD16+AE16</f>
+        <v>70</v>
+      </c>
+      <c r="AG16" s="71">
+        <f>AF16/AC16</f>
+        <v>17.5</v>
+      </c>
+      <c r="AH16" s="58"/>
+      <c r="AI16" s="41"/>
+      <c r="AJ16" s="41"/>
+      <c r="AK16" s="13"/>
+      <c r="AL16" s="59"/>
+    </row>
+    <row r="17" spans="1:38">
+      <c r="A17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="11">
+        <f>ROUND((AB17-(36*AC17))/AC17,0)</f>
         <v>18</v>
-      </c>
-      <c r="AF16" s="58"/>
-      <c r="AG16" s="41"/>
-      <c r="AH16" s="41"/>
-      <c r="AI16" s="13"/>
-      <c r="AJ16" s="59"/>
-    </row>
-    <row r="17" spans="1:36">
-      <c r="A17" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="11">
-        <f>ROUND((Z17-(36*AA17))/AA17,0)</f>
-        <v>22</v>
       </c>
       <c r="D17" s="51"/>
       <c r="E17" s="52"/>
-      <c r="F17" s="15">
-        <v>61</v>
+      <c r="F17" s="14">
+        <v>55</v>
       </c>
       <c r="G17" s="12">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H17" s="51"/>
       <c r="I17" s="52"/>
-      <c r="J17" s="15">
+      <c r="J17" s="14"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="14">
         <v>56</v>
-      </c>
-      <c r="K17" s="12">
-        <v>19</v>
-      </c>
-      <c r="L17" s="42">
-        <v>60</v>
       </c>
       <c r="M17" s="12">
         <v>15</v>
       </c>
-      <c r="N17" s="42">
+      <c r="N17" s="14">
+        <v>57</v>
+      </c>
+      <c r="O17" s="12">
+        <v>14</v>
+      </c>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="14"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="75">
+        <v>49</v>
+      </c>
+      <c r="U17" s="12">
+        <v>22</v>
+      </c>
+      <c r="V17" s="75">
+        <v>58</v>
+      </c>
+      <c r="W17" s="12">
+        <v>14</v>
+      </c>
+      <c r="X17" s="77">
+        <v>50</v>
+      </c>
+      <c r="Y17" s="12">
+        <v>23</v>
+      </c>
+      <c r="Z17" s="77">
         <v>56</v>
       </c>
-      <c r="O17" s="12">
-        <v>20</v>
-      </c>
-      <c r="P17" s="42">
-        <v>54</v>
-      </c>
-      <c r="Q17" s="12">
-        <v>22</v>
-      </c>
-      <c r="R17" s="42"/>
-      <c r="S17" s="12"/>
-      <c r="T17" s="42">
-        <v>66</v>
-      </c>
-      <c r="U17" s="12">
-        <v>9</v>
-      </c>
-      <c r="V17" s="42">
-        <v>55</v>
-      </c>
-      <c r="W17" s="12">
-        <v>22</v>
-      </c>
-      <c r="X17" s="42"/>
-      <c r="Y17" s="12"/>
-      <c r="Z17" s="65">
-        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17</f>
-        <v>408</v>
-      </c>
-      <c r="AA17" s="13">
-        <f>COUNTIF(D17:X17,"&gt;30")</f>
+      <c r="AA17" s="12">
+        <v>16</v>
+      </c>
+      <c r="AB17" s="65">
+        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17</f>
+        <v>381</v>
+      </c>
+      <c r="AC17" s="13">
+        <f>COUNTIF(D17:Z17,"&gt;30")</f>
         <v>7</v>
       </c>
-      <c r="AB17" s="40">
-        <v>2</v>
-      </c>
-      <c r="AC17" s="12"/>
-      <c r="AD17" s="41">
-        <f>SUMIF(G17:Y17, "&lt;30")+AB17+AC17</f>
-        <v>123</v>
-      </c>
-      <c r="AE17" s="71">
-        <f>AD17/AA17</f>
-        <v>17.571428571428573</v>
-      </c>
-      <c r="AF17" s="58"/>
-      <c r="AG17" s="41"/>
-      <c r="AH17" s="41"/>
-      <c r="AI17" s="13"/>
-      <c r="AJ17" s="59"/>
+      <c r="AD17" s="40">
+        <v>1</v>
+      </c>
+      <c r="AE17" s="12"/>
+      <c r="AF17" s="41">
+        <f>SUMIF(G17:AA17, "&lt;30")+AD17+AE17</f>
+        <v>121</v>
+      </c>
+      <c r="AG17" s="71">
+        <f>AF17/AC17</f>
+        <v>17.285714285714285</v>
+      </c>
+      <c r="AH17" s="61"/>
+      <c r="AI17" s="41"/>
+      <c r="AJ17" s="41"/>
+      <c r="AK17" s="13"/>
+      <c r="AL17" s="59"/>
     </row>
-    <row r="18" spans="1:36">
+    <row r="18" spans="1:38">
       <c r="A18" s="9" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C18" s="11">
-        <f>ROUND((Z18-(36*AA18))/AA18,0)</f>
-        <v>18</v>
+        <f>ROUND((AB18-(36*AC18))/AC18,0)</f>
+        <v>14</v>
       </c>
       <c r="D18" s="51"/>
       <c r="E18" s="52"/>
-      <c r="F18" s="14">
-        <v>55</v>
-      </c>
-      <c r="G18" s="12">
-        <v>16</v>
-      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="12"/>
       <c r="H18" s="51"/>
       <c r="I18" s="52"/>
       <c r="J18" s="14"/>
       <c r="K18" s="12"/>
-      <c r="L18" s="14">
-        <v>56</v>
-      </c>
-      <c r="M18" s="12">
-        <v>15</v>
-      </c>
-      <c r="N18" s="14">
-        <v>57</v>
-      </c>
-      <c r="O18" s="12">
+      <c r="L18" s="14"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="14">
+        <v>48</v>
+      </c>
+      <c r="Q18" s="12">
+        <v>18</v>
+      </c>
+      <c r="R18" s="14">
+        <v>51</v>
+      </c>
+      <c r="S18" s="12">
         <v>14</v>
       </c>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="14"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="75">
-        <v>49</v>
+      <c r="T18" s="14">
+        <v>51</v>
       </c>
       <c r="U18" s="12">
-        <v>22</v>
-      </c>
-      <c r="V18" s="75">
-        <v>58</v>
-      </c>
-      <c r="W18" s="12">
         <v>14</v>
       </c>
-      <c r="X18" s="107">
+      <c r="V18" s="14"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="14">
+        <v>48</v>
+      </c>
+      <c r="Y18" s="12">
+        <v>20</v>
+      </c>
+      <c r="Z18" s="14">
         <v>50</v>
       </c>
-      <c r="Y18" s="12">
-        <v>23</v>
-      </c>
-      <c r="Z18" s="65">
-        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18</f>
-        <v>325</v>
-      </c>
-      <c r="AA18" s="13">
-        <f>COUNTIF(D18:X18,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AB18" s="40">
-        <v>1</v>
-      </c>
-      <c r="AC18" s="12"/>
-      <c r="AD18" s="41">
-        <f>SUMIF(G18:Y18, "&lt;30")+AB18+AC18</f>
-        <v>105</v>
-      </c>
-      <c r="AE18" s="71">
-        <f>AD18/AA18</f>
-        <v>17.5</v>
-      </c>
-      <c r="AF18" s="61"/>
-      <c r="AG18" s="41"/>
-      <c r="AH18" s="41"/>
-      <c r="AI18" s="13"/>
-      <c r="AJ18" s="59"/>
+      <c r="AA18" s="12">
+        <v>18</v>
+      </c>
+      <c r="AB18" s="65">
+        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18</f>
+        <v>248</v>
+      </c>
+      <c r="AC18" s="13">
+        <f>COUNTIF(D18:Z18,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AD18" s="40"/>
+      <c r="AE18" s="12"/>
+      <c r="AF18" s="41">
+        <f>SUMIF(G18:AA18, "&lt;30")+AD18+AE18</f>
+        <v>84</v>
+      </c>
+      <c r="AG18" s="71">
+        <f>AF18/AC18</f>
+        <v>16.8</v>
+      </c>
+      <c r="AH18" s="58"/>
+      <c r="AI18" s="41"/>
+      <c r="AJ18" s="41"/>
+      <c r="AK18" s="13"/>
+      <c r="AL18" s="59"/>
     </row>
-    <row r="19" spans="1:36">
+    <row r="19" spans="1:38">
       <c r="A19" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>30</v>
-      </c>
       <c r="C19" s="11">
-        <f>ROUND((Z19-(36*AA19))/AA19,0)</f>
-        <v>11</v>
+        <f>ROUND((AB19-(36*AC19))/AC19,0)</f>
+        <v>12</v>
       </c>
       <c r="D19" s="51"/>
       <c r="E19" s="52"/>
@@ -3093,109 +3183,135 @@
       <c r="W19" s="12"/>
       <c r="X19" s="14"/>
       <c r="Y19" s="12"/>
-      <c r="Z19" s="65">
-        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19</f>
-        <v>283</v>
-      </c>
-      <c r="AA19" s="13">
-        <f>COUNTIF(D19:X19,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AB19" s="43"/>
-      <c r="AC19" s="33"/>
-      <c r="AD19" s="41">
-        <f>SUMIF(G19:Y19, "&lt;30")+AB19+AC19</f>
-        <v>99</v>
-      </c>
-      <c r="AE19" s="71">
-        <f>AD19/AA19</f>
-        <v>16.5</v>
-      </c>
-      <c r="AF19" s="61"/>
-      <c r="AG19" s="13"/>
-      <c r="AH19" s="13"/>
+      <c r="Z19" s="14">
+        <v>50</v>
+      </c>
+      <c r="AA19" s="12">
+        <v>15</v>
+      </c>
+      <c r="AB19" s="65">
+        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19</f>
+        <v>333</v>
+      </c>
+      <c r="AC19" s="13">
+        <f>COUNTIF(D19:Z19,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AD19" s="43"/>
+      <c r="AE19" s="33"/>
+      <c r="AF19" s="41">
+        <f>SUMIF(G19:AA19, "&lt;30")+AD19+AE19</f>
+        <v>114</v>
+      </c>
+      <c r="AG19" s="71">
+        <f>AF19/AC19</f>
+        <v>16.285714285714285</v>
+      </c>
+      <c r="AH19" s="61"/>
       <c r="AI19" s="13"/>
-      <c r="AJ19" s="59"/>
+      <c r="AJ19" s="13"/>
+      <c r="AK19" s="13"/>
+      <c r="AL19" s="59"/>
     </row>
-    <row r="20" spans="1:36">
+    <row r="20" spans="1:38">
       <c r="A20" s="9" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C20" s="11">
-        <f>ROUND((Z20-(36*AA20))/AA20,0)</f>
-        <v>14</v>
+        <f>ROUND((AB20-(36*AC20))/AC20,0)</f>
+        <v>24</v>
       </c>
       <c r="D20" s="51"/>
       <c r="E20" s="52"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="12"/>
+      <c r="F20" s="15">
+        <v>61</v>
+      </c>
+      <c r="G20" s="12">
+        <v>14</v>
+      </c>
       <c r="H20" s="51"/>
       <c r="I20" s="52"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="12"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="12"/>
-      <c r="P20" s="14">
-        <v>48</v>
+      <c r="J20" s="15">
+        <v>56</v>
+      </c>
+      <c r="K20" s="12">
+        <v>19</v>
+      </c>
+      <c r="L20" s="42">
+        <v>60</v>
+      </c>
+      <c r="M20" s="12">
+        <v>15</v>
+      </c>
+      <c r="N20" s="42">
+        <v>56</v>
+      </c>
+      <c r="O20" s="12">
+        <v>20</v>
+      </c>
+      <c r="P20" s="42">
+        <v>54</v>
       </c>
       <c r="Q20" s="12">
-        <v>18</v>
-      </c>
-      <c r="R20" s="14">
-        <v>51</v>
-      </c>
-      <c r="S20" s="12">
-        <v>14</v>
-      </c>
-      <c r="T20" s="14">
-        <v>51</v>
+        <v>22</v>
+      </c>
+      <c r="R20" s="42"/>
+      <c r="S20" s="12"/>
+      <c r="T20" s="42">
+        <v>66</v>
       </c>
       <c r="U20" s="12">
-        <v>14</v>
-      </c>
-      <c r="V20" s="14"/>
-      <c r="W20" s="12"/>
-      <c r="X20" s="14">
-        <v>48</v>
-      </c>
-      <c r="Y20" s="12">
-        <v>20</v>
-      </c>
-      <c r="Z20" s="65">
-        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20</f>
-        <v>198</v>
-      </c>
-      <c r="AA20" s="13">
-        <f>COUNTIF(D20:X20,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="AB20" s="40"/>
-      <c r="AC20" s="12"/>
-      <c r="AD20" s="41">
-        <f>SUMIF(G20:Y20, "&lt;30")+AB20+AC20</f>
-        <v>66</v>
-      </c>
-      <c r="AE20" s="71">
-        <f>AD20/AA20</f>
-        <v>16.5</v>
-      </c>
-      <c r="AF20" s="58"/>
-      <c r="AG20" s="41"/>
-      <c r="AH20" s="41"/>
-      <c r="AI20" s="13"/>
-      <c r="AJ20" s="59"/>
+        <v>9</v>
+      </c>
+      <c r="V20" s="42">
+        <v>55</v>
+      </c>
+      <c r="W20" s="12">
+        <v>22</v>
+      </c>
+      <c r="X20" s="42"/>
+      <c r="Y20" s="12"/>
+      <c r="Z20" s="42">
+        <v>70</v>
+      </c>
+      <c r="AA20" s="114">
+        <v>6</v>
+      </c>
+      <c r="AB20" s="65">
+        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20</f>
+        <v>478</v>
+      </c>
+      <c r="AC20" s="13">
+        <f>COUNTIF(D20:Z20,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AD20" s="40">
+        <v>2</v>
+      </c>
+      <c r="AE20" s="12"/>
+      <c r="AF20" s="41">
+        <f>SUMIF(G20:AA20, "&lt;30")+AD20+AE20</f>
+        <v>129</v>
+      </c>
+      <c r="AG20" s="71">
+        <f>AF20/AC20</f>
+        <v>16.125</v>
+      </c>
+      <c r="AH20" s="58"/>
+      <c r="AI20" s="41"/>
+      <c r="AJ20" s="41"/>
+      <c r="AK20" s="13"/>
+      <c r="AL20" s="59"/>
     </row>
-    <row r="21" spans="1:36">
+    <row r="21" spans="1:38">
       <c r="A21" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>22</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>23</v>
       </c>
       <c r="C21" s="11">
         <v>18</v>
@@ -3226,91 +3342,95 @@
       <c r="W21" s="12"/>
       <c r="X21" s="14"/>
       <c r="Y21" s="12"/>
-      <c r="Z21" s="65">
-        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21</f>
+      <c r="Z21" s="14"/>
+      <c r="AA21" s="12"/>
+      <c r="AB21" s="65">
+        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21</f>
         <v>56</v>
       </c>
-      <c r="AA21" s="13">
-        <f>COUNTIF(D21:X21,"&gt;30")</f>
+      <c r="AC21" s="13">
+        <f>COUNTIF(D21:Z21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AB21" s="40"/>
-      <c r="AC21" s="12"/>
-      <c r="AD21" s="41">
-        <f>SUMIF(G21:Y21, "&lt;30")+AB21+AC21</f>
+      <c r="AD21" s="40"/>
+      <c r="AE21" s="12"/>
+      <c r="AF21" s="41">
+        <f>SUMIF(G21:AA21, "&lt;30")+AD21+AE21</f>
         <v>16</v>
       </c>
-      <c r="AE21" s="71">
-        <f>AD21/AA21</f>
+      <c r="AG21" s="71">
+        <f>AF21/AC21</f>
         <v>16</v>
       </c>
-      <c r="AF21" s="61"/>
-      <c r="AG21" s="41"/>
-      <c r="AH21" s="41"/>
-      <c r="AI21" s="13"/>
-      <c r="AJ21" s="59"/>
+      <c r="AH21" s="61"/>
+      <c r="AI21" s="41"/>
+      <c r="AJ21" s="41"/>
+      <c r="AK21" s="13"/>
+      <c r="AL21" s="59"/>
     </row>
-    <row r="22" spans="1:36" ht="17" thickBot="1">
+    <row r="22" spans="1:38" ht="17" thickBot="1">
       <c r="A22" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>50</v>
-      </c>
       <c r="C22" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D22" s="53"/>
       <c r="E22" s="54"/>
-      <c r="F22" s="110"/>
+      <c r="F22" s="80"/>
       <c r="G22" s="21"/>
       <c r="H22" s="53"/>
       <c r="I22" s="54"/>
-      <c r="J22" s="110"/>
+      <c r="J22" s="80"/>
       <c r="K22" s="21"/>
-      <c r="L22" s="111">
+      <c r="L22" s="81">
         <v>50</v>
       </c>
       <c r="M22" s="21"/>
-      <c r="N22" s="111"/>
+      <c r="N22" s="81"/>
       <c r="O22" s="21"/>
-      <c r="P22" s="111"/>
+      <c r="P22" s="81"/>
       <c r="Q22" s="21"/>
-      <c r="R22" s="111"/>
+      <c r="R22" s="81"/>
       <c r="S22" s="21"/>
-      <c r="T22" s="111"/>
+      <c r="T22" s="81"/>
       <c r="U22" s="21"/>
-      <c r="V22" s="111"/>
+      <c r="V22" s="81"/>
       <c r="W22" s="21"/>
-      <c r="X22" s="111"/>
+      <c r="X22" s="81"/>
       <c r="Y22" s="21"/>
-      <c r="Z22" s="66">
-        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22</f>
+      <c r="Z22" s="81"/>
+      <c r="AA22" s="21"/>
+      <c r="AB22" s="66">
+        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22</f>
         <v>50</v>
       </c>
-      <c r="AA22" s="22">
-        <f>COUNTIF(D22:X22,"&gt;30")</f>
+      <c r="AC22" s="22">
+        <f>COUNTIF(D22:Z22,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AB22" s="44">
+      <c r="AD22" s="44">
         <v>1</v>
       </c>
-      <c r="AC22" s="21"/>
-      <c r="AD22" s="45">
-        <f>SUMIF(G22:Y22, "&lt;30")+AB22+AC22</f>
+      <c r="AE22" s="21"/>
+      <c r="AF22" s="45">
+        <f>SUMIF(G22:AA22, "&lt;30")+AD22+AE22</f>
         <v>1</v>
       </c>
-      <c r="AE22" s="72">
-        <f>AD22/AA22</f>
+      <c r="AG22" s="72">
+        <f>AF22/AC22</f>
         <v>1</v>
       </c>
-      <c r="AF22" s="62"/>
-      <c r="AG22" s="45"/>
-      <c r="AH22" s="45"/>
-      <c r="AI22" s="22"/>
-      <c r="AJ22" s="63"/>
+      <c r="AH22" s="62"/>
+      <c r="AI22" s="45"/>
+      <c r="AJ22" s="45"/>
+      <c r="AK22" s="22"/>
+      <c r="AL22" s="63"/>
     </row>
-    <row r="23" spans="1:36" s="23" customFormat="1" ht="17" thickBot="1">
+    <row r="23" spans="1:38" s="23" customFormat="1" ht="17" thickBot="1">
       <c r="A23" s="34"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -3363,23 +3483,28 @@
         <v>46.46153846153846</v>
       </c>
       <c r="Y23" s="36"/>
-      <c r="Z23" s="37"/>
+      <c r="Z23" s="36">
+        <f>AVERAGEIF(Z4:Z22,"&gt;0")</f>
+        <v>49.53846153846154</v>
+      </c>
+      <c r="AA23" s="36"/>
+      <c r="AB23" s="37"/>
     </row>
-    <row r="24" spans="1:36">
+    <row r="24" spans="1:38">
       <c r="C24" s="24"/>
-      <c r="Z24" s="25"/>
-      <c r="AA24" s="25"/>
-      <c r="AB24" s="26"/>
-      <c r="AC24" s="26"/>
-      <c r="AD24" s="25"/>
-      <c r="AE24" s="27"/>
+      <c r="AB24" s="25"/>
+      <c r="AC24" s="25"/>
+      <c r="AD24" s="26"/>
+      <c r="AE24" s="26"/>
+      <c r="AF24" s="25"/>
+      <c r="AG24" s="27"/>
     </row>
-    <row r="25" spans="1:36">
+    <row r="25" spans="1:38">
       <c r="C25" s="46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F25" s="28"/>
       <c r="H25" s="28"/>
@@ -3391,13 +3516,14 @@
       <c r="T25" s="28"/>
       <c r="V25" s="28"/>
       <c r="X25" s="28"/>
+      <c r="Z25" s="28"/>
     </row>
-    <row r="26" spans="1:36">
+    <row r="26" spans="1:38">
       <c r="C26" s="47" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F26" s="29"/>
       <c r="H26" s="29"/>
@@ -3409,14 +3535,15 @@
       <c r="T26" s="29"/>
       <c r="V26" s="29"/>
       <c r="X26" s="29"/>
-      <c r="Z26" s="30"/>
+      <c r="Z26" s="29"/>
+      <c r="AB26" s="30"/>
     </row>
-    <row r="27" spans="1:36">
+    <row r="27" spans="1:38">
       <c r="C27" s="48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D27" s="31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E27" s="32"/>
       <c r="F27" s="31"/>
@@ -3439,20 +3566,45 @@
       <c r="W27" s="32"/>
       <c r="X27" s="31"/>
       <c r="Y27" s="32"/>
+      <c r="Z27" s="31"/>
+      <c r="AA27" s="32"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AJ22">
-    <sortCondition descending="1" ref="AE4:AE22"/>
-    <sortCondition descending="1" ref="Z4:Z22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AL22">
+    <sortCondition descending="1" ref="AG4:AG22"/>
+    <sortCondition descending="1" ref="AB4:AB22"/>
   </sortState>
-  <mergeCells count="37">
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="AF1:AJ1"/>
+  <mergeCells count="39">
+    <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
     <mergeCell ref="AF2:AF3"/>
     <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="AB1:AB3"/>
+    <mergeCell ref="AC1:AG1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="AH1:AL1"/>
     <mergeCell ref="AH2:AH3"/>
     <mergeCell ref="AI2:AI3"/>
     <mergeCell ref="AJ2:AJ3"/>
+    <mergeCell ref="AK2:AK3"/>
+    <mergeCell ref="AL2:AL3"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="R2:S2"/>
     <mergeCell ref="T1:U1"/>
@@ -3461,28 +3613,7 @@
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="AB2:AB3"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="Z1:Z3"/>
-    <mergeCell ref="AA1:AE1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="Z1:AA1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
080525 - updated scores and skins results from 8/4
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94A3502-0EBB-1C4C-B4A9-72D954014F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B462733-2B02-A44E-8A60-B83CCB999AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10340" yWindow="2280" windowWidth="26960" windowHeight="15740" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="5380" yWindow="2280" windowWidth="31760" windowHeight="15740" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="68">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -238,13 +238,16 @@
   </si>
   <si>
     <t>WEEK 13</t>
+  </si>
+  <si>
+    <t>WEEK 14</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -376,6 +379,12 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -953,7 +962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1166,11 +1175,89 @@
     <xf numFmtId="1" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1196,82 +1283,49 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1608,7 +1662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AN27"/>
+  <dimension ref="A1:AP27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1623,188 +1677,198 @@
     <col min="27" max="27" width="6.33203125" customWidth="1"/>
     <col min="28" max="28" width="6" customWidth="1"/>
     <col min="29" max="29" width="6.33203125" customWidth="1"/>
-    <col min="30" max="30" width="8.83203125" customWidth="1"/>
-    <col min="31" max="31" width="6.1640625" customWidth="1"/>
-    <col min="32" max="32" width="5.83203125" customWidth="1"/>
-    <col min="33" max="33" width="5.6640625" customWidth="1"/>
-    <col min="34" max="34" width="5.5" customWidth="1"/>
-    <col min="35" max="35" width="8" customWidth="1"/>
-    <col min="36" max="36" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="37" max="38" width="6" hidden="1" customWidth="1"/>
-    <col min="39" max="39" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="40" max="40" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="6" customWidth="1"/>
+    <col min="31" max="31" width="6.33203125" customWidth="1"/>
+    <col min="32" max="32" width="7.1640625" customWidth="1"/>
+    <col min="33" max="33" width="6.1640625" customWidth="1"/>
+    <col min="34" max="34" width="5.83203125" customWidth="1"/>
+    <col min="35" max="35" width="5.6640625" customWidth="1"/>
+    <col min="36" max="36" width="5.5" customWidth="1"/>
+    <col min="37" max="37" width="8" customWidth="1"/>
+    <col min="38" max="38" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="39" max="40" width="6" hidden="1" customWidth="1"/>
+    <col min="41" max="41" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="42" max="42" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="54" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="80" t="s">
+    <row r="1" spans="1:42" s="54" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="86" t="s">
+      <c r="B1" s="107"/>
+      <c r="C1" s="112" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="88" t="s">
+      <c r="D1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="89"/>
-      <c r="F1" s="88" t="s">
+      <c r="E1" s="85"/>
+      <c r="F1" s="84" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="89"/>
-      <c r="H1" s="88" t="s">
+      <c r="G1" s="85"/>
+      <c r="H1" s="84" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="89"/>
-      <c r="J1" s="88" t="s">
+      <c r="I1" s="85"/>
+      <c r="J1" s="84" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="89"/>
-      <c r="L1" s="88" t="s">
+      <c r="K1" s="85"/>
+      <c r="L1" s="84" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="89"/>
-      <c r="N1" s="88" t="s">
+      <c r="M1" s="85"/>
+      <c r="N1" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="89"/>
-      <c r="P1" s="88" t="s">
+      <c r="O1" s="85"/>
+      <c r="P1" s="84" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="88" t="s">
+      <c r="Q1" s="85"/>
+      <c r="R1" s="84" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="89"/>
-      <c r="T1" s="88" t="s">
+      <c r="S1" s="85"/>
+      <c r="T1" s="84" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="89"/>
-      <c r="V1" s="88" t="s">
+      <c r="U1" s="85"/>
+      <c r="V1" s="84" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="89"/>
-      <c r="X1" s="88" t="s">
+      <c r="W1" s="85"/>
+      <c r="X1" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="89"/>
-      <c r="Z1" s="88" t="s">
+      <c r="Y1" s="85"/>
+      <c r="Z1" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="89"/>
-      <c r="AB1" s="88" t="s">
+      <c r="AA1" s="85"/>
+      <c r="AB1" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="89"/>
-      <c r="AD1" s="98" t="s">
+      <c r="AC1" s="85"/>
+      <c r="AD1" s="84" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE1" s="85"/>
+      <c r="AF1" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="AE1" s="100" t="s">
+      <c r="AG1" s="103" t="s">
         <v>65</v>
       </c>
-      <c r="AF1" s="101"/>
-      <c r="AG1" s="101"/>
-      <c r="AH1" s="101"/>
-      <c r="AI1" s="102"/>
-      <c r="AJ1" s="103" t="s">
+      <c r="AH1" s="104"/>
+      <c r="AI1" s="104"/>
+      <c r="AJ1" s="104"/>
+      <c r="AK1" s="105"/>
+      <c r="AL1" s="88" t="s">
         <v>57</v>
       </c>
-      <c r="AK1" s="104"/>
-      <c r="AL1" s="104"/>
-      <c r="AM1" s="104"/>
-      <c r="AN1" s="105"/>
+      <c r="AM1" s="89"/>
+      <c r="AN1" s="89"/>
+      <c r="AO1" s="89"/>
+      <c r="AP1" s="90"/>
     </row>
-    <row r="2" spans="1:40" s="54" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="82"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="78">
+    <row r="2" spans="1:42" s="54" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="108"/>
+      <c r="B2" s="109"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="86">
         <v>45782</v>
       </c>
-      <c r="E2" s="79"/>
-      <c r="F2" s="78">
+      <c r="E2" s="87"/>
+      <c r="F2" s="86">
         <v>45789</v>
       </c>
-      <c r="G2" s="79"/>
-      <c r="H2" s="78">
+      <c r="G2" s="87"/>
+      <c r="H2" s="86">
         <v>45796</v>
       </c>
-      <c r="I2" s="79"/>
-      <c r="J2" s="78">
+      <c r="I2" s="87"/>
+      <c r="J2" s="86">
         <v>45803</v>
       </c>
-      <c r="K2" s="79"/>
-      <c r="L2" s="78">
+      <c r="K2" s="87"/>
+      <c r="L2" s="86">
         <v>45810</v>
       </c>
-      <c r="M2" s="79"/>
-      <c r="N2" s="78">
+      <c r="M2" s="87"/>
+      <c r="N2" s="86">
         <v>45817</v>
       </c>
-      <c r="O2" s="79"/>
-      <c r="P2" s="78">
+      <c r="O2" s="87"/>
+      <c r="P2" s="86">
         <v>45824</v>
       </c>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="78">
+      <c r="Q2" s="87"/>
+      <c r="R2" s="86">
         <v>45831</v>
       </c>
-      <c r="S2" s="79"/>
-      <c r="T2" s="78">
+      <c r="S2" s="87"/>
+      <c r="T2" s="86">
         <v>45838</v>
       </c>
-      <c r="U2" s="79"/>
-      <c r="V2" s="78">
+      <c r="U2" s="87"/>
+      <c r="V2" s="86">
         <v>45845</v>
       </c>
-      <c r="W2" s="79"/>
-      <c r="X2" s="78">
+      <c r="W2" s="87"/>
+      <c r="X2" s="86">
         <v>45852</v>
       </c>
-      <c r="Y2" s="79"/>
-      <c r="Z2" s="78">
+      <c r="Y2" s="87"/>
+      <c r="Z2" s="86">
         <v>45859</v>
       </c>
-      <c r="AA2" s="79"/>
-      <c r="AB2" s="78">
+      <c r="AA2" s="87"/>
+      <c r="AB2" s="86">
         <v>45866</v>
       </c>
-      <c r="AC2" s="79"/>
-      <c r="AD2" s="99"/>
-      <c r="AE2" s="98" t="s">
+      <c r="AC2" s="87"/>
+      <c r="AD2" s="86">
+        <v>45873</v>
+      </c>
+      <c r="AE2" s="87"/>
+      <c r="AF2" s="102"/>
+      <c r="AG2" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="AF2" s="94" t="s">
+      <c r="AH2" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="AG2" s="96" t="s">
+      <c r="AI2" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="AH2" s="90" t="s">
+      <c r="AJ2" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="AI2" s="92" t="s">
+      <c r="AK2" s="95" t="s">
         <v>7</v>
       </c>
-      <c r="AJ2" s="106" t="s">
+      <c r="AL2" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AK2" s="106" t="s">
+      <c r="AM2" s="91" t="s">
         <v>4</v>
       </c>
-      <c r="AL2" s="106" t="s">
+      <c r="AN2" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="AM2" s="106" t="s">
+      <c r="AO2" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="AN2" s="106" t="s">
+      <c r="AP2" s="91" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:40" s="54" customFormat="1" ht="29" customHeight="1" thickBot="1">
-      <c r="A3" s="84"/>
-      <c r="B3" s="85"/>
-      <c r="C3" s="87"/>
+    <row r="3" spans="1:42" s="54" customFormat="1" ht="29" customHeight="1" thickBot="1">
+      <c r="A3" s="110"/>
+      <c r="B3" s="111"/>
+      <c r="C3" s="113"/>
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1883,19 +1947,25 @@
       <c r="AC3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="AD3" s="99"/>
-      <c r="AE3" s="99"/>
-      <c r="AF3" s="95"/>
-      <c r="AG3" s="97"/>
-      <c r="AH3" s="91"/>
-      <c r="AI3" s="93"/>
-      <c r="AJ3" s="107"/>
-      <c r="AK3" s="107"/>
-      <c r="AL3" s="107"/>
-      <c r="AM3" s="107"/>
-      <c r="AN3" s="107"/>
+      <c r="AD3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF3" s="102"/>
+      <c r="AG3" s="102"/>
+      <c r="AH3" s="98"/>
+      <c r="AI3" s="100"/>
+      <c r="AJ3" s="94"/>
+      <c r="AK3" s="96"/>
+      <c r="AL3" s="92"/>
+      <c r="AM3" s="92"/>
+      <c r="AN3" s="92"/>
+      <c r="AO3" s="92"/>
+      <c r="AP3" s="92"/>
     </row>
-    <row r="4" spans="1:40" ht="16" customHeight="1">
+    <row r="4" spans="1:42" ht="16" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>34</v>
       </c>
@@ -1903,268 +1973,295 @@
         <v>35</v>
       </c>
       <c r="C4" s="5">
-        <v>2</v>
+        <f t="shared" ref="C4:C14" si="0">ROUND((AF4-(36*AG4))/AG4,0)</f>
+        <v>1</v>
       </c>
       <c r="D4" s="47"/>
       <c r="E4" s="48"/>
-      <c r="F4" s="110"/>
+      <c r="F4" s="80"/>
       <c r="G4" s="6"/>
       <c r="H4" s="47"/>
       <c r="I4" s="48"/>
-      <c r="J4" s="110"/>
+      <c r="J4" s="80"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="110"/>
+      <c r="L4" s="80"/>
       <c r="M4" s="6"/>
-      <c r="N4" s="110"/>
+      <c r="N4" s="80"/>
       <c r="O4" s="6"/>
-      <c r="P4" s="111">
+      <c r="P4" s="81">
         <v>39</v>
       </c>
       <c r="Q4" s="6">
         <v>17</v>
       </c>
-      <c r="R4" s="111">
+      <c r="R4" s="81">
         <v>38</v>
       </c>
       <c r="S4" s="6">
         <v>18</v>
       </c>
-      <c r="T4" s="111"/>
+      <c r="T4" s="81"/>
       <c r="U4" s="6"/>
-      <c r="V4" s="112">
+      <c r="V4" s="82">
         <v>37</v>
       </c>
       <c r="W4" s="6">
         <v>19</v>
       </c>
-      <c r="X4" s="112">
+      <c r="X4" s="122">
         <v>36</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="123">
         <v>20</v>
       </c>
-      <c r="Z4" s="112">
+      <c r="Z4" s="122">
         <v>38</v>
       </c>
       <c r="AA4" s="75">
         <v>18</v>
       </c>
-      <c r="AB4" s="111">
+      <c r="AB4" s="121">
         <v>35</v>
       </c>
       <c r="AC4" s="75">
         <v>21</v>
       </c>
-      <c r="AD4" s="62">
-        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4</f>
-        <v>223</v>
-      </c>
-      <c r="AE4" s="7">
-        <f>COUNTIF(D4:AB4,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AF4" s="36">
+      <c r="AD4" s="120">
+        <v>37</v>
+      </c>
+      <c r="AE4" s="114">
+        <v>19</v>
+      </c>
+      <c r="AF4" s="62">
+        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4</f>
+        <v>260</v>
+      </c>
+      <c r="AG4" s="7">
+        <f>COUNTIF(D4:AD4,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AH4" s="36">
         <v>3</v>
       </c>
-      <c r="AG4" s="6">
-        <v>8</v>
-      </c>
-      <c r="AH4" s="37">
-        <f>SUMIF(G4:AC4, "&lt;30")+AF4+AG4</f>
-        <v>124</v>
-      </c>
-      <c r="AI4" s="66">
-        <f>AH4/AE4</f>
-        <v>20.666666666666668</v>
-      </c>
-      <c r="AJ4" s="108"/>
-      <c r="AK4" s="37"/>
-      <c r="AL4" s="37"/>
-      <c r="AM4" s="7"/>
-      <c r="AN4" s="55"/>
+      <c r="AI4" s="6">
+        <v>9</v>
+      </c>
+      <c r="AJ4" s="37">
+        <f>SUMIF(G4:AE4, "&lt;30")+AH4+AI4</f>
+        <v>144</v>
+      </c>
+      <c r="AK4" s="66">
+        <f t="shared" ref="AK4:AK22" si="1">AJ4/AG4</f>
+        <v>20.571428571428573</v>
+      </c>
+      <c r="AL4" s="78"/>
+      <c r="AM4" s="37"/>
+      <c r="AN4" s="37"/>
+      <c r="AO4" s="7"/>
+      <c r="AP4" s="55"/>
     </row>
-    <row r="5" spans="1:40">
+    <row r="5" spans="1:42">
       <c r="A5" s="8" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="C5" s="10">
-        <f>ROUND((AD5-(36*AE5))/AE5,0)</f>
-        <v>17</v>
+        <f>ROUND((AF5-(36*AG5))/AG5,0)</f>
+        <v>12</v>
       </c>
       <c r="D5" s="49"/>
       <c r="E5" s="50"/>
-      <c r="F5" s="13">
-        <v>53</v>
-      </c>
-      <c r="G5" s="11">
-        <v>23</v>
-      </c>
+      <c r="F5" s="13"/>
+      <c r="G5" s="11"/>
       <c r="H5" s="49"/>
       <c r="I5" s="50"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="11"/>
+      <c r="J5" s="13">
+        <v>52</v>
+      </c>
+      <c r="K5" s="11">
+        <v>17</v>
+      </c>
       <c r="L5" s="13"/>
       <c r="M5" s="11"/>
       <c r="N5" s="13">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="O5" s="11">
+        <v>23</v>
+      </c>
+      <c r="P5" s="13">
+        <v>46</v>
+      </c>
+      <c r="Q5" s="11">
+        <v>23</v>
+      </c>
+      <c r="R5" s="13">
+        <v>54</v>
+      </c>
+      <c r="S5" s="11">
+        <v>16</v>
+      </c>
+      <c r="T5" s="13">
+        <v>45</v>
+      </c>
+      <c r="U5" s="11">
+        <v>23</v>
+      </c>
+      <c r="V5" s="13">
+        <v>48</v>
+      </c>
+      <c r="W5" s="11">
         <v>19</v>
       </c>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="13">
-        <v>50</v>
-      </c>
-      <c r="S5" s="11">
-        <v>26</v>
-      </c>
-      <c r="T5" s="13">
-        <v>56</v>
-      </c>
-      <c r="U5" s="11">
+      <c r="X5" s="124">
+        <v>49</v>
+      </c>
+      <c r="Y5" s="125">
+        <v>18</v>
+      </c>
+      <c r="Z5" s="70"/>
+      <c r="AA5" s="76"/>
+      <c r="AB5" s="70">
+        <v>46</v>
+      </c>
+      <c r="AC5" s="76">
+        <v>21</v>
+      </c>
+      <c r="AD5" s="119">
+        <v>43</v>
+      </c>
+      <c r="AE5" s="116">
+        <v>23</v>
+      </c>
+      <c r="AF5" s="63">
+        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5+AD5</f>
+        <v>429</v>
+      </c>
+      <c r="AG5" s="12">
+        <f>COUNTIF(D5:AD5,"&gt;30")</f>
+        <v>9</v>
+      </c>
+      <c r="AH5" s="38">
+        <v>1</v>
+      </c>
+      <c r="AI5" s="11">
+        <v>1</v>
+      </c>
+      <c r="AJ5" s="39">
+        <f>SUMIF(G5:AE5, "&lt;30")+AH5+AI5</f>
+        <v>185</v>
+      </c>
+      <c r="AK5" s="67">
+        <f>AJ5/AG5</f>
+        <v>20.555555555555557</v>
+      </c>
+      <c r="AL5" s="56"/>
+      <c r="AM5" s="39"/>
+      <c r="AN5" s="39"/>
+      <c r="AO5" s="12"/>
+      <c r="AP5" s="57"/>
+    </row>
+    <row r="6" spans="1:42">
+      <c r="A6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="V5" s="13"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="13"/>
-      <c r="Y5" s="11"/>
-      <c r="Z5" s="70">
-        <v>54</v>
-      </c>
-      <c r="AA5" s="76">
-        <v>18</v>
-      </c>
-      <c r="AB5" s="70">
-        <v>50</v>
-      </c>
-      <c r="AC5" s="76">
-        <v>22</v>
-      </c>
-      <c r="AD5" s="63">
-        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5</f>
-        <v>320</v>
-      </c>
-      <c r="AE5" s="12">
-        <f>COUNTIF(D5:AB5,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AF5" s="38"/>
-      <c r="AG5" s="11"/>
-      <c r="AH5" s="39">
-        <f>SUMIF(G5:AC5, "&lt;30")+AF5+AG5</f>
-        <v>123</v>
-      </c>
-      <c r="AI5" s="67">
-        <f>AH5/AE5</f>
-        <v>20.5</v>
-      </c>
-      <c r="AJ5" s="56"/>
-      <c r="AK5" s="39"/>
-      <c r="AL5" s="39"/>
-      <c r="AM5" s="12"/>
-      <c r="AN5" s="57" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:40">
-      <c r="A6" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>37</v>
-      </c>
       <c r="C6" s="10">
-        <f>ROUND((AD6-(36*AE6))/AE6,0)</f>
-        <v>11</v>
+        <f>ROUND((AF6-(36*AG6))/AG6,0)</f>
+        <v>17</v>
       </c>
       <c r="D6" s="49"/>
       <c r="E6" s="50"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="11"/>
+      <c r="F6" s="13">
+        <v>53</v>
+      </c>
+      <c r="G6" s="11">
+        <v>23</v>
+      </c>
       <c r="H6" s="49"/>
       <c r="I6" s="50"/>
       <c r="J6" s="13"/>
       <c r="K6" s="11"/>
       <c r="L6" s="13"/>
       <c r="M6" s="11"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="13">
-        <v>43</v>
-      </c>
-      <c r="Q6" s="11">
+      <c r="N6" s="13">
+        <v>57</v>
+      </c>
+      <c r="O6" s="11">
+        <v>19</v>
+      </c>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="11"/>
+      <c r="R6" s="13">
+        <v>50</v>
+      </c>
+      <c r="S6" s="11">
         <v>26</v>
       </c>
-      <c r="R6" s="69">
-        <v>45</v>
-      </c>
-      <c r="S6" s="11">
-        <v>24</v>
-      </c>
-      <c r="T6" s="70"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="70">
+      <c r="T6" s="13">
+        <v>56</v>
+      </c>
+      <c r="U6" s="11">
+        <v>15</v>
+      </c>
+      <c r="V6" s="13"/>
+      <c r="W6" s="11"/>
+      <c r="X6" s="124"/>
+      <c r="Y6" s="125"/>
+      <c r="Z6" s="70">
+        <v>54</v>
+      </c>
+      <c r="AA6" s="76">
+        <v>18</v>
+      </c>
+      <c r="AB6" s="70">
         <v>50</v>
       </c>
-      <c r="W6" s="11">
-        <v>19</v>
-      </c>
-      <c r="X6" s="70">
-        <v>44</v>
-      </c>
-      <c r="Y6" s="11">
-        <v>20</v>
-      </c>
-      <c r="Z6" s="70"/>
-      <c r="AA6" s="76"/>
-      <c r="AB6" s="70">
-        <v>54</v>
-      </c>
       <c r="AC6" s="76">
+        <v>22</v>
+      </c>
+      <c r="AD6" s="115"/>
+      <c r="AE6" s="116"/>
+      <c r="AF6" s="63">
+        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6+AD6</f>
+        <v>320</v>
+      </c>
+      <c r="AG6" s="12">
+        <f>COUNTIF(D6:AD6,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AH6" s="38"/>
+      <c r="AI6" s="11"/>
+      <c r="AJ6" s="39">
+        <f>SUMIF(G6:AE6, "&lt;30")+AH6+AI6</f>
+        <v>123</v>
+      </c>
+      <c r="AK6" s="67">
+        <f>AJ6/AG6</f>
+        <v>20.5</v>
+      </c>
+      <c r="AL6" s="56"/>
+      <c r="AM6" s="39"/>
+      <c r="AN6" s="39"/>
+      <c r="AO6" s="12"/>
+      <c r="AP6" s="57" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:42">
+      <c r="A7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="10">
+        <f>ROUND((AF7-(36*AG7))/AG7,0)</f>
         <v>11</v>
-      </c>
-      <c r="AD6" s="63">
-        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6</f>
-        <v>236</v>
-      </c>
-      <c r="AE6" s="12">
-        <f>COUNTIF(D6:AB6,"&gt;30")</f>
-        <v>5</v>
-      </c>
-      <c r="AF6" s="38">
-        <v>1</v>
-      </c>
-      <c r="AG6" s="11">
-        <v>1</v>
-      </c>
-      <c r="AH6" s="39">
-        <f>SUMIF(G6:AC6, "&lt;30")+AF6+AG6</f>
-        <v>102</v>
-      </c>
-      <c r="AI6" s="67">
-        <f>AH6/AE6</f>
-        <v>20.399999999999999</v>
-      </c>
-      <c r="AJ6" s="59"/>
-      <c r="AK6" s="39"/>
-      <c r="AL6" s="39"/>
-      <c r="AM6" s="12"/>
-      <c r="AN6" s="57"/>
-    </row>
-    <row r="7" spans="1:40">
-      <c r="A7" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="10">
-        <f>ROUND((AD7-(36*AE7))/AE7,0)</f>
-        <v>12</v>
       </c>
       <c r="D7" s="49"/>
       <c r="E7" s="50"/>
@@ -2172,283 +2269,283 @@
       <c r="G7" s="11"/>
       <c r="H7" s="49"/>
       <c r="I7" s="50"/>
-      <c r="J7" s="72">
-        <v>52</v>
-      </c>
-      <c r="K7" s="11">
-        <v>17</v>
-      </c>
+      <c r="J7" s="72"/>
+      <c r="K7" s="11"/>
       <c r="L7" s="72"/>
       <c r="M7" s="11"/>
-      <c r="N7" s="72">
-        <v>46</v>
-      </c>
-      <c r="O7" s="11">
-        <v>23</v>
-      </c>
+      <c r="N7" s="72"/>
+      <c r="O7" s="11"/>
       <c r="P7" s="72">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="Q7" s="11">
-        <v>23</v>
-      </c>
-      <c r="R7" s="72">
-        <v>54</v>
+        <v>26</v>
+      </c>
+      <c r="R7" s="128">
+        <v>45</v>
       </c>
       <c r="S7" s="11">
-        <v>16</v>
-      </c>
-      <c r="T7" s="72">
-        <v>45</v>
-      </c>
-      <c r="U7" s="11">
-        <v>23</v>
-      </c>
-      <c r="V7" s="72">
-        <v>48</v>
+        <v>24</v>
+      </c>
+      <c r="T7" s="77"/>
+      <c r="U7" s="11"/>
+      <c r="V7" s="77">
+        <v>50</v>
       </c>
       <c r="W7" s="11">
         <v>19</v>
       </c>
-      <c r="X7" s="72">
-        <v>49</v>
-      </c>
-      <c r="Y7" s="11">
-        <v>18</v>
+      <c r="X7" s="77">
+        <v>44</v>
+      </c>
+      <c r="Y7" s="125">
+        <v>20</v>
       </c>
       <c r="Z7" s="77"/>
       <c r="AA7" s="76"/>
       <c r="AB7" s="77">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="AC7" s="76">
-        <v>21</v>
-      </c>
-      <c r="AD7" s="63">
-        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7</f>
-        <v>386</v>
-      </c>
-      <c r="AE7" s="12">
-        <f>COUNTIF(D7:AB7,"&gt;30")</f>
-        <v>8</v>
-      </c>
-      <c r="AF7" s="38"/>
-      <c r="AG7" s="11">
+        <v>11</v>
+      </c>
+      <c r="AD7" s="117"/>
+      <c r="AE7" s="116"/>
+      <c r="AF7" s="63">
+        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7+AD7</f>
+        <v>236</v>
+      </c>
+      <c r="AG7" s="12">
+        <f>COUNTIF(D7:AD7,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AH7" s="38">
         <v>1</v>
       </c>
-      <c r="AH7" s="39">
-        <f>SUMIF(G7:AC7, "&lt;30")+AF7+AG7</f>
-        <v>161</v>
-      </c>
-      <c r="AI7" s="67">
-        <f>AH7/AE7</f>
-        <v>20.125</v>
-      </c>
-      <c r="AJ7" s="56"/>
-      <c r="AK7" s="39"/>
-      <c r="AL7" s="39"/>
-      <c r="AM7" s="12"/>
-      <c r="AN7" s="57"/>
+      <c r="AI7" s="11">
+        <v>1</v>
+      </c>
+      <c r="AJ7" s="39">
+        <f>SUMIF(G7:AE7, "&lt;30")+AH7+AI7</f>
+        <v>102</v>
+      </c>
+      <c r="AK7" s="67">
+        <f>AJ7/AG7</f>
+        <v>20.399999999999999</v>
+      </c>
+      <c r="AL7" s="59"/>
+      <c r="AM7" s="39"/>
+      <c r="AN7" s="39"/>
+      <c r="AO7" s="12"/>
+      <c r="AP7" s="57"/>
     </row>
-    <row r="8" spans="1:40">
+    <row r="8" spans="1:42">
       <c r="A8" s="8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C8" s="10">
-        <f>ROUND((AD8-(36*AE8))/AE8,0)</f>
-        <v>14</v>
+        <f>ROUND((AF8-(36*AG8))/AG8,0)</f>
+        <v>7</v>
       </c>
       <c r="D8" s="49"/>
       <c r="E8" s="50"/>
-      <c r="F8" s="13">
-        <v>42</v>
+      <c r="F8" s="65">
+        <v>45</v>
       </c>
       <c r="G8" s="11">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="H8" s="49"/>
       <c r="I8" s="50"/>
-      <c r="J8" s="13"/>
+      <c r="J8" s="65"/>
       <c r="K8" s="11"/>
-      <c r="L8" s="13">
-        <v>54</v>
+      <c r="L8" s="65">
+        <v>43</v>
       </c>
       <c r="M8" s="11">
+        <v>19</v>
+      </c>
+      <c r="N8" s="14">
+        <v>41</v>
+      </c>
+      <c r="O8" s="11">
+        <v>21</v>
+      </c>
+      <c r="P8" s="40">
+        <v>47</v>
+      </c>
+      <c r="Q8" s="11">
         <v>15</v>
       </c>
-      <c r="N8" s="13"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="13">
-        <v>54</v>
-      </c>
-      <c r="Q8" s="11">
+      <c r="R8" s="40">
+        <v>42</v>
+      </c>
+      <c r="S8" s="11">
+        <v>20</v>
+      </c>
+      <c r="T8" s="40">
+        <v>43</v>
+      </c>
+      <c r="U8" s="11">
+        <v>19</v>
+      </c>
+      <c r="V8" s="40">
+        <v>44</v>
+      </c>
+      <c r="W8" s="11">
+        <v>18</v>
+      </c>
+      <c r="X8" s="70">
+        <v>48</v>
+      </c>
+      <c r="Y8" s="125">
         <v>16</v>
       </c>
-      <c r="R8" s="13">
-        <v>53</v>
-      </c>
-      <c r="S8" s="11">
-        <v>16</v>
-      </c>
-      <c r="T8" s="13"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="69">
-        <v>46</v>
-      </c>
-      <c r="W8" s="11">
+      <c r="Z8" s="70">
+        <v>40</v>
+      </c>
+      <c r="AA8" s="76">
+        <v>22</v>
+      </c>
+      <c r="AB8" s="70">
+        <v>40</v>
+      </c>
+      <c r="AC8" s="76">
+        <v>22</v>
+      </c>
+      <c r="AD8" s="115">
+        <v>38</v>
+      </c>
+      <c r="AE8" s="116">
         <v>23</v>
       </c>
-      <c r="X8" s="70">
-        <v>49</v>
-      </c>
-      <c r="Y8" s="11">
-        <v>19</v>
-      </c>
-      <c r="Z8" s="70">
-        <v>50</v>
-      </c>
-      <c r="AA8" s="76">
-        <v>18</v>
-      </c>
-      <c r="AB8" s="70"/>
-      <c r="AC8" s="76"/>
-      <c r="AD8" s="63">
-        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8</f>
-        <v>348</v>
-      </c>
-      <c r="AE8" s="12">
-        <f>COUNTIF(D8:AB8,"&gt;30")</f>
-        <v>7</v>
-      </c>
-      <c r="AF8" s="38">
+      <c r="AF8" s="63">
+        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8+AD8</f>
+        <v>471</v>
+      </c>
+      <c r="AG8" s="12">
+        <f>COUNTIF(D8:AD8,"&gt;30")</f>
+        <v>11</v>
+      </c>
+      <c r="AH8" s="38">
         <v>1</v>
       </c>
-      <c r="AG8" s="11">
-        <v>1</v>
-      </c>
-      <c r="AH8" s="39">
-        <f>SUMIF(G8:AC8, "&lt;30")+AF8+AG8</f>
-        <v>136</v>
-      </c>
-      <c r="AI8" s="67">
-        <f>AH8/AE8</f>
-        <v>19.428571428571427</v>
-      </c>
-      <c r="AJ8" s="58"/>
-      <c r="AK8" s="39"/>
-      <c r="AL8" s="39"/>
-      <c r="AM8" s="12"/>
-      <c r="AN8" s="57"/>
+      <c r="AI8" s="11">
+        <v>5</v>
+      </c>
+      <c r="AJ8" s="39">
+        <f>SUMIF(G8:AE8, "&lt;30")+AH8+AI8</f>
+        <v>218</v>
+      </c>
+      <c r="AK8" s="67">
+        <f>AJ8/AG8</f>
+        <v>19.818181818181817</v>
+      </c>
+      <c r="AL8" s="58"/>
+      <c r="AM8" s="39"/>
+      <c r="AN8" s="39"/>
+      <c r="AO8" s="12"/>
+      <c r="AP8" s="57"/>
     </row>
-    <row r="9" spans="1:40">
+    <row r="9" spans="1:42">
       <c r="A9" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C9" s="10">
-        <f>ROUND((AD9-(36*AE9))/AE9,0)</f>
-        <v>7</v>
+        <f>ROUND((AF9-(36*AG9))/AG9,0)</f>
+        <v>14</v>
       </c>
       <c r="D9" s="49"/>
       <c r="E9" s="50"/>
-      <c r="F9" s="65">
-        <v>45</v>
+      <c r="F9" s="13">
+        <v>42</v>
       </c>
       <c r="G9" s="11">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="H9" s="49"/>
       <c r="I9" s="50"/>
-      <c r="J9" s="65"/>
+      <c r="J9" s="13"/>
       <c r="K9" s="11"/>
-      <c r="L9" s="65">
-        <v>43</v>
+      <c r="L9" s="13">
+        <v>54</v>
       </c>
       <c r="M9" s="11">
+        <v>15</v>
+      </c>
+      <c r="N9" s="13"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="13">
+        <v>54</v>
+      </c>
+      <c r="Q9" s="11">
+        <v>16</v>
+      </c>
+      <c r="R9" s="13">
+        <v>53</v>
+      </c>
+      <c r="S9" s="11">
+        <v>16</v>
+      </c>
+      <c r="T9" s="13"/>
+      <c r="U9" s="11"/>
+      <c r="V9" s="69">
+        <v>46</v>
+      </c>
+      <c r="W9" s="11">
+        <v>23</v>
+      </c>
+      <c r="X9" s="70">
+        <v>49</v>
+      </c>
+      <c r="Y9" s="125">
         <v>19</v>
       </c>
-      <c r="N9" s="14">
-        <v>41</v>
-      </c>
-      <c r="O9" s="11">
-        <v>21</v>
-      </c>
-      <c r="P9" s="40">
-        <v>47</v>
-      </c>
-      <c r="Q9" s="11">
-        <v>15</v>
-      </c>
-      <c r="R9" s="40">
-        <v>42</v>
-      </c>
-      <c r="S9" s="11">
-        <v>20</v>
-      </c>
-      <c r="T9" s="40">
-        <v>43</v>
-      </c>
-      <c r="U9" s="11">
-        <v>19</v>
-      </c>
-      <c r="V9" s="40">
-        <v>44</v>
-      </c>
-      <c r="W9" s="11">
+      <c r="Z9" s="70">
+        <v>50</v>
+      </c>
+      <c r="AA9" s="76">
         <v>18</v>
       </c>
-      <c r="X9" s="40">
-        <v>48</v>
-      </c>
-      <c r="Y9" s="11">
-        <v>16</v>
-      </c>
-      <c r="Z9" s="40">
-        <v>40</v>
-      </c>
-      <c r="AA9" s="76">
-        <v>22</v>
-      </c>
-      <c r="AB9" s="40">
-        <v>40</v>
-      </c>
-      <c r="AC9" s="76">
-        <v>22</v>
-      </c>
-      <c r="AD9" s="63">
-        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9</f>
-        <v>433</v>
-      </c>
-      <c r="AE9" s="12">
-        <f>COUNTIF(D9:AB9,"&gt;30")</f>
-        <v>10</v>
-      </c>
-      <c r="AF9" s="38">
+      <c r="AB9" s="70"/>
+      <c r="AC9" s="76"/>
+      <c r="AD9" s="115"/>
+      <c r="AE9" s="116"/>
+      <c r="AF9" s="63">
+        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9+AD9</f>
+        <v>348</v>
+      </c>
+      <c r="AG9" s="12">
+        <f>COUNTIF(D9:AD9,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AH9" s="38">
         <v>1</v>
       </c>
-      <c r="AG9" s="11">
-        <v>4</v>
-      </c>
-      <c r="AH9" s="39">
-        <f>SUMIF(G9:AC9, "&lt;30")+AF9+AG9</f>
-        <v>194</v>
-      </c>
-      <c r="AI9" s="67">
-        <f>AH9/AE9</f>
-        <v>19.399999999999999</v>
-      </c>
-      <c r="AJ9" s="56"/>
-      <c r="AK9" s="39"/>
-      <c r="AL9" s="39"/>
-      <c r="AM9" s="12"/>
-      <c r="AN9" s="57"/>
+      <c r="AI9" s="11">
+        <v>1</v>
+      </c>
+      <c r="AJ9" s="39">
+        <f>SUMIF(G9:AE9, "&lt;30")+AH9+AI9</f>
+        <v>136</v>
+      </c>
+      <c r="AK9" s="67">
+        <f>AJ9/AG9</f>
+        <v>19.428571428571427</v>
+      </c>
+      <c r="AL9" s="56"/>
+      <c r="AM9" s="39"/>
+      <c r="AN9" s="39"/>
+      <c r="AO9" s="12"/>
+      <c r="AP9" s="57"/>
     </row>
-    <row r="10" spans="1:40">
+    <row r="10" spans="1:42">
       <c r="A10" s="8" t="s">
         <v>12</v>
       </c>
@@ -2456,8 +2553,8 @@
         <v>13</v>
       </c>
       <c r="C10" s="10">
-        <f>ROUND((AD10-(36*AE10))/AE10,0)</f>
-        <v>12</v>
+        <f>ROUND((AF10-(36*AG10))/AG10,0)</f>
+        <v>11</v>
       </c>
       <c r="D10" s="49"/>
       <c r="E10" s="50"/>
@@ -2503,142 +2600,154 @@
       <c r="W10" s="11">
         <v>19</v>
       </c>
-      <c r="X10" s="40">
+      <c r="X10" s="70">
         <v>53</v>
       </c>
-      <c r="Y10" s="11">
+      <c r="Y10" s="125">
         <v>13</v>
       </c>
-      <c r="Z10" s="40">
+      <c r="Z10" s="70">
         <v>52</v>
       </c>
       <c r="AA10" s="76">
         <v>13</v>
       </c>
-      <c r="AB10" s="40">
+      <c r="AB10" s="70">
         <v>44</v>
       </c>
       <c r="AC10" s="76">
         <v>22</v>
       </c>
-      <c r="AD10" s="63">
-        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10</f>
-        <v>428</v>
-      </c>
-      <c r="AE10" s="12">
-        <f>COUNTIF(D10:AB10,"&gt;30")</f>
-        <v>9</v>
-      </c>
-      <c r="AF10" s="38">
+      <c r="AD10" s="115">
+        <v>42</v>
+      </c>
+      <c r="AE10" s="116">
+        <v>24</v>
+      </c>
+      <c r="AF10" s="63">
+        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10+AD10</f>
+        <v>470</v>
+      </c>
+      <c r="AG10" s="12">
+        <f>COUNTIF(D10:AD10,"&gt;30")</f>
+        <v>10</v>
+      </c>
+      <c r="AH10" s="38">
         <v>2</v>
       </c>
-      <c r="AG10" s="11">
+      <c r="AI10" s="11">
         <v>1</v>
       </c>
-      <c r="AH10" s="39">
-        <f>SUMIF(G10:AC10, "&lt;30")+AF10+AG10</f>
-        <v>170</v>
-      </c>
-      <c r="AI10" s="67">
-        <f>AH10/AE10</f>
-        <v>18.888888888888889</v>
-      </c>
-      <c r="AJ10" s="113"/>
-      <c r="AK10" s="39"/>
-      <c r="AL10" s="39"/>
-      <c r="AM10" s="12"/>
-      <c r="AN10" s="57"/>
+      <c r="AJ10" s="39">
+        <f>SUMIF(G10:AE10, "&lt;30")+AH10+AI10</f>
+        <v>194</v>
+      </c>
+      <c r="AK10" s="67">
+        <f>AJ10/AG10</f>
+        <v>19.399999999999999</v>
+      </c>
+      <c r="AL10" s="83"/>
+      <c r="AM10" s="39"/>
+      <c r="AN10" s="39"/>
+      <c r="AO10" s="12"/>
+      <c r="AP10" s="57"/>
     </row>
-    <row r="11" spans="1:40">
+    <row r="11" spans="1:42">
       <c r="A11" s="8" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C11" s="10">
-        <f>ROUND((AD11-(36*AE11))/AE11,0)</f>
-        <v>12</v>
+        <f>ROUND((AF11-(36*AG11))/AG11,0)</f>
+        <v>8</v>
       </c>
       <c r="D11" s="49"/>
       <c r="E11" s="50"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="11"/>
+      <c r="F11" s="13">
+        <v>41</v>
+      </c>
+      <c r="G11" s="11">
+        <v>21</v>
+      </c>
       <c r="H11" s="49"/>
       <c r="I11" s="50"/>
-      <c r="J11" s="15"/>
+      <c r="J11" s="13"/>
       <c r="K11" s="11"/>
-      <c r="L11" s="15"/>
+      <c r="L11" s="13"/>
       <c r="M11" s="11"/>
-      <c r="N11" s="15"/>
-      <c r="O11" s="11"/>
+      <c r="N11" s="53">
+        <v>48</v>
+      </c>
+      <c r="O11" s="11">
+        <v>14</v>
+      </c>
       <c r="P11" s="40">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Q11" s="11">
+        <v>18</v>
+      </c>
+      <c r="R11" s="40"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="40"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="40"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="69">
+        <v>40</v>
+      </c>
+      <c r="Y11" s="125">
+        <v>22</v>
+      </c>
+      <c r="Z11" s="70">
+        <v>44</v>
+      </c>
+      <c r="AA11" s="76">
+        <v>17</v>
+      </c>
+      <c r="AB11" s="70">
+        <v>46</v>
+      </c>
+      <c r="AC11" s="76">
+        <v>16</v>
+      </c>
+      <c r="AD11" s="118">
+        <v>42</v>
+      </c>
+      <c r="AE11" s="116">
         <v>20</v>
       </c>
-      <c r="R11" s="40">
-        <v>50</v>
-      </c>
-      <c r="S11" s="11">
-        <v>17</v>
-      </c>
-      <c r="T11" s="40">
-        <v>46</v>
-      </c>
-      <c r="U11" s="11">
-        <v>21</v>
-      </c>
-      <c r="V11" s="40">
-        <v>47</v>
-      </c>
-      <c r="W11" s="11">
-        <v>19</v>
-      </c>
-      <c r="X11" s="40">
-        <v>44</v>
-      </c>
-      <c r="Y11" s="11">
-        <v>22</v>
-      </c>
-      <c r="Z11" s="40">
-        <v>52</v>
-      </c>
-      <c r="AA11" s="76">
-        <v>14</v>
-      </c>
-      <c r="AB11" s="40">
-        <v>47</v>
-      </c>
-      <c r="AC11" s="76">
-        <v>19</v>
-      </c>
-      <c r="AD11" s="63">
-        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11</f>
-        <v>333</v>
-      </c>
-      <c r="AE11" s="12">
-        <f>COUNTIF(D11:AB11,"&gt;30")</f>
+      <c r="AF11" s="63">
+        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11+AD11</f>
+        <v>305</v>
+      </c>
+      <c r="AG11" s="12">
+        <f>COUNTIF(D11:AD11,"&gt;30")</f>
         <v>7</v>
       </c>
-      <c r="AF11" s="38"/>
-      <c r="AG11" s="11"/>
-      <c r="AH11" s="39">
-        <f>SUMIF(G11:AC11, "&lt;30")+AF11+AG11</f>
-        <v>132</v>
-      </c>
-      <c r="AI11" s="67">
-        <f>AH11/AE11</f>
-        <v>18.857142857142858</v>
-      </c>
-      <c r="AJ11" s="56"/>
-      <c r="AK11" s="39"/>
-      <c r="AL11" s="39"/>
-      <c r="AM11" s="12"/>
-      <c r="AN11" s="57"/>
+      <c r="AH11" s="38">
+        <v>2</v>
+      </c>
+      <c r="AI11" s="11">
+        <v>1</v>
+      </c>
+      <c r="AJ11" s="39">
+        <f>SUMIF(G11:AE11, "&lt;30")+AH11+AI11</f>
+        <v>131</v>
+      </c>
+      <c r="AK11" s="67">
+        <f>AJ11/AG11</f>
+        <v>18.714285714285715</v>
+      </c>
+      <c r="AL11" s="59"/>
+      <c r="AM11" s="39"/>
+      <c r="AN11" s="39"/>
+      <c r="AO11" s="12"/>
+      <c r="AP11" s="57"/>
     </row>
-    <row r="12" spans="1:40">
+    <row r="12" spans="1:42">
       <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
@@ -2646,7 +2755,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="10">
-        <f>ROUND((AD12-(36*AE12))/AE12,0)</f>
+        <f>ROUND((AF12-(36*AG12))/AG12,0)</f>
         <v>15</v>
       </c>
       <c r="D12" s="49"/>
@@ -2681,10 +2790,10 @@
       <c r="U12" s="11"/>
       <c r="V12" s="13"/>
       <c r="W12" s="11"/>
-      <c r="X12" s="13">
+      <c r="X12" s="124">
         <v>48</v>
       </c>
-      <c r="Y12" s="11">
+      <c r="Y12" s="125">
         <v>21</v>
       </c>
       <c r="Z12" s="70"/>
@@ -2695,120 +2804,128 @@
       <c r="AC12" s="76">
         <v>18</v>
       </c>
-      <c r="AD12" s="63">
-        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12</f>
+      <c r="AD12" s="115"/>
+      <c r="AE12" s="116"/>
+      <c r="AF12" s="63">
+        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12+AD12</f>
         <v>253</v>
       </c>
-      <c r="AE12" s="12">
-        <f>COUNTIF(D12:AB12,"&gt;30")</f>
+      <c r="AG12" s="12">
+        <f>COUNTIF(D12:AD12,"&gt;30")</f>
         <v>5</v>
       </c>
-      <c r="AF12" s="38"/>
-      <c r="AG12" s="11"/>
-      <c r="AH12" s="39">
-        <f>SUMIF(G12:AC12, "&lt;30")+AF12+AG12</f>
+      <c r="AH12" s="38"/>
+      <c r="AI12" s="11"/>
+      <c r="AJ12" s="39">
+        <f>SUMIF(G12:AE12, "&lt;30")+AH12+AI12</f>
         <v>92</v>
       </c>
-      <c r="AI12" s="67">
-        <f>AH12/AE12</f>
+      <c r="AK12" s="67">
+        <f>AJ12/AG12</f>
         <v>18.399999999999999</v>
       </c>
-      <c r="AJ12" s="59"/>
-      <c r="AK12" s="39"/>
-      <c r="AL12" s="39"/>
-      <c r="AM12" s="12"/>
-      <c r="AN12" s="57"/>
+      <c r="AL12" s="59"/>
+      <c r="AM12" s="39"/>
+      <c r="AN12" s="39"/>
+      <c r="AO12" s="12"/>
+      <c r="AP12" s="57"/>
     </row>
-    <row r="13" spans="1:40">
+    <row r="13" spans="1:42">
       <c r="A13" s="8" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C13" s="10">
-        <f>ROUND((AD13-(36*AE13))/AE13,0)</f>
-        <v>8</v>
+        <f>ROUND((AF13-(36*AG13))/AG13,0)</f>
+        <v>12</v>
       </c>
       <c r="D13" s="49"/>
       <c r="E13" s="50"/>
-      <c r="F13" s="13">
-        <v>41</v>
-      </c>
-      <c r="G13" s="11">
-        <v>21</v>
-      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="11"/>
       <c r="H13" s="49"/>
       <c r="I13" s="50"/>
-      <c r="J13" s="13"/>
+      <c r="J13" s="15"/>
       <c r="K13" s="11"/>
-      <c r="L13" s="13"/>
+      <c r="L13" s="15"/>
       <c r="M13" s="11"/>
-      <c r="N13" s="53">
-        <v>48</v>
-      </c>
-      <c r="O13" s="11">
+      <c r="N13" s="15"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="40">
+        <v>47</v>
+      </c>
+      <c r="Q13" s="11">
+        <v>20</v>
+      </c>
+      <c r="R13" s="40">
+        <v>50</v>
+      </c>
+      <c r="S13" s="11">
+        <v>17</v>
+      </c>
+      <c r="T13" s="40">
+        <v>46</v>
+      </c>
+      <c r="U13" s="11">
+        <v>21</v>
+      </c>
+      <c r="V13" s="40">
+        <v>47</v>
+      </c>
+      <c r="W13" s="11">
+        <v>19</v>
+      </c>
+      <c r="X13" s="70">
+        <v>44</v>
+      </c>
+      <c r="Y13" s="125">
+        <v>22</v>
+      </c>
+      <c r="Z13" s="70">
+        <v>52</v>
+      </c>
+      <c r="AA13" s="76">
         <v>14</v>
       </c>
-      <c r="P13" s="40">
-        <v>44</v>
-      </c>
-      <c r="Q13" s="11">
-        <v>18</v>
-      </c>
-      <c r="R13" s="40"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="40"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="40"/>
-      <c r="W13" s="11"/>
-      <c r="X13" s="14">
-        <v>40</v>
-      </c>
-      <c r="Y13" s="11">
-        <v>22</v>
-      </c>
-      <c r="Z13" s="40">
-        <v>44</v>
-      </c>
-      <c r="AA13" s="76">
-        <v>17</v>
-      </c>
-      <c r="AB13" s="40">
-        <v>46</v>
+      <c r="AB13" s="70">
+        <v>47</v>
       </c>
       <c r="AC13" s="76">
-        <v>16</v>
-      </c>
-      <c r="AD13" s="63">
-        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13</f>
-        <v>263</v>
-      </c>
-      <c r="AE13" s="12">
-        <f>COUNTIF(D13:AB13,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AF13" s="38">
-        <v>1</v>
-      </c>
-      <c r="AG13" s="11">
-        <v>1</v>
-      </c>
-      <c r="AH13" s="39">
-        <f>SUMIF(G13:AC13, "&lt;30")+AF13+AG13</f>
-        <v>110</v>
-      </c>
-      <c r="AI13" s="67">
-        <f>AH13/AE13</f>
-        <v>18.333333333333332</v>
-      </c>
-      <c r="AJ13" s="59"/>
-      <c r="AK13" s="39"/>
-      <c r="AL13" s="39"/>
-      <c r="AM13" s="12"/>
-      <c r="AN13" s="57"/>
+        <v>19</v>
+      </c>
+      <c r="AD13" s="115">
+        <v>51</v>
+      </c>
+      <c r="AE13" s="116">
+        <v>15</v>
+      </c>
+      <c r="AF13" s="63">
+        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13+AD13</f>
+        <v>384</v>
+      </c>
+      <c r="AG13" s="12">
+        <f>COUNTIF(D13:AD13,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AH13" s="38"/>
+      <c r="AI13" s="11"/>
+      <c r="AJ13" s="39">
+        <f>SUMIF(G13:AE13, "&lt;30")+AH13+AI13</f>
+        <v>147</v>
+      </c>
+      <c r="AK13" s="67">
+        <f>AJ13/AG13</f>
+        <v>18.375</v>
+      </c>
+      <c r="AL13" s="56"/>
+      <c r="AM13" s="39"/>
+      <c r="AN13" s="39"/>
+      <c r="AO13" s="12"/>
+      <c r="AP13" s="57"/>
     </row>
-    <row r="14" spans="1:40">
+    <row r="14" spans="1:42">
       <c r="A14" s="8" t="s">
         <v>17</v>
       </c>
@@ -2816,6 +2933,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="10">
+        <f>ROUND((AF14-(36*AG14))/AG14,0)</f>
         <v>22</v>
       </c>
       <c r="D14" s="49"/>
@@ -2850,37 +2968,39 @@
       <c r="W14" s="11">
         <v>17</v>
       </c>
-      <c r="X14" s="13"/>
-      <c r="Y14" s="11"/>
+      <c r="X14" s="124"/>
+      <c r="Y14" s="125"/>
       <c r="Z14" s="70"/>
       <c r="AA14" s="76"/>
       <c r="AB14" s="70"/>
       <c r="AC14" s="76"/>
-      <c r="AD14" s="63">
-        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14</f>
+      <c r="AD14" s="115"/>
+      <c r="AE14" s="116"/>
+      <c r="AF14" s="63">
+        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14+AD14</f>
         <v>173</v>
       </c>
-      <c r="AE14" s="12">
-        <f>COUNTIF(D14:AB14,"&gt;30")</f>
+      <c r="AG14" s="12">
+        <f>COUNTIF(D14:AD14,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="AF14" s="38"/>
-      <c r="AG14" s="11"/>
-      <c r="AH14" s="39">
-        <f>SUMIF(G14:AC14, "&lt;30")+AF14+AG14</f>
+      <c r="AH14" s="38"/>
+      <c r="AI14" s="11"/>
+      <c r="AJ14" s="39">
+        <f>SUMIF(G14:AE14, "&lt;30")+AH14+AI14</f>
         <v>55</v>
       </c>
-      <c r="AI14" s="67">
-        <f>AH14/AE14</f>
+      <c r="AK14" s="67">
+        <f>AJ14/AG14</f>
         <v>18.333333333333332</v>
       </c>
-      <c r="AJ14" s="59"/>
-      <c r="AK14" s="39"/>
-      <c r="AL14" s="39"/>
-      <c r="AM14" s="12"/>
-      <c r="AN14" s="57"/>
+      <c r="AL14" s="59"/>
+      <c r="AM14" s="39"/>
+      <c r="AN14" s="39"/>
+      <c r="AO14" s="12"/>
+      <c r="AP14" s="57"/>
     </row>
-    <row r="15" spans="1:40">
+    <row r="15" spans="1:42">
       <c r="A15" s="8" t="s">
         <v>18</v>
       </c>
@@ -2888,7 +3008,7 @@
         <v>19</v>
       </c>
       <c r="C15" s="10">
-        <f>ROUND((AD15-(36*AE15))/AE15,0)</f>
+        <f>ROUND((AF15-(36*AG15))/AG15,0)</f>
         <v>9</v>
       </c>
       <c r="D15" s="49"/>
@@ -2923,10 +3043,10 @@
       <c r="U15" s="11"/>
       <c r="V15" s="13"/>
       <c r="W15" s="11"/>
-      <c r="X15" s="13">
+      <c r="X15" s="124">
         <v>47</v>
       </c>
-      <c r="Y15" s="11">
+      <c r="Y15" s="125">
         <v>16</v>
       </c>
       <c r="Z15" s="69">
@@ -2935,41 +3055,47 @@
       <c r="AA15" s="76">
         <v>22</v>
       </c>
-      <c r="AB15" s="109">
+      <c r="AB15" s="79">
         <v>50</v>
       </c>
       <c r="AC15" s="76">
         <v>13</v>
       </c>
-      <c r="AD15" s="63">
-        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15</f>
-        <v>269</v>
-      </c>
-      <c r="AE15" s="12">
-        <f>COUNTIF(D15:AB15,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AF15" s="38">
+      <c r="AD15" s="115">
+        <v>44</v>
+      </c>
+      <c r="AE15" s="116">
+        <v>19</v>
+      </c>
+      <c r="AF15" s="63">
+        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15+AD15</f>
+        <v>313</v>
+      </c>
+      <c r="AG15" s="12">
+        <f>COUNTIF(D15:AD15,"&gt;30")</f>
+        <v>7</v>
+      </c>
+      <c r="AH15" s="38">
         <v>2</v>
       </c>
-      <c r="AG15" s="11">
+      <c r="AI15" s="11">
         <v>1</v>
       </c>
-      <c r="AH15" s="39">
-        <f>SUMIF(G15:AC15, "&lt;30")+AF15+AG15</f>
-        <v>109</v>
-      </c>
-      <c r="AI15" s="67">
-        <f>AH15/AE15</f>
-        <v>18.166666666666668</v>
-      </c>
-      <c r="AJ15" s="59"/>
-      <c r="AK15" s="39"/>
-      <c r="AL15" s="39"/>
-      <c r="AM15" s="12"/>
-      <c r="AN15" s="57"/>
+      <c r="AJ15" s="39">
+        <f>SUMIF(G15:AE15, "&lt;30")+AH15+AI15</f>
+        <v>128</v>
+      </c>
+      <c r="AK15" s="67">
+        <f>AJ15/AG15</f>
+        <v>18.285714285714285</v>
+      </c>
+      <c r="AL15" s="59"/>
+      <c r="AM15" s="39"/>
+      <c r="AN15" s="39"/>
+      <c r="AO15" s="12"/>
+      <c r="AP15" s="57"/>
     </row>
-    <row r="16" spans="1:40">
+    <row r="16" spans="1:42">
       <c r="A16" s="8" t="s">
         <v>20</v>
       </c>
@@ -2977,7 +3103,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="10">
-        <f>ROUND((AD16-(36*AE16))/AE16,0)</f>
+        <f>ROUND((AF16-(36*AG16))/AG16,0)</f>
         <v>18</v>
       </c>
       <c r="D16" s="49"/>
@@ -3023,13 +3149,13 @@
       <c r="X16" s="70">
         <v>50</v>
       </c>
-      <c r="Y16" s="11">
+      <c r="Y16" s="125">
         <v>23</v>
       </c>
       <c r="Z16" s="70">
         <v>56</v>
       </c>
-      <c r="AA16" s="11">
+      <c r="AA16" s="125">
         <v>16</v>
       </c>
       <c r="AB16" s="69">
@@ -3038,33 +3164,39 @@
       <c r="AC16" s="76">
         <v>23</v>
       </c>
-      <c r="AD16" s="63">
-        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16</f>
-        <v>430</v>
-      </c>
-      <c r="AE16" s="12">
-        <f>COUNTIF(D16:AB16,"&gt;30")</f>
-        <v>8</v>
-      </c>
-      <c r="AF16" s="38">
+      <c r="AD16" s="115">
+        <v>54</v>
+      </c>
+      <c r="AE16" s="116">
+        <v>18</v>
+      </c>
+      <c r="AF16" s="63">
+        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16+AD16</f>
+        <v>484</v>
+      </c>
+      <c r="AG16" s="12">
+        <f>COUNTIF(D16:AD16,"&gt;30")</f>
+        <v>9</v>
+      </c>
+      <c r="AH16" s="38">
         <v>2</v>
       </c>
-      <c r="AG16" s="11"/>
-      <c r="AH16" s="39">
-        <f>SUMIF(G16:AC16, "&lt;30")+AF16+AG16</f>
-        <v>145</v>
-      </c>
-      <c r="AI16" s="67">
-        <f>AH16/AE16</f>
-        <v>18.125</v>
-      </c>
-      <c r="AJ16" s="59"/>
-      <c r="AK16" s="39"/>
-      <c r="AL16" s="39"/>
-      <c r="AM16" s="12"/>
-      <c r="AN16" s="57"/>
+      <c r="AI16" s="11"/>
+      <c r="AJ16" s="39">
+        <f>SUMIF(G16:AE16, "&lt;30")+AH16+AI16</f>
+        <v>163</v>
+      </c>
+      <c r="AK16" s="67">
+        <f>AJ16/AG16</f>
+        <v>18.111111111111111</v>
+      </c>
+      <c r="AL16" s="59"/>
+      <c r="AM16" s="39"/>
+      <c r="AN16" s="39"/>
+      <c r="AO16" s="12"/>
+      <c r="AP16" s="57"/>
     </row>
-    <row r="17" spans="1:40">
+    <row r="17" spans="1:42">
       <c r="A17" s="8" t="s">
         <v>30</v>
       </c>
@@ -3072,7 +3204,7 @@
         <v>38</v>
       </c>
       <c r="C17" s="10">
-        <f>ROUND((AD17-(36*AE17))/AE17,0)</f>
+        <f>ROUND((AF17-(36*AG17))/AG17,0)</f>
         <v>13</v>
       </c>
       <c r="D17" s="49"/>
@@ -3107,16 +3239,16 @@
       </c>
       <c r="V17" s="13"/>
       <c r="W17" s="11"/>
-      <c r="X17" s="13">
+      <c r="X17" s="124">
         <v>48</v>
       </c>
-      <c r="Y17" s="11">
+      <c r="Y17" s="125">
         <v>20</v>
       </c>
-      <c r="Z17" s="13">
+      <c r="Z17" s="124">
         <v>50</v>
       </c>
-      <c r="AA17" s="11">
+      <c r="AA17" s="125">
         <v>18</v>
       </c>
       <c r="AB17" s="70">
@@ -3125,198 +3257,213 @@
       <c r="AC17" s="76">
         <v>21</v>
       </c>
-      <c r="AD17" s="63">
-        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17</f>
+      <c r="AD17" s="115"/>
+      <c r="AE17" s="116"/>
+      <c r="AF17" s="63">
+        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17+AD17</f>
         <v>295</v>
       </c>
-      <c r="AE17" s="12">
-        <f>COUNTIF(D17:AB17,"&gt;30")</f>
+      <c r="AG17" s="12">
+        <f>COUNTIF(D17:AD17,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AF17" s="38"/>
-      <c r="AG17" s="11"/>
-      <c r="AH17" s="39">
-        <f>SUMIF(G17:AC17, "&lt;30")+AF17+AG17</f>
+      <c r="AH17" s="38"/>
+      <c r="AI17" s="11"/>
+      <c r="AJ17" s="39">
+        <f>SUMIF(G17:AE17, "&lt;30")+AH17+AI17</f>
         <v>105</v>
       </c>
-      <c r="AI17" s="67">
-        <f>AH17/AE17</f>
+      <c r="AK17" s="67">
+        <f>AJ17/AG17</f>
         <v>17.5</v>
       </c>
-      <c r="AJ17" s="56"/>
-      <c r="AK17" s="39"/>
-      <c r="AL17" s="39"/>
-      <c r="AM17" s="12"/>
-      <c r="AN17" s="57"/>
+      <c r="AL17" s="56"/>
+      <c r="AM17" s="39"/>
+      <c r="AN17" s="39"/>
+      <c r="AO17" s="12"/>
+      <c r="AP17" s="57"/>
     </row>
-    <row r="18" spans="1:40">
+    <row r="18" spans="1:42">
       <c r="A18" s="8" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C18" s="10">
-        <v>9</v>
+        <f>ROUND((AF18-(36*AG18))/AG18,0)</f>
+        <v>12</v>
       </c>
       <c r="D18" s="49"/>
       <c r="E18" s="50"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="11"/>
+      <c r="F18" s="13">
+        <v>46</v>
+      </c>
+      <c r="G18" s="11">
+        <v>18</v>
+      </c>
       <c r="H18" s="49"/>
       <c r="I18" s="50"/>
-      <c r="J18" s="15"/>
+      <c r="J18" s="13"/>
       <c r="K18" s="11"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="40">
-        <v>45</v>
+      <c r="L18" s="13">
+        <v>46</v>
+      </c>
+      <c r="M18" s="11">
+        <v>18</v>
+      </c>
+      <c r="N18" s="13">
+        <v>46</v>
       </c>
       <c r="O18" s="11">
         <v>18</v>
       </c>
-      <c r="P18" s="40">
-        <v>43</v>
+      <c r="P18" s="13">
+        <v>46</v>
       </c>
       <c r="Q18" s="11">
-        <v>20</v>
-      </c>
-      <c r="R18" s="40"/>
-      <c r="S18" s="11"/>
-      <c r="T18" s="40"/>
-      <c r="U18" s="11"/>
-      <c r="V18" s="40"/>
+        <v>18</v>
+      </c>
+      <c r="R18" s="13">
+        <v>47</v>
+      </c>
+      <c r="S18" s="11">
+        <v>14</v>
+      </c>
+      <c r="T18" s="13">
+        <v>52</v>
+      </c>
+      <c r="U18" s="11">
+        <v>13</v>
+      </c>
+      <c r="V18" s="13"/>
       <c r="W18" s="11"/>
-      <c r="X18" s="40">
-        <v>48</v>
-      </c>
-      <c r="Y18" s="11">
+      <c r="X18" s="124"/>
+      <c r="Y18" s="125"/>
+      <c r="Z18" s="124">
+        <v>50</v>
+      </c>
+      <c r="AA18" s="125">
         <v>15</v>
       </c>
-      <c r="Z18" s="40">
+      <c r="AB18" s="70"/>
+      <c r="AC18" s="76"/>
+      <c r="AD18" s="115">
         <v>47</v>
       </c>
-      <c r="AA18" s="76">
-        <v>16</v>
-      </c>
-      <c r="AB18" s="40"/>
-      <c r="AC18" s="76"/>
-      <c r="AD18" s="63">
-        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18</f>
-        <v>183</v>
-      </c>
-      <c r="AE18" s="12">
-        <f>COUNTIF(D18:AB18,"&gt;30")</f>
-        <v>4</v>
-      </c>
-      <c r="AF18" s="38"/>
-      <c r="AG18" s="11">
-        <v>1</v>
-      </c>
-      <c r="AH18" s="39">
-        <f>SUMIF(G18:AC18, "&lt;30")+AF18+AG18</f>
-        <v>70</v>
-      </c>
-      <c r="AI18" s="67">
-        <f>AH18/AE18</f>
-        <v>17.5</v>
-      </c>
-      <c r="AJ18" s="56"/>
-      <c r="AK18" s="39"/>
-      <c r="AL18" s="39"/>
+      <c r="AE18" s="116">
+        <v>19</v>
+      </c>
+      <c r="AF18" s="63">
+        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18+AD18</f>
+        <v>380</v>
+      </c>
+      <c r="AG18" s="12">
+        <f>COUNTIF(D18:AD18,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AH18" s="41"/>
+      <c r="AI18" s="31"/>
+      <c r="AJ18" s="39">
+        <f>SUMIF(G18:AE18, "&lt;30")+AH18+AI18</f>
+        <v>133</v>
+      </c>
+      <c r="AK18" s="67">
+        <f>AJ18/AG18</f>
+        <v>16.625</v>
+      </c>
+      <c r="AL18" s="59"/>
       <c r="AM18" s="12"/>
-      <c r="AN18" s="57"/>
+      <c r="AN18" s="12"/>
+      <c r="AO18" s="12"/>
+      <c r="AP18" s="57"/>
     </row>
-    <row r="19" spans="1:40">
+    <row r="19" spans="1:42">
       <c r="A19" s="8" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C19" s="10">
-        <f>ROUND((AD19-(36*AE19))/AE19,0)</f>
-        <v>12</v>
+        <f>ROUND((AF19-(36*AG19))/AG19,0)</f>
+        <v>11</v>
       </c>
       <c r="D19" s="49"/>
       <c r="E19" s="50"/>
-      <c r="F19" s="13">
-        <v>46</v>
-      </c>
-      <c r="G19" s="11">
-        <v>18</v>
-      </c>
+      <c r="F19" s="15"/>
+      <c r="G19" s="11"/>
       <c r="H19" s="49"/>
       <c r="I19" s="50"/>
-      <c r="J19" s="13"/>
+      <c r="J19" s="15"/>
       <c r="K19" s="11"/>
-      <c r="L19" s="13">
-        <v>46</v>
-      </c>
-      <c r="M19" s="11">
-        <v>18</v>
-      </c>
-      <c r="N19" s="13">
-        <v>46</v>
+      <c r="L19" s="15"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="40">
+        <v>45</v>
       </c>
       <c r="O19" s="11">
         <v>18</v>
       </c>
-      <c r="P19" s="13">
-        <v>46</v>
+      <c r="P19" s="40">
+        <v>43</v>
       </c>
       <c r="Q19" s="11">
-        <v>18</v>
-      </c>
-      <c r="R19" s="13">
+        <v>20</v>
+      </c>
+      <c r="R19" s="40"/>
+      <c r="S19" s="11"/>
+      <c r="T19" s="40"/>
+      <c r="U19" s="11"/>
+      <c r="V19" s="40"/>
+      <c r="W19" s="11"/>
+      <c r="X19" s="70">
+        <v>48</v>
+      </c>
+      <c r="Y19" s="125">
+        <v>15</v>
+      </c>
+      <c r="Z19" s="70">
         <v>47</v>
       </c>
-      <c r="S19" s="11">
-        <v>14</v>
-      </c>
-      <c r="T19" s="13">
-        <v>52</v>
-      </c>
-      <c r="U19" s="11">
-        <v>13</v>
-      </c>
-      <c r="V19" s="13"/>
-      <c r="W19" s="11"/>
-      <c r="X19" s="13"/>
-      <c r="Y19" s="11"/>
-      <c r="Z19" s="13">
-        <v>50</v>
-      </c>
-      <c r="AA19" s="11">
-        <v>15</v>
+      <c r="AA19" s="76">
+        <v>16</v>
       </c>
       <c r="AB19" s="70"/>
       <c r="AC19" s="76"/>
-      <c r="AD19" s="63">
-        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19</f>
-        <v>333</v>
-      </c>
-      <c r="AE19" s="12">
-        <f>COUNTIF(D19:AB19,"&gt;30")</f>
-        <v>7</v>
-      </c>
-      <c r="AF19" s="41"/>
-      <c r="AG19" s="31"/>
-      <c r="AH19" s="39">
-        <f>SUMIF(G19:AC19, "&lt;30")+AF19+AG19</f>
-        <v>114</v>
-      </c>
-      <c r="AI19" s="67">
-        <f>AH19/AE19</f>
-        <v>16.285714285714285</v>
-      </c>
-      <c r="AJ19" s="59"/>
-      <c r="AK19" s="12"/>
-      <c r="AL19" s="12"/>
-      <c r="AM19" s="12"/>
-      <c r="AN19" s="57"/>
+      <c r="AD19" s="115">
+        <v>51</v>
+      </c>
+      <c r="AE19" s="116">
+        <v>13</v>
+      </c>
+      <c r="AF19" s="63">
+        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19+AD19</f>
+        <v>234</v>
+      </c>
+      <c r="AG19" s="12">
+        <f>COUNTIF(D19:AD19,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AH19" s="38"/>
+      <c r="AI19" s="11">
+        <v>1</v>
+      </c>
+      <c r="AJ19" s="39">
+        <f>SUMIF(G19:AE19, "&lt;30")+AH19+AI19</f>
+        <v>83</v>
+      </c>
+      <c r="AK19" s="67">
+        <f>AJ19/AG19</f>
+        <v>16.600000000000001</v>
+      </c>
+      <c r="AL19" s="56"/>
+      <c r="AM19" s="39"/>
+      <c r="AN19" s="39"/>
+      <c r="AO19" s="12"/>
+      <c r="AP19" s="57"/>
     </row>
-    <row r="20" spans="1:40">
+    <row r="20" spans="1:42">
       <c r="A20" s="8" t="s">
         <v>23</v>
       </c>
@@ -3324,7 +3471,7 @@
         <v>24</v>
       </c>
       <c r="C20" s="10">
-        <f>ROUND((AD20-(36*AE20))/AE20,0)</f>
+        <f>ROUND((AF20-(36*AG20))/AG20,0)</f>
         <v>24</v>
       </c>
       <c r="D20" s="49"/>
@@ -3375,47 +3522,53 @@
       <c r="W20" s="11">
         <v>22</v>
       </c>
-      <c r="X20" s="40"/>
-      <c r="Y20" s="11"/>
-      <c r="Z20" s="40">
+      <c r="X20" s="70"/>
+      <c r="Y20" s="125"/>
+      <c r="Z20" s="70">
         <v>70</v>
       </c>
       <c r="AA20" s="76">
         <v>6</v>
       </c>
-      <c r="AB20" s="40">
+      <c r="AB20" s="70">
         <v>63</v>
       </c>
       <c r="AC20" s="76">
         <v>15</v>
       </c>
-      <c r="AD20" s="63">
-        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20</f>
-        <v>541</v>
-      </c>
-      <c r="AE20" s="12">
-        <f>COUNTIF(D20:AB20,"&gt;30")</f>
-        <v>9</v>
-      </c>
-      <c r="AF20" s="38">
+      <c r="AD20" s="115">
+        <v>58</v>
+      </c>
+      <c r="AE20" s="116">
+        <v>20</v>
+      </c>
+      <c r="AF20" s="63">
+        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20+AD20</f>
+        <v>599</v>
+      </c>
+      <c r="AG20" s="12">
+        <f>COUNTIF(D20:AD20,"&gt;30")</f>
+        <v>10</v>
+      </c>
+      <c r="AH20" s="38">
         <v>2</v>
       </c>
-      <c r="AG20" s="11"/>
-      <c r="AH20" s="39">
-        <f>SUMIF(G20:AC20, "&lt;30")+AF20+AG20</f>
-        <v>144</v>
-      </c>
-      <c r="AI20" s="67">
-        <f>AH20/AE20</f>
-        <v>16</v>
-      </c>
-      <c r="AJ20" s="56"/>
-      <c r="AK20" s="39"/>
-      <c r="AL20" s="39"/>
-      <c r="AM20" s="12"/>
-      <c r="AN20" s="57"/>
+      <c r="AI20" s="11"/>
+      <c r="AJ20" s="39">
+        <f>SUMIF(G20:AE20, "&lt;30")+AH20+AI20</f>
+        <v>164</v>
+      </c>
+      <c r="AK20" s="67">
+        <f>AJ20/AG20</f>
+        <v>16.399999999999999</v>
+      </c>
+      <c r="AL20" s="56"/>
+      <c r="AM20" s="39"/>
+      <c r="AN20" s="39"/>
+      <c r="AO20" s="12"/>
+      <c r="AP20" s="57"/>
     </row>
-    <row r="21" spans="1:40">
+    <row r="21" spans="1:42">
       <c r="A21" s="8" t="s">
         <v>21</v>
       </c>
@@ -3449,37 +3602,39 @@
       <c r="U21" s="11"/>
       <c r="V21" s="13"/>
       <c r="W21" s="11"/>
-      <c r="X21" s="13"/>
-      <c r="Y21" s="11"/>
-      <c r="Z21" s="13"/>
-      <c r="AA21" s="11"/>
+      <c r="X21" s="124"/>
+      <c r="Y21" s="125"/>
+      <c r="Z21" s="124"/>
+      <c r="AA21" s="125"/>
       <c r="AB21" s="70"/>
       <c r="AC21" s="76"/>
-      <c r="AD21" s="63">
-        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21</f>
+      <c r="AD21" s="115"/>
+      <c r="AE21" s="116"/>
+      <c r="AF21" s="63">
+        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21+AD21</f>
         <v>56</v>
       </c>
-      <c r="AE21" s="12">
-        <f>COUNTIF(D21:AB21,"&gt;30")</f>
+      <c r="AG21" s="12">
+        <f>COUNTIF(D21:AD21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AF21" s="38"/>
-      <c r="AG21" s="11"/>
-      <c r="AH21" s="39">
-        <f>SUMIF(G21:AC21, "&lt;30")+AF21+AG21</f>
+      <c r="AH21" s="38"/>
+      <c r="AI21" s="11"/>
+      <c r="AJ21" s="39">
+        <f>SUMIF(G21:AE21, "&lt;30")+AH21+AI21</f>
         <v>16</v>
       </c>
-      <c r="AI21" s="67">
-        <f>AH21/AE21</f>
+      <c r="AK21" s="67">
+        <f>AJ21/AG21</f>
         <v>16</v>
       </c>
-      <c r="AJ21" s="59"/>
-      <c r="AK21" s="39"/>
-      <c r="AL21" s="39"/>
-      <c r="AM21" s="12"/>
-      <c r="AN21" s="57"/>
+      <c r="AL21" s="59"/>
+      <c r="AM21" s="39"/>
+      <c r="AN21" s="39"/>
+      <c r="AO21" s="12"/>
+      <c r="AP21" s="57"/>
     </row>
-    <row r="22" spans="1:40" ht="17" thickBot="1">
+    <row r="22" spans="1:42" ht="17" thickBot="1">
       <c r="A22" s="16" t="s">
         <v>48</v>
       </c>
@@ -3511,39 +3666,41 @@
       <c r="U22" s="19"/>
       <c r="V22" s="74"/>
       <c r="W22" s="19"/>
-      <c r="X22" s="74"/>
-      <c r="Y22" s="19"/>
-      <c r="Z22" s="74"/>
-      <c r="AA22" s="19"/>
-      <c r="AB22" s="74"/>
-      <c r="AC22" s="19"/>
-      <c r="AD22" s="64">
-        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22</f>
+      <c r="X22" s="126"/>
+      <c r="Y22" s="127"/>
+      <c r="Z22" s="126"/>
+      <c r="AA22" s="127"/>
+      <c r="AB22" s="126"/>
+      <c r="AC22" s="127"/>
+      <c r="AD22" s="126"/>
+      <c r="AE22" s="127"/>
+      <c r="AF22" s="64">
+        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22+AD22</f>
         <v>50</v>
       </c>
-      <c r="AE22" s="20">
-        <f>COUNTIF(D22:AB22,"&gt;30")</f>
+      <c r="AG22" s="20">
+        <f>COUNTIF(D22:AD22,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AF22" s="42">
+      <c r="AH22" s="42">
         <v>1</v>
       </c>
-      <c r="AG22" s="19"/>
-      <c r="AH22" s="43">
-        <f>SUMIF(G22:AC22, "&lt;30")+AF22+AG22</f>
+      <c r="AI22" s="19"/>
+      <c r="AJ22" s="43">
+        <f>SUMIF(G22:AC22, "&lt;30")+AH22+AI22</f>
         <v>1</v>
       </c>
-      <c r="AI22" s="68">
-        <f>AH22/AE22</f>
+      <c r="AK22" s="68">
+        <f>AJ22/AG22</f>
         <v>1</v>
       </c>
-      <c r="AJ22" s="60"/>
-      <c r="AK22" s="43"/>
-      <c r="AL22" s="43"/>
-      <c r="AM22" s="20"/>
-      <c r="AN22" s="61"/>
+      <c r="AL22" s="60"/>
+      <c r="AM22" s="43"/>
+      <c r="AN22" s="43"/>
+      <c r="AO22" s="20"/>
+      <c r="AP22" s="61"/>
     </row>
-    <row r="23" spans="1:40" s="21" customFormat="1" ht="17" thickBot="1">
+    <row r="23" spans="1:42" s="21" customFormat="1" ht="17" thickBot="1">
       <c r="A23" s="32"/>
       <c r="B23" s="33"/>
       <c r="C23" s="33"/>
@@ -3606,18 +3763,23 @@
         <v>47.846153846153847</v>
       </c>
       <c r="AC23" s="34"/>
-      <c r="AD23" s="35"/>
+      <c r="AD23" s="34">
+        <f>AVERAGEIF(AD4:AD22,"&gt;0")</f>
+        <v>46.090909090909093</v>
+      </c>
+      <c r="AE23" s="34"/>
+      <c r="AF23" s="35"/>
     </row>
-    <row r="24" spans="1:40">
+    <row r="24" spans="1:42">
       <c r="C24" s="22"/>
-      <c r="AD24" s="23"/>
-      <c r="AE24" s="23"/>
-      <c r="AF24" s="24"/>
-      <c r="AG24" s="24"/>
-      <c r="AH24" s="23"/>
-      <c r="AI24" s="25"/>
+      <c r="AF24" s="23"/>
+      <c r="AG24" s="23"/>
+      <c r="AH24" s="24"/>
+      <c r="AI24" s="24"/>
+      <c r="AJ24" s="23"/>
+      <c r="AK24" s="25"/>
     </row>
-    <row r="25" spans="1:40">
+    <row r="25" spans="1:42">
       <c r="C25" s="44" t="s">
         <v>41</v>
       </c>
@@ -3636,8 +3798,9 @@
       <c r="X25" s="26"/>
       <c r="Z25" s="26"/>
       <c r="AB25" s="26"/>
+      <c r="AD25" s="26"/>
     </row>
-    <row r="26" spans="1:40">
+    <row r="26" spans="1:42">
       <c r="C26" s="45" t="s">
         <v>42</v>
       </c>
@@ -3656,9 +3819,10 @@
       <c r="X26" s="27"/>
       <c r="Z26" s="27"/>
       <c r="AB26" s="27"/>
-      <c r="AD26" s="28"/>
+      <c r="AD26" s="27"/>
+      <c r="AF26" s="28"/>
     </row>
-    <row r="27" spans="1:40">
+    <row r="27" spans="1:42">
       <c r="C27" s="46" t="s">
         <v>46</v>
       </c>
@@ -3690,32 +3854,39 @@
       <c r="AA27" s="30"/>
       <c r="AB27" s="29"/>
       <c r="AC27" s="30"/>
+      <c r="AD27" s="29"/>
+      <c r="AE27" s="30"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AN22">
-    <sortCondition descending="1" ref="AI4:AI22"/>
-    <sortCondition descending="1" ref="AD4:AD22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:AP22">
+    <sortCondition descending="1" ref="AK5:AK22"/>
+    <sortCondition descending="1" ref="AF5:AF22"/>
   </sortState>
-  <mergeCells count="41">
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="AB1:AC1"/>
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="AJ1:AN1"/>
-    <mergeCell ref="AJ2:AJ3"/>
-    <mergeCell ref="AK2:AK3"/>
-    <mergeCell ref="AL2:AL3"/>
-    <mergeCell ref="AM2:AM3"/>
-    <mergeCell ref="AN2:AN3"/>
+  <mergeCells count="43">
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="AD1:AE1"/>
+    <mergeCell ref="AD2:AE2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
     <mergeCell ref="AH2:AH3"/>
     <mergeCell ref="AI2:AI3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="AF2:AF3"/>
     <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="AE2:AE3"/>
     <mergeCell ref="N1:O1"/>
-    <mergeCell ref="AD1:AD3"/>
-    <mergeCell ref="AE1:AI1"/>
+    <mergeCell ref="AF1:AF3"/>
+    <mergeCell ref="AG1:AK1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="P2:Q2"/>
@@ -3723,21 +3894,18 @@
     <mergeCell ref="R2:S2"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="T2:U2"/>
     <mergeCell ref="V1:W1"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="AB1:AC1"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="AL1:AP1"/>
+    <mergeCell ref="AL2:AL3"/>
+    <mergeCell ref="AM2:AM3"/>
+    <mergeCell ref="AN2:AN3"/>
+    <mergeCell ref="AO2:AO3"/>
+    <mergeCell ref="AP2:AP3"/>
+    <mergeCell ref="AJ2:AJ3"/>
+    <mergeCell ref="AK2:AK3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
081125 - posted tee times for 8/11
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94A3502-0EBB-1C4C-B4A9-72D954014F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{F94A3502-0EBB-1C4C-B4A9-72D954014F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A7BFC1A-C7C6-4DB9-B4B8-215DAD07F51B}"/>
   <bookViews>
-    <workbookView xWindow="10340" yWindow="2280" windowWidth="26960" windowHeight="15740" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="43125" yWindow="3150" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -397,7 +397,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -949,11 +949,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -963,9 +989,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1166,11 +1189,38 @@
     <xf numFmtId="1" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="43" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1196,11 +1246,50 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1213,66 +1302,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1289,6 +1318,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1609,202 +1642,202 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
   <dimension ref="A1:AN27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" customWidth="1"/>
-    <col min="2" max="2" width="8.1640625" customWidth="1"/>
-    <col min="3" max="3" width="10.1640625" customWidth="1"/>
-    <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="8.625" customWidth="1"/>
+    <col min="2" max="2" width="8.125" customWidth="1"/>
+    <col min="3" max="3" width="10.125" customWidth="1"/>
+    <col min="4" max="10" width="6.875" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="23" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="23" width="6.375" hidden="1" customWidth="1"/>
     <col min="24" max="24" width="6" customWidth="1"/>
-    <col min="25" max="25" width="6.33203125" customWidth="1"/>
+    <col min="25" max="25" width="6.375" customWidth="1"/>
     <col min="26" max="26" width="6" customWidth="1"/>
-    <col min="27" max="27" width="6.33203125" customWidth="1"/>
+    <col min="27" max="27" width="6.375" customWidth="1"/>
     <col min="28" max="28" width="6" customWidth="1"/>
-    <col min="29" max="29" width="6.33203125" customWidth="1"/>
-    <col min="30" max="30" width="8.83203125" customWidth="1"/>
-    <col min="31" max="31" width="6.1640625" customWidth="1"/>
-    <col min="32" max="32" width="5.83203125" customWidth="1"/>
-    <col min="33" max="33" width="5.6640625" customWidth="1"/>
+    <col min="29" max="29" width="6.375" customWidth="1"/>
+    <col min="30" max="30" width="8.875" customWidth="1"/>
+    <col min="31" max="31" width="6.125" customWidth="1"/>
+    <col min="32" max="32" width="5.875" customWidth="1"/>
+    <col min="33" max="33" width="5.625" customWidth="1"/>
     <col min="34" max="34" width="5.5" customWidth="1"/>
     <col min="35" max="35" width="8" customWidth="1"/>
-    <col min="36" max="36" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="7.375" hidden="1" customWidth="1"/>
     <col min="37" max="38" width="6" hidden="1" customWidth="1"/>
-    <col min="39" max="39" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="40" max="40" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="39" max="39" width="7.375" hidden="1" customWidth="1"/>
+    <col min="40" max="40" width="9.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="54" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="80" t="s">
+    <row r="1" spans="1:40" s="53" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="86" t="s">
+      <c r="B1" s="89"/>
+      <c r="C1" s="94" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="88" t="s">
+      <c r="D1" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="89"/>
-      <c r="F1" s="88" t="s">
+      <c r="E1" s="87"/>
+      <c r="F1" s="86" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="89"/>
-      <c r="H1" s="88" t="s">
+      <c r="G1" s="87"/>
+      <c r="H1" s="86" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="89"/>
-      <c r="J1" s="88" t="s">
+      <c r="I1" s="87"/>
+      <c r="J1" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="89"/>
-      <c r="L1" s="88" t="s">
+      <c r="K1" s="87"/>
+      <c r="L1" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="89"/>
-      <c r="N1" s="88" t="s">
+      <c r="M1" s="87"/>
+      <c r="N1" s="86" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="89"/>
-      <c r="P1" s="88" t="s">
+      <c r="O1" s="87"/>
+      <c r="P1" s="86" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="88" t="s">
+      <c r="Q1" s="87"/>
+      <c r="R1" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="89"/>
-      <c r="T1" s="88" t="s">
+      <c r="S1" s="87"/>
+      <c r="T1" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="89"/>
-      <c r="V1" s="88" t="s">
+      <c r="U1" s="87"/>
+      <c r="V1" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="89"/>
-      <c r="X1" s="88" t="s">
+      <c r="W1" s="87"/>
+      <c r="X1" s="86" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="89"/>
-      <c r="Z1" s="88" t="s">
+      <c r="Y1" s="87"/>
+      <c r="Z1" s="86" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="89"/>
-      <c r="AB1" s="88" t="s">
+      <c r="AA1" s="87"/>
+      <c r="AB1" s="86" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="89"/>
-      <c r="AD1" s="98" t="s">
+      <c r="AC1" s="87"/>
+      <c r="AD1" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="AE1" s="100" t="s">
+      <c r="AE1" s="103" t="s">
         <v>65</v>
       </c>
-      <c r="AF1" s="101"/>
-      <c r="AG1" s="101"/>
-      <c r="AH1" s="101"/>
-      <c r="AI1" s="102"/>
-      <c r="AJ1" s="103" t="s">
+      <c r="AF1" s="104"/>
+      <c r="AG1" s="104"/>
+      <c r="AH1" s="104"/>
+      <c r="AI1" s="105"/>
+      <c r="AJ1" s="106" t="s">
         <v>57</v>
       </c>
-      <c r="AK1" s="104"/>
-      <c r="AL1" s="104"/>
-      <c r="AM1" s="104"/>
-      <c r="AN1" s="105"/>
+      <c r="AK1" s="107"/>
+      <c r="AL1" s="107"/>
+      <c r="AM1" s="107"/>
+      <c r="AN1" s="108"/>
     </row>
-    <row r="2" spans="1:40" s="54" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="82"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="78">
+    <row r="2" spans="1:40" s="53" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="90"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="84">
         <v>45782</v>
       </c>
-      <c r="E2" s="79"/>
-      <c r="F2" s="78">
+      <c r="E2" s="85"/>
+      <c r="F2" s="84">
         <v>45789</v>
       </c>
-      <c r="G2" s="79"/>
-      <c r="H2" s="78">
+      <c r="G2" s="85"/>
+      <c r="H2" s="84">
         <v>45796</v>
       </c>
-      <c r="I2" s="79"/>
-      <c r="J2" s="78">
+      <c r="I2" s="85"/>
+      <c r="J2" s="84">
         <v>45803</v>
       </c>
-      <c r="K2" s="79"/>
-      <c r="L2" s="78">
+      <c r="K2" s="85"/>
+      <c r="L2" s="84">
         <v>45810</v>
       </c>
-      <c r="M2" s="79"/>
-      <c r="N2" s="78">
+      <c r="M2" s="85"/>
+      <c r="N2" s="84">
         <v>45817</v>
       </c>
-      <c r="O2" s="79"/>
-      <c r="P2" s="78">
+      <c r="O2" s="85"/>
+      <c r="P2" s="84">
         <v>45824</v>
       </c>
-      <c r="Q2" s="79"/>
-      <c r="R2" s="78">
+      <c r="Q2" s="85"/>
+      <c r="R2" s="84">
         <v>45831</v>
       </c>
-      <c r="S2" s="79"/>
-      <c r="T2" s="78">
+      <c r="S2" s="85"/>
+      <c r="T2" s="84">
         <v>45838</v>
       </c>
-      <c r="U2" s="79"/>
-      <c r="V2" s="78">
+      <c r="U2" s="85"/>
+      <c r="V2" s="84">
         <v>45845</v>
       </c>
-      <c r="W2" s="79"/>
-      <c r="X2" s="78">
+      <c r="W2" s="85"/>
+      <c r="X2" s="84">
         <v>45852</v>
       </c>
-      <c r="Y2" s="79"/>
-      <c r="Z2" s="78">
+      <c r="Y2" s="85"/>
+      <c r="Z2" s="84">
         <v>45859</v>
       </c>
-      <c r="AA2" s="79"/>
-      <c r="AB2" s="78">
+      <c r="AA2" s="85"/>
+      <c r="AB2" s="84">
         <v>45866</v>
       </c>
-      <c r="AC2" s="79"/>
-      <c r="AD2" s="99"/>
-      <c r="AE2" s="98" t="s">
+      <c r="AC2" s="85"/>
+      <c r="AD2" s="102"/>
+      <c r="AE2" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="AF2" s="94" t="s">
+      <c r="AF2" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="AG2" s="96" t="s">
+      <c r="AG2" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="AH2" s="90" t="s">
+      <c r="AH2" s="111" t="s">
         <v>6</v>
       </c>
-      <c r="AI2" s="92" t="s">
+      <c r="AI2" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="AJ2" s="106" t="s">
+      <c r="AJ2" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="AK2" s="106" t="s">
+      <c r="AK2" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="AL2" s="106" t="s">
+      <c r="AL2" s="109" t="s">
         <v>5</v>
       </c>
-      <c r="AM2" s="106" t="s">
+      <c r="AM2" s="109" t="s">
         <v>6</v>
       </c>
-      <c r="AN2" s="106" t="s">
+      <c r="AN2" s="109" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:40" s="54" customFormat="1" ht="29" customHeight="1" thickBot="1">
-      <c r="A3" s="84"/>
-      <c r="B3" s="85"/>
-      <c r="C3" s="87"/>
+    <row r="3" spans="1:40" s="53" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
+      <c r="A3" s="92"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="96"/>
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1883,1813 +1916,1816 @@
       <c r="AC3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="AD3" s="99"/>
-      <c r="AE3" s="99"/>
-      <c r="AF3" s="95"/>
-      <c r="AG3" s="97"/>
-      <c r="AH3" s="91"/>
-      <c r="AI3" s="93"/>
-      <c r="AJ3" s="107"/>
-      <c r="AK3" s="107"/>
-      <c r="AL3" s="107"/>
-      <c r="AM3" s="107"/>
-      <c r="AN3" s="107"/>
+      <c r="AD3" s="102"/>
+      <c r="AE3" s="102"/>
+      <c r="AF3" s="98"/>
+      <c r="AG3" s="100"/>
+      <c r="AH3" s="112"/>
+      <c r="AI3" s="114"/>
+      <c r="AJ3" s="110"/>
+      <c r="AK3" s="110"/>
+      <c r="AL3" s="110"/>
+      <c r="AM3" s="110"/>
+      <c r="AN3" s="110"/>
     </row>
-    <row r="4" spans="1:40" ht="16" customHeight="1">
+    <row r="4" spans="1:40" ht="15.95" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="5">
-        <v>2</v>
-      </c>
-      <c r="D4" s="47"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="110"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="110"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="110"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="111">
+      <c r="C4" s="83">
+        <f t="shared" ref="C4:C14" si="0">ROUND((AD4-(36*AE4))/AE4,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="79"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="80">
         <v>39</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4" s="5">
         <v>17</v>
       </c>
-      <c r="R4" s="111">
+      <c r="R4" s="80">
         <v>38</v>
       </c>
-      <c r="S4" s="6">
+      <c r="S4" s="5">
         <v>18</v>
       </c>
-      <c r="T4" s="111"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="112">
+      <c r="T4" s="80"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="81">
         <v>37</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4" s="5">
         <v>19</v>
       </c>
-      <c r="X4" s="112">
+      <c r="X4" s="81">
         <v>36</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="5">
         <v>20</v>
       </c>
-      <c r="Z4" s="112">
+      <c r="Z4" s="81">
         <v>38</v>
       </c>
-      <c r="AA4" s="75">
+      <c r="AA4" s="74">
         <v>18</v>
       </c>
-      <c r="AB4" s="111">
+      <c r="AB4" s="80">
         <v>35</v>
       </c>
-      <c r="AC4" s="75">
+      <c r="AC4" s="74">
         <v>21</v>
       </c>
-      <c r="AD4" s="62">
-        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4</f>
+      <c r="AD4" s="61">
+        <f t="shared" ref="AD4:AD22" si="1">F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4</f>
         <v>223</v>
       </c>
-      <c r="AE4" s="7">
-        <f>COUNTIF(D4:AB4,"&gt;30")</f>
+      <c r="AE4" s="6">
+        <f t="shared" ref="AE4:AE22" si="2">COUNTIF(D4:AB4,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AF4" s="36">
+      <c r="AF4" s="35">
         <v>3</v>
       </c>
-      <c r="AG4" s="6">
+      <c r="AG4" s="5">
         <v>8</v>
       </c>
-      <c r="AH4" s="37">
-        <f>SUMIF(G4:AC4, "&lt;30")+AF4+AG4</f>
+      <c r="AH4" s="36">
+        <f t="shared" ref="AH4:AH22" si="3">SUMIF(G4:AC4, "&lt;30")+AF4+AG4</f>
         <v>124</v>
       </c>
-      <c r="AI4" s="66">
-        <f>AH4/AE4</f>
+      <c r="AI4" s="65">
+        <f t="shared" ref="AI4:AI22" si="4">AH4/AE4</f>
         <v>20.666666666666668</v>
       </c>
-      <c r="AJ4" s="108"/>
-      <c r="AK4" s="37"/>
-      <c r="AL4" s="37"/>
-      <c r="AM4" s="7"/>
-      <c r="AN4" s="55"/>
+      <c r="AJ4" s="77"/>
+      <c r="AK4" s="36"/>
+      <c r="AL4" s="36"/>
+      <c r="AM4" s="6"/>
+      <c r="AN4" s="54"/>
     </row>
     <row r="5" spans="1:40">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="10">
-        <f>ROUND((AD5-(36*AE5))/AE5,0)</f>
+      <c r="C5" s="9">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="D5" s="49"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="13">
+      <c r="D5" s="48"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="12">
         <v>53</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <v>23</v>
       </c>
-      <c r="H5" s="49"/>
-      <c r="I5" s="50"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="13">
+      <c r="H5" s="48"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="12">
         <v>57</v>
       </c>
-      <c r="O5" s="11">
+      <c r="O5" s="10">
         <v>19</v>
       </c>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="13">
+      <c r="P5" s="12"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="12">
         <v>50</v>
       </c>
-      <c r="S5" s="11">
+      <c r="S5" s="10">
         <v>26</v>
       </c>
-      <c r="T5" s="13">
+      <c r="T5" s="12">
         <v>56</v>
       </c>
-      <c r="U5" s="11">
+      <c r="U5" s="10">
         <v>15</v>
       </c>
-      <c r="V5" s="13"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="13"/>
-      <c r="Y5" s="11"/>
-      <c r="Z5" s="70">
+      <c r="V5" s="12"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="12"/>
+      <c r="Y5" s="10"/>
+      <c r="Z5" s="69">
         <v>54</v>
       </c>
-      <c r="AA5" s="76">
+      <c r="AA5" s="75">
         <v>18</v>
       </c>
-      <c r="AB5" s="70">
+      <c r="AB5" s="69">
         <v>50</v>
       </c>
-      <c r="AC5" s="76">
+      <c r="AC5" s="75">
         <v>22</v>
       </c>
-      <c r="AD5" s="63">
-        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5</f>
+      <c r="AD5" s="62">
+        <f t="shared" si="1"/>
         <v>320</v>
       </c>
-      <c r="AE5" s="12">
-        <f>COUNTIF(D5:AB5,"&gt;30")</f>
+      <c r="AE5" s="11">
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="AF5" s="38"/>
-      <c r="AG5" s="11"/>
-      <c r="AH5" s="39">
-        <f>SUMIF(G5:AC5, "&lt;30")+AF5+AG5</f>
+      <c r="AF5" s="37"/>
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="38">
+        <f t="shared" si="3"/>
         <v>123</v>
       </c>
-      <c r="AI5" s="67">
-        <f>AH5/AE5</f>
+      <c r="AI5" s="66">
+        <f t="shared" si="4"/>
         <v>20.5</v>
       </c>
-      <c r="AJ5" s="56"/>
-      <c r="AK5" s="39"/>
-      <c r="AL5" s="39"/>
-      <c r="AM5" s="12"/>
-      <c r="AN5" s="57" t="s">
+      <c r="AJ5" s="55"/>
+      <c r="AK5" s="38"/>
+      <c r="AL5" s="38"/>
+      <c r="AM5" s="11"/>
+      <c r="AN5" s="56" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:40">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="10">
-        <f>ROUND((AD6-(36*AE6))/AE6,0)</f>
+      <c r="C6" s="9">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D6" s="49"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="50"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="13">
+      <c r="D6" s="48"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="12">
         <v>43</v>
       </c>
-      <c r="Q6" s="11">
+      <c r="Q6" s="10">
         <v>26</v>
       </c>
-      <c r="R6" s="69">
+      <c r="R6" s="68">
         <v>45</v>
       </c>
-      <c r="S6" s="11">
+      <c r="S6" s="10">
         <v>24</v>
       </c>
-      <c r="T6" s="70"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="70">
+      <c r="T6" s="69"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="69">
         <v>50</v>
       </c>
-      <c r="W6" s="11">
+      <c r="W6" s="10">
         <v>19</v>
       </c>
-      <c r="X6" s="70">
+      <c r="X6" s="69">
         <v>44</v>
       </c>
-      <c r="Y6" s="11">
+      <c r="Y6" s="10">
         <v>20</v>
       </c>
-      <c r="Z6" s="70"/>
-      <c r="AA6" s="76"/>
-      <c r="AB6" s="70">
+      <c r="Z6" s="69"/>
+      <c r="AA6" s="75"/>
+      <c r="AB6" s="69">
         <v>54</v>
       </c>
-      <c r="AC6" s="76">
+      <c r="AC6" s="75">
         <v>11</v>
       </c>
-      <c r="AD6" s="63">
-        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6</f>
+      <c r="AD6" s="62">
+        <f t="shared" si="1"/>
         <v>236</v>
       </c>
-      <c r="AE6" s="12">
-        <f>COUNTIF(D6:AB6,"&gt;30")</f>
+      <c r="AE6" s="11">
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="AF6" s="38">
+      <c r="AF6" s="37">
         <v>1</v>
       </c>
-      <c r="AG6" s="11">
+      <c r="AG6" s="10">
         <v>1</v>
       </c>
-      <c r="AH6" s="39">
-        <f>SUMIF(G6:AC6, "&lt;30")+AF6+AG6</f>
+      <c r="AH6" s="38">
+        <f t="shared" si="3"/>
         <v>102</v>
       </c>
-      <c r="AI6" s="67">
-        <f>AH6/AE6</f>
+      <c r="AI6" s="66">
+        <f t="shared" si="4"/>
         <v>20.399999999999999</v>
       </c>
-      <c r="AJ6" s="59"/>
-      <c r="AK6" s="39"/>
-      <c r="AL6" s="39"/>
-      <c r="AM6" s="12"/>
-      <c r="AN6" s="57"/>
+      <c r="AJ6" s="58"/>
+      <c r="AK6" s="38"/>
+      <c r="AL6" s="38"/>
+      <c r="AM6" s="11"/>
+      <c r="AN6" s="56"/>
     </row>
     <row r="7" spans="1:40">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="10">
-        <f>ROUND((AD7-(36*AE7))/AE7,0)</f>
+      <c r="C7" s="9">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D7" s="49"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="72"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="50"/>
-      <c r="J7" s="72">
+      <c r="D7" s="48"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="71">
         <v>52</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="10">
         <v>17</v>
       </c>
-      <c r="L7" s="72"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="72">
+      <c r="L7" s="71"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="71">
         <v>46</v>
       </c>
-      <c r="O7" s="11">
+      <c r="O7" s="10">
         <v>23</v>
       </c>
-      <c r="P7" s="72">
+      <c r="P7" s="71">
         <v>46</v>
       </c>
-      <c r="Q7" s="11">
+      <c r="Q7" s="10">
         <v>23</v>
       </c>
-      <c r="R7" s="72">
+      <c r="R7" s="71">
         <v>54</v>
       </c>
-      <c r="S7" s="11">
+      <c r="S7" s="10">
         <v>16</v>
       </c>
-      <c r="T7" s="72">
+      <c r="T7" s="71">
         <v>45</v>
       </c>
-      <c r="U7" s="11">
+      <c r="U7" s="10">
         <v>23</v>
       </c>
-      <c r="V7" s="72">
+      <c r="V7" s="71">
         <v>48</v>
       </c>
-      <c r="W7" s="11">
+      <c r="W7" s="10">
         <v>19</v>
       </c>
-      <c r="X7" s="72">
+      <c r="X7" s="71">
         <v>49</v>
       </c>
-      <c r="Y7" s="11">
+      <c r="Y7" s="10">
         <v>18</v>
       </c>
-      <c r="Z7" s="77"/>
-      <c r="AA7" s="76"/>
-      <c r="AB7" s="77">
+      <c r="Z7" s="76"/>
+      <c r="AA7" s="75"/>
+      <c r="AB7" s="76">
         <v>46</v>
       </c>
-      <c r="AC7" s="76">
+      <c r="AC7" s="75">
         <v>21</v>
       </c>
-      <c r="AD7" s="63">
-        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7</f>
+      <c r="AD7" s="62">
+        <f t="shared" si="1"/>
         <v>386</v>
       </c>
-      <c r="AE7" s="12">
-        <f>COUNTIF(D7:AB7,"&gt;30")</f>
+      <c r="AE7" s="11">
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="AF7" s="38"/>
-      <c r="AG7" s="11">
+      <c r="AF7" s="37"/>
+      <c r="AG7" s="10">
         <v>1</v>
       </c>
-      <c r="AH7" s="39">
-        <f>SUMIF(G7:AC7, "&lt;30")+AF7+AG7</f>
+      <c r="AH7" s="38">
+        <f t="shared" si="3"/>
         <v>161</v>
       </c>
-      <c r="AI7" s="67">
-        <f>AH7/AE7</f>
+      <c r="AI7" s="66">
+        <f t="shared" si="4"/>
         <v>20.125</v>
       </c>
-      <c r="AJ7" s="56"/>
-      <c r="AK7" s="39"/>
-      <c r="AL7" s="39"/>
-      <c r="AM7" s="12"/>
-      <c r="AN7" s="57"/>
+      <c r="AJ7" s="55"/>
+      <c r="AK7" s="38"/>
+      <c r="AL7" s="38"/>
+      <c r="AM7" s="11"/>
+      <c r="AN7" s="56"/>
     </row>
     <row r="8" spans="1:40">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="10">
-        <f>ROUND((AD8-(36*AE8))/AE8,0)</f>
+      <c r="C8" s="9">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D8" s="49"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="13">
+      <c r="D8" s="48"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="12">
         <v>42</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <v>27</v>
       </c>
-      <c r="H8" s="49"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="13">
+      <c r="H8" s="48"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="12">
         <v>54</v>
       </c>
-      <c r="M8" s="11">
+      <c r="M8" s="10">
         <v>15</v>
       </c>
-      <c r="N8" s="13"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="13">
+      <c r="N8" s="12"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="12">
         <v>54</v>
       </c>
-      <c r="Q8" s="11">
+      <c r="Q8" s="10">
         <v>16</v>
       </c>
-      <c r="R8" s="13">
+      <c r="R8" s="12">
         <v>53</v>
       </c>
-      <c r="S8" s="11">
+      <c r="S8" s="10">
         <v>16</v>
       </c>
-      <c r="T8" s="13"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="69">
+      <c r="T8" s="12"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="68">
         <v>46</v>
       </c>
-      <c r="W8" s="11">
+      <c r="W8" s="10">
         <v>23</v>
       </c>
-      <c r="X8" s="70">
+      <c r="X8" s="69">
         <v>49</v>
       </c>
-      <c r="Y8" s="11">
+      <c r="Y8" s="10">
         <v>19</v>
       </c>
-      <c r="Z8" s="70">
+      <c r="Z8" s="69">
         <v>50</v>
       </c>
-      <c r="AA8" s="76">
+      <c r="AA8" s="75">
         <v>18</v>
       </c>
-      <c r="AB8" s="70"/>
-      <c r="AC8" s="76"/>
-      <c r="AD8" s="63">
-        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8</f>
+      <c r="AB8" s="69"/>
+      <c r="AC8" s="75"/>
+      <c r="AD8" s="62">
+        <f t="shared" si="1"/>
         <v>348</v>
       </c>
-      <c r="AE8" s="12">
-        <f>COUNTIF(D8:AB8,"&gt;30")</f>
+      <c r="AE8" s="11">
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AF8" s="38">
+      <c r="AF8" s="37">
         <v>1</v>
       </c>
-      <c r="AG8" s="11">
+      <c r="AG8" s="10">
         <v>1</v>
       </c>
-      <c r="AH8" s="39">
-        <f>SUMIF(G8:AC8, "&lt;30")+AF8+AG8</f>
+      <c r="AH8" s="38">
+        <f t="shared" si="3"/>
         <v>136</v>
       </c>
-      <c r="AI8" s="67">
-        <f>AH8/AE8</f>
+      <c r="AI8" s="66">
+        <f t="shared" si="4"/>
         <v>19.428571428571427</v>
       </c>
-      <c r="AJ8" s="58"/>
-      <c r="AK8" s="39"/>
-      <c r="AL8" s="39"/>
-      <c r="AM8" s="12"/>
-      <c r="AN8" s="57"/>
+      <c r="AJ8" s="57"/>
+      <c r="AK8" s="38"/>
+      <c r="AL8" s="38"/>
+      <c r="AM8" s="11"/>
+      <c r="AN8" s="56"/>
     </row>
     <row r="9" spans="1:40">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="10">
-        <f>ROUND((AD9-(36*AE9))/AE9,0)</f>
+      <c r="C9" s="9">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D9" s="49"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="65">
+      <c r="D9" s="48"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="64">
         <v>45</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="10">
         <v>17</v>
       </c>
-      <c r="H9" s="49"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="65"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="65">
+      <c r="H9" s="48"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="64">
         <v>43</v>
       </c>
-      <c r="M9" s="11">
+      <c r="M9" s="10">
         <v>19</v>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="13">
         <v>41</v>
       </c>
-      <c r="O9" s="11">
+      <c r="O9" s="10">
         <v>21</v>
       </c>
-      <c r="P9" s="40">
+      <c r="P9" s="39">
         <v>47</v>
       </c>
-      <c r="Q9" s="11">
+      <c r="Q9" s="10">
         <v>15</v>
       </c>
-      <c r="R9" s="40">
+      <c r="R9" s="39">
         <v>42</v>
       </c>
-      <c r="S9" s="11">
+      <c r="S9" s="10">
         <v>20</v>
       </c>
-      <c r="T9" s="40">
+      <c r="T9" s="39">
         <v>43</v>
       </c>
-      <c r="U9" s="11">
+      <c r="U9" s="10">
         <v>19</v>
       </c>
-      <c r="V9" s="40">
+      <c r="V9" s="39">
         <v>44</v>
       </c>
-      <c r="W9" s="11">
+      <c r="W9" s="10">
         <v>18</v>
       </c>
-      <c r="X9" s="40">
+      <c r="X9" s="39">
         <v>48</v>
       </c>
-      <c r="Y9" s="11">
+      <c r="Y9" s="10">
         <v>16</v>
       </c>
-      <c r="Z9" s="40">
+      <c r="Z9" s="39">
         <v>40</v>
       </c>
-      <c r="AA9" s="76">
+      <c r="AA9" s="75">
         <v>22</v>
       </c>
-      <c r="AB9" s="40">
+      <c r="AB9" s="39">
         <v>40</v>
       </c>
-      <c r="AC9" s="76">
+      <c r="AC9" s="75">
         <v>22</v>
       </c>
-      <c r="AD9" s="63">
-        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9</f>
+      <c r="AD9" s="62">
+        <f t="shared" si="1"/>
         <v>433</v>
       </c>
-      <c r="AE9" s="12">
-        <f>COUNTIF(D9:AB9,"&gt;30")</f>
+      <c r="AE9" s="11">
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AF9" s="38">
+      <c r="AF9" s="37">
         <v>1</v>
       </c>
-      <c r="AG9" s="11">
+      <c r="AG9" s="10">
         <v>4</v>
       </c>
-      <c r="AH9" s="39">
-        <f>SUMIF(G9:AC9, "&lt;30")+AF9+AG9</f>
+      <c r="AH9" s="38">
+        <f t="shared" si="3"/>
         <v>194</v>
       </c>
-      <c r="AI9" s="67">
-        <f>AH9/AE9</f>
+      <c r="AI9" s="66">
+        <f t="shared" si="4"/>
         <v>19.399999999999999</v>
       </c>
-      <c r="AJ9" s="56"/>
-      <c r="AK9" s="39"/>
-      <c r="AL9" s="39"/>
-      <c r="AM9" s="12"/>
-      <c r="AN9" s="57"/>
+      <c r="AJ9" s="55"/>
+      <c r="AK9" s="38"/>
+      <c r="AL9" s="38"/>
+      <c r="AM9" s="11"/>
+      <c r="AN9" s="56"/>
     </row>
     <row r="10" spans="1:40">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="10">
-        <f>ROUND((AD10-(36*AE10))/AE10,0)</f>
+      <c r="C10" s="9">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D10" s="49"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="71">
+      <c r="D10" s="48"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="70">
         <v>42</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="10">
         <v>25</v>
       </c>
-      <c r="H10" s="49"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="71"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="40">
+      <c r="H10" s="48"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="39">
         <v>51</v>
       </c>
-      <c r="M10" s="11">
+      <c r="M10" s="10">
         <v>16</v>
       </c>
-      <c r="N10" s="40"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="14">
+      <c r="N10" s="39"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="13">
         <v>49</v>
       </c>
-      <c r="Q10" s="11">
+      <c r="Q10" s="10">
         <v>18</v>
       </c>
-      <c r="R10" s="40">
+      <c r="R10" s="39">
         <v>46</v>
       </c>
-      <c r="S10" s="11">
+      <c r="S10" s="10">
         <v>21</v>
       </c>
-      <c r="T10" s="40">
+      <c r="T10" s="39">
         <v>45</v>
       </c>
-      <c r="U10" s="11">
+      <c r="U10" s="10">
         <v>20</v>
       </c>
-      <c r="V10" s="40">
+      <c r="V10" s="39">
         <v>46</v>
       </c>
-      <c r="W10" s="11">
+      <c r="W10" s="10">
         <v>19</v>
       </c>
-      <c r="X10" s="40">
+      <c r="X10" s="39">
         <v>53</v>
       </c>
-      <c r="Y10" s="11">
+      <c r="Y10" s="10">
         <v>13</v>
       </c>
-      <c r="Z10" s="40">
+      <c r="Z10" s="39">
         <v>52</v>
       </c>
-      <c r="AA10" s="76">
+      <c r="AA10" s="75">
         <v>13</v>
       </c>
-      <c r="AB10" s="40">
+      <c r="AB10" s="39">
         <v>44</v>
       </c>
-      <c r="AC10" s="76">
+      <c r="AC10" s="75">
         <v>22</v>
       </c>
-      <c r="AD10" s="63">
-        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10</f>
+      <c r="AD10" s="62">
+        <f t="shared" si="1"/>
         <v>428</v>
       </c>
-      <c r="AE10" s="12">
-        <f>COUNTIF(D10:AB10,"&gt;30")</f>
+      <c r="AE10" s="11">
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="AF10" s="38">
+      <c r="AF10" s="37">
         <v>2</v>
       </c>
-      <c r="AG10" s="11">
+      <c r="AG10" s="10">
         <v>1</v>
       </c>
-      <c r="AH10" s="39">
-        <f>SUMIF(G10:AC10, "&lt;30")+AF10+AG10</f>
+      <c r="AH10" s="38">
+        <f t="shared" si="3"/>
         <v>170</v>
       </c>
-      <c r="AI10" s="67">
-        <f>AH10/AE10</f>
+      <c r="AI10" s="66">
+        <f t="shared" si="4"/>
         <v>18.888888888888889</v>
       </c>
-      <c r="AJ10" s="113"/>
-      <c r="AK10" s="39"/>
-      <c r="AL10" s="39"/>
-      <c r="AM10" s="12"/>
-      <c r="AN10" s="57"/>
+      <c r="AJ10" s="82"/>
+      <c r="AK10" s="38"/>
+      <c r="AL10" s="38"/>
+      <c r="AM10" s="11"/>
+      <c r="AN10" s="56"/>
     </row>
     <row r="11" spans="1:40">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="10">
-        <f>ROUND((AD11-(36*AE11))/AE11,0)</f>
+      <c r="C11" s="9">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D11" s="49"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="49"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="15"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="40">
+      <c r="D11" s="48"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="39">
         <v>47</v>
       </c>
-      <c r="Q11" s="11">
+      <c r="Q11" s="10">
         <v>20</v>
       </c>
-      <c r="R11" s="40">
+      <c r="R11" s="39">
         <v>50</v>
       </c>
-      <c r="S11" s="11">
+      <c r="S11" s="10">
         <v>17</v>
       </c>
-      <c r="T11" s="40">
+      <c r="T11" s="39">
         <v>46</v>
       </c>
-      <c r="U11" s="11">
+      <c r="U11" s="10">
         <v>21</v>
       </c>
-      <c r="V11" s="40">
+      <c r="V11" s="39">
         <v>47</v>
       </c>
-      <c r="W11" s="11">
+      <c r="W11" s="10">
         <v>19</v>
       </c>
-      <c r="X11" s="40">
+      <c r="X11" s="39">
         <v>44</v>
       </c>
-      <c r="Y11" s="11">
+      <c r="Y11" s="10">
         <v>22</v>
       </c>
-      <c r="Z11" s="40">
+      <c r="Z11" s="39">
         <v>52</v>
       </c>
-      <c r="AA11" s="76">
+      <c r="AA11" s="75">
         <v>14</v>
       </c>
-      <c r="AB11" s="40">
+      <c r="AB11" s="39">
         <v>47</v>
       </c>
-      <c r="AC11" s="76">
+      <c r="AC11" s="75">
         <v>19</v>
       </c>
-      <c r="AD11" s="63">
-        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11</f>
+      <c r="AD11" s="62">
+        <f t="shared" si="1"/>
         <v>333</v>
       </c>
-      <c r="AE11" s="12">
-        <f>COUNTIF(D11:AB11,"&gt;30")</f>
+      <c r="AE11" s="11">
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AF11" s="38"/>
-      <c r="AG11" s="11"/>
-      <c r="AH11" s="39">
-        <f>SUMIF(G11:AC11, "&lt;30")+AF11+AG11</f>
+      <c r="AF11" s="37"/>
+      <c r="AG11" s="10"/>
+      <c r="AH11" s="38">
+        <f t="shared" si="3"/>
         <v>132</v>
       </c>
-      <c r="AI11" s="67">
-        <f>AH11/AE11</f>
+      <c r="AI11" s="66">
+        <f t="shared" si="4"/>
         <v>18.857142857142858</v>
       </c>
-      <c r="AJ11" s="56"/>
-      <c r="AK11" s="39"/>
-      <c r="AL11" s="39"/>
-      <c r="AM11" s="12"/>
-      <c r="AN11" s="57"/>
+      <c r="AJ11" s="55"/>
+      <c r="AK11" s="38"/>
+      <c r="AL11" s="38"/>
+      <c r="AM11" s="11"/>
+      <c r="AN11" s="56"/>
     </row>
     <row r="12" spans="1:40">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="10">
-        <f>ROUND((AD12-(36*AE12))/AE12,0)</f>
+      <c r="C12" s="9">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="D12" s="49"/>
-      <c r="E12" s="50"/>
-      <c r="F12" s="13">
+      <c r="D12" s="48"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="12">
         <v>51</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="10">
         <v>18</v>
       </c>
-      <c r="H12" s="49"/>
-      <c r="I12" s="50"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="13">
+      <c r="H12" s="48"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="12">
         <v>51</v>
       </c>
-      <c r="O12" s="11">
+      <c r="O12" s="10">
         <v>18</v>
       </c>
-      <c r="P12" s="13">
+      <c r="P12" s="12">
         <v>52</v>
       </c>
-      <c r="Q12" s="11">
+      <c r="Q12" s="10">
         <v>17</v>
       </c>
-      <c r="R12" s="13"/>
-      <c r="S12" s="11"/>
-      <c r="T12" s="13"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="13"/>
-      <c r="W12" s="11"/>
-      <c r="X12" s="13">
+      <c r="R12" s="12"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="12"/>
+      <c r="W12" s="10"/>
+      <c r="X12" s="12">
         <v>48</v>
       </c>
-      <c r="Y12" s="11">
+      <c r="Y12" s="10">
         <v>21</v>
       </c>
-      <c r="Z12" s="70"/>
-      <c r="AA12" s="76"/>
-      <c r="AB12" s="70">
+      <c r="Z12" s="69"/>
+      <c r="AA12" s="75"/>
+      <c r="AB12" s="69">
         <v>51</v>
       </c>
-      <c r="AC12" s="76">
+      <c r="AC12" s="75">
         <v>18</v>
       </c>
-      <c r="AD12" s="63">
-        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12</f>
+      <c r="AD12" s="62">
+        <f t="shared" si="1"/>
         <v>253</v>
       </c>
-      <c r="AE12" s="12">
-        <f>COUNTIF(D12:AB12,"&gt;30")</f>
+      <c r="AE12" s="11">
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="AF12" s="38"/>
-      <c r="AG12" s="11"/>
-      <c r="AH12" s="39">
-        <f>SUMIF(G12:AC12, "&lt;30")+AF12+AG12</f>
+      <c r="AF12" s="37"/>
+      <c r="AG12" s="10"/>
+      <c r="AH12" s="38">
+        <f t="shared" si="3"/>
         <v>92</v>
       </c>
-      <c r="AI12" s="67">
-        <f>AH12/AE12</f>
+      <c r="AI12" s="66">
+        <f t="shared" si="4"/>
         <v>18.399999999999999</v>
       </c>
-      <c r="AJ12" s="59"/>
-      <c r="AK12" s="39"/>
-      <c r="AL12" s="39"/>
-      <c r="AM12" s="12"/>
-      <c r="AN12" s="57"/>
+      <c r="AJ12" s="58"/>
+      <c r="AK12" s="38"/>
+      <c r="AL12" s="38"/>
+      <c r="AM12" s="11"/>
+      <c r="AN12" s="56"/>
     </row>
     <row r="13" spans="1:40">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="10">
-        <f>ROUND((AD13-(36*AE13))/AE13,0)</f>
+      <c r="C13" s="9">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="D13" s="49"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="13">
+      <c r="D13" s="48"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="12">
         <v>41</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="10">
         <v>21</v>
       </c>
-      <c r="H13" s="49"/>
-      <c r="I13" s="50"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="53">
+      <c r="H13" s="48"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="52">
         <v>48</v>
       </c>
-      <c r="O13" s="11">
+      <c r="O13" s="10">
         <v>14</v>
       </c>
-      <c r="P13" s="40">
+      <c r="P13" s="39">
         <v>44</v>
       </c>
-      <c r="Q13" s="11">
+      <c r="Q13" s="10">
         <v>18</v>
       </c>
-      <c r="R13" s="40"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="40"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="40"/>
-      <c r="W13" s="11"/>
-      <c r="X13" s="14">
+      <c r="R13" s="39"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="39"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="39"/>
+      <c r="W13" s="10"/>
+      <c r="X13" s="13">
         <v>40</v>
       </c>
-      <c r="Y13" s="11">
+      <c r="Y13" s="10">
         <v>22</v>
       </c>
-      <c r="Z13" s="40">
+      <c r="Z13" s="39">
         <v>44</v>
       </c>
-      <c r="AA13" s="76">
+      <c r="AA13" s="75">
         <v>17</v>
       </c>
-      <c r="AB13" s="40">
+      <c r="AB13" s="39">
         <v>46</v>
       </c>
-      <c r="AC13" s="76">
+      <c r="AC13" s="75">
         <v>16</v>
       </c>
-      <c r="AD13" s="63">
-        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13</f>
+      <c r="AD13" s="62">
+        <f t="shared" si="1"/>
         <v>263</v>
       </c>
-      <c r="AE13" s="12">
-        <f>COUNTIF(D13:AB13,"&gt;30")</f>
+      <c r="AE13" s="11">
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="AF13" s="38">
+      <c r="AF13" s="37">
         <v>1</v>
       </c>
-      <c r="AG13" s="11">
+      <c r="AG13" s="10">
         <v>1</v>
       </c>
-      <c r="AH13" s="39">
-        <f>SUMIF(G13:AC13, "&lt;30")+AF13+AG13</f>
+      <c r="AH13" s="38">
+        <f t="shared" si="3"/>
         <v>110</v>
       </c>
-      <c r="AI13" s="67">
-        <f>AH13/AE13</f>
+      <c r="AI13" s="66">
+        <f t="shared" si="4"/>
         <v>18.333333333333332</v>
       </c>
-      <c r="AJ13" s="59"/>
-      <c r="AK13" s="39"/>
-      <c r="AL13" s="39"/>
-      <c r="AM13" s="12"/>
-      <c r="AN13" s="57"/>
+      <c r="AJ13" s="58"/>
+      <c r="AK13" s="38"/>
+      <c r="AL13" s="38"/>
+      <c r="AM13" s="11"/>
+      <c r="AN13" s="56"/>
     </row>
     <row r="14" spans="1:40">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="9">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="D14" s="49"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="13">
+      <c r="D14" s="48"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="12">
         <v>59</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="10">
         <v>17</v>
       </c>
-      <c r="H14" s="49"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="13">
+      <c r="H14" s="48"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="12">
         <v>55</v>
       </c>
-      <c r="S14" s="11">
+      <c r="S14" s="10">
         <v>21</v>
       </c>
-      <c r="T14" s="13"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="13">
+      <c r="T14" s="12"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="12">
         <v>59</v>
       </c>
-      <c r="W14" s="11">
+      <c r="W14" s="10">
         <v>17</v>
       </c>
-      <c r="X14" s="13"/>
-      <c r="Y14" s="11"/>
-      <c r="Z14" s="70"/>
-      <c r="AA14" s="76"/>
-      <c r="AB14" s="70"/>
-      <c r="AC14" s="76"/>
-      <c r="AD14" s="63">
-        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14</f>
+      <c r="X14" s="12"/>
+      <c r="Y14" s="10"/>
+      <c r="Z14" s="69"/>
+      <c r="AA14" s="75"/>
+      <c r="AB14" s="69"/>
+      <c r="AC14" s="75"/>
+      <c r="AD14" s="62">
+        <f t="shared" si="1"/>
         <v>173</v>
       </c>
-      <c r="AE14" s="12">
-        <f>COUNTIF(D14:AB14,"&gt;30")</f>
+      <c r="AE14" s="11">
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AF14" s="38"/>
-      <c r="AG14" s="11"/>
-      <c r="AH14" s="39">
-        <f>SUMIF(G14:AC14, "&lt;30")+AF14+AG14</f>
+      <c r="AF14" s="37"/>
+      <c r="AG14" s="10"/>
+      <c r="AH14" s="38">
+        <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="AI14" s="67">
-        <f>AH14/AE14</f>
+      <c r="AI14" s="66">
+        <f t="shared" si="4"/>
         <v>18.333333333333332</v>
       </c>
-      <c r="AJ14" s="59"/>
-      <c r="AK14" s="39"/>
-      <c r="AL14" s="39"/>
-      <c r="AM14" s="12"/>
-      <c r="AN14" s="57"/>
+      <c r="AJ14" s="58"/>
+      <c r="AK14" s="38"/>
+      <c r="AL14" s="38"/>
+      <c r="AM14" s="11"/>
+      <c r="AN14" s="56"/>
     </row>
     <row r="15" spans="1:40">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="9">
         <f>ROUND((AD15-(36*AE15))/AE15,0)</f>
         <v>9</v>
       </c>
-      <c r="D15" s="49"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="13">
+      <c r="D15" s="48"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="12">
         <v>46</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="10">
         <v>16</v>
       </c>
-      <c r="H15" s="49"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="13">
+      <c r="H15" s="48"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="12">
         <v>42</v>
       </c>
-      <c r="O15" s="11">
+      <c r="O15" s="10">
         <v>20</v>
       </c>
-      <c r="P15" s="13">
+      <c r="P15" s="12">
         <v>43</v>
       </c>
-      <c r="Q15" s="11">
+      <c r="Q15" s="10">
         <v>19</v>
       </c>
-      <c r="R15" s="13"/>
-      <c r="S15" s="11"/>
-      <c r="T15" s="13"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="13"/>
-      <c r="W15" s="11"/>
-      <c r="X15" s="13">
+      <c r="R15" s="12"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="12"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="12"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="12">
         <v>47</v>
       </c>
-      <c r="Y15" s="11">
+      <c r="Y15" s="10">
         <v>16</v>
       </c>
-      <c r="Z15" s="69">
+      <c r="Z15" s="68">
         <v>41</v>
       </c>
-      <c r="AA15" s="76">
+      <c r="AA15" s="75">
         <v>22</v>
       </c>
-      <c r="AB15" s="109">
+      <c r="AB15" s="78">
         <v>50</v>
       </c>
-      <c r="AC15" s="76">
+      <c r="AC15" s="75">
         <v>13</v>
       </c>
-      <c r="AD15" s="63">
-        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15</f>
+      <c r="AD15" s="62">
+        <f t="shared" si="1"/>
         <v>269</v>
       </c>
-      <c r="AE15" s="12">
-        <f>COUNTIF(D15:AB15,"&gt;30")</f>
+      <c r="AE15" s="11">
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="AF15" s="38">
+      <c r="AF15" s="37">
         <v>2</v>
       </c>
-      <c r="AG15" s="11">
+      <c r="AG15" s="10">
         <v>1</v>
       </c>
-      <c r="AH15" s="39">
-        <f>SUMIF(G15:AC15, "&lt;30")+AF15+AG15</f>
+      <c r="AH15" s="38">
+        <f t="shared" si="3"/>
         <v>109</v>
       </c>
-      <c r="AI15" s="67">
-        <f>AH15/AE15</f>
+      <c r="AI15" s="66">
+        <f t="shared" si="4"/>
         <v>18.166666666666668</v>
       </c>
-      <c r="AJ15" s="59"/>
-      <c r="AK15" s="39"/>
-      <c r="AL15" s="39"/>
-      <c r="AM15" s="12"/>
-      <c r="AN15" s="57"/>
+      <c r="AJ15" s="58"/>
+      <c r="AK15" s="38"/>
+      <c r="AL15" s="38"/>
+      <c r="AM15" s="11"/>
+      <c r="AN15" s="56"/>
     </row>
     <row r="16" spans="1:40">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="9">
         <f>ROUND((AD16-(36*AE16))/AE16,0)</f>
         <v>18</v>
       </c>
-      <c r="D16" s="49"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="13">
+      <c r="D16" s="48"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="12">
         <v>55</v>
       </c>
-      <c r="G16" s="11">
+      <c r="G16" s="10">
         <v>16</v>
       </c>
-      <c r="H16" s="49"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="13">
+      <c r="H16" s="48"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="12">
         <v>56</v>
       </c>
-      <c r="M16" s="11">
+      <c r="M16" s="10">
         <v>15</v>
       </c>
-      <c r="N16" s="13">
+      <c r="N16" s="12">
         <v>57</v>
       </c>
-      <c r="O16" s="11">
+      <c r="O16" s="10">
         <v>14</v>
       </c>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="13"/>
-      <c r="S16" s="11"/>
-      <c r="T16" s="69">
+      <c r="P16" s="12"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="68">
         <v>49</v>
       </c>
-      <c r="U16" s="11">
+      <c r="U16" s="10">
         <v>22</v>
       </c>
-      <c r="V16" s="69">
+      <c r="V16" s="68">
         <v>58</v>
       </c>
-      <c r="W16" s="11">
+      <c r="W16" s="10">
         <v>14</v>
       </c>
-      <c r="X16" s="70">
+      <c r="X16" s="69">
         <v>50</v>
       </c>
-      <c r="Y16" s="11">
+      <c r="Y16" s="10">
         <v>23</v>
       </c>
-      <c r="Z16" s="70">
+      <c r="Z16" s="69">
         <v>56</v>
       </c>
-      <c r="AA16" s="11">
+      <c r="AA16" s="10">
         <v>16</v>
       </c>
-      <c r="AB16" s="69">
+      <c r="AB16" s="68">
         <v>49</v>
       </c>
-      <c r="AC16" s="76">
+      <c r="AC16" s="75">
         <v>23</v>
       </c>
-      <c r="AD16" s="63">
-        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16</f>
+      <c r="AD16" s="62">
+        <f t="shared" si="1"/>
         <v>430</v>
       </c>
-      <c r="AE16" s="12">
-        <f>COUNTIF(D16:AB16,"&gt;30")</f>
+      <c r="AE16" s="11">
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="AF16" s="38">
+      <c r="AF16" s="37">
         <v>2</v>
       </c>
-      <c r="AG16" s="11"/>
-      <c r="AH16" s="39">
-        <f>SUMIF(G16:AC16, "&lt;30")+AF16+AG16</f>
+      <c r="AG16" s="10"/>
+      <c r="AH16" s="38">
+        <f t="shared" si="3"/>
         <v>145</v>
       </c>
-      <c r="AI16" s="67">
-        <f>AH16/AE16</f>
+      <c r="AI16" s="66">
+        <f t="shared" si="4"/>
         <v>18.125</v>
       </c>
-      <c r="AJ16" s="59"/>
-      <c r="AK16" s="39"/>
-      <c r="AL16" s="39"/>
-      <c r="AM16" s="12"/>
-      <c r="AN16" s="57"/>
+      <c r="AJ16" s="58"/>
+      <c r="AK16" s="38"/>
+      <c r="AL16" s="38"/>
+      <c r="AM16" s="11"/>
+      <c r="AN16" s="56"/>
     </row>
     <row r="17" spans="1:40">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="9">
         <f>ROUND((AD17-(36*AE17))/AE17,0)</f>
         <v>13</v>
       </c>
-      <c r="D17" s="49"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="13">
+      <c r="D17" s="48"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="48"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="12">
         <v>48</v>
       </c>
-      <c r="Q17" s="11">
+      <c r="Q17" s="10">
         <v>18</v>
       </c>
-      <c r="R17" s="13">
+      <c r="R17" s="12">
         <v>51</v>
       </c>
-      <c r="S17" s="11">
+      <c r="S17" s="10">
         <v>14</v>
       </c>
-      <c r="T17" s="13">
+      <c r="T17" s="12">
         <v>51</v>
       </c>
-      <c r="U17" s="11">
+      <c r="U17" s="10">
         <v>14</v>
       </c>
-      <c r="V17" s="13"/>
-      <c r="W17" s="11"/>
-      <c r="X17" s="13">
+      <c r="V17" s="12"/>
+      <c r="W17" s="10"/>
+      <c r="X17" s="12">
         <v>48</v>
       </c>
-      <c r="Y17" s="11">
+      <c r="Y17" s="10">
         <v>20</v>
       </c>
-      <c r="Z17" s="13">
+      <c r="Z17" s="12">
         <v>50</v>
       </c>
-      <c r="AA17" s="11">
+      <c r="AA17" s="10">
         <v>18</v>
       </c>
-      <c r="AB17" s="70">
+      <c r="AB17" s="69">
         <v>47</v>
       </c>
-      <c r="AC17" s="76">
+      <c r="AC17" s="75">
         <v>21</v>
       </c>
-      <c r="AD17" s="63">
-        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17</f>
+      <c r="AD17" s="62">
+        <f t="shared" si="1"/>
         <v>295</v>
       </c>
-      <c r="AE17" s="12">
-        <f>COUNTIF(D17:AB17,"&gt;30")</f>
+      <c r="AE17" s="11">
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="AF17" s="38"/>
-      <c r="AG17" s="11"/>
-      <c r="AH17" s="39">
-        <f>SUMIF(G17:AC17, "&lt;30")+AF17+AG17</f>
+      <c r="AF17" s="37"/>
+      <c r="AG17" s="10"/>
+      <c r="AH17" s="38">
+        <f t="shared" si="3"/>
         <v>105</v>
       </c>
-      <c r="AI17" s="67">
-        <f>AH17/AE17</f>
+      <c r="AI17" s="66">
+        <f t="shared" si="4"/>
         <v>17.5</v>
       </c>
-      <c r="AJ17" s="56"/>
-      <c r="AK17" s="39"/>
-      <c r="AL17" s="39"/>
-      <c r="AM17" s="12"/>
-      <c r="AN17" s="57"/>
+      <c r="AJ17" s="55"/>
+      <c r="AK17" s="38"/>
+      <c r="AL17" s="38"/>
+      <c r="AM17" s="11"/>
+      <c r="AN17" s="56"/>
     </row>
     <row r="18" spans="1:40">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="10">
-        <v>9</v>
-      </c>
-      <c r="D18" s="49"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="49"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="40">
+      <c r="C18" s="9">
+        <f>ROUND((AD18-(36*AE18))/AE18,0)</f>
+        <v>10</v>
+      </c>
+      <c r="D18" s="48"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="39">
         <v>45</v>
       </c>
-      <c r="O18" s="11">
+      <c r="O18" s="10">
         <v>18</v>
       </c>
-      <c r="P18" s="40">
+      <c r="P18" s="39">
         <v>43</v>
       </c>
-      <c r="Q18" s="11">
+      <c r="Q18" s="10">
         <v>20</v>
       </c>
-      <c r="R18" s="40"/>
-      <c r="S18" s="11"/>
-      <c r="T18" s="40"/>
-      <c r="U18" s="11"/>
-      <c r="V18" s="40"/>
-      <c r="W18" s="11"/>
-      <c r="X18" s="40">
+      <c r="R18" s="39"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="39"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="39"/>
+      <c r="W18" s="10"/>
+      <c r="X18" s="39">
         <v>48</v>
       </c>
-      <c r="Y18" s="11">
+      <c r="Y18" s="10">
         <v>15</v>
       </c>
-      <c r="Z18" s="40">
+      <c r="Z18" s="39">
         <v>47</v>
       </c>
-      <c r="AA18" s="76">
+      <c r="AA18" s="75">
         <v>16</v>
       </c>
-      <c r="AB18" s="40"/>
-      <c r="AC18" s="76"/>
-      <c r="AD18" s="63">
-        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18</f>
+      <c r="AB18" s="39"/>
+      <c r="AC18" s="75"/>
+      <c r="AD18" s="62">
+        <f t="shared" si="1"/>
         <v>183</v>
       </c>
-      <c r="AE18" s="12">
-        <f>COUNTIF(D18:AB18,"&gt;30")</f>
+      <c r="AE18" s="11">
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="AF18" s="38"/>
-      <c r="AG18" s="11">
+      <c r="AF18" s="37"/>
+      <c r="AG18" s="10">
         <v>1</v>
       </c>
-      <c r="AH18" s="39">
-        <f>SUMIF(G18:AC18, "&lt;30")+AF18+AG18</f>
+      <c r="AH18" s="38">
+        <f t="shared" si="3"/>
         <v>70</v>
       </c>
-      <c r="AI18" s="67">
-        <f>AH18/AE18</f>
+      <c r="AI18" s="66">
+        <f t="shared" si="4"/>
         <v>17.5</v>
       </c>
-      <c r="AJ18" s="56"/>
-      <c r="AK18" s="39"/>
-      <c r="AL18" s="39"/>
-      <c r="AM18" s="12"/>
-      <c r="AN18" s="57"/>
+      <c r="AJ18" s="55"/>
+      <c r="AK18" s="38"/>
+      <c r="AL18" s="38"/>
+      <c r="AM18" s="11"/>
+      <c r="AN18" s="56"/>
     </row>
     <row r="19" spans="1:40">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <f>ROUND((AD19-(36*AE19))/AE19,0)</f>
         <v>12</v>
       </c>
-      <c r="D19" s="49"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="13">
+      <c r="D19" s="48"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="12">
         <v>46</v>
       </c>
-      <c r="G19" s="11">
+      <c r="G19" s="10">
         <v>18</v>
       </c>
-      <c r="H19" s="49"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="13">
+      <c r="H19" s="48"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="12">
         <v>46</v>
       </c>
-      <c r="M19" s="11">
+      <c r="M19" s="10">
         <v>18</v>
       </c>
-      <c r="N19" s="13">
+      <c r="N19" s="12">
         <v>46</v>
       </c>
-      <c r="O19" s="11">
+      <c r="O19" s="10">
         <v>18</v>
       </c>
-      <c r="P19" s="13">
+      <c r="P19" s="12">
         <v>46</v>
       </c>
-      <c r="Q19" s="11">
+      <c r="Q19" s="10">
         <v>18</v>
       </c>
-      <c r="R19" s="13">
+      <c r="R19" s="12">
         <v>47</v>
       </c>
-      <c r="S19" s="11">
+      <c r="S19" s="10">
         <v>14</v>
       </c>
-      <c r="T19" s="13">
+      <c r="T19" s="12">
         <v>52</v>
       </c>
-      <c r="U19" s="11">
+      <c r="U19" s="10">
         <v>13</v>
       </c>
-      <c r="V19" s="13"/>
-      <c r="W19" s="11"/>
-      <c r="X19" s="13"/>
-      <c r="Y19" s="11"/>
-      <c r="Z19" s="13">
+      <c r="V19" s="12"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="12"/>
+      <c r="Y19" s="10"/>
+      <c r="Z19" s="12">
         <v>50</v>
       </c>
-      <c r="AA19" s="11">
+      <c r="AA19" s="10">
         <v>15</v>
       </c>
-      <c r="AB19" s="70"/>
-      <c r="AC19" s="76"/>
-      <c r="AD19" s="63">
-        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19</f>
+      <c r="AB19" s="69"/>
+      <c r="AC19" s="75"/>
+      <c r="AD19" s="62">
+        <f t="shared" si="1"/>
         <v>333</v>
       </c>
-      <c r="AE19" s="12">
-        <f>COUNTIF(D19:AB19,"&gt;30")</f>
+      <c r="AE19" s="11">
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AF19" s="41"/>
-      <c r="AG19" s="31"/>
-      <c r="AH19" s="39">
-        <f>SUMIF(G19:AC19, "&lt;30")+AF19+AG19</f>
+      <c r="AF19" s="40"/>
+      <c r="AG19" s="30"/>
+      <c r="AH19" s="38">
+        <f t="shared" si="3"/>
         <v>114</v>
       </c>
-      <c r="AI19" s="67">
-        <f>AH19/AE19</f>
+      <c r="AI19" s="66">
+        <f t="shared" si="4"/>
         <v>16.285714285714285</v>
       </c>
-      <c r="AJ19" s="59"/>
-      <c r="AK19" s="12"/>
-      <c r="AL19" s="12"/>
-      <c r="AM19" s="12"/>
-      <c r="AN19" s="57"/>
+      <c r="AJ19" s="58"/>
+      <c r="AK19" s="11"/>
+      <c r="AL19" s="11"/>
+      <c r="AM19" s="11"/>
+      <c r="AN19" s="56"/>
     </row>
     <row r="20" spans="1:40">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <f>ROUND((AD20-(36*AE20))/AE20,0)</f>
         <v>24</v>
       </c>
-      <c r="D20" s="49"/>
-      <c r="E20" s="50"/>
-      <c r="F20" s="14">
+      <c r="D20" s="48"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="13">
         <v>61</v>
       </c>
-      <c r="G20" s="11">
+      <c r="G20" s="10">
         <v>14</v>
       </c>
-      <c r="H20" s="49"/>
-      <c r="I20" s="50"/>
-      <c r="J20" s="14">
+      <c r="H20" s="48"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="13">
         <v>56</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20" s="10">
         <v>19</v>
       </c>
-      <c r="L20" s="40">
+      <c r="L20" s="39">
         <v>60</v>
       </c>
-      <c r="M20" s="11">
+      <c r="M20" s="10">
         <v>15</v>
       </c>
-      <c r="N20" s="40">
+      <c r="N20" s="39">
         <v>56</v>
       </c>
-      <c r="O20" s="11">
+      <c r="O20" s="10">
         <v>20</v>
       </c>
-      <c r="P20" s="40">
+      <c r="P20" s="39">
         <v>54</v>
       </c>
-      <c r="Q20" s="11">
+      <c r="Q20" s="10">
         <v>22</v>
       </c>
-      <c r="R20" s="40"/>
-      <c r="S20" s="11"/>
-      <c r="T20" s="40">
+      <c r="R20" s="39"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="39">
         <v>66</v>
       </c>
-      <c r="U20" s="11">
+      <c r="U20" s="10">
         <v>9</v>
       </c>
-      <c r="V20" s="40">
+      <c r="V20" s="39">
         <v>55</v>
       </c>
-      <c r="W20" s="11">
+      <c r="W20" s="10">
         <v>22</v>
       </c>
-      <c r="X20" s="40"/>
-      <c r="Y20" s="11"/>
-      <c r="Z20" s="40">
+      <c r="X20" s="39"/>
+      <c r="Y20" s="10"/>
+      <c r="Z20" s="39">
         <v>70</v>
       </c>
-      <c r="AA20" s="76">
+      <c r="AA20" s="75">
         <v>6</v>
       </c>
-      <c r="AB20" s="40">
+      <c r="AB20" s="39">
         <v>63</v>
       </c>
-      <c r="AC20" s="76">
+      <c r="AC20" s="75">
         <v>15</v>
       </c>
-      <c r="AD20" s="63">
-        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20</f>
+      <c r="AD20" s="62">
+        <f t="shared" si="1"/>
         <v>541</v>
       </c>
-      <c r="AE20" s="12">
-        <f>COUNTIF(D20:AB20,"&gt;30")</f>
+      <c r="AE20" s="11">
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="AF20" s="38">
+      <c r="AF20" s="37">
         <v>2</v>
       </c>
-      <c r="AG20" s="11"/>
-      <c r="AH20" s="39">
-        <f>SUMIF(G20:AC20, "&lt;30")+AF20+AG20</f>
+      <c r="AG20" s="10"/>
+      <c r="AH20" s="38">
+        <f t="shared" si="3"/>
         <v>144</v>
       </c>
-      <c r="AI20" s="67">
-        <f>AH20/AE20</f>
+      <c r="AI20" s="66">
+        <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="AJ20" s="56"/>
-      <c r="AK20" s="39"/>
-      <c r="AL20" s="39"/>
-      <c r="AM20" s="12"/>
-      <c r="AN20" s="57"/>
+      <c r="AJ20" s="55"/>
+      <c r="AK20" s="38"/>
+      <c r="AL20" s="38"/>
+      <c r="AM20" s="11"/>
+      <c r="AN20" s="56"/>
     </row>
     <row r="21" spans="1:40">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="9">
         <v>18</v>
       </c>
-      <c r="D21" s="49"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="13">
+      <c r="D21" s="48"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="12">
         <v>56</v>
       </c>
-      <c r="G21" s="11">
+      <c r="G21" s="10">
         <v>16</v>
       </c>
-      <c r="H21" s="49"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="13"/>
-      <c r="S21" s="11"/>
-      <c r="T21" s="13"/>
-      <c r="U21" s="11"/>
-      <c r="V21" s="13"/>
-      <c r="W21" s="11"/>
-      <c r="X21" s="13"/>
-      <c r="Y21" s="11"/>
-      <c r="Z21" s="13"/>
-      <c r="AA21" s="11"/>
-      <c r="AB21" s="70"/>
-      <c r="AC21" s="76"/>
-      <c r="AD21" s="63">
-        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21</f>
+      <c r="H21" s="48"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="12"/>
+      <c r="U21" s="10"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="10"/>
+      <c r="X21" s="12"/>
+      <c r="Y21" s="10"/>
+      <c r="Z21" s="12"/>
+      <c r="AA21" s="10"/>
+      <c r="AB21" s="69"/>
+      <c r="AC21" s="75"/>
+      <c r="AD21" s="62">
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
-      <c r="AE21" s="12">
-        <f>COUNTIF(D21:AB21,"&gt;30")</f>
+      <c r="AE21" s="11">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AF21" s="38"/>
-      <c r="AG21" s="11"/>
-      <c r="AH21" s="39">
-        <f>SUMIF(G21:AC21, "&lt;30")+AF21+AG21</f>
+      <c r="AF21" s="37"/>
+      <c r="AG21" s="10"/>
+      <c r="AH21" s="38">
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="AI21" s="67">
-        <f>AH21/AE21</f>
+      <c r="AI21" s="66">
+        <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="AJ21" s="59"/>
-      <c r="AK21" s="39"/>
-      <c r="AL21" s="39"/>
-      <c r="AM21" s="12"/>
-      <c r="AN21" s="57"/>
+      <c r="AJ21" s="58"/>
+      <c r="AK21" s="38"/>
+      <c r="AL21" s="38"/>
+      <c r="AM21" s="11"/>
+      <c r="AN21" s="56"/>
     </row>
-    <row r="22" spans="1:40" ht="17" thickBot="1">
-      <c r="A22" s="16" t="s">
+    <row r="22" spans="1:40" ht="16.5" thickBot="1">
+      <c r="A22" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="51"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="51"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="73"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="74">
+      <c r="D22" s="50"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="72"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="51"/>
+      <c r="J22" s="72"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="73">
         <v>50</v>
       </c>
-      <c r="M22" s="19"/>
-      <c r="N22" s="74"/>
-      <c r="O22" s="19"/>
-      <c r="P22" s="74"/>
-      <c r="Q22" s="19"/>
-      <c r="R22" s="74"/>
-      <c r="S22" s="19"/>
-      <c r="T22" s="74"/>
-      <c r="U22" s="19"/>
-      <c r="V22" s="74"/>
-      <c r="W22" s="19"/>
-      <c r="X22" s="74"/>
-      <c r="Y22" s="19"/>
-      <c r="Z22" s="74"/>
-      <c r="AA22" s="19"/>
-      <c r="AB22" s="74"/>
-      <c r="AC22" s="19"/>
-      <c r="AD22" s="64">
-        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22</f>
+      <c r="M22" s="18"/>
+      <c r="N22" s="73"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="73"/>
+      <c r="Q22" s="18"/>
+      <c r="R22" s="73"/>
+      <c r="S22" s="18"/>
+      <c r="T22" s="73"/>
+      <c r="U22" s="18"/>
+      <c r="V22" s="73"/>
+      <c r="W22" s="18"/>
+      <c r="X22" s="73"/>
+      <c r="Y22" s="18"/>
+      <c r="Z22" s="73"/>
+      <c r="AA22" s="18"/>
+      <c r="AB22" s="73"/>
+      <c r="AC22" s="18"/>
+      <c r="AD22" s="63">
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="AE22" s="20">
-        <f>COUNTIF(D22:AB22,"&gt;30")</f>
+      <c r="AE22" s="19">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AF22" s="42">
+      <c r="AF22" s="41">
         <v>1</v>
       </c>
-      <c r="AG22" s="19"/>
-      <c r="AH22" s="43">
-        <f>SUMIF(G22:AC22, "&lt;30")+AF22+AG22</f>
+      <c r="AG22" s="18"/>
+      <c r="AH22" s="42">
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="AI22" s="68">
-        <f>AH22/AE22</f>
+      <c r="AI22" s="67">
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="AJ22" s="60"/>
-      <c r="AK22" s="43"/>
-      <c r="AL22" s="43"/>
-      <c r="AM22" s="20"/>
-      <c r="AN22" s="61"/>
+      <c r="AJ22" s="59"/>
+      <c r="AK22" s="42"/>
+      <c r="AL22" s="42"/>
+      <c r="AM22" s="19"/>
+      <c r="AN22" s="60"/>
     </row>
-    <row r="23" spans="1:40" s="21" customFormat="1" ht="17" thickBot="1">
-      <c r="A23" s="32"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34">
+    <row r="23" spans="1:40" s="20" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A23" s="31"/>
+      <c r="B23" s="32"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33">
         <f>AVERAGEIF(F4:F22,"&gt;0")</f>
         <v>49.75</v>
       </c>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="34">
+      <c r="G23" s="33"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+      <c r="J23" s="33">
         <f>AVERAGEIF(J4:J22,"&gt;0")</f>
         <v>54</v>
       </c>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34">
+      <c r="K23" s="33"/>
+      <c r="L23" s="33">
         <f>AVERAGEIF(L4:L22,"&gt;0")</f>
         <v>51.428571428571431</v>
       </c>
-      <c r="M23" s="34"/>
-      <c r="N23" s="34">
+      <c r="M23" s="33"/>
+      <c r="N23" s="33">
         <f>AVERAGEIF(N4:N22,"&gt;0")</f>
         <v>48.9</v>
       </c>
-      <c r="O23" s="34"/>
-      <c r="P23" s="34">
+      <c r="O23" s="33"/>
+      <c r="P23" s="33">
         <f>AVERAGEIF(P4:P22,"&gt;0")</f>
         <v>46.785714285714285</v>
       </c>
-      <c r="Q23" s="34"/>
-      <c r="R23" s="34">
+      <c r="Q23" s="33"/>
+      <c r="R23" s="33">
         <f>AVERAGEIF(R4:R22,"&gt;0")</f>
         <v>48.272727272727273</v>
       </c>
-      <c r="S23" s="34"/>
-      <c r="T23" s="34">
+      <c r="S23" s="33"/>
+      <c r="T23" s="33">
         <f>AVERAGEIF(T4:T22,"&gt;0")</f>
         <v>50.333333333333336</v>
       </c>
-      <c r="U23" s="34"/>
-      <c r="V23" s="34">
+      <c r="U23" s="33"/>
+      <c r="V23" s="33">
         <f>AVERAGEIF(V4:V22,"&gt;0")</f>
         <v>49</v>
       </c>
-      <c r="W23" s="34"/>
-      <c r="X23" s="34">
+      <c r="W23" s="33"/>
+      <c r="X23" s="33">
         <f>AVERAGEIF(X4:X22,"&gt;0")</f>
         <v>46.46153846153846</v>
       </c>
-      <c r="Y23" s="34"/>
-      <c r="Z23" s="34">
+      <c r="Y23" s="33"/>
+      <c r="Z23" s="33">
         <f>AVERAGEIF(Z4:Z22,"&gt;0")</f>
         <v>49.53846153846154</v>
       </c>
-      <c r="AA23" s="34"/>
-      <c r="AB23" s="34">
+      <c r="AA23" s="33"/>
+      <c r="AB23" s="33">
         <f>AVERAGEIF(AB4:AB22,"&gt;0")</f>
         <v>47.846153846153847</v>
       </c>
-      <c r="AC23" s="34"/>
-      <c r="AD23" s="35"/>
+      <c r="AC23" s="33"/>
+      <c r="AD23" s="34"/>
     </row>
     <row r="24" spans="1:40">
-      <c r="C24" s="22"/>
-      <c r="AD24" s="23"/>
-      <c r="AE24" s="23"/>
-      <c r="AF24" s="24"/>
-      <c r="AG24" s="24"/>
-      <c r="AH24" s="23"/>
-      <c r="AI24" s="25"/>
+      <c r="C24" s="21"/>
+      <c r="AD24" s="22"/>
+      <c r="AE24" s="22"/>
+      <c r="AF24" s="23"/>
+      <c r="AG24" s="23"/>
+      <c r="AH24" s="22"/>
+      <c r="AI24" s="24"/>
     </row>
     <row r="25" spans="1:40">
-      <c r="C25" s="44" t="s">
+      <c r="C25" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="F25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="J25" s="26"/>
-      <c r="L25" s="26"/>
-      <c r="N25" s="26"/>
-      <c r="P25" s="26"/>
-      <c r="R25" s="26"/>
-      <c r="T25" s="26"/>
-      <c r="V25" s="26"/>
-      <c r="X25" s="26"/>
-      <c r="Z25" s="26"/>
-      <c r="AB25" s="26"/>
+      <c r="F25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="J25" s="25"/>
+      <c r="L25" s="25"/>
+      <c r="N25" s="25"/>
+      <c r="P25" s="25"/>
+      <c r="R25" s="25"/>
+      <c r="T25" s="25"/>
+      <c r="V25" s="25"/>
+      <c r="X25" s="25"/>
+      <c r="Z25" s="25"/>
+      <c r="AB25" s="25"/>
     </row>
     <row r="26" spans="1:40">
-      <c r="C26" s="45" t="s">
+      <c r="C26" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="27" t="s">
+      <c r="D26" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="J26" s="27"/>
-      <c r="L26" s="27"/>
-      <c r="N26" s="27"/>
-      <c r="P26" s="27"/>
-      <c r="R26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="V26" s="27"/>
-      <c r="X26" s="27"/>
-      <c r="Z26" s="27"/>
-      <c r="AB26" s="27"/>
-      <c r="AD26" s="28"/>
+      <c r="F26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="N26" s="26"/>
+      <c r="P26" s="26"/>
+      <c r="R26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="V26" s="26"/>
+      <c r="X26" s="26"/>
+      <c r="Z26" s="26"/>
+      <c r="AB26" s="26"/>
+      <c r="AD26" s="27"/>
     </row>
     <row r="27" spans="1:40">
-      <c r="C27" s="46" t="s">
+      <c r="C27" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="D27" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="30"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="30"/>
-      <c r="L27" s="29"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="29"/>
-      <c r="O27" s="30"/>
-      <c r="P27" s="29"/>
-      <c r="Q27" s="30"/>
-      <c r="R27" s="29"/>
-      <c r="S27" s="30"/>
-      <c r="T27" s="29"/>
-      <c r="U27" s="30"/>
-      <c r="V27" s="29"/>
-      <c r="W27" s="30"/>
-      <c r="X27" s="29"/>
-      <c r="Y27" s="30"/>
-      <c r="Z27" s="29"/>
-      <c r="AA27" s="30"/>
-      <c r="AB27" s="29"/>
-      <c r="AC27" s="30"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="29"/>
+      <c r="L27" s="28"/>
+      <c r="M27" s="29"/>
+      <c r="N27" s="28"/>
+      <c r="O27" s="29"/>
+      <c r="P27" s="28"/>
+      <c r="Q27" s="29"/>
+      <c r="R27" s="28"/>
+      <c r="S27" s="29"/>
+      <c r="T27" s="28"/>
+      <c r="U27" s="29"/>
+      <c r="V27" s="28"/>
+      <c r="W27" s="29"/>
+      <c r="X27" s="28"/>
+      <c r="Y27" s="29"/>
+      <c r="Z27" s="28"/>
+      <c r="AA27" s="29"/>
+      <c r="AB27" s="28"/>
+      <c r="AC27" s="29"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AN22">
@@ -3697,8 +3733,6 @@
     <sortCondition descending="1" ref="AD4:AD22"/>
   </sortState>
   <mergeCells count="41">
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="AB1:AC1"/>
     <mergeCell ref="AB2:AC2"/>
     <mergeCell ref="AJ1:AN1"/>
     <mergeCell ref="AJ2:AJ3"/>
@@ -3708,8 +3742,6 @@
     <mergeCell ref="AN2:AN3"/>
     <mergeCell ref="AH2:AH3"/>
     <mergeCell ref="AI2:AI3"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
     <mergeCell ref="AF2:AF3"/>
     <mergeCell ref="AG2:AG3"/>
     <mergeCell ref="AE2:AE3"/>
@@ -3723,21 +3755,25 @@
     <mergeCell ref="R2:S2"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="AB1:AC1"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="X2:Y2"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
081925 - updated weeks 15/16 scores and week 15 skins
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{F94A3502-0EBB-1C4C-B4A9-72D954014F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A7BFC1A-C7C6-4DB9-B4B8-215DAD07F51B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAD6DB6-E3D7-F14D-BFB0-08DA4216CCD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43125" yWindow="3150" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="43100" yWindow="3160" windowWidth="30760" windowHeight="17120" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -238,6 +238,15 @@
   </si>
   <si>
     <t>WEEK 13</t>
+  </si>
+  <si>
+    <t>WEEK 14</t>
+  </si>
+  <si>
+    <t>WEEK 15</t>
+  </si>
+  <si>
+    <t>WEEK 16</t>
   </si>
 </sst>
 </file>
@@ -979,7 +988,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1129,9 +1138,6 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1195,18 +1201,6 @@
     <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="43" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1216,12 +1210,66 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1249,59 +1297,29 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1318,10 +1336,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1641,203 +1655,233 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
-  <dimension ref="A1:AN27"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AT27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="8.625" customWidth="1"/>
-    <col min="2" max="2" width="8.125" customWidth="1"/>
-    <col min="3" max="3" width="10.125" customWidth="1"/>
-    <col min="4" max="10" width="6.875" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="8.1640625" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" customWidth="1"/>
+    <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="23" width="6.375" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="6" customWidth="1"/>
-    <col min="25" max="25" width="6.375" customWidth="1"/>
-    <col min="26" max="26" width="6" customWidth="1"/>
-    <col min="27" max="27" width="6.375" customWidth="1"/>
-    <col min="28" max="28" width="6" customWidth="1"/>
-    <col min="29" max="29" width="6.375" customWidth="1"/>
-    <col min="30" max="30" width="8.875" customWidth="1"/>
-    <col min="31" max="31" width="6.125" customWidth="1"/>
-    <col min="32" max="32" width="5.875" customWidth="1"/>
-    <col min="33" max="33" width="5.625" customWidth="1"/>
-    <col min="34" max="34" width="5.5" customWidth="1"/>
-    <col min="35" max="35" width="8" customWidth="1"/>
-    <col min="36" max="36" width="7.375" hidden="1" customWidth="1"/>
-    <col min="37" max="38" width="6" hidden="1" customWidth="1"/>
-    <col min="39" max="39" width="7.375" hidden="1" customWidth="1"/>
-    <col min="40" max="40" width="9.375" hidden="1" customWidth="1"/>
+    <col min="12" max="23" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="6" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="6" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="6" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="6" customWidth="1"/>
+    <col min="31" max="31" width="6.33203125" customWidth="1"/>
+    <col min="32" max="32" width="6" customWidth="1"/>
+    <col min="33" max="33" width="6.33203125" customWidth="1"/>
+    <col min="34" max="34" width="6" customWidth="1"/>
+    <col min="35" max="35" width="6.33203125" customWidth="1"/>
+    <col min="36" max="36" width="8.83203125" customWidth="1"/>
+    <col min="37" max="37" width="6.1640625" customWidth="1"/>
+    <col min="38" max="38" width="5.83203125" customWidth="1"/>
+    <col min="39" max="39" width="5.6640625" customWidth="1"/>
+    <col min="40" max="40" width="5.5" customWidth="1"/>
+    <col min="41" max="41" width="8" customWidth="1"/>
+    <col min="42" max="42" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="43" max="44" width="6" hidden="1" customWidth="1"/>
+    <col min="45" max="45" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="46" max="46" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="53" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="88" t="s">
+    <row r="1" spans="1:46" s="53" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="94" t="s">
+      <c r="B1" s="102"/>
+      <c r="C1" s="107" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="86" t="s">
+      <c r="D1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="87"/>
-      <c r="F1" s="86" t="s">
+      <c r="E1" s="97"/>
+      <c r="F1" s="96" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="87"/>
-      <c r="H1" s="86" t="s">
+      <c r="G1" s="97"/>
+      <c r="H1" s="96" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="87"/>
-      <c r="J1" s="86" t="s">
+      <c r="I1" s="97"/>
+      <c r="J1" s="96" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="87"/>
-      <c r="L1" s="86" t="s">
+      <c r="K1" s="97"/>
+      <c r="L1" s="96" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="87"/>
-      <c r="N1" s="86" t="s">
+      <c r="M1" s="97"/>
+      <c r="N1" s="96" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="87"/>
-      <c r="P1" s="86" t="s">
+      <c r="O1" s="97"/>
+      <c r="P1" s="96" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="87"/>
-      <c r="R1" s="86" t="s">
+      <c r="Q1" s="97"/>
+      <c r="R1" s="96" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="87"/>
-      <c r="T1" s="86" t="s">
+      <c r="S1" s="97"/>
+      <c r="T1" s="96" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="87"/>
-      <c r="V1" s="86" t="s">
+      <c r="U1" s="97"/>
+      <c r="V1" s="96" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="87"/>
-      <c r="X1" s="86" t="s">
+      <c r="W1" s="97"/>
+      <c r="X1" s="96" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="87"/>
-      <c r="Z1" s="86" t="s">
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="96" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="87"/>
-      <c r="AB1" s="86" t="s">
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="96" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="87"/>
-      <c r="AD1" s="101" t="s">
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="96" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE1" s="97"/>
+      <c r="AF1" s="96" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="96" t="s">
+        <v>69</v>
+      </c>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="AE1" s="103" t="s">
+      <c r="AK1" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="AF1" s="104"/>
-      <c r="AG1" s="104"/>
-      <c r="AH1" s="104"/>
-      <c r="AI1" s="105"/>
-      <c r="AJ1" s="106" t="s">
+      <c r="AL1" s="99"/>
+      <c r="AM1" s="99"/>
+      <c r="AN1" s="99"/>
+      <c r="AO1" s="100"/>
+      <c r="AP1" s="81" t="s">
         <v>57</v>
       </c>
-      <c r="AK1" s="107"/>
-      <c r="AL1" s="107"/>
-      <c r="AM1" s="107"/>
-      <c r="AN1" s="108"/>
+      <c r="AQ1" s="82"/>
+      <c r="AR1" s="82"/>
+      <c r="AS1" s="82"/>
+      <c r="AT1" s="83"/>
     </row>
-    <row r="2" spans="1:40" s="53" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="90"/>
-      <c r="B2" s="91"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="84">
+    <row r="2" spans="1:46" s="53" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="103"/>
+      <c r="B2" s="104"/>
+      <c r="C2" s="108"/>
+      <c r="D2" s="79">
         <v>45782</v>
       </c>
-      <c r="E2" s="85"/>
-      <c r="F2" s="84">
+      <c r="E2" s="80"/>
+      <c r="F2" s="79">
         <v>45789</v>
       </c>
-      <c r="G2" s="85"/>
-      <c r="H2" s="84">
+      <c r="G2" s="80"/>
+      <c r="H2" s="79">
         <v>45796</v>
       </c>
-      <c r="I2" s="85"/>
-      <c r="J2" s="84">
+      <c r="I2" s="80"/>
+      <c r="J2" s="79">
         <v>45803</v>
       </c>
-      <c r="K2" s="85"/>
-      <c r="L2" s="84">
+      <c r="K2" s="80"/>
+      <c r="L2" s="79">
         <v>45810</v>
       </c>
-      <c r="M2" s="85"/>
-      <c r="N2" s="84">
+      <c r="M2" s="80"/>
+      <c r="N2" s="79">
         <v>45817</v>
       </c>
-      <c r="O2" s="85"/>
-      <c r="P2" s="84">
+      <c r="O2" s="80"/>
+      <c r="P2" s="79">
         <v>45824</v>
       </c>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="84">
+      <c r="Q2" s="80"/>
+      <c r="R2" s="79">
         <v>45831</v>
       </c>
-      <c r="S2" s="85"/>
-      <c r="T2" s="84">
+      <c r="S2" s="80"/>
+      <c r="T2" s="79">
         <v>45838</v>
       </c>
-      <c r="U2" s="85"/>
-      <c r="V2" s="84">
+      <c r="U2" s="80"/>
+      <c r="V2" s="79">
         <v>45845</v>
       </c>
-      <c r="W2" s="85"/>
-      <c r="X2" s="84">
+      <c r="W2" s="80"/>
+      <c r="X2" s="79">
         <v>45852</v>
       </c>
-      <c r="Y2" s="85"/>
-      <c r="Z2" s="84">
+      <c r="Y2" s="80"/>
+      <c r="Z2" s="79">
         <v>45859</v>
       </c>
-      <c r="AA2" s="85"/>
-      <c r="AB2" s="84">
+      <c r="AA2" s="80"/>
+      <c r="AB2" s="79">
         <v>45866</v>
       </c>
-      <c r="AC2" s="85"/>
-      <c r="AD2" s="102"/>
-      <c r="AE2" s="101" t="s">
+      <c r="AC2" s="80"/>
+      <c r="AD2" s="79">
+        <v>45873</v>
+      </c>
+      <c r="AE2" s="80"/>
+      <c r="AF2" s="79">
+        <v>45880</v>
+      </c>
+      <c r="AG2" s="80"/>
+      <c r="AH2" s="79">
+        <v>45887</v>
+      </c>
+      <c r="AI2" s="80"/>
+      <c r="AJ2" s="95"/>
+      <c r="AK2" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="AF2" s="97" t="s">
+      <c r="AL2" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="AG2" s="99" t="s">
+      <c r="AM2" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="AH2" s="111" t="s">
+      <c r="AN2" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="AI2" s="113" t="s">
+      <c r="AO2" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="AJ2" s="109" t="s">
+      <c r="AP2" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="AK2" s="109" t="s">
+      <c r="AQ2" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="AL2" s="109" t="s">
+      <c r="AR2" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="AM2" s="109" t="s">
+      <c r="AS2" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="AN2" s="109" t="s">
+      <c r="AT2" s="84" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:40" s="53" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
-      <c r="A3" s="92"/>
-      <c r="B3" s="93"/>
-      <c r="C3" s="96"/>
+    <row r="3" spans="1:46" s="53" customFormat="1" ht="29" customHeight="1" thickBot="1">
+      <c r="A3" s="105"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="109"/>
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1916,280 +1960,360 @@
       <c r="AC3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="AD3" s="102"/>
-      <c r="AE3" s="102"/>
-      <c r="AF3" s="98"/>
-      <c r="AG3" s="100"/>
-      <c r="AH3" s="112"/>
-      <c r="AI3" s="114"/>
-      <c r="AJ3" s="110"/>
-      <c r="AK3" s="110"/>
-      <c r="AL3" s="110"/>
-      <c r="AM3" s="110"/>
-      <c r="AN3" s="110"/>
+      <c r="AD3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AG3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ3" s="95"/>
+      <c r="AK3" s="95"/>
+      <c r="AL3" s="91"/>
+      <c r="AM3" s="93"/>
+      <c r="AN3" s="87"/>
+      <c r="AO3" s="89"/>
+      <c r="AP3" s="85"/>
+      <c r="AQ3" s="85"/>
+      <c r="AR3" s="85"/>
+      <c r="AS3" s="85"/>
+      <c r="AT3" s="85"/>
     </row>
-    <row r="4" spans="1:40" ht="15.95" customHeight="1">
+    <row r="4" spans="1:46" ht="16" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="83">
-        <f t="shared" ref="C4:C14" si="0">ROUND((AD4-(36*AE4))/AE4,0)</f>
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="C4" s="78">
+        <f>ROUND((AJ4-(36*AK4))/AK4,0)</f>
+        <v>17</v>
       </c>
       <c r="D4" s="46"/>
       <c r="E4" s="47"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="5"/>
+      <c r="F4" s="111">
+        <v>53</v>
+      </c>
+      <c r="G4" s="5">
+        <v>23</v>
+      </c>
       <c r="H4" s="46"/>
       <c r="I4" s="47"/>
-      <c r="J4" s="79"/>
+      <c r="J4" s="111"/>
       <c r="K4" s="5"/>
-      <c r="L4" s="79"/>
+      <c r="L4" s="111"/>
       <c r="M4" s="5"/>
-      <c r="N4" s="79"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="80">
-        <v>39</v>
-      </c>
-      <c r="Q4" s="5">
-        <v>17</v>
-      </c>
-      <c r="R4" s="80">
-        <v>38</v>
+      <c r="N4" s="111">
+        <v>57</v>
+      </c>
+      <c r="O4" s="5">
+        <v>19</v>
+      </c>
+      <c r="P4" s="111"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="111">
+        <v>50</v>
       </c>
       <c r="S4" s="5">
+        <v>26</v>
+      </c>
+      <c r="T4" s="111">
+        <v>56</v>
+      </c>
+      <c r="U4" s="5">
+        <v>15</v>
+      </c>
+      <c r="V4" s="111"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="111"/>
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="115">
+        <v>54</v>
+      </c>
+      <c r="AA4" s="73">
         <v>18</v>
       </c>
-      <c r="T4" s="80"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="81">
-        <v>37</v>
-      </c>
-      <c r="W4" s="5">
-        <v>19</v>
-      </c>
-      <c r="X4" s="81">
-        <v>36</v>
-      </c>
-      <c r="Y4" s="5">
-        <v>20</v>
-      </c>
-      <c r="Z4" s="81">
-        <v>38</v>
-      </c>
-      <c r="AA4" s="74">
-        <v>18</v>
-      </c>
-      <c r="AB4" s="80">
+      <c r="AB4" s="115">
+        <v>50</v>
+      </c>
+      <c r="AC4" s="73">
+        <v>22</v>
+      </c>
+      <c r="AD4" s="115"/>
+      <c r="AE4" s="73"/>
+      <c r="AF4" s="115"/>
+      <c r="AG4" s="73"/>
+      <c r="AH4" s="115"/>
+      <c r="AI4" s="73"/>
+      <c r="AJ4" s="60">
+        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4</f>
+        <v>320</v>
+      </c>
+      <c r="AK4" s="6">
+        <f>COUNTIF(D4:AH4,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AL4" s="35"/>
+      <c r="AM4" s="5"/>
+      <c r="AN4" s="36">
+        <f>SUMIF(G4:AI4, "&lt;30")+AL4+AM4</f>
+        <v>123</v>
+      </c>
+      <c r="AO4" s="64">
+        <f>AN4/AK4</f>
+        <v>20.5</v>
+      </c>
+      <c r="AP4" s="76"/>
+      <c r="AQ4" s="36"/>
+      <c r="AR4" s="36"/>
+      <c r="AS4" s="6"/>
+      <c r="AT4" s="54" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:46">
+      <c r="A5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="AC4" s="74">
-        <v>21</v>
-      </c>
-      <c r="AD4" s="61">
-        <f t="shared" ref="AD4:AD22" si="1">F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4</f>
-        <v>223</v>
-      </c>
-      <c r="AE4" s="6">
-        <f t="shared" ref="AE4:AE22" si="2">COUNTIF(D4:AB4,"&gt;30")</f>
-        <v>6</v>
-      </c>
-      <c r="AF4" s="35">
-        <v>3</v>
-      </c>
-      <c r="AG4" s="5">
-        <v>8</v>
-      </c>
-      <c r="AH4" s="36">
-        <f t="shared" ref="AH4:AH22" si="3">SUMIF(G4:AC4, "&lt;30")+AF4+AG4</f>
-        <v>124</v>
-      </c>
-      <c r="AI4" s="65">
-        <f t="shared" ref="AI4:AI22" si="4">AH4/AE4</f>
-        <v>20.666666666666668</v>
-      </c>
-      <c r="AJ4" s="77"/>
-      <c r="AK4" s="36"/>
-      <c r="AL4" s="36"/>
-      <c r="AM4" s="6"/>
-      <c r="AN4" s="54"/>
-    </row>
-    <row r="5" spans="1:40">
-      <c r="A5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>15</v>
-      </c>
       <c r="C5" s="9">
-        <f t="shared" si="0"/>
-        <v>17</v>
+        <f>ROUND((AJ5-(36*AK5))/AK5,0)</f>
+        <v>1</v>
       </c>
       <c r="D5" s="48"/>
       <c r="E5" s="49"/>
-      <c r="F5" s="12">
-        <v>53</v>
-      </c>
-      <c r="G5" s="10">
-        <v>23</v>
-      </c>
+      <c r="F5" s="112"/>
+      <c r="G5" s="10"/>
       <c r="H5" s="48"/>
       <c r="I5" s="49"/>
-      <c r="J5" s="12"/>
+      <c r="J5" s="112"/>
       <c r="K5" s="10"/>
-      <c r="L5" s="12"/>
+      <c r="L5" s="112"/>
       <c r="M5" s="10"/>
-      <c r="N5" s="12">
-        <v>57</v>
-      </c>
-      <c r="O5" s="10">
+      <c r="N5" s="112"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="113">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="10">
+        <v>17</v>
+      </c>
+      <c r="R5" s="113">
+        <v>38</v>
+      </c>
+      <c r="S5" s="10">
+        <v>18</v>
+      </c>
+      <c r="T5" s="113"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="114">
+        <v>37</v>
+      </c>
+      <c r="W5" s="10">
         <v>19</v>
       </c>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="12">
-        <v>50</v>
-      </c>
-      <c r="S5" s="10">
-        <v>26</v>
-      </c>
-      <c r="T5" s="12">
-        <v>56</v>
-      </c>
-      <c r="U5" s="10">
-        <v>15</v>
-      </c>
-      <c r="V5" s="12"/>
-      <c r="W5" s="10"/>
-      <c r="X5" s="12"/>
-      <c r="Y5" s="10"/>
-      <c r="Z5" s="69">
-        <v>54</v>
-      </c>
-      <c r="AA5" s="75">
+      <c r="X5" s="114">
+        <v>36</v>
+      </c>
+      <c r="Y5" s="10">
+        <v>20</v>
+      </c>
+      <c r="Z5" s="114">
+        <v>38</v>
+      </c>
+      <c r="AA5" s="74">
         <v>18</v>
       </c>
-      <c r="AB5" s="69">
-        <v>50</v>
-      </c>
-      <c r="AC5" s="75">
-        <v>22</v>
-      </c>
-      <c r="AD5" s="62">
-        <f t="shared" si="1"/>
-        <v>320</v>
-      </c>
-      <c r="AE5" s="11">
-        <f t="shared" si="2"/>
+      <c r="AB5" s="113">
+        <v>35</v>
+      </c>
+      <c r="AC5" s="74">
+        <v>21</v>
+      </c>
+      <c r="AD5" s="113">
+        <v>37</v>
+      </c>
+      <c r="AE5" s="74">
+        <v>19</v>
+      </c>
+      <c r="AF5" s="113">
+        <v>37</v>
+      </c>
+      <c r="AG5" s="74">
+        <v>18</v>
+      </c>
+      <c r="AH5" s="113">
+        <v>38</v>
+      </c>
+      <c r="AI5" s="74">
+        <v>17</v>
+      </c>
+      <c r="AJ5" s="61">
+        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5+AD5+AF5+AH5</f>
+        <v>335</v>
+      </c>
+      <c r="AK5" s="11">
+        <f>COUNTIF(D5:AH5,"&gt;30")</f>
+        <v>9</v>
+      </c>
+      <c r="AL5" s="37">
+        <v>3</v>
+      </c>
+      <c r="AM5" s="10">
+        <v>11</v>
+      </c>
+      <c r="AN5" s="38">
+        <f>SUMIF(G5:AI5, "&lt;30")+AL5+AM5</f>
+        <v>181</v>
+      </c>
+      <c r="AO5" s="65">
+        <f>AN5/AK5</f>
+        <v>20.111111111111111</v>
+      </c>
+      <c r="AP5" s="55"/>
+      <c r="AQ5" s="38"/>
+      <c r="AR5" s="38"/>
+      <c r="AS5" s="11"/>
+      <c r="AT5" s="56"/>
+    </row>
+    <row r="6" spans="1:46">
+      <c r="A6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="9">
+        <f>ROUND((AJ6-(36*AK6))/AK6,0)</f>
         <v>6</v>
-      </c>
-      <c r="AF5" s="37"/>
-      <c r="AG5" s="10"/>
-      <c r="AH5" s="38">
-        <f t="shared" si="3"/>
-        <v>123</v>
-      </c>
-      <c r="AI5" s="66">
-        <f t="shared" si="4"/>
-        <v>20.5</v>
-      </c>
-      <c r="AJ5" s="55"/>
-      <c r="AK5" s="38"/>
-      <c r="AL5" s="38"/>
-      <c r="AM5" s="11"/>
-      <c r="AN5" s="56" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:40">
-      <c r="A6" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="9">
-        <f t="shared" si="0"/>
-        <v>11</v>
       </c>
       <c r="D6" s="48"/>
       <c r="E6" s="49"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="10"/>
+      <c r="F6" s="63">
+        <v>45</v>
+      </c>
+      <c r="G6" s="10">
+        <v>17</v>
+      </c>
       <c r="H6" s="48"/>
       <c r="I6" s="49"/>
-      <c r="J6" s="12"/>
+      <c r="J6" s="63"/>
       <c r="K6" s="10"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="12">
+      <c r="L6" s="63">
         <v>43</v>
       </c>
+      <c r="M6" s="10">
+        <v>19</v>
+      </c>
+      <c r="N6" s="13">
+        <v>41</v>
+      </c>
+      <c r="O6" s="10">
+        <v>21</v>
+      </c>
+      <c r="P6" s="39">
+        <v>47</v>
+      </c>
       <c r="Q6" s="10">
-        <v>26</v>
-      </c>
-      <c r="R6" s="68">
-        <v>45</v>
+        <v>15</v>
+      </c>
+      <c r="R6" s="39">
+        <v>42</v>
       </c>
       <c r="S6" s="10">
-        <v>24</v>
-      </c>
-      <c r="T6" s="69"/>
-      <c r="U6" s="10"/>
-      <c r="V6" s="69">
-        <v>50</v>
+        <v>20</v>
+      </c>
+      <c r="T6" s="39">
+        <v>43</v>
+      </c>
+      <c r="U6" s="10">
+        <v>19</v>
+      </c>
+      <c r="V6" s="39">
+        <v>44</v>
       </c>
       <c r="W6" s="10">
-        <v>19</v>
-      </c>
-      <c r="X6" s="69">
-        <v>44</v>
+        <v>18</v>
+      </c>
+      <c r="X6" s="39">
+        <v>48</v>
       </c>
       <c r="Y6" s="10">
+        <v>16</v>
+      </c>
+      <c r="Z6" s="39">
+        <v>40</v>
+      </c>
+      <c r="AA6" s="74">
+        <v>22</v>
+      </c>
+      <c r="AB6" s="39">
+        <v>40</v>
+      </c>
+      <c r="AC6" s="74">
+        <v>22</v>
+      </c>
+      <c r="AD6" s="39">
+        <v>38</v>
+      </c>
+      <c r="AE6" s="74">
+        <v>23</v>
+      </c>
+      <c r="AF6" s="77">
+        <v>41</v>
+      </c>
+      <c r="AG6" s="74">
         <v>20</v>
       </c>
-      <c r="Z6" s="69"/>
-      <c r="AA6" s="75"/>
-      <c r="AB6" s="69">
-        <v>54</v>
-      </c>
-      <c r="AC6" s="75">
-        <v>11</v>
-      </c>
-      <c r="AD6" s="62">
-        <f t="shared" si="1"/>
-        <v>236</v>
-      </c>
-      <c r="AE6" s="11">
-        <f t="shared" si="2"/>
+      <c r="AH6" s="68">
+        <v>40</v>
+      </c>
+      <c r="AI6" s="74">
+        <v>21</v>
+      </c>
+      <c r="AJ6" s="61">
+        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6+AD6+AF6+AH6</f>
+        <v>552</v>
+      </c>
+      <c r="AK6" s="11">
+        <f>COUNTIF(D6:AH6,"&gt;30")</f>
+        <v>13</v>
+      </c>
+      <c r="AL6" s="37">
+        <v>2</v>
+      </c>
+      <c r="AM6" s="10">
         <v>5</v>
       </c>
-      <c r="AF6" s="37">
-        <v>1</v>
-      </c>
-      <c r="AG6" s="10">
-        <v>1</v>
-      </c>
-      <c r="AH6" s="38">
-        <f t="shared" si="3"/>
-        <v>102</v>
-      </c>
-      <c r="AI6" s="66">
-        <f t="shared" si="4"/>
-        <v>20.399999999999999</v>
-      </c>
-      <c r="AJ6" s="58"/>
-      <c r="AK6" s="38"/>
-      <c r="AL6" s="38"/>
-      <c r="AM6" s="11"/>
-      <c r="AN6" s="56"/>
+      <c r="AN6" s="38">
+        <f>SUMIF(G6:AI6, "&lt;30")+AL6+AM6</f>
+        <v>260</v>
+      </c>
+      <c r="AO6" s="65">
+        <f>AN6/AK6</f>
+        <v>20</v>
+      </c>
+      <c r="AP6" s="55"/>
+      <c r="AQ6" s="38"/>
+      <c r="AR6" s="38"/>
+      <c r="AS6" s="11"/>
+      <c r="AT6" s="56"/>
     </row>
-    <row r="7" spans="1:40">
+    <row r="7" spans="1:46">
       <c r="A7" s="7" t="s">
         <v>39</v>
       </c>
@@ -2197,580 +2321,662 @@
         <v>40</v>
       </c>
       <c r="C7" s="9">
-        <f t="shared" si="0"/>
+        <f>ROUND((AJ7-(36*AK7))/AK7,0)</f>
         <v>12</v>
       </c>
       <c r="D7" s="48"/>
       <c r="E7" s="49"/>
-      <c r="F7" s="71"/>
+      <c r="F7" s="70"/>
       <c r="G7" s="10"/>
       <c r="H7" s="48"/>
       <c r="I7" s="49"/>
-      <c r="J7" s="71">
+      <c r="J7" s="70">
         <v>52</v>
       </c>
       <c r="K7" s="10">
         <v>17</v>
       </c>
-      <c r="L7" s="71"/>
+      <c r="L7" s="70"/>
       <c r="M7" s="10"/>
-      <c r="N7" s="71">
+      <c r="N7" s="70">
         <v>46</v>
       </c>
       <c r="O7" s="10">
         <v>23</v>
       </c>
-      <c r="P7" s="71">
+      <c r="P7" s="70">
         <v>46</v>
       </c>
       <c r="Q7" s="10">
         <v>23</v>
       </c>
-      <c r="R7" s="71">
+      <c r="R7" s="70">
         <v>54</v>
       </c>
       <c r="S7" s="10">
         <v>16</v>
       </c>
-      <c r="T7" s="71">
+      <c r="T7" s="70">
         <v>45</v>
       </c>
       <c r="U7" s="10">
         <v>23</v>
       </c>
-      <c r="V7" s="71">
+      <c r="V7" s="70">
         <v>48</v>
       </c>
       <c r="W7" s="10">
         <v>19</v>
       </c>
-      <c r="X7" s="71">
+      <c r="X7" s="70">
         <v>49</v>
       </c>
       <c r="Y7" s="10">
         <v>18</v>
       </c>
-      <c r="Z7" s="76"/>
-      <c r="AA7" s="75"/>
-      <c r="AB7" s="76">
+      <c r="Z7" s="75"/>
+      <c r="AA7" s="74"/>
+      <c r="AB7" s="75">
         <v>46</v>
       </c>
-      <c r="AC7" s="75">
+      <c r="AC7" s="74">
         <v>21</v>
       </c>
-      <c r="AD7" s="62">
-        <f t="shared" si="1"/>
-        <v>386</v>
-      </c>
-      <c r="AE7" s="11">
-        <f t="shared" si="2"/>
-        <v>8</v>
-      </c>
-      <c r="AF7" s="37"/>
-      <c r="AG7" s="10">
+      <c r="AD7" s="110">
+        <v>43</v>
+      </c>
+      <c r="AE7" s="74">
+        <v>23</v>
+      </c>
+      <c r="AF7" s="75">
+        <v>47</v>
+      </c>
+      <c r="AG7" s="74">
+        <v>19</v>
+      </c>
+      <c r="AH7" s="75">
+        <v>51</v>
+      </c>
+      <c r="AI7" s="74">
+        <v>15</v>
+      </c>
+      <c r="AJ7" s="61">
+        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7+AD7+AF7+AH7</f>
+        <v>527</v>
+      </c>
+      <c r="AK7" s="11">
+        <f>COUNTIF(D7:AH7,"&gt;30")</f>
+        <v>11</v>
+      </c>
+      <c r="AL7" s="37">
         <v>1</v>
       </c>
-      <c r="AH7" s="38">
-        <f t="shared" si="3"/>
-        <v>161</v>
-      </c>
-      <c r="AI7" s="66">
-        <f t="shared" si="4"/>
-        <v>20.125</v>
-      </c>
-      <c r="AJ7" s="55"/>
-      <c r="AK7" s="38"/>
-      <c r="AL7" s="38"/>
-      <c r="AM7" s="11"/>
-      <c r="AN7" s="56"/>
+      <c r="AM7" s="10">
+        <v>1</v>
+      </c>
+      <c r="AN7" s="38">
+        <f>SUMIF(G7:AI7, "&lt;30")+AL7+AM7</f>
+        <v>219</v>
+      </c>
+      <c r="AO7" s="65">
+        <f>AN7/AK7</f>
+        <v>19.90909090909091</v>
+      </c>
+      <c r="AP7" s="55"/>
+      <c r="AQ7" s="38"/>
+      <c r="AR7" s="38"/>
+      <c r="AS7" s="11"/>
+      <c r="AT7" s="56"/>
     </row>
-    <row r="8" spans="1:40">
+    <row r="8" spans="1:46">
       <c r="A8" s="7" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="C8" s="9">
-        <f t="shared" si="0"/>
-        <v>14</v>
+        <f>ROUND((AJ8-(36*AK8))/AK8,0)</f>
+        <v>7</v>
       </c>
       <c r="D8" s="48"/>
       <c r="E8" s="49"/>
       <c r="F8" s="12">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G8" s="10">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="H8" s="48"/>
       <c r="I8" s="49"/>
       <c r="J8" s="12"/>
       <c r="K8" s="10"/>
-      <c r="L8" s="12">
-        <v>54</v>
-      </c>
-      <c r="M8" s="10">
-        <v>15</v>
-      </c>
-      <c r="N8" s="12"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="12">
-        <v>54</v>
+      <c r="L8" s="12"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="52">
+        <v>48</v>
+      </c>
+      <c r="O8" s="10">
+        <v>14</v>
+      </c>
+      <c r="P8" s="39">
+        <v>44</v>
       </c>
       <c r="Q8" s="10">
+        <v>18</v>
+      </c>
+      <c r="R8" s="39"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="39"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="39"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="13">
+        <v>40</v>
+      </c>
+      <c r="Y8" s="10">
+        <v>22</v>
+      </c>
+      <c r="Z8" s="39">
+        <v>44</v>
+      </c>
+      <c r="AA8" s="74">
+        <v>17</v>
+      </c>
+      <c r="AB8" s="39">
+        <v>46</v>
+      </c>
+      <c r="AC8" s="74">
         <v>16</v>
       </c>
-      <c r="R8" s="12">
-        <v>53</v>
-      </c>
-      <c r="S8" s="10">
-        <v>16</v>
-      </c>
-      <c r="T8" s="12"/>
-      <c r="U8" s="10"/>
-      <c r="V8" s="68">
-        <v>46</v>
-      </c>
-      <c r="W8" s="10">
+      <c r="AD8" s="52">
+        <v>42</v>
+      </c>
+      <c r="AE8" s="74">
+        <v>20</v>
+      </c>
+      <c r="AF8" s="39">
+        <v>44</v>
+      </c>
+      <c r="AG8" s="74">
+        <v>18</v>
+      </c>
+      <c r="AH8" s="52">
+        <v>39</v>
+      </c>
+      <c r="AI8" s="74">
         <v>23</v>
       </c>
-      <c r="X8" s="69">
-        <v>49</v>
-      </c>
-      <c r="Y8" s="10">
-        <v>19</v>
-      </c>
-      <c r="Z8" s="69">
-        <v>50</v>
-      </c>
-      <c r="AA8" s="75">
-        <v>18</v>
-      </c>
-      <c r="AB8" s="69"/>
-      <c r="AC8" s="75"/>
-      <c r="AD8" s="62">
-        <f t="shared" si="1"/>
-        <v>348</v>
-      </c>
-      <c r="AE8" s="11">
-        <f t="shared" si="2"/>
-        <v>7</v>
-      </c>
-      <c r="AF8" s="37">
-        <v>1</v>
-      </c>
-      <c r="AG8" s="10">
-        <v>1</v>
-      </c>
-      <c r="AH8" s="38">
-        <f t="shared" si="3"/>
-        <v>136</v>
-      </c>
-      <c r="AI8" s="66">
-        <f t="shared" si="4"/>
-        <v>19.428571428571427</v>
-      </c>
-      <c r="AJ8" s="57"/>
-      <c r="AK8" s="38"/>
-      <c r="AL8" s="38"/>
-      <c r="AM8" s="11"/>
-      <c r="AN8" s="56"/>
+      <c r="AJ8" s="61">
+        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8+AD8+AF8+AH8</f>
+        <v>388</v>
+      </c>
+      <c r="AK8" s="11">
+        <f>COUNTIF(D8:AH8,"&gt;30")</f>
+        <v>9</v>
+      </c>
+      <c r="AL8" s="37">
+        <v>3</v>
+      </c>
+      <c r="AM8" s="10">
+        <v>3</v>
+      </c>
+      <c r="AN8" s="38">
+        <f>SUMIF(G8:AI8, "&lt;30")+AL8+AM8</f>
+        <v>175</v>
+      </c>
+      <c r="AO8" s="65">
+        <f>AN8/AK8</f>
+        <v>19.444444444444443</v>
+      </c>
+      <c r="AP8" s="117"/>
+      <c r="AQ8" s="38"/>
+      <c r="AR8" s="38"/>
+      <c r="AS8" s="11"/>
+      <c r="AT8" s="56"/>
     </row>
-    <row r="9" spans="1:40">
+    <row r="9" spans="1:46">
       <c r="A9" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C9" s="9">
-        <f t="shared" si="0"/>
-        <v>7</v>
+        <f>ROUND((AJ9-(36*AK9))/AK9,0)</f>
+        <v>11</v>
       </c>
       <c r="D9" s="48"/>
       <c r="E9" s="49"/>
-      <c r="F9" s="64">
-        <v>45</v>
+      <c r="F9" s="69">
+        <v>42</v>
       </c>
       <c r="G9" s="10">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H9" s="48"/>
       <c r="I9" s="49"/>
-      <c r="J9" s="64"/>
+      <c r="J9" s="69"/>
       <c r="K9" s="10"/>
-      <c r="L9" s="64">
-        <v>43</v>
+      <c r="L9" s="39">
+        <v>51</v>
       </c>
       <c r="M9" s="10">
+        <v>16</v>
+      </c>
+      <c r="N9" s="39"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="13">
+        <v>49</v>
+      </c>
+      <c r="Q9" s="10">
+        <v>18</v>
+      </c>
+      <c r="R9" s="39">
+        <v>46</v>
+      </c>
+      <c r="S9" s="10">
+        <v>21</v>
+      </c>
+      <c r="T9" s="39">
+        <v>45</v>
+      </c>
+      <c r="U9" s="10">
+        <v>20</v>
+      </c>
+      <c r="V9" s="39">
+        <v>46</v>
+      </c>
+      <c r="W9" s="10">
         <v>19</v>
       </c>
-      <c r="N9" s="13">
-        <v>41</v>
-      </c>
-      <c r="O9" s="10">
-        <v>21</v>
-      </c>
-      <c r="P9" s="39">
-        <v>47</v>
-      </c>
-      <c r="Q9" s="10">
-        <v>15</v>
-      </c>
-      <c r="R9" s="39">
+      <c r="X9" s="39">
+        <v>53</v>
+      </c>
+      <c r="Y9" s="10">
+        <v>13</v>
+      </c>
+      <c r="Z9" s="39">
+        <v>52</v>
+      </c>
+      <c r="AA9" s="74">
+        <v>13</v>
+      </c>
+      <c r="AB9" s="39">
+        <v>44</v>
+      </c>
+      <c r="AC9" s="74">
+        <v>22</v>
+      </c>
+      <c r="AD9" s="39">
         <v>42</v>
       </c>
-      <c r="S9" s="10">
+      <c r="AE9" s="74">
+        <v>24</v>
+      </c>
+      <c r="AF9" s="39">
+        <v>45</v>
+      </c>
+      <c r="AG9" s="74">
         <v>20</v>
       </c>
-      <c r="T9" s="39">
-        <v>43</v>
-      </c>
-      <c r="U9" s="10">
-        <v>19</v>
-      </c>
-      <c r="V9" s="39">
-        <v>44</v>
-      </c>
-      <c r="W9" s="10">
-        <v>18</v>
-      </c>
-      <c r="X9" s="39">
+      <c r="AH9" s="39">
         <v>48</v>
       </c>
-      <c r="Y9" s="10">
-        <v>16</v>
-      </c>
-      <c r="Z9" s="39">
-        <v>40</v>
-      </c>
-      <c r="AA9" s="75">
-        <v>22</v>
-      </c>
-      <c r="AB9" s="39">
-        <v>40</v>
-      </c>
-      <c r="AC9" s="75">
-        <v>22</v>
-      </c>
-      <c r="AD9" s="62">
-        <f t="shared" si="1"/>
-        <v>433</v>
-      </c>
-      <c r="AE9" s="11">
-        <f t="shared" si="2"/>
-        <v>10</v>
-      </c>
-      <c r="AF9" s="37">
-        <v>1</v>
-      </c>
-      <c r="AG9" s="10">
-        <v>4</v>
-      </c>
-      <c r="AH9" s="38">
-        <f t="shared" si="3"/>
-        <v>194</v>
-      </c>
-      <c r="AI9" s="66">
-        <f t="shared" si="4"/>
-        <v>19.399999999999999</v>
-      </c>
-      <c r="AJ9" s="55"/>
-      <c r="AK9" s="38"/>
-      <c r="AL9" s="38"/>
-      <c r="AM9" s="11"/>
-      <c r="AN9" s="56"/>
+      <c r="AI9" s="74">
+        <v>17</v>
+      </c>
+      <c r="AJ9" s="61">
+        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9+AD9+AF9+AH9</f>
+        <v>563</v>
+      </c>
+      <c r="AK9" s="11">
+        <f>COUNTIF(D9:AH9,"&gt;30")</f>
+        <v>12</v>
+      </c>
+      <c r="AL9" s="37">
+        <v>2</v>
+      </c>
+      <c r="AM9" s="10">
+        <v>2</v>
+      </c>
+      <c r="AN9" s="38">
+        <f>SUMIF(G9:AI9, "&lt;30")+AL9+AM9</f>
+        <v>232</v>
+      </c>
+      <c r="AO9" s="65">
+        <f>AN9/AK9</f>
+        <v>19.333333333333332</v>
+      </c>
+      <c r="AP9" s="55"/>
+      <c r="AQ9" s="38"/>
+      <c r="AR9" s="38"/>
+      <c r="AS9" s="11"/>
+      <c r="AT9" s="56"/>
     </row>
-    <row r="10" spans="1:40">
+    <row r="10" spans="1:46">
       <c r="A10" s="7" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C10" s="9">
-        <f t="shared" si="0"/>
+        <f>ROUND((AJ10-(36*AK10))/AK10,0)</f>
         <v>12</v>
       </c>
       <c r="D10" s="48"/>
       <c r="E10" s="49"/>
-      <c r="F10" s="70">
-        <v>42</v>
-      </c>
-      <c r="G10" s="10">
-        <v>25</v>
-      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="10"/>
       <c r="H10" s="48"/>
       <c r="I10" s="49"/>
-      <c r="J10" s="70"/>
+      <c r="J10" s="12"/>
       <c r="K10" s="10"/>
-      <c r="L10" s="39">
-        <v>51</v>
-      </c>
-      <c r="M10" s="10">
-        <v>16</v>
-      </c>
-      <c r="N10" s="39"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="12"/>
       <c r="O10" s="10"/>
-      <c r="P10" s="13">
-        <v>49</v>
+      <c r="P10" s="12">
+        <v>43</v>
       </c>
       <c r="Q10" s="10">
-        <v>18</v>
-      </c>
-      <c r="R10" s="39">
-        <v>46</v>
+        <v>26</v>
+      </c>
+      <c r="R10" s="67">
+        <v>45</v>
       </c>
       <c r="S10" s="10">
-        <v>21</v>
-      </c>
-      <c r="T10" s="39">
-        <v>45</v>
-      </c>
-      <c r="U10" s="10">
-        <v>20</v>
-      </c>
-      <c r="V10" s="39">
-        <v>46</v>
+        <v>24</v>
+      </c>
+      <c r="T10" s="68"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="68">
+        <v>50</v>
       </c>
       <c r="W10" s="10">
         <v>19</v>
       </c>
-      <c r="X10" s="39">
-        <v>53</v>
+      <c r="X10" s="68">
+        <v>44</v>
       </c>
       <c r="Y10" s="10">
-        <v>13</v>
-      </c>
-      <c r="Z10" s="39">
-        <v>52</v>
-      </c>
-      <c r="AA10" s="75">
-        <v>13</v>
-      </c>
-      <c r="AB10" s="39">
-        <v>44</v>
-      </c>
-      <c r="AC10" s="75">
-        <v>22</v>
-      </c>
-      <c r="AD10" s="62">
-        <f t="shared" si="1"/>
-        <v>428</v>
-      </c>
-      <c r="AE10" s="11">
-        <f t="shared" si="2"/>
-        <v>9</v>
-      </c>
-      <c r="AF10" s="37">
-        <v>2</v>
-      </c>
-      <c r="AG10" s="10">
+        <v>20</v>
+      </c>
+      <c r="Z10" s="68"/>
+      <c r="AA10" s="74"/>
+      <c r="AB10" s="68">
+        <v>54</v>
+      </c>
+      <c r="AC10" s="74">
+        <v>11</v>
+      </c>
+      <c r="AD10" s="68"/>
+      <c r="AE10" s="74"/>
+      <c r="AF10" s="68">
+        <v>51</v>
+      </c>
+      <c r="AG10" s="74">
+        <v>14</v>
+      </c>
+      <c r="AH10" s="68"/>
+      <c r="AI10" s="74"/>
+      <c r="AJ10" s="61">
+        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10+AD10+AF10+AH10</f>
+        <v>287</v>
+      </c>
+      <c r="AK10" s="11">
+        <f>COUNTIF(D10:AH10,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AL10" s="37">
         <v>1</v>
       </c>
-      <c r="AH10" s="38">
-        <f t="shared" si="3"/>
-        <v>170</v>
-      </c>
-      <c r="AI10" s="66">
-        <f t="shared" si="4"/>
-        <v>18.888888888888889</v>
-      </c>
-      <c r="AJ10" s="82"/>
-      <c r="AK10" s="38"/>
-      <c r="AL10" s="38"/>
-      <c r="AM10" s="11"/>
-      <c r="AN10" s="56"/>
+      <c r="AM10" s="10">
+        <v>1</v>
+      </c>
+      <c r="AN10" s="38">
+        <f>SUMIF(G10:AI10, "&lt;30")+AL10+AM10</f>
+        <v>116</v>
+      </c>
+      <c r="AO10" s="65">
+        <f>AN10/AK10</f>
+        <v>19.333333333333332</v>
+      </c>
+      <c r="AP10" s="116"/>
+      <c r="AQ10" s="38"/>
+      <c r="AR10" s="38"/>
+      <c r="AS10" s="11"/>
+      <c r="AT10" s="56"/>
     </row>
-    <row r="11" spans="1:40">
+    <row r="11" spans="1:46">
       <c r="A11" s="7" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C11" s="9">
-        <f t="shared" si="0"/>
-        <v>12</v>
+        <f>ROUND((AJ11-(36*AK11))/AK11,0)</f>
+        <v>14</v>
       </c>
       <c r="D11" s="48"/>
       <c r="E11" s="49"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="10"/>
+      <c r="F11" s="12">
+        <v>42</v>
+      </c>
+      <c r="G11" s="10">
+        <v>27</v>
+      </c>
       <c r="H11" s="48"/>
       <c r="I11" s="49"/>
-      <c r="J11" s="14"/>
+      <c r="J11" s="12"/>
       <c r="K11" s="10"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="14"/>
+      <c r="L11" s="12">
+        <v>54</v>
+      </c>
+      <c r="M11" s="10">
+        <v>15</v>
+      </c>
+      <c r="N11" s="12"/>
       <c r="O11" s="10"/>
-      <c r="P11" s="39">
-        <v>47</v>
+      <c r="P11" s="12">
+        <v>54</v>
       </c>
       <c r="Q11" s="10">
-        <v>20</v>
-      </c>
-      <c r="R11" s="39">
+        <v>16</v>
+      </c>
+      <c r="R11" s="12">
+        <v>53</v>
+      </c>
+      <c r="S11" s="10">
+        <v>16</v>
+      </c>
+      <c r="T11" s="12"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="67">
+        <v>46</v>
+      </c>
+      <c r="W11" s="10">
+        <v>23</v>
+      </c>
+      <c r="X11" s="68">
+        <v>49</v>
+      </c>
+      <c r="Y11" s="10">
+        <v>19</v>
+      </c>
+      <c r="Z11" s="68">
         <v>50</v>
       </c>
-      <c r="S11" s="10">
-        <v>17</v>
-      </c>
-      <c r="T11" s="39">
-        <v>46</v>
-      </c>
-      <c r="U11" s="10">
-        <v>21</v>
-      </c>
-      <c r="V11" s="39">
-        <v>47</v>
-      </c>
-      <c r="W11" s="10">
-        <v>19</v>
-      </c>
-      <c r="X11" s="39">
-        <v>44</v>
-      </c>
-      <c r="Y11" s="10">
-        <v>22</v>
-      </c>
-      <c r="Z11" s="39">
-        <v>52</v>
-      </c>
-      <c r="AA11" s="75">
-        <v>14</v>
-      </c>
-      <c r="AB11" s="39">
-        <v>47</v>
-      </c>
-      <c r="AC11" s="75">
-        <v>19</v>
-      </c>
-      <c r="AD11" s="62">
-        <f t="shared" si="1"/>
-        <v>333</v>
-      </c>
-      <c r="AE11" s="11">
-        <f t="shared" si="2"/>
-        <v>7</v>
-      </c>
-      <c r="AF11" s="37"/>
-      <c r="AG11" s="10"/>
-      <c r="AH11" s="38">
-        <f t="shared" si="3"/>
-        <v>132</v>
-      </c>
-      <c r="AI11" s="66">
-        <f t="shared" si="4"/>
-        <v>18.857142857142858</v>
-      </c>
-      <c r="AJ11" s="55"/>
-      <c r="AK11" s="38"/>
-      <c r="AL11" s="38"/>
-      <c r="AM11" s="11"/>
-      <c r="AN11" s="56"/>
+      <c r="AA11" s="74">
+        <v>18</v>
+      </c>
+      <c r="AB11" s="68"/>
+      <c r="AC11" s="74"/>
+      <c r="AD11" s="68"/>
+      <c r="AE11" s="74"/>
+      <c r="AF11" s="68"/>
+      <c r="AG11" s="74"/>
+      <c r="AH11" s="68">
+        <v>50</v>
+      </c>
+      <c r="AI11" s="74">
+        <v>18</v>
+      </c>
+      <c r="AJ11" s="61">
+        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11+AD11+AF11+AH11</f>
+        <v>398</v>
+      </c>
+      <c r="AK11" s="11">
+        <f>COUNTIF(D11:AH11,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AL11" s="37">
+        <v>1</v>
+      </c>
+      <c r="AM11" s="10">
+        <v>1</v>
+      </c>
+      <c r="AN11" s="38">
+        <f>SUMIF(G11:AI11, "&lt;30")+AL11+AM11</f>
+        <v>154</v>
+      </c>
+      <c r="AO11" s="65">
+        <f>AN11/AK11</f>
+        <v>19.25</v>
+      </c>
+      <c r="AP11" s="55"/>
+      <c r="AQ11" s="38"/>
+      <c r="AR11" s="38"/>
+      <c r="AS11" s="11"/>
+      <c r="AT11" s="56"/>
     </row>
-    <row r="12" spans="1:40">
+    <row r="12" spans="1:46">
       <c r="A12" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C12" s="9">
-        <f t="shared" si="0"/>
-        <v>15</v>
+        <f>ROUND((AJ12-(36*AK12))/AK12,0)</f>
+        <v>12</v>
       </c>
       <c r="D12" s="48"/>
       <c r="E12" s="49"/>
-      <c r="F12" s="12">
-        <v>51</v>
-      </c>
-      <c r="G12" s="10">
-        <v>18</v>
-      </c>
+      <c r="F12" s="14"/>
+      <c r="G12" s="10"/>
       <c r="H12" s="48"/>
       <c r="I12" s="49"/>
-      <c r="J12" s="12"/>
+      <c r="J12" s="14"/>
       <c r="K12" s="10"/>
-      <c r="L12" s="12"/>
+      <c r="L12" s="14"/>
       <c r="M12" s="10"/>
-      <c r="N12" s="12">
+      <c r="N12" s="14"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="39">
+        <v>47</v>
+      </c>
+      <c r="Q12" s="10">
+        <v>20</v>
+      </c>
+      <c r="R12" s="39">
+        <v>50</v>
+      </c>
+      <c r="S12" s="10">
+        <v>17</v>
+      </c>
+      <c r="T12" s="39">
+        <v>46</v>
+      </c>
+      <c r="U12" s="10">
+        <v>21</v>
+      </c>
+      <c r="V12" s="39">
+        <v>47</v>
+      </c>
+      <c r="W12" s="10">
+        <v>19</v>
+      </c>
+      <c r="X12" s="39">
+        <v>44</v>
+      </c>
+      <c r="Y12" s="10">
+        <v>22</v>
+      </c>
+      <c r="Z12" s="39">
+        <v>52</v>
+      </c>
+      <c r="AA12" s="74">
+        <v>14</v>
+      </c>
+      <c r="AB12" s="39">
+        <v>47</v>
+      </c>
+      <c r="AC12" s="74">
+        <v>19</v>
+      </c>
+      <c r="AD12" s="39">
         <v>51</v>
       </c>
-      <c r="O12" s="10">
-        <v>18</v>
-      </c>
-      <c r="P12" s="12">
-        <v>52</v>
-      </c>
-      <c r="Q12" s="10">
+      <c r="AE12" s="74">
+        <v>15</v>
+      </c>
+      <c r="AF12" s="39">
+        <v>49</v>
+      </c>
+      <c r="AG12" s="74">
         <v>17</v>
       </c>
-      <c r="R12" s="12"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="12"/>
-      <c r="U12" s="10"/>
-      <c r="V12" s="12"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="12">
-        <v>48</v>
-      </c>
-      <c r="Y12" s="10">
-        <v>21</v>
-      </c>
-      <c r="Z12" s="69"/>
-      <c r="AA12" s="75"/>
-      <c r="AB12" s="69">
-        <v>51</v>
-      </c>
-      <c r="AC12" s="75">
-        <v>18</v>
-      </c>
-      <c r="AD12" s="62">
-        <f t="shared" si="1"/>
-        <v>253</v>
-      </c>
-      <c r="AE12" s="11">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="AF12" s="37"/>
-      <c r="AG12" s="10"/>
-      <c r="AH12" s="38">
-        <f t="shared" si="3"/>
-        <v>92</v>
-      </c>
-      <c r="AI12" s="66">
-        <f t="shared" si="4"/>
+      <c r="AH12" s="39">
+        <v>46</v>
+      </c>
+      <c r="AI12" s="74">
+        <v>20</v>
+      </c>
+      <c r="AJ12" s="61">
+        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12+AD12+AF12+AH12</f>
+        <v>479</v>
+      </c>
+      <c r="AK12" s="11">
+        <f>COUNTIF(D12:AH12,"&gt;30")</f>
+        <v>10</v>
+      </c>
+      <c r="AL12" s="37"/>
+      <c r="AM12" s="10"/>
+      <c r="AN12" s="38">
+        <f>SUMIF(G12:AI12, "&lt;30")+AL12+AM12</f>
+        <v>184</v>
+      </c>
+      <c r="AO12" s="65">
+        <f>AN12/AK12</f>
         <v>18.399999999999999</v>
       </c>
-      <c r="AJ12" s="58"/>
-      <c r="AK12" s="38"/>
-      <c r="AL12" s="38"/>
-      <c r="AM12" s="11"/>
-      <c r="AN12" s="56"/>
+      <c r="AP12" s="55"/>
+      <c r="AQ12" s="38"/>
+      <c r="AR12" s="38"/>
+      <c r="AS12" s="11"/>
+      <c r="AT12" s="56"/>
     </row>
-    <row r="13" spans="1:40">
+    <row r="13" spans="1:46">
       <c r="A13" s="7" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C13" s="9">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>ROUND((AJ13-(36*AK13))/AK13,0)</f>
+        <v>15</v>
       </c>
       <c r="D13" s="48"/>
       <c r="E13" s="49"/>
       <c r="F13" s="12">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="G13" s="10">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H13" s="48"/>
       <c r="I13" s="49"/>
@@ -2778,71 +2984,69 @@
       <c r="K13" s="10"/>
       <c r="L13" s="12"/>
       <c r="M13" s="10"/>
-      <c r="N13" s="52">
+      <c r="N13" s="12">
+        <v>51</v>
+      </c>
+      <c r="O13" s="10">
+        <v>18</v>
+      </c>
+      <c r="P13" s="12">
+        <v>52</v>
+      </c>
+      <c r="Q13" s="10">
+        <v>17</v>
+      </c>
+      <c r="R13" s="12"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="12"/>
+      <c r="W13" s="10"/>
+      <c r="X13" s="12">
         <v>48</v>
       </c>
-      <c r="O13" s="10">
-        <v>14</v>
-      </c>
-      <c r="P13" s="39">
-        <v>44</v>
-      </c>
-      <c r="Q13" s="10">
+      <c r="Y13" s="10">
+        <v>21</v>
+      </c>
+      <c r="Z13" s="68"/>
+      <c r="AA13" s="74"/>
+      <c r="AB13" s="68">
+        <v>51</v>
+      </c>
+      <c r="AC13" s="74">
         <v>18</v>
       </c>
-      <c r="R13" s="39"/>
-      <c r="S13" s="10"/>
-      <c r="T13" s="39"/>
-      <c r="U13" s="10"/>
-      <c r="V13" s="39"/>
-      <c r="W13" s="10"/>
-      <c r="X13" s="13">
-        <v>40</v>
-      </c>
-      <c r="Y13" s="10">
-        <v>22</v>
-      </c>
-      <c r="Z13" s="39">
-        <v>44</v>
-      </c>
-      <c r="AA13" s="75">
-        <v>17</v>
-      </c>
-      <c r="AB13" s="39">
-        <v>46</v>
-      </c>
-      <c r="AC13" s="75">
-        <v>16</v>
-      </c>
-      <c r="AD13" s="62">
-        <f t="shared" si="1"/>
-        <v>263</v>
-      </c>
-      <c r="AE13" s="11">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="AF13" s="37">
-        <v>1</v>
-      </c>
-      <c r="AG13" s="10">
-        <v>1</v>
-      </c>
-      <c r="AH13" s="38">
-        <f t="shared" si="3"/>
-        <v>110</v>
-      </c>
-      <c r="AI13" s="66">
-        <f t="shared" si="4"/>
-        <v>18.333333333333332</v>
-      </c>
-      <c r="AJ13" s="58"/>
-      <c r="AK13" s="38"/>
-      <c r="AL13" s="38"/>
-      <c r="AM13" s="11"/>
-      <c r="AN13" s="56"/>
+      <c r="AD13" s="68"/>
+      <c r="AE13" s="74"/>
+      <c r="AF13" s="68"/>
+      <c r="AG13" s="74"/>
+      <c r="AH13" s="68"/>
+      <c r="AI13" s="74"/>
+      <c r="AJ13" s="61">
+        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13+AD13+AF13+AH13</f>
+        <v>253</v>
+      </c>
+      <c r="AK13" s="11">
+        <f>COUNTIF(D13:AH13,"&gt;30")</f>
+        <v>5</v>
+      </c>
+      <c r="AL13" s="37"/>
+      <c r="AM13" s="10"/>
+      <c r="AN13" s="38">
+        <f>SUMIF(G13:AI13, "&lt;30")+AL13+AM13</f>
+        <v>92</v>
+      </c>
+      <c r="AO13" s="65">
+        <f>AN13/AK13</f>
+        <v>18.399999999999999</v>
+      </c>
+      <c r="AP13" s="57"/>
+      <c r="AQ13" s="38"/>
+      <c r="AR13" s="38"/>
+      <c r="AS13" s="11"/>
+      <c r="AT13" s="56"/>
     </row>
-    <row r="14" spans="1:40">
+    <row r="14" spans="1:46">
       <c r="A14" s="7" t="s">
         <v>17</v>
       </c>
@@ -2850,7 +3054,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="9">
-        <f t="shared" si="0"/>
+        <f>ROUND((AJ14-(36*AK14))/AK14,0)</f>
         <v>22</v>
       </c>
       <c r="D14" s="48"/>
@@ -2887,138 +3091,156 @@
       </c>
       <c r="X14" s="12"/>
       <c r="Y14" s="10"/>
-      <c r="Z14" s="69"/>
-      <c r="AA14" s="75"/>
-      <c r="AB14" s="69"/>
-      <c r="AC14" s="75"/>
-      <c r="AD14" s="62">
-        <f t="shared" si="1"/>
+      <c r="Z14" s="68"/>
+      <c r="AA14" s="74"/>
+      <c r="AB14" s="68"/>
+      <c r="AC14" s="74"/>
+      <c r="AD14" s="68"/>
+      <c r="AE14" s="74"/>
+      <c r="AF14" s="68"/>
+      <c r="AG14" s="74"/>
+      <c r="AH14" s="68"/>
+      <c r="AI14" s="74"/>
+      <c r="AJ14" s="61">
+        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14+AD14+AF14+AH14</f>
         <v>173</v>
       </c>
-      <c r="AE14" s="11">
-        <f t="shared" si="2"/>
+      <c r="AK14" s="11">
+        <f>COUNTIF(D14:AH14,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="AF14" s="37"/>
-      <c r="AG14" s="10"/>
-      <c r="AH14" s="38">
-        <f t="shared" si="3"/>
+      <c r="AL14" s="37"/>
+      <c r="AM14" s="10"/>
+      <c r="AN14" s="38">
+        <f>SUMIF(G14:AI14, "&lt;30")+AL14+AM14</f>
         <v>55</v>
       </c>
-      <c r="AI14" s="66">
-        <f t="shared" si="4"/>
+      <c r="AO14" s="65">
+        <f>AN14/AK14</f>
         <v>18.333333333333332</v>
       </c>
-      <c r="AJ14" s="58"/>
-      <c r="AK14" s="38"/>
-      <c r="AL14" s="38"/>
-      <c r="AM14" s="11"/>
-      <c r="AN14" s="56"/>
+      <c r="AP14" s="57"/>
+      <c r="AQ14" s="38"/>
+      <c r="AR14" s="38"/>
+      <c r="AS14" s="11"/>
+      <c r="AT14" s="56"/>
     </row>
-    <row r="15" spans="1:40">
+    <row r="15" spans="1:46">
       <c r="A15" s="7" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C15" s="9">
-        <f>ROUND((AD15-(36*AE15))/AE15,0)</f>
-        <v>9</v>
+        <f>ROUND((AJ15-(36*AK15))/AK15,0)</f>
+        <v>13</v>
       </c>
       <c r="D15" s="48"/>
       <c r="E15" s="49"/>
-      <c r="F15" s="12">
-        <v>46</v>
-      </c>
-      <c r="G15" s="10">
-        <v>16</v>
-      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="10"/>
       <c r="H15" s="48"/>
       <c r="I15" s="49"/>
       <c r="J15" s="12"/>
       <c r="K15" s="10"/>
       <c r="L15" s="12"/>
       <c r="M15" s="10"/>
-      <c r="N15" s="12">
-        <v>42</v>
-      </c>
-      <c r="O15" s="10">
-        <v>20</v>
-      </c>
+      <c r="N15" s="12"/>
+      <c r="O15" s="10"/>
       <c r="P15" s="12">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="Q15" s="10">
-        <v>19</v>
-      </c>
-      <c r="R15" s="12"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="10"/>
+        <v>18</v>
+      </c>
+      <c r="R15" s="12">
+        <v>51</v>
+      </c>
+      <c r="S15" s="10">
+        <v>14</v>
+      </c>
+      <c r="T15" s="12">
+        <v>51</v>
+      </c>
+      <c r="U15" s="10">
+        <v>14</v>
+      </c>
       <c r="V15" s="12"/>
       <c r="W15" s="10"/>
       <c r="X15" s="12">
+        <v>48</v>
+      </c>
+      <c r="Y15" s="10">
+        <v>20</v>
+      </c>
+      <c r="Z15" s="12">
+        <v>50</v>
+      </c>
+      <c r="AA15" s="10">
+        <v>18</v>
+      </c>
+      <c r="AB15" s="68">
         <v>47</v>
       </c>
-      <c r="Y15" s="10">
-        <v>16</v>
-      </c>
-      <c r="Z15" s="68">
-        <v>41</v>
-      </c>
-      <c r="AA15" s="75">
-        <v>22</v>
-      </c>
-      <c r="AB15" s="78">
-        <v>50</v>
-      </c>
-      <c r="AC15" s="75">
-        <v>13</v>
-      </c>
-      <c r="AD15" s="62">
-        <f t="shared" si="1"/>
-        <v>269</v>
-      </c>
-      <c r="AE15" s="11">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="AF15" s="37">
-        <v>2</v>
-      </c>
-      <c r="AG15" s="10">
+      <c r="AC15" s="74">
+        <v>21</v>
+      </c>
+      <c r="AD15" s="68"/>
+      <c r="AE15" s="74"/>
+      <c r="AF15" s="68">
+        <v>46</v>
+      </c>
+      <c r="AG15" s="74">
+        <v>21</v>
+      </c>
+      <c r="AH15" s="68">
+        <v>48</v>
+      </c>
+      <c r="AI15" s="74">
+        <v>19</v>
+      </c>
+      <c r="AJ15" s="61">
+        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15+AD15+AF15+AH15</f>
+        <v>389</v>
+      </c>
+      <c r="AK15" s="11">
+        <f>COUNTIF(D15:AH15,"&gt;30")</f>
+        <v>8</v>
+      </c>
+      <c r="AL15" s="37"/>
+      <c r="AM15" s="10">
         <v>1</v>
       </c>
-      <c r="AH15" s="38">
-        <f t="shared" si="3"/>
-        <v>109</v>
-      </c>
-      <c r="AI15" s="66">
-        <f t="shared" si="4"/>
-        <v>18.166666666666668</v>
-      </c>
-      <c r="AJ15" s="58"/>
-      <c r="AK15" s="38"/>
-      <c r="AL15" s="38"/>
-      <c r="AM15" s="11"/>
-      <c r="AN15" s="56"/>
+      <c r="AN15" s="38">
+        <f>SUMIF(G15:AI15, "&lt;30")+AL15+AM15</f>
+        <v>146</v>
+      </c>
+      <c r="AO15" s="65">
+        <f>AN15/AK15</f>
+        <v>18.25</v>
+      </c>
+      <c r="AP15" s="55"/>
+      <c r="AQ15" s="38"/>
+      <c r="AR15" s="38"/>
+      <c r="AS15" s="11"/>
+      <c r="AT15" s="56"/>
     </row>
-    <row r="16" spans="1:40">
+    <row r="16" spans="1:46">
       <c r="A16" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C16" s="9">
-        <f>ROUND((AD16-(36*AE16))/AE16,0)</f>
-        <v>18</v>
+        <f>ROUND((AJ16-(36*AK16))/AK16,0)</f>
+        <v>9</v>
       </c>
       <c r="D16" s="48"/>
       <c r="E16" s="49"/>
       <c r="F16" s="12">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="G16" s="10">
         <v>16</v>
@@ -3027,332 +3249,406 @@
       <c r="I16" s="49"/>
       <c r="J16" s="12"/>
       <c r="K16" s="10"/>
-      <c r="L16" s="12">
-        <v>56</v>
-      </c>
-      <c r="M16" s="10">
-        <v>15</v>
-      </c>
+      <c r="L16" s="12"/>
+      <c r="M16" s="10"/>
       <c r="N16" s="12">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="O16" s="10">
-        <v>14</v>
-      </c>
-      <c r="P16" s="12"/>
-      <c r="Q16" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="P16" s="12">
+        <v>43</v>
+      </c>
+      <c r="Q16" s="10">
+        <v>19</v>
+      </c>
       <c r="R16" s="12"/>
       <c r="S16" s="10"/>
-      <c r="T16" s="68">
+      <c r="T16" s="12"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="12"/>
+      <c r="W16" s="10"/>
+      <c r="X16" s="12">
+        <v>47</v>
+      </c>
+      <c r="Y16" s="10">
+        <v>16</v>
+      </c>
+      <c r="Z16" s="67">
+        <v>41</v>
+      </c>
+      <c r="AA16" s="74">
+        <v>22</v>
+      </c>
+      <c r="AB16" s="77">
+        <v>50</v>
+      </c>
+      <c r="AC16" s="74">
+        <v>13</v>
+      </c>
+      <c r="AD16" s="68">
+        <v>44</v>
+      </c>
+      <c r="AE16" s="74">
+        <v>19</v>
+      </c>
+      <c r="AF16" s="68">
+        <v>43</v>
+      </c>
+      <c r="AG16" s="74">
+        <v>20</v>
+      </c>
+      <c r="AH16" s="68">
         <v>49</v>
       </c>
-      <c r="U16" s="10">
-        <v>22</v>
-      </c>
-      <c r="V16" s="68">
-        <v>58</v>
-      </c>
-      <c r="W16" s="10">
-        <v>14</v>
-      </c>
-      <c r="X16" s="69">
-        <v>50</v>
-      </c>
-      <c r="Y16" s="10">
-        <v>23</v>
-      </c>
-      <c r="Z16" s="69">
-        <v>56</v>
-      </c>
-      <c r="AA16" s="10">
-        <v>16</v>
-      </c>
-      <c r="AB16" s="68">
-        <v>49</v>
-      </c>
-      <c r="AC16" s="75">
-        <v>23</v>
-      </c>
-      <c r="AD16" s="62">
-        <f t="shared" si="1"/>
-        <v>430</v>
-      </c>
-      <c r="AE16" s="11">
-        <f t="shared" si="2"/>
-        <v>8</v>
-      </c>
-      <c r="AF16" s="37">
+      <c r="AI16" s="74">
+        <v>15</v>
+      </c>
+      <c r="AJ16" s="61">
+        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16+AD16+AF16+AH16</f>
+        <v>405</v>
+      </c>
+      <c r="AK16" s="11">
+        <f>COUNTIF(D16:AH16,"&gt;30")</f>
+        <v>9</v>
+      </c>
+      <c r="AL16" s="37">
         <v>2</v>
       </c>
-      <c r="AG16" s="10"/>
-      <c r="AH16" s="38">
-        <f t="shared" si="3"/>
-        <v>145</v>
-      </c>
-      <c r="AI16" s="66">
-        <f t="shared" si="4"/>
-        <v>18.125</v>
-      </c>
-      <c r="AJ16" s="58"/>
-      <c r="AK16" s="38"/>
-      <c r="AL16" s="38"/>
-      <c r="AM16" s="11"/>
-      <c r="AN16" s="56"/>
+      <c r="AM16" s="10">
+        <v>1</v>
+      </c>
+      <c r="AN16" s="38">
+        <f>SUMIF(G16:AI16, "&lt;30")+AL16+AM16</f>
+        <v>163</v>
+      </c>
+      <c r="AO16" s="65">
+        <f>AN16/AK16</f>
+        <v>18.111111111111111</v>
+      </c>
+      <c r="AP16" s="57"/>
+      <c r="AQ16" s="38"/>
+      <c r="AR16" s="38"/>
+      <c r="AS16" s="11"/>
+      <c r="AT16" s="56"/>
     </row>
-    <row r="17" spans="1:40">
+    <row r="17" spans="1:46">
       <c r="A17" s="7" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="C17" s="9">
-        <f>ROUND((AD17-(36*AE17))/AE17,0)</f>
-        <v>13</v>
+        <f>ROUND((AJ17-(36*AK17))/AK17,0)</f>
+        <v>18</v>
       </c>
       <c r="D17" s="48"/>
       <c r="E17" s="49"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="10"/>
+      <c r="F17" s="12">
+        <v>55</v>
+      </c>
+      <c r="G17" s="10">
+        <v>16</v>
+      </c>
       <c r="H17" s="48"/>
       <c r="I17" s="49"/>
       <c r="J17" s="12"/>
       <c r="K17" s="10"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="12"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="12">
-        <v>48</v>
-      </c>
-      <c r="Q17" s="10">
+      <c r="L17" s="12">
+        <v>56</v>
+      </c>
+      <c r="M17" s="10">
+        <v>15</v>
+      </c>
+      <c r="N17" s="12">
+        <v>57</v>
+      </c>
+      <c r="O17" s="10">
+        <v>14</v>
+      </c>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="67">
+        <v>49</v>
+      </c>
+      <c r="U17" s="10">
+        <v>22</v>
+      </c>
+      <c r="V17" s="67">
+        <v>58</v>
+      </c>
+      <c r="W17" s="10">
+        <v>14</v>
+      </c>
+      <c r="X17" s="68">
+        <v>50</v>
+      </c>
+      <c r="Y17" s="10">
+        <v>23</v>
+      </c>
+      <c r="Z17" s="68">
+        <v>56</v>
+      </c>
+      <c r="AA17" s="10">
+        <v>16</v>
+      </c>
+      <c r="AB17" s="67">
+        <v>49</v>
+      </c>
+      <c r="AC17" s="74">
+        <v>23</v>
+      </c>
+      <c r="AD17" s="68">
+        <v>54</v>
+      </c>
+      <c r="AE17" s="74">
         <v>18</v>
       </c>
-      <c r="R17" s="12">
-        <v>51</v>
-      </c>
-      <c r="S17" s="10">
+      <c r="AF17" s="68">
+        <v>58</v>
+      </c>
+      <c r="AG17" s="74">
         <v>14</v>
       </c>
-      <c r="T17" s="12">
-        <v>51</v>
-      </c>
-      <c r="U17" s="10">
-        <v>14</v>
-      </c>
-      <c r="V17" s="12"/>
-      <c r="W17" s="10"/>
-      <c r="X17" s="12">
-        <v>48</v>
-      </c>
-      <c r="Y17" s="10">
+      <c r="AH17" s="68">
+        <v>52</v>
+      </c>
+      <c r="AI17" s="74">
         <v>20</v>
       </c>
-      <c r="Z17" s="12">
-        <v>50</v>
-      </c>
-      <c r="AA17" s="10">
-        <v>18</v>
-      </c>
-      <c r="AB17" s="69">
-        <v>47</v>
-      </c>
-      <c r="AC17" s="75">
-        <v>21</v>
-      </c>
-      <c r="AD17" s="62">
-        <f t="shared" si="1"/>
-        <v>295</v>
-      </c>
-      <c r="AE17" s="11">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="AF17" s="37"/>
-      <c r="AG17" s="10"/>
-      <c r="AH17" s="38">
-        <f t="shared" si="3"/>
-        <v>105</v>
-      </c>
-      <c r="AI17" s="66">
-        <f t="shared" si="4"/>
-        <v>17.5</v>
-      </c>
-      <c r="AJ17" s="55"/>
-      <c r="AK17" s="38"/>
-      <c r="AL17" s="38"/>
-      <c r="AM17" s="11"/>
-      <c r="AN17" s="56"/>
+      <c r="AJ17" s="61">
+        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17+AD17+AF17+AH17</f>
+        <v>594</v>
+      </c>
+      <c r="AK17" s="11">
+        <f>COUNTIF(D17:AH17,"&gt;30")</f>
+        <v>11</v>
+      </c>
+      <c r="AL17" s="37">
+        <v>2</v>
+      </c>
+      <c r="AM17" s="10"/>
+      <c r="AN17" s="38">
+        <f>SUMIF(G17:AI17, "&lt;30")+AL17+AM17</f>
+        <v>197</v>
+      </c>
+      <c r="AO17" s="65">
+        <f>AN17/AK17</f>
+        <v>17.90909090909091</v>
+      </c>
+      <c r="AP17" s="57"/>
+      <c r="AQ17" s="38"/>
+      <c r="AR17" s="38"/>
+      <c r="AS17" s="11"/>
+      <c r="AT17" s="56"/>
     </row>
-    <row r="18" spans="1:40">
+    <row r="18" spans="1:46">
       <c r="A18" s="7" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C18" s="9">
-        <f>ROUND((AD18-(36*AE18))/AE18,0)</f>
-        <v>10</v>
+        <f>ROUND((AJ18-(36*AK18))/AK18,0)</f>
+        <v>11</v>
       </c>
       <c r="D18" s="48"/>
       <c r="E18" s="49"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="10"/>
+      <c r="F18" s="12">
+        <v>46</v>
+      </c>
+      <c r="G18" s="10">
+        <v>18</v>
+      </c>
       <c r="H18" s="48"/>
       <c r="I18" s="49"/>
-      <c r="J18" s="14"/>
+      <c r="J18" s="12"/>
       <c r="K18" s="10"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="39">
-        <v>45</v>
+      <c r="L18" s="12">
+        <v>46</v>
+      </c>
+      <c r="M18" s="10">
+        <v>18</v>
+      </c>
+      <c r="N18" s="12">
+        <v>46</v>
       </c>
       <c r="O18" s="10">
         <v>18</v>
       </c>
-      <c r="P18" s="39">
-        <v>43</v>
+      <c r="P18" s="12">
+        <v>46</v>
       </c>
       <c r="Q18" s="10">
-        <v>20</v>
-      </c>
-      <c r="R18" s="39"/>
-      <c r="S18" s="10"/>
-      <c r="T18" s="39"/>
-      <c r="U18" s="10"/>
-      <c r="V18" s="39"/>
+        <v>18</v>
+      </c>
+      <c r="R18" s="12">
+        <v>47</v>
+      </c>
+      <c r="S18" s="10">
+        <v>14</v>
+      </c>
+      <c r="T18" s="12">
+        <v>52</v>
+      </c>
+      <c r="U18" s="10">
+        <v>13</v>
+      </c>
+      <c r="V18" s="12"/>
       <c r="W18" s="10"/>
-      <c r="X18" s="39">
+      <c r="X18" s="12"/>
+      <c r="Y18" s="10"/>
+      <c r="Z18" s="12">
+        <v>50</v>
+      </c>
+      <c r="AA18" s="10">
+        <v>15</v>
+      </c>
+      <c r="AB18" s="68"/>
+      <c r="AC18" s="74"/>
+      <c r="AD18" s="68">
+        <v>47</v>
+      </c>
+      <c r="AE18" s="74">
+        <v>19</v>
+      </c>
+      <c r="AF18" s="68">
         <v>48</v>
       </c>
-      <c r="Y18" s="10">
-        <v>15</v>
-      </c>
-      <c r="Z18" s="39">
-        <v>47</v>
-      </c>
-      <c r="AA18" s="75">
-        <v>16</v>
-      </c>
-      <c r="AB18" s="39"/>
-      <c r="AC18" s="75"/>
-      <c r="AD18" s="62">
-        <f t="shared" si="1"/>
-        <v>183</v>
-      </c>
-      <c r="AE18" s="11">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="AF18" s="37"/>
-      <c r="AG18" s="10">
+      <c r="AG18" s="74">
+        <v>18</v>
+      </c>
+      <c r="AH18" s="68">
+        <v>44</v>
+      </c>
+      <c r="AI18" s="74">
+        <v>22</v>
+      </c>
+      <c r="AJ18" s="61">
+        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18+AD18+AF18+AH18</f>
+        <v>472</v>
+      </c>
+      <c r="AK18" s="11">
+        <f>COUNTIF(D18:AH18,"&gt;30")</f>
+        <v>10</v>
+      </c>
+      <c r="AL18" s="40"/>
+      <c r="AM18" s="30">
         <v>1</v>
       </c>
-      <c r="AH18" s="38">
-        <f t="shared" si="3"/>
-        <v>70</v>
-      </c>
-      <c r="AI18" s="66">
-        <f t="shared" si="4"/>
-        <v>17.5</v>
-      </c>
-      <c r="AJ18" s="55"/>
-      <c r="AK18" s="38"/>
-      <c r="AL18" s="38"/>
-      <c r="AM18" s="11"/>
-      <c r="AN18" s="56"/>
+      <c r="AN18" s="38">
+        <f>SUMIF(G18:AI18, "&lt;30")+AL18+AM18</f>
+        <v>174</v>
+      </c>
+      <c r="AO18" s="65">
+        <f>AN18/AK18</f>
+        <v>17.399999999999999</v>
+      </c>
+      <c r="AP18" s="57"/>
+      <c r="AQ18" s="11"/>
+      <c r="AR18" s="11"/>
+      <c r="AS18" s="11"/>
+      <c r="AT18" s="56"/>
     </row>
-    <row r="19" spans="1:40">
+    <row r="19" spans="1:46">
       <c r="A19" s="7" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C19" s="9">
-        <f>ROUND((AD19-(36*AE19))/AE19,0)</f>
-        <v>12</v>
+        <f>ROUND((AJ19-(36*AK19))/AK19,0)</f>
+        <v>11</v>
       </c>
       <c r="D19" s="48"/>
       <c r="E19" s="49"/>
-      <c r="F19" s="12">
-        <v>46</v>
-      </c>
-      <c r="G19" s="10">
-        <v>18</v>
-      </c>
+      <c r="F19" s="14"/>
+      <c r="G19" s="10"/>
       <c r="H19" s="48"/>
       <c r="I19" s="49"/>
-      <c r="J19" s="12"/>
+      <c r="J19" s="14"/>
       <c r="K19" s="10"/>
-      <c r="L19" s="12">
-        <v>46</v>
-      </c>
-      <c r="M19" s="10">
-        <v>18</v>
-      </c>
-      <c r="N19" s="12">
-        <v>46</v>
+      <c r="L19" s="14"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="39">
+        <v>45</v>
       </c>
       <c r="O19" s="10">
         <v>18</v>
       </c>
-      <c r="P19" s="12">
-        <v>46</v>
+      <c r="P19" s="39">
+        <v>43</v>
       </c>
       <c r="Q19" s="10">
-        <v>18</v>
-      </c>
-      <c r="R19" s="12">
+        <v>20</v>
+      </c>
+      <c r="R19" s="39"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="39"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="39"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="39">
+        <v>48</v>
+      </c>
+      <c r="Y19" s="10">
+        <v>15</v>
+      </c>
+      <c r="Z19" s="39">
         <v>47</v>
       </c>
-      <c r="S19" s="10">
-        <v>14</v>
-      </c>
-      <c r="T19" s="12">
-        <v>52</v>
-      </c>
-      <c r="U19" s="10">
+      <c r="AA19" s="74">
+        <v>16</v>
+      </c>
+      <c r="AB19" s="39"/>
+      <c r="AC19" s="74"/>
+      <c r="AD19" s="39">
+        <v>51</v>
+      </c>
+      <c r="AE19" s="74">
         <v>13</v>
       </c>
-      <c r="V19" s="12"/>
-      <c r="W19" s="10"/>
-      <c r="X19" s="12"/>
-      <c r="Y19" s="10"/>
-      <c r="Z19" s="12">
-        <v>50</v>
-      </c>
-      <c r="AA19" s="10">
-        <v>15</v>
-      </c>
-      <c r="AB19" s="69"/>
-      <c r="AC19" s="75"/>
-      <c r="AD19" s="62">
-        <f t="shared" si="1"/>
-        <v>333</v>
-      </c>
-      <c r="AE19" s="11">
-        <f t="shared" si="2"/>
-        <v>7</v>
-      </c>
-      <c r="AF19" s="40"/>
-      <c r="AG19" s="30"/>
-      <c r="AH19" s="38">
-        <f t="shared" si="3"/>
-        <v>114</v>
-      </c>
-      <c r="AI19" s="66">
-        <f t="shared" si="4"/>
-        <v>16.285714285714285</v>
-      </c>
-      <c r="AJ19" s="58"/>
-      <c r="AK19" s="11"/>
-      <c r="AL19" s="11"/>
-      <c r="AM19" s="11"/>
-      <c r="AN19" s="56"/>
+      <c r="AF19" s="39">
+        <v>45</v>
+      </c>
+      <c r="AG19" s="74">
+        <v>20</v>
+      </c>
+      <c r="AH19" s="39"/>
+      <c r="AI19" s="74"/>
+      <c r="AJ19" s="61">
+        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19+AD19+AF19+AH19</f>
+        <v>279</v>
+      </c>
+      <c r="AK19" s="11">
+        <f>COUNTIF(D19:AH19,"&gt;30")</f>
+        <v>6</v>
+      </c>
+      <c r="AL19" s="37"/>
+      <c r="AM19" s="10">
+        <v>2</v>
+      </c>
+      <c r="AN19" s="38">
+        <f>SUMIF(G19:AI19, "&lt;30")+AL19+AM19</f>
+        <v>104</v>
+      </c>
+      <c r="AO19" s="65">
+        <f>AN19/AK19</f>
+        <v>17.333333333333332</v>
+      </c>
+      <c r="AP19" s="55"/>
+      <c r="AQ19" s="38"/>
+      <c r="AR19" s="38"/>
+      <c r="AS19" s="11"/>
+      <c r="AT19" s="56"/>
     </row>
-    <row r="20" spans="1:40">
+    <row r="20" spans="1:46">
       <c r="A20" s="7" t="s">
         <v>23</v>
       </c>
@@ -3360,7 +3656,7 @@
         <v>24</v>
       </c>
       <c r="C20" s="9">
-        <f>ROUND((AD20-(36*AE20))/AE20,0)</f>
+        <f>ROUND((AJ20-(36*AK20))/AK20,0)</f>
         <v>24</v>
       </c>
       <c r="D20" s="48"/>
@@ -3416,42 +3712,60 @@
       <c r="Z20" s="39">
         <v>70</v>
       </c>
-      <c r="AA20" s="75">
+      <c r="AA20" s="74">
         <v>6</v>
       </c>
       <c r="AB20" s="39">
         <v>63</v>
       </c>
-      <c r="AC20" s="75">
+      <c r="AC20" s="74">
         <v>15</v>
       </c>
-      <c r="AD20" s="62">
-        <f t="shared" si="1"/>
-        <v>541</v>
-      </c>
-      <c r="AE20" s="11">
-        <f t="shared" si="2"/>
-        <v>9</v>
-      </c>
-      <c r="AF20" s="37">
+      <c r="AD20" s="39">
+        <v>58</v>
+      </c>
+      <c r="AE20" s="74">
+        <v>20</v>
+      </c>
+      <c r="AF20" s="39">
+        <v>60</v>
+      </c>
+      <c r="AG20" s="74">
+        <v>18</v>
+      </c>
+      <c r="AH20" s="39">
+        <v>55</v>
+      </c>
+      <c r="AI20" s="74">
+        <v>23</v>
+      </c>
+      <c r="AJ20" s="61">
+        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20+AD20+AF20+AH20</f>
+        <v>714</v>
+      </c>
+      <c r="AK20" s="11">
+        <f>COUNTIF(D20:AH20,"&gt;30")</f>
+        <v>12</v>
+      </c>
+      <c r="AL20" s="37">
         <v>2</v>
       </c>
-      <c r="AG20" s="10"/>
-      <c r="AH20" s="38">
-        <f t="shared" si="3"/>
-        <v>144</v>
-      </c>
-      <c r="AI20" s="66">
-        <f t="shared" si="4"/>
-        <v>16</v>
-      </c>
-      <c r="AJ20" s="55"/>
-      <c r="AK20" s="38"/>
-      <c r="AL20" s="38"/>
-      <c r="AM20" s="11"/>
-      <c r="AN20" s="56"/>
+      <c r="AM20" s="10"/>
+      <c r="AN20" s="38">
+        <f>SUMIF(G20:AI20, "&lt;30")+AL20+AM20</f>
+        <v>205</v>
+      </c>
+      <c r="AO20" s="65">
+        <f>AN20/AK20</f>
+        <v>17.083333333333332</v>
+      </c>
+      <c r="AP20" s="55"/>
+      <c r="AQ20" s="38"/>
+      <c r="AR20" s="38"/>
+      <c r="AS20" s="11"/>
+      <c r="AT20" s="56"/>
     </row>
-    <row r="21" spans="1:40">
+    <row r="21" spans="1:46">
       <c r="A21" s="7" t="s">
         <v>21</v>
       </c>
@@ -3489,33 +3803,39 @@
       <c r="Y21" s="10"/>
       <c r="Z21" s="12"/>
       <c r="AA21" s="10"/>
-      <c r="AB21" s="69"/>
-      <c r="AC21" s="75"/>
-      <c r="AD21" s="62">
-        <f t="shared" si="1"/>
+      <c r="AB21" s="68"/>
+      <c r="AC21" s="74"/>
+      <c r="AD21" s="68"/>
+      <c r="AE21" s="74"/>
+      <c r="AF21" s="68"/>
+      <c r="AG21" s="74"/>
+      <c r="AH21" s="68"/>
+      <c r="AI21" s="74"/>
+      <c r="AJ21" s="61">
+        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21+AD21+AF21+AH21</f>
         <v>56</v>
       </c>
-      <c r="AE21" s="11">
-        <f t="shared" si="2"/>
+      <c r="AK21" s="11">
+        <f>COUNTIF(D21:AH21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AF21" s="37"/>
-      <c r="AG21" s="10"/>
-      <c r="AH21" s="38">
-        <f t="shared" si="3"/>
+      <c r="AL21" s="37"/>
+      <c r="AM21" s="10"/>
+      <c r="AN21" s="38">
+        <f>SUMIF(G21:AI21, "&lt;30")+AL21+AM21</f>
         <v>16</v>
       </c>
-      <c r="AI21" s="66">
-        <f t="shared" si="4"/>
+      <c r="AO21" s="65">
+        <f>AN21/AK21</f>
         <v>16</v>
       </c>
-      <c r="AJ21" s="58"/>
-      <c r="AK21" s="38"/>
-      <c r="AL21" s="38"/>
-      <c r="AM21" s="11"/>
-      <c r="AN21" s="56"/>
+      <c r="AP21" s="57"/>
+      <c r="AQ21" s="38"/>
+      <c r="AR21" s="38"/>
+      <c r="AS21" s="11"/>
+      <c r="AT21" s="56"/>
     </row>
-    <row r="22" spans="1:40" ht="16.5" thickBot="1">
+    <row r="22" spans="1:46" ht="17" thickBot="1">
       <c r="A22" s="15" t="s">
         <v>48</v>
       </c>
@@ -3527,59 +3847,65 @@
       </c>
       <c r="D22" s="50"/>
       <c r="E22" s="51"/>
-      <c r="F22" s="72"/>
+      <c r="F22" s="71"/>
       <c r="G22" s="18"/>
       <c r="H22" s="50"/>
       <c r="I22" s="51"/>
-      <c r="J22" s="72"/>
+      <c r="J22" s="71"/>
       <c r="K22" s="18"/>
-      <c r="L22" s="73">
+      <c r="L22" s="72">
         <v>50</v>
       </c>
       <c r="M22" s="18"/>
-      <c r="N22" s="73"/>
+      <c r="N22" s="72"/>
       <c r="O22" s="18"/>
-      <c r="P22" s="73"/>
+      <c r="P22" s="72"/>
       <c r="Q22" s="18"/>
-      <c r="R22" s="73"/>
+      <c r="R22" s="72"/>
       <c r="S22" s="18"/>
-      <c r="T22" s="73"/>
+      <c r="T22" s="72"/>
       <c r="U22" s="18"/>
-      <c r="V22" s="73"/>
+      <c r="V22" s="72"/>
       <c r="W22" s="18"/>
-      <c r="X22" s="73"/>
+      <c r="X22" s="72"/>
       <c r="Y22" s="18"/>
-      <c r="Z22" s="73"/>
+      <c r="Z22" s="72"/>
       <c r="AA22" s="18"/>
-      <c r="AB22" s="73"/>
+      <c r="AB22" s="72"/>
       <c r="AC22" s="18"/>
-      <c r="AD22" s="63">
-        <f t="shared" si="1"/>
+      <c r="AD22" s="72"/>
+      <c r="AE22" s="18"/>
+      <c r="AF22" s="72"/>
+      <c r="AG22" s="18"/>
+      <c r="AH22" s="72"/>
+      <c r="AI22" s="18"/>
+      <c r="AJ22" s="62">
+        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22+AD22+AF22+AH22</f>
         <v>50</v>
       </c>
-      <c r="AE22" s="19">
-        <f t="shared" si="2"/>
+      <c r="AK22" s="19">
+        <f>COUNTIF(D22:AH22,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AF22" s="41">
+      <c r="AL22" s="41">
         <v>1</v>
       </c>
-      <c r="AG22" s="18"/>
-      <c r="AH22" s="42">
-        <f t="shared" si="3"/>
+      <c r="AM22" s="18"/>
+      <c r="AN22" s="42">
+        <f>SUMIF(G22:AI22, "&lt;30")+AL22+AM22</f>
         <v>1</v>
       </c>
-      <c r="AI22" s="67">
-        <f t="shared" si="4"/>
+      <c r="AO22" s="66">
+        <f>AN22/AK22</f>
         <v>1</v>
       </c>
-      <c r="AJ22" s="59"/>
-      <c r="AK22" s="42"/>
-      <c r="AL22" s="42"/>
-      <c r="AM22" s="19"/>
-      <c r="AN22" s="60"/>
+      <c r="AP22" s="58"/>
+      <c r="AQ22" s="42"/>
+      <c r="AR22" s="42"/>
+      <c r="AS22" s="19"/>
+      <c r="AT22" s="59"/>
     </row>
-    <row r="23" spans="1:40" s="20" customFormat="1" ht="16.5" thickBot="1">
+    <row r="23" spans="1:46" s="20" customFormat="1" ht="17" thickBot="1">
       <c r="A23" s="31"/>
       <c r="B23" s="32"/>
       <c r="C23" s="32"/>
@@ -3642,18 +3968,33 @@
         <v>47.846153846153847</v>
       </c>
       <c r="AC23" s="33"/>
-      <c r="AD23" s="34"/>
+      <c r="AD23" s="33">
+        <f>AVERAGEIF(AD4:AD22,"&gt;0")</f>
+        <v>46.090909090909093</v>
+      </c>
+      <c r="AE23" s="33"/>
+      <c r="AF23" s="33">
+        <f>AVERAGEIF(AF4:AF22,"&gt;0")</f>
+        <v>47.230769230769234</v>
+      </c>
+      <c r="AG23" s="33"/>
+      <c r="AH23" s="33">
+        <f>AVERAGEIF(AH4:AH22,"&gt;0")</f>
+        <v>46.666666666666664</v>
+      </c>
+      <c r="AI23" s="33"/>
+      <c r="AJ23" s="34"/>
     </row>
-    <row r="24" spans="1:40">
+    <row r="24" spans="1:46">
       <c r="C24" s="21"/>
-      <c r="AD24" s="22"/>
-      <c r="AE24" s="22"/>
-      <c r="AF24" s="23"/>
-      <c r="AG24" s="23"/>
-      <c r="AH24" s="22"/>
-      <c r="AI24" s="24"/>
+      <c r="AJ24" s="22"/>
+      <c r="AK24" s="22"/>
+      <c r="AL24" s="23"/>
+      <c r="AM24" s="23"/>
+      <c r="AN24" s="22"/>
+      <c r="AO24" s="24"/>
     </row>
-    <row r="25" spans="1:40">
+    <row r="25" spans="1:46">
       <c r="C25" s="43" t="s">
         <v>41</v>
       </c>
@@ -3672,8 +4013,11 @@
       <c r="X25" s="25"/>
       <c r="Z25" s="25"/>
       <c r="AB25" s="25"/>
+      <c r="AD25" s="25"/>
+      <c r="AF25" s="25"/>
+      <c r="AH25" s="25"/>
     </row>
-    <row r="26" spans="1:40">
+    <row r="26" spans="1:46">
       <c r="C26" s="44" t="s">
         <v>42</v>
       </c>
@@ -3692,9 +4036,12 @@
       <c r="X26" s="26"/>
       <c r="Z26" s="26"/>
       <c r="AB26" s="26"/>
-      <c r="AD26" s="27"/>
+      <c r="AD26" s="26"/>
+      <c r="AF26" s="26"/>
+      <c r="AH26" s="26"/>
+      <c r="AJ26" s="27"/>
     </row>
-    <row r="27" spans="1:40">
+    <row r="27" spans="1:46">
       <c r="C27" s="45" t="s">
         <v>46</v>
       </c>
@@ -3726,28 +4073,37 @@
       <c r="AA27" s="29"/>
       <c r="AB27" s="28"/>
       <c r="AC27" s="29"/>
+      <c r="AD27" s="28"/>
+      <c r="AE27" s="29"/>
+      <c r="AF27" s="28"/>
+      <c r="AG27" s="29"/>
+      <c r="AH27" s="28"/>
+      <c r="AI27" s="29"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AN22">
-    <sortCondition descending="1" ref="AI4:AI22"/>
-    <sortCondition descending="1" ref="AD4:AD22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AT22">
+    <sortCondition descending="1" ref="AO4:AO22"/>
+    <sortCondition descending="1" ref="AJ4:AJ22"/>
   </sortState>
-  <mergeCells count="41">
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="AJ1:AN1"/>
-    <mergeCell ref="AJ2:AJ3"/>
-    <mergeCell ref="AK2:AK3"/>
-    <mergeCell ref="AL2:AL3"/>
-    <mergeCell ref="AM2:AM3"/>
-    <mergeCell ref="AN2:AN3"/>
-    <mergeCell ref="AH2:AH3"/>
-    <mergeCell ref="AI2:AI3"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="AE2:AE3"/>
+  <mergeCells count="47">
+    <mergeCell ref="AH1:AI1"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="N1:O1"/>
-    <mergeCell ref="AD1:AD3"/>
-    <mergeCell ref="AE1:AI1"/>
+    <mergeCell ref="AJ1:AJ3"/>
+    <mergeCell ref="AK1:AO1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="P2:Q2"/>
@@ -3758,22 +4114,25 @@
     <mergeCell ref="V1:W1"/>
     <mergeCell ref="Z1:AA1"/>
     <mergeCell ref="AB1:AC1"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="AP1:AT1"/>
+    <mergeCell ref="AP2:AP3"/>
+    <mergeCell ref="AQ2:AQ3"/>
+    <mergeCell ref="AR2:AR3"/>
+    <mergeCell ref="AS2:AS3"/>
+    <mergeCell ref="AT2:AT3"/>
+    <mergeCell ref="AN2:AN3"/>
+    <mergeCell ref="AO2:AO3"/>
+    <mergeCell ref="AL2:AL3"/>
+    <mergeCell ref="AM2:AM3"/>
+    <mergeCell ref="AK2:AK3"/>
+    <mergeCell ref="AD1:AE1"/>
+    <mergeCell ref="AD2:AE2"/>
+    <mergeCell ref="AF1:AG1"/>
+    <mergeCell ref="AF2:AG2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
090225 - updated results page
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="13_ncr:1_{3CAD6DB6-E3D7-F14D-BFB0-08DA4216CCD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94B1057E-DEFC-4505-B841-7BEFC0850F02}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="13_ncr:1_{3CAD6DB6-E3D7-F14D-BFB0-08DA4216CCD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19DCD355-21B6-4EEC-B38D-5D05928B7CFF}"/>
   <bookViews>
     <workbookView xWindow="3525" yWindow="2190" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
@@ -262,7 +262,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -395,12 +395,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="26"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF00B050"/>
@@ -429,7 +423,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -753,6 +747,168 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -760,7 +916,7 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -772,10 +928,17 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -790,22 +953,18 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -818,145 +977,81 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
+      <left/>
+      <right/>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -970,7 +1065,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -980,40 +1075,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1041,22 +1121,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1071,68 +1145,44 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1141,19 +1191,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="16" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1162,13 +1206,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1180,58 +1221,58 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1240,24 +1281,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1273,7 +1296,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1285,13 +1308,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1306,7 +1329,7 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1348,13 +1371,69 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="46" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="47" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="49" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1732,226 +1811,226 @@
     <col min="50" max="50" width="9.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" s="47" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="125" t="s">
+    <row r="1" spans="1:50" s="34" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="131" t="s">
+      <c r="B1" s="102"/>
+      <c r="C1" s="107" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="103" t="s">
+      <c r="D1" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="104"/>
-      <c r="F1" s="103" t="s">
+      <c r="E1" s="80"/>
+      <c r="F1" s="79" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="104"/>
-      <c r="H1" s="103" t="s">
+      <c r="G1" s="80"/>
+      <c r="H1" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="104"/>
-      <c r="J1" s="103" t="s">
+      <c r="I1" s="80"/>
+      <c r="J1" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="104"/>
-      <c r="L1" s="103" t="s">
+      <c r="K1" s="80"/>
+      <c r="L1" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="104"/>
-      <c r="N1" s="103" t="s">
+      <c r="M1" s="80"/>
+      <c r="N1" s="79" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="104"/>
-      <c r="P1" s="103" t="s">
+      <c r="O1" s="80"/>
+      <c r="P1" s="79" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="104"/>
-      <c r="R1" s="103" t="s">
+      <c r="Q1" s="80"/>
+      <c r="R1" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="104"/>
-      <c r="T1" s="103" t="s">
+      <c r="S1" s="80"/>
+      <c r="T1" s="79" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="104"/>
-      <c r="V1" s="103" t="s">
+      <c r="U1" s="80"/>
+      <c r="V1" s="79" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="104"/>
-      <c r="X1" s="103" t="s">
+      <c r="W1" s="80"/>
+      <c r="X1" s="79" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="104"/>
-      <c r="Z1" s="103" t="s">
+      <c r="Y1" s="80"/>
+      <c r="Z1" s="79" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="104"/>
-      <c r="AB1" s="103" t="s">
+      <c r="AA1" s="80"/>
+      <c r="AB1" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="104"/>
-      <c r="AD1" s="103" t="s">
+      <c r="AC1" s="80"/>
+      <c r="AD1" s="79" t="s">
         <v>67</v>
       </c>
-      <c r="AE1" s="104"/>
-      <c r="AF1" s="103" t="s">
+      <c r="AE1" s="80"/>
+      <c r="AF1" s="79" t="s">
         <v>68</v>
       </c>
-      <c r="AG1" s="104"/>
-      <c r="AH1" s="103" t="s">
+      <c r="AG1" s="80"/>
+      <c r="AH1" s="79" t="s">
         <v>69</v>
       </c>
-      <c r="AI1" s="104"/>
-      <c r="AJ1" s="103" t="s">
+      <c r="AI1" s="80"/>
+      <c r="AJ1" s="79" t="s">
         <v>70</v>
       </c>
-      <c r="AK1" s="104"/>
-      <c r="AL1" s="103" t="s">
+      <c r="AK1" s="80"/>
+      <c r="AL1" s="79" t="s">
         <v>71</v>
       </c>
-      <c r="AM1" s="104"/>
-      <c r="AN1" s="115" t="s">
+      <c r="AM1" s="80"/>
+      <c r="AN1" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="122" t="s">
+      <c r="AO1" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="AP1" s="123"/>
-      <c r="AQ1" s="123"/>
-      <c r="AR1" s="123"/>
-      <c r="AS1" s="124"/>
-      <c r="AT1" s="117" t="s">
+      <c r="AP1" s="99"/>
+      <c r="AQ1" s="99"/>
+      <c r="AR1" s="99"/>
+      <c r="AS1" s="100"/>
+      <c r="AT1" s="93" t="s">
         <v>57</v>
       </c>
-      <c r="AU1" s="118"/>
-      <c r="AV1" s="118"/>
-      <c r="AW1" s="118"/>
-      <c r="AX1" s="119"/>
+      <c r="AU1" s="94"/>
+      <c r="AV1" s="94"/>
+      <c r="AW1" s="94"/>
+      <c r="AX1" s="95"/>
     </row>
-    <row r="2" spans="1:50" s="47" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="127"/>
-      <c r="B2" s="128"/>
-      <c r="C2" s="132"/>
-      <c r="D2" s="105">
+    <row r="2" spans="1:50" s="34" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="103"/>
+      <c r="B2" s="104"/>
+      <c r="C2" s="108"/>
+      <c r="D2" s="81">
         <v>45782</v>
       </c>
-      <c r="E2" s="106"/>
-      <c r="F2" s="105">
+      <c r="E2" s="82"/>
+      <c r="F2" s="81">
         <v>45789</v>
       </c>
-      <c r="G2" s="106"/>
-      <c r="H2" s="105">
+      <c r="G2" s="82"/>
+      <c r="H2" s="81">
         <v>45796</v>
       </c>
-      <c r="I2" s="106"/>
-      <c r="J2" s="105">
+      <c r="I2" s="82"/>
+      <c r="J2" s="81">
         <v>45803</v>
       </c>
-      <c r="K2" s="106"/>
-      <c r="L2" s="105">
+      <c r="K2" s="82"/>
+      <c r="L2" s="81">
         <v>45810</v>
       </c>
-      <c r="M2" s="106"/>
-      <c r="N2" s="105">
+      <c r="M2" s="82"/>
+      <c r="N2" s="81">
         <v>45817</v>
       </c>
-      <c r="O2" s="106"/>
-      <c r="P2" s="105">
+      <c r="O2" s="82"/>
+      <c r="P2" s="81">
         <v>45824</v>
       </c>
-      <c r="Q2" s="106"/>
-      <c r="R2" s="105">
+      <c r="Q2" s="82"/>
+      <c r="R2" s="81">
         <v>45831</v>
       </c>
-      <c r="S2" s="106"/>
-      <c r="T2" s="105">
+      <c r="S2" s="82"/>
+      <c r="T2" s="81">
         <v>45838</v>
       </c>
-      <c r="U2" s="106"/>
-      <c r="V2" s="105">
+      <c r="U2" s="82"/>
+      <c r="V2" s="81">
         <v>45845</v>
       </c>
-      <c r="W2" s="106"/>
-      <c r="X2" s="105">
+      <c r="W2" s="82"/>
+      <c r="X2" s="81">
         <v>45852</v>
       </c>
-      <c r="Y2" s="106"/>
-      <c r="Z2" s="105">
+      <c r="Y2" s="82"/>
+      <c r="Z2" s="81">
         <v>45859</v>
       </c>
-      <c r="AA2" s="106"/>
-      <c r="AB2" s="105">
+      <c r="AA2" s="82"/>
+      <c r="AB2" s="81">
         <v>45866</v>
       </c>
-      <c r="AC2" s="106"/>
-      <c r="AD2" s="105">
+      <c r="AC2" s="82"/>
+      <c r="AD2" s="81">
         <v>45873</v>
       </c>
-      <c r="AE2" s="106"/>
-      <c r="AF2" s="105">
+      <c r="AE2" s="82"/>
+      <c r="AF2" s="81">
         <v>45880</v>
       </c>
-      <c r="AG2" s="106"/>
-      <c r="AH2" s="105">
+      <c r="AG2" s="82"/>
+      <c r="AH2" s="81">
         <v>45887</v>
       </c>
-      <c r="AI2" s="106"/>
-      <c r="AJ2" s="105">
+      <c r="AI2" s="82"/>
+      <c r="AJ2" s="81">
         <v>45894</v>
       </c>
-      <c r="AK2" s="106"/>
-      <c r="AL2" s="105">
+      <c r="AK2" s="82"/>
+      <c r="AL2" s="81">
         <v>45901</v>
       </c>
-      <c r="AM2" s="106"/>
-      <c r="AN2" s="116"/>
-      <c r="AO2" s="115" t="s">
+      <c r="AM2" s="82"/>
+      <c r="AN2" s="92"/>
+      <c r="AO2" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AP2" s="111" t="s">
+      <c r="AP2" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="AQ2" s="113" t="s">
+      <c r="AQ2" s="89" t="s">
         <v>5</v>
       </c>
-      <c r="AR2" s="107" t="s">
+      <c r="AR2" s="83" t="s">
         <v>6</v>
       </c>
-      <c r="AS2" s="109" t="s">
+      <c r="AS2" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="AT2" s="120" t="s">
+      <c r="AT2" s="96" t="s">
         <v>3</v>
       </c>
-      <c r="AU2" s="120" t="s">
+      <c r="AU2" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="AV2" s="120" t="s">
+      <c r="AV2" s="96" t="s">
         <v>5</v>
       </c>
-      <c r="AW2" s="120" t="s">
+      <c r="AW2" s="96" t="s">
         <v>6</v>
       </c>
-      <c r="AX2" s="120" t="s">
+      <c r="AX2" s="96" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:50" s="47" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
-      <c r="A3" s="129"/>
-      <c r="B3" s="130"/>
-      <c r="C3" s="133"/>
-      <c r="D3" s="1" t="s">
+    <row r="3" spans="1:50" s="34" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
+      <c r="A3" s="105"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="122" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="122" t="s">
         <v>9</v>
       </c>
       <c r="H3" s="1" t="s">
@@ -2050,17 +2129,17 @@
       <c r="AM3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="AN3" s="116"/>
-      <c r="AO3" s="116"/>
-      <c r="AP3" s="112"/>
-      <c r="AQ3" s="114"/>
-      <c r="AR3" s="108"/>
-      <c r="AS3" s="110"/>
-      <c r="AT3" s="121"/>
-      <c r="AU3" s="121"/>
-      <c r="AV3" s="121"/>
-      <c r="AW3" s="121"/>
-      <c r="AX3" s="121"/>
+      <c r="AN3" s="92"/>
+      <c r="AO3" s="92"/>
+      <c r="AP3" s="88"/>
+      <c r="AQ3" s="90"/>
+      <c r="AR3" s="84"/>
+      <c r="AS3" s="86"/>
+      <c r="AT3" s="97"/>
+      <c r="AU3" s="97"/>
+      <c r="AV3" s="97"/>
+      <c r="AW3" s="97"/>
+      <c r="AX3" s="97"/>
     </row>
     <row r="4" spans="1:50" ht="15.95" customHeight="1">
       <c r="A4" s="3" t="s">
@@ -2069,2278 +2148,2281 @@
       <c r="B4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="117">
         <f>ROUND((AN4-(36*AO4))/AO4,0)</f>
         <v>17</v>
       </c>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="70">
+      <c r="D4" s="125"/>
+      <c r="E4" s="128"/>
+      <c r="F4" s="53">
         <v>53</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="71">
         <v>23</v>
       </c>
-      <c r="H4" s="40"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="70"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="70"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="70">
+      <c r="H4" s="125"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="71"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="71"/>
+      <c r="N4" s="53">
         <v>57</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="71">
         <v>19</v>
       </c>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="70">
+      <c r="P4" s="53"/>
+      <c r="Q4" s="71"/>
+      <c r="R4" s="53">
         <v>50</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="71">
         <v>26</v>
       </c>
-      <c r="T4" s="70">
+      <c r="T4" s="53">
         <v>56</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="71">
         <v>15</v>
       </c>
-      <c r="V4" s="70"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="70"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="74">
+      <c r="V4" s="53"/>
+      <c r="W4" s="71"/>
+      <c r="X4" s="53"/>
+      <c r="Y4" s="71"/>
+      <c r="Z4" s="53">
         <v>54</v>
       </c>
-      <c r="AA4" s="64">
+      <c r="AA4" s="71">
         <v>18</v>
       </c>
-      <c r="AB4" s="74">
+      <c r="AB4" s="53">
         <v>50</v>
       </c>
-      <c r="AC4" s="64">
+      <c r="AC4" s="71">
         <v>22</v>
       </c>
-      <c r="AD4" s="74"/>
-      <c r="AE4" s="80"/>
-      <c r="AF4" s="74"/>
-      <c r="AG4" s="80"/>
-      <c r="AH4" s="74"/>
-      <c r="AI4" s="80"/>
-      <c r="AJ4" s="97"/>
-      <c r="AK4" s="98"/>
-      <c r="AL4" s="74"/>
-      <c r="AM4" s="80"/>
-      <c r="AN4" s="67">
+      <c r="AD4" s="56"/>
+      <c r="AE4" s="62"/>
+      <c r="AF4" s="56"/>
+      <c r="AG4" s="62"/>
+      <c r="AH4" s="56"/>
+      <c r="AI4" s="62"/>
+      <c r="AJ4" s="125"/>
+      <c r="AK4" s="128"/>
+      <c r="AL4" s="56"/>
+      <c r="AM4" s="62"/>
+      <c r="AN4" s="50">
         <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4+AJ4+AL4</f>
         <v>320</v>
       </c>
-      <c r="AO4" s="67">
+      <c r="AO4" s="50">
         <f>COUNTIF(D4:AL4,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AP4" s="88"/>
-      <c r="AQ4" s="89"/>
-      <c r="AR4" s="85">
+      <c r="AP4" s="70"/>
+      <c r="AQ4" s="71"/>
+      <c r="AR4" s="67">
         <f>SUMIF(G4:AM4, "&lt;30")+AP4+AQ4</f>
         <v>123</v>
       </c>
-      <c r="AS4" s="55">
+      <c r="AS4" s="42">
         <f>AR4/AO4</f>
         <v>20.5</v>
       </c>
-      <c r="AT4" s="67"/>
-      <c r="AU4" s="33"/>
-      <c r="AV4" s="33"/>
-      <c r="AW4" s="6"/>
-      <c r="AX4" s="48" t="s">
+      <c r="AT4" s="50"/>
+      <c r="AU4" s="26"/>
+      <c r="AV4" s="26"/>
+      <c r="AW4" s="5"/>
+      <c r="AX4" s="35" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:50">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="118">
         <f>ROUND((AN5-(36*AO5))/AO5,0)</f>
         <v>1</v>
       </c>
-      <c r="D5" s="42"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="71"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="71"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="72">
+      <c r="D5" s="126"/>
+      <c r="E5" s="129"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="126"/>
+      <c r="I5" s="129"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="65"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="65"/>
+      <c r="P5" s="54">
         <v>39</v>
       </c>
-      <c r="Q5" s="10">
+      <c r="Q5" s="65">
         <v>17</v>
       </c>
-      <c r="R5" s="72">
+      <c r="R5" s="54">
         <v>38</v>
       </c>
-      <c r="S5" s="10">
+      <c r="S5" s="65">
         <v>18</v>
       </c>
-      <c r="T5" s="72"/>
-      <c r="U5" s="10"/>
-      <c r="V5" s="73">
+      <c r="T5" s="54"/>
+      <c r="U5" s="65"/>
+      <c r="V5" s="54">
         <v>37</v>
       </c>
-      <c r="W5" s="10">
+      <c r="W5" s="65">
         <v>19</v>
       </c>
-      <c r="X5" s="73">
+      <c r="X5" s="54">
         <v>36</v>
       </c>
-      <c r="Y5" s="10">
+      <c r="Y5" s="65">
         <v>20</v>
       </c>
-      <c r="Z5" s="73">
+      <c r="Z5" s="54">
         <v>38</v>
       </c>
       <c r="AA5" s="65">
         <v>18</v>
       </c>
-      <c r="AB5" s="72">
+      <c r="AB5" s="54">
         <v>35</v>
       </c>
       <c r="AC5" s="65">
         <v>21</v>
       </c>
-      <c r="AD5" s="72">
+      <c r="AD5" s="55">
         <v>37</v>
       </c>
-      <c r="AE5" s="81">
+      <c r="AE5" s="63">
         <v>19</v>
       </c>
-      <c r="AF5" s="72">
+      <c r="AF5" s="55">
         <v>37</v>
       </c>
-      <c r="AG5" s="81">
+      <c r="AG5" s="63">
         <v>18</v>
       </c>
-      <c r="AH5" s="72">
+      <c r="AH5" s="55">
         <v>38</v>
       </c>
-      <c r="AI5" s="81">
+      <c r="AI5" s="63">
         <v>17</v>
       </c>
-      <c r="AJ5" s="99"/>
-      <c r="AK5" s="100"/>
-      <c r="AL5" s="72"/>
-      <c r="AM5" s="81"/>
-      <c r="AN5" s="49">
+      <c r="AJ5" s="126"/>
+      <c r="AK5" s="129"/>
+      <c r="AL5" s="55"/>
+      <c r="AM5" s="63"/>
+      <c r="AN5" s="36">
         <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5+AD5+AF5+AH5+AJ5+AL5</f>
         <v>335</v>
       </c>
-      <c r="AO5" s="49">
+      <c r="AO5" s="36">
         <f>COUNTIF(D5:AL5,"&gt;30")</f>
         <v>9</v>
       </c>
-      <c r="AP5" s="90">
+      <c r="AP5" s="72">
         <v>3</v>
       </c>
-      <c r="AQ5" s="83">
+      <c r="AQ5" s="65">
         <v>11</v>
       </c>
-      <c r="AR5" s="86">
+      <c r="AR5" s="68">
         <f>SUMIF(G5:AM5, "&lt;30")+AP5+AQ5</f>
         <v>181</v>
       </c>
-      <c r="AS5" s="56">
+      <c r="AS5" s="43">
         <f>AR5/AO5</f>
         <v>20.111111111111111</v>
       </c>
-      <c r="AT5" s="49"/>
-      <c r="AU5" s="34"/>
-      <c r="AV5" s="34"/>
-      <c r="AW5" s="11"/>
-      <c r="AX5" s="50"/>
+      <c r="AT5" s="36"/>
+      <c r="AU5" s="27"/>
+      <c r="AV5" s="27"/>
+      <c r="AW5" s="8"/>
+      <c r="AX5" s="37"/>
     </row>
     <row r="6" spans="1:50">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="118">
         <f>ROUND((AN6-(36*AO6))/AO6,0)</f>
         <v>6</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="54">
+      <c r="D6" s="126"/>
+      <c r="E6" s="129"/>
+      <c r="F6" s="41">
         <v>45</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="65">
         <v>17</v>
       </c>
-      <c r="H6" s="42"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="54">
+      <c r="H6" s="126"/>
+      <c r="I6" s="129"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="65"/>
+      <c r="L6" s="41">
         <v>43</v>
       </c>
-      <c r="M6" s="10">
+      <c r="M6" s="65">
         <v>19</v>
       </c>
-      <c r="N6" s="13">
+      <c r="N6" s="41">
         <v>41</v>
       </c>
-      <c r="O6" s="10">
+      <c r="O6" s="65">
         <v>21</v>
       </c>
-      <c r="P6" s="35">
+      <c r="P6" s="41">
         <v>47</v>
       </c>
-      <c r="Q6" s="10">
+      <c r="Q6" s="65">
         <v>15</v>
       </c>
-      <c r="R6" s="35">
+      <c r="R6" s="41">
         <v>42</v>
       </c>
-      <c r="S6" s="10">
+      <c r="S6" s="65">
         <v>20</v>
       </c>
-      <c r="T6" s="35">
+      <c r="T6" s="41">
         <v>43</v>
       </c>
-      <c r="U6" s="10">
+      <c r="U6" s="65">
         <v>19</v>
       </c>
-      <c r="V6" s="35">
+      <c r="V6" s="41">
         <v>44</v>
       </c>
-      <c r="W6" s="10">
+      <c r="W6" s="65">
         <v>18</v>
       </c>
-      <c r="X6" s="35">
+      <c r="X6" s="41">
         <v>48</v>
       </c>
-      <c r="Y6" s="10">
+      <c r="Y6" s="65">
         <v>16</v>
       </c>
-      <c r="Z6" s="35">
+      <c r="Z6" s="41">
         <v>40</v>
       </c>
       <c r="AA6" s="65">
         <v>22</v>
       </c>
-      <c r="AB6" s="35">
+      <c r="AB6" s="41">
         <v>40</v>
       </c>
       <c r="AC6" s="65">
         <v>22</v>
       </c>
-      <c r="AD6" s="35">
+      <c r="AD6" s="28">
         <v>38</v>
       </c>
-      <c r="AE6" s="81">
+      <c r="AE6" s="63">
         <v>23</v>
       </c>
-      <c r="AF6" s="68">
+      <c r="AF6" s="51">
         <v>41</v>
       </c>
-      <c r="AG6" s="81">
+      <c r="AG6" s="63">
         <v>20</v>
       </c>
-      <c r="AH6" s="59">
+      <c r="AH6" s="45">
         <v>40</v>
       </c>
-      <c r="AI6" s="81">
+      <c r="AI6" s="63">
         <v>21</v>
       </c>
-      <c r="AJ6" s="99"/>
-      <c r="AK6" s="100"/>
-      <c r="AL6" s="59"/>
-      <c r="AM6" s="81"/>
-      <c r="AN6" s="49">
+      <c r="AJ6" s="126"/>
+      <c r="AK6" s="129"/>
+      <c r="AL6" s="45"/>
+      <c r="AM6" s="63"/>
+      <c r="AN6" s="36">
         <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6+AD6+AF6+AH6+AJ6+AL6</f>
         <v>552</v>
       </c>
-      <c r="AO6" s="49">
+      <c r="AO6" s="36">
         <f>COUNTIF(D6:AL6,"&gt;30")</f>
         <v>13</v>
       </c>
-      <c r="AP6" s="90">
+      <c r="AP6" s="72">
         <v>2</v>
       </c>
-      <c r="AQ6" s="83">
+      <c r="AQ6" s="65">
         <v>5</v>
       </c>
-      <c r="AR6" s="86">
+      <c r="AR6" s="68">
         <f>SUMIF(G6:AM6, "&lt;30")+AP6+AQ6</f>
         <v>260</v>
       </c>
-      <c r="AS6" s="56">
+      <c r="AS6" s="43">
         <f>AR6/AO6</f>
         <v>20</v>
       </c>
-      <c r="AT6" s="49"/>
-      <c r="AU6" s="34"/>
-      <c r="AV6" s="34"/>
-      <c r="AW6" s="11"/>
-      <c r="AX6" s="50"/>
+      <c r="AT6" s="36"/>
+      <c r="AU6" s="27"/>
+      <c r="AV6" s="27"/>
+      <c r="AW6" s="8"/>
+      <c r="AX6" s="37"/>
     </row>
     <row r="7" spans="1:50">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="118">
         <f>ROUND((AN7-(36*AO7))/AO7,0)</f>
         <v>12</v>
       </c>
-      <c r="D7" s="42"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="61">
+      <c r="D7" s="126"/>
+      <c r="E7" s="129"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="126"/>
+      <c r="I7" s="129"/>
+      <c r="J7" s="9">
         <v>52</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K7" s="65">
         <v>17</v>
       </c>
-      <c r="L7" s="61"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="61">
+      <c r="L7" s="9"/>
+      <c r="M7" s="65"/>
+      <c r="N7" s="9">
         <v>46</v>
       </c>
-      <c r="O7" s="10">
+      <c r="O7" s="65">
         <v>23</v>
       </c>
-      <c r="P7" s="61">
+      <c r="P7" s="9">
         <v>46</v>
       </c>
-      <c r="Q7" s="10">
+      <c r="Q7" s="65">
         <v>23</v>
       </c>
-      <c r="R7" s="61">
+      <c r="R7" s="9">
         <v>54</v>
       </c>
-      <c r="S7" s="10">
+      <c r="S7" s="65">
         <v>16</v>
       </c>
-      <c r="T7" s="61">
+      <c r="T7" s="9">
         <v>45</v>
       </c>
-      <c r="U7" s="10">
+      <c r="U7" s="65">
         <v>23</v>
       </c>
-      <c r="V7" s="61">
+      <c r="V7" s="9">
         <v>48</v>
       </c>
-      <c r="W7" s="10">
+      <c r="W7" s="65">
         <v>19</v>
       </c>
-      <c r="X7" s="61">
+      <c r="X7" s="9">
         <v>49</v>
       </c>
-      <c r="Y7" s="10">
+      <c r="Y7" s="65">
         <v>18</v>
       </c>
-      <c r="Z7" s="66"/>
+      <c r="Z7" s="9"/>
       <c r="AA7" s="65"/>
-      <c r="AB7" s="66">
+      <c r="AB7" s="9">
         <v>46</v>
       </c>
       <c r="AC7" s="65">
         <v>21</v>
       </c>
-      <c r="AD7" s="69">
+      <c r="AD7" s="52">
         <v>43</v>
       </c>
-      <c r="AE7" s="81">
+      <c r="AE7" s="63">
         <v>23</v>
       </c>
-      <c r="AF7" s="66">
+      <c r="AF7" s="49">
         <v>47</v>
       </c>
-      <c r="AG7" s="81">
+      <c r="AG7" s="63">
         <v>19</v>
       </c>
-      <c r="AH7" s="66">
+      <c r="AH7" s="49">
         <v>51</v>
       </c>
-      <c r="AI7" s="81">
+      <c r="AI7" s="63">
         <v>15</v>
       </c>
-      <c r="AJ7" s="99"/>
-      <c r="AK7" s="100"/>
-      <c r="AL7" s="66">
+      <c r="AJ7" s="126"/>
+      <c r="AK7" s="129"/>
+      <c r="AL7" s="49">
         <v>50</v>
       </c>
-      <c r="AM7" s="81">
+      <c r="AM7" s="63">
         <v>16</v>
       </c>
-      <c r="AN7" s="49">
+      <c r="AN7" s="36">
         <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7+AD7+AF7+AH7+AJ7+AL7</f>
         <v>577</v>
       </c>
-      <c r="AO7" s="49">
+      <c r="AO7" s="36">
         <f>COUNTIF(D7:AL7,"&gt;30")</f>
         <v>12</v>
       </c>
-      <c r="AP7" s="90">
+      <c r="AP7" s="72">
         <v>1</v>
       </c>
-      <c r="AQ7" s="83">
+      <c r="AQ7" s="65">
         <v>1</v>
       </c>
-      <c r="AR7" s="86">
+      <c r="AR7" s="68">
         <f>SUMIF(G7:AM7, "&lt;30")+AP7+AQ7</f>
         <v>235</v>
       </c>
-      <c r="AS7" s="56">
+      <c r="AS7" s="43">
         <f>AR7/AO7</f>
         <v>19.583333333333332</v>
       </c>
-      <c r="AT7" s="49"/>
-      <c r="AU7" s="34"/>
-      <c r="AV7" s="34"/>
-      <c r="AW7" s="11"/>
-      <c r="AX7" s="50"/>
+      <c r="AT7" s="36"/>
+      <c r="AU7" s="27"/>
+      <c r="AV7" s="27"/>
+      <c r="AW7" s="8"/>
+      <c r="AX7" s="37"/>
     </row>
     <row r="8" spans="1:50">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="118">
         <f>ROUND((AN8-(36*AO8))/AO8,0)</f>
         <v>12</v>
       </c>
-      <c r="D8" s="42"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="12">
+      <c r="D8" s="126"/>
+      <c r="E8" s="129"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="126"/>
+      <c r="I8" s="129"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="65"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="65"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="65"/>
+      <c r="P8" s="9">
         <v>43</v>
       </c>
-      <c r="Q8" s="10">
+      <c r="Q8" s="65">
         <v>26</v>
       </c>
-      <c r="R8" s="58">
+      <c r="R8" s="9">
         <v>45</v>
       </c>
-      <c r="S8" s="10">
+      <c r="S8" s="65">
         <v>24</v>
       </c>
-      <c r="T8" s="59"/>
-      <c r="U8" s="10"/>
-      <c r="V8" s="59">
+      <c r="T8" s="9"/>
+      <c r="U8" s="65"/>
+      <c r="V8" s="9">
         <v>50</v>
       </c>
-      <c r="W8" s="10">
+      <c r="W8" s="65">
         <v>19</v>
       </c>
-      <c r="X8" s="59">
+      <c r="X8" s="9">
         <v>44</v>
       </c>
-      <c r="Y8" s="10">
+      <c r="Y8" s="65">
         <v>20</v>
       </c>
-      <c r="Z8" s="59"/>
+      <c r="Z8" s="9"/>
       <c r="AA8" s="65"/>
-      <c r="AB8" s="59">
+      <c r="AB8" s="9">
         <v>54</v>
       </c>
       <c r="AC8" s="65">
         <v>11</v>
       </c>
-      <c r="AD8" s="59"/>
-      <c r="AE8" s="81"/>
-      <c r="AF8" s="59">
+      <c r="AD8" s="45"/>
+      <c r="AE8" s="63"/>
+      <c r="AF8" s="45">
         <v>51</v>
       </c>
-      <c r="AG8" s="81">
+      <c r="AG8" s="63">
         <v>14</v>
       </c>
-      <c r="AH8" s="59"/>
-      <c r="AI8" s="81"/>
-      <c r="AJ8" s="99"/>
-      <c r="AK8" s="100"/>
-      <c r="AL8" s="134">
+      <c r="AH8" s="45"/>
+      <c r="AI8" s="63"/>
+      <c r="AJ8" s="126"/>
+      <c r="AK8" s="129"/>
+      <c r="AL8" s="110">
         <v>46</v>
       </c>
-      <c r="AM8" s="81">
+      <c r="AM8" s="63">
         <v>20</v>
       </c>
-      <c r="AN8" s="49">
+      <c r="AN8" s="36">
         <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8+AD8+AF8+AH8+AJ8+AL8</f>
         <v>333</v>
       </c>
-      <c r="AO8" s="49">
+      <c r="AO8" s="36">
         <f>COUNTIF(D8:AL8,"&gt;30")</f>
         <v>7</v>
       </c>
-      <c r="AP8" s="90">
+      <c r="AP8" s="72">
         <v>2</v>
       </c>
-      <c r="AQ8" s="83">
+      <c r="AQ8" s="65">
         <v>1</v>
       </c>
-      <c r="AR8" s="86">
+      <c r="AR8" s="68">
         <f>SUMIF(G8:AM8, "&lt;30")+AP8+AQ8</f>
         <v>137</v>
       </c>
-      <c r="AS8" s="56">
+      <c r="AS8" s="43">
         <f>AR8/AO8</f>
         <v>19.571428571428573</v>
       </c>
-      <c r="AT8" s="75"/>
-      <c r="AU8" s="34"/>
-      <c r="AV8" s="34"/>
-      <c r="AW8" s="11"/>
-      <c r="AX8" s="50"/>
+      <c r="AT8" s="57"/>
+      <c r="AU8" s="27"/>
+      <c r="AV8" s="27"/>
+      <c r="AW8" s="8"/>
+      <c r="AX8" s="37"/>
     </row>
     <row r="9" spans="1:50">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="118">
         <f>ROUND((AN9-(36*AO9))/AO9,0)</f>
         <v>7</v>
       </c>
-      <c r="D9" s="42"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="12">
+      <c r="D9" s="126"/>
+      <c r="E9" s="129"/>
+      <c r="F9" s="9">
         <v>41</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="65">
         <v>21</v>
       </c>
-      <c r="H9" s="42"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="46">
+      <c r="H9" s="126"/>
+      <c r="I9" s="129"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="65"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="65"/>
+      <c r="N9" s="9">
         <v>48</v>
       </c>
-      <c r="O9" s="10">
+      <c r="O9" s="65">
         <v>14</v>
       </c>
-      <c r="P9" s="35">
+      <c r="P9" s="9">
         <v>44</v>
       </c>
-      <c r="Q9" s="10">
+      <c r="Q9" s="65">
         <v>18</v>
       </c>
-      <c r="R9" s="35"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="35"/>
-      <c r="U9" s="10"/>
-      <c r="V9" s="35"/>
-      <c r="W9" s="10"/>
-      <c r="X9" s="13">
+      <c r="R9" s="9"/>
+      <c r="S9" s="65"/>
+      <c r="T9" s="9"/>
+      <c r="U9" s="65"/>
+      <c r="V9" s="9"/>
+      <c r="W9" s="65"/>
+      <c r="X9" s="9">
         <v>40</v>
       </c>
-      <c r="Y9" s="10">
+      <c r="Y9" s="65">
         <v>22</v>
       </c>
-      <c r="Z9" s="35">
+      <c r="Z9" s="9">
         <v>44</v>
       </c>
       <c r="AA9" s="65">
         <v>17</v>
       </c>
-      <c r="AB9" s="35">
+      <c r="AB9" s="9">
         <v>46</v>
       </c>
       <c r="AC9" s="65">
         <v>16</v>
       </c>
-      <c r="AD9" s="46">
+      <c r="AD9" s="33">
         <v>42</v>
       </c>
-      <c r="AE9" s="81">
+      <c r="AE9" s="63">
         <v>20</v>
       </c>
-      <c r="AF9" s="35">
+      <c r="AF9" s="28">
         <v>44</v>
       </c>
-      <c r="AG9" s="81">
+      <c r="AG9" s="63">
         <v>18</v>
       </c>
-      <c r="AH9" s="46">
+      <c r="AH9" s="33">
         <v>39</v>
       </c>
-      <c r="AI9" s="81">
+      <c r="AI9" s="63">
         <v>23</v>
       </c>
-      <c r="AJ9" s="99"/>
-      <c r="AK9" s="100"/>
-      <c r="AL9" s="135"/>
-      <c r="AM9" s="81"/>
-      <c r="AN9" s="49">
+      <c r="AJ9" s="126"/>
+      <c r="AK9" s="129"/>
+      <c r="AL9" s="131"/>
+      <c r="AM9" s="63"/>
+      <c r="AN9" s="36">
         <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9+AD9+AF9+AH9+AJ9+AL9</f>
         <v>388</v>
       </c>
-      <c r="AO9" s="49">
+      <c r="AO9" s="36">
         <f>COUNTIF(D9:AL9,"&gt;30")</f>
         <v>9</v>
       </c>
-      <c r="AP9" s="90">
+      <c r="AP9" s="72">
         <v>3</v>
       </c>
-      <c r="AQ9" s="83">
+      <c r="AQ9" s="65">
         <v>3</v>
       </c>
-      <c r="AR9" s="86">
+      <c r="AR9" s="68">
         <f>SUMIF(G9:AM9, "&lt;30")+AP9+AQ9</f>
         <v>175</v>
       </c>
-      <c r="AS9" s="56">
+      <c r="AS9" s="43">
         <f>AR9/AO9</f>
         <v>19.444444444444443</v>
       </c>
-      <c r="AT9" s="51"/>
-      <c r="AU9" s="34"/>
-      <c r="AV9" s="34"/>
-      <c r="AW9" s="11"/>
-      <c r="AX9" s="50"/>
+      <c r="AT9" s="38"/>
+      <c r="AU9" s="27"/>
+      <c r="AV9" s="27"/>
+      <c r="AW9" s="8"/>
+      <c r="AX9" s="37"/>
     </row>
     <row r="10" spans="1:50">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="118">
         <f>ROUND((AN10-(36*AO10))/AO10,0)</f>
         <v>14</v>
       </c>
-      <c r="D10" s="42"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="12">
+      <c r="D10" s="126"/>
+      <c r="E10" s="129"/>
+      <c r="F10" s="9">
         <v>42</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="65">
         <v>27</v>
       </c>
-      <c r="H10" s="42"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="12">
+      <c r="H10" s="126"/>
+      <c r="I10" s="129"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="65"/>
+      <c r="L10" s="9">
         <v>54</v>
       </c>
-      <c r="M10" s="10">
+      <c r="M10" s="65">
         <v>15</v>
       </c>
-      <c r="N10" s="12"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="12">
+      <c r="N10" s="9"/>
+      <c r="O10" s="65"/>
+      <c r="P10" s="9">
         <v>54</v>
       </c>
-      <c r="Q10" s="10">
+      <c r="Q10" s="65">
         <v>16</v>
       </c>
-      <c r="R10" s="12">
+      <c r="R10" s="9">
         <v>53</v>
       </c>
-      <c r="S10" s="10">
+      <c r="S10" s="65">
         <v>16</v>
       </c>
-      <c r="T10" s="12"/>
-      <c r="U10" s="10"/>
-      <c r="V10" s="58">
+      <c r="T10" s="9"/>
+      <c r="U10" s="65"/>
+      <c r="V10" s="9">
         <v>46</v>
       </c>
-      <c r="W10" s="10">
+      <c r="W10" s="65">
         <v>23</v>
       </c>
-      <c r="X10" s="59">
+      <c r="X10" s="9">
         <v>49</v>
       </c>
-      <c r="Y10" s="10">
+      <c r="Y10" s="65">
         <v>19</v>
       </c>
-      <c r="Z10" s="59">
+      <c r="Z10" s="9">
         <v>50</v>
       </c>
       <c r="AA10" s="65">
         <v>18</v>
       </c>
-      <c r="AB10" s="59"/>
+      <c r="AB10" s="9"/>
       <c r="AC10" s="65"/>
-      <c r="AD10" s="59"/>
-      <c r="AE10" s="81"/>
-      <c r="AF10" s="59"/>
-      <c r="AG10" s="81"/>
-      <c r="AH10" s="59">
+      <c r="AD10" s="45"/>
+      <c r="AE10" s="63"/>
+      <c r="AF10" s="45"/>
+      <c r="AG10" s="63"/>
+      <c r="AH10" s="45">
         <v>50</v>
       </c>
-      <c r="AI10" s="81">
+      <c r="AI10" s="63">
         <v>18</v>
       </c>
-      <c r="AJ10" s="99"/>
-      <c r="AK10" s="100"/>
-      <c r="AL10" s="59">
+      <c r="AJ10" s="126"/>
+      <c r="AK10" s="129"/>
+      <c r="AL10" s="45">
         <v>50</v>
       </c>
-      <c r="AM10" s="81">
+      <c r="AM10" s="63">
         <v>18</v>
       </c>
-      <c r="AN10" s="49">
+      <c r="AN10" s="36">
         <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10+AD10+AF10+AH10+AJ10+AL10</f>
         <v>448</v>
       </c>
-      <c r="AO10" s="49">
+      <c r="AO10" s="36">
         <f>COUNTIF(D10:AL10,"&gt;30")</f>
         <v>9</v>
       </c>
-      <c r="AP10" s="90">
+      <c r="AP10" s="72">
         <v>1</v>
       </c>
-      <c r="AQ10" s="83">
+      <c r="AQ10" s="65">
         <v>1</v>
       </c>
-      <c r="AR10" s="86">
+      <c r="AR10" s="68">
         <f>SUMIF(G10:AM10, "&lt;30")+AP10+AQ10</f>
         <v>172</v>
       </c>
-      <c r="AS10" s="56">
+      <c r="AS10" s="43">
         <f>AR10/AO10</f>
         <v>19.111111111111111</v>
       </c>
-      <c r="AT10" s="76"/>
-      <c r="AU10" s="34"/>
-      <c r="AV10" s="34"/>
-      <c r="AW10" s="11"/>
-      <c r="AX10" s="50"/>
+      <c r="AT10" s="58"/>
+      <c r="AU10" s="27"/>
+      <c r="AV10" s="27"/>
+      <c r="AW10" s="8"/>
+      <c r="AX10" s="37"/>
     </row>
     <row r="11" spans="1:50">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="118">
         <f>ROUND((AN11-(36*AO11))/AO11,0)</f>
         <v>11</v>
       </c>
-      <c r="D11" s="42"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="60">
+      <c r="D11" s="126"/>
+      <c r="E11" s="129"/>
+      <c r="F11" s="46">
         <v>42</v>
       </c>
-      <c r="G11" s="10">
+      <c r="G11" s="65">
         <v>25</v>
       </c>
-      <c r="H11" s="42"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="35">
+      <c r="H11" s="126"/>
+      <c r="I11" s="129"/>
+      <c r="J11" s="46"/>
+      <c r="K11" s="65"/>
+      <c r="L11" s="46">
         <v>51</v>
       </c>
-      <c r="M11" s="10">
+      <c r="M11" s="65">
         <v>16</v>
       </c>
-      <c r="N11" s="35"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="13">
+      <c r="N11" s="46"/>
+      <c r="O11" s="65"/>
+      <c r="P11" s="46">
         <v>49</v>
       </c>
-      <c r="Q11" s="10">
+      <c r="Q11" s="65">
         <v>18</v>
       </c>
-      <c r="R11" s="35">
+      <c r="R11" s="46">
         <v>46</v>
       </c>
-      <c r="S11" s="10">
+      <c r="S11" s="65">
         <v>21</v>
       </c>
-      <c r="T11" s="35">
+      <c r="T11" s="46">
         <v>45</v>
       </c>
-      <c r="U11" s="10">
+      <c r="U11" s="65">
         <v>20</v>
       </c>
-      <c r="V11" s="35">
+      <c r="V11" s="46">
         <v>46</v>
       </c>
-      <c r="W11" s="10">
+      <c r="W11" s="65">
         <v>19</v>
       </c>
-      <c r="X11" s="35">
+      <c r="X11" s="46">
         <v>53</v>
       </c>
-      <c r="Y11" s="10">
+      <c r="Y11" s="65">
         <v>13</v>
       </c>
-      <c r="Z11" s="35">
+      <c r="Z11" s="46">
         <v>52</v>
       </c>
       <c r="AA11" s="65">
         <v>13</v>
       </c>
-      <c r="AB11" s="35">
+      <c r="AB11" s="46">
         <v>44</v>
       </c>
       <c r="AC11" s="65">
         <v>22</v>
       </c>
-      <c r="AD11" s="35">
+      <c r="AD11" s="28">
         <v>42</v>
       </c>
-      <c r="AE11" s="81">
+      <c r="AE11" s="63">
         <v>24</v>
       </c>
-      <c r="AF11" s="35">
+      <c r="AF11" s="28">
         <v>45</v>
       </c>
-      <c r="AG11" s="81">
+      <c r="AG11" s="63">
         <v>20</v>
       </c>
-      <c r="AH11" s="35">
+      <c r="AH11" s="28">
         <v>48</v>
       </c>
-      <c r="AI11" s="81">
+      <c r="AI11" s="63">
         <v>17</v>
       </c>
-      <c r="AJ11" s="99"/>
-      <c r="AK11" s="100"/>
-      <c r="AL11" s="35">
+      <c r="AJ11" s="126"/>
+      <c r="AK11" s="129"/>
+      <c r="AL11" s="28">
         <v>50</v>
       </c>
-      <c r="AM11" s="81">
+      <c r="AM11" s="63">
         <v>15</v>
       </c>
-      <c r="AN11" s="49">
+      <c r="AN11" s="36">
         <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11+AD11+AF11+AH11+AJ11+AL11</f>
         <v>613</v>
       </c>
-      <c r="AO11" s="49">
+      <c r="AO11" s="36">
         <f>COUNTIF(D11:AL11,"&gt;30")</f>
         <v>13</v>
       </c>
-      <c r="AP11" s="90">
+      <c r="AP11" s="72">
         <v>2</v>
       </c>
-      <c r="AQ11" s="83">
+      <c r="AQ11" s="65">
         <v>2</v>
       </c>
-      <c r="AR11" s="86">
+      <c r="AR11" s="68">
         <f>SUMIF(G11:AM11, "&lt;30")+AP11+AQ11</f>
         <v>247</v>
       </c>
-      <c r="AS11" s="56">
+      <c r="AS11" s="43">
         <f>AR11/AO11</f>
         <v>19</v>
       </c>
-      <c r="AT11" s="49"/>
-      <c r="AU11" s="34"/>
-      <c r="AV11" s="34"/>
-      <c r="AW11" s="11"/>
-      <c r="AX11" s="50"/>
+      <c r="AT11" s="36"/>
+      <c r="AU11" s="27"/>
+      <c r="AV11" s="27"/>
+      <c r="AW11" s="8"/>
+      <c r="AX11" s="37"/>
     </row>
     <row r="12" spans="1:50">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="118">
         <f>ROUND((AN12-(36*AO12))/AO12,0)</f>
         <v>15</v>
       </c>
-      <c r="D12" s="42"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="12">
+      <c r="D12" s="126"/>
+      <c r="E12" s="129"/>
+      <c r="F12" s="9">
         <v>51</v>
       </c>
-      <c r="G12" s="10">
+      <c r="G12" s="65">
         <v>18</v>
       </c>
-      <c r="H12" s="42"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="12">
+      <c r="H12" s="126"/>
+      <c r="I12" s="129"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="65"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="65"/>
+      <c r="N12" s="9">
         <v>51</v>
       </c>
-      <c r="O12" s="10">
+      <c r="O12" s="65">
         <v>18</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="9">
         <v>52</v>
       </c>
-      <c r="Q12" s="10">
+      <c r="Q12" s="65">
         <v>17</v>
       </c>
-      <c r="R12" s="12"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="12"/>
-      <c r="U12" s="10"/>
-      <c r="V12" s="12"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="12">
+      <c r="R12" s="9"/>
+      <c r="S12" s="65"/>
+      <c r="T12" s="9"/>
+      <c r="U12" s="65"/>
+      <c r="V12" s="9"/>
+      <c r="W12" s="65"/>
+      <c r="X12" s="9">
         <v>48</v>
       </c>
-      <c r="Y12" s="10">
+      <c r="Y12" s="65">
         <v>21</v>
       </c>
-      <c r="Z12" s="59"/>
+      <c r="Z12" s="9"/>
       <c r="AA12" s="65"/>
-      <c r="AB12" s="59">
+      <c r="AB12" s="9">
         <v>51</v>
       </c>
       <c r="AC12" s="65">
         <v>18</v>
       </c>
-      <c r="AD12" s="59"/>
-      <c r="AE12" s="81"/>
-      <c r="AF12" s="59"/>
-      <c r="AG12" s="81"/>
-      <c r="AH12" s="59"/>
-      <c r="AI12" s="81"/>
-      <c r="AJ12" s="99"/>
-      <c r="AK12" s="100"/>
-      <c r="AL12" s="59"/>
-      <c r="AM12" s="81"/>
-      <c r="AN12" s="49">
+      <c r="AD12" s="45"/>
+      <c r="AE12" s="63"/>
+      <c r="AF12" s="45"/>
+      <c r="AG12" s="63"/>
+      <c r="AH12" s="45"/>
+      <c r="AI12" s="63"/>
+      <c r="AJ12" s="126"/>
+      <c r="AK12" s="129"/>
+      <c r="AL12" s="45"/>
+      <c r="AM12" s="63"/>
+      <c r="AN12" s="36">
         <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12+AD12+AF12+AH12+AJ12+AL12</f>
         <v>253</v>
       </c>
-      <c r="AO12" s="49">
+      <c r="AO12" s="36">
         <f>COUNTIF(D12:AL12,"&gt;30")</f>
         <v>5</v>
       </c>
-      <c r="AP12" s="90"/>
-      <c r="AQ12" s="83"/>
-      <c r="AR12" s="86">
+      <c r="AP12" s="72"/>
+      <c r="AQ12" s="65"/>
+      <c r="AR12" s="68">
         <f>SUMIF(G12:AM12, "&lt;30")+AP12+AQ12</f>
         <v>92</v>
       </c>
-      <c r="AS12" s="56">
+      <c r="AS12" s="43">
         <f>AR12/AO12</f>
         <v>18.399999999999999</v>
       </c>
-      <c r="AT12" s="51"/>
-      <c r="AU12" s="34"/>
-      <c r="AV12" s="34"/>
-      <c r="AW12" s="11"/>
-      <c r="AX12" s="50"/>
+      <c r="AT12" s="38"/>
+      <c r="AU12" s="27"/>
+      <c r="AV12" s="27"/>
+      <c r="AW12" s="8"/>
+      <c r="AX12" s="37"/>
     </row>
     <row r="13" spans="1:50">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="118">
         <f>ROUND((AN13-(36*AO13))/AO13,0)</f>
         <v>22</v>
       </c>
-      <c r="D13" s="42"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="12">
+      <c r="D13" s="126"/>
+      <c r="E13" s="129"/>
+      <c r="F13" s="9">
         <v>59</v>
       </c>
-      <c r="G13" s="10">
+      <c r="G13" s="65">
         <v>17</v>
       </c>
-      <c r="H13" s="42"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="12">
+      <c r="H13" s="126"/>
+      <c r="I13" s="129"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="65"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="65"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="65"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="65"/>
+      <c r="R13" s="9">
         <v>55</v>
       </c>
-      <c r="S13" s="10">
+      <c r="S13" s="65">
         <v>21</v>
       </c>
-      <c r="T13" s="12"/>
-      <c r="U13" s="10"/>
-      <c r="V13" s="12">
+      <c r="T13" s="9"/>
+      <c r="U13" s="65"/>
+      <c r="V13" s="9">
         <v>59</v>
       </c>
-      <c r="W13" s="10">
+      <c r="W13" s="65">
         <v>17</v>
       </c>
-      <c r="X13" s="12"/>
-      <c r="Y13" s="10"/>
-      <c r="Z13" s="59"/>
+      <c r="X13" s="9"/>
+      <c r="Y13" s="65"/>
+      <c r="Z13" s="9"/>
       <c r="AA13" s="65"/>
-      <c r="AB13" s="59"/>
+      <c r="AB13" s="9"/>
       <c r="AC13" s="65"/>
-      <c r="AD13" s="59"/>
-      <c r="AE13" s="81"/>
-      <c r="AF13" s="59"/>
-      <c r="AG13" s="81"/>
-      <c r="AH13" s="59"/>
-      <c r="AI13" s="81"/>
-      <c r="AJ13" s="99"/>
-      <c r="AK13" s="100"/>
-      <c r="AL13" s="59"/>
-      <c r="AM13" s="81"/>
-      <c r="AN13" s="49">
+      <c r="AD13" s="45"/>
+      <c r="AE13" s="63"/>
+      <c r="AF13" s="45"/>
+      <c r="AG13" s="63"/>
+      <c r="AH13" s="45"/>
+      <c r="AI13" s="63"/>
+      <c r="AJ13" s="126"/>
+      <c r="AK13" s="129"/>
+      <c r="AL13" s="45"/>
+      <c r="AM13" s="63"/>
+      <c r="AN13" s="36">
         <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13+AD13+AF13+AH13+AJ13+AL13</f>
         <v>173</v>
       </c>
-      <c r="AO13" s="49">
+      <c r="AO13" s="36">
         <f>COUNTIF(D13:AL13,"&gt;30")</f>
         <v>3</v>
       </c>
-      <c r="AP13" s="90"/>
-      <c r="AQ13" s="83"/>
-      <c r="AR13" s="86">
+      <c r="AP13" s="72"/>
+      <c r="AQ13" s="65"/>
+      <c r="AR13" s="68">
         <f>SUMIF(G13:AM13, "&lt;30")+AP13+AQ13</f>
         <v>55</v>
       </c>
-      <c r="AS13" s="56">
+      <c r="AS13" s="43">
         <f>AR13/AO13</f>
         <v>18.333333333333332</v>
       </c>
-      <c r="AT13" s="51"/>
-      <c r="AU13" s="34"/>
-      <c r="AV13" s="34"/>
-      <c r="AW13" s="11"/>
-      <c r="AX13" s="50"/>
+      <c r="AT13" s="38"/>
+      <c r="AU13" s="27"/>
+      <c r="AV13" s="27"/>
+      <c r="AW13" s="8"/>
+      <c r="AX13" s="37"/>
     </row>
     <row r="14" spans="1:50">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="118">
         <f>ROUND((AN14-(36*AO14))/AO14,0)</f>
         <v>13</v>
       </c>
-      <c r="D14" s="42"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="12">
+      <c r="D14" s="126"/>
+      <c r="E14" s="129"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="126"/>
+      <c r="I14" s="129"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="65"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="65"/>
+      <c r="P14" s="9">
         <v>48</v>
       </c>
-      <c r="Q14" s="10">
+      <c r="Q14" s="65">
         <v>18</v>
       </c>
-      <c r="R14" s="12">
+      <c r="R14" s="9">
         <v>51</v>
       </c>
-      <c r="S14" s="10">
+      <c r="S14" s="65">
         <v>14</v>
       </c>
-      <c r="T14" s="12">
+      <c r="T14" s="9">
         <v>51</v>
       </c>
-      <c r="U14" s="10">
+      <c r="U14" s="65">
         <v>14</v>
       </c>
-      <c r="V14" s="12"/>
-      <c r="W14" s="10"/>
-      <c r="X14" s="12">
+      <c r="V14" s="9"/>
+      <c r="W14" s="65"/>
+      <c r="X14" s="9">
         <v>48</v>
       </c>
-      <c r="Y14" s="10">
+      <c r="Y14" s="65">
         <v>20</v>
       </c>
-      <c r="Z14" s="12">
+      <c r="Z14" s="9">
         <v>50</v>
       </c>
-      <c r="AA14" s="10">
+      <c r="AA14" s="65">
         <v>18</v>
       </c>
-      <c r="AB14" s="59">
+      <c r="AB14" s="9">
         <v>47</v>
       </c>
       <c r="AC14" s="65">
         <v>21</v>
       </c>
-      <c r="AD14" s="59"/>
-      <c r="AE14" s="81"/>
-      <c r="AF14" s="59">
+      <c r="AD14" s="45"/>
+      <c r="AE14" s="63"/>
+      <c r="AF14" s="45">
         <v>46</v>
       </c>
-      <c r="AG14" s="81">
+      <c r="AG14" s="63">
         <v>21</v>
       </c>
-      <c r="AH14" s="59">
+      <c r="AH14" s="45">
         <v>48</v>
       </c>
-      <c r="AI14" s="81">
+      <c r="AI14" s="63">
         <v>19</v>
       </c>
-      <c r="AJ14" s="99"/>
-      <c r="AK14" s="100"/>
-      <c r="AL14" s="59"/>
-      <c r="AM14" s="81"/>
-      <c r="AN14" s="49">
+      <c r="AJ14" s="126"/>
+      <c r="AK14" s="129"/>
+      <c r="AL14" s="45"/>
+      <c r="AM14" s="63"/>
+      <c r="AN14" s="36">
         <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14+AD14+AF14+AH14+AJ14+AL14</f>
         <v>389</v>
       </c>
-      <c r="AO14" s="49">
+      <c r="AO14" s="36">
         <f>COUNTIF(D14:AL14,"&gt;30")</f>
         <v>8</v>
       </c>
-      <c r="AP14" s="90"/>
-      <c r="AQ14" s="83">
+      <c r="AP14" s="72"/>
+      <c r="AQ14" s="65">
         <v>1</v>
       </c>
-      <c r="AR14" s="86">
+      <c r="AR14" s="68">
         <f>SUMIF(G14:AM14, "&lt;30")+AP14+AQ14</f>
         <v>146</v>
       </c>
-      <c r="AS14" s="56">
+      <c r="AS14" s="43">
         <f>AR14/AO14</f>
         <v>18.25</v>
       </c>
-      <c r="AT14" s="49"/>
-      <c r="AU14" s="34"/>
-      <c r="AV14" s="34"/>
-      <c r="AW14" s="11"/>
-      <c r="AX14" s="50"/>
+      <c r="AT14" s="36"/>
+      <c r="AU14" s="27"/>
+      <c r="AV14" s="27"/>
+      <c r="AW14" s="8"/>
+      <c r="AX14" s="37"/>
     </row>
     <row r="15" spans="1:50">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="118">
         <f>ROUND((AN15-(36*AO15))/AO15,0)</f>
         <v>9</v>
       </c>
-      <c r="D15" s="42"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="12">
+      <c r="D15" s="126"/>
+      <c r="E15" s="129"/>
+      <c r="F15" s="9">
         <v>46</v>
       </c>
-      <c r="G15" s="10">
+      <c r="G15" s="65">
         <v>16</v>
       </c>
-      <c r="H15" s="42"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="12">
+      <c r="H15" s="126"/>
+      <c r="I15" s="129"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="65"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="65"/>
+      <c r="N15" s="9">
         <v>42</v>
       </c>
-      <c r="O15" s="10">
+      <c r="O15" s="65">
         <v>20</v>
       </c>
-      <c r="P15" s="12">
+      <c r="P15" s="9">
         <v>43</v>
       </c>
-      <c r="Q15" s="10">
+      <c r="Q15" s="65">
         <v>19</v>
       </c>
-      <c r="R15" s="12"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="10"/>
-      <c r="V15" s="12"/>
-      <c r="W15" s="10"/>
-      <c r="X15" s="12">
+      <c r="R15" s="9"/>
+      <c r="S15" s="65"/>
+      <c r="T15" s="9"/>
+      <c r="U15" s="65"/>
+      <c r="V15" s="9"/>
+      <c r="W15" s="65"/>
+      <c r="X15" s="9">
         <v>47</v>
       </c>
-      <c r="Y15" s="10">
+      <c r="Y15" s="65">
         <v>16</v>
       </c>
-      <c r="Z15" s="58">
+      <c r="Z15" s="9">
         <v>41</v>
       </c>
       <c r="AA15" s="65">
         <v>22</v>
       </c>
-      <c r="AB15" s="68">
+      <c r="AB15" s="9">
         <v>50</v>
       </c>
       <c r="AC15" s="65">
         <v>13</v>
       </c>
-      <c r="AD15" s="59">
+      <c r="AD15" s="45">
         <v>44</v>
       </c>
-      <c r="AE15" s="81">
+      <c r="AE15" s="63">
         <v>19</v>
       </c>
-      <c r="AF15" s="59">
+      <c r="AF15" s="45">
         <v>43</v>
       </c>
-      <c r="AG15" s="81">
+      <c r="AG15" s="63">
         <v>20</v>
       </c>
-      <c r="AH15" s="59">
+      <c r="AH15" s="45">
         <v>49</v>
       </c>
-      <c r="AI15" s="81">
+      <c r="AI15" s="63">
         <v>15</v>
       </c>
-      <c r="AJ15" s="99"/>
-      <c r="AK15" s="100"/>
-      <c r="AL15" s="59"/>
-      <c r="AM15" s="81"/>
-      <c r="AN15" s="49">
+      <c r="AJ15" s="126"/>
+      <c r="AK15" s="129"/>
+      <c r="AL15" s="45"/>
+      <c r="AM15" s="63"/>
+      <c r="AN15" s="36">
         <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15+AD15+AF15+AH15+AJ15+AL15</f>
         <v>405</v>
       </c>
-      <c r="AO15" s="49">
+      <c r="AO15" s="36">
         <f>COUNTIF(D15:AL15,"&gt;30")</f>
         <v>9</v>
       </c>
-      <c r="AP15" s="90">
+      <c r="AP15" s="72">
         <v>2</v>
       </c>
-      <c r="AQ15" s="83">
+      <c r="AQ15" s="65">
         <v>1</v>
       </c>
-      <c r="AR15" s="86">
+      <c r="AR15" s="68">
         <f>SUMIF(G15:AM15, "&lt;30")+AP15+AQ15</f>
         <v>163</v>
       </c>
-      <c r="AS15" s="56">
+      <c r="AS15" s="43">
         <f>AR15/AO15</f>
         <v>18.111111111111111</v>
       </c>
-      <c r="AT15" s="51"/>
-      <c r="AU15" s="34"/>
-      <c r="AV15" s="34"/>
-      <c r="AW15" s="11"/>
-      <c r="AX15" s="50"/>
+      <c r="AT15" s="38"/>
+      <c r="AU15" s="27"/>
+      <c r="AV15" s="27"/>
+      <c r="AW15" s="8"/>
+      <c r="AX15" s="37"/>
     </row>
     <row r="16" spans="1:50">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="118">
         <f>ROUND((AN16-(36*AO16))/AO16,0)</f>
         <v>12</v>
       </c>
-      <c r="D16" s="42"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="35">
+      <c r="D16" s="126"/>
+      <c r="E16" s="129"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="126"/>
+      <c r="I16" s="129"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="65"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="65"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="65"/>
+      <c r="P16" s="11">
         <v>47</v>
       </c>
-      <c r="Q16" s="10">
+      <c r="Q16" s="65">
         <v>20</v>
       </c>
-      <c r="R16" s="35">
+      <c r="R16" s="11">
         <v>50</v>
       </c>
-      <c r="S16" s="10">
+      <c r="S16" s="65">
         <v>17</v>
       </c>
-      <c r="T16" s="35">
+      <c r="T16" s="11">
         <v>46</v>
       </c>
-      <c r="U16" s="10">
+      <c r="U16" s="65">
         <v>21</v>
       </c>
-      <c r="V16" s="35">
+      <c r="V16" s="11">
         <v>47</v>
       </c>
-      <c r="W16" s="10">
+      <c r="W16" s="65">
         <v>19</v>
       </c>
-      <c r="X16" s="35">
+      <c r="X16" s="11">
         <v>44</v>
       </c>
-      <c r="Y16" s="10">
+      <c r="Y16" s="65">
         <v>22</v>
       </c>
-      <c r="Z16" s="35">
+      <c r="Z16" s="11">
         <v>52</v>
       </c>
       <c r="AA16" s="65">
         <v>14</v>
       </c>
-      <c r="AB16" s="35">
+      <c r="AB16" s="11">
         <v>47</v>
       </c>
       <c r="AC16" s="65">
         <v>19</v>
       </c>
-      <c r="AD16" s="35">
+      <c r="AD16" s="28">
         <v>51</v>
       </c>
-      <c r="AE16" s="81">
+      <c r="AE16" s="63">
         <v>15</v>
       </c>
-      <c r="AF16" s="35">
+      <c r="AF16" s="28">
         <v>49</v>
       </c>
-      <c r="AG16" s="81">
+      <c r="AG16" s="63">
         <v>17</v>
       </c>
-      <c r="AH16" s="35">
+      <c r="AH16" s="28">
         <v>46</v>
       </c>
-      <c r="AI16" s="81">
+      <c r="AI16" s="63">
         <v>20</v>
       </c>
-      <c r="AJ16" s="99"/>
-      <c r="AK16" s="100"/>
-      <c r="AL16" s="35">
+      <c r="AJ16" s="126"/>
+      <c r="AK16" s="129"/>
+      <c r="AL16" s="28">
         <v>51</v>
       </c>
-      <c r="AM16" s="81">
+      <c r="AM16" s="63">
         <v>15</v>
       </c>
-      <c r="AN16" s="49">
+      <c r="AN16" s="36">
         <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16+AD16+AF16+AH16+AJ16+AL16</f>
         <v>530</v>
       </c>
-      <c r="AO16" s="49">
+      <c r="AO16" s="36">
         <f>COUNTIF(D16:AL16,"&gt;30")</f>
         <v>11</v>
       </c>
-      <c r="AP16" s="90"/>
-      <c r="AQ16" s="83"/>
-      <c r="AR16" s="86">
+      <c r="AP16" s="72"/>
+      <c r="AQ16" s="65"/>
+      <c r="AR16" s="68">
         <f>SUMIF(G16:AM16, "&lt;30")+AP16+AQ16</f>
         <v>199</v>
       </c>
-      <c r="AS16" s="56">
+      <c r="AS16" s="43">
         <f>AR16/AO16</f>
         <v>18.09090909090909</v>
       </c>
-      <c r="AT16" s="49"/>
-      <c r="AU16" s="34"/>
-      <c r="AV16" s="34"/>
-      <c r="AW16" s="11"/>
-      <c r="AX16" s="50"/>
+      <c r="AT16" s="36"/>
+      <c r="AU16" s="27"/>
+      <c r="AV16" s="27"/>
+      <c r="AW16" s="8"/>
+      <c r="AX16" s="37"/>
     </row>
     <row r="17" spans="1:50">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="118">
         <f>ROUND((AN17-(36*AO17))/AO17,0)</f>
         <v>18</v>
       </c>
-      <c r="D17" s="42"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="12">
+      <c r="D17" s="126"/>
+      <c r="E17" s="129"/>
+      <c r="F17" s="9">
         <v>55</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="65">
         <v>16</v>
       </c>
-      <c r="H17" s="42"/>
-      <c r="I17" s="43"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="12">
+      <c r="H17" s="126"/>
+      <c r="I17" s="129"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="65"/>
+      <c r="L17" s="9">
         <v>56</v>
       </c>
-      <c r="M17" s="10">
+      <c r="M17" s="65">
         <v>15</v>
       </c>
-      <c r="N17" s="12">
+      <c r="N17" s="9">
         <v>57</v>
       </c>
-      <c r="O17" s="10">
+      <c r="O17" s="65">
         <v>14</v>
       </c>
-      <c r="P17" s="12"/>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="12"/>
-      <c r="S17" s="10"/>
-      <c r="T17" s="58">
+      <c r="P17" s="9"/>
+      <c r="Q17" s="65"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="65"/>
+      <c r="T17" s="9">
         <v>49</v>
       </c>
-      <c r="U17" s="10">
+      <c r="U17" s="65">
         <v>22</v>
       </c>
-      <c r="V17" s="58">
+      <c r="V17" s="9">
         <v>58</v>
       </c>
-      <c r="W17" s="10">
+      <c r="W17" s="65">
         <v>14</v>
       </c>
-      <c r="X17" s="59">
+      <c r="X17" s="9">
         <v>50</v>
       </c>
-      <c r="Y17" s="10">
+      <c r="Y17" s="65">
         <v>23</v>
       </c>
-      <c r="Z17" s="59">
+      <c r="Z17" s="9">
         <v>56</v>
       </c>
-      <c r="AA17" s="10">
+      <c r="AA17" s="65">
         <v>16</v>
       </c>
-      <c r="AB17" s="58">
+      <c r="AB17" s="9">
         <v>49</v>
       </c>
       <c r="AC17" s="65">
         <v>23</v>
       </c>
-      <c r="AD17" s="59">
+      <c r="AD17" s="45">
         <v>54</v>
       </c>
-      <c r="AE17" s="81">
+      <c r="AE17" s="63">
         <v>18</v>
       </c>
-      <c r="AF17" s="59">
+      <c r="AF17" s="45">
         <v>58</v>
       </c>
-      <c r="AG17" s="81">
+      <c r="AG17" s="63">
         <v>14</v>
       </c>
-      <c r="AH17" s="59">
+      <c r="AH17" s="45">
         <v>52</v>
       </c>
-      <c r="AI17" s="81">
+      <c r="AI17" s="63">
         <v>20</v>
       </c>
-      <c r="AJ17" s="99"/>
-      <c r="AK17" s="100"/>
-      <c r="AL17" s="59"/>
-      <c r="AM17" s="81"/>
-      <c r="AN17" s="49">
+      <c r="AJ17" s="126"/>
+      <c r="AK17" s="129"/>
+      <c r="AL17" s="45"/>
+      <c r="AM17" s="63"/>
+      <c r="AN17" s="36">
         <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17+AD17+AF17+AH17+AJ17+AL17</f>
         <v>594</v>
       </c>
-      <c r="AO17" s="49">
+      <c r="AO17" s="36">
         <f>COUNTIF(D17:AL17,"&gt;30")</f>
         <v>11</v>
       </c>
-      <c r="AP17" s="90">
+      <c r="AP17" s="72">
         <v>2</v>
       </c>
-      <c r="AQ17" s="83"/>
-      <c r="AR17" s="86">
+      <c r="AQ17" s="65"/>
+      <c r="AR17" s="68">
         <f>SUMIF(G17:AM17, "&lt;30")+AP17+AQ17</f>
         <v>197</v>
       </c>
-      <c r="AS17" s="56">
+      <c r="AS17" s="43">
         <f>AR17/AO17</f>
         <v>17.90909090909091</v>
       </c>
-      <c r="AT17" s="51"/>
-      <c r="AU17" s="34"/>
-      <c r="AV17" s="34"/>
-      <c r="AW17" s="11"/>
-      <c r="AX17" s="50"/>
+      <c r="AT17" s="38"/>
+      <c r="AU17" s="27"/>
+      <c r="AV17" s="27"/>
+      <c r="AW17" s="8"/>
+      <c r="AX17" s="37"/>
     </row>
     <row r="18" spans="1:50">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="118">
         <f>ROUND((AN18-(36*AO18))/AO18,0)</f>
         <v>11</v>
       </c>
-      <c r="D18" s="42"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="12">
+      <c r="D18" s="126"/>
+      <c r="E18" s="129"/>
+      <c r="F18" s="9">
         <v>46</v>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="65">
         <v>18</v>
       </c>
-      <c r="H18" s="42"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="12">
+      <c r="H18" s="126"/>
+      <c r="I18" s="129"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="65"/>
+      <c r="L18" s="9">
         <v>46</v>
       </c>
-      <c r="M18" s="10">
+      <c r="M18" s="65">
         <v>18</v>
       </c>
-      <c r="N18" s="12">
+      <c r="N18" s="9">
         <v>46</v>
       </c>
-      <c r="O18" s="10">
+      <c r="O18" s="65">
         <v>18</v>
       </c>
-      <c r="P18" s="12">
+      <c r="P18" s="9">
         <v>46</v>
       </c>
-      <c r="Q18" s="10">
+      <c r="Q18" s="65">
         <v>18</v>
       </c>
-      <c r="R18" s="12">
+      <c r="R18" s="9">
         <v>47</v>
       </c>
-      <c r="S18" s="10">
+      <c r="S18" s="65">
         <v>14</v>
       </c>
-      <c r="T18" s="12">
+      <c r="T18" s="9">
         <v>52</v>
       </c>
-      <c r="U18" s="10">
+      <c r="U18" s="65">
         <v>13</v>
       </c>
-      <c r="V18" s="12"/>
-      <c r="W18" s="10"/>
-      <c r="X18" s="12"/>
-      <c r="Y18" s="10"/>
-      <c r="Z18" s="12">
+      <c r="V18" s="9"/>
+      <c r="W18" s="65"/>
+      <c r="X18" s="9"/>
+      <c r="Y18" s="65"/>
+      <c r="Z18" s="9">
         <v>50</v>
       </c>
-      <c r="AA18" s="10">
+      <c r="AA18" s="65">
         <v>15</v>
       </c>
-      <c r="AB18" s="59"/>
+      <c r="AB18" s="9"/>
       <c r="AC18" s="65"/>
-      <c r="AD18" s="59">
+      <c r="AD18" s="45">
         <v>47</v>
       </c>
-      <c r="AE18" s="81">
+      <c r="AE18" s="63">
         <v>19</v>
       </c>
-      <c r="AF18" s="59">
+      <c r="AF18" s="45">
         <v>48</v>
       </c>
-      <c r="AG18" s="81">
+      <c r="AG18" s="63">
         <v>18</v>
       </c>
-      <c r="AH18" s="59">
+      <c r="AH18" s="45">
         <v>44</v>
       </c>
-      <c r="AI18" s="81">
+      <c r="AI18" s="63">
         <v>22</v>
       </c>
-      <c r="AJ18" s="99"/>
-      <c r="AK18" s="100"/>
-      <c r="AL18" s="59"/>
-      <c r="AM18" s="81"/>
-      <c r="AN18" s="49">
+      <c r="AJ18" s="126"/>
+      <c r="AK18" s="129"/>
+      <c r="AL18" s="45"/>
+      <c r="AM18" s="63"/>
+      <c r="AN18" s="36">
         <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18+AD18+AF18+AH18+AJ18+AL18</f>
         <v>472</v>
       </c>
-      <c r="AO18" s="49">
+      <c r="AO18" s="36">
         <f>COUNTIF(D18:AL18,"&gt;30")</f>
         <v>10</v>
       </c>
-      <c r="AP18" s="12"/>
-      <c r="AQ18" s="91">
+      <c r="AP18" s="9"/>
+      <c r="AQ18" s="73">
         <v>1</v>
       </c>
-      <c r="AR18" s="86">
+      <c r="AR18" s="68">
         <f>SUMIF(G18:AM18, "&lt;30")+AP18+AQ18</f>
         <v>174</v>
       </c>
-      <c r="AS18" s="56">
+      <c r="AS18" s="43">
         <f>AR18/AO18</f>
         <v>17.399999999999999</v>
       </c>
-      <c r="AT18" s="51"/>
-      <c r="AU18" s="11"/>
-      <c r="AV18" s="11"/>
-      <c r="AW18" s="11"/>
-      <c r="AX18" s="50"/>
+      <c r="AT18" s="38"/>
+      <c r="AU18" s="8"/>
+      <c r="AV18" s="8"/>
+      <c r="AW18" s="8"/>
+      <c r="AX18" s="37"/>
     </row>
     <row r="19" spans="1:50">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="118">
         <f>ROUND((AN19-(36*AO19))/AO19,0)</f>
         <v>11</v>
       </c>
-      <c r="D19" s="42"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="43"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="35">
+      <c r="D19" s="126"/>
+      <c r="E19" s="129"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="65"/>
+      <c r="H19" s="126"/>
+      <c r="I19" s="129"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="65"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="65"/>
+      <c r="N19" s="11">
         <v>45</v>
       </c>
-      <c r="O19" s="10">
+      <c r="O19" s="65">
         <v>18</v>
       </c>
-      <c r="P19" s="35">
+      <c r="P19" s="11">
         <v>43</v>
       </c>
-      <c r="Q19" s="10">
+      <c r="Q19" s="65">
         <v>20</v>
       </c>
-      <c r="R19" s="35"/>
-      <c r="S19" s="10"/>
-      <c r="T19" s="35"/>
-      <c r="U19" s="10"/>
-      <c r="V19" s="35"/>
-      <c r="W19" s="10"/>
-      <c r="X19" s="35">
+      <c r="R19" s="11"/>
+      <c r="S19" s="65"/>
+      <c r="T19" s="11"/>
+      <c r="U19" s="65"/>
+      <c r="V19" s="11"/>
+      <c r="W19" s="65"/>
+      <c r="X19" s="11">
         <v>48</v>
       </c>
-      <c r="Y19" s="10">
+      <c r="Y19" s="65">
         <v>15</v>
       </c>
-      <c r="Z19" s="35">
+      <c r="Z19" s="11">
         <v>47</v>
       </c>
       <c r="AA19" s="65">
         <v>16</v>
       </c>
-      <c r="AB19" s="35"/>
+      <c r="AB19" s="11"/>
       <c r="AC19" s="65"/>
-      <c r="AD19" s="35">
+      <c r="AD19" s="28">
         <v>51</v>
       </c>
-      <c r="AE19" s="81">
+      <c r="AE19" s="63">
         <v>13</v>
       </c>
-      <c r="AF19" s="35">
+      <c r="AF19" s="28">
         <v>45</v>
       </c>
-      <c r="AG19" s="81">
+      <c r="AG19" s="63">
         <v>20</v>
       </c>
-      <c r="AH19" s="35"/>
-      <c r="AI19" s="81"/>
-      <c r="AJ19" s="99"/>
-      <c r="AK19" s="100"/>
-      <c r="AL19" s="35"/>
-      <c r="AM19" s="81"/>
-      <c r="AN19" s="49">
+      <c r="AH19" s="28"/>
+      <c r="AI19" s="63"/>
+      <c r="AJ19" s="126"/>
+      <c r="AK19" s="129"/>
+      <c r="AL19" s="28"/>
+      <c r="AM19" s="63"/>
+      <c r="AN19" s="36">
         <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19+AD19+AF19+AH19+AJ19+AL19</f>
         <v>279</v>
       </c>
-      <c r="AO19" s="49">
+      <c r="AO19" s="36">
         <f>COUNTIF(D19:AL19,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AP19" s="90"/>
-      <c r="AQ19" s="83">
+      <c r="AP19" s="72"/>
+      <c r="AQ19" s="65">
         <v>2</v>
       </c>
-      <c r="AR19" s="86">
+      <c r="AR19" s="68">
         <f>SUMIF(G19:AM19, "&lt;30")+AP19+AQ19</f>
         <v>104</v>
       </c>
-      <c r="AS19" s="56">
+      <c r="AS19" s="43">
         <f>AR19/AO19</f>
         <v>17.333333333333332</v>
       </c>
-      <c r="AT19" s="49"/>
-      <c r="AU19" s="34"/>
-      <c r="AV19" s="34"/>
-      <c r="AW19" s="11"/>
-      <c r="AX19" s="50"/>
+      <c r="AT19" s="36"/>
+      <c r="AU19" s="27"/>
+      <c r="AV19" s="27"/>
+      <c r="AW19" s="8"/>
+      <c r="AX19" s="37"/>
     </row>
     <row r="20" spans="1:50">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="118">
         <f>ROUND((AN20-(36*AO20))/AO20,0)</f>
         <v>24</v>
       </c>
-      <c r="D20" s="42"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="13">
+      <c r="D20" s="126"/>
+      <c r="E20" s="129"/>
+      <c r="F20" s="10">
         <v>61</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="65">
         <v>14</v>
       </c>
-      <c r="H20" s="42"/>
-      <c r="I20" s="43"/>
-      <c r="J20" s="13">
+      <c r="H20" s="126"/>
+      <c r="I20" s="129"/>
+      <c r="J20" s="10">
         <v>56</v>
       </c>
-      <c r="K20" s="10">
+      <c r="K20" s="65">
         <v>19</v>
       </c>
-      <c r="L20" s="35">
+      <c r="L20" s="10">
         <v>60</v>
       </c>
-      <c r="M20" s="10">
+      <c r="M20" s="65">
         <v>15</v>
       </c>
-      <c r="N20" s="35">
+      <c r="N20" s="10">
         <v>56</v>
       </c>
-      <c r="O20" s="10">
+      <c r="O20" s="65">
         <v>20</v>
       </c>
-      <c r="P20" s="35">
+      <c r="P20" s="10">
         <v>54</v>
       </c>
-      <c r="Q20" s="10">
+      <c r="Q20" s="65">
         <v>22</v>
       </c>
-      <c r="R20" s="35"/>
-      <c r="S20" s="10"/>
-      <c r="T20" s="35">
+      <c r="R20" s="10"/>
+      <c r="S20" s="65"/>
+      <c r="T20" s="10">
         <v>66</v>
       </c>
-      <c r="U20" s="10">
+      <c r="U20" s="65">
         <v>9</v>
       </c>
-      <c r="V20" s="35">
+      <c r="V20" s="10">
         <v>55</v>
       </c>
-      <c r="W20" s="10">
+      <c r="W20" s="65">
         <v>22</v>
       </c>
-      <c r="X20" s="35"/>
-      <c r="Y20" s="10"/>
-      <c r="Z20" s="35">
+      <c r="X20" s="10"/>
+      <c r="Y20" s="65"/>
+      <c r="Z20" s="10">
         <v>70</v>
       </c>
       <c r="AA20" s="65">
         <v>6</v>
       </c>
-      <c r="AB20" s="35">
+      <c r="AB20" s="10">
         <v>63</v>
       </c>
       <c r="AC20" s="65">
         <v>15</v>
       </c>
-      <c r="AD20" s="35">
+      <c r="AD20" s="28">
         <v>58</v>
       </c>
-      <c r="AE20" s="81">
+      <c r="AE20" s="63">
         <v>20</v>
       </c>
-      <c r="AF20" s="35">
+      <c r="AF20" s="28">
         <v>60</v>
       </c>
-      <c r="AG20" s="81">
+      <c r="AG20" s="63">
         <v>18</v>
       </c>
-      <c r="AH20" s="35">
+      <c r="AH20" s="28">
         <v>55</v>
       </c>
-      <c r="AI20" s="81">
+      <c r="AI20" s="63">
         <v>23</v>
       </c>
-      <c r="AJ20" s="99"/>
-      <c r="AK20" s="100"/>
-      <c r="AL20" s="35"/>
-      <c r="AM20" s="81"/>
-      <c r="AN20" s="49">
+      <c r="AJ20" s="126"/>
+      <c r="AK20" s="129"/>
+      <c r="AL20" s="28"/>
+      <c r="AM20" s="63"/>
+      <c r="AN20" s="36">
         <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20+AD20+AF20+AH20+AJ20+AL20</f>
         <v>714</v>
       </c>
-      <c r="AO20" s="49">
+      <c r="AO20" s="36">
         <f>COUNTIF(D20:AL20,"&gt;30")</f>
         <v>12</v>
       </c>
-      <c r="AP20" s="90">
+      <c r="AP20" s="72">
         <v>2</v>
       </c>
-      <c r="AQ20" s="83"/>
-      <c r="AR20" s="86">
+      <c r="AQ20" s="65"/>
+      <c r="AR20" s="68">
         <f>SUMIF(G20:AM20, "&lt;30")+AP20+AQ20</f>
         <v>205</v>
       </c>
-      <c r="AS20" s="56">
+      <c r="AS20" s="43">
         <f>AR20/AO20</f>
         <v>17.083333333333332</v>
       </c>
-      <c r="AT20" s="49"/>
-      <c r="AU20" s="34"/>
-      <c r="AV20" s="34"/>
-      <c r="AW20" s="11"/>
-      <c r="AX20" s="50"/>
+      <c r="AT20" s="36"/>
+      <c r="AU20" s="27"/>
+      <c r="AV20" s="27"/>
+      <c r="AW20" s="8"/>
+      <c r="AX20" s="37"/>
     </row>
     <row r="21" spans="1:50">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="118">
         <v>18</v>
       </c>
-      <c r="D21" s="42"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="12">
+      <c r="D21" s="126"/>
+      <c r="E21" s="129"/>
+      <c r="F21" s="9">
         <v>56</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="65">
         <v>16</v>
       </c>
-      <c r="H21" s="42"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="12"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="12"/>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="12"/>
-      <c r="S21" s="10"/>
-      <c r="T21" s="12"/>
-      <c r="U21" s="10"/>
-      <c r="V21" s="12"/>
-      <c r="W21" s="10"/>
-      <c r="X21" s="12"/>
-      <c r="Y21" s="10"/>
-      <c r="Z21" s="12"/>
-      <c r="AA21" s="10"/>
-      <c r="AB21" s="59"/>
+      <c r="H21" s="126"/>
+      <c r="I21" s="129"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="65"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="65"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="65"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="65"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="65"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="65"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="65"/>
+      <c r="X21" s="9"/>
+      <c r="Y21" s="65"/>
+      <c r="Z21" s="9"/>
+      <c r="AA21" s="65"/>
+      <c r="AB21" s="9"/>
       <c r="AC21" s="65"/>
-      <c r="AD21" s="59"/>
-      <c r="AE21" s="81"/>
-      <c r="AF21" s="59"/>
-      <c r="AG21" s="81"/>
-      <c r="AH21" s="59"/>
-      <c r="AI21" s="81"/>
-      <c r="AJ21" s="99"/>
-      <c r="AK21" s="100"/>
-      <c r="AL21" s="59"/>
-      <c r="AM21" s="81"/>
-      <c r="AN21" s="49">
+      <c r="AD21" s="45"/>
+      <c r="AE21" s="63"/>
+      <c r="AF21" s="45"/>
+      <c r="AG21" s="63"/>
+      <c r="AH21" s="45"/>
+      <c r="AI21" s="63"/>
+      <c r="AJ21" s="126"/>
+      <c r="AK21" s="129"/>
+      <c r="AL21" s="45"/>
+      <c r="AM21" s="63"/>
+      <c r="AN21" s="36">
         <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21+AD21+AF21+AH21+AJ21+AL21</f>
         <v>56</v>
       </c>
-      <c r="AO21" s="49">
+      <c r="AO21" s="36">
         <f>COUNTIF(D21:AL21,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AP21" s="90"/>
-      <c r="AQ21" s="83"/>
-      <c r="AR21" s="86">
+      <c r="AP21" s="72"/>
+      <c r="AQ21" s="65"/>
+      <c r="AR21" s="68">
         <f>SUMIF(G21:AM21, "&lt;30")+AP21+AQ21</f>
         <v>16</v>
       </c>
-      <c r="AS21" s="56">
+      <c r="AS21" s="43">
         <f>AR21/AO21</f>
         <v>16</v>
       </c>
-      <c r="AT21" s="51"/>
-      <c r="AU21" s="34"/>
-      <c r="AV21" s="34"/>
-      <c r="AW21" s="11"/>
-      <c r="AX21" s="50"/>
+      <c r="AT21" s="38"/>
+      <c r="AU21" s="27"/>
+      <c r="AV21" s="27"/>
+      <c r="AW21" s="8"/>
+      <c r="AX21" s="37"/>
     </row>
     <row r="22" spans="1:50" ht="16.5" thickBot="1">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="111" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="112" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="119" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="62"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="44"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="62"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="63">
+      <c r="D22" s="126"/>
+      <c r="E22" s="129"/>
+      <c r="F22" s="54"/>
+      <c r="G22" s="65"/>
+      <c r="H22" s="126"/>
+      <c r="I22" s="129"/>
+      <c r="J22" s="54"/>
+      <c r="K22" s="65"/>
+      <c r="L22" s="54">
         <v>50</v>
       </c>
-      <c r="M22" s="18"/>
-      <c r="N22" s="63"/>
-      <c r="O22" s="18"/>
-      <c r="P22" s="63"/>
-      <c r="Q22" s="18"/>
-      <c r="R22" s="63"/>
-      <c r="S22" s="18"/>
-      <c r="T22" s="63"/>
-      <c r="U22" s="18"/>
-      <c r="V22" s="63"/>
-      <c r="W22" s="18"/>
-      <c r="X22" s="63"/>
-      <c r="Y22" s="18"/>
-      <c r="Z22" s="63"/>
-      <c r="AA22" s="18"/>
-      <c r="AB22" s="63"/>
-      <c r="AC22" s="18"/>
-      <c r="AD22" s="82"/>
-      <c r="AE22" s="83"/>
-      <c r="AF22" s="82"/>
-      <c r="AG22" s="83"/>
-      <c r="AH22" s="82"/>
-      <c r="AI22" s="83"/>
-      <c r="AJ22" s="99"/>
-      <c r="AK22" s="100"/>
-      <c r="AL22" s="82"/>
-      <c r="AM22" s="83"/>
-      <c r="AN22" s="49">
+      <c r="M22" s="65"/>
+      <c r="N22" s="54"/>
+      <c r="O22" s="65"/>
+      <c r="P22" s="54"/>
+      <c r="Q22" s="65"/>
+      <c r="R22" s="54"/>
+      <c r="S22" s="65"/>
+      <c r="T22" s="54"/>
+      <c r="U22" s="65"/>
+      <c r="V22" s="54"/>
+      <c r="W22" s="65"/>
+      <c r="X22" s="54"/>
+      <c r="Y22" s="65"/>
+      <c r="Z22" s="54"/>
+      <c r="AA22" s="65"/>
+      <c r="AB22" s="54"/>
+      <c r="AC22" s="65"/>
+      <c r="AD22" s="64"/>
+      <c r="AE22" s="65"/>
+      <c r="AF22" s="64"/>
+      <c r="AG22" s="65"/>
+      <c r="AH22" s="64"/>
+      <c r="AI22" s="65"/>
+      <c r="AJ22" s="126"/>
+      <c r="AK22" s="129"/>
+      <c r="AL22" s="64"/>
+      <c r="AM22" s="65"/>
+      <c r="AN22" s="36">
         <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22+AD22+AF22+AH22+AJ22+AL22</f>
         <v>50</v>
       </c>
-      <c r="AO22" s="49">
+      <c r="AO22" s="36">
         <f>COUNTIF(D22:AL22,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AP22" s="90">
+      <c r="AP22" s="72">
         <v>1</v>
       </c>
-      <c r="AQ22" s="83"/>
-      <c r="AR22" s="87">
+      <c r="AQ22" s="65"/>
+      <c r="AR22" s="69">
         <f>SUMIF(G22:AM22, "&lt;30")+AP22+AQ22</f>
         <v>1</v>
       </c>
-      <c r="AS22" s="57">
+      <c r="AS22" s="43">
         <f>AR22/AO22</f>
         <v>1</v>
       </c>
-      <c r="AT22" s="75"/>
-      <c r="AU22" s="78"/>
-      <c r="AV22" s="78"/>
-      <c r="AW22" s="77"/>
-      <c r="AX22" s="79"/>
+      <c r="AT22" s="57"/>
+      <c r="AU22" s="60"/>
+      <c r="AV22" s="60"/>
+      <c r="AW22" s="59"/>
+      <c r="AX22" s="61"/>
     </row>
     <row r="23" spans="1:50" ht="16.5" thickBot="1">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="120" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="44"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="62"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="63">
+      <c r="D23" s="127"/>
+      <c r="E23" s="130"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="66"/>
+      <c r="H23" s="127"/>
+      <c r="I23" s="130"/>
+      <c r="J23" s="47"/>
+      <c r="K23" s="66"/>
+      <c r="L23" s="47"/>
+      <c r="M23" s="66"/>
+      <c r="N23" s="47"/>
+      <c r="O23" s="66"/>
+      <c r="P23" s="47"/>
+      <c r="Q23" s="66"/>
+      <c r="R23" s="47"/>
+      <c r="S23" s="66"/>
+      <c r="T23" s="47"/>
+      <c r="U23" s="66"/>
+      <c r="V23" s="47"/>
+      <c r="W23" s="66"/>
+      <c r="X23" s="47"/>
+      <c r="Y23" s="66"/>
+      <c r="Z23" s="47"/>
+      <c r="AA23" s="66"/>
+      <c r="AB23" s="47"/>
+      <c r="AC23" s="66"/>
+      <c r="AD23" s="48"/>
+      <c r="AE23" s="66"/>
+      <c r="AF23" s="48"/>
+      <c r="AG23" s="66"/>
+      <c r="AH23" s="48"/>
+      <c r="AI23" s="66"/>
+      <c r="AJ23" s="127"/>
+      <c r="AK23" s="130"/>
+      <c r="AL23" s="116">
         <v>50</v>
       </c>
-      <c r="M23" s="18"/>
-      <c r="N23" s="63"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="63"/>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="63"/>
-      <c r="S23" s="18"/>
-      <c r="T23" s="63"/>
-      <c r="U23" s="18"/>
-      <c r="V23" s="63"/>
-      <c r="W23" s="18"/>
-      <c r="X23" s="63"/>
-      <c r="Y23" s="18"/>
-      <c r="Z23" s="63"/>
-      <c r="AA23" s="18"/>
-      <c r="AB23" s="63"/>
-      <c r="AC23" s="18"/>
-      <c r="AD23" s="63"/>
-      <c r="AE23" s="84"/>
-      <c r="AF23" s="63"/>
-      <c r="AG23" s="84"/>
-      <c r="AH23" s="63"/>
-      <c r="AI23" s="84"/>
-      <c r="AJ23" s="101"/>
-      <c r="AK23" s="102"/>
-      <c r="AL23" s="63"/>
-      <c r="AM23" s="84"/>
-      <c r="AN23" s="52">
+      <c r="AM23" s="66"/>
+      <c r="AN23" s="36">
         <f>F23+J23+L23+N23+P23+R23+T23+V23+X23+Z23+AB23+AD23+AF23+AH23+AJ23+AL23</f>
         <v>50</v>
       </c>
-      <c r="AO23" s="52">
+      <c r="AO23" s="39">
         <f>COUNTIF(D23:AL23,"&gt;30")</f>
         <v>1</v>
       </c>
-      <c r="AP23" s="92"/>
-      <c r="AQ23" s="84"/>
-      <c r="AR23" s="87">
+      <c r="AP23" s="74"/>
+      <c r="AQ23" s="66"/>
+      <c r="AR23" s="69">
         <f>SUMIF(G23:AM23, "&lt;30")+AP23+AQ23</f>
         <v>0</v>
       </c>
-      <c r="AS23" s="57">
+      <c r="AS23" s="44">
         <f>AR23/AO23</f>
         <v>0</v>
       </c>
-      <c r="AT23" s="52"/>
-      <c r="AU23" s="36"/>
-      <c r="AV23" s="36"/>
-      <c r="AW23" s="19"/>
-      <c r="AX23" s="53"/>
+      <c r="AT23" s="39"/>
+      <c r="AU23" s="29"/>
+      <c r="AV23" s="29"/>
+      <c r="AW23" s="14"/>
+      <c r="AX23" s="40"/>
     </row>
-    <row r="24" spans="1:50" s="20" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A24" s="30"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32">
+    <row r="24" spans="1:50" s="15" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A24" s="113"/>
+      <c r="B24" s="114"/>
+      <c r="C24" s="115"/>
+      <c r="D24" s="123"/>
+      <c r="E24" s="124"/>
+      <c r="F24" s="124">
         <f>AVERAGEIF(F4:F23,"&gt;0")</f>
         <v>49.75</v>
       </c>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32">
+      <c r="G24" s="124"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="25"/>
+      <c r="J24" s="25">
         <f>AVERAGEIF(J4:J23,"&gt;0")</f>
         <v>54</v>
       </c>
-      <c r="K24" s="32"/>
-      <c r="L24" s="32">
+      <c r="K24" s="25"/>
+      <c r="L24" s="25">
         <f>AVERAGEIF(L4:L23,"&gt;0")</f>
-        <v>51.25</v>
-      </c>
-      <c r="M24" s="32"/>
-      <c r="N24" s="32">
+        <v>51.428571428571431</v>
+      </c>
+      <c r="M24" s="25"/>
+      <c r="N24" s="25">
         <f>AVERAGEIF(N4:N23,"&gt;0")</f>
         <v>48.9</v>
       </c>
-      <c r="O24" s="32"/>
-      <c r="P24" s="32">
+      <c r="O24" s="25"/>
+      <c r="P24" s="25">
         <f>AVERAGEIF(P4:P23,"&gt;0")</f>
         <v>46.785714285714285</v>
       </c>
-      <c r="Q24" s="32"/>
-      <c r="R24" s="32">
+      <c r="Q24" s="25"/>
+      <c r="R24" s="25">
         <f>AVERAGEIF(R4:R23,"&gt;0")</f>
         <v>48.272727272727273</v>
       </c>
-      <c r="S24" s="32"/>
-      <c r="T24" s="32">
+      <c r="S24" s="25"/>
+      <c r="T24" s="25">
         <f>AVERAGEIF(T4:T23,"&gt;0")</f>
         <v>50.333333333333336</v>
       </c>
-      <c r="U24" s="32"/>
-      <c r="V24" s="32">
+      <c r="U24" s="25"/>
+      <c r="V24" s="25">
         <f>AVERAGEIF(V4:V23,"&gt;0")</f>
         <v>49</v>
       </c>
-      <c r="W24" s="32"/>
-      <c r="X24" s="32">
+      <c r="W24" s="25"/>
+      <c r="X24" s="25">
         <f>AVERAGEIF(X4:X23,"&gt;0")</f>
         <v>46.46153846153846</v>
       </c>
-      <c r="Y24" s="32"/>
-      <c r="Z24" s="32">
+      <c r="Y24" s="25"/>
+      <c r="Z24" s="25">
         <f>AVERAGEIF(Z4:Z23,"&gt;0")</f>
         <v>49.53846153846154</v>
       </c>
-      <c r="AA24" s="32"/>
-      <c r="AB24" s="32">
+      <c r="AA24" s="25"/>
+      <c r="AB24" s="25">
         <f>AVERAGEIF(AB4:AB23,"&gt;0")</f>
         <v>47.846153846153847</v>
       </c>
-      <c r="AC24" s="93"/>
-      <c r="AD24" s="94">
+      <c r="AC24" s="75"/>
+      <c r="AD24" s="76">
         <f>AVERAGEIF(AD4:AD23,"&gt;0")</f>
         <v>46.090909090909093</v>
       </c>
-      <c r="AE24" s="95"/>
-      <c r="AF24" s="94">
+      <c r="AE24" s="77"/>
+      <c r="AF24" s="76">
         <f>AVERAGEIF(AF4:AF23,"&gt;0")</f>
         <v>47.230769230769234</v>
       </c>
-      <c r="AG24" s="95"/>
-      <c r="AH24" s="94">
+      <c r="AG24" s="77"/>
+      <c r="AH24" s="76">
         <f>AVERAGEIF(AH4:AH23,"&gt;0")</f>
         <v>46.666666666666664</v>
       </c>
-      <c r="AI24" s="95"/>
-      <c r="AJ24" s="94"/>
-      <c r="AK24" s="95"/>
-      <c r="AL24" s="94">
+      <c r="AI24" s="77"/>
+      <c r="AJ24" s="76"/>
+      <c r="AK24" s="77"/>
+      <c r="AL24" s="76">
         <f>AVERAGEIF(AL4:AL23,"&gt;0")</f>
-        <v>49.4</v>
-      </c>
-      <c r="AM24" s="95"/>
-      <c r="AN24" s="96"/>
+        <v>49.5</v>
+      </c>
+      <c r="AM24" s="77"/>
+      <c r="AN24" s="78"/>
     </row>
     <row r="25" spans="1:50">
-      <c r="C25" s="21"/>
-      <c r="AN25" s="22"/>
-      <c r="AO25" s="22"/>
-      <c r="AP25" s="23"/>
-      <c r="AQ25" s="23"/>
-      <c r="AR25" s="22"/>
-      <c r="AS25" s="24"/>
+      <c r="C25" s="16"/>
+      <c r="AN25" s="17"/>
+      <c r="AO25" s="17"/>
+      <c r="AP25" s="18"/>
+      <c r="AQ25" s="18"/>
+      <c r="AR25" s="17"/>
+      <c r="AS25" s="19"/>
     </row>
     <row r="26" spans="1:50">
-      <c r="C26" s="37" t="s">
+      <c r="C26" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="D26" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="F26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="J26" s="25"/>
-      <c r="L26" s="25"/>
-      <c r="N26" s="25"/>
-      <c r="P26" s="25"/>
-      <c r="R26" s="25"/>
-      <c r="T26" s="25"/>
-      <c r="V26" s="25"/>
-      <c r="X26" s="25"/>
-      <c r="Z26" s="25"/>
-      <c r="AB26" s="25"/>
-      <c r="AD26" s="25"/>
-      <c r="AF26" s="25"/>
-      <c r="AH26" s="25"/>
-      <c r="AJ26" s="25"/>
-      <c r="AL26" s="25"/>
+      <c r="F26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="L26" s="20"/>
+      <c r="N26" s="20"/>
+      <c r="P26" s="20"/>
+      <c r="R26" s="20"/>
+      <c r="T26" s="20"/>
+      <c r="V26" s="20"/>
+      <c r="X26" s="20"/>
+      <c r="Z26" s="20"/>
+      <c r="AB26" s="20"/>
+      <c r="AD26" s="20"/>
+      <c r="AF26" s="20"/>
+      <c r="AH26" s="20"/>
+      <c r="AJ26" s="20"/>
+      <c r="AL26" s="20"/>
     </row>
     <row r="27" spans="1:50">
-      <c r="C27" s="38" t="s">
+      <c r="C27" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="F27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="J27" s="26"/>
-      <c r="L27" s="26"/>
-      <c r="N27" s="26"/>
-      <c r="P27" s="26"/>
-      <c r="R27" s="26"/>
-      <c r="T27" s="26"/>
-      <c r="V27" s="26"/>
-      <c r="X27" s="26"/>
-      <c r="Z27" s="26"/>
-      <c r="AB27" s="26"/>
-      <c r="AD27" s="26"/>
-      <c r="AF27" s="26"/>
-      <c r="AH27" s="26"/>
-      <c r="AJ27" s="26"/>
-      <c r="AL27" s="26"/>
-      <c r="AN27" s="27"/>
+      <c r="F27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="L27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="P27" s="21"/>
+      <c r="R27" s="21"/>
+      <c r="T27" s="21"/>
+      <c r="V27" s="21"/>
+      <c r="X27" s="21"/>
+      <c r="Z27" s="21"/>
+      <c r="AB27" s="21"/>
+      <c r="AD27" s="21"/>
+      <c r="AF27" s="21"/>
+      <c r="AH27" s="21"/>
+      <c r="AJ27" s="21"/>
+      <c r="AL27" s="21"/>
+      <c r="AN27" s="22"/>
     </row>
     <row r="28" spans="1:50">
-      <c r="C28" s="39" t="s">
+      <c r="C28" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="D28" s="28" t="s">
+      <c r="D28" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="E28" s="29"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="28"/>
-      <c r="K28" s="29"/>
-      <c r="L28" s="28"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="28"/>
-      <c r="O28" s="29"/>
-      <c r="P28" s="28"/>
-      <c r="Q28" s="29"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="29"/>
-      <c r="T28" s="28"/>
-      <c r="U28" s="29"/>
-      <c r="V28" s="28"/>
-      <c r="W28" s="29"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="29"/>
-      <c r="Z28" s="28"/>
-      <c r="AA28" s="29"/>
-      <c r="AB28" s="28"/>
-      <c r="AC28" s="29"/>
-      <c r="AD28" s="28"/>
-      <c r="AE28" s="29"/>
-      <c r="AF28" s="28"/>
-      <c r="AG28" s="29"/>
-      <c r="AH28" s="28"/>
-      <c r="AI28" s="29"/>
-      <c r="AJ28" s="28"/>
-      <c r="AK28" s="29"/>
-      <c r="AL28" s="28"/>
-      <c r="AM28" s="29"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="23"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="23"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="23"/>
+      <c r="U28" s="24"/>
+      <c r="V28" s="23"/>
+      <c r="W28" s="24"/>
+      <c r="X28" s="23"/>
+      <c r="Y28" s="24"/>
+      <c r="Z28" s="23"/>
+      <c r="AA28" s="24"/>
+      <c r="AB28" s="23"/>
+      <c r="AC28" s="24"/>
+      <c r="AD28" s="23"/>
+      <c r="AE28" s="24"/>
+      <c r="AF28" s="23"/>
+      <c r="AG28" s="24"/>
+      <c r="AH28" s="23"/>
+      <c r="AI28" s="24"/>
+      <c r="AJ28" s="23"/>
+      <c r="AK28" s="24"/>
+      <c r="AL28" s="23"/>
+      <c r="AM28" s="24"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:AX23">
     <sortCondition descending="1" ref="AS4:AS23"/>
     <sortCondition descending="1" ref="AN4:AN23"/>
   </sortState>
-  <mergeCells count="51">
+  <mergeCells count="54">
+    <mergeCell ref="D4:E23"/>
+    <mergeCell ref="H4:I23"/>
+    <mergeCell ref="AJ4:AK23"/>
     <mergeCell ref="AH1:AI1"/>
     <mergeCell ref="AH2:AI2"/>
     <mergeCell ref="H1:I1"/>

</xml_diff>

<commit_message>
091725 - updated CTTP identification
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96156276-B3B5-584D-BEB7-22207EAFAEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{96156276-B3B5-584D-BEB7-22207EAFAEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07A0D921-ACCE-4B0B-88B6-AD466FE12EAC}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="2640" windowWidth="30760" windowHeight="17120" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="4275" yWindow="2460" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -271,7 +271,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -411,6 +411,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1071,7 +1079,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1248,6 +1256,105 @@
     <xf numFmtId="1" fontId="0" fillId="2" borderId="42" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1260,6 +1367,60 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1287,157 +1448,10 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1775,272 +1789,272 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
   <dimension ref="A1:BB29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="8.6640625" customWidth="1"/>
-    <col min="2" max="2" width="8.1640625" customWidth="1"/>
-    <col min="3" max="3" width="10.1640625" customWidth="1"/>
-    <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="8.625" customWidth="1"/>
+    <col min="2" max="2" width="8.125" customWidth="1"/>
+    <col min="3" max="3" width="10.125" customWidth="1"/>
+    <col min="4" max="10" width="6.875" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="23" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="12" max="23" width="6.375" hidden="1" customWidth="1"/>
     <col min="24" max="24" width="6" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="6.375" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="6" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="6.375" hidden="1" customWidth="1"/>
     <col min="28" max="28" width="6" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.375" hidden="1" customWidth="1"/>
     <col min="30" max="30" width="6" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="6.375" hidden="1" customWidth="1"/>
     <col min="32" max="32" width="6" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="6.375" hidden="1" customWidth="1"/>
     <col min="34" max="34" width="6" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="6.375" hidden="1" customWidth="1"/>
     <col min="36" max="36" width="6" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="6.33203125" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="6.375" hidden="1" customWidth="1"/>
     <col min="38" max="38" width="6" customWidth="1"/>
-    <col min="39" max="39" width="6.33203125" customWidth="1"/>
+    <col min="39" max="39" width="6.375" customWidth="1"/>
     <col min="40" max="40" width="6" customWidth="1"/>
-    <col min="41" max="41" width="6.33203125" customWidth="1"/>
+    <col min="41" max="41" width="6.375" customWidth="1"/>
     <col min="42" max="42" width="6" customWidth="1"/>
-    <col min="43" max="43" width="6.33203125" customWidth="1"/>
-    <col min="44" max="44" width="8.83203125" customWidth="1"/>
-    <col min="45" max="45" width="6.1640625" customWidth="1"/>
-    <col min="46" max="46" width="5.83203125" customWidth="1"/>
-    <col min="47" max="47" width="5.6640625" customWidth="1"/>
+    <col min="43" max="43" width="6.375" customWidth="1"/>
+    <col min="44" max="44" width="8.875" customWidth="1"/>
+    <col min="45" max="45" width="6.125" customWidth="1"/>
+    <col min="46" max="46" width="5.875" customWidth="1"/>
+    <col min="47" max="47" width="5.625" customWidth="1"/>
     <col min="48" max="48" width="5.5" customWidth="1"/>
     <col min="49" max="49" width="8" customWidth="1"/>
-    <col min="50" max="50" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="50" max="50" width="7.375" hidden="1" customWidth="1"/>
     <col min="51" max="52" width="6" hidden="1" customWidth="1"/>
-    <col min="53" max="53" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="54" max="54" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="53" max="53" width="7.375" hidden="1" customWidth="1"/>
+    <col min="54" max="54" width="9.375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:54" s="32" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="121" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="76" t="s">
+      <c r="B1" s="122"/>
+      <c r="C1" s="127" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="67"/>
-      <c r="F1" s="66" t="s">
+      <c r="E1" s="100"/>
+      <c r="F1" s="99" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="67"/>
-      <c r="H1" s="66" t="s">
+      <c r="G1" s="100"/>
+      <c r="H1" s="99" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="67"/>
-      <c r="J1" s="66" t="s">
+      <c r="I1" s="100"/>
+      <c r="J1" s="99" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="67"/>
-      <c r="L1" s="66" t="s">
+      <c r="K1" s="100"/>
+      <c r="L1" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="67"/>
-      <c r="N1" s="66" t="s">
+      <c r="M1" s="100"/>
+      <c r="N1" s="99" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="67"/>
-      <c r="P1" s="66" t="s">
+      <c r="O1" s="100"/>
+      <c r="P1" s="99" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="66" t="s">
+      <c r="Q1" s="100"/>
+      <c r="R1" s="99" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="67"/>
-      <c r="T1" s="66" t="s">
+      <c r="S1" s="100"/>
+      <c r="T1" s="99" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="67"/>
-      <c r="V1" s="66" t="s">
+      <c r="U1" s="100"/>
+      <c r="V1" s="99" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="67"/>
-      <c r="X1" s="66" t="s">
+      <c r="W1" s="100"/>
+      <c r="X1" s="99" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="66" t="s">
+      <c r="Y1" s="100"/>
+      <c r="Z1" s="99" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="66" t="s">
+      <c r="AA1" s="100"/>
+      <c r="AB1" s="99" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="66" t="s">
+      <c r="AC1" s="100"/>
+      <c r="AD1" s="99" t="s">
         <v>67</v>
       </c>
-      <c r="AE1" s="67"/>
-      <c r="AF1" s="66" t="s">
+      <c r="AE1" s="100"/>
+      <c r="AF1" s="99" t="s">
         <v>68</v>
       </c>
-      <c r="AG1" s="67"/>
-      <c r="AH1" s="66" t="s">
+      <c r="AG1" s="100"/>
+      <c r="AH1" s="99" t="s">
         <v>69</v>
       </c>
-      <c r="AI1" s="67"/>
-      <c r="AJ1" s="66" t="s">
+      <c r="AI1" s="100"/>
+      <c r="AJ1" s="99" t="s">
         <v>70</v>
       </c>
-      <c r="AK1" s="67"/>
-      <c r="AL1" s="66" t="s">
+      <c r="AK1" s="100"/>
+      <c r="AL1" s="99" t="s">
         <v>71</v>
       </c>
-      <c r="AM1" s="67"/>
-      <c r="AN1" s="66" t="s">
+      <c r="AM1" s="100"/>
+      <c r="AN1" s="99" t="s">
         <v>73</v>
       </c>
-      <c r="AO1" s="67"/>
-      <c r="AP1" s="66" t="s">
+      <c r="AO1" s="100"/>
+      <c r="AP1" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="AQ1" s="67"/>
-      <c r="AR1" s="82" t="s">
+      <c r="AQ1" s="100"/>
+      <c r="AR1" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="AS1" s="89" t="s">
+      <c r="AS1" s="118" t="s">
         <v>65</v>
       </c>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="91"/>
-      <c r="AX1" s="84" t="s">
+      <c r="AT1" s="119"/>
+      <c r="AU1" s="119"/>
+      <c r="AV1" s="119"/>
+      <c r="AW1" s="120"/>
+      <c r="AX1" s="113" t="s">
         <v>57</v>
       </c>
-      <c r="AY1" s="85"/>
-      <c r="AZ1" s="85"/>
-      <c r="BA1" s="85"/>
-      <c r="BB1" s="86"/>
+      <c r="AY1" s="114"/>
+      <c r="AZ1" s="114"/>
+      <c r="BA1" s="114"/>
+      <c r="BB1" s="115"/>
     </row>
     <row r="2" spans="1:54" s="32" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="72"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="68">
+      <c r="A2" s="123"/>
+      <c r="B2" s="124"/>
+      <c r="C2" s="128"/>
+      <c r="D2" s="101">
         <v>45782</v>
       </c>
-      <c r="E2" s="69"/>
-      <c r="F2" s="68">
+      <c r="E2" s="102"/>
+      <c r="F2" s="101">
         <v>45789</v>
       </c>
-      <c r="G2" s="69"/>
-      <c r="H2" s="68">
+      <c r="G2" s="102"/>
+      <c r="H2" s="101">
         <v>45796</v>
       </c>
-      <c r="I2" s="69"/>
-      <c r="J2" s="68">
+      <c r="I2" s="102"/>
+      <c r="J2" s="101">
         <v>45803</v>
       </c>
-      <c r="K2" s="69"/>
-      <c r="L2" s="68">
+      <c r="K2" s="102"/>
+      <c r="L2" s="101">
         <v>45810</v>
       </c>
-      <c r="M2" s="69"/>
-      <c r="N2" s="68">
+      <c r="M2" s="102"/>
+      <c r="N2" s="101">
         <v>45817</v>
       </c>
-      <c r="O2" s="69"/>
-      <c r="P2" s="68">
+      <c r="O2" s="102"/>
+      <c r="P2" s="101">
         <v>45824</v>
       </c>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="68">
+      <c r="Q2" s="102"/>
+      <c r="R2" s="101">
         <v>45831</v>
       </c>
-      <c r="S2" s="69"/>
-      <c r="T2" s="68">
+      <c r="S2" s="102"/>
+      <c r="T2" s="101">
         <v>45838</v>
       </c>
-      <c r="U2" s="69"/>
-      <c r="V2" s="68">
+      <c r="U2" s="102"/>
+      <c r="V2" s="101">
         <v>45845</v>
       </c>
-      <c r="W2" s="69"/>
-      <c r="X2" s="68">
+      <c r="W2" s="102"/>
+      <c r="X2" s="101">
         <v>45852</v>
       </c>
-      <c r="Y2" s="69"/>
-      <c r="Z2" s="68">
+      <c r="Y2" s="102"/>
+      <c r="Z2" s="101">
         <v>45859</v>
       </c>
-      <c r="AA2" s="69"/>
-      <c r="AB2" s="68">
+      <c r="AA2" s="102"/>
+      <c r="AB2" s="101">
         <v>45866</v>
       </c>
-      <c r="AC2" s="69"/>
-      <c r="AD2" s="68">
+      <c r="AC2" s="102"/>
+      <c r="AD2" s="101">
         <v>45873</v>
       </c>
-      <c r="AE2" s="69"/>
-      <c r="AF2" s="68">
+      <c r="AE2" s="102"/>
+      <c r="AF2" s="101">
         <v>45880</v>
       </c>
-      <c r="AG2" s="69"/>
-      <c r="AH2" s="68">
+      <c r="AG2" s="102"/>
+      <c r="AH2" s="101">
         <v>45887</v>
       </c>
-      <c r="AI2" s="69"/>
-      <c r="AJ2" s="68">
+      <c r="AI2" s="102"/>
+      <c r="AJ2" s="101">
         <v>45894</v>
       </c>
-      <c r="AK2" s="69"/>
-      <c r="AL2" s="68">
+      <c r="AK2" s="102"/>
+      <c r="AL2" s="101">
         <v>45901</v>
       </c>
-      <c r="AM2" s="69"/>
-      <c r="AN2" s="68">
+      <c r="AM2" s="102"/>
+      <c r="AN2" s="101">
         <v>45908</v>
       </c>
-      <c r="AO2" s="69"/>
-      <c r="AP2" s="68">
+      <c r="AO2" s="102"/>
+      <c r="AP2" s="101">
         <v>45915</v>
       </c>
-      <c r="AQ2" s="69"/>
-      <c r="AR2" s="83"/>
-      <c r="AS2" s="82" t="s">
+      <c r="AQ2" s="102"/>
+      <c r="AR2" s="106"/>
+      <c r="AS2" s="105" t="s">
         <v>3</v>
       </c>
-      <c r="AT2" s="80" t="s">
+      <c r="AT2" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="AU2" s="81" t="s">
+      <c r="AU2" s="111" t="s">
         <v>5</v>
       </c>
-      <c r="AV2" s="92" t="s">
+      <c r="AV2" s="103" t="s">
         <v>6</v>
       </c>
-      <c r="AW2" s="79" t="s">
+      <c r="AW2" s="107" t="s">
         <v>7</v>
       </c>
-      <c r="AX2" s="87" t="s">
+      <c r="AX2" s="116" t="s">
         <v>3</v>
       </c>
-      <c r="AY2" s="87" t="s">
+      <c r="AY2" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="AZ2" s="87" t="s">
+      <c r="AZ2" s="116" t="s">
         <v>5</v>
       </c>
-      <c r="BA2" s="87" t="s">
+      <c r="BA2" s="116" t="s">
         <v>6</v>
       </c>
-      <c r="BB2" s="87" t="s">
+      <c r="BB2" s="116" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:54" s="32" customFormat="1" ht="29" customHeight="1" thickBot="1">
-      <c r="A3" s="74"/>
-      <c r="B3" s="75"/>
-      <c r="C3" s="78"/>
+    <row r="3" spans="1:54" s="32" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
+      <c r="A3" s="125"/>
+      <c r="B3" s="126"/>
+      <c r="C3" s="129"/>
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
@@ -2161,19 +2175,19 @@
       <c r="AQ3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="AR3" s="83"/>
-      <c r="AS3" s="83"/>
-      <c r="AT3" s="94"/>
-      <c r="AU3" s="95"/>
-      <c r="AV3" s="93"/>
-      <c r="AW3" s="96"/>
-      <c r="AX3" s="88"/>
-      <c r="AY3" s="88"/>
-      <c r="AZ3" s="88"/>
-      <c r="BA3" s="88"/>
-      <c r="BB3" s="88"/>
+      <c r="AR3" s="106"/>
+      <c r="AS3" s="106"/>
+      <c r="AT3" s="110"/>
+      <c r="AU3" s="112"/>
+      <c r="AV3" s="104"/>
+      <c r="AW3" s="108"/>
+      <c r="AX3" s="117"/>
+      <c r="AY3" s="117"/>
+      <c r="AZ3" s="117"/>
+      <c r="BA3" s="117"/>
+      <c r="BB3" s="117"/>
     </row>
-    <row r="4" spans="1:54" ht="16" customHeight="1">
+    <row r="4" spans="1:54" ht="15.95" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -2181,19 +2195,19 @@
         <v>15</v>
       </c>
       <c r="C4" s="63">
-        <f>ROUND((AR4-(36*AS4))/AS4,0)</f>
+        <f t="shared" ref="C4:C20" si="0">ROUND((AR4-(36*AS4))/AS4,0)</f>
         <v>17</v>
       </c>
-      <c r="D4" s="109"/>
-      <c r="E4" s="110"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="79"/>
       <c r="F4" s="46">
         <v>53</v>
       </c>
       <c r="G4" s="59">
         <v>23</v>
       </c>
-      <c r="H4" s="109"/>
-      <c r="I4" s="110"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="79"/>
       <c r="J4" s="46"/>
       <c r="K4" s="59"/>
       <c r="L4" s="46"/>
@@ -2240,30 +2254,30 @@
       <c r="AG4" s="55"/>
       <c r="AH4" s="49"/>
       <c r="AI4" s="55"/>
-      <c r="AJ4" s="109"/>
-      <c r="AK4" s="110"/>
+      <c r="AJ4" s="78"/>
+      <c r="AK4" s="79"/>
       <c r="AL4" s="49"/>
       <c r="AM4" s="55"/>
-      <c r="AN4" s="109"/>
-      <c r="AO4" s="113"/>
+      <c r="AN4" s="78"/>
+      <c r="AO4" s="82"/>
       <c r="AP4" s="49"/>
-      <c r="AQ4" s="97"/>
-      <c r="AR4" s="99">
-        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4+AJ4+AL4+AN4+AP4</f>
+      <c r="AQ4" s="66"/>
+      <c r="AR4" s="68">
+        <f t="shared" ref="AR4:AR24" si="1">F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4+AJ4+AL4+AN4+AP4</f>
         <v>320</v>
       </c>
       <c r="AS4" s="5">
-        <f>COUNTIF(D4:AP4,"&gt;30")</f>
+        <f t="shared" ref="AS4:AS24" si="2">COUNTIF(D4:AP4,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AT4" s="101"/>
-      <c r="AU4" s="105"/>
+      <c r="AT4" s="70"/>
+      <c r="AU4" s="74"/>
       <c r="AV4" s="24">
-        <f>SUMIF(G4:AQ4, "&lt;30")+AT4+AU4</f>
+        <f t="shared" ref="AV4:AV23" si="3">SUMIF(G4:AQ4, "&lt;30")+AT4+AU4</f>
         <v>123</v>
       </c>
       <c r="AW4" s="38">
-        <f>AV4/AS4</f>
+        <f t="shared" ref="AW4:AW24" si="4">AV4/AS4</f>
         <v>20.5</v>
       </c>
       <c r="AX4" s="44"/>
@@ -2282,15 +2296,15 @@
         <v>35</v>
       </c>
       <c r="C5" s="64">
-        <f>ROUND((AR5-(36*AS5))/AS5,0)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="D5" s="111"/>
-      <c r="E5" s="112"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="81"/>
       <c r="F5" s="47"/>
       <c r="G5" s="58"/>
-      <c r="H5" s="111"/>
-      <c r="I5" s="112"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="81"/>
       <c r="J5" s="47"/>
       <c r="K5" s="58"/>
       <c r="L5" s="47"/>
@@ -2353,38 +2367,38 @@
       <c r="AI5" s="56">
         <v>17</v>
       </c>
-      <c r="AJ5" s="111"/>
-      <c r="AK5" s="112"/>
+      <c r="AJ5" s="80"/>
+      <c r="AK5" s="81"/>
       <c r="AL5" s="48"/>
       <c r="AM5" s="56"/>
-      <c r="AN5" s="111"/>
-      <c r="AO5" s="114"/>
-      <c r="AP5" s="48">
+      <c r="AN5" s="80"/>
+      <c r="AO5" s="83"/>
+      <c r="AP5" s="130">
         <v>35</v>
       </c>
-      <c r="AQ5" s="98">
+      <c r="AQ5" s="67">
         <v>20</v>
       </c>
-      <c r="AR5" s="100">
-        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5+AD5+AF5+AH5+AJ5+AL5+AN5+AP5</f>
+      <c r="AR5" s="69">
+        <f t="shared" si="1"/>
         <v>370</v>
       </c>
       <c r="AS5" s="8">
-        <f>COUNTIF(D5:AP5,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT5" s="102">
+      <c r="AT5" s="71">
         <v>3</v>
       </c>
-      <c r="AU5" s="106">
+      <c r="AU5" s="75">
         <v>13</v>
       </c>
       <c r="AV5" s="25">
-        <f>SUMIF(G5:AQ5, "&lt;30")+AT5+AU5</f>
+        <f t="shared" si="3"/>
         <v>203</v>
       </c>
       <c r="AW5" s="39">
-        <f>AV5/AS5</f>
+        <f t="shared" si="4"/>
         <v>20.3</v>
       </c>
       <c r="AX5" s="34"/>
@@ -2401,19 +2415,19 @@
         <v>16</v>
       </c>
       <c r="C6" s="64">
-        <f>ROUND((AR6-(36*AS6))/AS6,0)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D6" s="111"/>
-      <c r="E6" s="112"/>
+      <c r="D6" s="80"/>
+      <c r="E6" s="81"/>
       <c r="F6" s="37">
         <v>45</v>
       </c>
       <c r="G6" s="58">
         <v>17</v>
       </c>
-      <c r="H6" s="111"/>
-      <c r="I6" s="112"/>
+      <c r="H6" s="80"/>
+      <c r="I6" s="81"/>
       <c r="J6" s="37"/>
       <c r="K6" s="58"/>
       <c r="L6" s="37">
@@ -2488,38 +2502,38 @@
       <c r="AI6" s="56">
         <v>21</v>
       </c>
-      <c r="AJ6" s="111"/>
-      <c r="AK6" s="112"/>
+      <c r="AJ6" s="80"/>
+      <c r="AK6" s="81"/>
       <c r="AL6" s="41"/>
       <c r="AM6" s="56"/>
-      <c r="AN6" s="111"/>
-      <c r="AO6" s="114"/>
+      <c r="AN6" s="80"/>
+      <c r="AO6" s="83"/>
       <c r="AP6" s="41">
         <v>43</v>
       </c>
-      <c r="AQ6" s="98">
+      <c r="AQ6" s="67">
         <v>17</v>
       </c>
-      <c r="AR6" s="100">
-        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6+AD6+AF6+AH6+AJ6+AL6+AN6+AP6</f>
+      <c r="AR6" s="69">
+        <f t="shared" si="1"/>
         <v>595</v>
       </c>
       <c r="AS6" s="8">
-        <f>COUNTIF(D6:AP6,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="AT6" s="102">
+      <c r="AT6" s="71">
         <v>2</v>
       </c>
-      <c r="AU6" s="106">
+      <c r="AU6" s="75">
         <v>6</v>
       </c>
       <c r="AV6" s="25">
-        <f>SUMIF(G6:AQ6, "&lt;30")+AT6+AU6</f>
+        <f t="shared" si="3"/>
         <v>278</v>
       </c>
       <c r="AW6" s="39">
-        <f>AV6/AS6</f>
+        <f t="shared" si="4"/>
         <v>19.857142857142858</v>
       </c>
       <c r="AX6" s="34"/>
@@ -2536,15 +2550,15 @@
         <v>37</v>
       </c>
       <c r="C7" s="64">
-        <f>ROUND((AR7-(36*AS7))/AS7,0)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D7" s="111"/>
-      <c r="E7" s="112"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="81"/>
       <c r="F7" s="9"/>
       <c r="G7" s="58"/>
-      <c r="H7" s="111"/>
-      <c r="I7" s="112"/>
+      <c r="H7" s="80"/>
+      <c r="I7" s="81"/>
       <c r="J7" s="9"/>
       <c r="K7" s="58"/>
       <c r="L7" s="9"/>
@@ -2595,38 +2609,38 @@
       </c>
       <c r="AH7" s="43"/>
       <c r="AI7" s="56"/>
-      <c r="AJ7" s="111"/>
-      <c r="AK7" s="112"/>
-      <c r="AL7" s="128">
+      <c r="AJ7" s="80"/>
+      <c r="AK7" s="81"/>
+      <c r="AL7" s="97">
         <v>46</v>
       </c>
       <c r="AM7" s="56">
         <v>20</v>
       </c>
-      <c r="AN7" s="111"/>
-      <c r="AO7" s="114"/>
-      <c r="AP7" s="129"/>
-      <c r="AQ7" s="98"/>
-      <c r="AR7" s="100">
-        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7+AD7+AF7+AH7+AJ7+AL7+AN7+AP7</f>
+      <c r="AN7" s="80"/>
+      <c r="AO7" s="83"/>
+      <c r="AP7" s="98"/>
+      <c r="AQ7" s="67"/>
+      <c r="AR7" s="69">
+        <f t="shared" si="1"/>
         <v>333</v>
       </c>
       <c r="AS7" s="8">
-        <f>COUNTIF(D7:AP7,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AT7" s="102">
+      <c r="AT7" s="71">
         <v>2</v>
       </c>
-      <c r="AU7" s="106">
+      <c r="AU7" s="75">
         <v>1</v>
       </c>
       <c r="AV7" s="25">
-        <f>SUMIF(G7:AQ7, "&lt;30")+AT7+AU7</f>
+        <f t="shared" si="3"/>
         <v>137</v>
       </c>
       <c r="AW7" s="39">
-        <f>AV7/AS7</f>
+        <f t="shared" si="4"/>
         <v>19.571428571428573</v>
       </c>
       <c r="AX7" s="36"/>
@@ -2643,19 +2657,19 @@
         <v>26</v>
       </c>
       <c r="C8" s="64">
-        <f>ROUND((AR8-(36*AS8))/AS8,0)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D8" s="111"/>
-      <c r="E8" s="112"/>
+      <c r="D8" s="80"/>
+      <c r="E8" s="81"/>
       <c r="F8" s="9">
         <v>41</v>
       </c>
       <c r="G8" s="58">
         <v>21</v>
       </c>
-      <c r="H8" s="111"/>
-      <c r="I8" s="112"/>
+      <c r="H8" s="80"/>
+      <c r="I8" s="81"/>
       <c r="J8" s="9"/>
       <c r="K8" s="58"/>
       <c r="L8" s="9"/>
@@ -2714,38 +2728,38 @@
       <c r="AI8" s="56">
         <v>23</v>
       </c>
-      <c r="AJ8" s="111"/>
-      <c r="AK8" s="112"/>
+      <c r="AJ8" s="80"/>
+      <c r="AK8" s="81"/>
       <c r="AL8" s="31"/>
       <c r="AM8" s="56"/>
-      <c r="AN8" s="111"/>
-      <c r="AO8" s="114"/>
+      <c r="AN8" s="80"/>
+      <c r="AO8" s="83"/>
       <c r="AP8" s="26">
         <v>41</v>
       </c>
-      <c r="AQ8" s="98">
+      <c r="AQ8" s="67">
         <v>20</v>
       </c>
-      <c r="AR8" s="100">
-        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8+AD8+AF8+AH8+AJ8+AL8+AN8+AP8</f>
+      <c r="AR8" s="69">
+        <f t="shared" si="1"/>
         <v>429</v>
       </c>
       <c r="AS8" s="8">
-        <f>COUNTIF(D8:AP8,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT8" s="102">
+      <c r="AT8" s="71">
         <v>3</v>
       </c>
-      <c r="AU8" s="106">
+      <c r="AU8" s="75">
         <v>3</v>
       </c>
       <c r="AV8" s="25">
-        <f>SUMIF(G8:AQ8, "&lt;30")+AT8+AU8</f>
+        <f t="shared" si="3"/>
         <v>195</v>
       </c>
       <c r="AW8" s="39">
-        <f>AV8/AS8</f>
+        <f t="shared" si="4"/>
         <v>19.5</v>
       </c>
       <c r="AX8" s="50"/>
@@ -2762,15 +2776,15 @@
         <v>40</v>
       </c>
       <c r="C9" s="64">
-        <f>ROUND((AR9-(36*AS9))/AS9,0)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D9" s="111"/>
-      <c r="E9" s="112"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="81"/>
       <c r="F9" s="9"/>
       <c r="G9" s="58"/>
-      <c r="H9" s="111"/>
-      <c r="I9" s="112"/>
+      <c r="H9" s="80"/>
+      <c r="I9" s="81"/>
       <c r="J9" s="9">
         <v>52</v>
       </c>
@@ -2823,7 +2837,7 @@
       <c r="AC9" s="58">
         <v>21</v>
       </c>
-      <c r="AD9" s="127">
+      <c r="AD9" s="96">
         <v>43</v>
       </c>
       <c r="AE9" s="56">
@@ -2841,42 +2855,42 @@
       <c r="AI9" s="56">
         <v>15</v>
       </c>
-      <c r="AJ9" s="111"/>
-      <c r="AK9" s="112"/>
+      <c r="AJ9" s="80"/>
+      <c r="AK9" s="81"/>
       <c r="AL9" s="43">
         <v>50</v>
       </c>
       <c r="AM9" s="56">
         <v>16</v>
       </c>
-      <c r="AN9" s="111"/>
-      <c r="AO9" s="114"/>
+      <c r="AN9" s="80"/>
+      <c r="AO9" s="83"/>
       <c r="AP9" s="43">
         <v>51</v>
       </c>
-      <c r="AQ9" s="98">
+      <c r="AQ9" s="67">
         <v>17</v>
       </c>
-      <c r="AR9" s="100">
-        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9+AD9+AF9+AH9+AJ9+AL9+AN9+AP9</f>
+      <c r="AR9" s="69">
+        <f t="shared" si="1"/>
         <v>628</v>
       </c>
       <c r="AS9" s="8">
-        <f>COUNTIF(D9:AP9,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="AT9" s="102">
+      <c r="AT9" s="71">
         <v>1</v>
       </c>
-      <c r="AU9" s="106">
+      <c r="AU9" s="75">
         <v>2</v>
       </c>
       <c r="AV9" s="25">
-        <f>SUMIF(G9:AQ9, "&lt;30")+AT9+AU9</f>
+        <f t="shared" si="3"/>
         <v>253</v>
       </c>
       <c r="AW9" s="39">
-        <f>AV9/AS9</f>
+        <f t="shared" si="4"/>
         <v>19.46153846153846</v>
       </c>
       <c r="AX9" s="34"/>
@@ -2893,19 +2907,19 @@
         <v>13</v>
       </c>
       <c r="C10" s="64">
-        <f>ROUND((AR10-(36*AS10))/AS10,0)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D10" s="111"/>
-      <c r="E10" s="112"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="81"/>
       <c r="F10" s="42">
         <v>42</v>
       </c>
       <c r="G10" s="58">
         <v>25</v>
       </c>
-      <c r="H10" s="111"/>
-      <c r="I10" s="112"/>
+      <c r="H10" s="80"/>
+      <c r="I10" s="81"/>
       <c r="J10" s="42"/>
       <c r="K10" s="58"/>
       <c r="L10" s="42">
@@ -2976,42 +2990,42 @@
       <c r="AI10" s="56">
         <v>17</v>
       </c>
-      <c r="AJ10" s="111"/>
-      <c r="AK10" s="112"/>
+      <c r="AJ10" s="80"/>
+      <c r="AK10" s="81"/>
       <c r="AL10" s="26">
         <v>50</v>
       </c>
       <c r="AM10" s="56">
         <v>15</v>
       </c>
-      <c r="AN10" s="111"/>
-      <c r="AO10" s="114"/>
+      <c r="AN10" s="80"/>
+      <c r="AO10" s="83"/>
       <c r="AP10" s="26">
         <v>42</v>
       </c>
-      <c r="AQ10" s="98">
+      <c r="AQ10" s="67">
         <v>23</v>
       </c>
-      <c r="AR10" s="100">
-        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10+AD10+AF10+AH10+AJ10+AL10+AN10+AP10</f>
+      <c r="AR10" s="69">
+        <f t="shared" si="1"/>
         <v>655</v>
       </c>
       <c r="AS10" s="8">
-        <f>COUNTIF(D10:AP10,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="AT10" s="102">
+      <c r="AT10" s="71">
         <v>2</v>
       </c>
-      <c r="AU10" s="106">
+      <c r="AU10" s="75">
         <v>3</v>
       </c>
       <c r="AV10" s="25">
-        <f>SUMIF(G10:AQ10, "&lt;30")+AT10+AU10</f>
+        <f t="shared" si="3"/>
         <v>271</v>
       </c>
       <c r="AW10" s="39">
-        <f>AV10/AS10</f>
+        <f t="shared" si="4"/>
         <v>19.357142857142858</v>
       </c>
       <c r="AX10" s="51"/>
@@ -3028,19 +3042,19 @@
         <v>11</v>
       </c>
       <c r="C11" s="64">
-        <f>ROUND((AR11-(36*AS11))/AS11,0)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D11" s="111"/>
-      <c r="E11" s="112"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="81"/>
       <c r="F11" s="9">
         <v>42</v>
       </c>
       <c r="G11" s="58">
         <v>27</v>
       </c>
-      <c r="H11" s="111"/>
-      <c r="I11" s="112"/>
+      <c r="H11" s="80"/>
+      <c r="I11" s="81"/>
       <c r="J11" s="9"/>
       <c r="K11" s="58"/>
       <c r="L11" s="9">
@@ -3095,42 +3109,42 @@
       <c r="AI11" s="56">
         <v>18</v>
       </c>
-      <c r="AJ11" s="111"/>
-      <c r="AK11" s="112"/>
+      <c r="AJ11" s="80"/>
+      <c r="AK11" s="81"/>
       <c r="AL11" s="41">
         <v>50</v>
       </c>
       <c r="AM11" s="56">
         <v>18</v>
       </c>
-      <c r="AN11" s="111"/>
-      <c r="AO11" s="114"/>
+      <c r="AN11" s="80"/>
+      <c r="AO11" s="83"/>
       <c r="AP11" s="41">
         <v>52</v>
       </c>
-      <c r="AQ11" s="98">
+      <c r="AQ11" s="67">
         <v>16</v>
       </c>
-      <c r="AR11" s="100">
-        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11+AD11+AF11+AH11+AJ11+AL11+AN11+AP11</f>
+      <c r="AR11" s="69">
+        <f t="shared" si="1"/>
         <v>500</v>
       </c>
       <c r="AS11" s="8">
-        <f>COUNTIF(D11:AP11,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT11" s="102">
+      <c r="AT11" s="71">
         <v>1</v>
       </c>
-      <c r="AU11" s="106">
+      <c r="AU11" s="75">
         <v>1</v>
       </c>
       <c r="AV11" s="25">
-        <f>SUMIF(G11:AQ11, "&lt;30")+AT11+AU11</f>
+        <f t="shared" si="3"/>
         <v>188</v>
       </c>
       <c r="AW11" s="39">
-        <f>AV11/AS11</f>
+        <f t="shared" si="4"/>
         <v>18.8</v>
       </c>
       <c r="AX11" s="34"/>
@@ -3147,19 +3161,19 @@
         <v>31</v>
       </c>
       <c r="C12" s="64">
-        <f>ROUND((AR12-(36*AS12))/AS12,0)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="D12" s="111"/>
-      <c r="E12" s="112"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="81"/>
       <c r="F12" s="9">
         <v>51</v>
       </c>
       <c r="G12" s="58">
         <v>18</v>
       </c>
-      <c r="H12" s="111"/>
-      <c r="I12" s="112"/>
+      <c r="H12" s="80"/>
+      <c r="I12" s="81"/>
       <c r="J12" s="9"/>
       <c r="K12" s="58"/>
       <c r="L12" s="9"/>
@@ -3202,34 +3216,34 @@
       <c r="AG12" s="56"/>
       <c r="AH12" s="41"/>
       <c r="AI12" s="56"/>
-      <c r="AJ12" s="111"/>
-      <c r="AK12" s="112"/>
+      <c r="AJ12" s="80"/>
+      <c r="AK12" s="81"/>
       <c r="AL12" s="41"/>
       <c r="AM12" s="56"/>
-      <c r="AN12" s="111"/>
-      <c r="AO12" s="114"/>
+      <c r="AN12" s="80"/>
+      <c r="AO12" s="83"/>
       <c r="AP12" s="41">
         <v>51</v>
       </c>
-      <c r="AQ12" s="98">
+      <c r="AQ12" s="67">
         <v>19</v>
       </c>
-      <c r="AR12" s="100">
-        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12+AD12+AF12+AH12+AJ12+AL12+AN12+AP12</f>
+      <c r="AR12" s="69">
+        <f t="shared" si="1"/>
         <v>304</v>
       </c>
       <c r="AS12" s="8">
-        <f>COUNTIF(D12:AP12,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="AT12" s="102"/>
-      <c r="AU12" s="106"/>
+      <c r="AT12" s="71"/>
+      <c r="AU12" s="75"/>
       <c r="AV12" s="25">
-        <f>SUMIF(G12:AQ12, "&lt;30")+AT12+AU12</f>
+        <f t="shared" si="3"/>
         <v>111</v>
       </c>
       <c r="AW12" s="39">
-        <f>AV12/AS12</f>
+        <f t="shared" si="4"/>
         <v>18.5</v>
       </c>
       <c r="AX12" s="36"/>
@@ -3246,15 +3260,15 @@
         <v>38</v>
       </c>
       <c r="C13" s="64">
-        <f>ROUND((AR13-(36*AS13))/AS13,0)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D13" s="111"/>
-      <c r="E13" s="112"/>
+      <c r="D13" s="80"/>
+      <c r="E13" s="81"/>
       <c r="F13" s="9"/>
       <c r="G13" s="58"/>
-      <c r="H13" s="111"/>
-      <c r="I13" s="112"/>
+      <c r="H13" s="80"/>
+      <c r="I13" s="81"/>
       <c r="J13" s="9"/>
       <c r="K13" s="58"/>
       <c r="L13" s="9"/>
@@ -3313,36 +3327,36 @@
       <c r="AI13" s="56">
         <v>19</v>
       </c>
-      <c r="AJ13" s="111"/>
-      <c r="AK13" s="112"/>
+      <c r="AJ13" s="80"/>
+      <c r="AK13" s="81"/>
       <c r="AL13" s="41"/>
       <c r="AM13" s="56"/>
-      <c r="AN13" s="111"/>
-      <c r="AO13" s="114"/>
+      <c r="AN13" s="80"/>
+      <c r="AO13" s="83"/>
       <c r="AP13" s="41">
         <v>47</v>
       </c>
-      <c r="AQ13" s="98">
+      <c r="AQ13" s="67">
         <v>20</v>
       </c>
-      <c r="AR13" s="100">
-        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13+AD13+AF13+AH13+AJ13+AL13+AN13+AP13</f>
+      <c r="AR13" s="69">
+        <f t="shared" si="1"/>
         <v>436</v>
       </c>
       <c r="AS13" s="8">
-        <f>COUNTIF(D13:AP13,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="AT13" s="102"/>
-      <c r="AU13" s="106">
+      <c r="AT13" s="71"/>
+      <c r="AU13" s="75">
         <v>1</v>
       </c>
       <c r="AV13" s="25">
-        <f>SUMIF(G13:AQ13, "&lt;30")+AT13+AU13</f>
+        <f t="shared" si="3"/>
         <v>166</v>
       </c>
       <c r="AW13" s="39">
-        <f>AV13/AS13</f>
+        <f t="shared" si="4"/>
         <v>18.444444444444443</v>
       </c>
       <c r="AX13" s="34"/>
@@ -3359,19 +3373,19 @@
         <v>11</v>
       </c>
       <c r="C14" s="64">
-        <f>ROUND((AR14-(36*AS14))/AS14,0)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="D14" s="111"/>
-      <c r="E14" s="112"/>
+      <c r="D14" s="80"/>
+      <c r="E14" s="81"/>
       <c r="F14" s="9">
         <v>59</v>
       </c>
       <c r="G14" s="58">
         <v>17</v>
       </c>
-      <c r="H14" s="111"/>
-      <c r="I14" s="112"/>
+      <c r="H14" s="80"/>
+      <c r="I14" s="81"/>
       <c r="J14" s="9"/>
       <c r="K14" s="58"/>
       <c r="L14" s="9"/>
@@ -3406,30 +3420,30 @@
       <c r="AG14" s="56"/>
       <c r="AH14" s="41"/>
       <c r="AI14" s="56"/>
-      <c r="AJ14" s="111"/>
-      <c r="AK14" s="112"/>
+      <c r="AJ14" s="80"/>
+      <c r="AK14" s="81"/>
       <c r="AL14" s="41"/>
       <c r="AM14" s="56"/>
-      <c r="AN14" s="111"/>
-      <c r="AO14" s="114"/>
+      <c r="AN14" s="80"/>
+      <c r="AO14" s="83"/>
       <c r="AP14" s="41"/>
-      <c r="AQ14" s="98"/>
-      <c r="AR14" s="100">
-        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14+AD14+AF14+AH14+AJ14+AL14+AN14+AP14</f>
+      <c r="AQ14" s="67"/>
+      <c r="AR14" s="69">
+        <f t="shared" si="1"/>
         <v>173</v>
       </c>
       <c r="AS14" s="8">
-        <f>COUNTIF(D14:AP14,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AT14" s="102"/>
-      <c r="AU14" s="106"/>
+      <c r="AT14" s="71"/>
+      <c r="AU14" s="75"/>
       <c r="AV14" s="25">
-        <f>SUMIF(G14:AQ14, "&lt;30")+AT14+AU14</f>
+        <f t="shared" si="3"/>
         <v>55</v>
       </c>
       <c r="AW14" s="39">
-        <f>AV14/AS14</f>
+        <f t="shared" si="4"/>
         <v>18.333333333333332</v>
       </c>
       <c r="AX14" s="36"/>
@@ -3446,15 +3460,15 @@
         <v>33</v>
       </c>
       <c r="C15" s="64">
-        <f>ROUND((AR15-(36*AS15))/AS15,0)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D15" s="111"/>
-      <c r="E15" s="112"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="81"/>
       <c r="F15" s="11"/>
       <c r="G15" s="58"/>
-      <c r="H15" s="111"/>
-      <c r="I15" s="112"/>
+      <c r="H15" s="80"/>
+      <c r="I15" s="81"/>
       <c r="J15" s="11"/>
       <c r="K15" s="58"/>
       <c r="L15" s="11"/>
@@ -3521,38 +3535,38 @@
       <c r="AI15" s="56">
         <v>20</v>
       </c>
-      <c r="AJ15" s="111"/>
-      <c r="AK15" s="112"/>
+      <c r="AJ15" s="80"/>
+      <c r="AK15" s="81"/>
       <c r="AL15" s="26">
         <v>51</v>
       </c>
       <c r="AM15" s="56">
         <v>15</v>
       </c>
-      <c r="AN15" s="111"/>
-      <c r="AO15" s="114"/>
+      <c r="AN15" s="80"/>
+      <c r="AO15" s="83"/>
       <c r="AP15" s="26">
         <v>49</v>
       </c>
-      <c r="AQ15" s="98">
+      <c r="AQ15" s="67">
         <v>17</v>
       </c>
-      <c r="AR15" s="100">
-        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15+AD15+AF15+AH15+AJ15+AL15+AN15+AP15</f>
+      <c r="AR15" s="69">
+        <f t="shared" si="1"/>
         <v>579</v>
       </c>
       <c r="AS15" s="8">
-        <f>COUNTIF(D15:AP15,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="AT15" s="102"/>
-      <c r="AU15" s="106"/>
+      <c r="AT15" s="71"/>
+      <c r="AU15" s="75"/>
       <c r="AV15" s="25">
-        <f>SUMIF(G15:AQ15, "&lt;30")+AT15+AU15</f>
+        <f t="shared" si="3"/>
         <v>216</v>
       </c>
       <c r="AW15" s="39">
-        <f>AV15/AS15</f>
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="AX15" s="34"/>
@@ -3569,19 +3583,19 @@
         <v>15</v>
       </c>
       <c r="C16" s="64">
-        <f>ROUND((AR16-(36*AS16))/AS16,0)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="D16" s="111"/>
-      <c r="E16" s="112"/>
+      <c r="D16" s="80"/>
+      <c r="E16" s="81"/>
       <c r="F16" s="9">
         <v>55</v>
       </c>
       <c r="G16" s="58">
         <v>16</v>
       </c>
-      <c r="H16" s="111"/>
-      <c r="I16" s="112"/>
+      <c r="H16" s="80"/>
+      <c r="I16" s="81"/>
       <c r="J16" s="9"/>
       <c r="K16" s="58"/>
       <c r="L16" s="9">
@@ -3648,32 +3662,32 @@
       <c r="AI16" s="56">
         <v>20</v>
       </c>
-      <c r="AJ16" s="111"/>
-      <c r="AK16" s="112"/>
+      <c r="AJ16" s="80"/>
+      <c r="AK16" s="81"/>
       <c r="AL16" s="41"/>
       <c r="AM16" s="56"/>
-      <c r="AN16" s="111"/>
-      <c r="AO16" s="114"/>
+      <c r="AN16" s="80"/>
+      <c r="AO16" s="83"/>
       <c r="AP16" s="41"/>
-      <c r="AQ16" s="98"/>
-      <c r="AR16" s="100">
-        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16+AD16+AF16+AH16+AJ16+AL16+AN16+AP16</f>
+      <c r="AQ16" s="67"/>
+      <c r="AR16" s="69">
+        <f t="shared" si="1"/>
         <v>594</v>
       </c>
       <c r="AS16" s="8">
-        <f>COUNTIF(D16:AP16,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AT16" s="102">
+      <c r="AT16" s="71">
         <v>2</v>
       </c>
-      <c r="AU16" s="106"/>
+      <c r="AU16" s="75"/>
       <c r="AV16" s="25">
-        <f>SUMIF(G16:AQ16, "&lt;30")+AT16+AU16</f>
+        <f t="shared" si="3"/>
         <v>197</v>
       </c>
       <c r="AW16" s="39">
-        <f>AV16/AS16</f>
+        <f t="shared" si="4"/>
         <v>17.90909090909091</v>
       </c>
       <c r="AX16" s="36"/>
@@ -3690,15 +3704,15 @@
         <v>56</v>
       </c>
       <c r="C17" s="64">
-        <f>ROUND((AR17-(36*AS17))/AS17,0)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D17" s="111"/>
-      <c r="E17" s="112"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="81"/>
       <c r="F17" s="11"/>
       <c r="G17" s="58"/>
-      <c r="H17" s="111"/>
-      <c r="I17" s="112"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
       <c r="J17" s="11"/>
       <c r="K17" s="58"/>
       <c r="L17" s="11"/>
@@ -3749,36 +3763,36 @@
       </c>
       <c r="AH17" s="26"/>
       <c r="AI17" s="56"/>
-      <c r="AJ17" s="111"/>
-      <c r="AK17" s="112"/>
+      <c r="AJ17" s="80"/>
+      <c r="AK17" s="81"/>
       <c r="AL17" s="26"/>
       <c r="AM17" s="56"/>
-      <c r="AN17" s="111"/>
-      <c r="AO17" s="114"/>
+      <c r="AN17" s="80"/>
+      <c r="AO17" s="83"/>
       <c r="AP17" s="26">
         <v>44</v>
       </c>
-      <c r="AQ17" s="98">
+      <c r="AQ17" s="67">
         <v>21</v>
       </c>
-      <c r="AR17" s="100">
-        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17+AD17+AF17+AH17+AJ17+AL17+AN17+AP17</f>
+      <c r="AR17" s="69">
+        <f t="shared" si="1"/>
         <v>323</v>
       </c>
       <c r="AS17" s="8">
-        <f>COUNTIF(D17:AP17,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AT17" s="102"/>
-      <c r="AU17" s="106">
+      <c r="AT17" s="71"/>
+      <c r="AU17" s="75">
         <v>2</v>
       </c>
       <c r="AV17" s="25">
-        <f>SUMIF(G17:AQ17, "&lt;30")+AT17+AU17</f>
+        <f t="shared" si="3"/>
         <v>125</v>
       </c>
       <c r="AW17" s="39">
-        <f>AV17/AS17</f>
+        <f t="shared" si="4"/>
         <v>17.857142857142858</v>
       </c>
       <c r="AX17" s="34"/>
@@ -3795,19 +3809,19 @@
         <v>19</v>
       </c>
       <c r="C18" s="64">
-        <f>ROUND((AR18-(36*AS18))/AS18,0)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D18" s="111"/>
-      <c r="E18" s="112"/>
+      <c r="D18" s="80"/>
+      <c r="E18" s="81"/>
       <c r="F18" s="9">
         <v>46</v>
       </c>
       <c r="G18" s="58">
         <v>16</v>
       </c>
-      <c r="H18" s="111"/>
-      <c r="I18" s="112"/>
+      <c r="H18" s="80"/>
+      <c r="I18" s="81"/>
       <c r="J18" s="9"/>
       <c r="K18" s="58"/>
       <c r="L18" s="9"/>
@@ -3866,38 +3880,38 @@
       <c r="AI18" s="56">
         <v>15</v>
       </c>
-      <c r="AJ18" s="111"/>
-      <c r="AK18" s="112"/>
+      <c r="AJ18" s="80"/>
+      <c r="AK18" s="81"/>
       <c r="AL18" s="41"/>
       <c r="AM18" s="56"/>
-      <c r="AN18" s="111"/>
-      <c r="AO18" s="114"/>
-      <c r="AP18" s="41">
+      <c r="AN18" s="80"/>
+      <c r="AO18" s="83"/>
+      <c r="AP18" s="131">
         <v>48</v>
       </c>
-      <c r="AQ18" s="98">
+      <c r="AQ18" s="67">
         <v>15</v>
       </c>
-      <c r="AR18" s="100">
-        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18+AD18+AF18+AH18+AJ18+AL18+AN18+AP18</f>
+      <c r="AR18" s="69">
+        <f t="shared" si="1"/>
         <v>453</v>
       </c>
       <c r="AS18" s="8">
-        <f>COUNTIF(D18:AP18,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT18" s="102">
+      <c r="AT18" s="71">
         <v>2</v>
       </c>
-      <c r="AU18" s="106">
+      <c r="AU18" s="75">
         <v>1</v>
       </c>
       <c r="AV18" s="25">
-        <f>SUMIF(G18:AQ18, "&lt;30")+AT18+AU18</f>
+        <f t="shared" si="3"/>
         <v>178</v>
       </c>
       <c r="AW18" s="39">
-        <f>AV18/AS18</f>
+        <f t="shared" si="4"/>
         <v>17.8</v>
       </c>
       <c r="AX18" s="36"/>
@@ -3914,19 +3928,19 @@
         <v>29</v>
       </c>
       <c r="C19" s="64">
-        <f>ROUND((AR19-(36*AS19))/AS19,0)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D19" s="111"/>
-      <c r="E19" s="112"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="81"/>
       <c r="F19" s="9">
         <v>46</v>
       </c>
       <c r="G19" s="58">
         <v>18</v>
       </c>
-      <c r="H19" s="111"/>
-      <c r="I19" s="112"/>
+      <c r="H19" s="80"/>
+      <c r="I19" s="81"/>
       <c r="J19" s="9"/>
       <c r="K19" s="58"/>
       <c r="L19" s="9">
@@ -3989,32 +4003,32 @@
       <c r="AI19" s="56">
         <v>22</v>
       </c>
-      <c r="AJ19" s="111"/>
-      <c r="AK19" s="112"/>
+      <c r="AJ19" s="80"/>
+      <c r="AK19" s="81"/>
       <c r="AL19" s="41"/>
       <c r="AM19" s="56"/>
-      <c r="AN19" s="111"/>
-      <c r="AO19" s="114"/>
+      <c r="AN19" s="80"/>
+      <c r="AO19" s="83"/>
       <c r="AP19" s="41"/>
-      <c r="AQ19" s="98"/>
-      <c r="AR19" s="100">
-        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19+AD19+AF19+AH19+AJ19+AL19+AN19+AP19</f>
+      <c r="AQ19" s="67"/>
+      <c r="AR19" s="69">
+        <f t="shared" si="1"/>
         <v>472</v>
       </c>
       <c r="AS19" s="8">
-        <f>COUNTIF(D19:AP19,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT19" s="103"/>
-      <c r="AU19" s="107">
+      <c r="AT19" s="72"/>
+      <c r="AU19" s="76">
         <v>1</v>
       </c>
       <c r="AV19" s="25">
-        <f>SUMIF(G19:AQ19, "&lt;30")+AT19+AU19</f>
+        <f t="shared" si="3"/>
         <v>174</v>
       </c>
       <c r="AW19" s="39">
-        <f>AV19/AS19</f>
+        <f t="shared" si="4"/>
         <v>17.399999999999999</v>
       </c>
       <c r="AX19" s="36"/>
@@ -4031,19 +4045,19 @@
         <v>24</v>
       </c>
       <c r="C20" s="64">
-        <f>ROUND((AR20-(36*AS20))/AS20,0)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="D20" s="111"/>
-      <c r="E20" s="112"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="81"/>
       <c r="F20" s="10">
         <v>61</v>
       </c>
       <c r="G20" s="58">
         <v>14</v>
       </c>
-      <c r="H20" s="111"/>
-      <c r="I20" s="112"/>
+      <c r="H20" s="80"/>
+      <c r="I20" s="81"/>
       <c r="J20" s="10">
         <v>56</v>
       </c>
@@ -4114,32 +4128,32 @@
       <c r="AI20" s="56">
         <v>23</v>
       </c>
-      <c r="AJ20" s="111"/>
-      <c r="AK20" s="112"/>
+      <c r="AJ20" s="80"/>
+      <c r="AK20" s="81"/>
       <c r="AL20" s="26"/>
       <c r="AM20" s="56"/>
-      <c r="AN20" s="111"/>
-      <c r="AO20" s="114"/>
+      <c r="AN20" s="80"/>
+      <c r="AO20" s="83"/>
       <c r="AP20" s="26"/>
-      <c r="AQ20" s="98"/>
-      <c r="AR20" s="100">
-        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20+AD20+AF20+AH20+AJ20+AL20+AN20+AP20</f>
+      <c r="AQ20" s="67"/>
+      <c r="AR20" s="69">
+        <f t="shared" si="1"/>
         <v>714</v>
       </c>
       <c r="AS20" s="8">
-        <f>COUNTIF(D20:AP20,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="AT20" s="102">
+      <c r="AT20" s="71">
         <v>2</v>
       </c>
-      <c r="AU20" s="106"/>
+      <c r="AU20" s="75"/>
       <c r="AV20" s="25">
-        <f>SUMIF(G20:AQ20, "&lt;30")+AT20+AU20</f>
+        <f t="shared" si="3"/>
         <v>205</v>
       </c>
       <c r="AW20" s="39">
-        <f>AV20/AS20</f>
+        <f t="shared" si="4"/>
         <v>17.083333333333332</v>
       </c>
       <c r="AX20" s="34"/>
@@ -4158,16 +4172,16 @@
       <c r="C21" s="64">
         <v>18</v>
       </c>
-      <c r="D21" s="111"/>
-      <c r="E21" s="112"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="81"/>
       <c r="F21" s="9">
         <v>56</v>
       </c>
       <c r="G21" s="58">
         <v>16</v>
       </c>
-      <c r="H21" s="111"/>
-      <c r="I21" s="112"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="81"/>
       <c r="J21" s="9"/>
       <c r="K21" s="58"/>
       <c r="L21" s="9"/>
@@ -4194,30 +4208,30 @@
       <c r="AG21" s="56"/>
       <c r="AH21" s="41"/>
       <c r="AI21" s="56"/>
-      <c r="AJ21" s="111"/>
-      <c r="AK21" s="112"/>
+      <c r="AJ21" s="80"/>
+      <c r="AK21" s="81"/>
       <c r="AL21" s="41"/>
       <c r="AM21" s="56"/>
-      <c r="AN21" s="111"/>
-      <c r="AO21" s="114"/>
+      <c r="AN21" s="80"/>
+      <c r="AO21" s="83"/>
       <c r="AP21" s="41"/>
-      <c r="AQ21" s="98"/>
-      <c r="AR21" s="100">
-        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21+AD21+AF21+AH21+AJ21+AL21+AN21+AP21</f>
+      <c r="AQ21" s="67"/>
+      <c r="AR21" s="69">
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="AS21" s="8">
-        <f>COUNTIF(D21:AP21,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT21" s="102"/>
-      <c r="AU21" s="106"/>
+      <c r="AT21" s="71"/>
+      <c r="AU21" s="75"/>
       <c r="AV21" s="25">
-        <f>SUMIF(G21:AQ21, "&lt;30")+AT21+AU21</f>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="AW21" s="39">
-        <f>AV21/AS21</f>
+        <f t="shared" si="4"/>
         <v>16</v>
       </c>
       <c r="AX21" s="36"/>
@@ -4236,12 +4250,12 @@
       <c r="C22" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="111"/>
-      <c r="E22" s="112"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="81"/>
       <c r="F22" s="47"/>
       <c r="G22" s="58"/>
-      <c r="H22" s="111"/>
-      <c r="I22" s="112"/>
+      <c r="H22" s="80"/>
+      <c r="I22" s="81"/>
       <c r="J22" s="47"/>
       <c r="K22" s="58"/>
       <c r="L22" s="47">
@@ -4270,32 +4284,32 @@
       <c r="AG22" s="58"/>
       <c r="AH22" s="57"/>
       <c r="AI22" s="58"/>
-      <c r="AJ22" s="111"/>
-      <c r="AK22" s="112"/>
+      <c r="AJ22" s="80"/>
+      <c r="AK22" s="81"/>
       <c r="AL22" s="57"/>
       <c r="AM22" s="58"/>
-      <c r="AN22" s="111"/>
-      <c r="AO22" s="114"/>
+      <c r="AN22" s="80"/>
+      <c r="AO22" s="83"/>
       <c r="AP22" s="48"/>
-      <c r="AQ22" s="98"/>
-      <c r="AR22" s="100">
-        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22+AD22+AF22+AH22+AJ22+AL22+AN22+AP22</f>
+      <c r="AQ22" s="67"/>
+      <c r="AR22" s="69">
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="AS22" s="8">
-        <f>COUNTIF(D22:AP22,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT22" s="102">
+      <c r="AT22" s="71">
         <v>1</v>
       </c>
-      <c r="AU22" s="106"/>
+      <c r="AU22" s="75"/>
       <c r="AV22" s="25">
-        <f>SUMIF(G22:AQ22, "&lt;30")+AT22+AU22</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="AW22" s="39">
-        <f>AV22/AS22</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AX22" s="50"/>
@@ -4314,12 +4328,12 @@
       <c r="C23" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="111"/>
-      <c r="E23" s="112"/>
+      <c r="D23" s="80"/>
+      <c r="E23" s="81"/>
       <c r="F23" s="47"/>
       <c r="G23" s="58"/>
-      <c r="H23" s="111"/>
-      <c r="I23" s="112"/>
+      <c r="H23" s="80"/>
+      <c r="I23" s="81"/>
       <c r="J23" s="47"/>
       <c r="K23" s="58"/>
       <c r="L23" s="47"/>
@@ -4346,32 +4360,32 @@
       <c r="AG23" s="58"/>
       <c r="AH23" s="57"/>
       <c r="AI23" s="58"/>
-      <c r="AJ23" s="111"/>
-      <c r="AK23" s="112"/>
+      <c r="AJ23" s="80"/>
+      <c r="AK23" s="81"/>
       <c r="AL23" s="57">
         <v>50</v>
       </c>
       <c r="AM23" s="58"/>
-      <c r="AN23" s="111"/>
-      <c r="AO23" s="114"/>
+      <c r="AN23" s="80"/>
+      <c r="AO23" s="83"/>
       <c r="AP23" s="48"/>
-      <c r="AQ23" s="98"/>
-      <c r="AR23" s="100">
-        <f>F23+J23+L23+N23+P23+R23+T23+V23+X23+Z23+AB23+AD23+AF23+AH23+AJ23+AL23+AN23+AP23</f>
+      <c r="AQ23" s="67"/>
+      <c r="AR23" s="69">
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="AS23" s="8">
-        <f>COUNTIF(D23:AP23,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT23" s="102"/>
-      <c r="AU23" s="106"/>
+      <c r="AT23" s="71"/>
+      <c r="AU23" s="75"/>
       <c r="AV23" s="25">
-        <f>SUMIF(G23:AQ23, "&lt;30")+AT23+AU23</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AW23" s="39">
-        <f>AV23/AS23</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AX23" s="50"/>
@@ -4380,7 +4394,7 @@
       <c r="BA23" s="52"/>
       <c r="BB23" s="54"/>
     </row>
-    <row r="24" spans="1:54" ht="17" thickBot="1">
+    <row r="24" spans="1:54" ht="16.5" thickBot="1">
       <c r="A24" s="61" t="s">
         <v>10</v>
       </c>
@@ -4390,63 +4404,63 @@
       <c r="C24" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="111"/>
-      <c r="E24" s="112"/>
-      <c r="F24" s="115"/>
-      <c r="G24" s="116"/>
-      <c r="H24" s="111"/>
-      <c r="I24" s="112"/>
-      <c r="J24" s="115"/>
-      <c r="K24" s="116"/>
-      <c r="L24" s="115"/>
-      <c r="M24" s="116"/>
-      <c r="N24" s="115"/>
-      <c r="O24" s="116"/>
-      <c r="P24" s="115"/>
-      <c r="Q24" s="116"/>
-      <c r="R24" s="115"/>
-      <c r="S24" s="116"/>
-      <c r="T24" s="115"/>
-      <c r="U24" s="116"/>
-      <c r="V24" s="115"/>
-      <c r="W24" s="116"/>
-      <c r="X24" s="115"/>
-      <c r="Y24" s="116"/>
-      <c r="Z24" s="115"/>
-      <c r="AA24" s="116"/>
-      <c r="AB24" s="115"/>
-      <c r="AC24" s="116"/>
-      <c r="AD24" s="117"/>
-      <c r="AE24" s="116"/>
-      <c r="AF24" s="117"/>
-      <c r="AG24" s="116"/>
-      <c r="AH24" s="117"/>
-      <c r="AI24" s="116"/>
-      <c r="AJ24" s="111"/>
-      <c r="AK24" s="112"/>
-      <c r="AL24" s="117"/>
-      <c r="AM24" s="116"/>
-      <c r="AN24" s="111"/>
-      <c r="AO24" s="114"/>
-      <c r="AP24" s="118">
+      <c r="D24" s="80"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="84"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="80"/>
+      <c r="I24" s="81"/>
+      <c r="J24" s="84"/>
+      <c r="K24" s="85"/>
+      <c r="L24" s="84"/>
+      <c r="M24" s="85"/>
+      <c r="N24" s="84"/>
+      <c r="O24" s="85"/>
+      <c r="P24" s="84"/>
+      <c r="Q24" s="85"/>
+      <c r="R24" s="84"/>
+      <c r="S24" s="85"/>
+      <c r="T24" s="84"/>
+      <c r="U24" s="85"/>
+      <c r="V24" s="84"/>
+      <c r="W24" s="85"/>
+      <c r="X24" s="84"/>
+      <c r="Y24" s="85"/>
+      <c r="Z24" s="84"/>
+      <c r="AA24" s="85"/>
+      <c r="AB24" s="84"/>
+      <c r="AC24" s="85"/>
+      <c r="AD24" s="86"/>
+      <c r="AE24" s="85"/>
+      <c r="AF24" s="86"/>
+      <c r="AG24" s="85"/>
+      <c r="AH24" s="86"/>
+      <c r="AI24" s="85"/>
+      <c r="AJ24" s="80"/>
+      <c r="AK24" s="81"/>
+      <c r="AL24" s="86"/>
+      <c r="AM24" s="85"/>
+      <c r="AN24" s="80"/>
+      <c r="AO24" s="83"/>
+      <c r="AP24" s="87">
         <v>45</v>
       </c>
-      <c r="AQ24" s="119"/>
-      <c r="AR24" s="100">
-        <f>F24+J24+L24+N24+P24+R24+T24+V24+X24+Z24+AB24+AD24+AF24+AH24+AJ24+AL24+AN24+AP24</f>
+      <c r="AQ24" s="88"/>
+      <c r="AR24" s="69">
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="AS24" s="12">
-        <f>COUNTIF(D24:AP24,"&gt;30")</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT24" s="104"/>
-      <c r="AU24" s="108"/>
+      <c r="AT24" s="73"/>
+      <c r="AU24" s="77"/>
       <c r="AV24" s="27">
         <v>0</v>
       </c>
       <c r="AW24" s="40">
-        <f>AV24/AS24</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AX24" s="50"/>
@@ -4455,11 +4469,11 @@
       <c r="BA24" s="52"/>
       <c r="BB24" s="54"/>
     </row>
-    <row r="25" spans="1:54" s="13" customFormat="1" ht="17" thickBot="1">
-      <c r="A25" s="120"/>
-      <c r="B25" s="121"/>
-      <c r="C25" s="122"/>
-      <c r="D25" s="123"/>
+    <row r="25" spans="1:54" s="13" customFormat="1" ht="16.5" thickBot="1">
+      <c r="A25" s="89"/>
+      <c r="B25" s="90"/>
+      <c r="C25" s="91"/>
+      <c r="D25" s="92"/>
       <c r="E25" s="23"/>
       <c r="F25" s="23">
         <f>AVERAGEIF(F4:F23,"&gt;0")</f>
@@ -4518,36 +4532,36 @@
         <v>47.846153846153847</v>
       </c>
       <c r="AC25" s="60"/>
-      <c r="AD25" s="124">
+      <c r="AD25" s="93">
         <f>AVERAGEIF(AD4:AD23,"&gt;0")</f>
         <v>46.090909090909093</v>
       </c>
-      <c r="AE25" s="125"/>
-      <c r="AF25" s="124">
+      <c r="AE25" s="94"/>
+      <c r="AF25" s="93">
         <f>AVERAGEIF(AF4:AF23,"&gt;0")</f>
         <v>47.230769230769234</v>
       </c>
-      <c r="AG25" s="125"/>
-      <c r="AH25" s="124">
+      <c r="AG25" s="94"/>
+      <c r="AH25" s="93">
         <f>AVERAGEIF(AH4:AH23,"&gt;0")</f>
         <v>46.666666666666664</v>
       </c>
-      <c r="AI25" s="125"/>
-      <c r="AJ25" s="124"/>
-      <c r="AK25" s="125"/>
-      <c r="AL25" s="124">
+      <c r="AI25" s="94"/>
+      <c r="AJ25" s="93"/>
+      <c r="AK25" s="94"/>
+      <c r="AL25" s="93">
         <f>AVERAGEIF(AL4:AL23,"&gt;0")</f>
         <v>49.5</v>
       </c>
-      <c r="AM25" s="125"/>
-      <c r="AN25" s="124"/>
-      <c r="AO25" s="125"/>
-      <c r="AP25" s="124">
+      <c r="AM25" s="94"/>
+      <c r="AN25" s="93"/>
+      <c r="AO25" s="94"/>
+      <c r="AP25" s="93">
         <f>AVERAGEIF(AP4:AP23,"&gt;0")</f>
         <v>45.727272727272727</v>
       </c>
-      <c r="AQ25" s="125"/>
-      <c r="AR25" s="126"/>
+      <c r="AQ25" s="94"/>
+      <c r="AR25" s="95"/>
     </row>
     <row r="26" spans="1:54">
       <c r="C26" s="14"/>
@@ -4666,32 +4680,19 @@
     <sortCondition descending="1" ref="AR4:AR24"/>
   </sortState>
   <mergeCells count="55">
-    <mergeCell ref="AP1:AQ1"/>
-    <mergeCell ref="AP2:AQ2"/>
-    <mergeCell ref="AJ1:AK1"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AL1:AM1"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AV2:AV3"/>
-    <mergeCell ref="AR1:AR3"/>
-    <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AN2:AO2"/>
-    <mergeCell ref="AW2:AW3"/>
-    <mergeCell ref="AT2:AT3"/>
-    <mergeCell ref="AU2:AU3"/>
-    <mergeCell ref="AS2:AS3"/>
-    <mergeCell ref="AX1:BB1"/>
-    <mergeCell ref="AX2:AX3"/>
-    <mergeCell ref="AY2:AY3"/>
-    <mergeCell ref="AZ2:AZ3"/>
-    <mergeCell ref="BA2:BA3"/>
-    <mergeCell ref="BB2:BB3"/>
-    <mergeCell ref="AS1:AW1"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="AH1:AI1"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="AD1:AE1"/>
+    <mergeCell ref="AD2:AE2"/>
+    <mergeCell ref="AF1:AG1"/>
     <mergeCell ref="AF2:AG2"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:C3"/>
@@ -4708,19 +4709,32 @@
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="AH1:AI1"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="AD1:AE1"/>
-    <mergeCell ref="AD2:AE2"/>
-    <mergeCell ref="AF1:AG1"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="AX2:AX3"/>
+    <mergeCell ref="AY2:AY3"/>
+    <mergeCell ref="AZ2:AZ3"/>
+    <mergeCell ref="BA2:BA3"/>
+    <mergeCell ref="BB2:BB3"/>
+    <mergeCell ref="AV2:AV3"/>
+    <mergeCell ref="AR1:AR3"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AN2:AO2"/>
+    <mergeCell ref="AW2:AW3"/>
+    <mergeCell ref="AT2:AT3"/>
+    <mergeCell ref="AU2:AU3"/>
+    <mergeCell ref="AS2:AS3"/>
+    <mergeCell ref="AS1:AW1"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AP2:AQ2"/>
+    <mergeCell ref="AJ1:AK1"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AL1:AM1"/>
+    <mergeCell ref="AL2:AM2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
091725 - removed CTTP id from Karla's round
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{96156276-B3B5-584D-BEB7-22207EAFAEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07A0D921-ACCE-4B0B-88B6-AD466FE12EAC}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{96156276-B3B5-584D-BEB7-22207EAFAEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C24F97C-6A44-4457-8851-C9EE5140AD87}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="2460" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="6255" yWindow="1950" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -1079,7 +1079,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1453,6 +1453,9 @@
     </xf>
     <xf numFmtId="1" fontId="19" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4362,7 +4365,7 @@
       <c r="AI23" s="58"/>
       <c r="AJ23" s="80"/>
       <c r="AK23" s="81"/>
-      <c r="AL23" s="57">
+      <c r="AL23" s="132">
         <v>50</v>
       </c>
       <c r="AM23" s="58"/>

</xml_diff>

<commit_message>
092125 - updated skinks and scores
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{96156276-B3B5-584D-BEB7-22207EAFAEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C24F97C-6A44-4457-8851-C9EE5140AD87}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D6A723-A405-444E-8774-8BE2B9E38855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6255" yWindow="1950" windowWidth="30765" windowHeight="17115" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="6380" yWindow="3200" windowWidth="30760" windowHeight="17120" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="77">
   <si>
     <t>PLAYERS</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>Ra</t>
+  </si>
+  <si>
+    <t>Weekly Average</t>
   </si>
 </sst>
 </file>
@@ -1079,14 +1082,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1355,6 +1352,15 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1367,6 +1373,48 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1397,21 +1445,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1421,41 +1454,14 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1792,144 +1798,144 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E0A73BD-DC86-AB41-8C3D-0D64B5D06628}">
   <dimension ref="A1:BB29"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="8.625" customWidth="1"/>
-    <col min="2" max="2" width="8.125" customWidth="1"/>
-    <col min="3" max="3" width="10.125" customWidth="1"/>
-    <col min="4" max="10" width="6.875" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="8.6640625" customWidth="1"/>
+    <col min="2" max="2" width="8.1640625" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" customWidth="1"/>
+    <col min="4" max="10" width="6.83203125" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="6" hidden="1" customWidth="1"/>
-    <col min="12" max="23" width="6.375" hidden="1" customWidth="1"/>
+    <col min="12" max="23" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="24" max="24" width="6" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="6.375" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="6" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="6.375" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="28" max="28" width="6" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="6.375" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="30" max="30" width="6" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="6.375" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="32" max="32" width="6" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="6.375" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="34" max="34" width="6" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="6.375" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="36" max="36" width="6" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="6.375" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="6.33203125" hidden="1" customWidth="1"/>
     <col min="38" max="38" width="6" customWidth="1"/>
-    <col min="39" max="39" width="6.375" customWidth="1"/>
+    <col min="39" max="39" width="6.33203125" customWidth="1"/>
     <col min="40" max="40" width="6" customWidth="1"/>
-    <col min="41" max="41" width="6.375" customWidth="1"/>
+    <col min="41" max="41" width="6.33203125" customWidth="1"/>
     <col min="42" max="42" width="6" customWidth="1"/>
-    <col min="43" max="43" width="6.375" customWidth="1"/>
-    <col min="44" max="44" width="8.875" customWidth="1"/>
-    <col min="45" max="45" width="6.125" customWidth="1"/>
-    <col min="46" max="46" width="5.875" customWidth="1"/>
-    <col min="47" max="47" width="5.625" customWidth="1"/>
+    <col min="43" max="43" width="6.33203125" customWidth="1"/>
+    <col min="44" max="44" width="8.83203125" customWidth="1"/>
+    <col min="45" max="45" width="6.1640625" customWidth="1"/>
+    <col min="46" max="46" width="5.83203125" customWidth="1"/>
+    <col min="47" max="47" width="5.6640625" customWidth="1"/>
     <col min="48" max="48" width="5.5" customWidth="1"/>
     <col min="49" max="49" width="8" customWidth="1"/>
-    <col min="50" max="50" width="7.375" hidden="1" customWidth="1"/>
+    <col min="50" max="50" width="7.33203125" hidden="1" customWidth="1"/>
     <col min="51" max="52" width="6" hidden="1" customWidth="1"/>
-    <col min="53" max="53" width="7.375" hidden="1" customWidth="1"/>
-    <col min="54" max="54" width="9.375" hidden="1" customWidth="1"/>
+    <col min="53" max="53" width="7.33203125" hidden="1" customWidth="1"/>
+    <col min="54" max="54" width="9.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" s="32" customFormat="1" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="121" t="s">
+    <row r="1" spans="1:54" s="30" customFormat="1" ht="17" customHeight="1" thickBot="1">
+      <c r="A1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="127" t="s">
+      <c r="B1" s="105"/>
+      <c r="C1" s="110" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="99" t="s">
+      <c r="D1" s="100" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="100"/>
-      <c r="F1" s="99" t="s">
+      <c r="E1" s="101"/>
+      <c r="F1" s="100" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="100"/>
-      <c r="H1" s="99" t="s">
+      <c r="G1" s="101"/>
+      <c r="H1" s="100" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="100"/>
-      <c r="J1" s="99" t="s">
+      <c r="I1" s="101"/>
+      <c r="J1" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="100"/>
-      <c r="L1" s="99" t="s">
+      <c r="K1" s="101"/>
+      <c r="L1" s="100" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="100"/>
-      <c r="N1" s="99" t="s">
+      <c r="M1" s="101"/>
+      <c r="N1" s="100" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="100"/>
-      <c r="P1" s="99" t="s">
+      <c r="O1" s="101"/>
+      <c r="P1" s="100" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="100"/>
-      <c r="R1" s="99" t="s">
+      <c r="Q1" s="101"/>
+      <c r="R1" s="100" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="100"/>
-      <c r="T1" s="99" t="s">
+      <c r="S1" s="101"/>
+      <c r="T1" s="100" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="100"/>
-      <c r="V1" s="99" t="s">
+      <c r="U1" s="101"/>
+      <c r="V1" s="100" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="100"/>
-      <c r="X1" s="99" t="s">
+      <c r="W1" s="101"/>
+      <c r="X1" s="100" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="100"/>
-      <c r="Z1" s="99" t="s">
+      <c r="Y1" s="101"/>
+      <c r="Z1" s="100" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="100"/>
-      <c r="AB1" s="99" t="s">
+      <c r="AA1" s="101"/>
+      <c r="AB1" s="100" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="100"/>
-      <c r="AD1" s="99" t="s">
+      <c r="AC1" s="101"/>
+      <c r="AD1" s="100" t="s">
         <v>67</v>
       </c>
-      <c r="AE1" s="100"/>
-      <c r="AF1" s="99" t="s">
+      <c r="AE1" s="101"/>
+      <c r="AF1" s="100" t="s">
         <v>68</v>
       </c>
-      <c r="AG1" s="100"/>
-      <c r="AH1" s="99" t="s">
+      <c r="AG1" s="101"/>
+      <c r="AH1" s="100" t="s">
         <v>69</v>
       </c>
-      <c r="AI1" s="100"/>
-      <c r="AJ1" s="99" t="s">
+      <c r="AI1" s="101"/>
+      <c r="AJ1" s="100" t="s">
         <v>70</v>
       </c>
-      <c r="AK1" s="100"/>
-      <c r="AL1" s="99" t="s">
+      <c r="AK1" s="101"/>
+      <c r="AL1" s="100" t="s">
         <v>71</v>
       </c>
-      <c r="AM1" s="100"/>
-      <c r="AN1" s="99" t="s">
+      <c r="AM1" s="101"/>
+      <c r="AN1" s="100" t="s">
         <v>73</v>
       </c>
-      <c r="AO1" s="100"/>
-      <c r="AP1" s="99" t="s">
+      <c r="AO1" s="101"/>
+      <c r="AP1" s="100" t="s">
         <v>74</v>
       </c>
-      <c r="AQ1" s="100"/>
-      <c r="AR1" s="105" t="s">
+      <c r="AQ1" s="101"/>
+      <c r="AR1" s="120" t="s">
         <v>2</v>
       </c>
-      <c r="AS1" s="118" t="s">
+      <c r="AS1" s="128" t="s">
         <v>65</v>
       </c>
-      <c r="AT1" s="119"/>
-      <c r="AU1" s="119"/>
-      <c r="AV1" s="119"/>
-      <c r="AW1" s="120"/>
+      <c r="AT1" s="129"/>
+      <c r="AU1" s="129"/>
+      <c r="AV1" s="129"/>
+      <c r="AW1" s="130"/>
       <c r="AX1" s="113" t="s">
         <v>57</v>
       </c>
@@ -1938,105 +1944,105 @@
       <c r="BA1" s="114"/>
       <c r="BB1" s="115"/>
     </row>
-    <row r="2" spans="1:54" s="32" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="123"/>
-      <c r="B2" s="124"/>
-      <c r="C2" s="128"/>
-      <c r="D2" s="101">
+    <row r="2" spans="1:54" s="30" customFormat="1" ht="17" customHeight="1">
+      <c r="A2" s="106"/>
+      <c r="B2" s="107"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="102">
         <v>45782</v>
       </c>
-      <c r="E2" s="102"/>
-      <c r="F2" s="101">
+      <c r="E2" s="103"/>
+      <c r="F2" s="102">
         <v>45789</v>
       </c>
-      <c r="G2" s="102"/>
-      <c r="H2" s="101">
+      <c r="G2" s="103"/>
+      <c r="H2" s="102">
         <v>45796</v>
       </c>
-      <c r="I2" s="102"/>
-      <c r="J2" s="101">
+      <c r="I2" s="103"/>
+      <c r="J2" s="102">
         <v>45803</v>
       </c>
-      <c r="K2" s="102"/>
-      <c r="L2" s="101">
+      <c r="K2" s="103"/>
+      <c r="L2" s="102">
         <v>45810</v>
       </c>
-      <c r="M2" s="102"/>
-      <c r="N2" s="101">
+      <c r="M2" s="103"/>
+      <c r="N2" s="102">
         <v>45817</v>
       </c>
-      <c r="O2" s="102"/>
-      <c r="P2" s="101">
+      <c r="O2" s="103"/>
+      <c r="P2" s="102">
         <v>45824</v>
       </c>
-      <c r="Q2" s="102"/>
-      <c r="R2" s="101">
+      <c r="Q2" s="103"/>
+      <c r="R2" s="102">
         <v>45831</v>
       </c>
-      <c r="S2" s="102"/>
-      <c r="T2" s="101">
+      <c r="S2" s="103"/>
+      <c r="T2" s="102">
         <v>45838</v>
       </c>
-      <c r="U2" s="102"/>
-      <c r="V2" s="101">
+      <c r="U2" s="103"/>
+      <c r="V2" s="102">
         <v>45845</v>
       </c>
-      <c r="W2" s="102"/>
-      <c r="X2" s="101">
+      <c r="W2" s="103"/>
+      <c r="X2" s="102">
         <v>45852</v>
       </c>
-      <c r="Y2" s="102"/>
-      <c r="Z2" s="101">
+      <c r="Y2" s="103"/>
+      <c r="Z2" s="102">
         <v>45859</v>
       </c>
-      <c r="AA2" s="102"/>
-      <c r="AB2" s="101">
+      <c r="AA2" s="103"/>
+      <c r="AB2" s="102">
         <v>45866</v>
       </c>
-      <c r="AC2" s="102"/>
-      <c r="AD2" s="101">
+      <c r="AC2" s="103"/>
+      <c r="AD2" s="102">
         <v>45873</v>
       </c>
-      <c r="AE2" s="102"/>
-      <c r="AF2" s="101">
+      <c r="AE2" s="103"/>
+      <c r="AF2" s="102">
         <v>45880</v>
       </c>
-      <c r="AG2" s="102"/>
-      <c r="AH2" s="101">
+      <c r="AG2" s="103"/>
+      <c r="AH2" s="102">
         <v>45887</v>
       </c>
-      <c r="AI2" s="102"/>
-      <c r="AJ2" s="101">
+      <c r="AI2" s="103"/>
+      <c r="AJ2" s="102">
         <v>45894</v>
       </c>
-      <c r="AK2" s="102"/>
-      <c r="AL2" s="101">
+      <c r="AK2" s="103"/>
+      <c r="AL2" s="102">
         <v>45901</v>
       </c>
-      <c r="AM2" s="102"/>
-      <c r="AN2" s="101">
+      <c r="AM2" s="103"/>
+      <c r="AN2" s="102">
         <v>45908</v>
       </c>
-      <c r="AO2" s="102"/>
-      <c r="AP2" s="101">
+      <c r="AO2" s="103"/>
+      <c r="AP2" s="102">
         <v>45915</v>
       </c>
-      <c r="AQ2" s="102"/>
-      <c r="AR2" s="106"/>
-      <c r="AS2" s="105" t="s">
+      <c r="AQ2" s="103"/>
+      <c r="AR2" s="121"/>
+      <c r="AS2" s="120" t="s">
         <v>3</v>
       </c>
-      <c r="AT2" s="109" t="s">
+      <c r="AT2" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="AU2" s="111" t="s">
+      <c r="AU2" s="126" t="s">
         <v>5</v>
       </c>
-      <c r="AV2" s="103" t="s">
+      <c r="AV2" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="AW2" s="107" t="s">
-        <v>7</v>
+      <c r="AW2" s="122" t="s">
+        <v>76</v>
       </c>
       <c r="AX2" s="116" t="s">
         <v>3</v>
@@ -2054,2628 +2060,2628 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:54" s="32" customFormat="1" ht="29.1" customHeight="1" thickBot="1">
-      <c r="A3" s="125"/>
-      <c r="B3" s="126"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="1" t="s">
+    <row r="3" spans="1:54" s="133" customFormat="1" ht="13" customHeight="1" thickBot="1">
+      <c r="A3" s="108"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="P3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="R3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="T3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="U3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="V3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="W3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="X3" s="1" t="s">
+      <c r="X3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="Y3" s="2" t="s">
+      <c r="Y3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="Z3" s="1" t="s">
+      <c r="Z3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AA3" s="2" t="s">
+      <c r="AA3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AB3" s="1" t="s">
+      <c r="AB3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AC3" s="2" t="s">
+      <c r="AC3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AD3" s="1" t="s">
+      <c r="AD3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AE3" s="2" t="s">
+      <c r="AE3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AF3" s="1" t="s">
+      <c r="AF3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AG3" s="2" t="s">
+      <c r="AG3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AH3" s="1" t="s">
+      <c r="AH3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AI3" s="2" t="s">
+      <c r="AI3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AJ3" s="1" t="s">
+      <c r="AJ3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AK3" s="2" t="s">
+      <c r="AK3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AL3" s="1" t="s">
+      <c r="AL3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AM3" s="2" t="s">
+      <c r="AM3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AN3" s="1" t="s">
+      <c r="AN3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AO3" s="2" t="s">
+      <c r="AO3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AP3" s="1" t="s">
+      <c r="AP3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="AQ3" s="2" t="s">
+      <c r="AQ3" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="AR3" s="106"/>
-      <c r="AS3" s="106"/>
-      <c r="AT3" s="110"/>
-      <c r="AU3" s="112"/>
-      <c r="AV3" s="104"/>
-      <c r="AW3" s="108"/>
+      <c r="AR3" s="121"/>
+      <c r="AS3" s="121"/>
+      <c r="AT3" s="125"/>
+      <c r="AU3" s="127"/>
+      <c r="AV3" s="119"/>
+      <c r="AW3" s="123"/>
       <c r="AX3" s="117"/>
       <c r="AY3" s="117"/>
       <c r="AZ3" s="117"/>
       <c r="BA3" s="117"/>
       <c r="BB3" s="117"/>
     </row>
-    <row r="4" spans="1:54" ht="15.95" customHeight="1">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:54" ht="16" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="63">
+      <c r="C4" s="61">
         <f t="shared" ref="C4:C20" si="0">ROUND((AR4-(36*AS4))/AS4,0)</f>
         <v>17</v>
       </c>
-      <c r="D4" s="78"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="46">
+      <c r="D4" s="76"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="44">
         <v>53</v>
       </c>
-      <c r="G4" s="59">
+      <c r="G4" s="57">
         <v>23</v>
       </c>
-      <c r="H4" s="78"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="46"/>
-      <c r="M4" s="59"/>
-      <c r="N4" s="46">
+      <c r="H4" s="76"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="44"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="57"/>
+      <c r="N4" s="44">
         <v>57</v>
       </c>
-      <c r="O4" s="59">
+      <c r="O4" s="57">
         <v>19</v>
       </c>
-      <c r="P4" s="46"/>
-      <c r="Q4" s="59"/>
-      <c r="R4" s="46">
+      <c r="P4" s="44"/>
+      <c r="Q4" s="57"/>
+      <c r="R4" s="44">
         <v>50</v>
       </c>
-      <c r="S4" s="59">
+      <c r="S4" s="57">
         <v>26</v>
       </c>
-      <c r="T4" s="46">
+      <c r="T4" s="44">
         <v>56</v>
       </c>
-      <c r="U4" s="59">
+      <c r="U4" s="57">
         <v>15</v>
       </c>
-      <c r="V4" s="46"/>
-      <c r="W4" s="59"/>
-      <c r="X4" s="46"/>
-      <c r="Y4" s="59"/>
-      <c r="Z4" s="46">
+      <c r="V4" s="44"/>
+      <c r="W4" s="57"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="57"/>
+      <c r="Z4" s="44">
         <v>54</v>
       </c>
-      <c r="AA4" s="59">
+      <c r="AA4" s="57">
         <v>18</v>
       </c>
-      <c r="AB4" s="46">
+      <c r="AB4" s="44">
         <v>50</v>
       </c>
-      <c r="AC4" s="59">
+      <c r="AC4" s="57">
         <v>22</v>
       </c>
-      <c r="AD4" s="49"/>
-      <c r="AE4" s="55"/>
-      <c r="AF4" s="49"/>
-      <c r="AG4" s="55"/>
-      <c r="AH4" s="49"/>
-      <c r="AI4" s="55"/>
-      <c r="AJ4" s="78"/>
-      <c r="AK4" s="79"/>
-      <c r="AL4" s="49"/>
-      <c r="AM4" s="55"/>
-      <c r="AN4" s="78"/>
-      <c r="AO4" s="82"/>
-      <c r="AP4" s="49"/>
-      <c r="AQ4" s="66"/>
-      <c r="AR4" s="68">
+      <c r="AD4" s="47"/>
+      <c r="AE4" s="53"/>
+      <c r="AF4" s="47"/>
+      <c r="AG4" s="53"/>
+      <c r="AH4" s="47"/>
+      <c r="AI4" s="53"/>
+      <c r="AJ4" s="76"/>
+      <c r="AK4" s="77"/>
+      <c r="AL4" s="47"/>
+      <c r="AM4" s="53"/>
+      <c r="AN4" s="76"/>
+      <c r="AO4" s="80"/>
+      <c r="AP4" s="47"/>
+      <c r="AQ4" s="64"/>
+      <c r="AR4" s="66">
         <f t="shared" ref="AR4:AR24" si="1">F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4+AJ4+AL4+AN4+AP4</f>
         <v>320</v>
       </c>
-      <c r="AS4" s="5">
+      <c r="AS4" s="3">
         <f t="shared" ref="AS4:AS24" si="2">COUNTIF(D4:AP4,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AT4" s="70"/>
-      <c r="AU4" s="74"/>
-      <c r="AV4" s="24">
+      <c r="AT4" s="68"/>
+      <c r="AU4" s="72"/>
+      <c r="AV4" s="22">
         <f t="shared" ref="AV4:AV23" si="3">SUMIF(G4:AQ4, "&lt;30")+AT4+AU4</f>
         <v>123</v>
       </c>
-      <c r="AW4" s="38">
+      <c r="AW4" s="36">
         <f t="shared" ref="AW4:AW24" si="4">AV4/AS4</f>
         <v>20.5</v>
       </c>
-      <c r="AX4" s="44"/>
-      <c r="AY4" s="24"/>
-      <c r="AZ4" s="24"/>
-      <c r="BA4" s="5"/>
-      <c r="BB4" s="33" t="s">
+      <c r="AX4" s="42"/>
+      <c r="AY4" s="22"/>
+      <c r="AZ4" s="22"/>
+      <c r="BA4" s="3"/>
+      <c r="BB4" s="31" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:54">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="64">
+      <c r="C5" s="62">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="D5" s="80"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="58"/>
-      <c r="L5" s="47"/>
-      <c r="M5" s="58"/>
-      <c r="N5" s="47"/>
-      <c r="O5" s="58"/>
-      <c r="P5" s="47">
+      <c r="D5" s="78"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="78"/>
+      <c r="I5" s="79"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="56"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="56"/>
+      <c r="P5" s="45">
         <v>39</v>
       </c>
-      <c r="Q5" s="58">
+      <c r="Q5" s="56">
         <v>17</v>
       </c>
-      <c r="R5" s="47">
+      <c r="R5" s="45">
         <v>38</v>
       </c>
-      <c r="S5" s="58">
+      <c r="S5" s="56">
         <v>18</v>
       </c>
-      <c r="T5" s="47"/>
-      <c r="U5" s="58"/>
-      <c r="V5" s="47">
+      <c r="T5" s="45"/>
+      <c r="U5" s="56"/>
+      <c r="V5" s="45">
         <v>37</v>
       </c>
-      <c r="W5" s="58">
+      <c r="W5" s="56">
         <v>19</v>
       </c>
-      <c r="X5" s="47">
+      <c r="X5" s="45">
         <v>36</v>
       </c>
-      <c r="Y5" s="58">
+      <c r="Y5" s="56">
         <v>20</v>
       </c>
-      <c r="Z5" s="47">
+      <c r="Z5" s="45">
         <v>38</v>
       </c>
-      <c r="AA5" s="58">
+      <c r="AA5" s="56">
         <v>18</v>
       </c>
-      <c r="AB5" s="47">
+      <c r="AB5" s="45">
         <v>35</v>
       </c>
-      <c r="AC5" s="58">
+      <c r="AC5" s="56">
         <v>21</v>
       </c>
-      <c r="AD5" s="48">
+      <c r="AD5" s="46">
         <v>37</v>
       </c>
-      <c r="AE5" s="56">
+      <c r="AE5" s="54">
         <v>19</v>
       </c>
-      <c r="AF5" s="48">
+      <c r="AF5" s="46">
         <v>37</v>
       </c>
-      <c r="AG5" s="56">
+      <c r="AG5" s="54">
         <v>18</v>
       </c>
-      <c r="AH5" s="48">
+      <c r="AH5" s="46">
         <v>38</v>
       </c>
-      <c r="AI5" s="56">
+      <c r="AI5" s="54">
         <v>17</v>
       </c>
-      <c r="AJ5" s="80"/>
-      <c r="AK5" s="81"/>
-      <c r="AL5" s="48"/>
-      <c r="AM5" s="56"/>
-      <c r="AN5" s="80"/>
-      <c r="AO5" s="83"/>
-      <c r="AP5" s="130">
+      <c r="AJ5" s="78"/>
+      <c r="AK5" s="79"/>
+      <c r="AL5" s="46"/>
+      <c r="AM5" s="54"/>
+      <c r="AN5" s="78"/>
+      <c r="AO5" s="81"/>
+      <c r="AP5" s="97">
         <v>35</v>
       </c>
-      <c r="AQ5" s="67">
+      <c r="AQ5" s="65">
         <v>20</v>
       </c>
-      <c r="AR5" s="69">
+      <c r="AR5" s="67">
         <f t="shared" si="1"/>
         <v>370</v>
       </c>
-      <c r="AS5" s="8">
+      <c r="AS5" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT5" s="71">
+      <c r="AT5" s="69">
         <v>3</v>
       </c>
-      <c r="AU5" s="75">
+      <c r="AU5" s="73">
         <v>13</v>
       </c>
-      <c r="AV5" s="25">
+      <c r="AV5" s="23">
         <f t="shared" si="3"/>
         <v>203</v>
       </c>
-      <c r="AW5" s="39">
+      <c r="AW5" s="37">
         <f t="shared" si="4"/>
         <v>20.3</v>
       </c>
-      <c r="AX5" s="34"/>
-      <c r="AY5" s="25"/>
-      <c r="AZ5" s="25"/>
-      <c r="BA5" s="8"/>
-      <c r="BB5" s="35"/>
+      <c r="AX5" s="32"/>
+      <c r="AY5" s="23"/>
+      <c r="AZ5" s="23"/>
+      <c r="BA5" s="6"/>
+      <c r="BB5" s="33"/>
     </row>
     <row r="6" spans="1:54">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="64">
+      <c r="C6" s="62">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D6" s="80"/>
-      <c r="E6" s="81"/>
-      <c r="F6" s="37">
+      <c r="D6" s="78"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="35">
         <v>45</v>
       </c>
-      <c r="G6" s="58">
+      <c r="G6" s="56">
         <v>17</v>
       </c>
-      <c r="H6" s="80"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="58"/>
-      <c r="L6" s="37">
+      <c r="H6" s="78"/>
+      <c r="I6" s="79"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="35">
         <v>43</v>
       </c>
-      <c r="M6" s="58">
+      <c r="M6" s="56">
         <v>19</v>
       </c>
-      <c r="N6" s="37">
+      <c r="N6" s="35">
         <v>41</v>
       </c>
-      <c r="O6" s="58">
+      <c r="O6" s="56">
         <v>21</v>
       </c>
-      <c r="P6" s="37">
+      <c r="P6" s="35">
         <v>47</v>
       </c>
-      <c r="Q6" s="58">
+      <c r="Q6" s="56">
         <v>15</v>
       </c>
-      <c r="R6" s="37">
+      <c r="R6" s="35">
         <v>42</v>
       </c>
-      <c r="S6" s="58">
+      <c r="S6" s="56">
         <v>20</v>
       </c>
-      <c r="T6" s="37">
+      <c r="T6" s="35">
         <v>43</v>
       </c>
-      <c r="U6" s="58">
+      <c r="U6" s="56">
         <v>19</v>
       </c>
-      <c r="V6" s="37">
+      <c r="V6" s="35">
         <v>44</v>
       </c>
-      <c r="W6" s="58">
+      <c r="W6" s="56">
         <v>18</v>
       </c>
-      <c r="X6" s="37">
+      <c r="X6" s="35">
         <v>48</v>
       </c>
-      <c r="Y6" s="58">
+      <c r="Y6" s="56">
         <v>16</v>
       </c>
-      <c r="Z6" s="37">
+      <c r="Z6" s="35">
         <v>40</v>
       </c>
-      <c r="AA6" s="58">
+      <c r="AA6" s="56">
         <v>22</v>
       </c>
-      <c r="AB6" s="37">
+      <c r="AB6" s="35">
         <v>40</v>
       </c>
-      <c r="AC6" s="58">
+      <c r="AC6" s="56">
         <v>22</v>
       </c>
-      <c r="AD6" s="26">
+      <c r="AD6" s="24">
         <v>38</v>
       </c>
-      <c r="AE6" s="56">
+      <c r="AE6" s="54">
         <v>23</v>
       </c>
-      <c r="AF6" s="45">
+      <c r="AF6" s="43">
         <v>41</v>
       </c>
-      <c r="AG6" s="56">
+      <c r="AG6" s="54">
         <v>20</v>
       </c>
-      <c r="AH6" s="41">
+      <c r="AH6" s="39">
         <v>40</v>
       </c>
-      <c r="AI6" s="56">
+      <c r="AI6" s="54">
         <v>21</v>
       </c>
-      <c r="AJ6" s="80"/>
-      <c r="AK6" s="81"/>
-      <c r="AL6" s="41"/>
-      <c r="AM6" s="56"/>
-      <c r="AN6" s="80"/>
-      <c r="AO6" s="83"/>
-      <c r="AP6" s="41">
+      <c r="AJ6" s="78"/>
+      <c r="AK6" s="79"/>
+      <c r="AL6" s="39"/>
+      <c r="AM6" s="54"/>
+      <c r="AN6" s="78"/>
+      <c r="AO6" s="81"/>
+      <c r="AP6" s="39">
         <v>43</v>
       </c>
-      <c r="AQ6" s="67">
+      <c r="AQ6" s="65">
         <v>17</v>
       </c>
-      <c r="AR6" s="69">
+      <c r="AR6" s="67">
         <f t="shared" si="1"/>
         <v>595</v>
       </c>
-      <c r="AS6" s="8">
+      <c r="AS6" s="6">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="AT6" s="71">
+      <c r="AT6" s="69">
         <v>2</v>
       </c>
-      <c r="AU6" s="75">
+      <c r="AU6" s="73">
         <v>6</v>
       </c>
-      <c r="AV6" s="25">
+      <c r="AV6" s="23">
         <f t="shared" si="3"/>
         <v>278</v>
       </c>
-      <c r="AW6" s="39">
+      <c r="AW6" s="37">
         <f t="shared" si="4"/>
         <v>19.857142857142858</v>
       </c>
-      <c r="AX6" s="34"/>
-      <c r="AY6" s="25"/>
-      <c r="AZ6" s="25"/>
-      <c r="BA6" s="8"/>
-      <c r="BB6" s="35"/>
+      <c r="AX6" s="32"/>
+      <c r="AY6" s="23"/>
+      <c r="AZ6" s="23"/>
+      <c r="BA6" s="6"/>
+      <c r="BB6" s="33"/>
     </row>
     <row r="7" spans="1:54">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="64">
+      <c r="C7" s="62">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D7" s="80"/>
-      <c r="E7" s="81"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="58"/>
-      <c r="H7" s="80"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="58"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="58"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="58"/>
-      <c r="P7" s="9">
+      <c r="D7" s="78"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="56"/>
+      <c r="H7" s="78"/>
+      <c r="I7" s="79"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="56"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="56"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="56"/>
+      <c r="P7" s="7">
         <v>43</v>
       </c>
-      <c r="Q7" s="58">
+      <c r="Q7" s="56">
         <v>26</v>
       </c>
-      <c r="R7" s="9">
+      <c r="R7" s="7">
         <v>45</v>
       </c>
-      <c r="S7" s="58">
+      <c r="S7" s="56">
         <v>24</v>
       </c>
-      <c r="T7" s="9"/>
-      <c r="U7" s="58"/>
-      <c r="V7" s="9">
+      <c r="T7" s="7"/>
+      <c r="U7" s="56"/>
+      <c r="V7" s="7">
         <v>50</v>
       </c>
-      <c r="W7" s="58">
+      <c r="W7" s="56">
         <v>19</v>
       </c>
-      <c r="X7" s="9">
+      <c r="X7" s="7">
         <v>44</v>
       </c>
-      <c r="Y7" s="58">
+      <c r="Y7" s="56">
         <v>20</v>
       </c>
-      <c r="Z7" s="9"/>
-      <c r="AA7" s="58"/>
-      <c r="AB7" s="9">
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="56"/>
+      <c r="AB7" s="7">
         <v>54</v>
       </c>
-      <c r="AC7" s="58">
+      <c r="AC7" s="56">
         <v>11</v>
       </c>
-      <c r="AD7" s="43"/>
-      <c r="AE7" s="56"/>
-      <c r="AF7" s="43">
+      <c r="AD7" s="41"/>
+      <c r="AE7" s="54"/>
+      <c r="AF7" s="41">
         <v>51</v>
       </c>
-      <c r="AG7" s="56">
+      <c r="AG7" s="54">
         <v>14</v>
       </c>
-      <c r="AH7" s="43"/>
-      <c r="AI7" s="56"/>
-      <c r="AJ7" s="80"/>
-      <c r="AK7" s="81"/>
-      <c r="AL7" s="97">
+      <c r="AH7" s="41"/>
+      <c r="AI7" s="54"/>
+      <c r="AJ7" s="78"/>
+      <c r="AK7" s="79"/>
+      <c r="AL7" s="95">
         <v>46</v>
       </c>
-      <c r="AM7" s="56">
+      <c r="AM7" s="54">
         <v>20</v>
       </c>
-      <c r="AN7" s="80"/>
-      <c r="AO7" s="83"/>
-      <c r="AP7" s="98"/>
-      <c r="AQ7" s="67"/>
-      <c r="AR7" s="69">
+      <c r="AN7" s="78"/>
+      <c r="AO7" s="81"/>
+      <c r="AP7" s="96"/>
+      <c r="AQ7" s="65"/>
+      <c r="AR7" s="67">
         <f t="shared" si="1"/>
         <v>333</v>
       </c>
-      <c r="AS7" s="8">
+      <c r="AS7" s="6">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AT7" s="71">
+      <c r="AT7" s="69">
         <v>2</v>
       </c>
-      <c r="AU7" s="75">
+      <c r="AU7" s="73">
         <v>1</v>
       </c>
-      <c r="AV7" s="25">
+      <c r="AV7" s="23">
         <f t="shared" si="3"/>
         <v>137</v>
       </c>
-      <c r="AW7" s="39">
+      <c r="AW7" s="37">
         <f t="shared" si="4"/>
         <v>19.571428571428573</v>
       </c>
-      <c r="AX7" s="36"/>
-      <c r="AY7" s="25"/>
-      <c r="AZ7" s="25"/>
-      <c r="BA7" s="8"/>
-      <c r="BB7" s="35"/>
+      <c r="AX7" s="34"/>
+      <c r="AY7" s="23"/>
+      <c r="AZ7" s="23"/>
+      <c r="BA7" s="6"/>
+      <c r="BB7" s="33"/>
     </row>
     <row r="8" spans="1:54">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="64">
+      <c r="C8" s="62">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D8" s="80"/>
-      <c r="E8" s="81"/>
-      <c r="F8" s="9">
+      <c r="D8" s="78"/>
+      <c r="E8" s="79"/>
+      <c r="F8" s="7">
         <v>41</v>
       </c>
-      <c r="G8" s="58">
+      <c r="G8" s="56">
         <v>21</v>
       </c>
-      <c r="H8" s="80"/>
-      <c r="I8" s="81"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="58"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="58"/>
-      <c r="N8" s="9">
+      <c r="H8" s="78"/>
+      <c r="I8" s="79"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="56"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="56"/>
+      <c r="N8" s="7">
         <v>48</v>
       </c>
-      <c r="O8" s="58">
+      <c r="O8" s="56">
         <v>14</v>
       </c>
-      <c r="P8" s="9">
+      <c r="P8" s="7">
         <v>44</v>
       </c>
-      <c r="Q8" s="58">
+      <c r="Q8" s="56">
         <v>18</v>
       </c>
-      <c r="R8" s="9"/>
-      <c r="S8" s="58"/>
-      <c r="T8" s="9"/>
-      <c r="U8" s="58"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="58"/>
-      <c r="X8" s="9">
+      <c r="R8" s="7"/>
+      <c r="S8" s="56"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="56"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="56"/>
+      <c r="X8" s="7">
         <v>40</v>
       </c>
-      <c r="Y8" s="58">
+      <c r="Y8" s="56">
         <v>22</v>
       </c>
-      <c r="Z8" s="9">
+      <c r="Z8" s="7">
         <v>44</v>
       </c>
-      <c r="AA8" s="58">
+      <c r="AA8" s="56">
         <v>17</v>
       </c>
-      <c r="AB8" s="9">
+      <c r="AB8" s="7">
         <v>46</v>
       </c>
-      <c r="AC8" s="58">
+      <c r="AC8" s="56">
         <v>16</v>
       </c>
-      <c r="AD8" s="31">
+      <c r="AD8" s="29">
         <v>42</v>
       </c>
-      <c r="AE8" s="56">
+      <c r="AE8" s="54">
         <v>20</v>
       </c>
-      <c r="AF8" s="26">
+      <c r="AF8" s="24">
         <v>44</v>
       </c>
-      <c r="AG8" s="56">
+      <c r="AG8" s="54">
         <v>18</v>
       </c>
-      <c r="AH8" s="31">
+      <c r="AH8" s="29">
         <v>39</v>
       </c>
-      <c r="AI8" s="56">
+      <c r="AI8" s="54">
         <v>23</v>
       </c>
-      <c r="AJ8" s="80"/>
-      <c r="AK8" s="81"/>
-      <c r="AL8" s="31"/>
-      <c r="AM8" s="56"/>
-      <c r="AN8" s="80"/>
-      <c r="AO8" s="83"/>
-      <c r="AP8" s="26">
+      <c r="AJ8" s="78"/>
+      <c r="AK8" s="79"/>
+      <c r="AL8" s="29"/>
+      <c r="AM8" s="54"/>
+      <c r="AN8" s="78"/>
+      <c r="AO8" s="81"/>
+      <c r="AP8" s="24">
         <v>41</v>
       </c>
-      <c r="AQ8" s="67">
+      <c r="AQ8" s="65">
         <v>20</v>
       </c>
-      <c r="AR8" s="69">
+      <c r="AR8" s="67">
         <f t="shared" si="1"/>
         <v>429</v>
       </c>
-      <c r="AS8" s="8">
+      <c r="AS8" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT8" s="71">
+      <c r="AT8" s="69">
         <v>3</v>
       </c>
-      <c r="AU8" s="75">
+      <c r="AU8" s="73">
         <v>3</v>
       </c>
-      <c r="AV8" s="25">
+      <c r="AV8" s="23">
         <f t="shared" si="3"/>
         <v>195</v>
       </c>
-      <c r="AW8" s="39">
+      <c r="AW8" s="37">
         <f t="shared" si="4"/>
         <v>19.5</v>
       </c>
-      <c r="AX8" s="50"/>
-      <c r="AY8" s="25"/>
-      <c r="AZ8" s="25"/>
-      <c r="BA8" s="8"/>
-      <c r="BB8" s="35"/>
+      <c r="AX8" s="48"/>
+      <c r="AY8" s="23"/>
+      <c r="AZ8" s="23"/>
+      <c r="BA8" s="6"/>
+      <c r="BB8" s="33"/>
     </row>
     <row r="9" spans="1:54">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="64">
+      <c r="C9" s="62">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D9" s="80"/>
-      <c r="E9" s="81"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="58"/>
-      <c r="H9" s="80"/>
-      <c r="I9" s="81"/>
-      <c r="J9" s="9">
+      <c r="D9" s="78"/>
+      <c r="E9" s="79"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="78"/>
+      <c r="I9" s="79"/>
+      <c r="J9" s="7">
         <v>52</v>
       </c>
-      <c r="K9" s="58">
+      <c r="K9" s="56">
         <v>17</v>
       </c>
-      <c r="L9" s="9"/>
-      <c r="M9" s="58"/>
-      <c r="N9" s="9">
+      <c r="L9" s="7"/>
+      <c r="M9" s="56"/>
+      <c r="N9" s="7">
         <v>46</v>
       </c>
-      <c r="O9" s="58">
+      <c r="O9" s="56">
         <v>23</v>
       </c>
-      <c r="P9" s="9">
+      <c r="P9" s="7">
         <v>46</v>
       </c>
-      <c r="Q9" s="58">
+      <c r="Q9" s="56">
         <v>23</v>
       </c>
-      <c r="R9" s="9">
+      <c r="R9" s="7">
         <v>54</v>
       </c>
-      <c r="S9" s="58">
+      <c r="S9" s="56">
         <v>16</v>
       </c>
-      <c r="T9" s="9">
+      <c r="T9" s="7">
         <v>45</v>
       </c>
-      <c r="U9" s="58">
+      <c r="U9" s="56">
         <v>23</v>
       </c>
-      <c r="V9" s="9">
+      <c r="V9" s="7">
         <v>48</v>
       </c>
-      <c r="W9" s="58">
+      <c r="W9" s="56">
         <v>19</v>
       </c>
-      <c r="X9" s="9">
+      <c r="X9" s="7">
         <v>49</v>
       </c>
-      <c r="Y9" s="58">
+      <c r="Y9" s="56">
         <v>18</v>
       </c>
-      <c r="Z9" s="9"/>
-      <c r="AA9" s="58"/>
-      <c r="AB9" s="9">
+      <c r="Z9" s="7"/>
+      <c r="AA9" s="56"/>
+      <c r="AB9" s="7">
         <v>46</v>
       </c>
-      <c r="AC9" s="58">
+      <c r="AC9" s="56">
         <v>21</v>
       </c>
-      <c r="AD9" s="96">
+      <c r="AD9" s="94">
         <v>43</v>
       </c>
-      <c r="AE9" s="56">
+      <c r="AE9" s="54">
         <v>23</v>
       </c>
-      <c r="AF9" s="41">
+      <c r="AF9" s="39">
         <v>47</v>
       </c>
-      <c r="AG9" s="56">
+      <c r="AG9" s="54">
         <v>19</v>
       </c>
-      <c r="AH9" s="41">
+      <c r="AH9" s="39">
         <v>51</v>
       </c>
-      <c r="AI9" s="56">
+      <c r="AI9" s="54">
         <v>15</v>
       </c>
-      <c r="AJ9" s="80"/>
-      <c r="AK9" s="81"/>
-      <c r="AL9" s="43">
+      <c r="AJ9" s="78"/>
+      <c r="AK9" s="79"/>
+      <c r="AL9" s="41">
         <v>50</v>
       </c>
-      <c r="AM9" s="56">
+      <c r="AM9" s="54">
         <v>16</v>
       </c>
-      <c r="AN9" s="80"/>
-      <c r="AO9" s="83"/>
-      <c r="AP9" s="43">
+      <c r="AN9" s="78"/>
+      <c r="AO9" s="81"/>
+      <c r="AP9" s="41">
         <v>51</v>
       </c>
-      <c r="AQ9" s="67">
+      <c r="AQ9" s="65">
         <v>17</v>
       </c>
-      <c r="AR9" s="69">
+      <c r="AR9" s="67">
         <f t="shared" si="1"/>
         <v>628</v>
       </c>
-      <c r="AS9" s="8">
+      <c r="AS9" s="6">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="AT9" s="71">
+      <c r="AT9" s="69">
         <v>1</v>
       </c>
-      <c r="AU9" s="75">
+      <c r="AU9" s="73">
         <v>2</v>
       </c>
-      <c r="AV9" s="25">
+      <c r="AV9" s="23">
         <f t="shared" si="3"/>
         <v>253</v>
       </c>
-      <c r="AW9" s="39">
+      <c r="AW9" s="37">
         <f t="shared" si="4"/>
         <v>19.46153846153846</v>
       </c>
-      <c r="AX9" s="34"/>
-      <c r="AY9" s="25"/>
-      <c r="AZ9" s="25"/>
-      <c r="BA9" s="8"/>
-      <c r="BB9" s="35"/>
+      <c r="AX9" s="32"/>
+      <c r="AY9" s="23"/>
+      <c r="AZ9" s="23"/>
+      <c r="BA9" s="6"/>
+      <c r="BB9" s="33"/>
     </row>
     <row r="10" spans="1:54">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="64">
+      <c r="C10" s="62">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D10" s="80"/>
-      <c r="E10" s="81"/>
-      <c r="F10" s="42">
+      <c r="D10" s="78"/>
+      <c r="E10" s="79"/>
+      <c r="F10" s="40">
         <v>42</v>
       </c>
-      <c r="G10" s="58">
+      <c r="G10" s="56">
         <v>25</v>
       </c>
-      <c r="H10" s="80"/>
-      <c r="I10" s="81"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="58"/>
-      <c r="L10" s="42">
+      <c r="H10" s="78"/>
+      <c r="I10" s="79"/>
+      <c r="J10" s="40"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="40">
         <v>51</v>
       </c>
-      <c r="M10" s="58">
+      <c r="M10" s="56">
         <v>16</v>
       </c>
-      <c r="N10" s="42"/>
-      <c r="O10" s="58"/>
-      <c r="P10" s="42">
+      <c r="N10" s="40"/>
+      <c r="O10" s="56"/>
+      <c r="P10" s="40">
         <v>49</v>
       </c>
-      <c r="Q10" s="58">
+      <c r="Q10" s="56">
         <v>18</v>
       </c>
-      <c r="R10" s="42">
+      <c r="R10" s="40">
         <v>46</v>
       </c>
-      <c r="S10" s="58">
+      <c r="S10" s="56">
         <v>21</v>
       </c>
-      <c r="T10" s="42">
+      <c r="T10" s="40">
         <v>45</v>
       </c>
-      <c r="U10" s="58">
+      <c r="U10" s="56">
         <v>20</v>
       </c>
-      <c r="V10" s="42">
+      <c r="V10" s="40">
         <v>46</v>
       </c>
-      <c r="W10" s="58">
+      <c r="W10" s="56">
         <v>19</v>
       </c>
-      <c r="X10" s="42">
+      <c r="X10" s="40">
         <v>53</v>
       </c>
-      <c r="Y10" s="58">
+      <c r="Y10" s="56">
         <v>13</v>
       </c>
-      <c r="Z10" s="42">
+      <c r="Z10" s="40">
         <v>52</v>
       </c>
-      <c r="AA10" s="58">
+      <c r="AA10" s="56">
         <v>13</v>
       </c>
-      <c r="AB10" s="42">
+      <c r="AB10" s="40">
         <v>44</v>
       </c>
-      <c r="AC10" s="58">
+      <c r="AC10" s="56">
         <v>22</v>
       </c>
-      <c r="AD10" s="26">
+      <c r="AD10" s="24">
         <v>42</v>
       </c>
-      <c r="AE10" s="56">
+      <c r="AE10" s="54">
         <v>24</v>
       </c>
-      <c r="AF10" s="26">
+      <c r="AF10" s="24">
         <v>45</v>
       </c>
-      <c r="AG10" s="56">
+      <c r="AG10" s="54">
         <v>20</v>
       </c>
-      <c r="AH10" s="26">
+      <c r="AH10" s="24">
         <v>48</v>
       </c>
-      <c r="AI10" s="56">
+      <c r="AI10" s="54">
         <v>17</v>
       </c>
-      <c r="AJ10" s="80"/>
-      <c r="AK10" s="81"/>
-      <c r="AL10" s="26">
+      <c r="AJ10" s="78"/>
+      <c r="AK10" s="79"/>
+      <c r="AL10" s="24">
         <v>50</v>
       </c>
-      <c r="AM10" s="56">
+      <c r="AM10" s="54">
         <v>15</v>
       </c>
-      <c r="AN10" s="80"/>
-      <c r="AO10" s="83"/>
-      <c r="AP10" s="26">
+      <c r="AN10" s="78"/>
+      <c r="AO10" s="81"/>
+      <c r="AP10" s="24">
         <v>42</v>
       </c>
-      <c r="AQ10" s="67">
+      <c r="AQ10" s="65">
         <v>23</v>
       </c>
-      <c r="AR10" s="69">
+      <c r="AR10" s="67">
         <f t="shared" si="1"/>
         <v>655</v>
       </c>
-      <c r="AS10" s="8">
+      <c r="AS10" s="6">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="AT10" s="71">
+      <c r="AT10" s="69">
         <v>2</v>
       </c>
-      <c r="AU10" s="75">
+      <c r="AU10" s="73">
         <v>3</v>
       </c>
-      <c r="AV10" s="25">
+      <c r="AV10" s="23">
         <f t="shared" si="3"/>
         <v>271</v>
       </c>
-      <c r="AW10" s="39">
+      <c r="AW10" s="37">
         <f t="shared" si="4"/>
         <v>19.357142857142858</v>
       </c>
-      <c r="AX10" s="51"/>
-      <c r="AY10" s="25"/>
-      <c r="AZ10" s="25"/>
-      <c r="BA10" s="8"/>
-      <c r="BB10" s="35"/>
+      <c r="AX10" s="49"/>
+      <c r="AY10" s="23"/>
+      <c r="AZ10" s="23"/>
+      <c r="BA10" s="6"/>
+      <c r="BB10" s="33"/>
     </row>
     <row r="11" spans="1:54">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="64">
+      <c r="C11" s="62">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D11" s="80"/>
-      <c r="E11" s="81"/>
-      <c r="F11" s="9">
+      <c r="D11" s="78"/>
+      <c r="E11" s="79"/>
+      <c r="F11" s="7">
         <v>42</v>
       </c>
-      <c r="G11" s="58">
+      <c r="G11" s="56">
         <v>27</v>
       </c>
-      <c r="H11" s="80"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="58"/>
-      <c r="L11" s="9">
+      <c r="H11" s="78"/>
+      <c r="I11" s="79"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="7">
         <v>54</v>
       </c>
-      <c r="M11" s="58">
+      <c r="M11" s="56">
         <v>15</v>
       </c>
-      <c r="N11" s="9"/>
-      <c r="O11" s="58"/>
-      <c r="P11" s="9">
+      <c r="N11" s="7"/>
+      <c r="O11" s="56"/>
+      <c r="P11" s="7">
         <v>54</v>
       </c>
-      <c r="Q11" s="58">
+      <c r="Q11" s="56">
         <v>16</v>
       </c>
-      <c r="R11" s="9">
+      <c r="R11" s="7">
         <v>53</v>
       </c>
-      <c r="S11" s="58">
+      <c r="S11" s="56">
         <v>16</v>
       </c>
-      <c r="T11" s="9"/>
-      <c r="U11" s="58"/>
-      <c r="V11" s="9">
+      <c r="T11" s="7"/>
+      <c r="U11" s="56"/>
+      <c r="V11" s="7">
         <v>46</v>
       </c>
-      <c r="W11" s="58">
+      <c r="W11" s="56">
         <v>23</v>
       </c>
-      <c r="X11" s="9">
+      <c r="X11" s="7">
         <v>49</v>
       </c>
-      <c r="Y11" s="58">
+      <c r="Y11" s="56">
         <v>19</v>
       </c>
-      <c r="Z11" s="9">
+      <c r="Z11" s="7">
         <v>50</v>
       </c>
-      <c r="AA11" s="58">
+      <c r="AA11" s="56">
         <v>18</v>
       </c>
-      <c r="AB11" s="9"/>
-      <c r="AC11" s="58"/>
-      <c r="AD11" s="41"/>
-      <c r="AE11" s="56"/>
-      <c r="AF11" s="41"/>
-      <c r="AG11" s="56"/>
-      <c r="AH11" s="41">
+      <c r="AB11" s="7"/>
+      <c r="AC11" s="56"/>
+      <c r="AD11" s="39"/>
+      <c r="AE11" s="54"/>
+      <c r="AF11" s="39"/>
+      <c r="AG11" s="54"/>
+      <c r="AH11" s="39">
         <v>50</v>
       </c>
-      <c r="AI11" s="56">
+      <c r="AI11" s="54">
         <v>18</v>
       </c>
-      <c r="AJ11" s="80"/>
-      <c r="AK11" s="81"/>
-      <c r="AL11" s="41">
+      <c r="AJ11" s="78"/>
+      <c r="AK11" s="79"/>
+      <c r="AL11" s="39">
         <v>50</v>
       </c>
-      <c r="AM11" s="56">
+      <c r="AM11" s="54">
         <v>18</v>
       </c>
-      <c r="AN11" s="80"/>
-      <c r="AO11" s="83"/>
-      <c r="AP11" s="41">
+      <c r="AN11" s="78"/>
+      <c r="AO11" s="81"/>
+      <c r="AP11" s="39">
         <v>52</v>
       </c>
-      <c r="AQ11" s="67">
+      <c r="AQ11" s="65">
         <v>16</v>
       </c>
-      <c r="AR11" s="69">
+      <c r="AR11" s="67">
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="AS11" s="8">
+      <c r="AS11" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT11" s="71">
+      <c r="AT11" s="69">
         <v>1</v>
       </c>
-      <c r="AU11" s="75">
+      <c r="AU11" s="73">
         <v>1</v>
       </c>
-      <c r="AV11" s="25">
+      <c r="AV11" s="23">
         <f t="shared" si="3"/>
         <v>188</v>
       </c>
-      <c r="AW11" s="39">
+      <c r="AW11" s="37">
         <f t="shared" si="4"/>
         <v>18.8</v>
       </c>
-      <c r="AX11" s="34"/>
-      <c r="AY11" s="25"/>
-      <c r="AZ11" s="25"/>
-      <c r="BA11" s="8"/>
-      <c r="BB11" s="35"/>
+      <c r="AX11" s="32"/>
+      <c r="AY11" s="23"/>
+      <c r="AZ11" s="23"/>
+      <c r="BA11" s="6"/>
+      <c r="BB11" s="33"/>
     </row>
     <row r="12" spans="1:54">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="64">
+      <c r="C12" s="62">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="D12" s="80"/>
-      <c r="E12" s="81"/>
-      <c r="F12" s="9">
+      <c r="D12" s="78"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="7">
         <v>51</v>
       </c>
-      <c r="G12" s="58">
+      <c r="G12" s="56">
         <v>18</v>
       </c>
-      <c r="H12" s="80"/>
-      <c r="I12" s="81"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="58"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="58"/>
-      <c r="N12" s="9">
+      <c r="H12" s="78"/>
+      <c r="I12" s="79"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="56"/>
+      <c r="N12" s="7">
         <v>51</v>
       </c>
-      <c r="O12" s="58">
+      <c r="O12" s="56">
         <v>18</v>
       </c>
-      <c r="P12" s="9">
+      <c r="P12" s="7">
         <v>52</v>
       </c>
-      <c r="Q12" s="58">
+      <c r="Q12" s="56">
         <v>17</v>
       </c>
-      <c r="R12" s="9"/>
-      <c r="S12" s="58"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="58"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="58"/>
-      <c r="X12" s="9">
+      <c r="R12" s="7"/>
+      <c r="S12" s="56"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="56"/>
+      <c r="V12" s="7"/>
+      <c r="W12" s="56"/>
+      <c r="X12" s="7">
         <v>48</v>
       </c>
-      <c r="Y12" s="58">
+      <c r="Y12" s="56">
         <v>21</v>
       </c>
-      <c r="Z12" s="9"/>
-      <c r="AA12" s="58"/>
-      <c r="AB12" s="9">
+      <c r="Z12" s="7"/>
+      <c r="AA12" s="56"/>
+      <c r="AB12" s="7">
         <v>51</v>
       </c>
-      <c r="AC12" s="58">
+      <c r="AC12" s="56">
         <v>18</v>
       </c>
-      <c r="AD12" s="41"/>
-      <c r="AE12" s="56"/>
-      <c r="AF12" s="41"/>
-      <c r="AG12" s="56"/>
-      <c r="AH12" s="41"/>
-      <c r="AI12" s="56"/>
-      <c r="AJ12" s="80"/>
-      <c r="AK12" s="81"/>
-      <c r="AL12" s="41"/>
-      <c r="AM12" s="56"/>
-      <c r="AN12" s="80"/>
-      <c r="AO12" s="83"/>
-      <c r="AP12" s="41">
+      <c r="AD12" s="39"/>
+      <c r="AE12" s="54"/>
+      <c r="AF12" s="39"/>
+      <c r="AG12" s="54"/>
+      <c r="AH12" s="39"/>
+      <c r="AI12" s="54"/>
+      <c r="AJ12" s="78"/>
+      <c r="AK12" s="79"/>
+      <c r="AL12" s="39"/>
+      <c r="AM12" s="54"/>
+      <c r="AN12" s="78"/>
+      <c r="AO12" s="81"/>
+      <c r="AP12" s="39">
         <v>51</v>
       </c>
-      <c r="AQ12" s="67">
+      <c r="AQ12" s="65">
         <v>19</v>
       </c>
-      <c r="AR12" s="69">
+      <c r="AR12" s="67">
         <f t="shared" si="1"/>
         <v>304</v>
       </c>
-      <c r="AS12" s="8">
+      <c r="AS12" s="6">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="AT12" s="71"/>
-      <c r="AU12" s="75"/>
-      <c r="AV12" s="25">
+      <c r="AT12" s="69"/>
+      <c r="AU12" s="73"/>
+      <c r="AV12" s="23">
         <f t="shared" si="3"/>
         <v>111</v>
       </c>
-      <c r="AW12" s="39">
+      <c r="AW12" s="37">
         <f t="shared" si="4"/>
         <v>18.5</v>
       </c>
-      <c r="AX12" s="36"/>
-      <c r="AY12" s="25"/>
-      <c r="AZ12" s="25"/>
-      <c r="BA12" s="8"/>
-      <c r="BB12" s="35"/>
+      <c r="AX12" s="34"/>
+      <c r="AY12" s="23"/>
+      <c r="AZ12" s="23"/>
+      <c r="BA12" s="6"/>
+      <c r="BB12" s="33"/>
     </row>
     <row r="13" spans="1:54">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="64">
+      <c r="C13" s="62">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D13" s="80"/>
-      <c r="E13" s="81"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="58"/>
-      <c r="H13" s="80"/>
-      <c r="I13" s="81"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="58"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="58"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="58"/>
-      <c r="P13" s="9">
+      <c r="D13" s="78"/>
+      <c r="E13" s="79"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="78"/>
+      <c r="I13" s="79"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="56"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="56"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="56"/>
+      <c r="P13" s="7">
         <v>48</v>
       </c>
-      <c r="Q13" s="58">
+      <c r="Q13" s="56">
         <v>18</v>
       </c>
-      <c r="R13" s="9">
+      <c r="R13" s="7">
         <v>51</v>
       </c>
-      <c r="S13" s="58">
+      <c r="S13" s="56">
         <v>14</v>
       </c>
-      <c r="T13" s="9">
+      <c r="T13" s="7">
         <v>51</v>
       </c>
-      <c r="U13" s="58">
+      <c r="U13" s="56">
         <v>14</v>
       </c>
-      <c r="V13" s="9"/>
-      <c r="W13" s="58"/>
-      <c r="X13" s="9">
+      <c r="V13" s="7"/>
+      <c r="W13" s="56"/>
+      <c r="X13" s="7">
         <v>48</v>
       </c>
-      <c r="Y13" s="58">
+      <c r="Y13" s="56">
         <v>20</v>
       </c>
-      <c r="Z13" s="9">
+      <c r="Z13" s="7">
         <v>50</v>
       </c>
-      <c r="AA13" s="58">
+      <c r="AA13" s="56">
         <v>18</v>
       </c>
-      <c r="AB13" s="9">
+      <c r="AB13" s="7">
         <v>47</v>
       </c>
-      <c r="AC13" s="58">
+      <c r="AC13" s="56">
         <v>21</v>
       </c>
-      <c r="AD13" s="41"/>
-      <c r="AE13" s="56"/>
-      <c r="AF13" s="41">
+      <c r="AD13" s="39"/>
+      <c r="AE13" s="54"/>
+      <c r="AF13" s="39">
         <v>46</v>
       </c>
-      <c r="AG13" s="56">
+      <c r="AG13" s="54">
         <v>21</v>
       </c>
-      <c r="AH13" s="41">
+      <c r="AH13" s="39">
         <v>48</v>
       </c>
-      <c r="AI13" s="56">
+      <c r="AI13" s="54">
         <v>19</v>
       </c>
-      <c r="AJ13" s="80"/>
-      <c r="AK13" s="81"/>
-      <c r="AL13" s="41"/>
-      <c r="AM13" s="56"/>
-      <c r="AN13" s="80"/>
-      <c r="AO13" s="83"/>
-      <c r="AP13" s="41">
+      <c r="AJ13" s="78"/>
+      <c r="AK13" s="79"/>
+      <c r="AL13" s="39"/>
+      <c r="AM13" s="54"/>
+      <c r="AN13" s="78"/>
+      <c r="AO13" s="81"/>
+      <c r="AP13" s="39">
         <v>47</v>
       </c>
-      <c r="AQ13" s="67">
+      <c r="AQ13" s="65">
         <v>20</v>
       </c>
-      <c r="AR13" s="69">
+      <c r="AR13" s="67">
         <f t="shared" si="1"/>
         <v>436</v>
       </c>
-      <c r="AS13" s="8">
+      <c r="AS13" s="6">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="AT13" s="71"/>
-      <c r="AU13" s="75">
+      <c r="AT13" s="69"/>
+      <c r="AU13" s="73">
         <v>1</v>
       </c>
-      <c r="AV13" s="25">
+      <c r="AV13" s="23">
         <f t="shared" si="3"/>
         <v>166</v>
       </c>
-      <c r="AW13" s="39">
+      <c r="AW13" s="37">
         <f t="shared" si="4"/>
         <v>18.444444444444443</v>
       </c>
-      <c r="AX13" s="34"/>
-      <c r="AY13" s="25"/>
-      <c r="AZ13" s="25"/>
-      <c r="BA13" s="8"/>
-      <c r="BB13" s="35"/>
+      <c r="AX13" s="32"/>
+      <c r="AY13" s="23"/>
+      <c r="AZ13" s="23"/>
+      <c r="BA13" s="6"/>
+      <c r="BB13" s="33"/>
     </row>
     <row r="14" spans="1:54">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="64">
+      <c r="C14" s="62">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="D14" s="80"/>
-      <c r="E14" s="81"/>
-      <c r="F14" s="9">
+      <c r="D14" s="78"/>
+      <c r="E14" s="79"/>
+      <c r="F14" s="7">
         <v>59</v>
       </c>
-      <c r="G14" s="58">
+      <c r="G14" s="56">
         <v>17</v>
       </c>
-      <c r="H14" s="80"/>
-      <c r="I14" s="81"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="58"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="58"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="58"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="58"/>
-      <c r="R14" s="9">
+      <c r="H14" s="78"/>
+      <c r="I14" s="79"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="56"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="56"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="56"/>
+      <c r="R14" s="7">
         <v>55</v>
       </c>
-      <c r="S14" s="58">
+      <c r="S14" s="56">
         <v>21</v>
       </c>
-      <c r="T14" s="9"/>
-      <c r="U14" s="58"/>
-      <c r="V14" s="9">
+      <c r="T14" s="7"/>
+      <c r="U14" s="56"/>
+      <c r="V14" s="7">
         <v>59</v>
       </c>
-      <c r="W14" s="58">
+      <c r="W14" s="56">
         <v>17</v>
       </c>
-      <c r="X14" s="9"/>
-      <c r="Y14" s="58"/>
-      <c r="Z14" s="9"/>
-      <c r="AA14" s="58"/>
-      <c r="AB14" s="9"/>
-      <c r="AC14" s="58"/>
-      <c r="AD14" s="41"/>
-      <c r="AE14" s="56"/>
-      <c r="AF14" s="41"/>
-      <c r="AG14" s="56"/>
-      <c r="AH14" s="41"/>
-      <c r="AI14" s="56"/>
-      <c r="AJ14" s="80"/>
-      <c r="AK14" s="81"/>
-      <c r="AL14" s="41"/>
-      <c r="AM14" s="56"/>
-      <c r="AN14" s="80"/>
-      <c r="AO14" s="83"/>
-      <c r="AP14" s="41"/>
-      <c r="AQ14" s="67"/>
-      <c r="AR14" s="69">
+      <c r="X14" s="7"/>
+      <c r="Y14" s="56"/>
+      <c r="Z14" s="7"/>
+      <c r="AA14" s="56"/>
+      <c r="AB14" s="7"/>
+      <c r="AC14" s="56"/>
+      <c r="AD14" s="39"/>
+      <c r="AE14" s="54"/>
+      <c r="AF14" s="39"/>
+      <c r="AG14" s="54"/>
+      <c r="AH14" s="39"/>
+      <c r="AI14" s="54"/>
+      <c r="AJ14" s="78"/>
+      <c r="AK14" s="79"/>
+      <c r="AL14" s="39"/>
+      <c r="AM14" s="54"/>
+      <c r="AN14" s="78"/>
+      <c r="AO14" s="81"/>
+      <c r="AP14" s="39"/>
+      <c r="AQ14" s="65"/>
+      <c r="AR14" s="67">
         <f t="shared" si="1"/>
         <v>173</v>
       </c>
-      <c r="AS14" s="8">
+      <c r="AS14" s="6">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AT14" s="71"/>
-      <c r="AU14" s="75"/>
-      <c r="AV14" s="25">
+      <c r="AT14" s="69"/>
+      <c r="AU14" s="73"/>
+      <c r="AV14" s="23">
         <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="AW14" s="39">
+      <c r="AW14" s="37">
         <f t="shared" si="4"/>
         <v>18.333333333333332</v>
       </c>
-      <c r="AX14" s="36"/>
-      <c r="AY14" s="25"/>
-      <c r="AZ14" s="25"/>
-      <c r="BA14" s="8"/>
-      <c r="BB14" s="35"/>
+      <c r="AX14" s="34"/>
+      <c r="AY14" s="23"/>
+      <c r="AZ14" s="23"/>
+      <c r="BA14" s="6"/>
+      <c r="BB14" s="33"/>
     </row>
     <row r="15" spans="1:54">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="64">
+      <c r="C15" s="62">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D15" s="80"/>
-      <c r="E15" s="81"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="80"/>
-      <c r="I15" s="81"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="58"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="58"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="58"/>
-      <c r="P15" s="11">
+      <c r="D15" s="78"/>
+      <c r="E15" s="79"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="79"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="56"/>
+      <c r="P15" s="9">
         <v>47</v>
       </c>
-      <c r="Q15" s="58">
+      <c r="Q15" s="56">
         <v>20</v>
       </c>
-      <c r="R15" s="11">
+      <c r="R15" s="9">
         <v>50</v>
       </c>
-      <c r="S15" s="58">
+      <c r="S15" s="56">
         <v>17</v>
       </c>
-      <c r="T15" s="11">
+      <c r="T15" s="9">
         <v>46</v>
       </c>
-      <c r="U15" s="58">
+      <c r="U15" s="56">
         <v>21</v>
       </c>
-      <c r="V15" s="11">
+      <c r="V15" s="9">
         <v>47</v>
       </c>
-      <c r="W15" s="58">
+      <c r="W15" s="56">
         <v>19</v>
       </c>
-      <c r="X15" s="11">
+      <c r="X15" s="9">
         <v>44</v>
       </c>
-      <c r="Y15" s="58">
+      <c r="Y15" s="56">
         <v>22</v>
       </c>
-      <c r="Z15" s="11">
+      <c r="Z15" s="9">
         <v>52</v>
       </c>
-      <c r="AA15" s="58">
+      <c r="AA15" s="56">
         <v>14</v>
       </c>
-      <c r="AB15" s="11">
+      <c r="AB15" s="9">
         <v>47</v>
       </c>
-      <c r="AC15" s="58">
+      <c r="AC15" s="56">
         <v>19</v>
       </c>
-      <c r="AD15" s="26">
+      <c r="AD15" s="24">
         <v>51</v>
       </c>
-      <c r="AE15" s="56">
+      <c r="AE15" s="54">
         <v>15</v>
       </c>
-      <c r="AF15" s="26">
+      <c r="AF15" s="24">
         <v>49</v>
       </c>
-      <c r="AG15" s="56">
+      <c r="AG15" s="54">
         <v>17</v>
       </c>
-      <c r="AH15" s="26">
+      <c r="AH15" s="24">
         <v>46</v>
       </c>
-      <c r="AI15" s="56">
+      <c r="AI15" s="54">
         <v>20</v>
       </c>
-      <c r="AJ15" s="80"/>
-      <c r="AK15" s="81"/>
-      <c r="AL15" s="26">
+      <c r="AJ15" s="78"/>
+      <c r="AK15" s="79"/>
+      <c r="AL15" s="24">
         <v>51</v>
       </c>
-      <c r="AM15" s="56">
+      <c r="AM15" s="54">
         <v>15</v>
       </c>
-      <c r="AN15" s="80"/>
-      <c r="AO15" s="83"/>
-      <c r="AP15" s="26">
+      <c r="AN15" s="78"/>
+      <c r="AO15" s="81"/>
+      <c r="AP15" s="24">
         <v>49</v>
       </c>
-      <c r="AQ15" s="67">
+      <c r="AQ15" s="65">
         <v>17</v>
       </c>
-      <c r="AR15" s="69">
+      <c r="AR15" s="67">
         <f t="shared" si="1"/>
         <v>579</v>
       </c>
-      <c r="AS15" s="8">
+      <c r="AS15" s="6">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="AT15" s="71"/>
-      <c r="AU15" s="75"/>
-      <c r="AV15" s="25">
+      <c r="AT15" s="69"/>
+      <c r="AU15" s="73"/>
+      <c r="AV15" s="23">
         <f t="shared" si="3"/>
         <v>216</v>
       </c>
-      <c r="AW15" s="39">
+      <c r="AW15" s="37">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="AX15" s="34"/>
-      <c r="AY15" s="25"/>
-      <c r="AZ15" s="25"/>
-      <c r="BA15" s="8"/>
-      <c r="BB15" s="35"/>
+      <c r="AX15" s="32"/>
+      <c r="AY15" s="23"/>
+      <c r="AZ15" s="23"/>
+      <c r="BA15" s="6"/>
+      <c r="BB15" s="33"/>
     </row>
     <row r="16" spans="1:54">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="64">
+      <c r="C16" s="62">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="D16" s="80"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="9">
+      <c r="D16" s="78"/>
+      <c r="E16" s="79"/>
+      <c r="F16" s="7">
         <v>55</v>
       </c>
-      <c r="G16" s="58">
+      <c r="G16" s="56">
         <v>16</v>
       </c>
-      <c r="H16" s="80"/>
-      <c r="I16" s="81"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="58"/>
-      <c r="L16" s="9">
+      <c r="H16" s="78"/>
+      <c r="I16" s="79"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="7">
         <v>56</v>
       </c>
-      <c r="M16" s="58">
+      <c r="M16" s="56">
         <v>15</v>
       </c>
-      <c r="N16" s="9">
+      <c r="N16" s="7">
         <v>57</v>
       </c>
-      <c r="O16" s="58">
+      <c r="O16" s="56">
         <v>14</v>
       </c>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="58"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="58"/>
-      <c r="T16" s="9">
+      <c r="P16" s="7"/>
+      <c r="Q16" s="56"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="56"/>
+      <c r="T16" s="7">
         <v>49</v>
       </c>
-      <c r="U16" s="58">
+      <c r="U16" s="56">
         <v>22</v>
       </c>
-      <c r="V16" s="9">
+      <c r="V16" s="7">
         <v>58</v>
       </c>
-      <c r="W16" s="58">
+      <c r="W16" s="56">
         <v>14</v>
       </c>
-      <c r="X16" s="9">
+      <c r="X16" s="7">
         <v>50</v>
       </c>
-      <c r="Y16" s="58">
+      <c r="Y16" s="56">
         <v>23</v>
       </c>
-      <c r="Z16" s="9">
+      <c r="Z16" s="7">
         <v>56</v>
       </c>
-      <c r="AA16" s="58">
+      <c r="AA16" s="56">
         <v>16</v>
       </c>
-      <c r="AB16" s="9">
+      <c r="AB16" s="7">
         <v>49</v>
       </c>
-      <c r="AC16" s="58">
+      <c r="AC16" s="56">
         <v>23</v>
       </c>
-      <c r="AD16" s="41">
+      <c r="AD16" s="39">
         <v>54</v>
       </c>
-      <c r="AE16" s="56">
+      <c r="AE16" s="54">
         <v>18</v>
       </c>
-      <c r="AF16" s="41">
+      <c r="AF16" s="39">
         <v>58</v>
       </c>
-      <c r="AG16" s="56">
+      <c r="AG16" s="54">
         <v>14</v>
       </c>
-      <c r="AH16" s="41">
+      <c r="AH16" s="39">
         <v>52</v>
       </c>
-      <c r="AI16" s="56">
+      <c r="AI16" s="54">
         <v>20</v>
       </c>
-      <c r="AJ16" s="80"/>
-      <c r="AK16" s="81"/>
-      <c r="AL16" s="41"/>
-      <c r="AM16" s="56"/>
-      <c r="AN16" s="80"/>
-      <c r="AO16" s="83"/>
-      <c r="AP16" s="41"/>
-      <c r="AQ16" s="67"/>
-      <c r="AR16" s="69">
+      <c r="AJ16" s="78"/>
+      <c r="AK16" s="79"/>
+      <c r="AL16" s="39"/>
+      <c r="AM16" s="54"/>
+      <c r="AN16" s="78"/>
+      <c r="AO16" s="81"/>
+      <c r="AP16" s="39"/>
+      <c r="AQ16" s="65"/>
+      <c r="AR16" s="67">
         <f t="shared" si="1"/>
         <v>594</v>
       </c>
-      <c r="AS16" s="8">
+      <c r="AS16" s="6">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AT16" s="71">
+      <c r="AT16" s="69">
         <v>2</v>
       </c>
-      <c r="AU16" s="75"/>
-      <c r="AV16" s="25">
+      <c r="AU16" s="73"/>
+      <c r="AV16" s="23">
         <f t="shared" si="3"/>
         <v>197</v>
       </c>
-      <c r="AW16" s="39">
+      <c r="AW16" s="37">
         <f t="shared" si="4"/>
         <v>17.90909090909091</v>
       </c>
-      <c r="AX16" s="36"/>
-      <c r="AY16" s="25"/>
-      <c r="AZ16" s="25"/>
-      <c r="BA16" s="8"/>
-      <c r="BB16" s="35"/>
+      <c r="AX16" s="34"/>
+      <c r="AY16" s="23"/>
+      <c r="AZ16" s="23"/>
+      <c r="BA16" s="6"/>
+      <c r="BB16" s="33"/>
     </row>
     <row r="17" spans="1:54">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="64">
+      <c r="C17" s="62">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D17" s="80"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="58"/>
-      <c r="H17" s="80"/>
-      <c r="I17" s="81"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="58"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="58"/>
-      <c r="N17" s="11">
+      <c r="D17" s="78"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="78"/>
+      <c r="I17" s="79"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="9">
         <v>45</v>
       </c>
-      <c r="O17" s="58">
+      <c r="O17" s="56">
         <v>18</v>
       </c>
-      <c r="P17" s="11">
+      <c r="P17" s="9">
         <v>43</v>
       </c>
-      <c r="Q17" s="58">
+      <c r="Q17" s="56">
         <v>20</v>
       </c>
-      <c r="R17" s="11"/>
-      <c r="S17" s="58"/>
-      <c r="T17" s="11"/>
-      <c r="U17" s="58"/>
-      <c r="V17" s="11"/>
-      <c r="W17" s="58"/>
-      <c r="X17" s="11">
+      <c r="R17" s="9"/>
+      <c r="S17" s="56"/>
+      <c r="T17" s="9"/>
+      <c r="U17" s="56"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="56"/>
+      <c r="X17" s="9">
         <v>48</v>
       </c>
-      <c r="Y17" s="58">
+      <c r="Y17" s="56">
         <v>15</v>
       </c>
-      <c r="Z17" s="11">
+      <c r="Z17" s="9">
         <v>47</v>
       </c>
-      <c r="AA17" s="58">
+      <c r="AA17" s="56">
         <v>16</v>
       </c>
-      <c r="AB17" s="11"/>
-      <c r="AC17" s="58"/>
-      <c r="AD17" s="26">
+      <c r="AB17" s="9"/>
+      <c r="AC17" s="56"/>
+      <c r="AD17" s="24">
         <v>51</v>
       </c>
-      <c r="AE17" s="56">
+      <c r="AE17" s="54">
         <v>13</v>
       </c>
-      <c r="AF17" s="26">
+      <c r="AF17" s="24">
         <v>45</v>
       </c>
-      <c r="AG17" s="56">
+      <c r="AG17" s="54">
         <v>20</v>
       </c>
-      <c r="AH17" s="26"/>
-      <c r="AI17" s="56"/>
-      <c r="AJ17" s="80"/>
-      <c r="AK17" s="81"/>
-      <c r="AL17" s="26"/>
-      <c r="AM17" s="56"/>
-      <c r="AN17" s="80"/>
-      <c r="AO17" s="83"/>
-      <c r="AP17" s="26">
+      <c r="AH17" s="24"/>
+      <c r="AI17" s="54"/>
+      <c r="AJ17" s="78"/>
+      <c r="AK17" s="79"/>
+      <c r="AL17" s="24"/>
+      <c r="AM17" s="54"/>
+      <c r="AN17" s="78"/>
+      <c r="AO17" s="81"/>
+      <c r="AP17" s="24">
         <v>44</v>
       </c>
-      <c r="AQ17" s="67">
+      <c r="AQ17" s="65">
         <v>21</v>
       </c>
-      <c r="AR17" s="69">
+      <c r="AR17" s="67">
         <f t="shared" si="1"/>
         <v>323</v>
       </c>
-      <c r="AS17" s="8">
+      <c r="AS17" s="6">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AT17" s="71"/>
-      <c r="AU17" s="75">
+      <c r="AT17" s="69"/>
+      <c r="AU17" s="73">
         <v>2</v>
       </c>
-      <c r="AV17" s="25">
+      <c r="AV17" s="23">
         <f t="shared" si="3"/>
         <v>125</v>
       </c>
-      <c r="AW17" s="39">
+      <c r="AW17" s="37">
         <f t="shared" si="4"/>
         <v>17.857142857142858</v>
       </c>
-      <c r="AX17" s="34"/>
-      <c r="AY17" s="25"/>
-      <c r="AZ17" s="25"/>
-      <c r="BA17" s="8"/>
-      <c r="BB17" s="35"/>
+      <c r="AX17" s="32"/>
+      <c r="AY17" s="23"/>
+      <c r="AZ17" s="23"/>
+      <c r="BA17" s="6"/>
+      <c r="BB17" s="33"/>
     </row>
     <row r="18" spans="1:54">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="64">
+      <c r="C18" s="62">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D18" s="80"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="9">
+      <c r="D18" s="78"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="7">
         <v>46</v>
       </c>
-      <c r="G18" s="58">
+      <c r="G18" s="56">
         <v>16</v>
       </c>
-      <c r="H18" s="80"/>
-      <c r="I18" s="81"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="58"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="58"/>
-      <c r="N18" s="9">
+      <c r="H18" s="78"/>
+      <c r="I18" s="79"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="7">
         <v>42</v>
       </c>
-      <c r="O18" s="58">
+      <c r="O18" s="56">
         <v>20</v>
       </c>
-      <c r="P18" s="9">
+      <c r="P18" s="7">
         <v>43</v>
       </c>
-      <c r="Q18" s="58">
+      <c r="Q18" s="56">
         <v>19</v>
       </c>
-      <c r="R18" s="9"/>
-      <c r="S18" s="58"/>
-      <c r="T18" s="9"/>
-      <c r="U18" s="58"/>
-      <c r="V18" s="9"/>
-      <c r="W18" s="58"/>
-      <c r="X18" s="9">
+      <c r="R18" s="7"/>
+      <c r="S18" s="56"/>
+      <c r="T18" s="7"/>
+      <c r="U18" s="56"/>
+      <c r="V18" s="7"/>
+      <c r="W18" s="56"/>
+      <c r="X18" s="7">
         <v>47</v>
       </c>
-      <c r="Y18" s="58">
+      <c r="Y18" s="56">
         <v>16</v>
       </c>
-      <c r="Z18" s="9">
+      <c r="Z18" s="7">
         <v>41</v>
       </c>
-      <c r="AA18" s="58">
+      <c r="AA18" s="56">
         <v>22</v>
       </c>
-      <c r="AB18" s="9">
+      <c r="AB18" s="7">
         <v>50</v>
       </c>
-      <c r="AC18" s="58">
+      <c r="AC18" s="56">
         <v>13</v>
       </c>
-      <c r="AD18" s="41">
+      <c r="AD18" s="39">
         <v>44</v>
       </c>
-      <c r="AE18" s="56">
+      <c r="AE18" s="54">
         <v>19</v>
       </c>
-      <c r="AF18" s="41">
+      <c r="AF18" s="39">
         <v>43</v>
       </c>
-      <c r="AG18" s="56">
+      <c r="AG18" s="54">
         <v>20</v>
       </c>
-      <c r="AH18" s="41">
+      <c r="AH18" s="39">
         <v>49</v>
       </c>
-      <c r="AI18" s="56">
+      <c r="AI18" s="54">
         <v>15</v>
       </c>
-      <c r="AJ18" s="80"/>
-      <c r="AK18" s="81"/>
-      <c r="AL18" s="41"/>
-      <c r="AM18" s="56"/>
-      <c r="AN18" s="80"/>
-      <c r="AO18" s="83"/>
-      <c r="AP18" s="131">
+      <c r="AJ18" s="78"/>
+      <c r="AK18" s="79"/>
+      <c r="AL18" s="39"/>
+      <c r="AM18" s="54"/>
+      <c r="AN18" s="78"/>
+      <c r="AO18" s="81"/>
+      <c r="AP18" s="98">
         <v>48</v>
       </c>
-      <c r="AQ18" s="67">
+      <c r="AQ18" s="65">
         <v>15</v>
       </c>
-      <c r="AR18" s="69">
+      <c r="AR18" s="67">
         <f t="shared" si="1"/>
         <v>453</v>
       </c>
-      <c r="AS18" s="8">
+      <c r="AS18" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT18" s="71">
+      <c r="AT18" s="69">
         <v>2</v>
       </c>
-      <c r="AU18" s="75">
+      <c r="AU18" s="73">
         <v>1</v>
       </c>
-      <c r="AV18" s="25">
+      <c r="AV18" s="23">
         <f t="shared" si="3"/>
         <v>178</v>
       </c>
-      <c r="AW18" s="39">
+      <c r="AW18" s="37">
         <f t="shared" si="4"/>
         <v>17.8</v>
       </c>
-      <c r="AX18" s="36"/>
-      <c r="AY18" s="25"/>
-      <c r="AZ18" s="25"/>
-      <c r="BA18" s="8"/>
-      <c r="BB18" s="35"/>
+      <c r="AX18" s="34"/>
+      <c r="AY18" s="23"/>
+      <c r="AZ18" s="23"/>
+      <c r="BA18" s="6"/>
+      <c r="BB18" s="33"/>
     </row>
     <row r="19" spans="1:54">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="64">
+      <c r="C19" s="62">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D19" s="80"/>
-      <c r="E19" s="81"/>
-      <c r="F19" s="9">
+      <c r="D19" s="78"/>
+      <c r="E19" s="79"/>
+      <c r="F19" s="7">
         <v>46</v>
       </c>
-      <c r="G19" s="58">
+      <c r="G19" s="56">
         <v>18</v>
       </c>
-      <c r="H19" s="80"/>
-      <c r="I19" s="81"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="58"/>
-      <c r="L19" s="9">
+      <c r="H19" s="78"/>
+      <c r="I19" s="79"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="56"/>
+      <c r="L19" s="7">
         <v>46</v>
       </c>
-      <c r="M19" s="58">
+      <c r="M19" s="56">
         <v>18</v>
       </c>
-      <c r="N19" s="9">
+      <c r="N19" s="7">
         <v>46</v>
       </c>
-      <c r="O19" s="58">
+      <c r="O19" s="56">
         <v>18</v>
       </c>
-      <c r="P19" s="9">
+      <c r="P19" s="7">
         <v>46</v>
       </c>
-      <c r="Q19" s="58">
+      <c r="Q19" s="56">
         <v>18</v>
       </c>
-      <c r="R19" s="9">
+      <c r="R19" s="7">
         <v>47</v>
       </c>
-      <c r="S19" s="58">
+      <c r="S19" s="56">
         <v>14</v>
       </c>
-      <c r="T19" s="9">
+      <c r="T19" s="7">
         <v>52</v>
       </c>
-      <c r="U19" s="58">
+      <c r="U19" s="56">
         <v>13</v>
       </c>
-      <c r="V19" s="9"/>
-      <c r="W19" s="58"/>
-      <c r="X19" s="9"/>
-      <c r="Y19" s="58"/>
-      <c r="Z19" s="9">
+      <c r="V19" s="7"/>
+      <c r="W19" s="56"/>
+      <c r="X19" s="7"/>
+      <c r="Y19" s="56"/>
+      <c r="Z19" s="7">
         <v>50</v>
       </c>
-      <c r="AA19" s="58">
+      <c r="AA19" s="56">
         <v>15</v>
       </c>
-      <c r="AB19" s="9"/>
-      <c r="AC19" s="58"/>
-      <c r="AD19" s="41">
+      <c r="AB19" s="7"/>
+      <c r="AC19" s="56"/>
+      <c r="AD19" s="39">
         <v>47</v>
       </c>
-      <c r="AE19" s="56">
+      <c r="AE19" s="54">
         <v>19</v>
       </c>
-      <c r="AF19" s="41">
+      <c r="AF19" s="39">
         <v>48</v>
       </c>
-      <c r="AG19" s="56">
+      <c r="AG19" s="54">
         <v>18</v>
       </c>
-      <c r="AH19" s="41">
+      <c r="AH19" s="39">
         <v>44</v>
       </c>
-      <c r="AI19" s="56">
+      <c r="AI19" s="54">
         <v>22</v>
       </c>
-      <c r="AJ19" s="80"/>
-      <c r="AK19" s="81"/>
-      <c r="AL19" s="41"/>
-      <c r="AM19" s="56"/>
-      <c r="AN19" s="80"/>
-      <c r="AO19" s="83"/>
-      <c r="AP19" s="41"/>
-      <c r="AQ19" s="67"/>
-      <c r="AR19" s="69">
+      <c r="AJ19" s="78"/>
+      <c r="AK19" s="79"/>
+      <c r="AL19" s="39"/>
+      <c r="AM19" s="54"/>
+      <c r="AN19" s="78"/>
+      <c r="AO19" s="81"/>
+      <c r="AP19" s="39"/>
+      <c r="AQ19" s="65"/>
+      <c r="AR19" s="67">
         <f t="shared" si="1"/>
         <v>472</v>
       </c>
-      <c r="AS19" s="8">
+      <c r="AS19" s="6">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AT19" s="72"/>
-      <c r="AU19" s="76">
+      <c r="AT19" s="70"/>
+      <c r="AU19" s="74">
         <v>1</v>
       </c>
-      <c r="AV19" s="25">
+      <c r="AV19" s="23">
         <f t="shared" si="3"/>
         <v>174</v>
       </c>
-      <c r="AW19" s="39">
+      <c r="AW19" s="37">
         <f t="shared" si="4"/>
         <v>17.399999999999999</v>
       </c>
-      <c r="AX19" s="36"/>
-      <c r="AY19" s="8"/>
-      <c r="AZ19" s="8"/>
-      <c r="BA19" s="8"/>
-      <c r="BB19" s="35"/>
+      <c r="AX19" s="34"/>
+      <c r="AY19" s="6"/>
+      <c r="AZ19" s="6"/>
+      <c r="BA19" s="6"/>
+      <c r="BB19" s="33"/>
     </row>
     <row r="20" spans="1:54">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="64">
+      <c r="C20" s="62">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="D20" s="80"/>
-      <c r="E20" s="81"/>
-      <c r="F20" s="10">
+      <c r="D20" s="78"/>
+      <c r="E20" s="79"/>
+      <c r="F20" s="8">
         <v>61</v>
       </c>
-      <c r="G20" s="58">
+      <c r="G20" s="56">
         <v>14</v>
       </c>
-      <c r="H20" s="80"/>
-      <c r="I20" s="81"/>
-      <c r="J20" s="10">
+      <c r="H20" s="78"/>
+      <c r="I20" s="79"/>
+      <c r="J20" s="8">
         <v>56</v>
       </c>
-      <c r="K20" s="58">
+      <c r="K20" s="56">
         <v>19</v>
       </c>
-      <c r="L20" s="10">
+      <c r="L20" s="8">
         <v>60</v>
       </c>
-      <c r="M20" s="58">
+      <c r="M20" s="56">
         <v>15</v>
       </c>
-      <c r="N20" s="10">
+      <c r="N20" s="8">
         <v>56</v>
       </c>
-      <c r="O20" s="58">
+      <c r="O20" s="56">
         <v>20</v>
       </c>
-      <c r="P20" s="10">
+      <c r="P20" s="8">
         <v>54</v>
       </c>
-      <c r="Q20" s="58">
+      <c r="Q20" s="56">
         <v>22</v>
       </c>
-      <c r="R20" s="10"/>
-      <c r="S20" s="58"/>
-      <c r="T20" s="10">
+      <c r="R20" s="8"/>
+      <c r="S20" s="56"/>
+      <c r="T20" s="8">
         <v>66</v>
       </c>
-      <c r="U20" s="58">
+      <c r="U20" s="56">
         <v>9</v>
       </c>
-      <c r="V20" s="10">
+      <c r="V20" s="8">
         <v>55</v>
       </c>
-      <c r="W20" s="58">
+      <c r="W20" s="56">
         <v>22</v>
       </c>
-      <c r="X20" s="10"/>
-      <c r="Y20" s="58"/>
-      <c r="Z20" s="10">
+      <c r="X20" s="8"/>
+      <c r="Y20" s="56"/>
+      <c r="Z20" s="8">
         <v>70</v>
       </c>
-      <c r="AA20" s="58">
+      <c r="AA20" s="56">
         <v>6</v>
       </c>
-      <c r="AB20" s="10">
+      <c r="AB20" s="8">
         <v>63</v>
       </c>
-      <c r="AC20" s="58">
+      <c r="AC20" s="56">
         <v>15</v>
       </c>
-      <c r="AD20" s="26">
+      <c r="AD20" s="24">
         <v>58</v>
       </c>
-      <c r="AE20" s="56">
+      <c r="AE20" s="54">
         <v>20</v>
       </c>
-      <c r="AF20" s="26">
+      <c r="AF20" s="24">
         <v>60</v>
       </c>
-      <c r="AG20" s="56">
+      <c r="AG20" s="54">
         <v>18</v>
       </c>
-      <c r="AH20" s="26">
+      <c r="AH20" s="24">
         <v>55</v>
       </c>
-      <c r="AI20" s="56">
+      <c r="AI20" s="54">
         <v>23</v>
       </c>
-      <c r="AJ20" s="80"/>
-      <c r="AK20" s="81"/>
-      <c r="AL20" s="26"/>
-      <c r="AM20" s="56"/>
-      <c r="AN20" s="80"/>
-      <c r="AO20" s="83"/>
-      <c r="AP20" s="26"/>
-      <c r="AQ20" s="67"/>
-      <c r="AR20" s="69">
+      <c r="AJ20" s="78"/>
+      <c r="AK20" s="79"/>
+      <c r="AL20" s="24"/>
+      <c r="AM20" s="54"/>
+      <c r="AN20" s="78"/>
+      <c r="AO20" s="81"/>
+      <c r="AP20" s="24"/>
+      <c r="AQ20" s="65"/>
+      <c r="AR20" s="67">
         <f t="shared" si="1"/>
         <v>714</v>
       </c>
-      <c r="AS20" s="8">
+      <c r="AS20" s="6">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="AT20" s="71">
+      <c r="AT20" s="69">
         <v>2</v>
       </c>
-      <c r="AU20" s="75"/>
-      <c r="AV20" s="25">
+      <c r="AU20" s="73"/>
+      <c r="AV20" s="23">
         <f t="shared" si="3"/>
         <v>205</v>
       </c>
-      <c r="AW20" s="39">
+      <c r="AW20" s="37">
         <f t="shared" si="4"/>
         <v>17.083333333333332</v>
       </c>
-      <c r="AX20" s="34"/>
-      <c r="AY20" s="25"/>
-      <c r="AZ20" s="25"/>
-      <c r="BA20" s="8"/>
-      <c r="BB20" s="35"/>
+      <c r="AX20" s="32"/>
+      <c r="AY20" s="23"/>
+      <c r="AZ20" s="23"/>
+      <c r="BA20" s="6"/>
+      <c r="BB20" s="33"/>
     </row>
     <row r="21" spans="1:54">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="64">
+      <c r="C21" s="62">
         <v>18</v>
       </c>
-      <c r="D21" s="80"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="9">
+      <c r="D21" s="78"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="7">
         <v>56</v>
       </c>
-      <c r="G21" s="58">
+      <c r="G21" s="56">
         <v>16</v>
       </c>
-      <c r="H21" s="80"/>
-      <c r="I21" s="81"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="58"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="58"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="58"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="58"/>
-      <c r="R21" s="9"/>
-      <c r="S21" s="58"/>
-      <c r="T21" s="9"/>
-      <c r="U21" s="58"/>
-      <c r="V21" s="9"/>
-      <c r="W21" s="58"/>
-      <c r="X21" s="9"/>
-      <c r="Y21" s="58"/>
-      <c r="Z21" s="9"/>
-      <c r="AA21" s="58"/>
-      <c r="AB21" s="9"/>
-      <c r="AC21" s="58"/>
-      <c r="AD21" s="41"/>
-      <c r="AE21" s="56"/>
-      <c r="AF21" s="41"/>
-      <c r="AG21" s="56"/>
-      <c r="AH21" s="41"/>
-      <c r="AI21" s="56"/>
-      <c r="AJ21" s="80"/>
-      <c r="AK21" s="81"/>
-      <c r="AL21" s="41"/>
-      <c r="AM21" s="56"/>
-      <c r="AN21" s="80"/>
-      <c r="AO21" s="83"/>
-      <c r="AP21" s="41"/>
-      <c r="AQ21" s="67"/>
-      <c r="AR21" s="69">
+      <c r="H21" s="78"/>
+      <c r="I21" s="79"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="56"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="56"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="56"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="56"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="56"/>
+      <c r="T21" s="7"/>
+      <c r="U21" s="56"/>
+      <c r="V21" s="7"/>
+      <c r="W21" s="56"/>
+      <c r="X21" s="7"/>
+      <c r="Y21" s="56"/>
+      <c r="Z21" s="7"/>
+      <c r="AA21" s="56"/>
+      <c r="AB21" s="7"/>
+      <c r="AC21" s="56"/>
+      <c r="AD21" s="39"/>
+      <c r="AE21" s="54"/>
+      <c r="AF21" s="39"/>
+      <c r="AG21" s="54"/>
+      <c r="AH21" s="39"/>
+      <c r="AI21" s="54"/>
+      <c r="AJ21" s="78"/>
+      <c r="AK21" s="79"/>
+      <c r="AL21" s="39"/>
+      <c r="AM21" s="54"/>
+      <c r="AN21" s="78"/>
+      <c r="AO21" s="81"/>
+      <c r="AP21" s="39"/>
+      <c r="AQ21" s="65"/>
+      <c r="AR21" s="67">
         <f t="shared" si="1"/>
         <v>56</v>
       </c>
-      <c r="AS21" s="8">
+      <c r="AS21" s="6">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT21" s="71"/>
-      <c r="AU21" s="75"/>
-      <c r="AV21" s="25">
+      <c r="AT21" s="69"/>
+      <c r="AU21" s="73"/>
+      <c r="AV21" s="23">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="AW21" s="39">
+      <c r="AW21" s="37">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="AX21" s="36"/>
-      <c r="AY21" s="25"/>
-      <c r="AZ21" s="25"/>
-      <c r="BA21" s="8"/>
-      <c r="BB21" s="35"/>
+      <c r="AX21" s="34"/>
+      <c r="AY21" s="23"/>
+      <c r="AZ21" s="23"/>
+      <c r="BA21" s="6"/>
+      <c r="BB21" s="33"/>
     </row>
     <row r="22" spans="1:54">
-      <c r="A22" s="61" t="s">
+      <c r="A22" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="62" t="s">
+      <c r="B22" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="65" t="s">
+      <c r="C22" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="80"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="47"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="80"/>
-      <c r="I22" s="81"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="58"/>
-      <c r="L22" s="47">
+      <c r="D22" s="78"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="56"/>
+      <c r="H22" s="78"/>
+      <c r="I22" s="79"/>
+      <c r="J22" s="45"/>
+      <c r="K22" s="56"/>
+      <c r="L22" s="45">
         <v>50</v>
       </c>
-      <c r="M22" s="58"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="58"/>
-      <c r="P22" s="47"/>
-      <c r="Q22" s="58"/>
-      <c r="R22" s="47"/>
-      <c r="S22" s="58"/>
-      <c r="T22" s="47"/>
-      <c r="U22" s="58"/>
-      <c r="V22" s="47"/>
-      <c r="W22" s="58"/>
-      <c r="X22" s="47"/>
-      <c r="Y22" s="58"/>
-      <c r="Z22" s="47"/>
-      <c r="AA22" s="58"/>
-      <c r="AB22" s="47"/>
-      <c r="AC22" s="58"/>
-      <c r="AD22" s="57"/>
-      <c r="AE22" s="58"/>
-      <c r="AF22" s="57"/>
-      <c r="AG22" s="58"/>
-      <c r="AH22" s="57"/>
-      <c r="AI22" s="58"/>
-      <c r="AJ22" s="80"/>
-      <c r="AK22" s="81"/>
-      <c r="AL22" s="57"/>
-      <c r="AM22" s="58"/>
-      <c r="AN22" s="80"/>
-      <c r="AO22" s="83"/>
-      <c r="AP22" s="48"/>
-      <c r="AQ22" s="67"/>
-      <c r="AR22" s="69">
+      <c r="M22" s="56"/>
+      <c r="N22" s="45"/>
+      <c r="O22" s="56"/>
+      <c r="P22" s="45"/>
+      <c r="Q22" s="56"/>
+      <c r="R22" s="45"/>
+      <c r="S22" s="56"/>
+      <c r="T22" s="45"/>
+      <c r="U22" s="56"/>
+      <c r="V22" s="45"/>
+      <c r="W22" s="56"/>
+      <c r="X22" s="45"/>
+      <c r="Y22" s="56"/>
+      <c r="Z22" s="45"/>
+      <c r="AA22" s="56"/>
+      <c r="AB22" s="45"/>
+      <c r="AC22" s="56"/>
+      <c r="AD22" s="55"/>
+      <c r="AE22" s="56"/>
+      <c r="AF22" s="55"/>
+      <c r="AG22" s="56"/>
+      <c r="AH22" s="55"/>
+      <c r="AI22" s="56"/>
+      <c r="AJ22" s="78"/>
+      <c r="AK22" s="79"/>
+      <c r="AL22" s="55"/>
+      <c r="AM22" s="56"/>
+      <c r="AN22" s="78"/>
+      <c r="AO22" s="81"/>
+      <c r="AP22" s="46"/>
+      <c r="AQ22" s="65"/>
+      <c r="AR22" s="67">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="AS22" s="8">
+      <c r="AS22" s="6">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT22" s="71">
+      <c r="AT22" s="69">
         <v>1</v>
       </c>
-      <c r="AU22" s="75"/>
-      <c r="AV22" s="25">
+      <c r="AU22" s="73"/>
+      <c r="AV22" s="23">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="AW22" s="39">
+      <c r="AW22" s="37">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="AX22" s="50"/>
-      <c r="AY22" s="53"/>
-      <c r="AZ22" s="53"/>
-      <c r="BA22" s="52"/>
-      <c r="BB22" s="54"/>
+      <c r="AX22" s="48"/>
+      <c r="AY22" s="51"/>
+      <c r="AZ22" s="51"/>
+      <c r="BA22" s="50"/>
+      <c r="BB22" s="52"/>
     </row>
     <row r="23" spans="1:54">
-      <c r="A23" s="61" t="s">
+      <c r="A23" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="62" t="s">
+      <c r="B23" s="60" t="s">
         <v>72</v>
       </c>
-      <c r="C23" s="65" t="s">
+      <c r="C23" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="80"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="47"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="80"/>
-      <c r="I23" s="81"/>
-      <c r="J23" s="47"/>
-      <c r="K23" s="58"/>
-      <c r="L23" s="47"/>
-      <c r="M23" s="58"/>
-      <c r="N23" s="47"/>
-      <c r="O23" s="58"/>
-      <c r="P23" s="47"/>
-      <c r="Q23" s="58"/>
-      <c r="R23" s="47"/>
-      <c r="S23" s="58"/>
-      <c r="T23" s="47"/>
-      <c r="U23" s="58"/>
-      <c r="V23" s="47"/>
-      <c r="W23" s="58"/>
-      <c r="X23" s="47"/>
-      <c r="Y23" s="58"/>
-      <c r="Z23" s="47"/>
-      <c r="AA23" s="58"/>
-      <c r="AB23" s="47"/>
-      <c r="AC23" s="58"/>
-      <c r="AD23" s="57"/>
-      <c r="AE23" s="58"/>
-      <c r="AF23" s="57"/>
-      <c r="AG23" s="58"/>
-      <c r="AH23" s="57"/>
-      <c r="AI23" s="58"/>
-      <c r="AJ23" s="80"/>
-      <c r="AK23" s="81"/>
-      <c r="AL23" s="132">
+      <c r="D23" s="78"/>
+      <c r="E23" s="79"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="79"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="56"/>
+      <c r="L23" s="45"/>
+      <c r="M23" s="56"/>
+      <c r="N23" s="45"/>
+      <c r="O23" s="56"/>
+      <c r="P23" s="45"/>
+      <c r="Q23" s="56"/>
+      <c r="R23" s="45"/>
+      <c r="S23" s="56"/>
+      <c r="T23" s="45"/>
+      <c r="U23" s="56"/>
+      <c r="V23" s="45"/>
+      <c r="W23" s="56"/>
+      <c r="X23" s="45"/>
+      <c r="Y23" s="56"/>
+      <c r="Z23" s="45"/>
+      <c r="AA23" s="56"/>
+      <c r="AB23" s="45"/>
+      <c r="AC23" s="56"/>
+      <c r="AD23" s="55"/>
+      <c r="AE23" s="56"/>
+      <c r="AF23" s="55"/>
+      <c r="AG23" s="56"/>
+      <c r="AH23" s="55"/>
+      <c r="AI23" s="56"/>
+      <c r="AJ23" s="78"/>
+      <c r="AK23" s="79"/>
+      <c r="AL23" s="99">
         <v>50</v>
       </c>
-      <c r="AM23" s="58"/>
-      <c r="AN23" s="80"/>
-      <c r="AO23" s="83"/>
-      <c r="AP23" s="48"/>
-      <c r="AQ23" s="67"/>
-      <c r="AR23" s="69">
+      <c r="AM23" s="56"/>
+      <c r="AN23" s="78"/>
+      <c r="AO23" s="81"/>
+      <c r="AP23" s="46"/>
+      <c r="AQ23" s="65"/>
+      <c r="AR23" s="67">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="AS23" s="8">
+      <c r="AS23" s="6">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT23" s="71"/>
-      <c r="AU23" s="75"/>
-      <c r="AV23" s="25">
+      <c r="AT23" s="69"/>
+      <c r="AU23" s="73"/>
+      <c r="AV23" s="23">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AW23" s="39">
+      <c r="AW23" s="37">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="AX23" s="50"/>
-      <c r="AY23" s="53"/>
-      <c r="AZ23" s="53"/>
-      <c r="BA23" s="52"/>
-      <c r="BB23" s="54"/>
+      <c r="AX23" s="48"/>
+      <c r="AY23" s="51"/>
+      <c r="AZ23" s="51"/>
+      <c r="BA23" s="50"/>
+      <c r="BB23" s="52"/>
     </row>
-    <row r="24" spans="1:54" ht="16.5" thickBot="1">
-      <c r="A24" s="61" t="s">
+    <row r="24" spans="1:54" ht="17" thickBot="1">
+      <c r="A24" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="62" t="s">
+      <c r="B24" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="65" t="s">
+      <c r="C24" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="80"/>
-      <c r="E24" s="81"/>
-      <c r="F24" s="84"/>
-      <c r="G24" s="85"/>
-      <c r="H24" s="80"/>
-      <c r="I24" s="81"/>
-      <c r="J24" s="84"/>
-      <c r="K24" s="85"/>
-      <c r="L24" s="84"/>
-      <c r="M24" s="85"/>
-      <c r="N24" s="84"/>
-      <c r="O24" s="85"/>
-      <c r="P24" s="84"/>
-      <c r="Q24" s="85"/>
-      <c r="R24" s="84"/>
-      <c r="S24" s="85"/>
-      <c r="T24" s="84"/>
-      <c r="U24" s="85"/>
-      <c r="V24" s="84"/>
-      <c r="W24" s="85"/>
-      <c r="X24" s="84"/>
-      <c r="Y24" s="85"/>
-      <c r="Z24" s="84"/>
-      <c r="AA24" s="85"/>
-      <c r="AB24" s="84"/>
-      <c r="AC24" s="85"/>
-      <c r="AD24" s="86"/>
-      <c r="AE24" s="85"/>
-      <c r="AF24" s="86"/>
-      <c r="AG24" s="85"/>
-      <c r="AH24" s="86"/>
-      <c r="AI24" s="85"/>
-      <c r="AJ24" s="80"/>
-      <c r="AK24" s="81"/>
-      <c r="AL24" s="86"/>
-      <c r="AM24" s="85"/>
-      <c r="AN24" s="80"/>
-      <c r="AO24" s="83"/>
-      <c r="AP24" s="87">
+      <c r="D24" s="78"/>
+      <c r="E24" s="79"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="83"/>
+      <c r="H24" s="78"/>
+      <c r="I24" s="79"/>
+      <c r="J24" s="82"/>
+      <c r="K24" s="83"/>
+      <c r="L24" s="82"/>
+      <c r="M24" s="83"/>
+      <c r="N24" s="82"/>
+      <c r="O24" s="83"/>
+      <c r="P24" s="82"/>
+      <c r="Q24" s="83"/>
+      <c r="R24" s="82"/>
+      <c r="S24" s="83"/>
+      <c r="T24" s="82"/>
+      <c r="U24" s="83"/>
+      <c r="V24" s="82"/>
+      <c r="W24" s="83"/>
+      <c r="X24" s="82"/>
+      <c r="Y24" s="83"/>
+      <c r="Z24" s="82"/>
+      <c r="AA24" s="83"/>
+      <c r="AB24" s="82"/>
+      <c r="AC24" s="83"/>
+      <c r="AD24" s="84"/>
+      <c r="AE24" s="83"/>
+      <c r="AF24" s="84"/>
+      <c r="AG24" s="83"/>
+      <c r="AH24" s="84"/>
+      <c r="AI24" s="83"/>
+      <c r="AJ24" s="78"/>
+      <c r="AK24" s="79"/>
+      <c r="AL24" s="84"/>
+      <c r="AM24" s="83"/>
+      <c r="AN24" s="78"/>
+      <c r="AO24" s="81"/>
+      <c r="AP24" s="85">
         <v>45</v>
       </c>
-      <c r="AQ24" s="88"/>
-      <c r="AR24" s="69">
+      <c r="AQ24" s="86"/>
+      <c r="AR24" s="67">
         <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="AS24" s="12">
+      <c r="AS24" s="10">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AT24" s="73"/>
-      <c r="AU24" s="77"/>
-      <c r="AV24" s="27">
+      <c r="AT24" s="71"/>
+      <c r="AU24" s="75"/>
+      <c r="AV24" s="25">
         <v>0</v>
       </c>
-      <c r="AW24" s="40">
+      <c r="AW24" s="38">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="AX24" s="50"/>
-      <c r="AY24" s="53"/>
-      <c r="AZ24" s="53"/>
-      <c r="BA24" s="52"/>
-      <c r="BB24" s="54"/>
+      <c r="AX24" s="48"/>
+      <c r="AY24" s="51"/>
+      <c r="AZ24" s="51"/>
+      <c r="BA24" s="50"/>
+      <c r="BB24" s="52"/>
     </row>
-    <row r="25" spans="1:54" s="13" customFormat="1" ht="16.5" thickBot="1">
-      <c r="A25" s="89"/>
-      <c r="B25" s="90"/>
-      <c r="C25" s="91"/>
-      <c r="D25" s="92"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23">
+    <row r="25" spans="1:54" s="11" customFormat="1" ht="17" thickBot="1">
+      <c r="A25" s="87"/>
+      <c r="B25" s="88"/>
+      <c r="C25" s="89"/>
+      <c r="D25" s="90"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21">
         <f>AVERAGEIF(F4:F23,"&gt;0")</f>
         <v>49.75</v>
       </c>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21">
         <f>AVERAGEIF(J4:J23,"&gt;0")</f>
         <v>54</v>
       </c>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23">
+      <c r="K25" s="21"/>
+      <c r="L25" s="21">
         <f>AVERAGEIF(L4:L23,"&gt;0")</f>
         <v>51.428571428571431</v>
       </c>
-      <c r="M25" s="23"/>
-      <c r="N25" s="23">
+      <c r="M25" s="21"/>
+      <c r="N25" s="21">
         <f>AVERAGEIF(N4:N23,"&gt;0")</f>
         <v>48.9</v>
       </c>
-      <c r="O25" s="23"/>
-      <c r="P25" s="23">
+      <c r="O25" s="21"/>
+      <c r="P25" s="21">
         <f>AVERAGEIF(P4:P23,"&gt;0")</f>
         <v>46.785714285714285</v>
       </c>
-      <c r="Q25" s="23"/>
-      <c r="R25" s="23">
+      <c r="Q25" s="21"/>
+      <c r="R25" s="21">
         <f>AVERAGEIF(R4:R23,"&gt;0")</f>
         <v>48.272727272727273</v>
       </c>
-      <c r="S25" s="23"/>
-      <c r="T25" s="23">
+      <c r="S25" s="21"/>
+      <c r="T25" s="21">
         <f>AVERAGEIF(T4:T23,"&gt;0")</f>
         <v>50.333333333333336</v>
       </c>
-      <c r="U25" s="23"/>
-      <c r="V25" s="23">
+      <c r="U25" s="21"/>
+      <c r="V25" s="21">
         <f>AVERAGEIF(V4:V23,"&gt;0")</f>
         <v>49</v>
       </c>
-      <c r="W25" s="23"/>
-      <c r="X25" s="23">
+      <c r="W25" s="21"/>
+      <c r="X25" s="21">
         <f>AVERAGEIF(X4:X23,"&gt;0")</f>
         <v>46.46153846153846</v>
       </c>
-      <c r="Y25" s="23"/>
-      <c r="Z25" s="23">
+      <c r="Y25" s="21"/>
+      <c r="Z25" s="21">
         <f>AVERAGEIF(Z4:Z23,"&gt;0")</f>
         <v>49.53846153846154</v>
       </c>
-      <c r="AA25" s="23"/>
-      <c r="AB25" s="23">
+      <c r="AA25" s="21"/>
+      <c r="AB25" s="21">
         <f>AVERAGEIF(AB4:AB23,"&gt;0")</f>
         <v>47.846153846153847</v>
       </c>
-      <c r="AC25" s="60"/>
-      <c r="AD25" s="93">
+      <c r="AC25" s="58"/>
+      <c r="AD25" s="91">
         <f>AVERAGEIF(AD4:AD23,"&gt;0")</f>
         <v>46.090909090909093</v>
       </c>
-      <c r="AE25" s="94"/>
-      <c r="AF25" s="93">
+      <c r="AE25" s="92"/>
+      <c r="AF25" s="91">
         <f>AVERAGEIF(AF4:AF23,"&gt;0")</f>
         <v>47.230769230769234</v>
       </c>
-      <c r="AG25" s="94"/>
-      <c r="AH25" s="93">
+      <c r="AG25" s="92"/>
+      <c r="AH25" s="91">
         <f>AVERAGEIF(AH4:AH23,"&gt;0")</f>
         <v>46.666666666666664</v>
       </c>
-      <c r="AI25" s="94"/>
-      <c r="AJ25" s="93"/>
-      <c r="AK25" s="94"/>
-      <c r="AL25" s="93">
+      <c r="AI25" s="92"/>
+      <c r="AJ25" s="91"/>
+      <c r="AK25" s="92"/>
+      <c r="AL25" s="91">
         <f>AVERAGEIF(AL4:AL23,"&gt;0")</f>
         <v>49.5</v>
       </c>
-      <c r="AM25" s="94"/>
-      <c r="AN25" s="93"/>
-      <c r="AO25" s="94"/>
-      <c r="AP25" s="93">
+      <c r="AM25" s="92"/>
+      <c r="AN25" s="91"/>
+      <c r="AO25" s="92"/>
+      <c r="AP25" s="91">
         <f>AVERAGEIF(AP4:AP23,"&gt;0")</f>
         <v>45.727272727272727</v>
       </c>
-      <c r="AQ25" s="94"/>
-      <c r="AR25" s="95"/>
+      <c r="AQ25" s="92"/>
+      <c r="AR25" s="93"/>
     </row>
     <row r="26" spans="1:54">
-      <c r="C26" s="14"/>
-      <c r="AR26" s="15"/>
-      <c r="AS26" s="15"/>
-      <c r="AT26" s="16"/>
-      <c r="AU26" s="16"/>
-      <c r="AV26" s="15"/>
-      <c r="AW26" s="17"/>
+      <c r="C26" s="12"/>
+      <c r="AR26" s="13"/>
+      <c r="AS26" s="13"/>
+      <c r="AT26" s="14"/>
+      <c r="AU26" s="14"/>
+      <c r="AV26" s="13"/>
+      <c r="AW26" s="15"/>
     </row>
     <row r="27" spans="1:54">
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="D27" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="J27" s="18"/>
-      <c r="L27" s="18"/>
-      <c r="N27" s="18"/>
-      <c r="P27" s="18"/>
-      <c r="R27" s="18"/>
-      <c r="T27" s="18"/>
-      <c r="V27" s="18"/>
-      <c r="X27" s="18"/>
-      <c r="Z27" s="18"/>
-      <c r="AB27" s="18"/>
-      <c r="AD27" s="18"/>
-      <c r="AF27" s="18"/>
-      <c r="AH27" s="18"/>
-      <c r="AJ27" s="18"/>
-      <c r="AL27" s="18"/>
-      <c r="AN27" s="18"/>
-      <c r="AP27" s="18"/>
+      <c r="F27" s="16"/>
+      <c r="H27" s="16"/>
+      <c r="J27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="T27" s="16"/>
+      <c r="V27" s="16"/>
+      <c r="X27" s="16"/>
+      <c r="Z27" s="16"/>
+      <c r="AB27" s="16"/>
+      <c r="AD27" s="16"/>
+      <c r="AF27" s="16"/>
+      <c r="AH27" s="16"/>
+      <c r="AJ27" s="16"/>
+      <c r="AL27" s="16"/>
+      <c r="AN27" s="16"/>
+      <c r="AP27" s="16"/>
     </row>
     <row r="28" spans="1:54">
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="F28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="N28" s="19"/>
-      <c r="P28" s="19"/>
-      <c r="R28" s="19"/>
-      <c r="T28" s="19"/>
-      <c r="V28" s="19"/>
-      <c r="X28" s="19"/>
-      <c r="Z28" s="19"/>
-      <c r="AB28" s="19"/>
-      <c r="AD28" s="19"/>
-      <c r="AF28" s="19"/>
-      <c r="AH28" s="19"/>
-      <c r="AJ28" s="19"/>
-      <c r="AL28" s="19"/>
-      <c r="AN28" s="19"/>
-      <c r="AP28" s="19"/>
-      <c r="AR28" s="20"/>
+      <c r="F28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="L28" s="17"/>
+      <c r="N28" s="17"/>
+      <c r="P28" s="17"/>
+      <c r="R28" s="17"/>
+      <c r="T28" s="17"/>
+      <c r="V28" s="17"/>
+      <c r="X28" s="17"/>
+      <c r="Z28" s="17"/>
+      <c r="AB28" s="17"/>
+      <c r="AD28" s="17"/>
+      <c r="AF28" s="17"/>
+      <c r="AH28" s="17"/>
+      <c r="AJ28" s="17"/>
+      <c r="AL28" s="17"/>
+      <c r="AN28" s="17"/>
+      <c r="AP28" s="17"/>
+      <c r="AR28" s="18"/>
     </row>
     <row r="29" spans="1:54">
-      <c r="C29" s="30" t="s">
+      <c r="C29" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="22"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="22"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="21"/>
-      <c r="O29" s="22"/>
-      <c r="P29" s="21"/>
-      <c r="Q29" s="22"/>
-      <c r="R29" s="21"/>
-      <c r="S29" s="22"/>
-      <c r="T29" s="21"/>
-      <c r="U29" s="22"/>
-      <c r="V29" s="21"/>
-      <c r="W29" s="22"/>
-      <c r="X29" s="21"/>
-      <c r="Y29" s="22"/>
-      <c r="Z29" s="21"/>
-      <c r="AA29" s="22"/>
-      <c r="AB29" s="21"/>
-      <c r="AC29" s="22"/>
-      <c r="AD29" s="21"/>
-      <c r="AE29" s="22"/>
-      <c r="AF29" s="21"/>
-      <c r="AG29" s="22"/>
-      <c r="AH29" s="21"/>
-      <c r="AI29" s="22"/>
-      <c r="AJ29" s="21"/>
-      <c r="AK29" s="22"/>
-      <c r="AL29" s="21"/>
-      <c r="AM29" s="22"/>
-      <c r="AN29" s="21"/>
-      <c r="AO29" s="22"/>
-      <c r="AP29" s="21"/>
-      <c r="AQ29" s="22"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="20"/>
+      <c r="N29" s="19"/>
+      <c r="O29" s="20"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="20"/>
+      <c r="R29" s="19"/>
+      <c r="S29" s="20"/>
+      <c r="T29" s="19"/>
+      <c r="U29" s="20"/>
+      <c r="V29" s="19"/>
+      <c r="W29" s="20"/>
+      <c r="X29" s="19"/>
+      <c r="Y29" s="20"/>
+      <c r="Z29" s="19"/>
+      <c r="AA29" s="20"/>
+      <c r="AB29" s="19"/>
+      <c r="AC29" s="20"/>
+      <c r="AD29" s="19"/>
+      <c r="AE29" s="20"/>
+      <c r="AF29" s="19"/>
+      <c r="AG29" s="20"/>
+      <c r="AH29" s="19"/>
+      <c r="AI29" s="20"/>
+      <c r="AJ29" s="19"/>
+      <c r="AK29" s="20"/>
+      <c r="AL29" s="19"/>
+      <c r="AM29" s="20"/>
+      <c r="AN29" s="19"/>
+      <c r="AO29" s="20"/>
+      <c r="AP29" s="19"/>
+      <c r="AQ29" s="20"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:BB24">
@@ -4683,6 +4689,45 @@
     <sortCondition descending="1" ref="AR4:AR24"/>
   </sortState>
   <mergeCells count="55">
+    <mergeCell ref="AJ1:AK1"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AL1:AM1"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AV2:AV3"/>
+    <mergeCell ref="AR1:AR3"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AN2:AO2"/>
+    <mergeCell ref="AW2:AW3"/>
+    <mergeCell ref="AT2:AT3"/>
+    <mergeCell ref="AU2:AU3"/>
+    <mergeCell ref="AS2:AS3"/>
+    <mergeCell ref="AS1:AW1"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AP2:AQ2"/>
+    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="AX2:AX3"/>
+    <mergeCell ref="AY2:AY3"/>
+    <mergeCell ref="AZ2:AZ3"/>
+    <mergeCell ref="BA2:BA3"/>
+    <mergeCell ref="BB2:BB3"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="AB1:AC1"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="AH1:AI1"/>
     <mergeCell ref="AH2:AI2"/>
     <mergeCell ref="H1:I1"/>
@@ -4697,47 +4742,8 @@
     <mergeCell ref="AD2:AE2"/>
     <mergeCell ref="AF1:AG1"/>
     <mergeCell ref="AF2:AG2"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="AB1:AC1"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="AX1:BB1"/>
-    <mergeCell ref="AX2:AX3"/>
-    <mergeCell ref="AY2:AY3"/>
-    <mergeCell ref="AZ2:AZ3"/>
-    <mergeCell ref="BA2:BA3"/>
-    <mergeCell ref="BB2:BB3"/>
-    <mergeCell ref="AV2:AV3"/>
-    <mergeCell ref="AR1:AR3"/>
-    <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AN2:AO2"/>
-    <mergeCell ref="AW2:AW3"/>
-    <mergeCell ref="AT2:AT3"/>
-    <mergeCell ref="AU2:AU3"/>
-    <mergeCell ref="AS2:AS3"/>
-    <mergeCell ref="AS1:AW1"/>
-    <mergeCell ref="AP1:AQ1"/>
-    <mergeCell ref="AP2:AQ2"/>
-    <mergeCell ref="AJ1:AK1"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AL1:AM1"/>
-    <mergeCell ref="AL2:AM2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
092325 - fixed a couple of names
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Overall Standings.xlsx
+++ b/public/results/2025/2025 Overall Standings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DA6B2A-580F-44C5-9A65-6C3CA4E654D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8B5DDA-51CE-401D-875E-33BF25358092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="90" yWindow="90" windowWidth="20475" windowHeight="10980" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
+    <workbookView xWindow="930" yWindow="45" windowWidth="10245" windowHeight="10755" xr2:uid="{1A9894EE-562E-3246-9111-2FABF9BD81D0}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 Overall" sheetId="1" r:id="rId1"/>
@@ -1172,99 +1172,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1471,6 +1378,99 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1850,239 +1850,239 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:56" s="14" customFormat="1" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="56" t="s">
+      <c r="B1" s="106"/>
+      <c r="C1" s="111" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="D1" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="29"/>
-      <c r="F1" s="28" t="s">
+      <c r="E1" s="102"/>
+      <c r="F1" s="101" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="29"/>
-      <c r="H1" s="28" t="s">
+      <c r="G1" s="102"/>
+      <c r="H1" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="28" t="s">
+      <c r="I1" s="102"/>
+      <c r="J1" s="101" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="29"/>
-      <c r="L1" s="28" t="s">
+      <c r="K1" s="102"/>
+      <c r="L1" s="101" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="29"/>
-      <c r="N1" s="28" t="s">
+      <c r="M1" s="102"/>
+      <c r="N1" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="O1" s="29"/>
-      <c r="P1" s="28" t="s">
+      <c r="O1" s="102"/>
+      <c r="P1" s="101" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="28" t="s">
+      <c r="Q1" s="102"/>
+      <c r="R1" s="101" t="s">
         <v>60</v>
       </c>
-      <c r="S1" s="29"/>
-      <c r="T1" s="28" t="s">
+      <c r="S1" s="102"/>
+      <c r="T1" s="101" t="s">
         <v>61</v>
       </c>
-      <c r="U1" s="29"/>
-      <c r="V1" s="28" t="s">
+      <c r="U1" s="102"/>
+      <c r="V1" s="101" t="s">
         <v>62</v>
       </c>
-      <c r="W1" s="29"/>
-      <c r="X1" s="28" t="s">
+      <c r="W1" s="102"/>
+      <c r="X1" s="101" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="29"/>
-      <c r="Z1" s="28" t="s">
+      <c r="Y1" s="102"/>
+      <c r="Z1" s="101" t="s">
         <v>64</v>
       </c>
-      <c r="AA1" s="29"/>
-      <c r="AB1" s="28" t="s">
+      <c r="AA1" s="102"/>
+      <c r="AB1" s="101" t="s">
         <v>66</v>
       </c>
-      <c r="AC1" s="29"/>
-      <c r="AD1" s="28" t="s">
+      <c r="AC1" s="102"/>
+      <c r="AD1" s="101" t="s">
         <v>67</v>
       </c>
-      <c r="AE1" s="29"/>
-      <c r="AF1" s="28" t="s">
+      <c r="AE1" s="102"/>
+      <c r="AF1" s="101" t="s">
         <v>68</v>
       </c>
-      <c r="AG1" s="29"/>
-      <c r="AH1" s="28" t="s">
+      <c r="AG1" s="102"/>
+      <c r="AH1" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="AI1" s="29"/>
-      <c r="AJ1" s="28" t="s">
+      <c r="AI1" s="102"/>
+      <c r="AJ1" s="101" t="s">
         <v>70</v>
       </c>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="28" t="s">
+      <c r="AK1" s="102"/>
+      <c r="AL1" s="101" t="s">
         <v>71</v>
       </c>
-      <c r="AM1" s="29"/>
-      <c r="AN1" s="28" t="s">
+      <c r="AM1" s="102"/>
+      <c r="AN1" s="101" t="s">
         <v>73</v>
       </c>
-      <c r="AO1" s="29"/>
-      <c r="AP1" s="28" t="s">
+      <c r="AO1" s="102"/>
+      <c r="AP1" s="101" t="s">
         <v>74</v>
       </c>
-      <c r="AQ1" s="29"/>
-      <c r="AR1" s="28" t="s">
+      <c r="AQ1" s="102"/>
+      <c r="AR1" s="101" t="s">
         <v>77</v>
       </c>
-      <c r="AS1" s="29"/>
-      <c r="AT1" s="34" t="s">
+      <c r="AS1" s="102"/>
+      <c r="AT1" s="125" t="s">
         <v>2</v>
       </c>
-      <c r="AU1" s="42" t="s">
+      <c r="AU1" s="127" t="s">
         <v>65</v>
       </c>
-      <c r="AV1" s="43"/>
-      <c r="AW1" s="43"/>
-      <c r="AX1" s="43"/>
-      <c r="AY1" s="44"/>
-      <c r="AZ1" s="45" t="s">
+      <c r="AV1" s="128"/>
+      <c r="AW1" s="128"/>
+      <c r="AX1" s="128"/>
+      <c r="AY1" s="129"/>
+      <c r="AZ1" s="114" t="s">
         <v>57</v>
       </c>
-      <c r="BA1" s="46"/>
-      <c r="BB1" s="46"/>
-      <c r="BC1" s="46"/>
-      <c r="BD1" s="47"/>
+      <c r="BA1" s="115"/>
+      <c r="BB1" s="115"/>
+      <c r="BC1" s="115"/>
+      <c r="BD1" s="116"/>
     </row>
     <row r="2" spans="1:56" s="14" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="30">
+      <c r="A2" s="107"/>
+      <c r="B2" s="108"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="103">
         <v>45782</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="30">
+      <c r="E2" s="104"/>
+      <c r="F2" s="103">
         <v>45789</v>
       </c>
-      <c r="G2" s="31"/>
-      <c r="H2" s="30">
+      <c r="G2" s="104"/>
+      <c r="H2" s="103">
         <v>45796</v>
       </c>
-      <c r="I2" s="31"/>
-      <c r="J2" s="30">
+      <c r="I2" s="104"/>
+      <c r="J2" s="103">
         <v>45803</v>
       </c>
-      <c r="K2" s="31"/>
-      <c r="L2" s="30">
+      <c r="K2" s="104"/>
+      <c r="L2" s="103">
         <v>45810</v>
       </c>
-      <c r="M2" s="31"/>
-      <c r="N2" s="30">
+      <c r="M2" s="104"/>
+      <c r="N2" s="103">
         <v>45817</v>
       </c>
-      <c r="O2" s="31"/>
-      <c r="P2" s="30">
+      <c r="O2" s="104"/>
+      <c r="P2" s="103">
         <v>45824</v>
       </c>
-      <c r="Q2" s="31"/>
-      <c r="R2" s="30">
+      <c r="Q2" s="104"/>
+      <c r="R2" s="103">
         <v>45831</v>
       </c>
-      <c r="S2" s="31"/>
-      <c r="T2" s="30">
+      <c r="S2" s="104"/>
+      <c r="T2" s="103">
         <v>45838</v>
       </c>
-      <c r="U2" s="31"/>
-      <c r="V2" s="30">
+      <c r="U2" s="104"/>
+      <c r="V2" s="103">
         <v>45845</v>
       </c>
-      <c r="W2" s="31"/>
-      <c r="X2" s="30">
+      <c r="W2" s="104"/>
+      <c r="X2" s="103">
         <v>45852</v>
       </c>
-      <c r="Y2" s="31"/>
-      <c r="Z2" s="30">
+      <c r="Y2" s="104"/>
+      <c r="Z2" s="103">
         <v>45859</v>
       </c>
-      <c r="AA2" s="31"/>
-      <c r="AB2" s="30">
+      <c r="AA2" s="104"/>
+      <c r="AB2" s="103">
         <v>45866</v>
       </c>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="30">
+      <c r="AC2" s="104"/>
+      <c r="AD2" s="103">
         <v>45873</v>
       </c>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="30">
+      <c r="AE2" s="104"/>
+      <c r="AF2" s="103">
         <v>45880</v>
       </c>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="30">
+      <c r="AG2" s="104"/>
+      <c r="AH2" s="103">
         <v>45887</v>
       </c>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="30">
+      <c r="AI2" s="104"/>
+      <c r="AJ2" s="103">
         <v>45894</v>
       </c>
-      <c r="AK2" s="31"/>
-      <c r="AL2" s="30">
+      <c r="AK2" s="104"/>
+      <c r="AL2" s="103">
         <v>45901</v>
       </c>
-      <c r="AM2" s="31"/>
-      <c r="AN2" s="30">
+      <c r="AM2" s="104"/>
+      <c r="AN2" s="103">
         <v>45908</v>
       </c>
-      <c r="AO2" s="31"/>
-      <c r="AP2" s="30">
+      <c r="AO2" s="104"/>
+      <c r="AP2" s="103">
         <v>45915</v>
       </c>
-      <c r="AQ2" s="31"/>
-      <c r="AR2" s="30">
+      <c r="AQ2" s="104"/>
+      <c r="AR2" s="103">
         <v>45922</v>
       </c>
-      <c r="AS2" s="31"/>
-      <c r="AT2" s="35"/>
-      <c r="AU2" s="34" t="s">
+      <c r="AS2" s="104"/>
+      <c r="AT2" s="126"/>
+      <c r="AU2" s="125" t="s">
         <v>3</v>
       </c>
-      <c r="AV2" s="38" t="s">
+      <c r="AV2" s="121" t="s">
         <v>4</v>
       </c>
-      <c r="AW2" s="40" t="s">
+      <c r="AW2" s="123" t="s">
         <v>5</v>
       </c>
-      <c r="AX2" s="32" t="s">
+      <c r="AX2" s="130" t="s">
         <v>6</v>
       </c>
-      <c r="AY2" s="36" t="s">
+      <c r="AY2" s="119" t="s">
         <v>76</v>
       </c>
-      <c r="AZ2" s="48" t="s">
+      <c r="AZ2" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="BA2" s="48" t="s">
+      <c r="BA2" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="BB2" s="48" t="s">
+      <c r="BB2" s="117" t="s">
         <v>5</v>
       </c>
-      <c r="BC2" s="48" t="s">
+      <c r="BC2" s="117" t="s">
         <v>6</v>
       </c>
-      <c r="BD2" s="48" t="s">
+      <c r="BD2" s="117" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:56" s="27" customFormat="1" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="54"/>
-      <c r="B3" s="55"/>
-      <c r="C3" s="58"/>
+      <c r="A3" s="109"/>
+      <c r="B3" s="110"/>
+      <c r="C3" s="113"/>
       <c r="D3" s="25" t="s">
         <v>8</v>
       </c>
@@ -2209,111 +2209,111 @@
       <c r="AS3" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="AT3" s="35"/>
-      <c r="AU3" s="35"/>
-      <c r="AV3" s="39"/>
-      <c r="AW3" s="41"/>
-      <c r="AX3" s="33"/>
-      <c r="AY3" s="37"/>
-      <c r="AZ3" s="49"/>
-      <c r="BA3" s="49"/>
-      <c r="BB3" s="49"/>
-      <c r="BC3" s="49"/>
-      <c r="BD3" s="49"/>
+      <c r="AT3" s="126"/>
+      <c r="AU3" s="126"/>
+      <c r="AV3" s="122"/>
+      <c r="AW3" s="124"/>
+      <c r="AX3" s="131"/>
+      <c r="AY3" s="120"/>
+      <c r="AZ3" s="118"/>
+      <c r="BA3" s="118"/>
+      <c r="BB3" s="118"/>
+      <c r="BC3" s="118"/>
+      <c r="BD3" s="118"/>
     </row>
     <row r="4" spans="1:56" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="61" t="s">
+      <c r="B4" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="62">
-        <f>ROUND((AT4-(36*AU4))/AU4,0)</f>
+      <c r="C4" s="31">
+        <f t="shared" ref="C4:C20" si="0">ROUND((AT4-(36*AU4))/AU4,0)</f>
         <v>17</v>
       </c>
-      <c r="D4" s="63"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="65">
+      <c r="D4" s="32"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="34">
         <v>53</v>
       </c>
-      <c r="G4" s="66">
+      <c r="G4" s="35">
         <v>23</v>
       </c>
-      <c r="H4" s="63"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="65"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="66"/>
-      <c r="N4" s="65">
+      <c r="H4" s="32"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="34">
         <v>57</v>
       </c>
-      <c r="O4" s="66">
+      <c r="O4" s="35">
         <v>19</v>
       </c>
-      <c r="P4" s="65"/>
-      <c r="Q4" s="66"/>
-      <c r="R4" s="65">
+      <c r="P4" s="34"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="34">
         <v>50</v>
       </c>
-      <c r="S4" s="66">
+      <c r="S4" s="35">
         <v>26</v>
       </c>
-      <c r="T4" s="65">
+      <c r="T4" s="34">
         <v>56</v>
       </c>
-      <c r="U4" s="66">
+      <c r="U4" s="35">
         <v>15</v>
       </c>
-      <c r="V4" s="65"/>
-      <c r="W4" s="66"/>
-      <c r="X4" s="65"/>
-      <c r="Y4" s="66"/>
-      <c r="Z4" s="65">
+      <c r="V4" s="34"/>
+      <c r="W4" s="35"/>
+      <c r="X4" s="34"/>
+      <c r="Y4" s="35"/>
+      <c r="Z4" s="34">
         <v>54</v>
       </c>
-      <c r="AA4" s="66">
+      <c r="AA4" s="35">
         <v>18</v>
       </c>
-      <c r="AB4" s="65">
+      <c r="AB4" s="34">
         <v>50</v>
       </c>
-      <c r="AC4" s="66">
+      <c r="AC4" s="35">
         <v>22</v>
       </c>
-      <c r="AD4" s="67"/>
-      <c r="AE4" s="68"/>
-      <c r="AF4" s="67"/>
-      <c r="AG4" s="68"/>
-      <c r="AH4" s="67"/>
-      <c r="AI4" s="68"/>
-      <c r="AJ4" s="63"/>
-      <c r="AK4" s="64"/>
-      <c r="AL4" s="67"/>
-      <c r="AM4" s="68"/>
-      <c r="AN4" s="63"/>
-      <c r="AO4" s="69"/>
-      <c r="AP4" s="67"/>
-      <c r="AQ4" s="70"/>
-      <c r="AR4" s="67"/>
-      <c r="AS4" s="70"/>
-      <c r="AT4" s="71">
-        <f>F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4+AJ4+AL4+AN4+AP4+AR4</f>
+      <c r="AD4" s="36"/>
+      <c r="AE4" s="37"/>
+      <c r="AF4" s="36"/>
+      <c r="AG4" s="37"/>
+      <c r="AH4" s="36"/>
+      <c r="AI4" s="37"/>
+      <c r="AJ4" s="32"/>
+      <c r="AK4" s="33"/>
+      <c r="AL4" s="36"/>
+      <c r="AM4" s="37"/>
+      <c r="AN4" s="32"/>
+      <c r="AO4" s="38"/>
+      <c r="AP4" s="36"/>
+      <c r="AQ4" s="39"/>
+      <c r="AR4" s="36"/>
+      <c r="AS4" s="39"/>
+      <c r="AT4" s="40">
+        <f t="shared" ref="AT4:AT26" si="1">F4+J4+L4+N4+P4+R4+T4+V4+X4+Z4+AB4+AD4+AF4+AH4+AJ4+AL4+AN4+AP4+AR4</f>
         <v>320</v>
       </c>
-      <c r="AU4" s="72">
-        <f>COUNTIF(D4:AR4,"&gt;30")</f>
+      <c r="AU4" s="41">
+        <f t="shared" ref="AU4:AU26" si="2">COUNTIF(D4:AR4,"&gt;30")</f>
         <v>6</v>
       </c>
-      <c r="AV4" s="73"/>
-      <c r="AW4" s="74"/>
-      <c r="AX4" s="75">
-        <f>SUMIF(G4:AS4, "&lt;30")+AV4+AW4</f>
+      <c r="AV4" s="42"/>
+      <c r="AW4" s="43"/>
+      <c r="AX4" s="44">
+        <f t="shared" ref="AX4:AX26" si="3">SUMIF(G4:AS4, "&lt;30")+AV4+AW4</f>
         <v>123</v>
       </c>
-      <c r="AY4" s="76">
-        <f>AX4/AU4</f>
+      <c r="AY4" s="45">
+        <f t="shared" ref="AY4:AY26" si="4">AX4/AU4</f>
         <v>20.5</v>
       </c>
       <c r="AZ4" s="19"/>
@@ -2325,118 +2325,118 @@
       </c>
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="78" t="s">
+      <c r="B5" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="79">
-        <f>ROUND((AT5-(36*AU5))/AU5,0)</f>
+      <c r="C5" s="48">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="D5" s="80"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="82"/>
-      <c r="G5" s="83"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="82"/>
-      <c r="K5" s="83"/>
-      <c r="L5" s="82"/>
-      <c r="M5" s="83"/>
-      <c r="N5" s="82"/>
-      <c r="O5" s="83"/>
-      <c r="P5" s="82">
+      <c r="D5" s="49"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="50"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="52"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="52"/>
+      <c r="N5" s="51"/>
+      <c r="O5" s="52"/>
+      <c r="P5" s="51">
         <v>39</v>
       </c>
-      <c r="Q5" s="83">
+      <c r="Q5" s="52">
         <v>17</v>
       </c>
-      <c r="R5" s="82">
+      <c r="R5" s="51">
         <v>38</v>
       </c>
-      <c r="S5" s="83">
+      <c r="S5" s="52">
         <v>18</v>
       </c>
-      <c r="T5" s="82"/>
-      <c r="U5" s="83"/>
-      <c r="V5" s="82">
+      <c r="T5" s="51"/>
+      <c r="U5" s="52"/>
+      <c r="V5" s="51">
         <v>37</v>
       </c>
-      <c r="W5" s="83">
+      <c r="W5" s="52">
         <v>19</v>
       </c>
-      <c r="X5" s="82">
+      <c r="X5" s="51">
         <v>36</v>
       </c>
-      <c r="Y5" s="83">
+      <c r="Y5" s="52">
         <v>20</v>
       </c>
-      <c r="Z5" s="82">
+      <c r="Z5" s="51">
         <v>38</v>
       </c>
-      <c r="AA5" s="83">
+      <c r="AA5" s="52">
         <v>18</v>
       </c>
-      <c r="AB5" s="82">
+      <c r="AB5" s="51">
         <v>35</v>
       </c>
-      <c r="AC5" s="83">
+      <c r="AC5" s="52">
         <v>21</v>
       </c>
-      <c r="AD5" s="84">
+      <c r="AD5" s="53">
         <v>37</v>
       </c>
-      <c r="AE5" s="85">
+      <c r="AE5" s="54">
         <v>19</v>
       </c>
-      <c r="AF5" s="84">
+      <c r="AF5" s="53">
         <v>37</v>
       </c>
-      <c r="AG5" s="85">
+      <c r="AG5" s="54">
         <v>18</v>
       </c>
-      <c r="AH5" s="84">
+      <c r="AH5" s="53">
         <v>38</v>
       </c>
-      <c r="AI5" s="85">
+      <c r="AI5" s="54">
         <v>17</v>
       </c>
-      <c r="AJ5" s="80"/>
-      <c r="AK5" s="81"/>
-      <c r="AL5" s="84"/>
-      <c r="AM5" s="85"/>
-      <c r="AN5" s="80"/>
-      <c r="AO5" s="86"/>
-      <c r="AP5" s="87">
+      <c r="AJ5" s="49"/>
+      <c r="AK5" s="50"/>
+      <c r="AL5" s="53"/>
+      <c r="AM5" s="54"/>
+      <c r="AN5" s="49"/>
+      <c r="AO5" s="55"/>
+      <c r="AP5" s="56">
         <v>35</v>
       </c>
-      <c r="AQ5" s="88">
+      <c r="AQ5" s="57">
         <v>20</v>
       </c>
-      <c r="AR5" s="84"/>
-      <c r="AS5" s="88"/>
-      <c r="AT5" s="89">
-        <f>F5+J5+L5+N5+P5+R5+T5+V5+X5+Z5+AB5+AD5+AF5+AH5+AJ5+AL5+AN5+AP5+AR5</f>
+      <c r="AR5" s="53"/>
+      <c r="AS5" s="57"/>
+      <c r="AT5" s="58">
+        <f t="shared" si="1"/>
         <v>370</v>
       </c>
-      <c r="AU5" s="90">
-        <f>COUNTIF(D5:AR5,"&gt;30")</f>
+      <c r="AU5" s="59">
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="AV5" s="91">
+      <c r="AV5" s="60">
         <v>3</v>
       </c>
-      <c r="AW5" s="92">
+      <c r="AW5" s="61">
         <v>13</v>
       </c>
-      <c r="AX5" s="93">
-        <f>SUMIF(G5:AS5, "&lt;30")+AV5+AW5</f>
+      <c r="AX5" s="62">
+        <f t="shared" si="3"/>
         <v>203</v>
       </c>
-      <c r="AY5" s="94">
-        <f>AX5/AU5</f>
+      <c r="AY5" s="63">
+        <f t="shared" si="4"/>
         <v>20.3</v>
       </c>
       <c r="AZ5" s="16"/>
@@ -2446,110 +2446,110 @@
       <c r="BD5" s="17"/>
     </row>
     <row r="6" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A6" s="77" t="s">
+      <c r="A6" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="78" t="s">
+      <c r="B6" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="79">
-        <f>ROUND((AT6-(36*AU6))/AU6,0)</f>
+      <c r="C6" s="48">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D6" s="80"/>
-      <c r="E6" s="81"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="83"/>
-      <c r="H6" s="80"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="95"/>
-      <c r="K6" s="83"/>
-      <c r="L6" s="95"/>
-      <c r="M6" s="83"/>
-      <c r="N6" s="95"/>
-      <c r="O6" s="83"/>
-      <c r="P6" s="95">
+      <c r="D6" s="49"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="50"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="52"/>
+      <c r="L6" s="64"/>
+      <c r="M6" s="52"/>
+      <c r="N6" s="64"/>
+      <c r="O6" s="52"/>
+      <c r="P6" s="64">
         <v>43</v>
       </c>
-      <c r="Q6" s="83">
+      <c r="Q6" s="52">
         <v>26</v>
       </c>
-      <c r="R6" s="95">
+      <c r="R6" s="64">
         <v>45</v>
       </c>
-      <c r="S6" s="83">
+      <c r="S6" s="52">
         <v>24</v>
       </c>
-      <c r="T6" s="95"/>
-      <c r="U6" s="83"/>
-      <c r="V6" s="95">
+      <c r="T6" s="64"/>
+      <c r="U6" s="52"/>
+      <c r="V6" s="64">
         <v>50</v>
       </c>
-      <c r="W6" s="83">
+      <c r="W6" s="52">
         <v>19</v>
       </c>
-      <c r="X6" s="95">
+      <c r="X6" s="64">
         <v>44</v>
       </c>
-      <c r="Y6" s="83">
+      <c r="Y6" s="52">
         <v>20</v>
       </c>
-      <c r="Z6" s="95"/>
-      <c r="AA6" s="83"/>
-      <c r="AB6" s="95">
+      <c r="Z6" s="64"/>
+      <c r="AA6" s="52"/>
+      <c r="AB6" s="64">
         <v>54</v>
       </c>
-      <c r="AC6" s="83">
+      <c r="AC6" s="52">
         <v>11</v>
       </c>
-      <c r="AD6" s="96"/>
-      <c r="AE6" s="85"/>
-      <c r="AF6" s="96">
+      <c r="AD6" s="65"/>
+      <c r="AE6" s="54"/>
+      <c r="AF6" s="65">
         <v>51</v>
       </c>
-      <c r="AG6" s="85">
+      <c r="AG6" s="54">
         <v>14</v>
       </c>
-      <c r="AH6" s="96"/>
-      <c r="AI6" s="85"/>
-      <c r="AJ6" s="80"/>
-      <c r="AK6" s="81"/>
-      <c r="AL6" s="97">
+      <c r="AH6" s="65"/>
+      <c r="AI6" s="54"/>
+      <c r="AJ6" s="49"/>
+      <c r="AK6" s="50"/>
+      <c r="AL6" s="66">
         <v>46</v>
       </c>
-      <c r="AM6" s="85">
+      <c r="AM6" s="54">
         <v>20</v>
       </c>
-      <c r="AN6" s="80"/>
-      <c r="AO6" s="86"/>
-      <c r="AP6" s="98"/>
-      <c r="AQ6" s="88"/>
-      <c r="AR6" s="98">
+      <c r="AN6" s="49"/>
+      <c r="AO6" s="55"/>
+      <c r="AP6" s="67"/>
+      <c r="AQ6" s="57"/>
+      <c r="AR6" s="67">
         <v>42</v>
       </c>
-      <c r="AS6" s="88">
+      <c r="AS6" s="57">
         <v>24</v>
       </c>
-      <c r="AT6" s="89">
-        <f>F6+J6+L6+N6+P6+R6+T6+V6+X6+Z6+AB6+AD6+AF6+AH6+AJ6+AL6+AN6+AP6+AR6</f>
+      <c r="AT6" s="58">
+        <f t="shared" si="1"/>
         <v>375</v>
       </c>
-      <c r="AU6" s="90">
-        <f>COUNTIF(D6:AR6,"&gt;30")</f>
+      <c r="AU6" s="59">
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="AV6" s="91">
+      <c r="AV6" s="60">
         <v>2</v>
       </c>
-      <c r="AW6" s="92">
+      <c r="AW6" s="61">
         <v>1</v>
       </c>
-      <c r="AX6" s="93">
-        <f>SUMIF(G6:AS6, "&lt;30")+AV6+AW6</f>
+      <c r="AX6" s="62">
+        <f t="shared" si="3"/>
         <v>161</v>
       </c>
-      <c r="AY6" s="94">
-        <f>AX6/AU6</f>
+      <c r="AY6" s="63">
+        <f t="shared" si="4"/>
         <v>20.125</v>
       </c>
       <c r="AZ6" s="18"/>
@@ -2559,122 +2559,122 @@
       <c r="BD6" s="17"/>
     </row>
     <row r="7" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A7" s="77" t="s">
+      <c r="A7" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="78" t="s">
+      <c r="B7" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="79">
-        <f>ROUND((AT7-(36*AU7))/AU7,0)</f>
+      <c r="C7" s="48">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D7" s="80"/>
-      <c r="E7" s="81"/>
-      <c r="F7" s="95">
+      <c r="D7" s="49"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="64">
         <v>41</v>
       </c>
-      <c r="G7" s="83">
+      <c r="G7" s="52">
         <v>21</v>
       </c>
-      <c r="H7" s="80"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="95"/>
-      <c r="K7" s="83"/>
-      <c r="L7" s="95"/>
-      <c r="M7" s="83"/>
-      <c r="N7" s="95">
+      <c r="H7" s="49"/>
+      <c r="I7" s="50"/>
+      <c r="J7" s="64"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="64"/>
+      <c r="M7" s="52"/>
+      <c r="N7" s="64">
         <v>48</v>
       </c>
-      <c r="O7" s="83">
+      <c r="O7" s="52">
         <v>14</v>
       </c>
-      <c r="P7" s="95">
+      <c r="P7" s="64">
         <v>44</v>
       </c>
-      <c r="Q7" s="83">
+      <c r="Q7" s="52">
         <v>18</v>
       </c>
-      <c r="R7" s="95"/>
-      <c r="S7" s="83"/>
-      <c r="T7" s="95"/>
-      <c r="U7" s="83"/>
-      <c r="V7" s="95"/>
-      <c r="W7" s="83"/>
-      <c r="X7" s="95">
+      <c r="R7" s="64"/>
+      <c r="S7" s="52"/>
+      <c r="T7" s="64"/>
+      <c r="U7" s="52"/>
+      <c r="V7" s="64"/>
+      <c r="W7" s="52"/>
+      <c r="X7" s="64">
         <v>40</v>
       </c>
-      <c r="Y7" s="83">
+      <c r="Y7" s="52">
         <v>22</v>
       </c>
-      <c r="Z7" s="95">
+      <c r="Z7" s="64">
         <v>44</v>
       </c>
-      <c r="AA7" s="83">
+      <c r="AA7" s="52">
         <v>17</v>
       </c>
-      <c r="AB7" s="95">
+      <c r="AB7" s="64">
         <v>46</v>
       </c>
-      <c r="AC7" s="83">
+      <c r="AC7" s="52">
         <v>16</v>
       </c>
-      <c r="AD7" s="99">
+      <c r="AD7" s="68">
         <v>42</v>
       </c>
-      <c r="AE7" s="85">
+      <c r="AE7" s="54">
         <v>20</v>
       </c>
-      <c r="AF7" s="100">
+      <c r="AF7" s="69">
         <v>44</v>
       </c>
-      <c r="AG7" s="85">
+      <c r="AG7" s="54">
         <v>18</v>
       </c>
-      <c r="AH7" s="99">
+      <c r="AH7" s="68">
         <v>39</v>
       </c>
-      <c r="AI7" s="85">
+      <c r="AI7" s="54">
         <v>23</v>
       </c>
-      <c r="AJ7" s="80"/>
-      <c r="AK7" s="81"/>
-      <c r="AL7" s="99"/>
-      <c r="AM7" s="85"/>
-      <c r="AN7" s="80"/>
-      <c r="AO7" s="86"/>
-      <c r="AP7" s="100">
+      <c r="AJ7" s="49"/>
+      <c r="AK7" s="50"/>
+      <c r="AL7" s="68"/>
+      <c r="AM7" s="54"/>
+      <c r="AN7" s="49"/>
+      <c r="AO7" s="55"/>
+      <c r="AP7" s="69">
         <v>41</v>
       </c>
-      <c r="AQ7" s="88">
+      <c r="AQ7" s="57">
         <v>20</v>
       </c>
-      <c r="AR7" s="100">
+      <c r="AR7" s="69">
         <v>38</v>
       </c>
-      <c r="AS7" s="88">
+      <c r="AS7" s="57">
         <v>23</v>
       </c>
-      <c r="AT7" s="89">
-        <f>F7+J7+L7+N7+P7+R7+T7+V7+X7+Z7+AB7+AD7+AF7+AH7+AJ7+AL7+AN7+AP7+AR7</f>
+      <c r="AT7" s="58">
+        <f t="shared" si="1"/>
         <v>467</v>
       </c>
-      <c r="AU7" s="90">
-        <f>COUNTIF(D7:AR7,"&gt;30")</f>
+      <c r="AU7" s="59">
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AV7" s="91">
+      <c r="AV7" s="60">
         <v>3</v>
       </c>
-      <c r="AW7" s="92">
+      <c r="AW7" s="61">
         <v>3</v>
       </c>
-      <c r="AX7" s="93">
-        <f>SUMIF(G7:AS7, "&lt;30")+AV7+AW7</f>
+      <c r="AX7" s="62">
+        <f t="shared" si="3"/>
         <v>218</v>
       </c>
-      <c r="AY7" s="94">
-        <f>AX7/AU7</f>
+      <c r="AY7" s="63">
+        <f t="shared" si="4"/>
         <v>19.818181818181817</v>
       </c>
       <c r="AZ7" s="18"/>
@@ -2684,275 +2684,275 @@
       <c r="BD7" s="17"/>
     </row>
     <row r="8" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A8" s="77" t="s">
+      <c r="A8" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="78" t="s">
+      <c r="B8" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="79">
-        <f>ROUND((AT8-(36*AU8))/AU8,0)</f>
+      <c r="C8" s="48">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D8" s="80"/>
-      <c r="E8" s="81"/>
-      <c r="F8" s="96">
+      <c r="D8" s="49"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="65">
         <v>45</v>
       </c>
-      <c r="G8" s="83">
+      <c r="G8" s="52">
         <v>17</v>
       </c>
-      <c r="H8" s="80"/>
-      <c r="I8" s="81"/>
-      <c r="J8" s="96"/>
-      <c r="K8" s="83"/>
-      <c r="L8" s="96">
+      <c r="H8" s="49"/>
+      <c r="I8" s="50"/>
+      <c r="J8" s="65"/>
+      <c r="K8" s="52"/>
+      <c r="L8" s="65">
         <v>43</v>
       </c>
-      <c r="M8" s="83">
+      <c r="M8" s="52">
         <v>19</v>
       </c>
-      <c r="N8" s="96">
+      <c r="N8" s="65">
         <v>41</v>
       </c>
-      <c r="O8" s="83">
+      <c r="O8" s="52">
         <v>21</v>
       </c>
-      <c r="P8" s="96">
+      <c r="P8" s="65">
         <v>47</v>
       </c>
-      <c r="Q8" s="83">
+      <c r="Q8" s="52">
         <v>15</v>
       </c>
-      <c r="R8" s="96">
+      <c r="R8" s="65">
         <v>42</v>
       </c>
-      <c r="S8" s="83">
+      <c r="S8" s="52">
         <v>20</v>
       </c>
-      <c r="T8" s="96">
+      <c r="T8" s="65">
         <v>43</v>
       </c>
-      <c r="U8" s="83">
+      <c r="U8" s="52">
         <v>19</v>
       </c>
-      <c r="V8" s="96">
+      <c r="V8" s="65">
         <v>44</v>
       </c>
-      <c r="W8" s="83">
+      <c r="W8" s="52">
         <v>18</v>
       </c>
-      <c r="X8" s="96">
+      <c r="X8" s="65">
         <v>48</v>
       </c>
-      <c r="Y8" s="83">
+      <c r="Y8" s="52">
         <v>16</v>
       </c>
-      <c r="Z8" s="96">
+      <c r="Z8" s="65">
         <v>40</v>
       </c>
-      <c r="AA8" s="83">
+      <c r="AA8" s="52">
         <v>22</v>
       </c>
-      <c r="AB8" s="96">
+      <c r="AB8" s="65">
         <v>40</v>
       </c>
-      <c r="AC8" s="83">
+      <c r="AC8" s="52">
         <v>22</v>
       </c>
-      <c r="AD8" s="96">
+      <c r="AD8" s="65">
         <v>38</v>
       </c>
-      <c r="AE8" s="85">
+      <c r="AE8" s="54">
         <v>23</v>
       </c>
-      <c r="AF8" s="101">
+      <c r="AF8" s="70">
         <v>41</v>
       </c>
-      <c r="AG8" s="85">
+      <c r="AG8" s="54">
         <v>20</v>
       </c>
-      <c r="AH8" s="96">
+      <c r="AH8" s="65">
         <v>40</v>
       </c>
-      <c r="AI8" s="85">
+      <c r="AI8" s="54">
         <v>21</v>
       </c>
-      <c r="AJ8" s="80"/>
-      <c r="AK8" s="81"/>
-      <c r="AL8" s="96"/>
-      <c r="AM8" s="85"/>
-      <c r="AN8" s="80"/>
-      <c r="AO8" s="86"/>
-      <c r="AP8" s="96">
+      <c r="AJ8" s="49"/>
+      <c r="AK8" s="50"/>
+      <c r="AL8" s="65"/>
+      <c r="AM8" s="54"/>
+      <c r="AN8" s="49"/>
+      <c r="AO8" s="55"/>
+      <c r="AP8" s="65">
         <v>43</v>
       </c>
-      <c r="AQ8" s="88">
+      <c r="AQ8" s="57">
         <v>17</v>
       </c>
-      <c r="AR8" s="96">
+      <c r="AR8" s="65">
         <v>43</v>
       </c>
-      <c r="AS8" s="88">
+      <c r="AS8" s="57">
         <v>18</v>
       </c>
-      <c r="AT8" s="89">
-        <f>F8+J8+L8+N8+P8+R8+T8+V8+X8+Z8+AB8+AD8+AF8+AH8+AJ8+AL8+AN8+AP8+AR8</f>
+      <c r="AT8" s="58">
+        <f t="shared" si="1"/>
         <v>638</v>
       </c>
-      <c r="AU8" s="90">
-        <f>COUNTIF(D8:AR8,"&gt;30")</f>
+      <c r="AU8" s="59">
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="AV8" s="91">
+      <c r="AV8" s="60">
         <v>2</v>
       </c>
-      <c r="AW8" s="92">
+      <c r="AW8" s="61">
         <v>6</v>
       </c>
-      <c r="AX8" s="93">
-        <f>SUMIF(G8:AS8, "&lt;30")+AV8+AW8</f>
+      <c r="AX8" s="62">
+        <f t="shared" si="3"/>
         <v>296</v>
       </c>
-      <c r="AY8" s="94">
-        <f>AX8/AU8</f>
+      <c r="AY8" s="63">
+        <f t="shared" si="4"/>
         <v>19.733333333333334</v>
       </c>
-      <c r="AZ8" s="59"/>
+      <c r="AZ8" s="28"/>
       <c r="BA8" s="10"/>
       <c r="BB8" s="10"/>
       <c r="BC8" s="2"/>
       <c r="BD8" s="17"/>
     </row>
     <row r="9" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A9" s="77" t="s">
+      <c r="A9" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="78" t="s">
+      <c r="B9" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="79">
-        <f>ROUND((AT9-(36*AU9))/AU9,0)</f>
+      <c r="C9" s="48">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D9" s="80"/>
-      <c r="E9" s="81"/>
-      <c r="F9" s="95"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="80"/>
-      <c r="I9" s="81"/>
-      <c r="J9" s="95">
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="64">
         <v>52</v>
       </c>
-      <c r="K9" s="83">
+      <c r="K9" s="52">
         <v>17</v>
       </c>
-      <c r="L9" s="95"/>
-      <c r="M9" s="83"/>
-      <c r="N9" s="95">
+      <c r="L9" s="64"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="64">
         <v>46</v>
       </c>
-      <c r="O9" s="83">
+      <c r="O9" s="52">
         <v>23</v>
       </c>
-      <c r="P9" s="95">
+      <c r="P9" s="64">
         <v>46</v>
       </c>
-      <c r="Q9" s="83">
+      <c r="Q9" s="52">
         <v>23</v>
       </c>
-      <c r="R9" s="95">
+      <c r="R9" s="64">
         <v>54</v>
       </c>
-      <c r="S9" s="83">
+      <c r="S9" s="52">
         <v>16</v>
       </c>
-      <c r="T9" s="95">
+      <c r="T9" s="64">
         <v>45</v>
       </c>
-      <c r="U9" s="83">
+      <c r="U9" s="52">
         <v>23</v>
       </c>
-      <c r="V9" s="95">
+      <c r="V9" s="64">
         <v>48</v>
       </c>
-      <c r="W9" s="83">
+      <c r="W9" s="52">
         <v>19</v>
       </c>
-      <c r="X9" s="95">
+      <c r="X9" s="64">
         <v>49</v>
       </c>
-      <c r="Y9" s="83">
+      <c r="Y9" s="52">
         <v>18</v>
       </c>
-      <c r="Z9" s="95"/>
-      <c r="AA9" s="83"/>
-      <c r="AB9" s="95">
+      <c r="Z9" s="64"/>
+      <c r="AA9" s="52"/>
+      <c r="AB9" s="64">
         <v>46</v>
       </c>
-      <c r="AC9" s="83">
+      <c r="AC9" s="52">
         <v>21</v>
       </c>
-      <c r="AD9" s="102">
+      <c r="AD9" s="71">
         <v>43</v>
       </c>
-      <c r="AE9" s="85">
+      <c r="AE9" s="54">
         <v>23</v>
       </c>
-      <c r="AF9" s="96">
+      <c r="AF9" s="65">
         <v>47</v>
       </c>
-      <c r="AG9" s="85">
+      <c r="AG9" s="54">
         <v>19</v>
       </c>
-      <c r="AH9" s="96">
+      <c r="AH9" s="65">
         <v>51</v>
       </c>
-      <c r="AI9" s="85">
+      <c r="AI9" s="54">
         <v>15</v>
       </c>
-      <c r="AJ9" s="80"/>
-      <c r="AK9" s="81"/>
-      <c r="AL9" s="100">
+      <c r="AJ9" s="49"/>
+      <c r="AK9" s="50"/>
+      <c r="AL9" s="69">
         <v>50</v>
       </c>
-      <c r="AM9" s="85">
+      <c r="AM9" s="54">
         <v>16</v>
       </c>
-      <c r="AN9" s="80"/>
-      <c r="AO9" s="86"/>
-      <c r="AP9" s="100">
+      <c r="AN9" s="49"/>
+      <c r="AO9" s="55"/>
+      <c r="AP9" s="69">
         <v>51</v>
       </c>
-      <c r="AQ9" s="88">
+      <c r="AQ9" s="57">
         <v>17</v>
       </c>
-      <c r="AR9" s="100">
+      <c r="AR9" s="69">
         <v>46</v>
       </c>
-      <c r="AS9" s="88">
+      <c r="AS9" s="57">
         <v>20</v>
       </c>
-      <c r="AT9" s="89">
-        <f>F9+J9+L9+N9+P9+R9+T9+V9+X9+Z9+AB9+AD9+AF9+AH9+AJ9+AL9+AN9+AP9+AR9</f>
+      <c r="AT9" s="58">
+        <f t="shared" si="1"/>
         <v>674</v>
       </c>
-      <c r="AU9" s="90">
-        <f>COUNTIF(D9:AR9,"&gt;30")</f>
+      <c r="AU9" s="59">
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="AV9" s="91">
+      <c r="AV9" s="60">
         <v>1</v>
       </c>
-      <c r="AW9" s="92">
+      <c r="AW9" s="61">
         <v>2</v>
       </c>
-      <c r="AX9" s="93">
-        <f>SUMIF(G9:AS9, "&lt;30")+AV9+AW9</f>
+      <c r="AX9" s="62">
+        <f t="shared" si="3"/>
         <v>273</v>
       </c>
-      <c r="AY9" s="94">
-        <f>AX9/AU9</f>
+      <c r="AY9" s="63">
+        <f t="shared" si="4"/>
         <v>19.5</v>
       </c>
       <c r="AZ9" s="16"/>
@@ -2962,138 +2962,138 @@
       <c r="BD9" s="17"/>
     </row>
     <row r="10" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A10" s="77" t="s">
+      <c r="A10" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="78" t="s">
+      <c r="B10" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="79">
-        <f>ROUND((AT10-(36*AU10))/AU10,0)</f>
+      <c r="C10" s="48">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D10" s="80"/>
-      <c r="E10" s="81"/>
-      <c r="F10" s="103">
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="72">
         <v>42</v>
       </c>
-      <c r="G10" s="83">
+      <c r="G10" s="52">
         <v>25</v>
       </c>
-      <c r="H10" s="80"/>
-      <c r="I10" s="81"/>
-      <c r="J10" s="103"/>
-      <c r="K10" s="83"/>
-      <c r="L10" s="103">
+      <c r="H10" s="49"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="72"/>
+      <c r="K10" s="52"/>
+      <c r="L10" s="72">
         <v>51</v>
       </c>
-      <c r="M10" s="83">
+      <c r="M10" s="52">
         <v>16</v>
       </c>
-      <c r="N10" s="103"/>
-      <c r="O10" s="83"/>
-      <c r="P10" s="103">
+      <c r="N10" s="72"/>
+      <c r="O10" s="52"/>
+      <c r="P10" s="72">
         <v>49</v>
       </c>
-      <c r="Q10" s="83">
+      <c r="Q10" s="52">
         <v>18</v>
       </c>
-      <c r="R10" s="103">
+      <c r="R10" s="72">
         <v>46</v>
       </c>
-      <c r="S10" s="83">
+      <c r="S10" s="52">
         <v>21</v>
       </c>
-      <c r="T10" s="103">
+      <c r="T10" s="72">
         <v>45</v>
       </c>
-      <c r="U10" s="83">
+      <c r="U10" s="52">
         <v>20</v>
       </c>
-      <c r="V10" s="103">
+      <c r="V10" s="72">
         <v>46</v>
       </c>
-      <c r="W10" s="83">
+      <c r="W10" s="52">
         <v>19</v>
       </c>
-      <c r="X10" s="103">
+      <c r="X10" s="72">
         <v>53</v>
       </c>
-      <c r="Y10" s="83">
+      <c r="Y10" s="52">
         <v>13</v>
       </c>
-      <c r="Z10" s="103">
+      <c r="Z10" s="72">
         <v>52</v>
       </c>
-      <c r="AA10" s="83">
+      <c r="AA10" s="52">
         <v>13</v>
       </c>
-      <c r="AB10" s="103">
+      <c r="AB10" s="72">
         <v>44</v>
       </c>
-      <c r="AC10" s="83">
+      <c r="AC10" s="52">
         <v>22</v>
       </c>
-      <c r="AD10" s="96">
+      <c r="AD10" s="65">
         <v>42</v>
       </c>
-      <c r="AE10" s="85">
+      <c r="AE10" s="54">
         <v>24</v>
       </c>
-      <c r="AF10" s="96">
+      <c r="AF10" s="65">
         <v>45</v>
       </c>
-      <c r="AG10" s="85">
+      <c r="AG10" s="54">
         <v>20</v>
       </c>
-      <c r="AH10" s="96">
+      <c r="AH10" s="65">
         <v>48</v>
       </c>
-      <c r="AI10" s="85">
+      <c r="AI10" s="54">
         <v>17</v>
       </c>
-      <c r="AJ10" s="80"/>
-      <c r="AK10" s="81"/>
-      <c r="AL10" s="96">
+      <c r="AJ10" s="49"/>
+      <c r="AK10" s="50"/>
+      <c r="AL10" s="65">
         <v>50</v>
       </c>
-      <c r="AM10" s="85">
+      <c r="AM10" s="54">
         <v>15</v>
       </c>
-      <c r="AN10" s="80"/>
-      <c r="AO10" s="86"/>
-      <c r="AP10" s="96">
+      <c r="AN10" s="49"/>
+      <c r="AO10" s="55"/>
+      <c r="AP10" s="65">
         <v>42</v>
       </c>
-      <c r="AQ10" s="88">
+      <c r="AQ10" s="57">
         <v>23</v>
       </c>
-      <c r="AR10" s="96">
+      <c r="AR10" s="65">
         <v>46</v>
       </c>
-      <c r="AS10" s="88">
+      <c r="AS10" s="57">
         <v>20</v>
       </c>
-      <c r="AT10" s="89">
-        <f>F10+J10+L10+N10+P10+R10+T10+V10+X10+Z10+AB10+AD10+AF10+AH10+AJ10+AL10+AN10+AP10+AR10</f>
+      <c r="AT10" s="58">
+        <f t="shared" si="1"/>
         <v>701</v>
       </c>
-      <c r="AU10" s="90">
-        <f>COUNTIF(D10:AR10,"&gt;30")</f>
+      <c r="AU10" s="59">
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="AV10" s="91">
+      <c r="AV10" s="60">
         <v>2</v>
       </c>
-      <c r="AW10" s="92">
+      <c r="AW10" s="61">
         <v>4</v>
       </c>
-      <c r="AX10" s="93">
-        <f>SUMIF(G10:AS10, "&lt;30")+AV10+AW10</f>
+      <c r="AX10" s="62">
+        <f t="shared" si="3"/>
         <v>292</v>
       </c>
-      <c r="AY10" s="94">
-        <f>AX10/AU10</f>
+      <c r="AY10" s="63">
+        <f t="shared" si="4"/>
         <v>19.466666666666665</v>
       </c>
       <c r="AZ10" s="21"/>
@@ -3103,102 +3103,102 @@
       <c r="BD10" s="17"/>
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A11" s="77" t="s">
+      <c r="A11" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="78" t="s">
+      <c r="B11" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="79">
-        <f>ROUND((AT11-(36*AU11))/AU11,0)</f>
+      <c r="C11" s="48">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D11" s="80"/>
-      <c r="E11" s="81"/>
-      <c r="F11" s="95">
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="64">
         <v>51</v>
       </c>
-      <c r="G11" s="83">
+      <c r="G11" s="52">
         <v>18</v>
       </c>
-      <c r="H11" s="80"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="95"/>
-      <c r="K11" s="83"/>
-      <c r="L11" s="95"/>
-      <c r="M11" s="83"/>
-      <c r="N11" s="95">
+      <c r="H11" s="49"/>
+      <c r="I11" s="50"/>
+      <c r="J11" s="64"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="64"/>
+      <c r="M11" s="52"/>
+      <c r="N11" s="64">
         <v>51</v>
       </c>
-      <c r="O11" s="83">
+      <c r="O11" s="52">
         <v>18</v>
       </c>
-      <c r="P11" s="95">
+      <c r="P11" s="64">
         <v>52</v>
       </c>
-      <c r="Q11" s="83">
+      <c r="Q11" s="52">
         <v>17</v>
       </c>
-      <c r="R11" s="95"/>
-      <c r="S11" s="83"/>
-      <c r="T11" s="95"/>
-      <c r="U11" s="83"/>
-      <c r="V11" s="95"/>
-      <c r="W11" s="83"/>
-      <c r="X11" s="95">
+      <c r="R11" s="64"/>
+      <c r="S11" s="52"/>
+      <c r="T11" s="64"/>
+      <c r="U11" s="52"/>
+      <c r="V11" s="64"/>
+      <c r="W11" s="52"/>
+      <c r="X11" s="64">
         <v>48</v>
       </c>
-      <c r="Y11" s="83">
+      <c r="Y11" s="52">
         <v>21</v>
       </c>
-      <c r="Z11" s="95"/>
-      <c r="AA11" s="83"/>
-      <c r="AB11" s="95">
+      <c r="Z11" s="64"/>
+      <c r="AA11" s="52"/>
+      <c r="AB11" s="64">
         <v>51</v>
       </c>
-      <c r="AC11" s="83">
+      <c r="AC11" s="52">
         <v>18</v>
       </c>
-      <c r="AD11" s="96"/>
-      <c r="AE11" s="85"/>
-      <c r="AF11" s="96"/>
-      <c r="AG11" s="85"/>
-      <c r="AH11" s="96"/>
-      <c r="AI11" s="85"/>
-      <c r="AJ11" s="80"/>
-      <c r="AK11" s="81"/>
-      <c r="AL11" s="96"/>
-      <c r="AM11" s="85"/>
-      <c r="AN11" s="80"/>
-      <c r="AO11" s="86"/>
-      <c r="AP11" s="96">
+      <c r="AD11" s="65"/>
+      <c r="AE11" s="54"/>
+      <c r="AF11" s="65"/>
+      <c r="AG11" s="54"/>
+      <c r="AH11" s="65"/>
+      <c r="AI11" s="54"/>
+      <c r="AJ11" s="49"/>
+      <c r="AK11" s="50"/>
+      <c r="AL11" s="65"/>
+      <c r="AM11" s="54"/>
+      <c r="AN11" s="49"/>
+      <c r="AO11" s="55"/>
+      <c r="AP11" s="65">
         <v>51</v>
       </c>
-      <c r="AQ11" s="88">
+      <c r="AQ11" s="57">
         <v>19</v>
       </c>
-      <c r="AR11" s="96">
+      <c r="AR11" s="65">
         <v>47</v>
       </c>
-      <c r="AS11" s="88">
+      <c r="AS11" s="57">
         <v>22</v>
       </c>
-      <c r="AT11" s="89">
-        <f>F11+J11+L11+N11+P11+R11+T11+V11+X11+Z11+AB11+AD11+AF11+AH11+AJ11+AL11+AN11+AP11+AR11</f>
+      <c r="AT11" s="58">
+        <f t="shared" si="1"/>
         <v>351</v>
       </c>
-      <c r="AU11" s="90">
-        <f>COUNTIF(D11:AR11,"&gt;30")</f>
+      <c r="AU11" s="59">
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="AV11" s="91"/>
-      <c r="AW11" s="92"/>
-      <c r="AX11" s="93">
-        <f>SUMIF(G11:AS11, "&lt;30")+AV11+AW11</f>
+      <c r="AV11" s="60"/>
+      <c r="AW11" s="61"/>
+      <c r="AX11" s="62">
+        <f t="shared" si="3"/>
         <v>133</v>
       </c>
-      <c r="AY11" s="94">
-        <f>AX11/AU11</f>
+      <c r="AY11" s="63">
+        <f t="shared" si="4"/>
         <v>19</v>
       </c>
       <c r="AZ11" s="18"/>
@@ -3208,122 +3208,122 @@
       <c r="BD11" s="17"/>
     </row>
     <row r="12" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="78" t="s">
+      <c r="B12" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="79">
-        <f>ROUND((AT12-(36*AU12))/AU12,0)</f>
+      <c r="C12" s="48">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D12" s="80"/>
-      <c r="E12" s="81"/>
-      <c r="F12" s="95">
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="64">
         <v>42</v>
       </c>
-      <c r="G12" s="83">
+      <c r="G12" s="52">
         <v>27</v>
       </c>
-      <c r="H12" s="80"/>
-      <c r="I12" s="81"/>
-      <c r="J12" s="95"/>
-      <c r="K12" s="83"/>
-      <c r="L12" s="95">
+      <c r="H12" s="49"/>
+      <c r="I12" s="50"/>
+      <c r="J12" s="64"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="64">
         <v>54</v>
       </c>
-      <c r="M12" s="83">
+      <c r="M12" s="52">
         <v>15</v>
       </c>
-      <c r="N12" s="95"/>
-      <c r="O12" s="83"/>
-      <c r="P12" s="95">
+      <c r="N12" s="64"/>
+      <c r="O12" s="52"/>
+      <c r="P12" s="64">
         <v>54</v>
       </c>
-      <c r="Q12" s="83">
+      <c r="Q12" s="52">
         <v>16</v>
       </c>
-      <c r="R12" s="95">
+      <c r="R12" s="64">
         <v>53</v>
       </c>
-      <c r="S12" s="83">
+      <c r="S12" s="52">
         <v>16</v>
       </c>
-      <c r="T12" s="95"/>
-      <c r="U12" s="83"/>
-      <c r="V12" s="95">
+      <c r="T12" s="64"/>
+      <c r="U12" s="52"/>
+      <c r="V12" s="64">
         <v>46</v>
       </c>
-      <c r="W12" s="83">
+      <c r="W12" s="52">
         <v>23</v>
       </c>
-      <c r="X12" s="95">
+      <c r="X12" s="64">
         <v>49</v>
       </c>
-      <c r="Y12" s="83">
+      <c r="Y12" s="52">
         <v>19</v>
       </c>
-      <c r="Z12" s="95">
+      <c r="Z12" s="64">
         <v>50</v>
       </c>
-      <c r="AA12" s="83">
+      <c r="AA12" s="52">
         <v>18</v>
       </c>
-      <c r="AB12" s="95"/>
-      <c r="AC12" s="83"/>
-      <c r="AD12" s="96"/>
-      <c r="AE12" s="85"/>
-      <c r="AF12" s="96"/>
-      <c r="AG12" s="85"/>
-      <c r="AH12" s="96">
+      <c r="AB12" s="64"/>
+      <c r="AC12" s="52"/>
+      <c r="AD12" s="65"/>
+      <c r="AE12" s="54"/>
+      <c r="AF12" s="65"/>
+      <c r="AG12" s="54"/>
+      <c r="AH12" s="65">
         <v>50</v>
       </c>
-      <c r="AI12" s="85">
+      <c r="AI12" s="54">
         <v>18</v>
       </c>
-      <c r="AJ12" s="80"/>
-      <c r="AK12" s="81"/>
-      <c r="AL12" s="96">
+      <c r="AJ12" s="49"/>
+      <c r="AK12" s="50"/>
+      <c r="AL12" s="65">
         <v>50</v>
       </c>
-      <c r="AM12" s="85">
+      <c r="AM12" s="54">
         <v>18</v>
       </c>
-      <c r="AN12" s="80"/>
-      <c r="AO12" s="86"/>
-      <c r="AP12" s="96">
+      <c r="AN12" s="49"/>
+      <c r="AO12" s="55"/>
+      <c r="AP12" s="65">
         <v>52</v>
       </c>
-      <c r="AQ12" s="88">
+      <c r="AQ12" s="57">
         <v>16</v>
       </c>
-      <c r="AR12" s="96">
+      <c r="AR12" s="65">
         <v>52</v>
       </c>
-      <c r="AS12" s="88">
+      <c r="AS12" s="57">
         <v>16</v>
       </c>
-      <c r="AT12" s="89">
-        <f>F12+J12+L12+N12+P12+R12+T12+V12+X12+Z12+AB12+AD12+AF12+AH12+AJ12+AL12+AN12+AP12+AR12</f>
+      <c r="AT12" s="58">
+        <f t="shared" si="1"/>
         <v>552</v>
       </c>
-      <c r="AU12" s="90">
-        <f>COUNTIF(D12:AR12,"&gt;30")</f>
+      <c r="AU12" s="59">
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AV12" s="91">
+      <c r="AV12" s="60">
         <v>1</v>
       </c>
-      <c r="AW12" s="92">
+      <c r="AW12" s="61">
         <v>1</v>
       </c>
-      <c r="AX12" s="93">
-        <f>SUMIF(G12:AS12, "&lt;30")+AV12+AW12</f>
+      <c r="AX12" s="62">
+        <f t="shared" si="3"/>
         <v>204</v>
       </c>
-      <c r="AY12" s="94">
-        <f>AX12/AU12</f>
+      <c r="AY12" s="63">
+        <f t="shared" si="4"/>
         <v>18.545454545454547</v>
       </c>
       <c r="AZ12" s="16"/>
@@ -3333,112 +3333,112 @@
       <c r="BD12" s="17"/>
     </row>
     <row r="13" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A13" s="77" t="s">
+      <c r="A13" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="78" t="s">
+      <c r="B13" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="79">
-        <f>ROUND((AT13-(36*AU13))/AU13,0)</f>
+      <c r="C13" s="48">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D13" s="80"/>
-      <c r="E13" s="81"/>
-      <c r="F13" s="95"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="80"/>
-      <c r="I13" s="81"/>
-      <c r="J13" s="95"/>
-      <c r="K13" s="83"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="83"/>
-      <c r="N13" s="95"/>
-      <c r="O13" s="83"/>
-      <c r="P13" s="95">
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="50"/>
+      <c r="J13" s="64"/>
+      <c r="K13" s="52"/>
+      <c r="L13" s="64"/>
+      <c r="M13" s="52"/>
+      <c r="N13" s="64"/>
+      <c r="O13" s="52"/>
+      <c r="P13" s="64">
         <v>48</v>
       </c>
-      <c r="Q13" s="83">
+      <c r="Q13" s="52">
         <v>18</v>
       </c>
-      <c r="R13" s="95">
+      <c r="R13" s="64">
         <v>51</v>
       </c>
-      <c r="S13" s="83">
+      <c r="S13" s="52">
         <v>14</v>
       </c>
-      <c r="T13" s="95">
+      <c r="T13" s="64">
         <v>51</v>
       </c>
-      <c r="U13" s="83">
+      <c r="U13" s="52">
         <v>14</v>
       </c>
-      <c r="V13" s="95"/>
-      <c r="W13" s="83"/>
-      <c r="X13" s="95">
+      <c r="V13" s="64"/>
+      <c r="W13" s="52"/>
+      <c r="X13" s="64">
         <v>48</v>
       </c>
-      <c r="Y13" s="83">
+      <c r="Y13" s="52">
         <v>20</v>
       </c>
-      <c r="Z13" s="95">
+      <c r="Z13" s="64">
         <v>50</v>
       </c>
-      <c r="AA13" s="83">
+      <c r="AA13" s="52">
         <v>18</v>
       </c>
-      <c r="AB13" s="95">
+      <c r="AB13" s="64">
         <v>47</v>
       </c>
-      <c r="AC13" s="83">
+      <c r="AC13" s="52">
         <v>21</v>
       </c>
-      <c r="AD13" s="96"/>
-      <c r="AE13" s="85"/>
-      <c r="AF13" s="96">
+      <c r="AD13" s="65"/>
+      <c r="AE13" s="54"/>
+      <c r="AF13" s="65">
         <v>46</v>
       </c>
-      <c r="AG13" s="85">
+      <c r="AG13" s="54">
         <v>21</v>
       </c>
-      <c r="AH13" s="96">
+      <c r="AH13" s="65">
         <v>48</v>
       </c>
-      <c r="AI13" s="85">
+      <c r="AI13" s="54">
         <v>19</v>
       </c>
-      <c r="AJ13" s="80"/>
-      <c r="AK13" s="81"/>
-      <c r="AL13" s="96"/>
-      <c r="AM13" s="85"/>
-      <c r="AN13" s="80"/>
-      <c r="AO13" s="86"/>
-      <c r="AP13" s="96">
+      <c r="AJ13" s="49"/>
+      <c r="AK13" s="50"/>
+      <c r="AL13" s="65"/>
+      <c r="AM13" s="54"/>
+      <c r="AN13" s="49"/>
+      <c r="AO13" s="55"/>
+      <c r="AP13" s="65">
         <v>47</v>
       </c>
-      <c r="AQ13" s="88">
+      <c r="AQ13" s="57">
         <v>20</v>
       </c>
-      <c r="AR13" s="96"/>
-      <c r="AS13" s="88"/>
-      <c r="AT13" s="89">
-        <f>F13+J13+L13+N13+P13+R13+T13+V13+X13+Z13+AB13+AD13+AF13+AH13+AJ13+AL13+AN13+AP13+AR13</f>
+      <c r="AR13" s="65"/>
+      <c r="AS13" s="57"/>
+      <c r="AT13" s="58">
+        <f t="shared" si="1"/>
         <v>436</v>
       </c>
-      <c r="AU13" s="90">
-        <f>COUNTIF(D13:AR13,"&gt;30")</f>
+      <c r="AU13" s="59">
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="AV13" s="91"/>
-      <c r="AW13" s="92">
+      <c r="AV13" s="60"/>
+      <c r="AW13" s="61">
         <v>1</v>
       </c>
-      <c r="AX13" s="93">
-        <f>SUMIF(G13:AS13, "&lt;30")+AV13+AW13</f>
+      <c r="AX13" s="62">
+        <f t="shared" si="3"/>
         <v>166</v>
       </c>
-      <c r="AY13" s="94">
-        <f>AX13/AU13</f>
+      <c r="AY13" s="63">
+        <f t="shared" si="4"/>
         <v>18.444444444444443</v>
       </c>
       <c r="AZ13" s="16"/>
@@ -3448,86 +3448,86 @@
       <c r="BD13" s="17"/>
     </row>
     <row r="14" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A14" s="77" t="s">
+      <c r="A14" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="78" t="s">
+      <c r="B14" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="79">
-        <f>ROUND((AT14-(36*AU14))/AU14,0)</f>
+      <c r="C14" s="48">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="D14" s="80"/>
-      <c r="E14" s="81"/>
-      <c r="F14" s="95">
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="64">
         <v>59</v>
       </c>
-      <c r="G14" s="83">
+      <c r="G14" s="52">
         <v>17</v>
       </c>
-      <c r="H14" s="80"/>
-      <c r="I14" s="81"/>
-      <c r="J14" s="95"/>
-      <c r="K14" s="83"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="83"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="83"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="83"/>
-      <c r="R14" s="95">
+      <c r="H14" s="49"/>
+      <c r="I14" s="50"/>
+      <c r="J14" s="64"/>
+      <c r="K14" s="52"/>
+      <c r="L14" s="64"/>
+      <c r="M14" s="52"/>
+      <c r="N14" s="64"/>
+      <c r="O14" s="52"/>
+      <c r="P14" s="64"/>
+      <c r="Q14" s="52"/>
+      <c r="R14" s="64">
         <v>55</v>
       </c>
-      <c r="S14" s="83">
+      <c r="S14" s="52">
         <v>21</v>
       </c>
-      <c r="T14" s="95"/>
-      <c r="U14" s="83"/>
-      <c r="V14" s="95">
+      <c r="T14" s="64"/>
+      <c r="U14" s="52"/>
+      <c r="V14" s="64">
         <v>59</v>
       </c>
-      <c r="W14" s="83">
+      <c r="W14" s="52">
         <v>17</v>
       </c>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="83"/>
-      <c r="Z14" s="95"/>
-      <c r="AA14" s="83"/>
-      <c r="AB14" s="95"/>
-      <c r="AC14" s="83"/>
-      <c r="AD14" s="96"/>
-      <c r="AE14" s="85"/>
-      <c r="AF14" s="96"/>
-      <c r="AG14" s="85"/>
-      <c r="AH14" s="96"/>
-      <c r="AI14" s="85"/>
-      <c r="AJ14" s="80"/>
-      <c r="AK14" s="81"/>
-      <c r="AL14" s="96"/>
-      <c r="AM14" s="85"/>
-      <c r="AN14" s="80"/>
-      <c r="AO14" s="86"/>
-      <c r="AP14" s="96"/>
-      <c r="AQ14" s="88"/>
-      <c r="AR14" s="96"/>
-      <c r="AS14" s="88"/>
-      <c r="AT14" s="89">
-        <f>F14+J14+L14+N14+P14+R14+T14+V14+X14+Z14+AB14+AD14+AF14+AH14+AJ14+AL14+AN14+AP14+AR14</f>
+      <c r="X14" s="64"/>
+      <c r="Y14" s="52"/>
+      <c r="Z14" s="64"/>
+      <c r="AA14" s="52"/>
+      <c r="AB14" s="64"/>
+      <c r="AC14" s="52"/>
+      <c r="AD14" s="65"/>
+      <c r="AE14" s="54"/>
+      <c r="AF14" s="65"/>
+      <c r="AG14" s="54"/>
+      <c r="AH14" s="65"/>
+      <c r="AI14" s="54"/>
+      <c r="AJ14" s="49"/>
+      <c r="AK14" s="50"/>
+      <c r="AL14" s="65"/>
+      <c r="AM14" s="54"/>
+      <c r="AN14" s="49"/>
+      <c r="AO14" s="55"/>
+      <c r="AP14" s="65"/>
+      <c r="AQ14" s="57"/>
+      <c r="AR14" s="65"/>
+      <c r="AS14" s="57"/>
+      <c r="AT14" s="58">
+        <f t="shared" si="1"/>
         <v>173</v>
       </c>
-      <c r="AU14" s="90">
-        <f>COUNTIF(D14:AR14,"&gt;30")</f>
+      <c r="AU14" s="59">
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AV14" s="91"/>
-      <c r="AW14" s="92"/>
-      <c r="AX14" s="93">
-        <f>SUMIF(G14:AS14, "&lt;30")+AV14+AW14</f>
+      <c r="AV14" s="60"/>
+      <c r="AW14" s="61"/>
+      <c r="AX14" s="62">
+        <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="AY14" s="94">
-        <f>AX14/AU14</f>
+      <c r="AY14" s="63">
+        <f t="shared" si="4"/>
         <v>18.333333333333332</v>
       </c>
       <c r="AZ14" s="18"/>
@@ -3537,122 +3537,122 @@
       <c r="BD14" s="17"/>
     </row>
     <row r="15" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A15" s="77" t="s">
+      <c r="A15" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="78" t="s">
+      <c r="B15" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="79">
-        <f>ROUND((AT15-(36*AU15))/AU15,0)</f>
+      <c r="C15" s="48">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D15" s="80"/>
-      <c r="E15" s="81"/>
-      <c r="F15" s="95">
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="64">
         <v>46</v>
       </c>
-      <c r="G15" s="83">
+      <c r="G15" s="52">
         <v>16</v>
       </c>
-      <c r="H15" s="80"/>
-      <c r="I15" s="81"/>
-      <c r="J15" s="95"/>
-      <c r="K15" s="83"/>
-      <c r="L15" s="95"/>
-      <c r="M15" s="83"/>
-      <c r="N15" s="95">
+      <c r="H15" s="49"/>
+      <c r="I15" s="50"/>
+      <c r="J15" s="64"/>
+      <c r="K15" s="52"/>
+      <c r="L15" s="64"/>
+      <c r="M15" s="52"/>
+      <c r="N15" s="64">
         <v>42</v>
       </c>
-      <c r="O15" s="83">
+      <c r="O15" s="52">
         <v>20</v>
       </c>
-      <c r="P15" s="95">
+      <c r="P15" s="64">
         <v>43</v>
       </c>
-      <c r="Q15" s="83">
+      <c r="Q15" s="52">
         <v>19</v>
       </c>
-      <c r="R15" s="95"/>
-      <c r="S15" s="83"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="83"/>
-      <c r="V15" s="95"/>
-      <c r="W15" s="83"/>
-      <c r="X15" s="95">
+      <c r="R15" s="64"/>
+      <c r="S15" s="52"/>
+      <c r="T15" s="64"/>
+      <c r="U15" s="52"/>
+      <c r="V15" s="64"/>
+      <c r="W15" s="52"/>
+      <c r="X15" s="64">
         <v>47</v>
       </c>
-      <c r="Y15" s="83">
+      <c r="Y15" s="52">
         <v>16</v>
       </c>
-      <c r="Z15" s="95">
+      <c r="Z15" s="64">
         <v>41</v>
       </c>
-      <c r="AA15" s="83">
+      <c r="AA15" s="52">
         <v>22</v>
       </c>
-      <c r="AB15" s="95">
+      <c r="AB15" s="64">
         <v>50</v>
       </c>
-      <c r="AC15" s="83">
+      <c r="AC15" s="52">
         <v>13</v>
       </c>
-      <c r="AD15" s="96">
+      <c r="AD15" s="65">
         <v>44</v>
       </c>
-      <c r="AE15" s="85">
+      <c r="AE15" s="54">
         <v>19</v>
       </c>
-      <c r="AF15" s="96">
+      <c r="AF15" s="65">
         <v>43</v>
       </c>
-      <c r="AG15" s="85">
+      <c r="AG15" s="54">
         <v>20</v>
       </c>
-      <c r="AH15" s="96">
+      <c r="AH15" s="65">
         <v>49</v>
       </c>
-      <c r="AI15" s="85">
+      <c r="AI15" s="54">
         <v>15</v>
       </c>
-      <c r="AJ15" s="80"/>
-      <c r="AK15" s="81"/>
-      <c r="AL15" s="96"/>
-      <c r="AM15" s="85"/>
-      <c r="AN15" s="80"/>
-      <c r="AO15" s="86"/>
-      <c r="AP15" s="101">
+      <c r="AJ15" s="49"/>
+      <c r="AK15" s="50"/>
+      <c r="AL15" s="65"/>
+      <c r="AM15" s="54"/>
+      <c r="AN15" s="49"/>
+      <c r="AO15" s="55"/>
+      <c r="AP15" s="70">
         <v>48</v>
       </c>
-      <c r="AQ15" s="88">
+      <c r="AQ15" s="57">
         <v>15</v>
       </c>
-      <c r="AR15" s="101">
+      <c r="AR15" s="70">
         <v>43</v>
       </c>
-      <c r="AS15" s="88">
+      <c r="AS15" s="57">
         <v>20</v>
       </c>
-      <c r="AT15" s="89">
-        <f>F15+J15+L15+N15+P15+R15+T15+V15+X15+Z15+AB15+AD15+AF15+AH15+AJ15+AL15+AN15+AP15+AR15</f>
+      <c r="AT15" s="58">
+        <f t="shared" si="1"/>
         <v>496</v>
       </c>
-      <c r="AU15" s="90">
-        <f>COUNTIF(D15:AR15,"&gt;30")</f>
+      <c r="AU15" s="59">
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AV15" s="91">
+      <c r="AV15" s="60">
         <v>3</v>
       </c>
-      <c r="AW15" s="92">
+      <c r="AW15" s="61">
         <v>2</v>
       </c>
-      <c r="AX15" s="93">
-        <f>SUMIF(G15:AS15, "&lt;30")+AV15+AW15</f>
+      <c r="AX15" s="62">
+        <f t="shared" si="3"/>
         <v>200</v>
       </c>
-      <c r="AY15" s="94">
-        <f>AX15/AU15</f>
+      <c r="AY15" s="63">
+        <f t="shared" si="4"/>
         <v>18.181818181818183</v>
       </c>
       <c r="AZ15" s="18"/>
@@ -3662,126 +3662,126 @@
       <c r="BD15" s="17"/>
     </row>
     <row r="16" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A16" s="77" t="s">
+      <c r="A16" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="78" t="s">
+      <c r="B16" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="79">
-        <f>ROUND((AT16-(36*AU16))/AU16,0)</f>
+      <c r="C16" s="48">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D16" s="80"/>
-      <c r="E16" s="81"/>
-      <c r="F16" s="102"/>
-      <c r="G16" s="83"/>
-      <c r="H16" s="80"/>
-      <c r="I16" s="81"/>
-      <c r="J16" s="102"/>
-      <c r="K16" s="83"/>
-      <c r="L16" s="102"/>
-      <c r="M16" s="83"/>
-      <c r="N16" s="102"/>
-      <c r="O16" s="83"/>
-      <c r="P16" s="102">
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="71"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="50"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="71"/>
+      <c r="M16" s="52"/>
+      <c r="N16" s="71"/>
+      <c r="O16" s="52"/>
+      <c r="P16" s="71">
         <v>47</v>
       </c>
-      <c r="Q16" s="83">
+      <c r="Q16" s="52">
         <v>20</v>
       </c>
-      <c r="R16" s="102">
+      <c r="R16" s="71">
         <v>50</v>
       </c>
-      <c r="S16" s="83">
+      <c r="S16" s="52">
         <v>17</v>
       </c>
-      <c r="T16" s="102">
+      <c r="T16" s="71">
         <v>46</v>
       </c>
-      <c r="U16" s="83">
+      <c r="U16" s="52">
         <v>21</v>
       </c>
-      <c r="V16" s="102">
+      <c r="V16" s="71">
         <v>47</v>
       </c>
-      <c r="W16" s="83">
+      <c r="W16" s="52">
         <v>19</v>
       </c>
-      <c r="X16" s="102">
+      <c r="X16" s="71">
         <v>44</v>
       </c>
-      <c r="Y16" s="83">
+      <c r="Y16" s="52">
         <v>22</v>
       </c>
-      <c r="Z16" s="102">
+      <c r="Z16" s="71">
         <v>52</v>
       </c>
-      <c r="AA16" s="83">
+      <c r="AA16" s="52">
         <v>14</v>
       </c>
-      <c r="AB16" s="102">
+      <c r="AB16" s="71">
         <v>47</v>
       </c>
-      <c r="AC16" s="83">
+      <c r="AC16" s="52">
         <v>19</v>
       </c>
-      <c r="AD16" s="96">
+      <c r="AD16" s="65">
         <v>51</v>
       </c>
-      <c r="AE16" s="85">
+      <c r="AE16" s="54">
         <v>15</v>
       </c>
-      <c r="AF16" s="96">
+      <c r="AF16" s="65">
         <v>49</v>
       </c>
-      <c r="AG16" s="85">
+      <c r="AG16" s="54">
         <v>17</v>
       </c>
-      <c r="AH16" s="96">
+      <c r="AH16" s="65">
         <v>46</v>
       </c>
-      <c r="AI16" s="85">
+      <c r="AI16" s="54">
         <v>20</v>
       </c>
-      <c r="AJ16" s="80"/>
-      <c r="AK16" s="81"/>
-      <c r="AL16" s="96">
+      <c r="AJ16" s="49"/>
+      <c r="AK16" s="50"/>
+      <c r="AL16" s="65">
         <v>51</v>
       </c>
-      <c r="AM16" s="85">
+      <c r="AM16" s="54">
         <v>15</v>
       </c>
-      <c r="AN16" s="80"/>
-      <c r="AO16" s="86"/>
-      <c r="AP16" s="96">
+      <c r="AN16" s="49"/>
+      <c r="AO16" s="55"/>
+      <c r="AP16" s="65">
         <v>49</v>
       </c>
-      <c r="AQ16" s="88">
+      <c r="AQ16" s="57">
         <v>17</v>
       </c>
-      <c r="AR16" s="96">
+      <c r="AR16" s="65">
         <v>48</v>
       </c>
-      <c r="AS16" s="88">
+      <c r="AS16" s="57">
         <v>18</v>
       </c>
-      <c r="AT16" s="89">
-        <f>F16+J16+L16+N16+P16+R16+T16+V16+X16+Z16+AB16+AD16+AF16+AH16+AJ16+AL16+AN16+AP16+AR16</f>
+      <c r="AT16" s="58">
+        <f t="shared" si="1"/>
         <v>627</v>
       </c>
-      <c r="AU16" s="90">
-        <f>COUNTIF(D16:AR16,"&gt;30")</f>
+      <c r="AU16" s="59">
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="AV16" s="91"/>
-      <c r="AW16" s="92"/>
-      <c r="AX16" s="93">
-        <f>SUMIF(G16:AS16, "&lt;30")+AV16+AW16</f>
+      <c r="AV16" s="60"/>
+      <c r="AW16" s="61"/>
+      <c r="AX16" s="62">
+        <f t="shared" si="3"/>
         <v>234</v>
       </c>
-      <c r="AY16" s="94">
-        <f>AX16/AU16</f>
+      <c r="AY16" s="63">
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="AZ16" s="16"/>
@@ -3791,120 +3791,120 @@
       <c r="BD16" s="17"/>
     </row>
     <row r="17" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A17" s="77" t="s">
+      <c r="A17" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="78" t="s">
+      <c r="B17" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="79">
-        <f>ROUND((AT17-(36*AU17))/AU17,0)</f>
+      <c r="C17" s="48">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="D17" s="80"/>
-      <c r="E17" s="81"/>
-      <c r="F17" s="95">
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="64">
         <v>55</v>
       </c>
-      <c r="G17" s="83">
+      <c r="G17" s="52">
         <v>16</v>
       </c>
-      <c r="H17" s="80"/>
-      <c r="I17" s="81"/>
-      <c r="J17" s="95"/>
-      <c r="K17" s="83"/>
-      <c r="L17" s="95">
+      <c r="H17" s="49"/>
+      <c r="I17" s="50"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="52"/>
+      <c r="L17" s="64">
         <v>56</v>
       </c>
-      <c r="M17" s="83">
+      <c r="M17" s="52">
         <v>15</v>
       </c>
-      <c r="N17" s="95">
+      <c r="N17" s="64">
         <v>57</v>
       </c>
-      <c r="O17" s="83">
+      <c r="O17" s="52">
         <v>14</v>
       </c>
-      <c r="P17" s="95"/>
-      <c r="Q17" s="83"/>
-      <c r="R17" s="95"/>
-      <c r="S17" s="83"/>
-      <c r="T17" s="95">
+      <c r="P17" s="64"/>
+      <c r="Q17" s="52"/>
+      <c r="R17" s="64"/>
+      <c r="S17" s="52"/>
+      <c r="T17" s="64">
         <v>49</v>
       </c>
-      <c r="U17" s="83">
+      <c r="U17" s="52">
         <v>22</v>
       </c>
-      <c r="V17" s="95">
+      <c r="V17" s="64">
         <v>58</v>
       </c>
-      <c r="W17" s="83">
+      <c r="W17" s="52">
         <v>14</v>
       </c>
-      <c r="X17" s="95">
+      <c r="X17" s="64">
         <v>50</v>
       </c>
-      <c r="Y17" s="83">
+      <c r="Y17" s="52">
         <v>23</v>
       </c>
-      <c r="Z17" s="95">
+      <c r="Z17" s="64">
         <v>56</v>
       </c>
-      <c r="AA17" s="83">
+      <c r="AA17" s="52">
         <v>16</v>
       </c>
-      <c r="AB17" s="95">
+      <c r="AB17" s="64">
         <v>49</v>
       </c>
-      <c r="AC17" s="83">
+      <c r="AC17" s="52">
         <v>23</v>
       </c>
-      <c r="AD17" s="96">
+      <c r="AD17" s="65">
         <v>54</v>
       </c>
-      <c r="AE17" s="85">
+      <c r="AE17" s="54">
         <v>18</v>
       </c>
-      <c r="AF17" s="96">
+      <c r="AF17" s="65">
         <v>58</v>
       </c>
-      <c r="AG17" s="85">
+      <c r="AG17" s="54">
         <v>14</v>
       </c>
-      <c r="AH17" s="96">
+      <c r="AH17" s="65">
         <v>52</v>
       </c>
-      <c r="AI17" s="85">
+      <c r="AI17" s="54">
         <v>20</v>
       </c>
-      <c r="AJ17" s="80"/>
-      <c r="AK17" s="81"/>
-      <c r="AL17" s="96"/>
-      <c r="AM17" s="85"/>
-      <c r="AN17" s="80"/>
-      <c r="AO17" s="86"/>
-      <c r="AP17" s="96"/>
-      <c r="AQ17" s="88"/>
-      <c r="AR17" s="96"/>
-      <c r="AS17" s="88"/>
-      <c r="AT17" s="89">
-        <f>F17+J17+L17+N17+P17+R17+T17+V17+X17+Z17+AB17+AD17+AF17+AH17+AJ17+AL17+AN17+AP17+AR17</f>
+      <c r="AJ17" s="49"/>
+      <c r="AK17" s="50"/>
+      <c r="AL17" s="65"/>
+      <c r="AM17" s="54"/>
+      <c r="AN17" s="49"/>
+      <c r="AO17" s="55"/>
+      <c r="AP17" s="65"/>
+      <c r="AQ17" s="57"/>
+      <c r="AR17" s="65"/>
+      <c r="AS17" s="57"/>
+      <c r="AT17" s="58">
+        <f t="shared" si="1"/>
         <v>594</v>
       </c>
-      <c r="AU17" s="90">
-        <f>COUNTIF(D17:AR17,"&gt;30")</f>
+      <c r="AU17" s="59">
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AV17" s="91">
+      <c r="AV17" s="60">
         <v>2</v>
       </c>
-      <c r="AW17" s="92"/>
-      <c r="AX17" s="93">
-        <f>SUMIF(G17:AS17, "&lt;30")+AV17+AW17</f>
+      <c r="AW17" s="61"/>
+      <c r="AX17" s="62">
+        <f t="shared" si="3"/>
         <v>197</v>
       </c>
-      <c r="AY17" s="94">
-        <f>AX17/AU17</f>
+      <c r="AY17" s="63">
+        <f t="shared" si="4"/>
         <v>17.90909090909091</v>
       </c>
       <c r="AZ17" s="18"/>
@@ -3914,108 +3914,108 @@
       <c r="BD17" s="17"/>
     </row>
     <row r="18" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A18" s="77" t="s">
+      <c r="A18" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="78" t="s">
+      <c r="B18" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="79">
-        <f>ROUND((AT18-(36*AU18))/AU18,0)</f>
+      <c r="C18" s="48">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D18" s="80"/>
-      <c r="E18" s="81"/>
-      <c r="F18" s="102"/>
-      <c r="G18" s="83"/>
-      <c r="H18" s="80"/>
-      <c r="I18" s="81"/>
-      <c r="J18" s="102"/>
-      <c r="K18" s="83"/>
-      <c r="L18" s="102"/>
-      <c r="M18" s="83"/>
-      <c r="N18" s="102">
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="71"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="50"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="52"/>
+      <c r="L18" s="71"/>
+      <c r="M18" s="52"/>
+      <c r="N18" s="71">
         <v>45</v>
       </c>
-      <c r="O18" s="83">
+      <c r="O18" s="52">
         <v>18</v>
       </c>
-      <c r="P18" s="102">
+      <c r="P18" s="71">
         <v>43</v>
       </c>
-      <c r="Q18" s="83">
+      <c r="Q18" s="52">
         <v>20</v>
       </c>
-      <c r="R18" s="102"/>
-      <c r="S18" s="83"/>
-      <c r="T18" s="102"/>
-      <c r="U18" s="83"/>
-      <c r="V18" s="102"/>
-      <c r="W18" s="83"/>
-      <c r="X18" s="102">
+      <c r="R18" s="71"/>
+      <c r="S18" s="52"/>
+      <c r="T18" s="71"/>
+      <c r="U18" s="52"/>
+      <c r="V18" s="71"/>
+      <c r="W18" s="52"/>
+      <c r="X18" s="71">
         <v>48</v>
       </c>
-      <c r="Y18" s="83">
+      <c r="Y18" s="52">
         <v>15</v>
       </c>
-      <c r="Z18" s="102">
+      <c r="Z18" s="71">
         <v>47</v>
       </c>
-      <c r="AA18" s="83">
+      <c r="AA18" s="52">
         <v>16</v>
       </c>
-      <c r="AB18" s="102"/>
-      <c r="AC18" s="83"/>
-      <c r="AD18" s="96">
+      <c r="AB18" s="71"/>
+      <c r="AC18" s="52"/>
+      <c r="AD18" s="65">
         <v>51</v>
       </c>
-      <c r="AE18" s="85">
+      <c r="AE18" s="54">
         <v>13</v>
       </c>
-      <c r="AF18" s="96">
+      <c r="AF18" s="65">
         <v>45</v>
       </c>
-      <c r="AG18" s="85">
+      <c r="AG18" s="54">
         <v>20</v>
       </c>
-      <c r="AH18" s="96"/>
-      <c r="AI18" s="85"/>
-      <c r="AJ18" s="80"/>
-      <c r="AK18" s="81"/>
-      <c r="AL18" s="96"/>
-      <c r="AM18" s="85"/>
-      <c r="AN18" s="80"/>
-      <c r="AO18" s="86"/>
-      <c r="AP18" s="96">
+      <c r="AH18" s="65"/>
+      <c r="AI18" s="54"/>
+      <c r="AJ18" s="49"/>
+      <c r="AK18" s="50"/>
+      <c r="AL18" s="65"/>
+      <c r="AM18" s="54"/>
+      <c r="AN18" s="49"/>
+      <c r="AO18" s="55"/>
+      <c r="AP18" s="65">
         <v>44</v>
       </c>
-      <c r="AQ18" s="88">
+      <c r="AQ18" s="57">
         <v>21</v>
       </c>
-      <c r="AR18" s="96">
+      <c r="AR18" s="65">
         <v>47</v>
       </c>
-      <c r="AS18" s="88">
+      <c r="AS18" s="57">
         <v>17</v>
       </c>
-      <c r="AT18" s="89">
-        <f>F18+J18+L18+N18+P18+R18+T18+V18+X18+Z18+AB18+AD18+AF18+AH18+AJ18+AL18+AN18+AP18+AR18</f>
+      <c r="AT18" s="58">
+        <f t="shared" si="1"/>
         <v>370</v>
       </c>
-      <c r="AU18" s="90">
-        <f>COUNTIF(D18:AR18,"&gt;30")</f>
+      <c r="AU18" s="59">
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="AV18" s="91"/>
-      <c r="AW18" s="92">
+      <c r="AV18" s="60"/>
+      <c r="AW18" s="61">
         <v>2</v>
       </c>
-      <c r="AX18" s="93">
-        <f>SUMIF(G18:AS18, "&lt;30")+AV18+AW18</f>
+      <c r="AX18" s="62">
+        <f t="shared" si="3"/>
         <v>142</v>
       </c>
-      <c r="AY18" s="94">
-        <f>AX18/AU18</f>
+      <c r="AY18" s="63">
+        <f t="shared" si="4"/>
         <v>17.75</v>
       </c>
       <c r="AZ18" s="16"/>
@@ -4025,120 +4025,120 @@
       <c r="BD18" s="17"/>
     </row>
     <row r="19" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A19" s="77" t="s">
+      <c r="A19" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="78" t="s">
+      <c r="B19" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="79">
-        <f>ROUND((AT19-(36*AU19))/AU19,0)</f>
+      <c r="C19" s="48">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D19" s="80"/>
-      <c r="E19" s="81"/>
-      <c r="F19" s="95">
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="64">
         <v>46</v>
       </c>
-      <c r="G19" s="83">
+      <c r="G19" s="52">
         <v>18</v>
       </c>
-      <c r="H19" s="80"/>
-      <c r="I19" s="81"/>
-      <c r="J19" s="95"/>
-      <c r="K19" s="83"/>
-      <c r="L19" s="95">
+      <c r="H19" s="49"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="64"/>
+      <c r="K19" s="52"/>
+      <c r="L19" s="64">
         <v>46</v>
       </c>
-      <c r="M19" s="83">
+      <c r="M19" s="52">
         <v>18</v>
       </c>
-      <c r="N19" s="95">
+      <c r="N19" s="64">
         <v>46</v>
       </c>
-      <c r="O19" s="83">
+      <c r="O19" s="52">
         <v>18</v>
       </c>
-      <c r="P19" s="95">
+      <c r="P19" s="64">
         <v>46</v>
       </c>
-      <c r="Q19" s="83">
+      <c r="Q19" s="52">
         <v>18</v>
       </c>
-      <c r="R19" s="95">
+      <c r="R19" s="64">
         <v>47</v>
       </c>
-      <c r="S19" s="83">
+      <c r="S19" s="52">
         <v>14</v>
       </c>
-      <c r="T19" s="95">
+      <c r="T19" s="64">
         <v>52</v>
       </c>
-      <c r="U19" s="83">
+      <c r="U19" s="52">
         <v>13</v>
       </c>
-      <c r="V19" s="95"/>
-      <c r="W19" s="83"/>
-      <c r="X19" s="95"/>
-      <c r="Y19" s="83"/>
-      <c r="Z19" s="95">
+      <c r="V19" s="64"/>
+      <c r="W19" s="52"/>
+      <c r="X19" s="64"/>
+      <c r="Y19" s="52"/>
+      <c r="Z19" s="64">
         <v>50</v>
       </c>
-      <c r="AA19" s="83">
+      <c r="AA19" s="52">
         <v>15</v>
       </c>
-      <c r="AB19" s="95"/>
-      <c r="AC19" s="83"/>
-      <c r="AD19" s="96">
+      <c r="AB19" s="64"/>
+      <c r="AC19" s="52"/>
+      <c r="AD19" s="65">
         <v>47</v>
       </c>
-      <c r="AE19" s="85">
+      <c r="AE19" s="54">
         <v>19</v>
       </c>
-      <c r="AF19" s="96">
+      <c r="AF19" s="65">
         <v>48</v>
       </c>
-      <c r="AG19" s="85">
+      <c r="AG19" s="54">
         <v>18</v>
       </c>
-      <c r="AH19" s="96">
+      <c r="AH19" s="65">
         <v>44</v>
       </c>
-      <c r="AI19" s="85">
+      <c r="AI19" s="54">
         <v>22</v>
       </c>
-      <c r="AJ19" s="80"/>
-      <c r="AK19" s="81"/>
-      <c r="AL19" s="96"/>
-      <c r="AM19" s="85"/>
-      <c r="AN19" s="80"/>
-      <c r="AO19" s="86"/>
-      <c r="AP19" s="96"/>
-      <c r="AQ19" s="88"/>
-      <c r="AR19" s="96">
+      <c r="AJ19" s="49"/>
+      <c r="AK19" s="50"/>
+      <c r="AL19" s="65"/>
+      <c r="AM19" s="54"/>
+      <c r="AN19" s="49"/>
+      <c r="AO19" s="55"/>
+      <c r="AP19" s="65"/>
+      <c r="AQ19" s="57"/>
+      <c r="AR19" s="65">
         <v>46</v>
       </c>
-      <c r="AS19" s="88">
+      <c r="AS19" s="57">
         <v>19</v>
       </c>
-      <c r="AT19" s="89">
-        <f>F19+J19+L19+N19+P19+R19+T19+V19+X19+Z19+AB19+AD19+AF19+AH19+AJ19+AL19+AN19+AP19+AR19</f>
+      <c r="AT19" s="58">
+        <f t="shared" si="1"/>
         <v>518</v>
       </c>
-      <c r="AU19" s="90">
-        <f>COUNTIF(D19:AR19,"&gt;30")</f>
+      <c r="AU19" s="59">
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="AV19" s="104"/>
-      <c r="AW19" s="105">
+      <c r="AV19" s="73"/>
+      <c r="AW19" s="74">
         <v>1</v>
       </c>
-      <c r="AX19" s="93">
-        <f>SUMIF(G19:AS19, "&lt;30")+AV19+AW19</f>
+      <c r="AX19" s="62">
+        <f t="shared" si="3"/>
         <v>193</v>
       </c>
-      <c r="AY19" s="94">
-        <f>AX19/AU19</f>
+      <c r="AY19" s="63">
+        <f t="shared" si="4"/>
         <v>17.545454545454547</v>
       </c>
       <c r="AZ19" s="18"/>
@@ -4148,124 +4148,124 @@
       <c r="BD19" s="17"/>
     </row>
     <row r="20" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A20" s="77" t="s">
+      <c r="A20" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="78" t="s">
+      <c r="B20" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="79">
-        <f>ROUND((AT20-(36*AU20))/AU20,0)</f>
+      <c r="C20" s="48">
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="D20" s="80"/>
-      <c r="E20" s="81"/>
-      <c r="F20" s="102">
+      <c r="D20" s="49"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="71">
         <v>61</v>
       </c>
-      <c r="G20" s="83">
+      <c r="G20" s="52">
         <v>14</v>
       </c>
-      <c r="H20" s="80"/>
-      <c r="I20" s="81"/>
-      <c r="J20" s="102">
+      <c r="H20" s="49"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="71">
         <v>56</v>
       </c>
-      <c r="K20" s="83">
+      <c r="K20" s="52">
         <v>19</v>
       </c>
-      <c r="L20" s="102">
+      <c r="L20" s="71">
         <v>60</v>
       </c>
-      <c r="M20" s="83">
+      <c r="M20" s="52">
         <v>15</v>
       </c>
-      <c r="N20" s="102">
+      <c r="N20" s="71">
         <v>56</v>
       </c>
-      <c r="O20" s="83">
+      <c r="O20" s="52">
         <v>20</v>
       </c>
-      <c r="P20" s="102">
+      <c r="P20" s="71">
         <v>54</v>
       </c>
-      <c r="Q20" s="83">
+      <c r="Q20" s="52">
         <v>22</v>
       </c>
-      <c r="R20" s="102"/>
-      <c r="S20" s="83"/>
-      <c r="T20" s="102">
+      <c r="R20" s="71"/>
+      <c r="S20" s="52"/>
+      <c r="T20" s="71">
         <v>66</v>
       </c>
-      <c r="U20" s="83">
+      <c r="U20" s="52">
         <v>9</v>
       </c>
-      <c r="V20" s="102">
+      <c r="V20" s="71">
         <v>55</v>
       </c>
-      <c r="W20" s="83">
+      <c r="W20" s="52">
         <v>22</v>
       </c>
-      <c r="X20" s="102"/>
-      <c r="Y20" s="83"/>
-      <c r="Z20" s="102">
+      <c r="X20" s="71"/>
+      <c r="Y20" s="52"/>
+      <c r="Z20" s="71">
         <v>70</v>
       </c>
-      <c r="AA20" s="83">
+      <c r="AA20" s="52">
         <v>6</v>
       </c>
-      <c r="AB20" s="102">
+      <c r="AB20" s="71">
         <v>63</v>
       </c>
-      <c r="AC20" s="83">
+      <c r="AC20" s="52">
         <v>15</v>
       </c>
-      <c r="AD20" s="96">
+      <c r="AD20" s="65">
         <v>58</v>
       </c>
-      <c r="AE20" s="85">
+      <c r="AE20" s="54">
         <v>20</v>
       </c>
-      <c r="AF20" s="96">
+      <c r="AF20" s="65">
         <v>60</v>
       </c>
-      <c r="AG20" s="85">
+      <c r="AG20" s="54">
         <v>18</v>
       </c>
-      <c r="AH20" s="96">
+      <c r="AH20" s="65">
         <v>55</v>
       </c>
-      <c r="AI20" s="85">
+      <c r="AI20" s="54">
         <v>23</v>
       </c>
-      <c r="AJ20" s="80"/>
-      <c r="AK20" s="81"/>
-      <c r="AL20" s="96"/>
-      <c r="AM20" s="85"/>
-      <c r="AN20" s="80"/>
-      <c r="AO20" s="86"/>
-      <c r="AP20" s="96"/>
-      <c r="AQ20" s="88"/>
-      <c r="AR20" s="96"/>
-      <c r="AS20" s="88"/>
-      <c r="AT20" s="89">
-        <f>F20+J20+L20+N20+P20+R20+T20+V20+X20+Z20+AB20+AD20+AF20+AH20+AJ20+AL20+AN20+AP20+AR20</f>
+      <c r="AJ20" s="49"/>
+      <c r="AK20" s="50"/>
+      <c r="AL20" s="65"/>
+      <c r="AM20" s="54"/>
+      <c r="AN20" s="49"/>
+      <c r="AO20" s="55"/>
+      <c r="AP20" s="65"/>
+      <c r="AQ20" s="57"/>
+      <c r="AR20" s="65"/>
+      <c r="AS20" s="57"/>
+      <c r="AT20" s="58">
+        <f t="shared" si="1"/>
         <v>714</v>
       </c>
-      <c r="AU20" s="90">
-        <f>COUNTIF(D20:AR20,"&gt;30")</f>
+      <c r="AU20" s="59">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="AV20" s="91">
+      <c r="AV20" s="60">
         <v>2</v>
       </c>
-      <c r="AW20" s="92"/>
-      <c r="AX20" s="93">
-        <f>SUMIF(G20:AS20, "&lt;30")+AV20+AW20</f>
+      <c r="AW20" s="61"/>
+      <c r="AX20" s="62">
+        <f t="shared" si="3"/>
         <v>205</v>
       </c>
-      <c r="AY20" s="94">
-        <f>AX20/AU20</f>
+      <c r="AY20" s="63">
+        <f t="shared" si="4"/>
         <v>17.083333333333332</v>
       </c>
       <c r="AZ20" s="16"/>
@@ -4275,77 +4275,77 @@
       <c r="BD20" s="17"/>
     </row>
     <row r="21" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A21" s="77" t="s">
+      <c r="A21" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="78" t="s">
+      <c r="B21" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="79">
+      <c r="C21" s="48">
         <v>18</v>
       </c>
-      <c r="D21" s="80"/>
-      <c r="E21" s="81"/>
-      <c r="F21" s="95">
+      <c r="D21" s="49"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="64">
         <v>56</v>
       </c>
-      <c r="G21" s="83">
+      <c r="G21" s="52">
         <v>16</v>
       </c>
-      <c r="H21" s="80"/>
-      <c r="I21" s="81"/>
-      <c r="J21" s="95"/>
-      <c r="K21" s="83"/>
-      <c r="L21" s="95"/>
-      <c r="M21" s="83"/>
-      <c r="N21" s="95"/>
-      <c r="O21" s="83"/>
-      <c r="P21" s="95"/>
-      <c r="Q21" s="83"/>
-      <c r="R21" s="95"/>
-      <c r="S21" s="83"/>
-      <c r="T21" s="95"/>
-      <c r="U21" s="83"/>
-      <c r="V21" s="95"/>
-      <c r="W21" s="83"/>
-      <c r="X21" s="95"/>
-      <c r="Y21" s="83"/>
-      <c r="Z21" s="95"/>
-      <c r="AA21" s="83"/>
-      <c r="AB21" s="95"/>
-      <c r="AC21" s="83"/>
-      <c r="AD21" s="96"/>
-      <c r="AE21" s="85"/>
-      <c r="AF21" s="96"/>
-      <c r="AG21" s="85"/>
-      <c r="AH21" s="96"/>
-      <c r="AI21" s="85"/>
-      <c r="AJ21" s="80"/>
-      <c r="AK21" s="81"/>
-      <c r="AL21" s="96"/>
-      <c r="AM21" s="85"/>
-      <c r="AN21" s="80"/>
-      <c r="AO21" s="86"/>
-      <c r="AP21" s="96"/>
-      <c r="AQ21" s="88"/>
-      <c r="AR21" s="96"/>
-      <c r="AS21" s="88"/>
-      <c r="AT21" s="89">
-        <f>F21+J21+L21+N21+P21+R21+T21+V21+X21+Z21+AB21+AD21+AF21+AH21+AJ21+AL21+AN21+AP21+AR21</f>
+      <c r="H21" s="49"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="64"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="64"/>
+      <c r="M21" s="52"/>
+      <c r="N21" s="64"/>
+      <c r="O21" s="52"/>
+      <c r="P21" s="64"/>
+      <c r="Q21" s="52"/>
+      <c r="R21" s="64"/>
+      <c r="S21" s="52"/>
+      <c r="T21" s="64"/>
+      <c r="U21" s="52"/>
+      <c r="V21" s="64"/>
+      <c r="W21" s="52"/>
+      <c r="X21" s="64"/>
+      <c r="Y21" s="52"/>
+      <c r="Z21" s="64"/>
+      <c r="AA21" s="52"/>
+      <c r="AB21" s="64"/>
+      <c r="AC21" s="52"/>
+      <c r="AD21" s="65"/>
+      <c r="AE21" s="54"/>
+      <c r="AF21" s="65"/>
+      <c r="AG21" s="54"/>
+      <c r="AH21" s="65"/>
+      <c r="AI21" s="54"/>
+      <c r="AJ21" s="49"/>
+      <c r="AK21" s="50"/>
+      <c r="AL21" s="65"/>
+      <c r="AM21" s="54"/>
+      <c r="AN21" s="49"/>
+      <c r="AO21" s="55"/>
+      <c r="AP21" s="65"/>
+      <c r="AQ21" s="57"/>
+      <c r="AR21" s="65"/>
+      <c r="AS21" s="57"/>
+      <c r="AT21" s="58">
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
-      <c r="AU21" s="90">
-        <f>COUNTIF(D21:AR21,"&gt;30")</f>
+      <c r="AU21" s="59">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AV21" s="91"/>
-      <c r="AW21" s="92"/>
-      <c r="AX21" s="93">
-        <f>SUMIF(G21:AS21, "&lt;30")+AV21+AW21</f>
+      <c r="AV21" s="60"/>
+      <c r="AW21" s="61"/>
+      <c r="AX21" s="62">
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="AY21" s="94">
-        <f>AX21/AU21</f>
+      <c r="AY21" s="63">
+        <f t="shared" si="4"/>
         <v>16</v>
       </c>
       <c r="AZ21" s="18"/>
@@ -4355,77 +4355,77 @@
       <c r="BD21" s="17"/>
     </row>
     <row r="22" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A22" s="106" t="s">
+      <c r="A22" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="107" t="s">
+      <c r="B22" s="76" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="108" t="s">
+      <c r="C22" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="80"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="82"/>
-      <c r="G22" s="83"/>
-      <c r="H22" s="80"/>
-      <c r="I22" s="81"/>
-      <c r="J22" s="82"/>
-      <c r="K22" s="83"/>
-      <c r="L22" s="82">
+      <c r="D22" s="49"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="50"/>
+      <c r="J22" s="51"/>
+      <c r="K22" s="52"/>
+      <c r="L22" s="51">
         <v>50</v>
       </c>
-      <c r="M22" s="83"/>
-      <c r="N22" s="82"/>
-      <c r="O22" s="83"/>
-      <c r="P22" s="82"/>
-      <c r="Q22" s="83"/>
-      <c r="R22" s="82"/>
-      <c r="S22" s="83"/>
-      <c r="T22" s="82"/>
-      <c r="U22" s="83"/>
-      <c r="V22" s="82"/>
-      <c r="W22" s="83"/>
-      <c r="X22" s="82"/>
-      <c r="Y22" s="83"/>
-      <c r="Z22" s="82"/>
-      <c r="AA22" s="83"/>
-      <c r="AB22" s="82"/>
-      <c r="AC22" s="83"/>
-      <c r="AD22" s="87"/>
-      <c r="AE22" s="83"/>
-      <c r="AF22" s="87"/>
-      <c r="AG22" s="83"/>
-      <c r="AH22" s="87"/>
-      <c r="AI22" s="83"/>
-      <c r="AJ22" s="80"/>
-      <c r="AK22" s="81"/>
-      <c r="AL22" s="87"/>
-      <c r="AM22" s="83"/>
-      <c r="AN22" s="80"/>
-      <c r="AO22" s="86"/>
-      <c r="AP22" s="84"/>
-      <c r="AQ22" s="88"/>
-      <c r="AR22" s="84"/>
-      <c r="AS22" s="88"/>
-      <c r="AT22" s="89">
-        <f>F22+J22+L22+N22+P22+R22+T22+V22+X22+Z22+AB22+AD22+AF22+AH22+AJ22+AL22+AN22+AP22+AR22</f>
+      <c r="M22" s="52"/>
+      <c r="N22" s="51"/>
+      <c r="O22" s="52"/>
+      <c r="P22" s="51"/>
+      <c r="Q22" s="52"/>
+      <c r="R22" s="51"/>
+      <c r="S22" s="52"/>
+      <c r="T22" s="51"/>
+      <c r="U22" s="52"/>
+      <c r="V22" s="51"/>
+      <c r="W22" s="52"/>
+      <c r="X22" s="51"/>
+      <c r="Y22" s="52"/>
+      <c r="Z22" s="51"/>
+      <c r="AA22" s="52"/>
+      <c r="AB22" s="51"/>
+      <c r="AC22" s="52"/>
+      <c r="AD22" s="56"/>
+      <c r="AE22" s="52"/>
+      <c r="AF22" s="56"/>
+      <c r="AG22" s="52"/>
+      <c r="AH22" s="56"/>
+      <c r="AI22" s="52"/>
+      <c r="AJ22" s="49"/>
+      <c r="AK22" s="50"/>
+      <c r="AL22" s="56"/>
+      <c r="AM22" s="52"/>
+      <c r="AN22" s="49"/>
+      <c r="AO22" s="55"/>
+      <c r="AP22" s="53"/>
+      <c r="AQ22" s="57"/>
+      <c r="AR22" s="53"/>
+      <c r="AS22" s="57"/>
+      <c r="AT22" s="58">
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="AU22" s="90">
-        <f>COUNTIF(D22:AR22,"&gt;30")</f>
+      <c r="AU22" s="59">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AV22" s="91">
+      <c r="AV22" s="60">
         <v>1</v>
       </c>
-      <c r="AW22" s="92"/>
-      <c r="AX22" s="93">
-        <f>SUMIF(G22:AS22, "&lt;30")+AV22+AW22</f>
+      <c r="AW22" s="61"/>
+      <c r="AX22" s="62">
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="AY22" s="94">
-        <f>AX22/AU22</f>
+      <c r="AY22" s="63">
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="AZ22" s="20"/>
@@ -4435,75 +4435,75 @@
       <c r="BD22" s="24"/>
     </row>
     <row r="23" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A23" s="106" t="s">
+      <c r="A23" s="75" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="107" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" s="108" t="s">
+      <c r="C23" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="80"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="82"/>
-      <c r="G23" s="83"/>
-      <c r="H23" s="80"/>
-      <c r="I23" s="81"/>
-      <c r="J23" s="82"/>
-      <c r="K23" s="83"/>
-      <c r="L23" s="82"/>
-      <c r="M23" s="83"/>
-      <c r="N23" s="82"/>
-      <c r="O23" s="83"/>
-      <c r="P23" s="82"/>
-      <c r="Q23" s="83"/>
-      <c r="R23" s="82"/>
-      <c r="S23" s="83"/>
-      <c r="T23" s="82"/>
-      <c r="U23" s="83"/>
-      <c r="V23" s="82"/>
-      <c r="W23" s="83"/>
-      <c r="X23" s="82"/>
-      <c r="Y23" s="83"/>
-      <c r="Z23" s="82"/>
-      <c r="AA23" s="83"/>
-      <c r="AB23" s="82"/>
-      <c r="AC23" s="83"/>
-      <c r="AD23" s="87"/>
-      <c r="AE23" s="83"/>
-      <c r="AF23" s="87"/>
-      <c r="AG23" s="83"/>
-      <c r="AH23" s="87"/>
-      <c r="AI23" s="83"/>
-      <c r="AJ23" s="80"/>
-      <c r="AK23" s="81"/>
-      <c r="AL23" s="84">
+      <c r="D23" s="49"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="50"/>
+      <c r="J23" s="51"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="51"/>
+      <c r="M23" s="52"/>
+      <c r="N23" s="51"/>
+      <c r="O23" s="52"/>
+      <c r="P23" s="51"/>
+      <c r="Q23" s="52"/>
+      <c r="R23" s="51"/>
+      <c r="S23" s="52"/>
+      <c r="T23" s="51"/>
+      <c r="U23" s="52"/>
+      <c r="V23" s="51"/>
+      <c r="W23" s="52"/>
+      <c r="X23" s="51"/>
+      <c r="Y23" s="52"/>
+      <c r="Z23" s="51"/>
+      <c r="AA23" s="52"/>
+      <c r="AB23" s="51"/>
+      <c r="AC23" s="52"/>
+      <c r="AD23" s="56"/>
+      <c r="AE23" s="52"/>
+      <c r="AF23" s="56"/>
+      <c r="AG23" s="52"/>
+      <c r="AH23" s="56"/>
+      <c r="AI23" s="52"/>
+      <c r="AJ23" s="49"/>
+      <c r="AK23" s="50"/>
+      <c r="AL23" s="53">
         <v>50</v>
       </c>
-      <c r="AM23" s="83"/>
-      <c r="AN23" s="80"/>
-      <c r="AO23" s="86"/>
-      <c r="AP23" s="84"/>
-      <c r="AQ23" s="88"/>
-      <c r="AR23" s="84"/>
-      <c r="AS23" s="88"/>
-      <c r="AT23" s="89">
-        <f>F23+J23+L23+N23+P23+R23+T23+V23+X23+Z23+AB23+AD23+AF23+AH23+AJ23+AL23+AN23+AP23+AR23</f>
+      <c r="AM23" s="52"/>
+      <c r="AN23" s="49"/>
+      <c r="AO23" s="55"/>
+      <c r="AP23" s="53"/>
+      <c r="AQ23" s="57"/>
+      <c r="AR23" s="53"/>
+      <c r="AS23" s="57"/>
+      <c r="AT23" s="58">
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="AU23" s="90">
-        <f>COUNTIF(D23:AR23,"&gt;30")</f>
+      <c r="AU23" s="59">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AV23" s="91"/>
-      <c r="AW23" s="92"/>
-      <c r="AX23" s="93">
-        <f>SUMIF(G23:AS23, "&lt;30")+AV23+AW23</f>
+      <c r="AV23" s="60"/>
+      <c r="AW23" s="61"/>
+      <c r="AX23" s="62">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AY23" s="94">
-        <f>AX23/AU23</f>
+      <c r="AY23" s="63">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AZ23" s="20"/>
@@ -4513,75 +4513,75 @@
       <c r="BD23" s="24"/>
     </row>
     <row r="24" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A24" s="106" t="s">
+      <c r="A24" s="75" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="B24" s="107" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="108" t="s">
+      <c r="C24" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="80"/>
-      <c r="E24" s="81"/>
-      <c r="F24" s="109"/>
-      <c r="G24" s="110"/>
-      <c r="H24" s="80"/>
-      <c r="I24" s="81"/>
-      <c r="J24" s="109"/>
-      <c r="K24" s="110"/>
-      <c r="L24" s="109"/>
-      <c r="M24" s="110"/>
-      <c r="N24" s="109"/>
-      <c r="O24" s="110"/>
-      <c r="P24" s="109"/>
-      <c r="Q24" s="110"/>
-      <c r="R24" s="109"/>
-      <c r="S24" s="110"/>
-      <c r="T24" s="109"/>
-      <c r="U24" s="110"/>
-      <c r="V24" s="109"/>
-      <c r="W24" s="110"/>
-      <c r="X24" s="109"/>
-      <c r="Y24" s="110"/>
-      <c r="Z24" s="109"/>
-      <c r="AA24" s="110"/>
-      <c r="AB24" s="109"/>
-      <c r="AC24" s="110"/>
-      <c r="AD24" s="111"/>
-      <c r="AE24" s="110"/>
-      <c r="AF24" s="111"/>
-      <c r="AG24" s="110"/>
-      <c r="AH24" s="111"/>
-      <c r="AI24" s="110"/>
-      <c r="AJ24" s="80"/>
-      <c r="AK24" s="81"/>
-      <c r="AL24" s="112"/>
-      <c r="AM24" s="110"/>
-      <c r="AN24" s="80"/>
-      <c r="AO24" s="86"/>
-      <c r="AP24" s="112"/>
-      <c r="AQ24" s="113"/>
-      <c r="AR24" s="112">
+      <c r="D24" s="49"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="79"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="78"/>
+      <c r="K24" s="79"/>
+      <c r="L24" s="78"/>
+      <c r="M24" s="79"/>
+      <c r="N24" s="78"/>
+      <c r="O24" s="79"/>
+      <c r="P24" s="78"/>
+      <c r="Q24" s="79"/>
+      <c r="R24" s="78"/>
+      <c r="S24" s="79"/>
+      <c r="T24" s="78"/>
+      <c r="U24" s="79"/>
+      <c r="V24" s="78"/>
+      <c r="W24" s="79"/>
+      <c r="X24" s="78"/>
+      <c r="Y24" s="79"/>
+      <c r="Z24" s="78"/>
+      <c r="AA24" s="79"/>
+      <c r="AB24" s="78"/>
+      <c r="AC24" s="79"/>
+      <c r="AD24" s="80"/>
+      <c r="AE24" s="79"/>
+      <c r="AF24" s="80"/>
+      <c r="AG24" s="79"/>
+      <c r="AH24" s="80"/>
+      <c r="AI24" s="79"/>
+      <c r="AJ24" s="49"/>
+      <c r="AK24" s="50"/>
+      <c r="AL24" s="81"/>
+      <c r="AM24" s="79"/>
+      <c r="AN24" s="49"/>
+      <c r="AO24" s="55"/>
+      <c r="AP24" s="81"/>
+      <c r="AQ24" s="82"/>
+      <c r="AR24" s="81">
         <v>49</v>
       </c>
-      <c r="AS24" s="113"/>
-      <c r="AT24" s="89">
-        <f>F24+J24+L24+N24+P24+R24+T24+V24+X24+Z24+AB24+AD24+AF24+AH24+AJ24+AL24+AN24+AP24+AR24</f>
+      <c r="AS24" s="82"/>
+      <c r="AT24" s="58">
+        <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="AU24" s="90">
-        <f>COUNTIF(D24:AR24,"&gt;30")</f>
+      <c r="AU24" s="59">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AV24" s="114"/>
-      <c r="AW24" s="115"/>
-      <c r="AX24" s="93">
-        <f>SUMIF(G24:AS24, "&lt;30")+AV24+AW24</f>
+      <c r="AV24" s="83"/>
+      <c r="AW24" s="84"/>
+      <c r="AX24" s="62">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AY24" s="94">
-        <f>AX24/AU24</f>
+      <c r="AY24" s="63">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AZ24" s="20"/>
@@ -4591,75 +4591,75 @@
       <c r="BD24" s="24"/>
     </row>
     <row r="25" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A25" s="106" t="s">
+      <c r="A25" s="75" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="76" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="107" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="108" t="s">
+      <c r="C25" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="80"/>
-      <c r="E25" s="81"/>
-      <c r="F25" s="109"/>
-      <c r="G25" s="110"/>
-      <c r="H25" s="80"/>
-      <c r="I25" s="81"/>
-      <c r="J25" s="109"/>
-      <c r="K25" s="110"/>
-      <c r="L25" s="109"/>
-      <c r="M25" s="110"/>
-      <c r="N25" s="109"/>
-      <c r="O25" s="110"/>
-      <c r="P25" s="109"/>
-      <c r="Q25" s="110"/>
-      <c r="R25" s="109"/>
-      <c r="S25" s="110"/>
-      <c r="T25" s="109"/>
-      <c r="U25" s="110"/>
-      <c r="V25" s="109"/>
-      <c r="W25" s="110"/>
-      <c r="X25" s="109"/>
-      <c r="Y25" s="110"/>
-      <c r="Z25" s="109"/>
-      <c r="AA25" s="110"/>
-      <c r="AB25" s="109"/>
-      <c r="AC25" s="110"/>
-      <c r="AD25" s="111"/>
-      <c r="AE25" s="110"/>
-      <c r="AF25" s="111"/>
-      <c r="AG25" s="110"/>
-      <c r="AH25" s="111"/>
-      <c r="AI25" s="110"/>
-      <c r="AJ25" s="80"/>
-      <c r="AK25" s="81"/>
-      <c r="AL25" s="112"/>
-      <c r="AM25" s="110"/>
-      <c r="AN25" s="80"/>
-      <c r="AO25" s="86"/>
-      <c r="AP25" s="112"/>
-      <c r="AQ25" s="113"/>
-      <c r="AR25" s="112">
+      <c r="D25" s="49"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="78"/>
+      <c r="G25" s="79"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="78"/>
+      <c r="K25" s="79"/>
+      <c r="L25" s="78"/>
+      <c r="M25" s="79"/>
+      <c r="N25" s="78"/>
+      <c r="O25" s="79"/>
+      <c r="P25" s="78"/>
+      <c r="Q25" s="79"/>
+      <c r="R25" s="78"/>
+      <c r="S25" s="79"/>
+      <c r="T25" s="78"/>
+      <c r="U25" s="79"/>
+      <c r="V25" s="78"/>
+      <c r="W25" s="79"/>
+      <c r="X25" s="78"/>
+      <c r="Y25" s="79"/>
+      <c r="Z25" s="78"/>
+      <c r="AA25" s="79"/>
+      <c r="AB25" s="78"/>
+      <c r="AC25" s="79"/>
+      <c r="AD25" s="80"/>
+      <c r="AE25" s="79"/>
+      <c r="AF25" s="80"/>
+      <c r="AG25" s="79"/>
+      <c r="AH25" s="80"/>
+      <c r="AI25" s="79"/>
+      <c r="AJ25" s="49"/>
+      <c r="AK25" s="50"/>
+      <c r="AL25" s="81"/>
+      <c r="AM25" s="79"/>
+      <c r="AN25" s="49"/>
+      <c r="AO25" s="55"/>
+      <c r="AP25" s="81"/>
+      <c r="AQ25" s="82"/>
+      <c r="AR25" s="81">
         <v>49</v>
       </c>
-      <c r="AS25" s="113"/>
-      <c r="AT25" s="89">
-        <f>F25+J25+L25+N25+P25+R25+T25+V25+X25+Z25+AB25+AD25+AF25+AH25+AJ25+AL25+AN25+AP25+AR25</f>
+      <c r="AS25" s="82"/>
+      <c r="AT25" s="58">
+        <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="AU25" s="90">
-        <f>COUNTIF(D25:AR25,"&gt;30")</f>
+      <c r="AU25" s="59">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AV25" s="114"/>
-      <c r="AW25" s="115"/>
-      <c r="AX25" s="93">
-        <f>SUMIF(G25:AS25, "&lt;30")+AV25+AW25</f>
+      <c r="AV25" s="83"/>
+      <c r="AW25" s="84"/>
+      <c r="AX25" s="62">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AY25" s="94">
-        <f>AX25/AU25</f>
+      <c r="AY25" s="63">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AZ25" s="20"/>
@@ -4669,75 +4669,75 @@
       <c r="BD25" s="24"/>
     </row>
     <row r="26" spans="1:56" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="106" t="s">
+      <c r="A26" s="75" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="107" t="s">
+      <c r="B26" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="C26" s="108" t="s">
+      <c r="C26" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="D26" s="80"/>
-      <c r="E26" s="81"/>
-      <c r="F26" s="109"/>
-      <c r="G26" s="110"/>
-      <c r="H26" s="80"/>
-      <c r="I26" s="81"/>
-      <c r="J26" s="109"/>
-      <c r="K26" s="110"/>
-      <c r="L26" s="109"/>
-      <c r="M26" s="110"/>
-      <c r="N26" s="109"/>
-      <c r="O26" s="110"/>
-      <c r="P26" s="109"/>
-      <c r="Q26" s="110"/>
-      <c r="R26" s="109"/>
-      <c r="S26" s="110"/>
-      <c r="T26" s="109"/>
-      <c r="U26" s="110"/>
-      <c r="V26" s="109"/>
-      <c r="W26" s="110"/>
-      <c r="X26" s="109"/>
-      <c r="Y26" s="110"/>
-      <c r="Z26" s="109"/>
-      <c r="AA26" s="110"/>
-      <c r="AB26" s="109"/>
-      <c r="AC26" s="110"/>
-      <c r="AD26" s="111"/>
-      <c r="AE26" s="110"/>
-      <c r="AF26" s="111"/>
-      <c r="AG26" s="110"/>
-      <c r="AH26" s="111"/>
-      <c r="AI26" s="110"/>
-      <c r="AJ26" s="80"/>
-      <c r="AK26" s="81"/>
-      <c r="AL26" s="111"/>
-      <c r="AM26" s="110"/>
-      <c r="AN26" s="80"/>
-      <c r="AO26" s="86"/>
-      <c r="AP26" s="112">
+      <c r="D26" s="49"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="79"/>
+      <c r="H26" s="49"/>
+      <c r="I26" s="50"/>
+      <c r="J26" s="78"/>
+      <c r="K26" s="79"/>
+      <c r="L26" s="78"/>
+      <c r="M26" s="79"/>
+      <c r="N26" s="78"/>
+      <c r="O26" s="79"/>
+      <c r="P26" s="78"/>
+      <c r="Q26" s="79"/>
+      <c r="R26" s="78"/>
+      <c r="S26" s="79"/>
+      <c r="T26" s="78"/>
+      <c r="U26" s="79"/>
+      <c r="V26" s="78"/>
+      <c r="W26" s="79"/>
+      <c r="X26" s="78"/>
+      <c r="Y26" s="79"/>
+      <c r="Z26" s="78"/>
+      <c r="AA26" s="79"/>
+      <c r="AB26" s="78"/>
+      <c r="AC26" s="79"/>
+      <c r="AD26" s="80"/>
+      <c r="AE26" s="79"/>
+      <c r="AF26" s="80"/>
+      <c r="AG26" s="79"/>
+      <c r="AH26" s="80"/>
+      <c r="AI26" s="79"/>
+      <c r="AJ26" s="49"/>
+      <c r="AK26" s="50"/>
+      <c r="AL26" s="80"/>
+      <c r="AM26" s="79"/>
+      <c r="AN26" s="49"/>
+      <c r="AO26" s="55"/>
+      <c r="AP26" s="81">
         <v>45</v>
       </c>
-      <c r="AQ26" s="113"/>
-      <c r="AR26" s="112"/>
-      <c r="AS26" s="113"/>
-      <c r="AT26" s="116">
-        <f>F26+J26+L26+N26+P26+R26+T26+V26+X26+Z26+AB26+AD26+AF26+AH26+AJ26+AL26+AN26+AP26+AR26</f>
+      <c r="AQ26" s="82"/>
+      <c r="AR26" s="81"/>
+      <c r="AS26" s="82"/>
+      <c r="AT26" s="85">
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
-      <c r="AU26" s="117">
-        <f>COUNTIF(D26:AR26,"&gt;30")</f>
+      <c r="AU26" s="86">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AV26" s="118"/>
-      <c r="AW26" s="119"/>
-      <c r="AX26" s="120">
-        <f>SUMIF(G26:AS26, "&lt;30")+AV26+AW26</f>
+      <c r="AV26" s="87"/>
+      <c r="AW26" s="88"/>
+      <c r="AX26" s="89">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="AY26" s="121">
-        <f>AX26/AU26</f>
+      <c r="AY26" s="90">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AZ26" s="20"/>
@@ -4747,108 +4747,108 @@
       <c r="BD26" s="24"/>
     </row>
     <row r="27" spans="1:56" s="3" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="122"/>
-      <c r="B27" s="123"/>
-      <c r="C27" s="124"/>
-      <c r="D27" s="125"/>
-      <c r="E27" s="126"/>
-      <c r="F27" s="126">
+      <c r="A27" s="91"/>
+      <c r="B27" s="92"/>
+      <c r="C27" s="93"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="95"/>
+      <c r="F27" s="95">
         <f>AVERAGEIF(F4:F23,"&gt;0")</f>
         <v>49.75</v>
       </c>
-      <c r="G27" s="126"/>
-      <c r="H27" s="126"/>
-      <c r="I27" s="126"/>
-      <c r="J27" s="126">
+      <c r="G27" s="95"/>
+      <c r="H27" s="95"/>
+      <c r="I27" s="95"/>
+      <c r="J27" s="95">
         <f>AVERAGEIF(J4:J23,"&gt;0")</f>
         <v>54</v>
       </c>
-      <c r="K27" s="126"/>
-      <c r="L27" s="126">
+      <c r="K27" s="95"/>
+      <c r="L27" s="95">
         <f>AVERAGEIF(L4:L23,"&gt;0")</f>
         <v>51.428571428571431</v>
       </c>
-      <c r="M27" s="126"/>
-      <c r="N27" s="126">
+      <c r="M27" s="95"/>
+      <c r="N27" s="95">
         <f>AVERAGEIF(N4:N23,"&gt;0")</f>
         <v>48.9</v>
       </c>
-      <c r="O27" s="126"/>
-      <c r="P27" s="126">
+      <c r="O27" s="95"/>
+      <c r="P27" s="95">
         <f>AVERAGEIF(P4:P23,"&gt;0")</f>
         <v>46.785714285714285</v>
       </c>
-      <c r="Q27" s="126"/>
-      <c r="R27" s="126">
+      <c r="Q27" s="95"/>
+      <c r="R27" s="95">
         <f>AVERAGEIF(R4:R23,"&gt;0")</f>
         <v>48.272727272727273</v>
       </c>
-      <c r="S27" s="126"/>
-      <c r="T27" s="126">
+      <c r="S27" s="95"/>
+      <c r="T27" s="95">
         <f>AVERAGEIF(T4:T23,"&gt;0")</f>
         <v>50.333333333333336</v>
       </c>
-      <c r="U27" s="126"/>
-      <c r="V27" s="126">
+      <c r="U27" s="95"/>
+      <c r="V27" s="95">
         <f>AVERAGEIF(V4:V23,"&gt;0")</f>
         <v>49</v>
       </c>
-      <c r="W27" s="126"/>
-      <c r="X27" s="126">
+      <c r="W27" s="95"/>
+      <c r="X27" s="95">
         <f>AVERAGEIF(X4:X23,"&gt;0")</f>
         <v>46.46153846153846</v>
       </c>
-      <c r="Y27" s="126"/>
-      <c r="Z27" s="126">
+      <c r="Y27" s="95"/>
+      <c r="Z27" s="95">
         <f>AVERAGEIF(Z4:Z23,"&gt;0")</f>
         <v>49.53846153846154</v>
       </c>
-      <c r="AA27" s="126"/>
-      <c r="AB27" s="126">
+      <c r="AA27" s="95"/>
+      <c r="AB27" s="95">
         <f>AVERAGEIF(AB4:AB23,"&gt;0")</f>
         <v>47.846153846153847</v>
       </c>
-      <c r="AC27" s="127"/>
-      <c r="AD27" s="128">
+      <c r="AC27" s="96"/>
+      <c r="AD27" s="97">
         <f>AVERAGEIF(AD4:AD23,"&gt;0")</f>
         <v>46.090909090909093</v>
       </c>
-      <c r="AE27" s="129"/>
-      <c r="AF27" s="128">
+      <c r="AE27" s="98"/>
+      <c r="AF27" s="97">
         <f>AVERAGEIF(AF4:AF23,"&gt;0")</f>
         <v>47.230769230769234</v>
       </c>
-      <c r="AG27" s="129"/>
-      <c r="AH27" s="128">
+      <c r="AG27" s="98"/>
+      <c r="AH27" s="97">
         <f>AVERAGEIF(AH4:AH23,"&gt;0")</f>
         <v>46.666666666666664</v>
       </c>
-      <c r="AI27" s="129"/>
-      <c r="AJ27" s="128"/>
-      <c r="AK27" s="129"/>
-      <c r="AL27" s="128">
+      <c r="AI27" s="98"/>
+      <c r="AJ27" s="97"/>
+      <c r="AK27" s="98"/>
+      <c r="AL27" s="97">
         <f>AVERAGEIF(AL4:AL23,"&gt;0")</f>
         <v>49.5</v>
       </c>
-      <c r="AM27" s="129"/>
-      <c r="AN27" s="128"/>
-      <c r="AO27" s="129"/>
-      <c r="AP27" s="128">
+      <c r="AM27" s="98"/>
+      <c r="AN27" s="97"/>
+      <c r="AO27" s="98"/>
+      <c r="AP27" s="97">
         <f>AVERAGEIF(AP4:AP23,"&gt;0")</f>
         <v>45.727272727272727</v>
       </c>
-      <c r="AQ27" s="129"/>
-      <c r="AR27" s="128">
+      <c r="AQ27" s="98"/>
+      <c r="AR27" s="97">
         <f>AVERAGEIF(AR4:AR23,"&gt;0")</f>
         <v>45.272727272727273</v>
       </c>
-      <c r="AS27" s="129"/>
-      <c r="AT27" s="130"/>
-      <c r="AU27" s="131"/>
-      <c r="AV27" s="131"/>
-      <c r="AW27" s="131"/>
-      <c r="AX27" s="131"/>
-      <c r="AY27" s="131"/>
+      <c r="AS27" s="98"/>
+      <c r="AT27" s="99"/>
+      <c r="AU27" s="100"/>
+      <c r="AV27" s="100"/>
+      <c r="AW27" s="100"/>
+      <c r="AX27" s="100"/>
+      <c r="AY27" s="100"/>
     </row>
     <row r="28" spans="1:56" x14ac:dyDescent="0.25">
       <c r="C28" s="11" t="s">
@@ -4962,6 +4962,47 @@
     <sortCondition descending="1" ref="AT4:AT26"/>
   </sortState>
   <mergeCells count="57">
+    <mergeCell ref="AJ1:AK1"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AL1:AM1"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AX2:AX3"/>
+    <mergeCell ref="AT1:AT3"/>
+    <mergeCell ref="AN1:AO1"/>
+    <mergeCell ref="AN2:AO2"/>
+    <mergeCell ref="AP1:AQ1"/>
+    <mergeCell ref="AP2:AQ2"/>
+    <mergeCell ref="AR1:AS1"/>
+    <mergeCell ref="AR2:AS2"/>
+    <mergeCell ref="AY2:AY3"/>
+    <mergeCell ref="AV2:AV3"/>
+    <mergeCell ref="AW2:AW3"/>
+    <mergeCell ref="AU2:AU3"/>
+    <mergeCell ref="AU1:AY1"/>
+    <mergeCell ref="AZ1:BD1"/>
+    <mergeCell ref="AZ2:AZ3"/>
+    <mergeCell ref="BA2:BA3"/>
+    <mergeCell ref="BB2:BB3"/>
+    <mergeCell ref="BC2:BC3"/>
+    <mergeCell ref="BD2:BD3"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="Z1:AA1"/>
+    <mergeCell ref="AB1:AC1"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="AH1:AI1"/>
     <mergeCell ref="AH2:AI2"/>
     <mergeCell ref="H1:I1"/>
@@ -4978,47 +5019,6 @@
     <mergeCell ref="AF2:AG2"/>
     <mergeCell ref="T1:U1"/>
     <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="AB1:AC1"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="AZ1:BD1"/>
-    <mergeCell ref="AZ2:AZ3"/>
-    <mergeCell ref="BA2:BA3"/>
-    <mergeCell ref="BB2:BB3"/>
-    <mergeCell ref="BC2:BC3"/>
-    <mergeCell ref="BD2:BD3"/>
-    <mergeCell ref="AY2:AY3"/>
-    <mergeCell ref="AV2:AV3"/>
-    <mergeCell ref="AW2:AW3"/>
-    <mergeCell ref="AU2:AU3"/>
-    <mergeCell ref="AU1:AY1"/>
-    <mergeCell ref="AJ1:AK1"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AL1:AM1"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AX2:AX3"/>
-    <mergeCell ref="AT1:AT3"/>
-    <mergeCell ref="AN1:AO1"/>
-    <mergeCell ref="AN2:AO2"/>
-    <mergeCell ref="AP1:AQ1"/>
-    <mergeCell ref="AP2:AQ2"/>
-    <mergeCell ref="AR1:AS1"/>
-    <mergeCell ref="AR2:AS2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>